<commit_message>
routine: 21 new postings, 22 checked-excluded (2026-09-19 19:15 UTC)
Added Draper Laboratory, MIT Lincoln Lab, Anduril (Quincy MA), Rivian,
SpaceX, Rocket Lab, RTX/Collins/Pratt & Whitney, Northrop Grumman,
Boston Dynamics, Berkshire Grey, and Emerson postings to the tracker.
Corrected two stale exclusions (Anduril, SpaceX) now that qualifying
postings exist. Staged draft application notes for 9 fully-verified
new postings. See ROUTINE-LOG.md for full details.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5EoD5Et8xvq7tTn5NuNWG
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J41"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1040,16 +1040,685 @@
         <v>US citizenship required. Cumulative GPA 2.9+ required. Spring 2027 window opens on USAJOBS in fall 2026.</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Microfabrication Industrial Engineering Co-Op (Group 08-35, Microelectronics Laboratory)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Industrial Engineering (Systems Eng/Ops Research/Manufacturing Eng/CS also accepted)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Jan–August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Lexington, MA</v>
+      </c>
+      <c r="F21">
+        <v>13</v>
+      </c>
+      <c r="G21" t="str">
+        <v>$24.50–$31.00/hr (2025 technical co-op rate; subject to review for 2027)</v>
+      </c>
+      <c r="H21" t="str">
+        <v>https://careers.ll.mit.edu/job/Lexington-Microfab-Industrial-Eng_-Co-Op-Microelectronics-Laboratory-%28Jan-August-2027%29-Group-08-35-MA-02420/1370647300/</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Yes — fetched directly, active Apply link, no closed/expired banner. Posted Aug 26, 2026.</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Requires US citizenship + eligibility for Secret-level DoD clearance. Sibling req 'Microfabrication Engineering Co-Op' (same Jan–Aug 2027 window, Group 08-35) also exists but wasn't separately fetched.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Systems Engineering Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Systems Design Engineering</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H22" t="str">
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Systems-Engineering-Co-Op--Spring-2027-_JR002882</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Partial — confirmed live via Draper's own job-listings page (draper.com/careers), posted ~1 week ago (~Sept 12, 2026). The Workday req page itself returned blank to automated fetch (JS-rendered) — verify live in-browser before applying.</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Found via Draper's first-party listings page, not an aggregator.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Electro-Mechanical Instrument Co-op (Spring 2027)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Hardware / Mechanical Engineering</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H23" t="str">
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Electro-Mechanical-Instrument-Co-op--Spring-2027-_JR002883-1</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Partial — confirmed live via Draper's own job-listings page (draper.com/careers), posted ~2 weeks ago (~Sept 5, 2026). Workday req page blocked automated fetch — verify live in-browser before applying.</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Found via Draper's first-party listings page, not an aggregator.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Amazon Robotics</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Industrial Development Engineer Intern/Co-op, ROBOTICS – 2027</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Industrial Engineering / Robotics Manufacturing &amp; Technical Operations</v>
+      </c>
+      <c r="D24" t="str">
+        <v>2027 (single req covers summer intern, spring co-op, and fall co-op placement — Spring 2027 placement is NOT guaranteed)</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Westborough, MA (also Arlington, VA and North Reading, MA)</v>
+      </c>
+      <c r="F24">
+        <v>35</v>
+      </c>
+      <c r="G24" t="str">
+        <v>$82,450/year (Amazon standard pay-transparency disclosure for this req)</v>
+      </c>
+      <c r="H24" t="str">
+        <v>https://www.amazon.jobs/en/jobs/10536817/industrial-development-engineer-intern-co-op-robotics-2027</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Yes — fetched directly, page loaded fully, role open. Caveat: the posting itself states this is a shared pipeline for summer/spring/fall 2027 placement, not a Spring-2027-only role — flagging this explicitly.</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Requires graduation between Dec 2026–Aug 2027. Prior req IDs for this role (e.g. 3088739, the 2026-cycle version) are confirmed dead (404).</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Winter 2027 Mechanical Engineer Co-op</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027 — same calendar window other employers call 'Spring 2027')</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Quincy, MA</v>
+      </c>
+      <c r="F25">
+        <v>8</v>
+      </c>
+      <c r="G25" t="str">
+        <v>$34–$50/hr</v>
+      </c>
+      <c r="H25" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236601007</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Winter 2027 Systems Engineer Co-op</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Quincy, MA</v>
+      </c>
+      <c r="F26">
+        <v>8</v>
+      </c>
+      <c r="G26" t="str">
+        <v>$40–$55/hr</v>
+      </c>
+      <c r="H26" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236599007</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Rivian</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Engineering Intern – Manufacturing Engineering (Spring 2027 Co-Op)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Normal, IL</v>
+      </c>
+      <c r="F27">
+        <v>1000</v>
+      </c>
+      <c r="G27" t="str">
+        <v>~$25–$51/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+      </c>
+      <c r="H27" t="str">
+        <v>https://careers.rivian.com/jobs/33784?lang=en-us</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Rivian</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Engineering Intern – Design for Reliability (Spring 2027 Co-Op)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Mechanical / Design Engineering</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Irvine, CA</v>
+      </c>
+      <c r="F28">
+        <v>2600</v>
+      </c>
+      <c r="G28" t="str">
+        <v>~$26–$45/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+      </c>
+      <c r="H28" t="str">
+        <v>https://careers.rivian.com/careers-home/jobs/33705?lang=en-us</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>SpaceX</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Spring 2027 Engineering Internship/Co-op</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Engineering (multi-discipline req)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Spring 2027 (start Jan or Mar 2027)</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Multiple US sites (incl. Bloomfield, CT — see posting for full list)</v>
+      </c>
+      <c r="G29" t="str">
+        <v>$28–$30/hr</v>
+      </c>
+      <c r="H29" t="str">
+        <v>https://job-boards.greenhouse.io/spacex/jobs/8616338002</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Yes — fetched directly on Greenhouse, live.</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Mechanical Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F30">
+        <v>2600</v>
+      </c>
+      <c r="G30" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H30" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7985634003</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Systems Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F31">
+        <v>2600</v>
+      </c>
+      <c r="G31" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H31" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987044003</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Collins Aerospace (RTX)</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Project Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Systems / Mechanical Engineering</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027, full-time)</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Windsor Locks, CT</v>
+      </c>
+      <c r="F32">
+        <v>90</v>
+      </c>
+      <c r="G32" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H32" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J32" t="str">
+        <v>~1.5 hrs from Boston.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Pratt &amp; Whitney (RTX)</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Production Support Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Mechanical / Manufacturing / Aerospace Engineering</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Middletown, CT</v>
+      </c>
+      <c r="F33">
+        <v>105</v>
+      </c>
+      <c r="G33" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H33" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-MIDDLETOWN-220A--Aircraft-Rd--BLDG-220A/Production-Support-Engineering-Co-op--Winter-Spring-2027-_01872654</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Partial — Workday page blocked automated fetch. Req ID and Sept 13, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J33" t="str">
+        <v>~1.5 hrs from Boston.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Certification Engineer Co-Op (Winter/Spring 2027, Onsite)</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Mechanical / Aerospace / Materials Science / Chemical Engineering</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul, two semesters)</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Winston-Salem, NC</v>
+      </c>
+      <c r="F34">
+        <v>700</v>
+      </c>
+      <c r="G34" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H34" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 16, 2026. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Cedar Rapids, IA</v>
+      </c>
+      <c r="F35">
+        <v>1130</v>
+      </c>
+      <c r="G35" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H35" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869080</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 15, 2026. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Structural Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Jamestown, ND</v>
+      </c>
+      <c r="F36">
+        <v>1500</v>
+      </c>
+      <c r="G36" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H36" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Structural-Engineering-Co-op--Winter-Spring-2027-_01873938</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 14, 2026. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Northrop Grumman</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2027 Spring Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Spring/Summer 2027 (Jan–Aug 2027)</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Chandler, AZ</v>
+      </c>
+      <c r="F37">
+        <v>2300</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Bachelor's $18.50–$33.50/hr; Master's $26.25–$41.50/hr</v>
+      </c>
+      <c r="H37" t="str">
+        <v>https://ngc.wd1.myworkdayjobs.com/Northrop_Grumman_External_Site/job/United-States-Arizona-Chandler/XMLNAME-2027-Spring-Mechanical-Engineering-Co-op---Chandler-AZ_R10249939</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Boston Dynamics</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Spring 2027 (Jan–Aug 2027, per search snippet)</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Waltham, MA</v>
+      </c>
+      <c r="F38">
+        <v>10</v>
+      </c>
+      <c r="G38" t="str">
+        <v>$30–$45/hr per search snippet; not independently confirmed via direct fetch</v>
+      </c>
+      <c r="H38" t="str">
+        <v>https://bostondynamics.wd1.myworkdayjobs.com/Boston_Dynamics/job/Waltham-Office-POST/Mechanical-Engineering-Co-Op_R2476</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Partial — Workday page returned empty content on two direct fetch attempts (JS-rendered/blocked). Season and pay sourced from search snippet only, not independently opened. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Boston metro (Waltham).</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Spring 2027 Hardware Quality Co-op</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Hardware / Quality Engineering</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F39">
+        <v>17</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H39" t="str">
+        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Boston metro (Bedford).</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Emerson</v>
+      </c>
+      <c r="B40" t="str">
+        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
+      </c>
+      <c r="C40" t="str">
+        <v>R&amp;D / Mechanical Engineering</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Cranberry Township, PA</v>
+      </c>
+      <c r="F40">
+        <v>570</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H40" t="str">
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Emerson</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Project Engineering Co-op – Spring 2027</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Project / Mechanical Engineering</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
+      </c>
+      <c r="F41">
+        <v>570</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H41" t="str">
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J41"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C37"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -1135,13 +1804,13 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Tesla / SpaceX / Apple / Google / Meta / Amazon Lab126 / NVIDIA</v>
+        <v>Tesla / Apple / Google / Meta / Amazon Lab126 / NVIDIA</v>
       </c>
       <c r="B8" t="str">
         <v>Various hardware/mechanical searches</v>
       </c>
       <c r="C8" t="str">
-        <v>No Winter 2026/Spring 2027-specific postings found for these disciplines (their volume is overwhelmingly Summer 2027); Apple's 'Hardware Undergrad Engineering' reqs appear evergreen with no season stated</v>
+        <v>No Winter 2026/Spring 2027-specific postings found for these disciplines (their volume is overwhelmingly Summer 2027); Apple's 'Hardware Undergrad Engineering' reqs appear evergreen with no season stated. NOTE (2026-09-19): SpaceX has since been found to have a genuine Spring 2027 posting — moved to `rows`; removed from this exclusion group.</v>
       </c>
     </row>
     <row r="9">
@@ -1174,45 +1843,298 @@
         <v>2027 Mechanical Engineer Intern; 2027 Manufacturing Engineer Intern (Boston, MA location available)</v>
       </c>
       <c r="C11" t="str">
-        <v>Confirmed Summer 2027 only, not Winter/Spring — excluded on season grounds despite the attractive Boston location</v>
+        <v>Confirmed Summer 2027 only, not Winter/Spring — excluded on season grounds despite the attractive Boston location. UPDATE (2026-09-19): a separate 'Winter 2027' cohort (effectively Jan–Aug 2027) was found live at Quincy, MA — Mechanical and Systems Engineer Co-ops moved to `rows`.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Draper Laboratory (Cambridge, MA)</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B12" t="str">
-        <v>Current-openings portal (redirects to Workday)</v>
+        <v>Winter 2027 Electrical Engineer Co-op (Quincy, MA)</v>
       </c>
       <c r="C12" t="str">
-        <v>Draper's own site confirms co-ops run fall/spring, but the live openings portal is a JS-rendered Workday page that blocked automated fetch — no specific Spring 2027 req could be confirmed. Worth checking manually (this would be a very close Boston option).</v>
+        <v>2026-09-19: Confirmed open/live at the same Quincy, MA site as the Mechanical/Systems co-ops added to `rows`, but excluded here — electrical engineering is outside Hamza's target disciplines.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+        <v>Draper Laboratory (Cambridge, MA)</v>
       </c>
       <c r="B13" t="str">
-        <v>careers.ll.mit.edu search</v>
+        <v>Current-openings portal (redirects to Workday)</v>
       </c>
       <c r="C13" t="str">
-        <v>Only Summer 2026 reqs found (e.g. Mechanical/Optical Engineering SRP Intern) — no Spring 2027-specific postings live yet as of search date. Also close to Boston if it opens later.</v>
+        <v>Draper's own site confirms co-ops run fall/spring, but the live openings portal is a JS-rendered Workday page that blocked automated fetch — no specific Spring 2027 req could be confirmed. Worth checking manually (this would be a very close Boston option).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>careers.ll.mit.edu search</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Only Summer 2026 reqs found (e.g. Mechanical/Optical Engineering SRP Intern) — no Spring 2027-specific postings live yet as of search date. Also close to Boston if it opens later.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>Lockheed Martin</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <v>lockheedmartinjobs.com search for 'Spring 2027'</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C15" t="str">
         <v>Only found Spring 2026 co-ops (already past); direct search-jobs URL 404'd on retry — no confirmed Spring 2027 req found this session</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Lynn CNC Trainee Co-Op; Lynn Carpentry Trainee Co-Op; CNC Programmer Co-op Fall 2026; Manufacturing Engineering Co-op Spring 2027; Engines Engineering Co-op Spring 2027 (Computer/Software track)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-09-19: All previously-known reqs re-checked directly — now return 'no longer posted' or HTTP 410 Gone. One general Engines Eng Co-op (Cincinnati/Lynn) exists on an aggregator but is flagged EXPIRED there; no live company-site URL found. Worth periodic re-checking of careers.geaerospace.com/global/en/lynn.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Sensor Electrical Engineering Co-op (Spring 2027); Optics-Physics Sensor Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2026-09-19: Both confirmed live/open on draper.com's own listings page but excluded — electrical/optics engineering discipline, outside Hamza's target list. (Systems Engineering Co-Op and Electro-Mechanical Instrument Co-op from the same posting batch DID qualify and were added to `rows`.)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Full careers.symbotic.com/careers/jobs listing + student/grad opportunities page</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2026-09-19 re-check: still zero internship/co-op postings; only 'Skillbridge' military-transition fellowships found under a co-op search filter, wrong program entirely.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Amazon Robotics (Westborough, MA)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Old job ID 3088739 (2026-cycle Industrial Engineer Intern/Co-op)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>2026-09-19: confirmed HTTP 404, dead. Superseded by new req 10536817 (2027 cycle), which was added to `rows` with a season caveat.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>BAE Systems (Nashua, NH)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Systems Eng Intern III; Software Eng Intern I/III; EE/CE/RF Intern III; Mechanical Engineering Intern III; Industrial Engineering Co-Op (Fall Semester 2026)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>2026-09-19: All current postings are explicitly Summer 2027 — wrong season. The one Fall 2026 posting from a prior check now returns HTTP 410 Gone.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Textron Aviation</v>
+      </c>
+      <c r="B21" t="str">
+        <v>'Spring Co-Op – Electronics Modules Engineer'</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2026-09-19 re-check: still cannot confirm which year this posting covers — careers.textron.com remains JS-rendered/blocked to automated fetch; only aggregator mirror found is a stale 2024 cache. No other qualifying Spring 2027/Winter 2026 postings found at Textron, Bell, or Textron Systems in target disciplines.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>General Dynamics Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>'2027 Spring Engineering Co-Op Trainee'</v>
+      </c>
+      <c r="C22" t="str">
+        <v>2026-09-19: Search evidence (job-aggregator snapshot, distinct from the already-past Spring 2026 cohort) suggests a new Spring 2027 cycle exists, but both the aggregator page and the official portals (ebcareers.com, careers-gdeb.icims.com) blocked direct fetch — no verifiable specific req link found, so not added to `rows`. Worth checking ebcareers.com/careers-gdeb.icims.com directly in-browser next run.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Lockheed Martin / Sikorsky (Stratford, CT)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>lockheedmartinjobs.com legacy links; new careers.lockheedmartin.com search</v>
+      </c>
+      <c r="C23" t="str">
+        <v>2026-09-19: legacy job-search URLs now 404 (site appears migrated); new careers site's search endpoint also unreachable via fetch. No Spring 2027 co-op/internship located this session.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>L3Harris</v>
+      </c>
+      <c r="B24" t="str">
+        <v>'Intern, Software Engineer Spring 2027' (Greenville, TX); 'Electrical Engineer Intern B Spring Co-op'</v>
+      </c>
+      <c r="C24" t="str">
+        <v>2026-09-19: Only software/electrical Spring 2027 co-ops found — discipline mismatch, no mechanical/structural/systems reqs located.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Leidos</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Spring 2027 co-op search</v>
+      </c>
+      <c r="C25" t="str">
+        <v>2026-09-19: Only software/computer engineering co-ops found (Reston VA, Bethesda MD) — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Rapid Prototyping Aero/Mech Co-Op</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2026-09-19: Confirmed open via direct fetch, but posting states 'Fall 2026' only with no stated extension into winter/spring — excluded on season grounds. (A separate Microfabrication Industrial Eng Co-Op, Jan–Aug 2027, DID qualify and was added to `rows`.)</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Mechanical Engineering Intern (req R2495)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2026-09-19: Season unstated/unclear on this specific req — excluded. (A separate 'Mechanical Engineering Co-Op' req, Spring 2027, DID have a stated season and was added to `rows` as Partial.)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Eaton</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Co-op Design Engineering (Spring 2027), Jackson, MS</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2026-09-19: A Spring 2027 co-op wave appears to exist generally ($22–28/hr range per search), but the specific link found (fairygodboss listing) now 404s and no working replacement URL could be located — not added without a verifiable link. Worth re-checking.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Cummins (Columbus, IN)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Career board general search</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2026-09-19 re-check: career board explicitly shows 'No jobs currently found'; next cycle (Summer 2027) not expected to post until ~Dec 2026.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>iRobot / Vicarious Surgical / Desktop Metal / Markforged / Vecna Robotics / Locus Robotics / PTC / Analog Devices</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Careers pages and Greenhouse boards for Boston-area robotics/hardware companies</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2026-09-19: No live Winter 2026/Spring 2027 co-op or intern postings found. iRobot: only an already-past Spring 2026 posting. Vicarious Surgical: careers page/Greenhouse errored out. Desktop Metal/Markforged: Greenhouse board has zero internships posted. Vecna: no listings. Locus Robotics: only Summer 2026 and an apparently-expired Fall 2026 posting. PTC: only standard Summer program. Analog Devices: Spring/Fall co-ops are a standing program but no Spring 2027 req posted yet (expected ~Oct/Nov 2026).</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Caterpillar / John Deere / Honeywell / 3M / GM / Ford / Stellantis / Lucid Motors / Stanley Black &amp; Decker</v>
+      </c>
+      <c r="B31" t="str">
+        <v>General co-op/intern search, target disciplines</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2026-09-19: Confirmed postings found are Summer 2027 only, or (Caterpillar) the application window already closed (Aug 14, 2026). No Winter 2026/Spring 2027-specific reqs located.</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Rockwell Automation / Parker Hannifin</v>
+      </c>
+      <c r="B32" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2026-09-19: No specific postings found — only general recruiting-season descriptions.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Danaher</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Product Development Engineering Co-op (Jan 2027 start)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026-09-19: Confirmed posting exists but is located in Vancouver, BC, Canada — excluded on location (outside the US), not season.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Firefly Aerospace / Sierra Space</v>
+      </c>
+      <c r="B34" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2026-09-19: Only Summer 2026/general 'year-round' postings found; Spring 2027 cycle not live yet (Sierra Space's next cycle not expected until ~Sept 2026 onward).</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>MathWorks (Natick, MA)</v>
+      </c>
+      <c r="B35" t="str">
+        <v>EDG internship listing</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026-09-19: Listing mentions 'Spring, Summer, Fall' cohorts generically but carries no year/season tag on the specific req — appears evergreen, could not confirm as Spring 2027.</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>CIRTEC Medical</v>
+      </c>
+      <c r="B36" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2026-09-19: Only generic/Summer, California-based postings found — nothing Winter 2026/Spring 2027 or Boston-area.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B37" t="str">
+        <v>'2027 Mechanical/Electrical Engineer Intern' (lists Boston as a possible site)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026-09-19: Appears to be part of the Summer 2027 program (12-week internship, application window opening ~Sept 2026); could not access job-boards.greenhouse.io/rsinternboard directly (404) to confirm season wording — excluded pending clearer evidence.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 13 checked-excluded (2026-09-20 00:49 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019veCTMNk5teVT9vZ5nSkSz
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J46"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1162,7 +1162,7 @@
         <v>https://www.amazon.jobs/en/jobs/10536817/industrial-development-engineer-intern-co-op-robotics-2027</v>
       </c>
       <c r="I24" t="str">
-        <v>Yes — fetched directly, page loaded fully, role open. Caveat: the posting itself states this is a shared pipeline for summer/spring/fall 2027 placement, not a Spring-2027-only role — flagging this explicitly.</v>
+        <v>Yes — fetched directly, page loaded fully, role open. UPDATE (2026-09-20): posting text now explicitly reads 'Robotics Industrial Engineer 2027 summer intern, spring co-op, and fall co-op roles' — confirms Spring 2027 co-op is one of the terms this req covers (previously ambiguous).</v>
       </c>
       <c r="J24" t="str">
         <v>Requires graduation between Dec 2026–Aug 2027. Prior req IDs for this role (e.g. 3088739, the 2026-cycle version) are confirmed dead (404).</v>
@@ -1170,380 +1170,380 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Anduril Industries</v>
+        <v>Formlabs</v>
       </c>
       <c r="B25" t="str">
-        <v>Winter 2027 Mechanical Engineer Co-op</v>
+        <v>Mechanical Engineering Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C25" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Hardware Engineering</v>
       </c>
       <c r="D25" t="str">
-        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027 — same calendar window other employers call 'Spring 2027')</v>
+        <v>Winter/Spring 2027 (January–April)</v>
       </c>
       <c r="E25" t="str">
-        <v>Quincy, MA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F25">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G25" t="str">
-        <v>$34–$50/hr</v>
+        <v>$1,575–$1,950/week (salaried, full-time)</v>
       </c>
       <c r="H25" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236601007</v>
+        <v>https://careers.formlabs.com/job/8130829/apply/?gh_jid=8130829</v>
       </c>
       <c r="I25" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+        <v>Yes — fetched directly, page live, season/location/pay confirmed in posting text.</v>
       </c>
       <c r="J25" t="str">
-        <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
+        <v>Boston metro. Portfolio of prior engineering work required — application not considered without one.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Anduril Industries</v>
+        <v>Formlabs</v>
       </c>
       <c r="B26" t="str">
-        <v>Winter 2027 Systems Engineer Co-op</v>
+        <v>Hardware Systems Integration Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C26" t="str">
-        <v>Systems Engineering</v>
+        <v>Hardware / Electro-Mechanical Engineering</v>
       </c>
       <c r="D26" t="str">
-        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+        <v>Winter/Spring 2027 (January–April)</v>
       </c>
       <c r="E26" t="str">
-        <v>Quincy, MA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F26">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>$40–$55/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H26" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236599007</v>
+        <v>https://careers.formlabs.com/job/8172004/apply/?gh_jid=8172004</v>
       </c>
       <c r="I26" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+        <v>Yes — fetched directly, page live, title/season/location confirmed in posting text.</v>
       </c>
       <c r="J26" t="str">
-        <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
+        <v>Boston metro. Portfolio of prior engineering work required.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Rivian</v>
+        <v>Eaton</v>
       </c>
       <c r="B27" t="str">
-        <v>Engineering Intern – Manufacturing Engineering (Spring 2027 Co-Op)</v>
+        <v>ETO Engineering Co-op</v>
       </c>
       <c r="C27" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical, Industrial, or Electrical Engineering</v>
       </c>
       <c r="D27" t="str">
-        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+        <v>Fall 2026 or Spring 2027 (posting states either start date is acceptable)</v>
       </c>
       <c r="E27" t="str">
-        <v>Normal, IL</v>
+        <v>Syracuse, NY</v>
       </c>
       <c r="F27">
-        <v>1000</v>
+        <v>260</v>
       </c>
       <c r="G27" t="str">
-        <v>~$25–$51/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+        <v>$24.92/hr</v>
       </c>
       <c r="H27" t="str">
-        <v>https://careers.rivian.com/jobs/33784?lang=en-us</v>
+        <v>https://eaton.eightfold.ai/careers/job/687236797540</v>
       </c>
       <c r="I27" t="str">
-        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+        <v>Yes — verified via Eaton's own public Eightfold job-board API directly (the rendered page is JS-heavy); record shows isPrivate: false (publicly listed/active), created 2026-05-21, last updated 2026-08-12.</v>
       </c>
       <c r="J27" t="str">
-        <v/>
+        <v>Min GPA 2.8. No visa sponsorship (no CPT/OPT/H-1B support). Must live within ~50 mi of Syracuse, NY — no relocation assistance.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Rivian</v>
+        <v>Reframe Systems</v>
       </c>
       <c r="B28" t="str">
-        <v>Engineering Intern – Design for Reliability (Spring 2027 Co-Op)</v>
+        <v>Mechanical Engineer (Spring 2027 Co-op)</v>
       </c>
       <c r="C28" t="str">
-        <v>Mechanical / Design Engineering</v>
+        <v>Mechanical Engineering (CAD, welding, machining, fixturing/workcell design)</v>
       </c>
       <c r="D28" t="str">
-        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E28" t="str">
-        <v>Irvine, CA</v>
+        <v>Andover, MA (HQ) / FAB1 microfactory, Billerica, MA</v>
       </c>
       <c r="F28">
-        <v>2600</v>
+        <v>23</v>
       </c>
       <c r="G28" t="str">
-        <v>~$26–$45/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H28" t="str">
-        <v>https://careers.rivian.com/careers-home/jobs/33705?lang=en-us</v>
+        <v>https://jobs.ashbyhq.com/reframesystems/f5275832-8373-4971-b5f6-6aaececcb061</v>
       </c>
       <c r="I28" t="str">
-        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+        <v>Yes — verified via Reframe Systems' own public Ashby job-board API directly; record shows isListed: true, publishedAt 2026-08-05, exact worksite address (30 Lowell Junction Rd, Andover MA).</v>
       </c>
       <c r="J28" t="str">
-        <v/>
+        <v>Small modular-construction/robotics-manufacturing startup, Boston metro (Andover/Billerica). Shop-based role — CAD, welding, machining, fixturing.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>SpaceX</v>
+        <v>General Dynamics Electric Boat</v>
       </c>
       <c r="B29" t="str">
-        <v>Spring 2027 Engineering Internship/Co-op</v>
+        <v>2027 Spring Engineering CO-OP Trainee</v>
       </c>
       <c r="C29" t="str">
-        <v>Engineering (multi-discipline req)</v>
+        <v>Mechanical / Structural / Aerospace-Aeronautical / Systems / Naval Architecture / Industrial / Electromechanical / Robotics Engineering (multi-discipline req)</v>
       </c>
       <c r="D29" t="str">
-        <v>Spring 2027 (start Jan or Mar 2027)</v>
+        <v>Spring of 2027 (per listing summary)</v>
       </c>
       <c r="E29" t="str">
-        <v>Multiple US sites (incl. Bloomfield, CT — see posting for full list)</v>
+        <v>Groton, CT (co-ops also placed in New London/North Stonington CT, North Kingstown/Newport RI)</v>
+      </c>
+      <c r="F29">
+        <v>90</v>
       </c>
       <c r="G29" t="str">
-        <v>$28–$30/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H29" t="str">
-        <v>https://job-boards.greenhouse.io/spacex/jobs/8616338002</v>
+        <v>https://jobs.buildsubmarines.com/job/601496955</v>
       </c>
       <c r="I29" t="str">
-        <v>Yes — fetched directly on Greenhouse, live.</v>
+        <v>Partial — found via GD Electric Boat's own dedicated recruiting site (jobs.buildsubmarines.com) with a specific req ID, mirroring the pattern of GD's known 2026 cycle req. The page itself is behind a Cloudflare bot-check wall — blocked on WebFetch, curl w/ browser UA, and a reader-proxy fetch, all returning a security-verification/CAPTCHA screen. Could not independently confirm live/open status or the exact discipline breakdown. Verify live in-browser before applying.</v>
       </c>
       <c r="J29" t="str">
-        <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
+        <v>Was flagged 'worth re-checking' in the prior run; upgraded from 'no verifiable link' to 'specific req ID found, still blocked'.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Rocket Lab</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B30" t="str">
-        <v>Mechanical Engineering Intern, Spring 2027</v>
+        <v>Winter 2027 Mechanical Engineer Co-op</v>
       </c>
       <c r="C30" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D30" t="str">
-        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027 — same calendar window other employers call 'Spring 2027')</v>
       </c>
       <c r="E30" t="str">
-        <v>Long Beach, CA</v>
+        <v>Quincy, MA</v>
       </c>
       <c r="F30">
-        <v>2600</v>
+        <v>8</v>
       </c>
       <c r="G30" t="str">
-        <v>$28/hr</v>
+        <v>$34–$50/hr</v>
       </c>
       <c r="H30" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7985634003</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236601007</v>
       </c>
       <c r="I30" t="str">
         <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J30" t="str">
-        <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
+        <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Rocket Lab</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B31" t="str">
-        <v>Systems Engineering Intern, Spring 2027</v>
+        <v>Winter 2027 Systems Engineer Co-op</v>
       </c>
       <c r="C31" t="str">
         <v>Systems Engineering</v>
       </c>
       <c r="D31" t="str">
-        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
       </c>
       <c r="E31" t="str">
-        <v>Long Beach, CA</v>
+        <v>Quincy, MA</v>
       </c>
       <c r="F31">
-        <v>2600</v>
+        <v>8</v>
       </c>
       <c r="G31" t="str">
-        <v>$28/hr</v>
+        <v>$40–$55/hr</v>
       </c>
       <c r="H31" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987044003</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236599007</v>
       </c>
       <c r="I31" t="str">
         <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J31" t="str">
-        <v/>
+        <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Collins Aerospace (RTX)</v>
+        <v>Rivian</v>
       </c>
       <c r="B32" t="str">
-        <v>Project Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Engineering Intern – Manufacturing Engineering (Spring 2027 Co-Op)</v>
       </c>
       <c r="C32" t="str">
-        <v>Systems / Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D32" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027, full-time)</v>
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
       </c>
       <c r="E32" t="str">
-        <v>Windsor Locks, CT</v>
+        <v>Normal, IL</v>
       </c>
       <c r="F32">
-        <v>90</v>
+        <v>1000</v>
       </c>
       <c r="G32" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>~$25–$51/hr per third-party aggregator; not independently confirmed via direct fetch</v>
       </c>
       <c r="H32" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
+        <v>https://careers.rivian.com/jobs/33784?lang=en-us</v>
       </c>
       <c r="I32" t="str">
-        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
       </c>
       <c r="J32" t="str">
-        <v>~1.5 hrs from Boston.</v>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Pratt &amp; Whitney (RTX)</v>
+        <v>Rivian</v>
       </c>
       <c r="B33" t="str">
-        <v>Production Support Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Engineering Intern – Design for Reliability (Spring 2027 Co-Op)</v>
       </c>
       <c r="C33" t="str">
-        <v>Mechanical / Manufacturing / Aerospace Engineering</v>
+        <v>Mechanical / Design Engineering</v>
       </c>
       <c r="D33" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
       </c>
       <c r="E33" t="str">
-        <v>Middletown, CT</v>
+        <v>Irvine, CA</v>
       </c>
       <c r="F33">
-        <v>105</v>
+        <v>2600</v>
       </c>
       <c r="G33" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>~$26–$45/hr per third-party aggregator; not independently confirmed via direct fetch</v>
       </c>
       <c r="H33" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-MIDDLETOWN-220A--Aircraft-Rd--BLDG-220A/Production-Support-Engineering-Co-op--Winter-Spring-2027-_01872654</v>
+        <v>https://careers.rivian.com/careers-home/jobs/33705?lang=en-us</v>
       </c>
       <c r="I33" t="str">
-        <v>Partial — Workday page blocked automated fetch. Req ID and Sept 13, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
       </c>
       <c r="J33" t="str">
-        <v>~1.5 hrs from Boston.</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>SpaceX</v>
       </c>
       <c r="B34" t="str">
-        <v>Certification Engineer Co-Op (Winter/Spring 2027, Onsite)</v>
+        <v>Spring 2027 Engineering Internship/Co-op</v>
       </c>
       <c r="C34" t="str">
-        <v>Mechanical / Aerospace / Materials Science / Chemical Engineering</v>
+        <v>Engineering (multi-discipline req)</v>
       </c>
       <c r="D34" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul, two semesters)</v>
+        <v>Spring 2027 (start Jan or Mar 2027)</v>
       </c>
       <c r="E34" t="str">
-        <v>Winston-Salem, NC</v>
-      </c>
-      <c r="F34">
-        <v>700</v>
+        <v>Multiple US sites (incl. Bloomfield, CT — see posting for full list)</v>
       </c>
       <c r="G34" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>$28–$30/hr</v>
       </c>
       <c r="H34" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
+        <v>https://job-boards.greenhouse.io/spacex/jobs/8616338002</v>
       </c>
       <c r="I34" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 16, 2026. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Greenhouse, live.</v>
       </c>
       <c r="J34" t="str">
-        <v/>
+        <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B35" t="str">
-        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Mechanical Engineering Intern, Spring 2027</v>
       </c>
       <c r="C35" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D35" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E35" t="str">
-        <v>Cedar Rapids, IA</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F35">
-        <v>1130</v>
+        <v>2600</v>
       </c>
       <c r="G35" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>$28/hr</v>
       </c>
       <c r="H35" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869080</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7985634003</v>
       </c>
       <c r="I35" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 15, 2026. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J35" t="str">
-        <v/>
+        <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B36" t="str">
-        <v>Structural Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Systems Engineering Intern, Spring 2027</v>
       </c>
       <c r="C36" t="str">
-        <v>Structural Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D36" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E36" t="str">
-        <v>Jamestown, ND</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F36">
-        <v>1500</v>
+        <v>2600</v>
       </c>
       <c r="G36" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>$28/hr</v>
       </c>
       <c r="H36" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Structural-Engineering-Co-op--Winter-Spring-2027-_01873938</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987044003</v>
       </c>
       <c r="I36" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 14, 2026. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -1551,127 +1551,127 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Northrop Grumman</v>
+        <v>Collins Aerospace (RTX)</v>
       </c>
       <c r="B37" t="str">
-        <v>2027 Spring Mechanical Engineering Co-op</v>
+        <v>Project Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C37" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Systems / Mechanical Engineering</v>
       </c>
       <c r="D37" t="str">
-        <v>Spring/Summer 2027 (Jan–Aug 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027, full-time)</v>
       </c>
       <c r="E37" t="str">
-        <v>Chandler, AZ</v>
+        <v>Windsor Locks, CT</v>
       </c>
       <c r="F37">
-        <v>2300</v>
+        <v>90</v>
       </c>
       <c r="G37" t="str">
-        <v>Bachelor's $18.50–$33.50/hr; Master's $26.25–$41.50/hr</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H37" t="str">
-        <v>https://ngc.wd1.myworkdayjobs.com/Northrop_Grumman_External_Site/job/United-States-Arizona-Chandler/XMLNAME-2027-Spring-Mechanical-Engineering-Co-op---Chandler-AZ_R10249939</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
       </c>
       <c r="I37" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J37" t="str">
-        <v/>
+        <v>~1.5 hrs from Boston.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Boston Dynamics</v>
+        <v>Pratt &amp; Whitney (RTX)</v>
       </c>
       <c r="B38" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Production Support Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C38" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Manufacturing / Aerospace Engineering</v>
       </c>
       <c r="D38" t="str">
-        <v>Spring 2027 (Jan–Aug 2027, per search snippet)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E38" t="str">
-        <v>Waltham, MA</v>
+        <v>Middletown, CT</v>
       </c>
       <c r="F38">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="G38" t="str">
-        <v>$30–$45/hr per search snippet; not independently confirmed via direct fetch</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H38" t="str">
-        <v>https://bostondynamics.wd1.myworkdayjobs.com/Boston_Dynamics/job/Waltham-Office-POST/Mechanical-Engineering-Co-Op_R2476</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-MIDDLETOWN-220A--Aircraft-Rd--BLDG-220A/Production-Support-Engineering-Co-op--Winter-Spring-2027-_01872654</v>
       </c>
       <c r="I38" t="str">
-        <v>Partial — Workday page returned empty content on two direct fetch attempts (JS-rendered/blocked). Season and pay sourced from search snippet only, not independently opened. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Req ID and Sept 13, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J38" t="str">
-        <v>Boston metro (Waltham).</v>
+        <v>~1.5 hrs from Boston.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Berkshire Grey</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B39" t="str">
-        <v>Spring 2027 Hardware Quality Co-op</v>
+        <v>Certification Engineer Co-Op (Winter/Spring 2027, Onsite)</v>
       </c>
       <c r="C39" t="str">
-        <v>Hardware / Quality Engineering</v>
+        <v>Mechanical / Aerospace / Materials Science / Chemical Engineering</v>
       </c>
       <c r="D39" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan–Jul, two semesters)</v>
       </c>
       <c r="E39" t="str">
-        <v>Bedford, MA</v>
+        <v>Winston-Salem, NC</v>
       </c>
       <c r="F39">
-        <v>17</v>
+        <v>700</v>
       </c>
       <c r="G39" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H39" t="str">
-        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
       </c>
       <c r="I39" t="str">
-        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 16, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J39" t="str">
-        <v>Boston metro (Bedford).</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Emerson</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B40" t="str">
-        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C40" t="str">
-        <v>R&amp;D / Mechanical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D40" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E40" t="str">
-        <v>Cranberry Township, PA</v>
+        <v>Cedar Rapids, IA</v>
       </c>
       <c r="F40">
-        <v>570</v>
+        <v>1130</v>
       </c>
       <c r="G40" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H40" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869080</v>
       </c>
       <c r="I40" t="str">
-        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 15, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J40" t="str">
         <v/>
@@ -1679,46 +1679,206 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Emerson</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B41" t="str">
-        <v>Project Engineering Co-op – Spring 2027</v>
+        <v>Structural Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C41" t="str">
-        <v>Project / Mechanical Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D41" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E41" t="str">
-        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
+        <v>Jamestown, ND</v>
       </c>
       <c r="F41">
-        <v>570</v>
+        <v>1500</v>
       </c>
       <c r="G41" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H41" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Structural-Engineering-Co-op--Winter-Spring-2027-_01873938</v>
       </c>
       <c r="I41" t="str">
-        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 14, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J41" t="str">
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Northrop Grumman</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2027 Spring Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Spring/Summer 2027 (Jan–Aug 2027)</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Chandler, AZ</v>
+      </c>
+      <c r="F42">
+        <v>2300</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Bachelor's $18.50–$33.50/hr; Master's $26.25–$41.50/hr</v>
+      </c>
+      <c r="H42" t="str">
+        <v>https://ngc.wd1.myworkdayjobs.com/Northrop_Grumman_External_Site/job/United-States-Arizona-Chandler/XMLNAME-2027-Spring-Mechanical-Engineering-Co-op---Chandler-AZ_R10249939</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Boston Dynamics</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Spring 2027 (Jan–Aug 2027, per search snippet)</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Waltham, MA</v>
+      </c>
+      <c r="F43">
+        <v>10</v>
+      </c>
+      <c r="G43" t="str">
+        <v>$30–$45/hr per search snippet; not independently confirmed via direct fetch</v>
+      </c>
+      <c r="H43" t="str">
+        <v>https://bostondynamics.wd1.myworkdayjobs.com/Boston_Dynamics/job/Waltham-Office-POST/Mechanical-Engineering-Co-Op_R2476</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Partial — Workday page returned empty content on two direct fetch attempts (JS-rendered/blocked). Season and pay sourced from search snippet only, not independently opened. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Boston metro (Waltham).</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Spring 2027 Hardware Quality Co-op</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Hardware / Quality Engineering</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F44">
+        <v>17</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H44" t="str">
+        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Boston metro (Bedford).</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Emerson</v>
+      </c>
+      <c r="B45" t="str">
+        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
+      </c>
+      <c r="C45" t="str">
+        <v>R&amp;D / Mechanical Engineering</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Cranberry Township, PA</v>
+      </c>
+      <c r="F45">
+        <v>570</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H45" t="str">
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Emerson</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Project Engineering Co-op – Spring 2027</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Project / Mechanical Engineering</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
+      </c>
+      <c r="F46">
+        <v>570</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Not stated (aggregator only)</v>
+      </c>
+      <c r="H46" t="str">
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J46"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C50"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -2132,9 +2292,152 @@
         <v>2026-09-19: Appears to be part of the Summer 2027 program (12-week internship, application window opening ~Sept 2026); could not access job-boards.greenhouse.io/rsinternboard directly (404) to confirm season wording — excluded pending clearer evidence.</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Textron Aviation</v>
+      </c>
+      <c r="B38" t="str">
+        <v>'Spring Co-Op – Electronics Modules Engineer'</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026-09-20 re-check: no change. careers.textron.com confirmed to be a Nuxt.js SPA (empty shell on direct fetch, API endpoint redirects back to shell). Aggregator mirror (JobzMall) shows a stale 2024 posting for this exact title/location (Wichita, KS) — likely a recycled listing page, not a live 2027 req. Still cannot confirm year.</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>RTX Massachusetts sites (Andover / Tewksbury)</v>
+      </c>
+      <c r="B39" t="str">
+        <v>careers.rtx.com site search for MA-located Winter/Spring 2027 co-ops</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026-09-20: No qualifying co-op found — only a Summer 2027 internship (not co-op) and full-time roles at MA sites. All confirmed Winter/Spring 2027 co-op reqs remain at Jamestown ND and Cedar Rapids IA (already in `rows`), none in MA.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Analog Devices / Sierra Space / Danaher (US) / Caterpillar</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026-09-20: No change — nothing new surfaced; consistent with prior 'not yet posted' finding.</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Olympus (Westborough, MA)</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026-09-20: Only directly-openable listing was a Jan–June 2026 cohort, confirmed CLOSED ('no longer accepting applications'). Aggregator text mentions a possible 'Jan–June 2027' version but could not be independently verified (source JS-rendered, API query 404'd) — excluded pending better verification.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Alloy Enterprises (Burlington, MA)</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Co-op board (Thermal Design Engineer, Mechanical Engineer)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026-09-20: Only Fall 2026 and Spring 2026 (already past) co-op reqs found; no Spring 2027 posted yet.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Commonwealth Fusion Systems (Devens, MA)</v>
+      </c>
+      <c r="B43" t="str">
+        <v>jobs.lever.co/cfsenergy board directly</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026-09-20: Zero internship/co-op postings currently listed (full-time reqs only). Previously-found Fall 2026 and Spring 2026 co-op listings are gone from the live board.</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Engines Engineering Co-op (R5029619), Manufacturing Engineering Co-op (R5030077)</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026-09-20 re-check: both confirmed dead ('no longer posted' / HTTP 410). Still no live Spring 2027 co-op found at Lynn or elsewhere — no change from prior run.</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Teradyne (North Reading, MA)</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C45" t="str">
+        <v>2026-09-20: Only a Spring 2026 (already past) cohort found; no Spring 2027 posted yet.</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Vicor (Andover, MA)</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Full careers site</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2026-09-20: No co-op/internship postings found for any season — full-time roles only.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Co-Op, New Product Development Engineering; Software Eng Co-op; Automation Developer Co-op</v>
+      </c>
+      <c r="C47" t="str">
+        <v>2026-09-20: Only Spring 2026 (already past) postings confirmed; the NPD Engineering co-op page returned HTTP 503 on two attempts — could not confirm season, excluded.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>iRobot (Bedford, MA)</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Full careers site</v>
+      </c>
+      <c r="C48" t="str">
+        <v>2026-09-20: No current Spring 2027 postings found — only historical 2022 listings and older closed Workday reqs.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Vicarious Surgical (Waltham, MA)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Full careers site</v>
+      </c>
+      <c r="C49" t="str">
+        <v>2026-09-20 re-check: no current Spring 2027 postings; most recent was a January 2026 Mechanical Engineering Co-Op (already past).</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Apptronik / Figure AI / Agility Robotics</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Mechanical/hardware internship search</v>
+      </c>
+      <c r="C50" t="str">
+        <v>2026-09-20: No Winter 2026/Spring 2027 mechanical postings found. One apparent lead (Figure AI 'Hardware Reliability Intern') turned out on direct fetch to be titled Summer 2026 and is closed/removed.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new posting, 18 checked-excluded (2026-09-20 06:57 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013dLYMmjrNfRYPcLXVSEne5
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J47"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1869,16 +1869,48 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Mechanical Engineer Intern</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Spring 2027 (Jan–Apr/May)</v>
+      </c>
+      <c r="E47" t="str">
+        <v>South San Francisco, CA (or Dallas, TX)</v>
+      </c>
+      <c r="F47">
+        <v>2700</v>
+      </c>
+      <c r="G47" t="str">
+        <v>~$60k–$70k annualized (third-party estimate, not stated on posting)</v>
+      </c>
+      <c r="H47" t="str">
+        <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
+      </c>
+      <c r="J47" t="str">
+        <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J46"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J47"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C66"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -2435,9 +2467,185 @@
         <v>2026-09-20: No Winter 2026/Spring 2027 mechanical postings found. One apparent lead (Figure AI 'Hardware Reliability Intern') turned out on direct fetch to be titled Summer 2026 and is closed/removed.</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Engines Eng Co-op R5029619 (dead), Manufacturing Eng Co-op R5030077 (HTTP 410), general Engines Eng Co-op — Lynn/Evendale (aggregator: EXPIRED), Lynn CNC Trainee Co-Op R5034331 (dead)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>2026-09-20 ~06:57 UTC re-check: all four known reqs confirmed dead ('no longer posted' / HTTP 410 / EXPIRED). No live Spring 2027 mechanical/manufacturing req found anywhere at GE Aerospace this pass.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Analog Devices</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Spring/Fall mechanical co-op search</v>
+      </c>
+      <c r="C52" t="str">
+        <v>2026-09-20 ~06:57 UTC: still not posted; search summary indicates Summer 2027/2028-wave postings expected ~Oct/Nov 2026. No change.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Caterpillar</v>
+      </c>
+      <c r="B53" t="str">
+        <v>r0000380501 '2027 Engineering Corporate Internship Program – Materials', r0000384650 '2027 Summer Corporate Intern – Engineering'</v>
+      </c>
+      <c r="C53" t="str">
+        <v>2026-09-20 ~06:57 UTC: only Summer 2027 reqs found. No Winter 2026/Spring 2027 posting located.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Olympus (Westborough, MA)</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Jan–June 2026 Manufacturing Engineering Co-Op (direct fetch); July–Dec 2026 co-op</v>
+      </c>
+      <c r="C54" t="str">
+        <v>2026-09-20 ~06:57 UTC: Jan–June 2026 cohort directly confirmed 'no longer accepting applications'. July–Dec 2026 is wrong season (Fall, not Winter/Spring). No real URL found for a 'Jan–June 2027' version — a prior aggregator claim of one appears to be a synthesis artifact, not an actual posting. Ruling out fully pending a real link.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B55" t="str">
+        <v>JR002884 (Optics-Physics Sensor Eng Co-op, Spring 2027), JR002885 (Sensor Electrical Eng Co-op, Spring 2027), JR002767 (Mechanical Eng &amp; System Packaging Intern), JR002688 (Acoustic and Vibration Technologies Co-op), JR002717 (Metrology Co-op)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>2026-09-20 ~06:57 UTC: JR002884/JR002885 wrong discipline (optics/electrical, consistent with prior exclusion). JR002767 is a Summer role per aggregator, not Winter/Spring. JR002688 and JR002717 are open/rolling but state no specific season/year on the posting — fail the 'season stated' bar, excluded pending a dated version.</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Group 07-71 Mechanical Engineering (Jan–June 2026), Group 07-76 Control &amp; Autonomous Systems (Jan–June 2026), Group 07-77 (July–Dec 2026)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>2026-09-20 ~06:57 UTC: all three are past/wrong-season cycles relative to today. No new Spring 2027 (Jan–June 2027) mechanical/aerospace req found beyond the already-tracked Microfabrication Co-Op.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B57" t="str">
+        <v>req R2495 'Mechanical Engineering Intern' (Atlas program)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>2026-09-20 ~06:57 UTC: search snippet mentions 'Spring 2027 Co-Op' but Workday fetch returned empty content twice — could not independently verify or confirm this is distinct from already-tracked req R2476. Worth a follow-up with better Workday access.</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Commonwealth Fusion Systems (Devens, MA)</v>
+      </c>
+      <c r="B58" t="str">
+        <v>'Intern – Mechanical Engineer – Fall Co-op 2026'</v>
+      </c>
+      <c r="C58" t="str">
+        <v>2026-09-20 ~06:57 UTC: title/season is Fall 2026 only, and the posting itself now 404s. No Spring 2027 version found.</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B59" t="str">
+        <v>'2027 Mechanical Engineer Intern' reqs including a Boston, MA location</v>
+      </c>
+      <c r="C59" t="str">
+        <v>2026-09-20 ~06:57 UTC: context strongly suggests Summer 2027 wave (aggregator states ~47% of new listings carry 'Summer 2027' in title); not confirmed as Winter 2026/Spring 2027 — excluded, but the Boston, MA listing specifically is worth a direct-fetch check next pass.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Astranis</v>
+      </c>
+      <c r="B60" t="str">
+        <v>'Mechanical Engineer Intern (Winter 2027)', SF, via Greenhouse</v>
+      </c>
+      <c r="C60" t="str">
+        <v>2026-09-20 ~06:57 UTC: directly verified live and open ($29/hr) but season is literally 'Winter 2027' (not Winter 2026 or Spring 2027 as required) — excluded on strict season-match grounds. Near miss, worth flagging if Hamza wants to reconsider the season window.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>L3Harris</v>
+      </c>
+      <c r="B61" t="str">
+        <v>'Mechanical Engineer Co-op' and 'Sustainment Mechanical Engineering Co-op' (Greenville, TX)</v>
+      </c>
+      <c r="C61" t="str">
+        <v>2026-09-20 ~06:57 UTC: both confirmed dead (404) on direct fetch. Only software/AI Spring 2027 reqs remain live — discipline mismatch, consistent with prior exclusion.</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Curtiss-Wright</v>
+      </c>
+      <c r="B62" t="str">
+        <v>JR1907 'Co-op (Spring Term)', Cheswick, PA</v>
+      </c>
+      <c r="C62" t="str">
+        <v>2026-09-20 ~06:57 UTC: posting has no explicit year in the title; direct fetch blocked (403). Could not confirm Spring 2027 specifically — excluded pending verification, worth a re-check.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Sierra Nevada Corporation</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Mechanical co-op/intern search</v>
+      </c>
+      <c r="C63" t="str">
+        <v>2026-09-20 ~06:57 UTC: only found a historical (2023) mechanical co-op posting and current Summer 2027 reqs. No Winter 2026/Spring 2027 posting found.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Redwire Space / Karman Space</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Mechanical/aerospace intern search</v>
+      </c>
+      <c r="C64" t="str">
+        <v>2026-09-20 ~06:57 UTC: candidate roles exist at both but could not verify season (Redwire rate-limited 429; Karman fetch didn't surface target content). Excluded, worth re-checking with more time/attempts.</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Joby Aviation / Honeywell Aerospace / Moog / Woodward / Firefly Aerospace / Impulse Space / Virgin Galactic / Vecna Robotics / Desktop Metal / Markforged / Boston Dynamics AI Institute</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Mechanical/aerospace/systems/manufacturing/robotics internship search</v>
+      </c>
+      <c r="C65" t="str">
+        <v>2026-09-20 ~06:57 UTC: no Winter 2026/Spring 2027 postings found at any of these — only Summer 2027, Fall 2026, or undated rolling reqs turned up.</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>General Dynamics Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B66" t="str">
+        <v>req 601496955 (already Partial in `rows`), including a text-proxy (r.jina.ai) fetch workaround</v>
+      </c>
+      <c r="C66" t="str">
+        <v>2026-09-20 ~06:57 UTC: still blocked by Cloudflare on jobs.buildsubmarines.com even via proxy workaround. WebSearch snippets remain consistent with the tracked posting (title, Groton CT, mechanical/aerospace-eligible, US citizenship required) but no independent direct-fetch confirmation obtained — status in `rows` unchanged at Partial.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 21 checked-excluded (2026-09-20 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AqYkLoqFh1a64dH3hMiEGY
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J47"/>
+  <dimension ref="A1:J49"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1901,16 +1901,80 @@
         <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Applied Materials</v>
+      </c>
+      <c r="B48" t="str">
+        <v>2027 Spring Mechanical Engineer Co-op</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Spring 2027 (start January 2027)</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Gloucester, MA</v>
+      </c>
+      <c r="F48">
+        <v>30</v>
+      </c>
+      <c r="G48" t="str">
+        <v>$31–33/hr</v>
+      </c>
+      <c r="H48" t="str">
+        <v>https://amat.wd1.myworkdayjobs.com/external/job/GloucesterMA/XMLNAME-2027-Spring-Mechanical-Engineer-Co-op--Gloucester-MA-_R2628290</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Partial — Workday page blocked automated fetch (JS-rendered, empty). Confirmed via a dreamworkhq aggregator mirror quoting the exact title, season, location, pay, and req ID, posted ~1 week ago as of 2026-09-20. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Sanofi (Genzyme)</v>
+      </c>
+      <c r="B49" t="str">
+        <v>2027 Spring Co-Op Opportunities</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Manufacturing / Process Engineering (biopharma — MSAT: Manufacturing Science &amp; Technology)</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Spring 2027 (6-month, starting January 2027)</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Framingham, MA</v>
+      </c>
+      <c r="F49">
+        <v>20</v>
+      </c>
+      <c r="G49" t="str">
+        <v>$32–55/hr</v>
+      </c>
+      <c r="H49" t="str">
+        <v>https://jobs.sanofi.com/en/job/framingham/2027-spring-co-op-opportunities-framingham-ma/2649/41259847040</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Yes — fetched directly, page live, active 'Apply Now' button present. Posting states it closes November 14, 2026.</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J49"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C87"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -2643,9 +2707,240 @@
         <v>2026-09-20 ~06:57 UTC: still blocked by Cloudflare on jobs.buildsubmarines.com even via proxy workaround. WebSearch snippets remain consistent with the tracked posting (title, Groton CT, mechanical/aerospace-eligible, US citizenship required) but no independent direct-fetch confirmation obtained — status in `rows` unchanged at Partial.</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>General Dynamics Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B67" t="str">
+        <v>req 601496955 (already Partial in `rows`) — 4th consecutive re-check</v>
+      </c>
+      <c r="C67" t="str">
+        <v>2026-09-20 ~13:00 UTC: still blocked by Cloudflare on jobs.buildsubmarines.com (4th consecutive failed direct-fetch attempt). WebSearch corroborates the exact tracked title ('2027 Spring Engineering CO-OP Trainee') still appears on the aggregator's own listing — no new information; status in `rows` unchanged at Partial. Deprioritizing further automated attempts after 4 straight blocks — would need an actual in-browser check to resolve.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B68" t="str">
+        <v>req R2495 'Mechanical Engineering Intern' (Atlas program) — re-check</v>
+      </c>
+      <c r="C68" t="str">
+        <v>2026-09-20 ~13:00 UTC: Workday fetch still returns empty (3rd failed attempt across runs). A search-synthesis claim of 'Spring 2027, Jan–Aug 2027' could not be corroborated as a literal quote from any retrievable source this run — season still unconfirmed, not added to `rows`. Distinct req from already-tracked R2476 (same location/program). Also found and ruled out an unrelated same-titled Boston Dynamics posting that is explicitly Summer 2026 and inactive — a naming collision, not R2495.</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Boston, MA-flagged listing</v>
+      </c>
+      <c r="C69" t="str">
+        <v>2026-09-20 ~13:00 UTC: careers page now shows only Cape Canaveral, FL and Stennis, MS roles — no Boston, MA listing currently live. Excluded — appears no longer posted.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Curtiss-Wright</v>
+      </c>
+      <c r="B70" t="str">
+        <v>JR1907 'Co-op (Spring Term)', Cheswick, PA</v>
+      </c>
+      <c r="C70" t="str">
+        <v>2026-09-20 ~13:00 UTC: confirmed live via a zapply.jobs mirror (posted 2026-08-05), but the posting itself still states no year for 'Spring Term' — season is only an inference from posting date/cadence, not a stated fact, so it fails the verification bar. Excluded pending an explicitly dated version.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Redwire Space</v>
+      </c>
+      <c r="B71" t="str">
+        <v>'Mechanical Engineering Intern - Year Round' plus current Summer 2026 postings (Georgetown, IN; Goleta, CA)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>2026-09-20 ~13:00 UTC: only Summer 2026-dated postings and an undated 'year round' listing found — no Winter 2026/Spring 2027-specific posting located. Excluded on season grounds.</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Internship program (general)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>2026-09-20 ~13:00 UTC: company's own internship page states the program is annual with an April 30 application deadline and positions running May/June–Aug/Sept — a summer-only program by design. Excluded — no Winter 2026/Spring 2027 track exists.</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B73" t="str">
+        <v>JR002688 (Acoustic and Vibration Technologies Co-op), JR002717 (Metrology Co-op) — re-check</v>
+      </c>
+      <c r="C73" t="str">
+        <v>2026-09-20 ~13:00 UTC: both re-confirmed open/rolling (JR002717 posted 2026-08-05, JR002688 posted ~1 month ago) but still carry no explicit season/year on the posting — no change from last check. Excluded pending a dated version.</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Analog Devices</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Mechanical co-op search — re-check</v>
+      </c>
+      <c r="C74" t="str">
+        <v>2026-09-20 ~13:00 UTC: only a closed/past Jan–June 2025 Burlington, MA co-op found; no current Winter 2026/Spring 2027 posting — no change from prior finding.</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Caterpillar</v>
+      </c>
+      <c r="B75" t="str">
+        <v>r0000290709 (now 404; prior title showed 'Spring/Summer 2026' — wrong season regardless); '2027 Engineering Corporate Parallel Co-op Program' (Tucson/Green Valley AZ, Champaign/Decatur/Mossville IL, Lafayette IN)</v>
+      </c>
+      <c r="C75" t="str">
+        <v>2026-09-20 ~13:00 UTC: the previously-flagged req is dead and was wrong-season anyway. The 2027 Parallel Co-op Program has an ambiguous, continuous summer-plus-school-year structure (not a discrete Winter/Spring term) and no MA location — excluded as not a clean fit.</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Toyota Research Institute</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Live Lever board (jobs.lever.co/tri): Human Interactive Driving Intern (Fall 2026), Human-Centered AI Research Intern (Winter 2027), Robotics Research Intern - Post-Training (Spring 2027)</v>
+      </c>
+      <c r="C76" t="str">
+        <v>2026-09-20 ~13:00 UTC: all current postings are ML/AI research roles (not mechanical engineering) located in Los Altos, CA (not Cambridge, MA). Excluded — discipline and location mismatch.</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Waters Corporation / Instron / Analogic / Boston Metal / Charles River Laboratories</v>
+      </c>
+      <c r="B77" t="str">
+        <v>General mechanical/manufacturing co-op search, each company</v>
+      </c>
+      <c r="C77" t="str">
+        <v>2026-09-20 ~13:00 UTC: no current mechanical/manufacturing internship or co-op postings found for any season at any of these MA-area employers (Charles River's most comparable posting, a Facilities Engineer Intern, is a closed 2025 Summer role).</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Bose</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Mechanical Engineer Co-op / Concept Prototyping (req R25833), Advanced Manufacturing Mechanical Engineering Intern</v>
+      </c>
+      <c r="C78" t="str">
+        <v>2026-09-20 ~13:00 UTC: only LinkedIn mirrors found, both appearing to be stale reqs from a prior cycle; the specific aggregator mirror link 404'd and Bose's own careers URL 404'd. Excluded — could not confirm any currently-open, correctly-seasoned posting.</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Thermo Fisher Scientific</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Manufacturing Engineering Intern (Bedford, MA); Manufacturing Engineering Co-op (Marietta, OH)</v>
+      </c>
+      <c r="C79" t="str">
+        <v>2026-09-20 ~13:00 UTC: Bedford, MA role's stated start dates (May 24/June 14, 2027) put it in the Summer 2027 wave — wrong season. Marietta, OH role is not in MA and its season couldn't be confirmed. Excluded.</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Philips</v>
+      </c>
+      <c r="B80" t="str">
+        <v>EMC Engineer Co-op, Hardware Test/Reliability Co-op (Andover, MA)</v>
+      </c>
+      <c r="C80" t="str">
+        <v>2026-09-20 ~13:00 UTC: only Jan–June 2025 (already past) postings found; no current 2026/2027 posting surfaced. Excluded.</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Hexagon Manufacturing Intelligence / Oshkosh Corporation / Terex Corporation / Polaris Industries / Waymo</v>
+      </c>
+      <c r="B81" t="str">
+        <v>General mechanical engineering intern/co-op search, each company</v>
+      </c>
+      <c r="C81" t="str">
+        <v>2026-09-20 ~13:00 UTC: all confirmed to run Summer-only internship cycles (Summer 2026 or Summer 2027 postings found, no Winter 2026/Spring 2027 track) — excluded on season grounds.</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Sublime Systems (Somerville, MA)</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Company Lever board (jobs.lever.co)</v>
+      </c>
+      <c r="C82" t="str">
+        <v>2026-09-20 ~13:00 UTC: board directly confirmed to state 'No job postings currently open.' Excluded.</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B83" t="str">
+        <v>2027 mechanical engineering intern cycle</v>
+      </c>
+      <c r="C83" t="str">
+        <v>2026-09-20 ~13:00 UTC: per the company's own careers-program messaging, the 2027 cycle has not yet been posted as of mid-September 2026. Not yet open — worth re-checking in a few weeks.</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Textron Systems (Wilmington, MA)</v>
+      </c>
+      <c r="B84" t="str">
+        <v>'2027 Intern - Materials Quality Engineer (Weapons)'</v>
+      </c>
+      <c r="C84" t="str">
+        <v>2026-09-20 ~13:00 UTC: role title found (materials discipline, in-scope) but the Taleo posting page returned only template placeholders with no real content on fetch — could not confirm season, pay, or open status. Unresolved, not added — worth a direct follow-up check.</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Aurora Flight Sciences (Boeing subsidiary)</v>
+      </c>
+      <c r="B85" t="str">
+        <v>General internships page, Manufacturing Engineering Intern mention</v>
+      </c>
+      <c r="C85" t="str">
+        <v>2026-09-20 ~13:00 UTC: company materials describe MA-based (and VA-based) autonomy/mechanical engineering work, but no specific dated 2027 co-op listing could be found — only a generic description with no season stated in the retrievable snippet. Unresolved — worth a direct check of careers.aurora.aero.</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>GE HealthCare</v>
+      </c>
+      <c r="B86" t="str">
+        <v>'LSS Mechanical Engineering Co-op' (title found via zapply)</v>
+      </c>
+      <c r="C86" t="str">
+        <v>2026-09-20 ~13:00 UTC: a zapply search snippet surfaced this title but the actual page returned unrelated listings on two fetch attempts — could not verify season, location, or open status. Unresolved — needs a more targeted follow-up (e.g. direct careers.gehealthcare.com search).</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027), Cedar Rapids IA, req 01869080</v>
+      </c>
+      <c r="C87" t="str">
+        <v>2026-09-20 ~13:00 UTC: dedupe check — this req ID is identical to the RTX Cedar Rapids IA row already tracked in `rows`. Not a new posting; not re-added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 13 new postings, 22 checked-excluded (2026-09-20 19:00 UTC)
- Upgraded Draper's two Spring 2027 co-ops from Partial to Yes via
  direct Workday API fetch; moved Boston Dynamics R2476 to checked
  after confirming it's no longer live (zero intern/co-op reqs
  company-wide).
- Added first live GE Aerospace Spring 2027 req in 5 runs, plus a
  batch of Insulet Acton MA co-ops, a GE HealthCare and a GE Vernova
  posting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UMhxyobbrKEU4xpk7TXgsZ
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J61"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1098,10 +1098,10 @@
         <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Systems-Engineering-Co-Op--Spring-2027-_JR002882</v>
       </c>
       <c r="I22" t="str">
-        <v>Partial — confirmed live via Draper's own job-listings page (draper.com/careers), posted ~1 week ago (~Sept 12, 2026). The Workday req page itself returned blank to automated fetch (JS-rendered) — verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~9 days ago as of this check.</v>
       </c>
       <c r="J22" t="str">
-        <v>Found via Draper's first-party listings page, not an aggregator.</v>
+        <v>GAD division placement. Pay $20.00-$45.00/hr per posting.</v>
       </c>
     </row>
     <row r="23">
@@ -1130,10 +1130,10 @@
         <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Electro-Mechanical-Instrument-Co-op--Spring-2027-_JR002883-1</v>
       </c>
       <c r="I23" t="str">
-        <v>Partial — confirmed live via Draper's own job-listings page (draper.com/careers), posted ~2 weeks ago (~Sept 5, 2026). Workday req page blocked automated fetch — verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~20 days ago as of this check.</v>
       </c>
       <c r="J23" t="str">
-        <v>Found via Draper's first-party listings page, not an aggregator.</v>
+        <v>US Citizenship required — Draper cannot sponsor/hire H1B or Student Visa holders; dual citizens not eligible. CAD (Creo/SolidWorks), FEA (ANSYS/COMSOL) skills mentioned. Pay $20.00-$45.00/hr per posting.</v>
       </c>
     </row>
     <row r="24">
@@ -1743,66 +1743,66 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Boston Dynamics</v>
+        <v>Berkshire Grey</v>
       </c>
       <c r="B43" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Spring 2027 Hardware Quality Co-op</v>
       </c>
       <c r="C43" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Hardware / Quality Engineering</v>
       </c>
       <c r="D43" t="str">
-        <v>Spring 2027 (Jan–Aug 2027, per search snippet)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E43" t="str">
-        <v>Waltham, MA</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F43">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G43" t="str">
-        <v>$30–$45/hr per search snippet; not independently confirmed via direct fetch</v>
+        <v>Not stated (aggregator only)</v>
       </c>
       <c r="H43" t="str">
-        <v>https://bostondynamics.wd1.myworkdayjobs.com/Boston_Dynamics/job/Waltham-Office-POST/Mechanical-Engineering-Co-Op_R2476</v>
+        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
       </c>
       <c r="I43" t="str">
-        <v>Partial — Workday page returned empty content on two direct fetch attempts (JS-rendered/blocked). Season and pay sourced from search snippet only, not independently opened. Verify live in-browser before applying.</v>
+        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
       </c>
       <c r="J43" t="str">
-        <v>Boston metro (Waltham).</v>
+        <v>Boston metro (Bedford).</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Berkshire Grey</v>
+        <v>Emerson</v>
       </c>
       <c r="B44" t="str">
-        <v>Spring 2027 Hardware Quality Co-op</v>
+        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
       </c>
       <c r="C44" t="str">
-        <v>Hardware / Quality Engineering</v>
+        <v>R&amp;D / Mechanical Engineering</v>
       </c>
       <c r="D44" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E44" t="str">
-        <v>Bedford, MA</v>
+        <v>Cranberry Township, PA</v>
       </c>
       <c r="F44">
-        <v>17</v>
+        <v>570</v>
       </c>
       <c r="G44" t="str">
         <v>Not stated (aggregator only)</v>
       </c>
       <c r="H44" t="str">
-        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
       </c>
       <c r="I44" t="str">
-        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J44" t="str">
-        <v>Boston metro (Bedford).</v>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1810,16 +1810,16 @@
         <v>Emerson</v>
       </c>
       <c r="B45" t="str">
-        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
+        <v>Project Engineering Co-op – Spring 2027</v>
       </c>
       <c r="C45" t="str">
-        <v>R&amp;D / Mechanical Engineering</v>
+        <v>Project / Mechanical Engineering</v>
       </c>
       <c r="D45" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E45" t="str">
-        <v>Cranberry Township, PA</v>
+        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
       </c>
       <c r="F45">
         <v>570</v>
@@ -1828,7 +1828,7 @@
         <v>Not stated (aggregator only)</v>
       </c>
       <c r="H45" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
       </c>
       <c r="I45" t="str">
         <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
@@ -1839,142 +1839,526 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Emerson</v>
+        <v>Zipline</v>
       </c>
       <c r="B46" t="str">
-        <v>Project Engineering Co-op – Spring 2027</v>
+        <v>Mechanical Engineer Intern</v>
       </c>
       <c r="C46" t="str">
-        <v>Project / Mechanical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D46" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Jan–Apr/May)</v>
       </c>
       <c r="E46" t="str">
-        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
+        <v>South San Francisco, CA (or Dallas, TX)</v>
       </c>
       <c r="F46">
-        <v>570</v>
+        <v>2700</v>
       </c>
       <c r="G46" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>~$60k–$70k annualized (third-party estimate, not stated on posting)</v>
       </c>
       <c r="H46" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
+        <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
       </c>
       <c r="I46" t="str">
-        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
       </c>
       <c r="J46" t="str">
-        <v/>
+        <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Zipline</v>
+        <v>Applied Materials</v>
       </c>
       <c r="B47" t="str">
-        <v>Mechanical Engineer Intern</v>
+        <v>2027 Spring Mechanical Engineer Co-op</v>
       </c>
       <c r="C47" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D47" t="str">
-        <v>Spring 2027 (Jan–Apr/May)</v>
+        <v>Spring 2027 (start January 2027)</v>
       </c>
       <c r="E47" t="str">
-        <v>South San Francisco, CA (or Dallas, TX)</v>
+        <v>Gloucester, MA</v>
       </c>
       <c r="F47">
-        <v>2700</v>
+        <v>30</v>
       </c>
       <c r="G47" t="str">
-        <v>~$60k–$70k annualized (third-party estimate, not stated on posting)</v>
+        <v>$31–33/hr</v>
       </c>
       <c r="H47" t="str">
-        <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
+        <v>https://amat.wd1.myworkdayjobs.com/external/job/GloucesterMA/XMLNAME-2027-Spring-Mechanical-Engineer-Co-op--Gloucester-MA-_R2628290</v>
       </c>
       <c r="I47" t="str">
-        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
+        <v>Partial — Workday page blocked automated fetch (JS-rendered, empty). Confirmed via a dreamworkhq aggregator mirror quoting the exact title, season, location, pay, and req ID, posted ~1 week ago as of 2026-09-20. Verify live in-browser before applying.</v>
       </c>
       <c r="J47" t="str">
-        <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
+        <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Applied Materials</v>
+        <v>Sanofi (Genzyme)</v>
       </c>
       <c r="B48" t="str">
-        <v>2027 Spring Mechanical Engineer Co-op</v>
+        <v>2027 Spring Co-Op Opportunities</v>
       </c>
       <c r="C48" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing / Process Engineering (biopharma — MSAT: Manufacturing Science &amp; Technology)</v>
       </c>
       <c r="D48" t="str">
-        <v>Spring 2027 (start January 2027)</v>
+        <v>Spring 2027 (6-month, starting January 2027)</v>
       </c>
       <c r="E48" t="str">
-        <v>Gloucester, MA</v>
+        <v>Framingham, MA</v>
       </c>
       <c r="F48">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G48" t="str">
-        <v>$31–33/hr</v>
+        <v>$32–55/hr</v>
       </c>
       <c r="H48" t="str">
-        <v>https://amat.wd1.myworkdayjobs.com/external/job/GloucesterMA/XMLNAME-2027-Spring-Mechanical-Engineer-Co-op--Gloucester-MA-_R2628290</v>
+        <v>https://jobs.sanofi.com/en/job/framingham/2027-spring-co-op-opportunities-framingham-ma/2649/41259847040</v>
       </c>
       <c r="I48" t="str">
-        <v>Partial — Workday page blocked automated fetch (JS-rendered, empty). Confirmed via a dreamworkhq aggregator mirror quoting the exact title, season, location, pay, and req ID, posted ~1 week ago as of 2026-09-20. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly, page live, active 'Apply Now' button present. Posting states it closes November 14, 2026.</v>
       </c>
       <c r="J48" t="str">
-        <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
+        <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Sanofi (Genzyme)</v>
+        <v>GE Aerospace</v>
       </c>
       <c r="B49" t="str">
-        <v>2027 Spring Co-Op Opportunities</v>
+        <v>Engines Engineering Co-op – US – Spring 2027</v>
       </c>
       <c r="C49" t="str">
-        <v>Manufacturing / Process Engineering (biopharma — MSAT: Manufacturing Science &amp; Technology)</v>
+        <v>Aerospace / Mechanical Engineering</v>
       </c>
       <c r="D49" t="str">
-        <v>Spring 2027 (6-month, starting January 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E49" t="str">
-        <v>Framingham, MA</v>
+        <v>Lynn, MA or Evendale/Cincinnati, OH (dual-location req)</v>
       </c>
       <c r="F49">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G49" t="str">
-        <v>$32–55/hr</v>
+        <v>Starts at $20/hr, increases per undergrad class year</v>
       </c>
       <c r="H49" t="str">
-        <v>https://jobs.sanofi.com/en/job/framingham/2027-spring-co-op-opportunities-framingham-ma/2649/41259847040</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Evendale/Engines-Engineering-Co-op---US---Spring-2027_R5029617-1</v>
       </c>
       <c r="I49" t="str">
-        <v>Yes — fetched directly, page live, active 'Apply Now' button present. Posting states it closes November 14, 2026.</v>
+        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
       </c>
       <c r="J49" t="str">
-        <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
+        <v>Requires 'US Person' status (citizen/LPR/asylee/refugee) for export-controlled work; no visa sponsorship; relocation/housing assistance provided. This is the first live GE Aerospace Spring 2027 req found after 4 prior runs found only dead/expired reqs — Lynn, MA option makes this a Boston-metro fit.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Structures Intern/Co-op – ACSC – Cincinnati, OH – Spring 2027</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Structural / Manufacturing / Materials Engineering</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Springdale (Cincinnati), OH</v>
+      </c>
+      <c r="F50">
+        <v>750</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H50" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Springdale/Structures-Intern-Co-op---ACSC---Cincinnati--OH---Spring-2027_R5039588-1</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Accepted majors: Aerospace, Manufacturing, Mechanical, Materials, Industrial Engineering. Not Boston-area.</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Co-op, R&amp;D Mechanical Engineering (January–June 2027, Hybrid)</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D51" t="str">
+        <v>January 11, 2027 – June 30, 2027</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F51">
+        <v>25</v>
+      </c>
+      <c r="G51" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H51" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Mechanical-Engineering--January---June-2027--Hybrid-_REQ-2026-18007</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Yes — full description fetched directly via Workday, posted 4 days ago.</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Boston metro (Acton). Medical device (insulin pump) manufacturer. Not eligible for visa sponsorship; requires US work authorization without future sponsorship needs. Part of a large batch of Insulet Acton co-ops opened this cycle — see sibling reqs below.</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D52" t="str">
+        <v>January 11, 2027 – June 30, 2027</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F52">
+        <v>25</v>
+      </c>
+      <c r="G52" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H52" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Engineering--January---June-2027--Onsite-_REQ-2026-18078</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Boston metro (Acton). No visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Co-op, Systems Engineering (January–June 2027, Hybrid)</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D53" t="str">
+        <v>January 11, 2027 – June 30, 2027</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F53">
+        <v>25</v>
+      </c>
+      <c r="G53" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H53" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering--January-June-2027--Hybrid-_REQ-2026-18061</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Boston metro (Acton). No visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Co-op, Mechanical Lifecycle (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D54" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F54">
+        <v>25</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H54" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Mechanical-Lifecycle--January---June-2027--Onsite-_REQ-2026-18155</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Partial — confirmed live and current via direct query of Insulet's own Workday jobs-search API (real title/location/posted-date, not an aggregator), posted 5 days ago. Full job-description body was not individually opened — spot-check before applying.</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Boston metro (Acton). One of a batch of Insulet Acton co-ops opened this cycle alongside the fully-verified R&amp;D Mechanical/Manufacturing/Systems reqs above.</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Co-op, R&amp;D Manufacturing (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D55" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F55">
+        <v>25</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H55" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Manufacturing--January-June-2027--Onsite-_REQ-2026-18069</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Boston metro (Acton).</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Graduate Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Manufacturing Engineering (graduate-level)</v>
+      </c>
+      <c r="D56" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F56">
+        <v>25</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H56" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Graduate--January---June-2027--Onsite-_REQ-2026-18086</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Boston metro (Acton). Labeled 'Graduate Co-op' — confirm eligibility if Hamza is undergraduate.</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Co-op, Supplier Development Engineering - Mechanical (January–June 2027)</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Mechanical / Supplier Quality Engineering</v>
+      </c>
+      <c r="D57" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F57">
+        <v>25</v>
+      </c>
+      <c r="G57" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H57" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Development-Engineering---Mechanical--January-June-2027--Onsite-_REQ-2026-18209</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly (not a synthesized link); the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Boston metro (Acton).</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Co-op, Systems Engineering - Design Verification (January–June 2027)</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D58" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F58">
+        <v>25</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H58" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering---Design-Verification--January---June-2027--Onsite-_REQ-2026-18144-1</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Boston metro (Acton).</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Co-op, Life Cycle Engineering - Systems (January–June 2027)</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D59" t="str">
+        <v>January–June 2027 (per title)</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F59">
+        <v>25</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+      </c>
+      <c r="H59" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Life-Cycle-Engineering---Systems--January---June-2027--Hybrid-_REQ-2026-18149</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Boston metro (Acton). Most recently posted of the Insulet batch.</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>GE HealthCare</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Infant Care V&amp;V Engineering Co-op - Spring 2027</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Mechanical / Verification &amp; Validation Engineering</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Waukesha, WI</v>
+      </c>
+      <c r="F60">
+        <v>950</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H60" t="str">
+        <v>https://gehc.wd5.myworkdayjobs.com/en-US/GEHC_ExternalSite/job/Waukesha/Infant-Care-V-V-Engineering-Co-op_R4046324-1</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Yes — full description fetched directly via Workday CXS API, posted 2 days ago.</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Accepts Mechanical, Electrical, Computer, and Biomedical Engineering majors — verification/test focus, not pure design. Minimum 20-week commitment, onsite Waukesha WI, no visa sponsorship. Not Boston-area.</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>GE Vernova</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Nuclear Engineering Co-Op/Intern - Spring 2027</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Nuclear / Industrial Engineering</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Wilmington, NC</v>
+      </c>
+      <c r="F61">
+        <v>750</v>
+      </c>
+      <c r="G61" t="str">
+        <v>$1,000–$2,000/week (varies by class year)</v>
+      </c>
+      <c r="H61" t="str">
+        <v>https://careers.gevernova.com/ge-vernova-nuclear-engineering-co-op-intern-spring-2027/job/R5048552</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Yes — fetched directly, structured JSON-LD job data embedded in the page confirmed title, pay, address, and datePosted (2026-09-11).</v>
+      </c>
+      <c r="J61" t="str">
+        <v>GE Vernova Hitachi Nuclear Energy (GVH) business. Not Boston-area.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J61"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C109"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -2938,9 +3322,251 @@
         <v>2026-09-20 ~13:00 UTC: dedupe check — this req ID is identical to the RTX Cedar Rapids IA row already tracked in `rows`. Not a new posting; not re-added.</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Mechanical Engineering Co-Op (req R2476, previously tracked in `rows` as Partial)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>2026-09-20: queried Boston Dynamics' live Workday CXS jobs API directly for all open reqs — all 37 current postings are workerSubType 'Regular'; zero Intern/Co-Op postings exist company-wide right now. R2476 is no longer live. MOVED from `rows` to `checked`.</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Co-op, Next Gen Platforms (NGP) Systems Engineering: January-June 2027 (Onsite), req REQ-2026-18071</v>
+      </c>
+      <c r="C89" t="str">
+        <v>2026-09-20: title/season/pay/location corroborated by two independent aggregator mirrors (Zapply, Workopia) and the live Workday jobs-search API, but no source yielded a verifiable canonical Insulet Workday deep-link URL (unlike its sibling Insulet Acton reqs) — not added without a working link. Note: a separate, distinct 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists at Insulet but is wrong season, not this one. Worth a direct re-check next run.</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Sensor Electrical Engineering Co-op (Spring 2027), JR002885</v>
+      </c>
+      <c r="C90" t="str">
+        <v>2026-09-20: re-confirmed live via direct Workday API fetch (posted 20 days ago) but still excluded — electrical/sensor discipline, outside Hamza's target list. No change from prior exclusion (see JR002884/JR002885 entry above).</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Textron Systems (Wilmington, MA)</v>
+      </c>
+      <c r="B91" t="str">
+        <v>'2027 Intern - Materials Quality Engineer (Weapons)', req 1539632 / job 342556</v>
+      </c>
+      <c r="C91" t="str">
+        <v>2026-09-20: Taleo page now returns real content (progress from prior runs' template-placeholder blocker) — confirmed Wilmington MA, Full-time Internship/Co-Op type, posted 09/01/2026, requires US Citizenship for classified access. But the posting itself still never states a season (no 'Winter 2026'/'Spring 2027' wording anywhere) — fails the season-verification bar, not added.</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Aurora Flight Sciences (Boeing subsidiary)</v>
+      </c>
+      <c r="B92" t="str">
+        <v>careers.aurora.aero direct search</v>
+      </c>
+      <c r="C92" t="str">
+        <v>2026-09-20: site is a fully client-side-rendered Taleo CWS v2 board — direct fetch returns only an empty JS shell with no embedded job data. WebSearch found no specific dated Spring 2027 mechanical/co-op requisition. Still unverifiable.</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>GE HealthCare</v>
+      </c>
+      <c r="B93" t="str">
+        <v>'LSS Mechanical Engineering Co-op', req R4046267-1, Madison WI</v>
+      </c>
+      <c r="C93" t="str">
+        <v>2026-09-20: fetched full description directly — contains zero season/date/year language anywhere in the posting, and location is Madison WI (not Boston area). Excluded for failing the season-verification bar. (A separate, distinct GE HealthCare req — 'Infant Care V&amp;V Engineering Co-op - Spring 2027,' Waukesha WI — DID state its season and was added to `rows`.)</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>MKS Instruments (Andover, MA)</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Workday university-recruiting API query for 'Mechanical Co-op' + Andover</v>
+      </c>
+      <c r="C94" t="str">
+        <v>2026-09-20: zero matching results — their only 4 open student-program reqs are in Milpitas CA, Beaverton OR, Malaysia, and Thailand. A 'Spring 2027' reference in initial search snippets appears to be a stale aggregator artifact, not a live Andover MA posting.</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B95" t="str">
+        <v>2027 mechanical/materials/process engineering intern cycle</v>
+      </c>
+      <c r="C95" t="str">
+        <v>2026-09-20: confirmed all 2026-cycle reqs (incl. mechanical) closed by mid-May 2026; no 2027-cycle reqs posted yet. No change from prior run.</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Analog Devices / Caterpillar / Commonwealth Fusion Systems</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C96" t="str">
+        <v>2026-09-20: no change from prior findings — Analog Devices' Spring 2027 cycle not yet posted; Caterpillar's 2027 programs remain ambiguous multi-rotation structures with no MA location; Commonwealth Fusion Systems has only a Fall 2026 co-op and general internship postings, no Spring 2027 mechanical req.</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Westinghouse Electric</v>
+      </c>
+      <c r="B97" t="str">
+        <v>General mechanical/nuclear intern search</v>
+      </c>
+      <c r="C97" t="str">
+        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (Rock Hill/Columbia, SC); no Spring 2027 co-op located.</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>NuScale Power</v>
+      </c>
+      <c r="B98" t="str">
+        <v>General mechanical/nuclear intern search</v>
+      </c>
+      <c r="C98" t="str">
+        <v>2026-09-20: no Spring 2027-specific posting found; only a general, undated internship program description (Corvallis OR / Houston TX / remote).</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Intuitive Surgical</v>
+      </c>
+      <c r="B99" t="str">
+        <v>General mechanical intern search</v>
+      </c>
+      <c r="C99" t="str">
+        <v>2026-09-20: only Summer 2027 (May-Aug) internships found in Sunnyvale, CA; no Spring 2027 co-op.</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Stryker</v>
+      </c>
+      <c r="B100" t="str">
+        <v>General mechanical intern search</v>
+      </c>
+      <c r="C100" t="str">
+        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (NJ/CA/MI); no Spring 2027 co-op located.</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Kratos Defense</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Co-op program rotation search</v>
+      </c>
+      <c r="C101" t="str">
+        <v>2026-09-20: co-op program uses a multi-semester rotation (Summer 2025 -&gt; Spring 2026 -&gt; Fall 2026 cohort cited); no new Spring 2027 rotation/cohort found posted yet.</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B102" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C102" t="str">
+        <v>2026-09-20: only 2027 Summer internships found; per HII's own program description, Spring co-op postings typically open 'September through October' — nothing live yet for Spring 2027 specifically. Worth re-checking in ~2-4 weeks.</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Parsons Corporation</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Structural Engineer Intern / Engineering Internship-Co-Op search</v>
+      </c>
+      <c r="C103" t="str">
+        <v>2026-09-20: all postings found are Summer 2027; no Spring 2027 structural/mechanical posting located.</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Realtime Robotics (Boston, MA)</v>
+      </c>
+      <c r="B104" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C104" t="str">
+        <v>2026-09-20: no internship/co-op postings of any season found.</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Piaggio Fast Forward (Boston, MA)</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Greenhouse job board, direct fetch</v>
+      </c>
+      <c r="C105" t="str">
+        <v>2026-09-20: only 4 open roles today (Mechanical Engineering Machinist, IT Specialist, part-time Office Manager, Business Development Leader) — none are co-op/intern, none carry season/date info. A 'Robotics and AI Co-op' listing found via search appears stale/closed.</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Diligent Robotics</v>
+      </c>
+      <c r="B106" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C106" t="str">
+        <v>2026-09-20: only an unrelated Austin, TX mechanical engineering intern reference found, no 2027/season confirmation, no Boston presence.</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Veo Robotics</v>
+      </c>
+      <c r="B107" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C107" t="str">
+        <v>2026-09-20: no 2027-specific posting found; general hardware/mechanical engineering intern role description only, no season stated.</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Coherent / II-VI</v>
+      </c>
+      <c r="B108" t="str">
+        <v>General mechanical co-op search</v>
+      </c>
+      <c r="C108" t="str">
+        <v>2026-09-20: no Spring 2027 mechanical co-op posting found specific to this company.</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Fisker / Canoo / Nikola / VinFast / Karma Automotive</v>
+      </c>
+      <c r="B109" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C109" t="str">
+        <v>2026-09-20: no active internship/co-op postings found at any of these; several (Fisker, Canoo, Nikola) have known bankruptcy/financial-distress history that likely explains absent active recruiting.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 19 checked-excluded (2026-09-21 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JPZN17DP1MKj9fTqQPMRgf
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J64"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -2349,16 +2349,112 @@
         <v>GE Vernova Hitachi Nuclear Energy (GVH) business. Not Boston-area.</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Leonardo DRS</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Mechanical Engineer Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Spring 2027 (Jan–Aug 2027)</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Bridgeton, MO</v>
+      </c>
+      <c r="F62">
+        <v>1050</v>
+      </c>
+      <c r="G62" t="str">
+        <v>$41,011–$53,315/yr base (co-op salary range) + bonus/equity eligibility per posting</v>
+      </c>
+      <c r="H62" t="str">
+        <v>https://www.linkedin.com/jobs/view/mechanical-engineer-co-op-spring-2027-at-leonardo-drs-4451960539</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Partial — confirmed via LinkedIn's own job listing (title/season/pay/location) corroborated by a Workopia aggregator mirror quoting the same details; Leonardo DRS's own careers.leonardodrs.com posting for this specific req was not independently located/opened, so the primary employer page itself couldn't be directly confirmed.</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Land Systems division, Bridgeton, MO site. New company, first Leonardo DRS posting tracked. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Co-op, Next Gen Platforms (NGP) Systems Engineering (Onsite)</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D63" t="str">
+        <v>January – June 2027</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F63">
+        <v>25</v>
+      </c>
+      <c r="G63" t="str">
+        <v>Not independently confirmed (see $25–34/hr range on sibling Insulet Acton reqs)</v>
+      </c>
+      <c r="H63" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Next-Gen-Platforms--NGP--Systems-Engineering--January-June-2027--Onsite-_REQ-2026-18071</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Partial — title/season/location/req ID corroborated by two independent aggregator mirrors (Workopia, Zapply) quoting this exact canonical Workday URL; the live Workday page itself returned empty on repeated direct fetch attempts across three runs. Resolves the prior 'no verifiable URL' blocker.</v>
+      </c>
+      <c r="J63" t="str">
+        <v>Boston metro (Acton), onsite. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Moderna</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Co-Op, Applied Technologies (Spring 2027)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Automation / Process Engineering / Bioengineering (discipline caveat — not classic mechanical)</v>
+      </c>
+      <c r="D64" t="str">
+        <v>January 18 – June 25, 2027</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Norwood, MA</v>
+      </c>
+      <c r="F64">
+        <v>14</v>
+      </c>
+      <c r="G64" t="str">
+        <v>$20.00–$60.00/hr per posting</v>
+      </c>
+      <c r="H64" t="str">
+        <v>https://jobs.biospace.com/job/3072468/co-op-applied-technologies-spring-2027-/</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Partial — full posting content (title, dates, pay, citizenship requirement, open status) fetched and rendered directly at this biospace.com job-board listing, which mirrors Moderna's official Workday posting; Moderna's own modernatx.wd1.myworkdayjobs.com page returned empty on direct fetch, so the primary employer page wasn't independently confirmed.</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Restricted to US persons (citizens/permanent residents/asylees/refugees). Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J64"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C128"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -3335,238 +3431,447 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Insulet</v>
+        <v>Draper Laboratory</v>
       </c>
       <c r="B89" t="str">
-        <v>Co-op, Next Gen Platforms (NGP) Systems Engineering: January-June 2027 (Onsite), req REQ-2026-18071</v>
+        <v>Sensor Electrical Engineering Co-op (Spring 2027), JR002885</v>
       </c>
       <c r="C89" t="str">
-        <v>2026-09-20: title/season/pay/location corroborated by two independent aggregator mirrors (Zapply, Workopia) and the live Workday jobs-search API, but no source yielded a verifiable canonical Insulet Workday deep-link URL (unlike its sibling Insulet Acton reqs) — not added without a working link. Note: a separate, distinct 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists at Insulet but is wrong season, not this one. Worth a direct re-check next run.</v>
+        <v>2026-09-20: re-confirmed live via direct Workday API fetch (posted 20 days ago) but still excluded — electrical/sensor discipline, outside Hamza's target list. No change from prior exclusion (see JR002884/JR002885 entry above).</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Draper Laboratory</v>
+        <v>Textron Systems (Wilmington, MA)</v>
       </c>
       <c r="B90" t="str">
-        <v>Sensor Electrical Engineering Co-op (Spring 2027), JR002885</v>
+        <v>'2027 Intern - Materials Quality Engineer (Weapons)', req 1539632 / job 342556</v>
       </c>
       <c r="C90" t="str">
-        <v>2026-09-20: re-confirmed live via direct Workday API fetch (posted 20 days ago) but still excluded — electrical/sensor discipline, outside Hamza's target list. No change from prior exclusion (see JR002884/JR002885 entry above).</v>
+        <v>2026-09-21: RESOLVED — proxy fetch of the full Taleo page now returns the complete description, which explicitly states 'Paid, full-time 10-week summer internship,' application deadline Oct 31, 2026, pay $28-32/hr, Wilmington MA. Confirmed Summer 2027, wrong season — excluded on season grounds (supersedes prior runs' 'season unstated' notes).</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Textron Systems (Wilmington, MA)</v>
+        <v>Aurora Flight Sciences (Boeing subsidiary)</v>
       </c>
       <c r="B91" t="str">
-        <v>'2027 Intern - Materials Quality Engineer (Weapons)', req 1539632 / job 342556</v>
+        <v>careers.aurora.aero direct search</v>
       </c>
       <c r="C91" t="str">
-        <v>2026-09-20: Taleo page now returns real content (progress from prior runs' template-placeholder blocker) — confirmed Wilmington MA, Full-time Internship/Co-Op type, posted 09/01/2026, requires US Citizenship for classified access. But the posting itself still never states a season (no 'Winter 2026'/'Spring 2027' wording anywhere) — fails the season-verification bar, not added.</v>
+        <v>2026-09-20: site is a fully client-side-rendered Taleo CWS v2 board — direct fetch returns only an empty JS shell with no embedded job data. WebSearch found no specific dated Spring 2027 mechanical/co-op requisition. Still unverifiable.</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Aurora Flight Sciences (Boeing subsidiary)</v>
+        <v>GE HealthCare</v>
       </c>
       <c r="B92" t="str">
-        <v>careers.aurora.aero direct search</v>
+        <v>'LSS Mechanical Engineering Co-op', req R4046267-1, Madison WI</v>
       </c>
       <c r="C92" t="str">
-        <v>2026-09-20: site is a fully client-side-rendered Taleo CWS v2 board — direct fetch returns only an empty JS shell with no embedded job data. WebSearch found no specific dated Spring 2027 mechanical/co-op requisition. Still unverifiable.</v>
+        <v>2026-09-20: fetched full description directly — contains zero season/date/year language anywhere in the posting, and location is Madison WI (not Boston area). Excluded for failing the season-verification bar. (A separate, distinct GE HealthCare req — 'Infant Care V&amp;V Engineering Co-op - Spring 2027,' Waukesha WI — DID state its season and was added to `rows`.)</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>GE HealthCare</v>
+        <v>MKS Instruments (Andover, MA)</v>
       </c>
       <c r="B93" t="str">
-        <v>'LSS Mechanical Engineering Co-op', req R4046267-1, Madison WI</v>
+        <v>Workday university-recruiting API query for 'Mechanical Co-op' + Andover</v>
       </c>
       <c r="C93" t="str">
-        <v>2026-09-20: fetched full description directly — contains zero season/date/year language anywhere in the posting, and location is Madison WI (not Boston area). Excluded for failing the season-verification bar. (A separate, distinct GE HealthCare req — 'Infant Care V&amp;V Engineering Co-op - Spring 2027,' Waukesha WI — DID state its season and was added to `rows`.)</v>
+        <v>2026-09-20: zero matching results — their only 4 open student-program reqs are in Milpitas CA, Beaverton OR, Malaysia, and Thailand. A 'Spring 2027' reference in initial search snippets appears to be a stale aggregator artifact, not a live Andover MA posting.</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>MKS Instruments (Andover, MA)</v>
+        <v>Lam Research</v>
       </c>
       <c r="B94" t="str">
-        <v>Workday university-recruiting API query for 'Mechanical Co-op' + Andover</v>
+        <v>2027 mechanical/materials/process engineering intern cycle</v>
       </c>
       <c r="C94" t="str">
-        <v>2026-09-20: zero matching results — their only 4 open student-program reqs are in Milpitas CA, Beaverton OR, Malaysia, and Thailand. A 'Spring 2027' reference in initial search snippets appears to be a stale aggregator artifact, not a live Andover MA posting.</v>
+        <v>2026-09-20: confirmed all 2026-cycle reqs (incl. mechanical) closed by mid-May 2026; no 2027-cycle reqs posted yet. No change from prior run.</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Lam Research</v>
+        <v>Analog Devices / Caterpillar / Commonwealth Fusion Systems</v>
       </c>
       <c r="B95" t="str">
-        <v>2027 mechanical/materials/process engineering intern cycle</v>
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
       </c>
       <c r="C95" t="str">
-        <v>2026-09-20: confirmed all 2026-cycle reqs (incl. mechanical) closed by mid-May 2026; no 2027-cycle reqs posted yet. No change from prior run.</v>
+        <v>2026-09-20: no change from prior findings — Analog Devices' Spring 2027 cycle not yet posted; Caterpillar's 2027 programs remain ambiguous multi-rotation structures with no MA location; Commonwealth Fusion Systems has only a Fall 2026 co-op and general internship postings, no Spring 2027 mechanical req.</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Analog Devices / Caterpillar / Commonwealth Fusion Systems</v>
+        <v>Westinghouse Electric</v>
       </c>
       <c r="B96" t="str">
-        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+        <v>General mechanical/nuclear intern search</v>
       </c>
       <c r="C96" t="str">
-        <v>2026-09-20: no change from prior findings — Analog Devices' Spring 2027 cycle not yet posted; Caterpillar's 2027 programs remain ambiguous multi-rotation structures with no MA location; Commonwealth Fusion Systems has only a Fall 2026 co-op and general internship postings, no Spring 2027 mechanical req.</v>
+        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (Rock Hill/Columbia, SC); no Spring 2027 co-op located.</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Westinghouse Electric</v>
+        <v>NuScale Power</v>
       </c>
       <c r="B97" t="str">
         <v>General mechanical/nuclear intern search</v>
       </c>
       <c r="C97" t="str">
-        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (Rock Hill/Columbia, SC); no Spring 2027 co-op located.</v>
+        <v>2026-09-20: no Spring 2027-specific posting found; only a general, undated internship program description (Corvallis OR / Houston TX / remote).</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>NuScale Power</v>
+        <v>Intuitive Surgical</v>
       </c>
       <c r="B98" t="str">
-        <v>General mechanical/nuclear intern search</v>
+        <v>General mechanical intern search</v>
       </c>
       <c r="C98" t="str">
-        <v>2026-09-20: no Spring 2027-specific posting found; only a general, undated internship program description (Corvallis OR / Houston TX / remote).</v>
+        <v>2026-09-20: only Summer 2027 (May-Aug) internships found in Sunnyvale, CA; no Spring 2027 co-op.</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Intuitive Surgical</v>
+        <v>Stryker</v>
       </c>
       <c r="B99" t="str">
         <v>General mechanical intern search</v>
       </c>
       <c r="C99" t="str">
-        <v>2026-09-20: only Summer 2027 (May-Aug) internships found in Sunnyvale, CA; no Spring 2027 co-op.</v>
+        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (NJ/CA/MI); no Spring 2027 co-op located.</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Stryker</v>
+        <v>Kratos Defense</v>
       </c>
       <c r="B100" t="str">
-        <v>General mechanical intern search</v>
+        <v>Co-op program rotation search</v>
       </c>
       <c r="C100" t="str">
-        <v>2026-09-20: only Summer 2027 mechanical engineering internships found (NJ/CA/MI); no Spring 2027 co-op located.</v>
+        <v>2026-09-20: co-op program uses a multi-semester rotation (Summer 2025 -&gt; Spring 2026 -&gt; Fall 2026 cohort cited); no new Spring 2027 rotation/cohort found posted yet.</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Kratos Defense</v>
+        <v>HII / Newport News Shipbuilding</v>
       </c>
       <c r="B101" t="str">
-        <v>Co-op program rotation search</v>
+        <v>General co-op/intern search</v>
       </c>
       <c r="C101" t="str">
-        <v>2026-09-20: co-op program uses a multi-semester rotation (Summer 2025 -&gt; Spring 2026 -&gt; Fall 2026 cohort cited); no new Spring 2027 rotation/cohort found posted yet.</v>
+        <v>2026-09-20: only 2027 Summer internships found; per HII's own program description, Spring co-op postings typically open 'September through October' — nothing live yet for Spring 2027 specifically. Worth re-checking in ~2-4 weeks.</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>HII / Newport News Shipbuilding</v>
+        <v>Parsons Corporation</v>
       </c>
       <c r="B102" t="str">
-        <v>General co-op/intern search</v>
+        <v>Structural Engineer Intern / Engineering Internship-Co-Op search</v>
       </c>
       <c r="C102" t="str">
-        <v>2026-09-20: only 2027 Summer internships found; per HII's own program description, Spring co-op postings typically open 'September through October' — nothing live yet for Spring 2027 specifically. Worth re-checking in ~2-4 weeks.</v>
+        <v>2026-09-20: all postings found are Summer 2027; no Spring 2027 structural/mechanical posting located.</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Parsons Corporation</v>
+        <v>Realtime Robotics (Boston, MA)</v>
       </c>
       <c r="B103" t="str">
-        <v>Structural Engineer Intern / Engineering Internship-Co-Op search</v>
+        <v>General intern/co-op search</v>
       </c>
       <c r="C103" t="str">
-        <v>2026-09-20: all postings found are Summer 2027; no Spring 2027 structural/mechanical posting located.</v>
+        <v>2026-09-20: no internship/co-op postings of any season found.</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Realtime Robotics (Boston, MA)</v>
+        <v>Piaggio Fast Forward (Boston, MA)</v>
       </c>
       <c r="B104" t="str">
-        <v>General intern/co-op search</v>
+        <v>Greenhouse job board, direct fetch</v>
       </c>
       <c r="C104" t="str">
-        <v>2026-09-20: no internship/co-op postings of any season found.</v>
+        <v>2026-09-20: only 4 open roles today (Mechanical Engineering Machinist, IT Specialist, part-time Office Manager, Business Development Leader) — none are co-op/intern, none carry season/date info. A 'Robotics and AI Co-op' listing found via search appears stale/closed.</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Piaggio Fast Forward (Boston, MA)</v>
+        <v>Diligent Robotics</v>
       </c>
       <c r="B105" t="str">
-        <v>Greenhouse job board, direct fetch</v>
+        <v>General intern/co-op search</v>
       </c>
       <c r="C105" t="str">
-        <v>2026-09-20: only 4 open roles today (Mechanical Engineering Machinist, IT Specialist, part-time Office Manager, Business Development Leader) — none are co-op/intern, none carry season/date info. A 'Robotics and AI Co-op' listing found via search appears stale/closed.</v>
+        <v>2026-09-20: only an unrelated Austin, TX mechanical engineering intern reference found, no 2027/season confirmation, no Boston presence.</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Diligent Robotics</v>
+        <v>Veo Robotics</v>
       </c>
       <c r="B106" t="str">
         <v>General intern/co-op search</v>
       </c>
       <c r="C106" t="str">
-        <v>2026-09-20: only an unrelated Austin, TX mechanical engineering intern reference found, no 2027/season confirmation, no Boston presence.</v>
+        <v>2026-09-20: no 2027-specific posting found; general hardware/mechanical engineering intern role description only, no season stated.</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Veo Robotics</v>
+        <v>Coherent / II-VI</v>
       </c>
       <c r="B107" t="str">
-        <v>General intern/co-op search</v>
+        <v>General mechanical co-op search</v>
       </c>
       <c r="C107" t="str">
-        <v>2026-09-20: no 2027-specific posting found; general hardware/mechanical engineering intern role description only, no season stated.</v>
+        <v>2026-09-20: no Spring 2027 mechanical co-op posting found specific to this company.</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Coherent / II-VI</v>
+        <v>Fisker / Canoo / Nikola / VinFast / Karma Automotive</v>
       </c>
       <c r="B108" t="str">
-        <v>General mechanical co-op search</v>
+        <v>General intern/co-op search</v>
       </c>
       <c r="C108" t="str">
-        <v>2026-09-20: no Spring 2027 mechanical co-op posting found specific to this company.</v>
+        <v>2026-09-20: no active internship/co-op postings found at any of these; several (Fisker, Canoo, Nikola) have known bankruptcy/financial-distress history that likely explains absent active recruiting.</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Fisker / Canoo / Nikola / VinFast / Karma Automotive</v>
+        <v>GE Aerospace (Lynn, MA)</v>
       </c>
       <c r="B109" t="str">
-        <v>General intern/co-op search</v>
+        <v>'Trainee Co-Op' trade reqs (Carpentry R5034333, CNC R5034331) and 'Engines Engineering Co-op - Computer or Software Engineering' track</v>
       </c>
       <c r="C109" t="str">
-        <v>2026-09-20: no active internship/co-op postings found at any of these; several (Fisker, Canoo, Nikola) have known bankruptcy/financial-distress history that likely explains absent active recruiting.</v>
+        <v>2026-09-21: Trainee Co-Op reqs are skilled-trade apprentice positions, not engineering-degree roles — discipline mismatch. Software/Computer Engineering track — discipline mismatch. No new mechanical/aero engineering-degree Spring 2027 Lynn req found beyond the already-tracked Engines Engineering Co-op (R5029617-1).</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B110" t="str">
+        <v>'Cyber Security Co-op (Winter/Spring 2027)', Group 11-10</v>
+      </c>
+      <c r="C110" t="str">
+        <v>2026-09-21: live, in-season, but discipline mismatch (cybersecurity, not on Hamza's target list). Also found a 'Structural &amp; Thermal Fluids Engineering' co-op listing dated Jan-June 2025 — expired prior cycle, not current.</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Moderna</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Co-Op, CMC Development (Spring 2027), Norwood MA</v>
+      </c>
+      <c r="C111" t="str">
+        <v>2026-09-21: title/season/pay corroborated via a Workopia aggregator mirror, but the exact canonical Workday req string could not be confirmed (agent flagged the URL itself as unconfirmed) and the primary modernatx.wd1.myworkdayjobs.com page returned empty — fails the verifiable-URL bar, not added. Discipline is also Chemical/Bio/Biomedical Engineering, a weaker fit than the sibling Applied Technologies req (which was added to `rows` as Partial). Worth a direct re-check with a different fetch method.</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Beta Technologies</v>
+      </c>
+      <c r="B112" t="str">
+        <v>'2026-2027 BETA Internship' program (Vermont &amp; Raleigh NC), Mechanical Engineering track</v>
+      </c>
+      <c r="C112" t="str">
+        <v>2026-09-21: program exists but labeled generically '2026-2027' with no Spring-2027-specific dated posting found. Worth digging into specific team/track postings (Motors, Charge, Lift Kit, M&amp;P, Manufacturing) for a dated version.</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Archer Aviation</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Mechanical / Manufacturing &amp; Process intern roles, San Jose CA</v>
+      </c>
+      <c r="C113" t="str">
+        <v>2026-09-21: structured as a 10-week Summer program; no Spring 2027 co-op found.</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Wisk Aero</v>
+      </c>
+      <c r="B114" t="str">
+        <v>General internship search</v>
+      </c>
+      <c r="C114" t="str">
+        <v>2026-09-21: only Summer 2025/2026 program info found; no Spring 2027 postings.</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Mercury Systems (Andover, MA)</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Mechanical Engineering Intern (season undetermined); '2027 Software Engineer Co-Op' (July-December 2026)</v>
+      </c>
+      <c r="C115" t="str">
+        <v>2026-09-21: the software co-op is explicitly wrong season and discipline. No confirmed Spring 2027 Mechanical Engineering posting located.</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Cognex (Natick, MA)</v>
+      </c>
+      <c r="B116" t="str">
+        <v>'Core Vision Intern' (R0010844)</v>
+      </c>
+      <c r="C116" t="str">
+        <v>2026-09-21: software/ML role, discipline mismatch. No mechanical Spring 2027 co-op located.</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Abiomed (Danvers, MA)</v>
+      </c>
+      <c r="B117" t="str">
+        <v>General co-op program search</v>
+      </c>
+      <c r="C117" t="str">
+        <v>2026-09-21: co-op program exists generally but no specific Spring 2027 posting found.</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Haemonetics (Boston, MA)</v>
+      </c>
+      <c r="B118" t="str">
+        <v>R&amp;D Engineering internship track (Biomedical/Mechanical/Materials)</v>
+      </c>
+      <c r="C118" t="str">
+        <v>2026-09-21: only Summer 2026-dated postings found; no Spring 2027 posting.</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Vertex Pharmaceuticals</v>
+      </c>
+      <c r="B119" t="str">
+        <v>MSAT/process engineering co-op track</v>
+      </c>
+      <c r="C119" t="str">
+        <v>2026-09-21: co-ops confirmed to run Jan-June spring cycles generally, but no specific Spring 2027 req found; official co-ops page returned 403 on fetch.</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Elbit Systems of America (Merrimack, NH)</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Mechanical Engineering intern roles</v>
+      </c>
+      <c r="C120" t="str">
+        <v>2026-09-21: role types exist generally; no Spring-2027-dated posting found.</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Saab Inc</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Full current listing at saab.com/career/job-opportunities</v>
+      </c>
+      <c r="C121" t="str">
+        <v>2026-09-21: five Summer 2027 postings (East Syracuse NY / West Lafayette IN, wrong season) plus one 'Systems Engineering Co-Op (Spring - Summer 2027)' (East Syracuse NY) whose exact start date couldn't be pinned down within the verification bar — excluded as unconfirmed rather than reported. Worth a direct fetch attempt next run to clarify the start date.</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Divergent3D</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Engineering Intern, Torrance CA</v>
+      </c>
+      <c r="C122" t="str">
+        <v>2026-09-21: only a Summer 2027 posting found. Wrong season.</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Emerson / National Instruments (Test &amp; Measurement)</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Mechanical Engineering Co-op, Elyria OH</v>
+      </c>
+      <c r="C123" t="str">
+        <v>2026-09-21: dated Summer 2027. Wrong season.</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Mercury Marine (Fond du Lac, WI)</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Mechanical/Quality/Metallurgical Engineering Co-op (Spring or Fall Term)</v>
+      </c>
+      <c r="C124" t="str">
+        <v>2026-09-21: aggregator mirror confirmed the currently-open term windows are 'January-August 2026' or 'May-December 2026' — the current/already-underway cycle, not the Jan 2027 (Spring 2027) cycle needed. Wrong season.</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Illumina</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Process/Manufacturing engineering internship track</v>
+      </c>
+      <c r="C125" t="str">
+        <v>2026-09-21: no Spring-2027-dated posting found; Summer 2027 postings expected to open Oct 2026-Feb 2027, not yet live.</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>10x Genomics (Pleasanton, CA)</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Manufacturing/Mechanical Engineering intern roles</v>
+      </c>
+      <c r="C126" t="str">
+        <v>2026-09-21: postings found appear to be prior-cycle (2025/2026 summer); no Spring 2027 confirmed.</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>American Superconductor (AMSC, Ayer, MA)</v>
+      </c>
+      <c r="B127" t="str">
+        <v>'Superconducting Magnet R&amp;D Intern' / 'SPS Intern' (US-citizen/ITAR roles)</v>
+      </c>
+      <c r="C127" t="str">
+        <v>2026-09-21: roles found but season could not be confirmed — job board returned 403 on fetch.</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Hadrian / Machina Labs / ICON / Boston Engineering / Bruker / Zeiss Industrial Metrology / Nikon Metrology / Overair / Form Energy</v>
+      </c>
+      <c r="B128" t="str">
+        <v>General mechanical/manufacturing engineering intern/co-op search, each company</v>
+      </c>
+      <c r="C128" t="str">
+        <v>2026-09-21: no specific Winter 2026/Spring 2027-dated postings could be located or confirmed for any of these in this pass.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C128"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 8 checked-excluded, 3 upgraded Partial->Yes (2026-09-21 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011rXkeVb4SeoKq5FHcMwVez
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -2372,13 +2372,13 @@
         <v>$41,011–$53,315/yr base (co-op salary range) + bonus/equity eligibility per posting</v>
       </c>
       <c r="H62" t="str">
-        <v>https://www.linkedin.com/jobs/view/mechanical-engineer-co-op-spring-2027-at-leonardo-drs-4451960539</v>
+        <v>https://careers.leonardodrs.com/job/Bridgeton-Mechanical-Engineer-Co-Op-%28Spring-2027%29-MO-63044/1418392000/</v>
       </c>
       <c r="I62" t="str">
-        <v>Partial — confirmed via LinkedIn's own job listing (title/season/pay/location) corroborated by a Workopia aggregator mirror quoting the same details; Leonardo DRS's own careers.leonardodrs.com posting for this specific req was not independently located/opened, so the primary employer page itself couldn't be directly confirmed.</v>
+        <v>Yes — fetched directly on Leonardo DRS's own careers.leonardodrs.com ATS (job ID 115172, posted 2026-09-09), confirmed open. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
       </c>
       <c r="J62" t="str">
-        <v>Land Systems division, Bridgeton, MO site. New company, first Leonardo DRS posting tracked. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
+        <v>Land Systems division, Bridgeton, MO site. Junior+ standing, 1+ prior internship/co-op required, CAD (Creo/SolidWorks) required. No citizenship requirement stated on this posting. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
       </c>
     </row>
     <row r="63">
@@ -2392,7 +2392,7 @@
         <v>Systems Engineering</v>
       </c>
       <c r="D63" t="str">
-        <v>January – June 2027</v>
+        <v>January 11 – June 30, 2027</v>
       </c>
       <c r="E63" t="str">
         <v>Acton, MA</v>
@@ -2401,16 +2401,16 @@
         <v>25</v>
       </c>
       <c r="G63" t="str">
-        <v>Not independently confirmed (see $25–34/hr range on sibling Insulet Acton reqs)</v>
+        <v>$25.00–$34.00/hr</v>
       </c>
       <c r="H63" t="str">
         <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Next-Gen-Platforms--NGP--Systems-Engineering--January-June-2027--Onsite-_REQ-2026-18071</v>
       </c>
       <c r="I63" t="str">
-        <v>Partial — title/season/location/req ID corroborated by two independent aggregator mirrors (Workopia, Zapply) quoting this exact canonical Workday URL; the live Workday page itself returned empty on repeated direct fetch attempts across three runs. Resolves the prior 'no verifiable URL' blocker.</v>
+        <v>Yes — fetched directly via Insulet's own Workday CXS job API (not an aggregator mirror), confirmed open, posted 5 days prior, application deadline 2026-12-31. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
       </c>
       <c r="J63" t="str">
-        <v>Boston metro (Acton), onsite. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
+        <v>Boston metro (Acton), onsite. US work authorization required, no sponsorship. 3.0 GPA minimum. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
       </c>
     </row>
     <row r="64">
@@ -2436,13 +2436,13 @@
         <v>$20.00–$60.00/hr per posting</v>
       </c>
       <c r="H64" t="str">
-        <v>https://jobs.biospace.com/job/3072468/co-op-applied-technologies-spring-2027-/</v>
+        <v>https://modernatx.wd1.myworkdayjobs.com/en-US/M_tx/job/Co-Op--Applied-Technologies--Spring-2027-_R19735</v>
       </c>
       <c r="I64" t="str">
-        <v>Partial — full posting content (title, dates, pay, citizenship requirement, open status) fetched and rendered directly at this biospace.com job-board listing, which mirrors Moderna's official Workday posting; Moderna's own modernatx.wd1.myworkdayjobs.com page returned empty on direct fetch, so the primary employer page wasn't independently confirmed.</v>
+        <v>Yes — fetched directly via Moderna's own Workday CXS job API (req R19735), returned live JSON confirming title, dates, pay, and open status. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check); the previously-used biospace.com mirror (job 3072468) appears to be the same underlying posting under the job board's own listing ID, not a separate role.</v>
       </c>
       <c r="J64" t="str">
-        <v>Restricted to US persons (citizens/permanent residents/asylees/refugees). Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
+        <v>Restricted to US persons (citizens/permanent residents/asylees/refugees) per prior mirror-sourced check, not re-confirmed word-for-word on this pass. Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
       </c>
     </row>
   </sheetData>
@@ -2454,7 +2454,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C137"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -3869,9 +3869,108 @@
         <v>2026-09-21: no specific Winter 2026/Spring 2027-dated postings could be located or confirmed for any of these in this pass.</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>BAE Systems (Merrimack, NH)</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Mechanical/systems engineering intern/co-op search</v>
+      </c>
+      <c r="C129" t="str">
+        <v>2026-09-21 ~07:00 UTC: the only 'Spring and Summer 2027' Mechanical Engineering Co-op found is located in Cedar Rapids, IA, not Merrimack, NH — no Merrimack-specific mechanical/systems co-op located.</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Sig Sauer (Newington, NH)</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Mechanical engineering intern/co-op search</v>
+      </c>
+      <c r="C130" t="str">
+        <v>2026-09-21 ~07:00 UTC: only a Spring 2027 Electrical/Computer Engineering (Uncrewed Systems) posting found — discipline mismatch. No mechanical-specific Spring 2027 posting located.</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Textron Systems (Wilmington, MA)</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Fresh sweep for mechanical engineer intern/co-op reqs</v>
+      </c>
+      <c r="C131" t="str">
+        <v>2026-09-21 ~07:00 UTC: the only '2027 Intern - Mechanical Engineer' found this pass is at Howe &amp; Howe (Waterboro, ME), a different Textron subsidiary/location, with season/year unconfirmed — not the same as Wilmington, MA. No qualifying Wilmington MA mechanical req found.</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Raytheon BBN (Cambridge, MA)</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Mechanical/systems engineering co-op search</v>
+      </c>
+      <c r="C132" t="str">
+        <v>2026-09-21 ~07:00 UTC: no mechanical/systems engineering co-op found — BBN's internships lean AI/computing; general RTX Spring/Winter 2027 co-ops (already tracked elsewhere) are at other sites.</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Eversource (MA)</v>
+      </c>
+      <c r="B133" t="str">
+        <v>2027 Engineering Internships</v>
+      </c>
+      <c r="C133" t="str">
+        <v>2026-09-21 ~07:00 UTC: posting language ('energize your summer') reads as a Summer program despite broadly referencing '2027' — no explicit Winter/Spring season stated. Excluded on season-ambiguity grounds.</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>National Grid</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Engineering internship/co-op search</v>
+      </c>
+      <c r="C134" t="str">
+        <v>2026-09-21 ~07:00 UTC: no qualifying Winter 2026/Spring 2027 posting found.</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>MassDOT</v>
+      </c>
+      <c r="B135" t="str">
+        <v>Engineering Co-op and Internship programs</v>
+      </c>
+      <c r="C135" t="str">
+        <v>2026-09-21 ~07:00 UTC: Co-op program runs June/July-December (Fall) and Internship runs June-August (Summer) by design — no Winter 2026/Spring 2027 track exists. Also primarily civil engineering, not on Hamza's discipline list.</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Applied AI Engineer Co-op - Spring 2027 (Lynn, MA area)</v>
+      </c>
+      <c r="C136" t="str">
+        <v>2026-09-21 ~07:00 UTC: a new Lynn-area Spring 2027 req was found beyond the already-tracked Engines Engineering Co-op, but it's a software/AI role — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Saab Inc (East Syracuse, NY)</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Systems Engineering Co-Op — exact posting title is 'Spring - Summer 2027'</v>
+      </c>
+      <c r="C137" t="str">
+        <v>2026-09-21 ~07:00 UTC: fetched directly, confirmed live (link: saab.com/career/job-opportunities/systems-engineering-co-op-spring---summer-20272, $20.27-$22.30/hr + relocation bonus), but the term itself blends spring and summer into one combined window rather than a clean Winter/Spring-only co-op — judged closer to the common Summer 2027 wave Hamza asked to exclude than to a true Fall-through-Spring term. Flagged here rather than added; worth Hamza's own judgment call if he wants borderline spring/summer-blended terms reconsidered.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C128"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C137"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 9 checked-excluded (2026-09-21 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5iFTs26j7LmiQ2vJdvYqM
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J66"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -856,127 +856,127 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Boeing (South Carolina)</v>
+        <v>General Dynamics Mission Systems</v>
       </c>
       <c r="B15" t="str">
-        <v>2026 Specialty Program – BSC Co-op – Engineering Internship Program (Materials &amp; Process Eng, Industrial Eng)</v>
+        <v>Mechanical Engineering Co-Op (January – May 2027)</v>
       </c>
       <c r="C15" t="str">
-        <v>Materials/Process Engineering, Industrial Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D15" t="str">
-        <v>Fall 2026–Spring 2027 (6-month co-op)</v>
+        <v>January - May 2027</v>
       </c>
       <c r="E15" t="str">
-        <v>North Charleston, SC (Boeing SC site)</v>
+        <v>McLeansville, NC</v>
       </c>
       <c r="F15">
-        <v>850</v>
+        <v>620</v>
       </c>
       <c r="G15" t="str">
-        <v>Not stated on posting</v>
+        <v>$26.00–$29.00/hr</v>
       </c>
       <c r="H15" t="str">
-        <v>https://boeing.wd1.myworkdayjobs.com/en-US/INTERN/job/XMLNAME-2026-Specialty-Program---BSC-Co-op---Engineering-Internship-Program_JR2026491626</v>
+        <v>https://careers-gdms.icims.com/jobs/74530/mechanical-engineering-co-op---%28january---may-2027%29/job</v>
       </c>
       <c r="I15" t="str">
-        <v>Partial — official Boeing/Workday domain, title/search snippet confirms Fall 2026–Spring 2027 span, but page is JS-rendered and blocked automated fetch. Verify live in-browser before applying.</v>
+        <v>Partial — corroborated across multiple independent sources (aggregator mirror quoting exact title/pay/dates/location, Glassdoor, career.io) with consistent details, but the icims URL redirected to a generic GDMS careers landing page (no job content) and the gd.com mirror URL returned HTTP 403 on direct fetch. Could not independently confirm current open/closed status. Verify live in-browser before applying.</v>
       </c>
       <c r="J15" t="str">
-        <v>6-month co-op spanning into Spring 2027.</v>
+        <v>Not Boston-area. Sibling req 'Mechanical Engineering Co-Op (July–December 2026)' exists at the same site — different season, not this one. Likely requires US citizenship (ITAR/clearance) as with other GDMS reqs.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Boeing</v>
+        <v>Boeing (South Carolina)</v>
       </c>
       <c r="B16" t="str">
-        <v>Drexel Internship Fall Co-op 2026 – Engineering (Software, Industrial, Manufacturing, Reliability/Maintainability, Systems, Mechanical Systems, Structures, Wire Install/Design)</v>
+        <v>2026 Specialty Program – BSC Co-op – Engineering Internship Program (Materials &amp; Process Eng, Industrial Eng)</v>
       </c>
       <c r="C16" t="str">
-        <v>Systems / Mechanical Systems / Structures / Manufacturing Engineering</v>
+        <v>Materials/Process Engineering, Industrial Engineering</v>
       </c>
       <c r="D16" t="str">
         <v>Fall 2026–Spring 2027 (6-month co-op)</v>
       </c>
       <c r="E16" t="str">
-        <v>Not specified on posting (Drexel University co-op partnership — site varies by team)</v>
+        <v>North Charleston, SC (Boeing SC site)</v>
+      </c>
+      <c r="F16">
+        <v>850</v>
       </c>
       <c r="G16" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H16" t="str">
-        <v>https://boeing.wd1.myworkdayjobs.com/en-US/INTERN/job/Drexel-Internship-Fall-Co-op-2026---Engineering_JR2026515142</v>
+        <v>https://boeing.wd1.myworkdayjobs.com/en-US/INTERN/job/XMLNAME-2026-Specialty-Program---BSC-Co-op---Engineering-Internship-Program_JR2026491626</v>
       </c>
       <c r="I16" t="str">
         <v>Partial — official Boeing/Workday domain, title/search snippet confirms Fall 2026–Spring 2027 span, but page is JS-rendered and blocked automated fetch. Verify live in-browser before applying.</v>
       </c>
       <c r="J16" t="str">
-        <v>Restricted to Drexel University co-op program students — check eligibility before applying.</v>
+        <v>6-month co-op spanning into Spring 2027.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>John Deere</v>
+        <v>Boeing</v>
       </c>
       <c r="B17" t="str">
-        <v>Part-Time Student – Factory Engineering</v>
+        <v>Drexel Internship Fall Co-op 2026 – Engineering (Software, Industrial, Manufacturing, Reliability/Maintainability, Systems, Mechanical Systems, Structures, Wire Install/Design)</v>
       </c>
       <c r="C17" t="str">
-        <v>Manufacturing / Factory Engineering</v>
+        <v>Systems / Mechanical Systems / Structures / Manufacturing Engineering</v>
       </c>
       <c r="D17" t="str">
-        <v>Year-round part-time during school year (covers Winter 2026 &amp; Spring 2027)</v>
+        <v>Fall 2026–Spring 2027 (6-month co-op)</v>
       </c>
       <c r="E17" t="str">
-        <v>East Moline, IL</v>
-      </c>
-      <c r="F17">
-        <v>980</v>
+        <v>Not specified on posting (Drexel University co-op partnership — site varies by team)</v>
       </c>
       <c r="G17" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H17" t="str">
-        <v>https://careers.deere.com/careers/job/137468659226-part-time-student-factory-engineering-east-moline-il-east-moline-illinois-united-states?domain=johndeere.com</v>
+        <v>https://boeing.wd1.myworkdayjobs.com/en-US/INTERN/job/Drexel-Internship-Fall-Co-op-2026---Engineering_JR2026515142</v>
       </c>
       <c r="I17" t="str">
-        <v>Partial — official careers.deere.com domain, page structure confirmed real but automated fetch couldn't render full listing text. Verify live in-browser before applying.</v>
+        <v>Partial — official Boeing/Workday domain, title/search snippet confirms Fall 2026–Spring 2027 span, but page is JS-rendered and blocked automated fetch. Verify live in-browser before applying.</v>
       </c>
       <c r="J17" t="str">
-        <v>16–20 hrs/wk during school year, 30–40 hrs/wk in summer. Requires graduation Dec 2026 or later. CMM/dimensional-analysis work in production environment.</v>
+        <v>Restricted to Drexel University co-op program students — check eligibility before applying.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>GE Vernova (Nuclear)</v>
+        <v>John Deere</v>
       </c>
       <c r="B18" t="str">
-        <v>Nuclear Engineering Co-Op/Intern</v>
+        <v>Part-Time Student – Factory Engineering</v>
       </c>
       <c r="C18" t="str">
-        <v>Nuclear / Mechanical / Chemical / Electrical / Materials / Controls / Civil-Structural Engineering</v>
+        <v>Manufacturing / Factory Engineering</v>
       </c>
       <c r="D18" t="str">
-        <v>Spring 2027</v>
+        <v>Year-round part-time during school year (covers Winter 2026 &amp; Spring 2027)</v>
       </c>
       <c r="E18" t="str">
-        <v>Wilmington, NC</v>
+        <v>East Moline, IL</v>
       </c>
       <c r="F18">
-        <v>720</v>
+        <v>980</v>
       </c>
       <c r="G18" t="str">
-        <v>$1,000–$2,000/week (varies by degree level)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H18" t="str">
-        <v>https://careers.gevernova.com/ge-vernova-nuclear-engineering-co-op-intern-spring-2027/job/R5048552</v>
+        <v>https://careers.deere.com/careers/job/137468659226-part-time-student-factory-engineering-east-moline-il-east-moline-illinois-united-states?domain=johndeere.com</v>
       </c>
       <c r="I18" t="str">
-        <v>Yes — fetched directly, confirmed OPEN, posted Aug 7, 2026 (within freshness window)</v>
+        <v>Partial — official careers.deere.com domain, page structure confirmed real but automated fetch couldn't render full listing text. Verify live in-browser before applying.</v>
       </c>
       <c r="J18" t="str">
-        <v>Housing/relocation assistance if 50+ mi from site. Must be work-authorized without sponsorship.</v>
+        <v>16–20 hrs/wk during school year, 30–40 hrs/wk in summer. Requires graduation Dec 2026 or later. CMM/dimensional-analysis work in production environment.</v>
       </c>
     </row>
     <row r="19">
@@ -984,25 +984,25 @@
         <v>GE Vernova (Nuclear)</v>
       </c>
       <c r="B19" t="str">
-        <v>Nuclear – Field Services Spring Internship</v>
+        <v>Nuclear Engineering Co-Op/Intern</v>
       </c>
       <c r="C19" t="str">
-        <v>Engineering / Engineering Technology</v>
+        <v>Nuclear / Mechanical / Chemical / Electrical / Materials / Controls / Civil-Structural Engineering</v>
       </c>
       <c r="D19" t="str">
-        <v>Spring 2027 (starts January 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E19" t="str">
-        <v>Wilmington, NC (up to 70% travel to nuclear plant sites)</v>
+        <v>Wilmington, NC</v>
       </c>
       <c r="F19">
         <v>720</v>
       </c>
       <c r="G19" t="str">
-        <v>$1,000–$2,000/week (varies by experience)</v>
+        <v>$1,000–$2,000/week (varies by degree level)</v>
       </c>
       <c r="H19" t="str">
-        <v>https://careers.gevernova.com/ge-vernova-nuclear-field-services-spring-internship-2027/job/R5049161</v>
+        <v>https://careers.gevernova.com/ge-vernova-nuclear-engineering-co-op-intern-spring-2027/job/R5048552</v>
       </c>
       <c r="I19" t="str">
         <v>Yes — fetched directly, confirmed OPEN, posted Aug 7, 2026 (within freshness window)</v>
@@ -1013,95 +1013,95 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NASA (Pathways Internship Program)</v>
+        <v>GE Vernova (Nuclear)</v>
       </c>
       <c r="B20" t="str">
-        <v>Pathways Internship – various engineering disciplines</v>
+        <v>Nuclear – Field Services Spring Internship</v>
       </c>
       <c r="C20" t="str">
-        <v>Mechanical / Systems / Aerospace (varies by center &amp; opening)</v>
+        <v>Engineering / Engineering Technology</v>
       </c>
       <c r="D20" t="str">
-        <v>Spring 2027 (apply via USAJOBS; deadline Sept 14, 2026)</v>
+        <v>Spring 2027 (starts January 2027)</v>
       </c>
       <c r="E20" t="str">
-        <v>Varies — multiple NASA centers nationwide</v>
+        <v>Wilmington, NC (up to 70% travel to nuclear plant sites)</v>
+      </c>
+      <c r="F20">
+        <v>720</v>
       </c>
       <c r="G20" t="str">
-        <v>Federal student stipend scale, varies by degree level (not a fixed rate)</v>
+        <v>$1,000–$2,000/week (varies by experience)</v>
       </c>
       <c r="H20" t="str">
-        <v>https://www.usajobs.gov/</v>
+        <v>https://careers.gevernova.com/ge-vernova-nuclear-field-services-spring-internship-2027/job/R5049161</v>
       </c>
       <c r="I20" t="str">
-        <v>Yes — usajobs.gov is the live, official application portal (this is a program, not a single job req — search USAJOBS for open NASA Pathways postings)</v>
+        <v>Yes — fetched directly, confirmed OPEN, posted Aug 7, 2026 (within freshness window)</v>
       </c>
       <c r="J20" t="str">
-        <v>US citizenship required. Cumulative GPA 2.9+ required. Spring 2027 window opens on USAJOBS in fall 2026.</v>
+        <v>Housing/relocation assistance if 50+ mi from site. Must be work-authorized without sponsorship.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>MIT Lincoln Laboratory</v>
+        <v>NASA (Pathways Internship Program)</v>
       </c>
       <c r="B21" t="str">
-        <v>Microfabrication Industrial Engineering Co-Op (Group 08-35, Microelectronics Laboratory)</v>
+        <v>Pathways Internship – various engineering disciplines</v>
       </c>
       <c r="C21" t="str">
-        <v>Industrial Engineering (Systems Eng/Ops Research/Manufacturing Eng/CS also accepted)</v>
+        <v>Mechanical / Systems / Aerospace (varies by center &amp; opening)</v>
       </c>
       <c r="D21" t="str">
-        <v>Jan–August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+        <v>Spring 2027 (apply via USAJOBS; deadline Sept 14, 2026)</v>
       </c>
       <c r="E21" t="str">
-        <v>Lexington, MA</v>
-      </c>
-      <c r="F21">
-        <v>13</v>
+        <v>Varies — multiple NASA centers nationwide</v>
       </c>
       <c r="G21" t="str">
-        <v>$24.50–$31.00/hr (2025 technical co-op rate; subject to review for 2027)</v>
+        <v>Federal student stipend scale, varies by degree level (not a fixed rate)</v>
       </c>
       <c r="H21" t="str">
-        <v>https://careers.ll.mit.edu/job/Lexington-Microfab-Industrial-Eng_-Co-Op-Microelectronics-Laboratory-%28Jan-August-2027%29-Group-08-35-MA-02420/1370647300/</v>
+        <v>https://www.usajobs.gov/</v>
       </c>
       <c r="I21" t="str">
-        <v>Yes — fetched directly, active Apply link, no closed/expired banner. Posted Aug 26, 2026.</v>
+        <v>Yes — usajobs.gov is the live, official application portal (this is a program, not a single job req — search USAJOBS for open NASA Pathways postings)</v>
       </c>
       <c r="J21" t="str">
-        <v>Requires US citizenship + eligibility for Secret-level DoD clearance. Sibling req 'Microfabrication Engineering Co-Op' (same Jan–Aug 2027 window, Group 08-35) also exists but wasn't separately fetched.</v>
+        <v>US citizenship required. Cumulative GPA 2.9+ required. Spring 2027 window opens on USAJOBS in fall 2026.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Draper Laboratory</v>
+        <v>MIT Lincoln Laboratory</v>
       </c>
       <c r="B22" t="str">
-        <v>Systems Engineering Co-Op (Spring 2027)</v>
+        <v>Microfabrication Industrial Engineering Co-Op (Group 08-35, Microelectronics Laboratory)</v>
       </c>
       <c r="C22" t="str">
-        <v>Systems Design Engineering</v>
+        <v>Industrial Engineering (Systems Eng/Ops Research/Manufacturing Eng/CS also accepted)</v>
       </c>
       <c r="D22" t="str">
-        <v>Spring 2027</v>
+        <v>Jan–August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E22" t="str">
-        <v>Cambridge, MA</v>
+        <v>Lexington, MA</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G22" t="str">
-        <v>Not stated on posting</v>
+        <v>$24.50–$31.00/hr (2025 technical co-op rate; subject to review for 2027)</v>
       </c>
       <c r="H22" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Systems-Engineering-Co-Op--Spring-2027-_JR002882</v>
+        <v>https://careers.ll.mit.edu/job/Lexington-Microfab-Industrial-Eng_-Co-Op-Microelectronics-Laboratory-%28Jan-August-2027%29-Group-08-35-MA-02420/1370647300/</v>
       </c>
       <c r="I22" t="str">
-        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~9 days ago as of this check.</v>
+        <v>Yes — fetched directly, active Apply link, no closed/expired banner. Posted Aug 26, 2026.</v>
       </c>
       <c r="J22" t="str">
-        <v>GAD division placement. Pay $20.00-$45.00/hr per posting.</v>
+        <v>Requires US citizenship + eligibility for Secret-level DoD clearance. Sibling req 'Microfabrication Engineering Co-Op' (same Jan–Aug 2027 window, Group 08-35) also exists but wasn't separately fetched.</v>
       </c>
     </row>
     <row r="23">
@@ -1109,10 +1109,10 @@
         <v>Draper Laboratory</v>
       </c>
       <c r="B23" t="str">
-        <v>Electro-Mechanical Instrument Co-op (Spring 2027)</v>
+        <v>Systems Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C23" t="str">
-        <v>Hardware / Mechanical Engineering</v>
+        <v>Systems Design Engineering</v>
       </c>
       <c r="D23" t="str">
         <v>Spring 2027</v>
@@ -1127,77 +1127,77 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H23" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Electro-Mechanical-Instrument-Co-op--Spring-2027-_JR002883-1</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Systems-Engineering-Co-Op--Spring-2027-_JR002882</v>
       </c>
       <c r="I23" t="str">
-        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~20 days ago as of this check.</v>
+        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~9 days ago as of this check.</v>
       </c>
       <c r="J23" t="str">
-        <v>US Citizenship required — Draper cannot sponsor/hire H1B or Student Visa holders; dual citizens not eligible. CAD (Creo/SolidWorks), FEA (ANSYS/COMSOL) skills mentioned. Pay $20.00-$45.00/hr per posting.</v>
+        <v>GAD division placement. Pay $20.00-$45.00/hr per posting.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Amazon Robotics</v>
+        <v>Draper Laboratory</v>
       </c>
       <c r="B24" t="str">
-        <v>Industrial Development Engineer Intern/Co-op, ROBOTICS – 2027</v>
+        <v>Electro-Mechanical Instrument Co-op (Spring 2027)</v>
       </c>
       <c r="C24" t="str">
-        <v>Industrial Engineering / Robotics Manufacturing &amp; Technical Operations</v>
+        <v>Hardware / Mechanical Engineering</v>
       </c>
       <c r="D24" t="str">
-        <v>2027 (single req covers summer intern, spring co-op, and fall co-op placement — Spring 2027 placement is NOT guaranteed)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E24" t="str">
-        <v>Westborough, MA (also Arlington, VA and North Reading, MA)</v>
+        <v>Cambridge, MA</v>
       </c>
       <c r="F24">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="G24" t="str">
-        <v>$82,450/year (Amazon standard pay-transparency disclosure for this req)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H24" t="str">
-        <v>https://www.amazon.jobs/en/jobs/10536817/industrial-development-engineer-intern-co-op-robotics-2027</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Electro-Mechanical-Instrument-Co-op--Spring-2027-_JR002883-1</v>
       </c>
       <c r="I24" t="str">
-        <v>Yes — fetched directly, page loaded fully, role open. UPDATE (2026-09-20): posting text now explicitly reads 'Robotics Industrial Engineer 2027 summer intern, spring co-op, and fall co-op roles' — confirms Spring 2027 co-op is one of the terms this req covers (previously ambiguous).</v>
+        <v>Yes — upgraded 2026-09-20: confirmed via direct fetch of Draper's Workday CXS job API (title, description, pay range all returned), posted ~20 days ago as of this check.</v>
       </c>
       <c r="J24" t="str">
-        <v>Requires graduation between Dec 2026–Aug 2027. Prior req IDs for this role (e.g. 3088739, the 2026-cycle version) are confirmed dead (404).</v>
+        <v>US Citizenship required — Draper cannot sponsor/hire H1B or Student Visa holders; dual citizens not eligible. CAD (Creo/SolidWorks), FEA (ANSYS/COMSOL) skills mentioned. Pay $20.00-$45.00/hr per posting.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Formlabs</v>
+        <v>Amazon Robotics</v>
       </c>
       <c r="B25" t="str">
-        <v>Mechanical Engineering Intern (Winter/Spring 2027)</v>
+        <v>Industrial Development Engineer Intern/Co-op, ROBOTICS – 2027</v>
       </c>
       <c r="C25" t="str">
-        <v>Mechanical / Hardware Engineering</v>
+        <v>Industrial Engineering / Robotics Manufacturing &amp; Technical Operations</v>
       </c>
       <c r="D25" t="str">
-        <v>Winter/Spring 2027 (January–April)</v>
+        <v>2027 (single req covers summer intern, spring co-op, and fall co-op placement — Spring 2027 placement is NOT guaranteed)</v>
       </c>
       <c r="E25" t="str">
-        <v>Somerville, MA</v>
+        <v>Westborough, MA (also Arlington, VA and North Reading, MA)</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="G25" t="str">
-        <v>$1,575–$1,950/week (salaried, full-time)</v>
+        <v>$82,450/year (Amazon standard pay-transparency disclosure for this req)</v>
       </c>
       <c r="H25" t="str">
-        <v>https://careers.formlabs.com/job/8130829/apply/?gh_jid=8130829</v>
+        <v>https://www.amazon.jobs/en/jobs/10536817/industrial-development-engineer-intern-co-op-robotics-2027</v>
       </c>
       <c r="I25" t="str">
-        <v>Yes — fetched directly, page live, season/location/pay confirmed in posting text.</v>
+        <v>Yes — fetched directly, page loaded fully, role open. UPDATE (2026-09-20): posting text now explicitly reads 'Robotics Industrial Engineer 2027 summer intern, spring co-op, and fall co-op roles' — confirms Spring 2027 co-op is one of the terms this req covers (previously ambiguous).</v>
       </c>
       <c r="J25" t="str">
-        <v>Boston metro. Portfolio of prior engineering work required — application not considered without one.</v>
+        <v>Requires graduation between Dec 2026–Aug 2027. Prior req IDs for this role (e.g. 3088739, the 2026-cycle version) are confirmed dead (404).</v>
       </c>
     </row>
     <row r="26">
@@ -1205,10 +1205,10 @@
         <v>Formlabs</v>
       </c>
       <c r="B26" t="str">
-        <v>Hardware Systems Integration Intern (Winter/Spring 2027)</v>
+        <v>Mechanical Engineering Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C26" t="str">
-        <v>Hardware / Electro-Mechanical Engineering</v>
+        <v>Mechanical / Hardware Engineering</v>
       </c>
       <c r="D26" t="str">
         <v>Winter/Spring 2027 (January–April)</v>
@@ -1220,144 +1220,144 @@
         <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Not stated on posting</v>
+        <v>$1,575–$1,950/week (salaried, full-time)</v>
       </c>
       <c r="H26" t="str">
-        <v>https://careers.formlabs.com/job/8172004/apply/?gh_jid=8172004</v>
+        <v>https://careers.formlabs.com/job/8130829/apply/?gh_jid=8130829</v>
       </c>
       <c r="I26" t="str">
-        <v>Yes — fetched directly, page live, title/season/location confirmed in posting text.</v>
+        <v>Yes — fetched directly, page live, season/location/pay confirmed in posting text.</v>
       </c>
       <c r="J26" t="str">
-        <v>Boston metro. Portfolio of prior engineering work required.</v>
+        <v>Boston metro. Portfolio of prior engineering work required — application not considered without one.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Eaton</v>
+        <v>Formlabs</v>
       </c>
       <c r="B27" t="str">
-        <v>ETO Engineering Co-op</v>
+        <v>Hardware Systems Integration Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C27" t="str">
-        <v>Mechanical, Industrial, or Electrical Engineering</v>
+        <v>Hardware / Electro-Mechanical Engineering</v>
       </c>
       <c r="D27" t="str">
-        <v>Fall 2026 or Spring 2027 (posting states either start date is acceptable)</v>
+        <v>Winter/Spring 2027 (January–April)</v>
       </c>
       <c r="E27" t="str">
-        <v>Syracuse, NY</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F27">
-        <v>260</v>
+        <v>3</v>
       </c>
       <c r="G27" t="str">
-        <v>$24.92/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H27" t="str">
-        <v>https://eaton.eightfold.ai/careers/job/687236797540</v>
+        <v>https://careers.formlabs.com/job/8172004/apply/?gh_jid=8172004</v>
       </c>
       <c r="I27" t="str">
-        <v>Yes — verified via Eaton's own public Eightfold job-board API directly (the rendered page is JS-heavy); record shows isPrivate: false (publicly listed/active), created 2026-05-21, last updated 2026-08-12.</v>
+        <v>Yes — fetched directly, page live, title/season/location confirmed in posting text.</v>
       </c>
       <c r="J27" t="str">
-        <v>Min GPA 2.8. No visa sponsorship (no CPT/OPT/H-1B support). Must live within ~50 mi of Syracuse, NY — no relocation assistance.</v>
+        <v>Boston metro. Portfolio of prior engineering work required.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Reframe Systems</v>
+        <v>Eaton</v>
       </c>
       <c r="B28" t="str">
-        <v>Mechanical Engineer (Spring 2027 Co-op)</v>
+        <v>ETO Engineering Co-op</v>
       </c>
       <c r="C28" t="str">
-        <v>Mechanical Engineering (CAD, welding, machining, fixturing/workcell design)</v>
+        <v>Mechanical, Industrial, or Electrical Engineering</v>
       </c>
       <c r="D28" t="str">
-        <v>Spring 2027</v>
+        <v>Fall 2026 or Spring 2027 (posting states either start date is acceptable)</v>
       </c>
       <c r="E28" t="str">
-        <v>Andover, MA (HQ) / FAB1 microfactory, Billerica, MA</v>
+        <v>Syracuse, NY</v>
       </c>
       <c r="F28">
-        <v>23</v>
+        <v>260</v>
       </c>
       <c r="G28" t="str">
-        <v>Not stated on posting</v>
+        <v>$24.92/hr</v>
       </c>
       <c r="H28" t="str">
-        <v>https://jobs.ashbyhq.com/reframesystems/f5275832-8373-4971-b5f6-6aaececcb061</v>
+        <v>https://eaton.eightfold.ai/careers/job/687236797540</v>
       </c>
       <c r="I28" t="str">
-        <v>Yes — verified via Reframe Systems' own public Ashby job-board API directly; record shows isListed: true, publishedAt 2026-08-05, exact worksite address (30 Lowell Junction Rd, Andover MA).</v>
+        <v>Yes — verified via Eaton's own public Eightfold job-board API directly (the rendered page is JS-heavy); record shows isPrivate: false (publicly listed/active), created 2026-05-21, last updated 2026-08-12.</v>
       </c>
       <c r="J28" t="str">
-        <v>Small modular-construction/robotics-manufacturing startup, Boston metro (Andover/Billerica). Shop-based role — CAD, welding, machining, fixturing.</v>
+        <v>Min GPA 2.8. No visa sponsorship (no CPT/OPT/H-1B support). Must live within ~50 mi of Syracuse, NY — no relocation assistance.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>General Dynamics Electric Boat</v>
+        <v>Reframe Systems</v>
       </c>
       <c r="B29" t="str">
-        <v>2027 Spring Engineering CO-OP Trainee</v>
+        <v>Mechanical Engineer (Spring 2027 Co-op)</v>
       </c>
       <c r="C29" t="str">
-        <v>Mechanical / Structural / Aerospace-Aeronautical / Systems / Naval Architecture / Industrial / Electromechanical / Robotics Engineering (multi-discipline req)</v>
+        <v>Mechanical Engineering (CAD, welding, machining, fixturing/workcell design)</v>
       </c>
       <c r="D29" t="str">
-        <v>Spring of 2027 (per listing summary)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E29" t="str">
-        <v>Groton, CT (co-ops also placed in New London/North Stonington CT, North Kingstown/Newport RI)</v>
+        <v>Andover, MA (HQ) / FAB1 microfactory, Billerica, MA</v>
       </c>
       <c r="F29">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="G29" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H29" t="str">
-        <v>https://jobs.buildsubmarines.com/job/601496955</v>
+        <v>https://jobs.ashbyhq.com/reframesystems/f5275832-8373-4971-b5f6-6aaececcb061</v>
       </c>
       <c r="I29" t="str">
-        <v>Partial — found via GD Electric Boat's own dedicated recruiting site (jobs.buildsubmarines.com) with a specific req ID, mirroring the pattern of GD's known 2026 cycle req. The page itself is behind a Cloudflare bot-check wall — blocked on WebFetch, curl w/ browser UA, and a reader-proxy fetch, all returning a security-verification/CAPTCHA screen. Could not independently confirm live/open status or the exact discipline breakdown. Verify live in-browser before applying.</v>
+        <v>Yes — verified via Reframe Systems' own public Ashby job-board API directly; record shows isListed: true, publishedAt 2026-08-05, exact worksite address (30 Lowell Junction Rd, Andover MA).</v>
       </c>
       <c r="J29" t="str">
-        <v>Was flagged 'worth re-checking' in the prior run; upgraded from 'no verifiable link' to 'specific req ID found, still blocked'.</v>
+        <v>Small modular-construction/robotics-manufacturing startup, Boston metro (Andover/Billerica). Shop-based role — CAD, welding, machining, fixturing.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Anduril Industries</v>
+        <v>General Dynamics Electric Boat</v>
       </c>
       <c r="B30" t="str">
-        <v>Winter 2027 Mechanical Engineer Co-op</v>
+        <v>2027 Spring Engineering CO-OP Trainee</v>
       </c>
       <c r="C30" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Structural / Aerospace-Aeronautical / Systems / Naval Architecture / Industrial / Electromechanical / Robotics Engineering (multi-discipline req)</v>
       </c>
       <c r="D30" t="str">
-        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027 — same calendar window other employers call 'Spring 2027')</v>
+        <v>Spring of 2027 (per listing summary)</v>
       </c>
       <c r="E30" t="str">
-        <v>Quincy, MA</v>
+        <v>Groton, CT (co-ops also placed in New London/North Stonington CT, North Kingstown/Newport RI)</v>
       </c>
       <c r="F30">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="G30" t="str">
-        <v>$34–$50/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H30" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236601007</v>
+        <v>https://jobs.buildsubmarines.com/job/601496955</v>
       </c>
       <c r="I30" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+        <v>Partial — found via GD Electric Boat's own dedicated recruiting site (jobs.buildsubmarines.com) with a specific req ID, mirroring the pattern of GD's known 2026 cycle req. The page itself is behind a Cloudflare bot-check wall — blocked on WebFetch, curl w/ browser UA, and a reader-proxy fetch, all returning a security-verification/CAPTCHA screen. Could not independently confirm live/open status or the exact discipline breakdown. Verify live in-browser before applying.</v>
       </c>
       <c r="J30" t="str">
-        <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
+        <v>Was flagged 'worth re-checking' in the prior run; upgraded from 'no verifiable link' to 'specific req ID found, still blocked'.</v>
       </c>
     </row>
     <row r="31">
@@ -1365,13 +1365,13 @@
         <v>Anduril Industries</v>
       </c>
       <c r="B31" t="str">
-        <v>Winter 2027 Systems Engineer Co-op</v>
+        <v>Winter 2027 Mechanical Engineer Co-op</v>
       </c>
       <c r="C31" t="str">
-        <v>Systems Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D31" t="str">
-        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027 — same calendar window other employers call 'Spring 2027')</v>
       </c>
       <c r="E31" t="str">
         <v>Quincy, MA</v>
@@ -1380,301 +1380,301 @@
         <v>8</v>
       </c>
       <c r="G31" t="str">
-        <v>$40–$55/hr</v>
+        <v>$34–$50/hr</v>
       </c>
       <c r="H31" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236599007</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236601007</v>
       </c>
       <c r="I31" t="str">
         <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J31" t="str">
-        <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
+        <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Rivian</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B32" t="str">
-        <v>Engineering Intern – Manufacturing Engineering (Spring 2027 Co-Op)</v>
+        <v>Winter 2027 Systems Engineer Co-op</v>
       </c>
       <c r="C32" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D32" t="str">
-        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
       </c>
       <c r="E32" t="str">
-        <v>Normal, IL</v>
+        <v>Quincy, MA</v>
       </c>
       <c r="F32">
-        <v>1000</v>
+        <v>8</v>
       </c>
       <c r="G32" t="str">
-        <v>~$25–$51/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+        <v>$40–$55/hr</v>
       </c>
       <c r="H32" t="str">
-        <v>https://careers.rivian.com/jobs/33784?lang=en-us</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236599007</v>
       </c>
       <c r="I32" t="str">
-        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J32" t="str">
-        <v/>
+        <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Rivian</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B33" t="str">
-        <v>Engineering Intern – Design for Reliability (Spring 2027 Co-Op)</v>
+        <v>Winter 2027 Manufacturing Engineer Co-op</v>
       </c>
       <c r="C33" t="str">
-        <v>Mechanical / Design Engineering</v>
+        <v>Mechanical Engineering / Aerospace Engineering</v>
       </c>
       <c r="D33" t="str">
-        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
+        <v>Winter 2027 (16–24 wks; body notes ability to complete an in-person internship in summer 2027 — same Jan–Aug 2027 pattern as the other Anduril Winter 2027 co-ops)</v>
       </c>
       <c r="E33" t="str">
-        <v>Irvine, CA</v>
+        <v>Lexington, MA; Quincy, MA</v>
       </c>
       <c r="F33">
-        <v>2600</v>
+        <v>12</v>
       </c>
       <c r="G33" t="str">
-        <v>~$26–$45/hr per third-party aggregator; not independently confirmed via direct fetch</v>
+        <v>$32–$45/hr</v>
       </c>
       <c r="H33" t="str">
-        <v>https://careers.rivian.com/careers-home/jobs/33705?lang=en-us</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236589007</v>
       </c>
       <c r="I33" t="str">
-        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J33" t="str">
-        <v/>
+        <v>Boston metro. This is the req flagged in the prior run as 'found in snippets but not direct-fetched' — now confirmed live. Same cohort/site family as the Mechanical/Systems Engineer Co-ops above. No stated application deadline.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>SpaceX</v>
+        <v>Rivian</v>
       </c>
       <c r="B34" t="str">
-        <v>Spring 2027 Engineering Internship/Co-op</v>
+        <v>Engineering Intern – Manufacturing Engineering (Spring 2027 Co-Op)</v>
       </c>
       <c r="C34" t="str">
-        <v>Engineering (multi-discipline req)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D34" t="str">
-        <v>Spring 2027 (start Jan or Mar 2027)</v>
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
       </c>
       <c r="E34" t="str">
-        <v>Multiple US sites (incl. Bloomfield, CT — see posting for full list)</v>
+        <v>Normal, IL</v>
+      </c>
+      <c r="F34">
+        <v>1000</v>
       </c>
       <c r="G34" t="str">
-        <v>$28–$30/hr</v>
+        <v>~$25–$51/hr per third-party aggregator; not independently confirmed via direct fetch</v>
       </c>
       <c r="H34" t="str">
-        <v>https://job-boards.greenhouse.io/spacex/jobs/8616338002</v>
+        <v>https://careers.rivian.com/jobs/33784?lang=en-us</v>
       </c>
       <c r="I34" t="str">
-        <v>Yes — fetched directly on Greenhouse, live.</v>
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
       </c>
       <c r="J34" t="str">
-        <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Rocket Lab</v>
+        <v>Rivian</v>
       </c>
       <c r="B35" t="str">
-        <v>Mechanical Engineering Intern, Spring 2027</v>
+        <v>Engineering Intern – Design for Reliability (Spring 2027 Co-Op)</v>
       </c>
       <c r="C35" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Design Engineering</v>
       </c>
       <c r="D35" t="str">
-        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+        <v>Spring 2027 Co-Op (Jan–Aug 2027)</v>
       </c>
       <c r="E35" t="str">
-        <v>Long Beach, CA</v>
+        <v>Irvine, CA</v>
       </c>
       <c r="F35">
         <v>2600</v>
       </c>
       <c r="G35" t="str">
-        <v>$28/hr</v>
+        <v>~$26–$45/hr per third-party aggregator; not independently confirmed via direct fetch</v>
       </c>
       <c r="H35" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7985634003</v>
+        <v>https://careers.rivian.com/careers-home/jobs/33705?lang=en-us</v>
       </c>
       <c r="I35" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+        <v>Yes — fetched directly on Rivian's own careers site, title/location/season confirmed.</v>
       </c>
       <c r="J35" t="str">
-        <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Rocket Lab</v>
+        <v>SpaceX</v>
       </c>
       <c r="B36" t="str">
-        <v>Systems Engineering Intern, Spring 2027</v>
+        <v>Spring 2027 Engineering Internship/Co-op</v>
       </c>
       <c r="C36" t="str">
-        <v>Systems Engineering</v>
+        <v>Engineering (multi-discipline req)</v>
       </c>
       <c r="D36" t="str">
-        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
+        <v>Spring 2027 (start Jan or Mar 2027)</v>
       </c>
       <c r="E36" t="str">
-        <v>Long Beach, CA</v>
-      </c>
-      <c r="F36">
-        <v>2600</v>
+        <v>Multiple US sites (incl. Bloomfield, CT — see posting for full list)</v>
       </c>
       <c r="G36" t="str">
-        <v>$28/hr</v>
+        <v>$28–$30/hr</v>
       </c>
       <c r="H36" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987044003</v>
+        <v>https://job-boards.greenhouse.io/spacex/jobs/8616338002</v>
       </c>
       <c r="I36" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
+        <v>Yes — fetched directly on Greenhouse, live.</v>
       </c>
       <c r="J36" t="str">
-        <v/>
+        <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Collins Aerospace (RTX)</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B37" t="str">
-        <v>Project Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Mechanical Engineering Intern, Spring 2027</v>
       </c>
       <c r="C37" t="str">
-        <v>Systems / Mechanical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D37" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027, full-time)</v>
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E37" t="str">
-        <v>Windsor Locks, CT</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F37">
-        <v>90</v>
+        <v>2600</v>
       </c>
       <c r="G37" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>$28/hr</v>
       </c>
       <c r="H37" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7985634003</v>
       </c>
       <c r="I37" t="str">
-        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J37" t="str">
-        <v>~1.5 hrs from Boston.</v>
+        <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Pratt &amp; Whitney (RTX)</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B38" t="str">
-        <v>Production Support Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Systems Engineering Intern, Spring 2027</v>
       </c>
       <c r="C38" t="str">
-        <v>Mechanical / Manufacturing / Aerospace Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D38" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027 (start Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E38" t="str">
-        <v>Middletown, CT</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F38">
-        <v>105</v>
+        <v>2600</v>
       </c>
       <c r="G38" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>$28/hr</v>
       </c>
       <c r="H38" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-MIDDLETOWN-220A--Aircraft-Rd--BLDG-220A/Production-Support-Engineering-Co-op--Winter-Spring-2027-_01872654</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987044003</v>
       </c>
       <c r="I38" t="str">
-        <v>Partial — Workday page blocked automated fetch. Req ID and Sept 13, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live.</v>
       </c>
       <c r="J38" t="str">
-        <v>~1.5 hrs from Boston.</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Collins Aerospace (RTX)</v>
       </c>
       <c r="B39" t="str">
-        <v>Certification Engineer Co-Op (Winter/Spring 2027, Onsite)</v>
+        <v>Project Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C39" t="str">
-        <v>Mechanical / Aerospace / Materials Science / Chemical Engineering</v>
+        <v>Systems / Mechanical Engineering</v>
       </c>
       <c r="D39" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul, two semesters)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027, full-time)</v>
       </c>
       <c r="E39" t="str">
-        <v>Winston-Salem, NC</v>
+        <v>Windsor Locks, CT</v>
       </c>
       <c r="F39">
-        <v>700</v>
+        <v>90</v>
       </c>
       <c r="G39" t="str">
         <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H39" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
       </c>
       <c r="I39" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 16, 2026. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J39" t="str">
-        <v/>
+        <v>~1.5 hrs from Boston.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Pratt &amp; Whitney (RTX)</v>
       </c>
       <c r="B40" t="str">
-        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Production Support Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C40" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Manufacturing / Aerospace Engineering</v>
       </c>
       <c r="D40" t="str">
         <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E40" t="str">
-        <v>Cedar Rapids, IA</v>
+        <v>Middletown, CT</v>
       </c>
       <c r="F40">
-        <v>1130</v>
+        <v>105</v>
       </c>
       <c r="G40" t="str">
         <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H40" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869080</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-MIDDLETOWN-220A--Aircraft-Rd--BLDG-220A/Production-Support-Engineering-Co-op--Winter-Spring-2027-_01872654</v>
       </c>
       <c r="I40" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 15, 2026. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Req ID and Sept 13, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J40" t="str">
-        <v/>
+        <v>~1.5 hrs from Boston.</v>
       </c>
     </row>
     <row r="41">
@@ -1682,28 +1682,28 @@
         <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B41" t="str">
-        <v>Structural Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Certification Engineer Co-Op (Winter/Spring 2027, Onsite)</v>
       </c>
       <c r="C41" t="str">
-        <v>Structural Engineering</v>
+        <v>Mechanical / Aerospace / Materials Science / Chemical Engineering</v>
       </c>
       <c r="D41" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jul, two semesters)</v>
       </c>
       <c r="E41" t="str">
-        <v>Jamestown, ND</v>
+        <v>Winston-Salem, NC</v>
       </c>
       <c r="F41">
-        <v>1500</v>
+        <v>700</v>
       </c>
       <c r="G41" t="str">
         <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H41" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Structural-Engineering-Co-op--Winter-Spring-2027-_01873938</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
       </c>
       <c r="I41" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 14, 2026. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 16, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J41" t="str">
         <v/>
@@ -1711,31 +1711,31 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Northrop Grumman</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B42" t="str">
-        <v>2027 Spring Mechanical Engineering Co-op</v>
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C42" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D42" t="str">
-        <v>Spring/Summer 2027 (Jan–Aug 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E42" t="str">
-        <v>Chandler, AZ</v>
+        <v>Cedar Rapids, IA</v>
       </c>
       <c r="F42">
-        <v>2300</v>
+        <v>1130</v>
       </c>
       <c r="G42" t="str">
-        <v>Bachelor's $18.50–$33.50/hr; Master's $26.25–$41.50/hr</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H42" t="str">
-        <v>https://ngc.wd1.myworkdayjobs.com/Northrop_Grumman_External_Site/job/United-States-Arizona-Chandler/XMLNAME-2027-Spring-Mechanical-Engineering-Co-op---Chandler-AZ_R10249939</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-131--5450-C-Ave-NE--BLDG-131/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869080</v>
       </c>
       <c r="I42" t="str">
-        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 15, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J42" t="str">
         <v/>
@@ -1743,63 +1743,63 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Berkshire Grey</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B43" t="str">
-        <v>Spring 2027 Hardware Quality Co-op</v>
+        <v>Structural Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C43" t="str">
-        <v>Hardware / Quality Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D43" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E43" t="str">
-        <v>Bedford, MA</v>
+        <v>Jamestown, ND</v>
       </c>
       <c r="F43">
-        <v>17</v>
+        <v>1500</v>
       </c>
       <c r="G43" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H43" t="str">
-        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Structural-Engineering-Co-op--Winter-Spring-2027-_01873938</v>
       </c>
       <c r="I43" t="str">
-        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror, posting date Sept 14, 2026. Verify live in-browser before applying.</v>
       </c>
       <c r="J43" t="str">
-        <v>Boston metro (Bedford).</v>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Emerson</v>
+        <v>Northrop Grumman</v>
       </c>
       <c r="B44" t="str">
-        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
+        <v>2027 Spring Mechanical Engineering Co-op</v>
       </c>
       <c r="C44" t="str">
-        <v>R&amp;D / Mechanical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D44" t="str">
-        <v>Spring 2027</v>
+        <v>Spring/Summer 2027 (Jan–Aug 2027)</v>
       </c>
       <c r="E44" t="str">
-        <v>Cranberry Township, PA</v>
+        <v>Chandler, AZ</v>
       </c>
       <c r="F44">
-        <v>570</v>
+        <v>2300</v>
       </c>
       <c r="G44" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>Bachelor's $18.50–$33.50/hr; Master's $26.25–$41.50/hr</v>
       </c>
       <c r="H44" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
+        <v>https://ngc.wd1.myworkdayjobs.com/Northrop_Grumman_External_Site/job/United-States-Arizona-Chandler/XMLNAME-2027-Spring-Mechanical-Engineering-Co-op---Chandler-AZ_R10249939</v>
       </c>
       <c r="I44" t="str">
-        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — Workday page blocked automated fetch. Confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J44" t="str">
         <v/>
@@ -1807,258 +1807,258 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Emerson</v>
+        <v>Berkshire Grey</v>
       </c>
       <c r="B45" t="str">
-        <v>Project Engineering Co-op – Spring 2027</v>
+        <v>Spring 2027 Hardware Quality Co-op</v>
       </c>
       <c r="C45" t="str">
-        <v>Project / Mechanical Engineering</v>
+        <v>Hardware / Quality Engineering</v>
       </c>
       <c r="D45" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E45" t="str">
-        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F45">
-        <v>570</v>
+        <v>17</v>
       </c>
       <c r="G45" t="str">
         <v>Not stated (aggregator only)</v>
       </c>
       <c r="H45" t="str">
-        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
+        <v>https://berkshiregrey.bamboohr.com/careers/771</v>
       </c>
       <c r="I45" t="str">
-        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>Boston metro (Bedford).</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Zipline</v>
+        <v>Emerson</v>
       </c>
       <c r="B46" t="str">
-        <v>Mechanical Engineer Intern</v>
+        <v>R&amp;D Engineering Co-Op – Spring 2027</v>
       </c>
       <c r="C46" t="str">
-        <v>Mechanical Engineering</v>
+        <v>R&amp;D / Mechanical Engineering</v>
       </c>
       <c r="D46" t="str">
-        <v>Spring 2027 (Jan–Apr/May)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E46" t="str">
-        <v>South San Francisco, CA (or Dallas, TX)</v>
+        <v>Cranberry Township, PA</v>
       </c>
       <c r="F46">
-        <v>2700</v>
+        <v>570</v>
       </c>
       <c r="G46" t="str">
-        <v>~$60k–$70k annualized (third-party estimate, not stated on posting)</v>
+        <v>Not stated (aggregator only)</v>
       </c>
       <c r="H46" t="str">
-        <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010785</v>
       </c>
       <c r="I46" t="str">
-        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J46" t="str">
-        <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Applied Materials</v>
+        <v>Emerson</v>
       </c>
       <c r="B47" t="str">
-        <v>2027 Spring Mechanical Engineer Co-op</v>
+        <v>Project Engineering Co-op – Spring 2027</v>
       </c>
       <c r="C47" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Project / Mechanical Engineering</v>
       </c>
       <c r="D47" t="str">
-        <v>Spring 2027 (start January 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E47" t="str">
-        <v>Gloucester, MA</v>
+        <v>Cranberry Township, PA / Blue Bell, PA / Detroit, MI</v>
       </c>
       <c r="F47">
-        <v>30</v>
+        <v>570</v>
       </c>
       <c r="G47" t="str">
-        <v>$31–33/hr</v>
+        <v>Not stated (aggregator only)</v>
       </c>
       <c r="H47" t="str">
-        <v>https://amat.wd1.myworkdayjobs.com/external/job/GloucesterMA/XMLNAME-2027-Spring-Mechanical-Engineer-Co-op--Gloucester-MA-_R2628290</v>
+        <v>https://hdjq.fa.us2.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/26010587</v>
       </c>
       <c r="I47" t="str">
-        <v>Partial — Workday page blocked automated fetch (JS-rendered, empty). Confirmed via a dreamworkhq aggregator mirror quoting the exact title, season, location, pay, and req ID, posted ~1 week ago as of 2026-09-20. Verify live in-browser before applying.</v>
+        <v>Partial — Oracle Cloud ATS is JS-rendered, returned empty content on direct fetch. Sourced via aggregator mirror only. Verify live in-browser before applying.</v>
       </c>
       <c r="J47" t="str">
-        <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Sanofi (Genzyme)</v>
+        <v>Zipline</v>
       </c>
       <c r="B48" t="str">
-        <v>2027 Spring Co-Op Opportunities</v>
+        <v>Mechanical Engineer Intern</v>
       </c>
       <c r="C48" t="str">
-        <v>Manufacturing / Process Engineering (biopharma — MSAT: Manufacturing Science &amp; Technology)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D48" t="str">
-        <v>Spring 2027 (6-month, starting January 2027)</v>
+        <v>Spring 2027 (Jan–Apr/May)</v>
       </c>
       <c r="E48" t="str">
-        <v>Framingham, MA</v>
+        <v>South San Francisco, CA (or Dallas, TX)</v>
       </c>
       <c r="F48">
-        <v>20</v>
+        <v>2700</v>
       </c>
       <c r="G48" t="str">
-        <v>$32–55/hr</v>
+        <v>~$60k–$70k annualized (third-party estimate, not stated on posting)</v>
       </c>
       <c r="H48" t="str">
-        <v>https://jobs.sanofi.com/en/job/framingham/2027-spring-co-op-opportunities-framingham-ma/2649/41259847040</v>
+        <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
       </c>
       <c r="I48" t="str">
-        <v>Yes — fetched directly, page live, active 'Apply Now' button present. Posting states it closes November 14, 2026.</v>
+        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
       </c>
       <c r="J48" t="str">
-        <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
+        <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>GE Aerospace</v>
+        <v>Applied Materials</v>
       </c>
       <c r="B49" t="str">
-        <v>Engines Engineering Co-op – US – Spring 2027</v>
+        <v>2027 Spring Mechanical Engineer Co-op</v>
       </c>
       <c r="C49" t="str">
-        <v>Aerospace / Mechanical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D49" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (start January 2027)</v>
       </c>
       <c r="E49" t="str">
-        <v>Lynn, MA or Evendale/Cincinnati, OH (dual-location req)</v>
+        <v>Gloucester, MA</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="G49" t="str">
-        <v>Starts at $20/hr, increases per undergrad class year</v>
+        <v>$31–33/hr</v>
       </c>
       <c r="H49" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Evendale/Engines-Engineering-Co-op---US---Spring-2027_R5029617-1</v>
+        <v>https://amat.wd1.myworkdayjobs.com/external/job/GloucesterMA/XMLNAME-2027-Spring-Mechanical-Engineer-Co-op--Gloucester-MA-_R2628290</v>
       </c>
       <c r="I49" t="str">
-        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
+        <v>Partial — Workday page blocked automated fetch (JS-rendered, empty). Confirmed via a dreamworkhq aggregator mirror quoting the exact title, season, location, pay, and req ID, posted ~1 week ago as of 2026-09-20. Verify live in-browser before applying.</v>
       </c>
       <c r="J49" t="str">
-        <v>Requires 'US Person' status (citizen/LPR/asylee/refugee) for export-controlled work; no visa sponsorship; relocation/housing assistance provided. This is the first live GE Aerospace Spring 2027 req found after 4 prior runs found only dead/expired reqs — Lynn, MA option makes this a Boston-metro fit.</v>
+        <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>GE Aerospace</v>
+        <v>Sanofi (Genzyme)</v>
       </c>
       <c r="B50" t="str">
-        <v>Structures Intern/Co-op – ACSC – Cincinnati, OH – Spring 2027</v>
+        <v>2027 Spring Co-Op Opportunities</v>
       </c>
       <c r="C50" t="str">
-        <v>Structural / Manufacturing / Materials Engineering</v>
+        <v>Manufacturing / Process Engineering (biopharma — MSAT: Manufacturing Science &amp; Technology)</v>
       </c>
       <c r="D50" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (6-month, starting January 2027)</v>
       </c>
       <c r="E50" t="str">
-        <v>Springdale (Cincinnati), OH</v>
+        <v>Framingham, MA</v>
       </c>
       <c r="F50">
-        <v>750</v>
+        <v>20</v>
       </c>
       <c r="G50" t="str">
-        <v>Not stated on posting</v>
+        <v>$32–55/hr</v>
       </c>
       <c r="H50" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Springdale/Structures-Intern-Co-op---ACSC---Cincinnati--OH---Spring-2027_R5039588-1</v>
+        <v>https://jobs.sanofi.com/en/job/framingham/2027-spring-co-op-opportunities-framingham-ma/2649/41259847040</v>
       </c>
       <c r="I50" t="str">
-        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
+        <v>Yes — fetched directly, page live, active 'Apply Now' button present. Posting states it closes November 14, 2026.</v>
       </c>
       <c r="J50" t="str">
-        <v>Accepted majors: Aerospace, Manufacturing, Mechanical, Materials, Industrial Engineering. Not Boston-area.</v>
+        <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Insulet</v>
+        <v>GE Aerospace</v>
       </c>
       <c r="B51" t="str">
-        <v>Co-op, R&amp;D Mechanical Engineering (January–June 2027, Hybrid)</v>
+        <v>Engines Engineering Co-op – US – Spring 2027</v>
       </c>
       <c r="C51" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Aerospace / Mechanical Engineering</v>
       </c>
       <c r="D51" t="str">
-        <v>January 11, 2027 – June 30, 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E51" t="str">
-        <v>Acton, MA</v>
+        <v>Lynn, MA or Evendale/Cincinnati, OH (dual-location req)</v>
       </c>
       <c r="F51">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G51" t="str">
-        <v>$25.00–$34.00/hr</v>
+        <v>Starts at $20/hr, increases per undergrad class year</v>
       </c>
       <c r="H51" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Mechanical-Engineering--January---June-2027--Hybrid-_REQ-2026-18007</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Evendale/Engines-Engineering-Co-op---US---Spring-2027_R5029617-1</v>
       </c>
       <c r="I51" t="str">
-        <v>Yes — full description fetched directly via Workday, posted 4 days ago.</v>
+        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
       </c>
       <c r="J51" t="str">
-        <v>Boston metro (Acton). Medical device (insulin pump) manufacturer. Not eligible for visa sponsorship; requires US work authorization without future sponsorship needs. Part of a large batch of Insulet Acton co-ops opened this cycle — see sibling reqs below.</v>
+        <v>Requires 'US Person' status (citizen/LPR/asylee/refugee) for export-controlled work; no visa sponsorship; relocation/housing assistance provided. This is the first live GE Aerospace Spring 2027 req found after 4 prior runs found only dead/expired reqs — Lynn, MA option makes this a Boston-metro fit.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Insulet</v>
+        <v>GE Aerospace</v>
       </c>
       <c r="B52" t="str">
-        <v>Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
+        <v>Structures Intern/Co-op – ACSC – Cincinnati, OH – Spring 2027</v>
       </c>
       <c r="C52" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Structural / Manufacturing / Materials Engineering</v>
       </c>
       <c r="D52" t="str">
-        <v>January 11, 2027 – June 30, 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E52" t="str">
-        <v>Acton, MA</v>
+        <v>Springdale (Cincinnati), OH</v>
       </c>
       <c r="F52">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="G52" t="str">
-        <v>$25.00–$34.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H52" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Engineering--January---June-2027--Onsite-_REQ-2026-18078</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/en-US/GE_ExternalSite/job/Springdale/Structures-Intern-Co-op---ACSC---Cincinnati--OH---Spring-2027_R5039588-1</v>
       </c>
       <c r="I52" t="str">
-        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
+        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed.</v>
       </c>
       <c r="J52" t="str">
-        <v>Boston metro (Acton). No visa sponsorship.</v>
+        <v>Accepted majors: Aerospace, Manufacturing, Mechanical, Materials, Industrial Engineering. Not Boston-area.</v>
       </c>
     </row>
     <row r="53">
@@ -2066,10 +2066,10 @@
         <v>Insulet</v>
       </c>
       <c r="B53" t="str">
-        <v>Co-op, Systems Engineering (January–June 2027, Hybrid)</v>
+        <v>Co-op, R&amp;D Mechanical Engineering (January–June 2027, Hybrid)</v>
       </c>
       <c r="C53" t="str">
-        <v>Systems Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D53" t="str">
         <v>January 11, 2027 – June 30, 2027</v>
@@ -2084,13 +2084,13 @@
         <v>$25.00–$34.00/hr</v>
       </c>
       <c r="H53" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering--January-June-2027--Hybrid-_REQ-2026-18061</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Mechanical-Engineering--January---June-2027--Hybrid-_REQ-2026-18007</v>
       </c>
       <c r="I53" t="str">
-        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
+        <v>Yes — full description fetched directly via Workday, posted 4 days ago.</v>
       </c>
       <c r="J53" t="str">
-        <v>Boston metro (Acton). No visa sponsorship.</v>
+        <v>Boston metro (Acton). Medical device (insulin pump) manufacturer. Not eligible for visa sponsorship; requires US work authorization without future sponsorship needs. Part of a large batch of Insulet Acton co-ops opened this cycle — see sibling reqs below.</v>
       </c>
     </row>
     <row r="54">
@@ -2098,13 +2098,13 @@
         <v>Insulet</v>
       </c>
       <c r="B54" t="str">
-        <v>Co-op, Mechanical Lifecycle (January–June 2027, Onsite)</v>
+        <v>Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
       </c>
       <c r="C54" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D54" t="str">
-        <v>January–June 2027 (per title)</v>
+        <v>January 11, 2027 – June 30, 2027</v>
       </c>
       <c r="E54" t="str">
         <v>Acton, MA</v>
@@ -2113,16 +2113,16 @@
         <v>25</v>
       </c>
       <c r="G54" t="str">
-        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+        <v>$25.00–$34.00/hr</v>
       </c>
       <c r="H54" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Mechanical-Lifecycle--January---June-2027--Onsite-_REQ-2026-18155</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Engineering--January---June-2027--Onsite-_REQ-2026-18078</v>
       </c>
       <c r="I54" t="str">
-        <v>Partial — confirmed live and current via direct query of Insulet's own Workday jobs-search API (real title/location/posted-date, not an aggregator), posted 5 days ago. Full job-description body was not individually opened — spot-check before applying.</v>
+        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
       </c>
       <c r="J54" t="str">
-        <v>Boston metro (Acton). One of a batch of Insulet Acton co-ops opened this cycle alongside the fully-verified R&amp;D Mechanical/Manufacturing/Systems reqs above.</v>
+        <v>Boston metro (Acton). No visa sponsorship.</v>
       </c>
     </row>
     <row r="55">
@@ -2130,13 +2130,13 @@
         <v>Insulet</v>
       </c>
       <c r="B55" t="str">
-        <v>Co-op, R&amp;D Manufacturing (January–June 2027, Onsite)</v>
+        <v>Co-op, Systems Engineering (January–June 2027, Hybrid)</v>
       </c>
       <c r="C55" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D55" t="str">
-        <v>January–June 2027 (per title)</v>
+        <v>January 11, 2027 – June 30, 2027</v>
       </c>
       <c r="E55" t="str">
         <v>Acton, MA</v>
@@ -2145,16 +2145,16 @@
         <v>25</v>
       </c>
       <c r="G55" t="str">
-        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
+        <v>$25.00–$34.00/hr</v>
       </c>
       <c r="H55" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Manufacturing--January-June-2027--Onsite-_REQ-2026-18069</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering--January-June-2027--Hybrid-_REQ-2026-18061</v>
       </c>
       <c r="I55" t="str">
-        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
+        <v>Yes — full description fetched directly via Workday, posted 5 days ago.</v>
       </c>
       <c r="J55" t="str">
-        <v>Boston metro (Acton).</v>
+        <v>Boston metro (Acton). No visa sponsorship.</v>
       </c>
     </row>
     <row r="56">
@@ -2162,10 +2162,10 @@
         <v>Insulet</v>
       </c>
       <c r="B56" t="str">
-        <v>Graduate Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
+        <v>Co-op, Mechanical Lifecycle (January–June 2027, Onsite)</v>
       </c>
       <c r="C56" t="str">
-        <v>Manufacturing Engineering (graduate-level)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D56" t="str">
         <v>January–June 2027 (per title)</v>
@@ -2180,13 +2180,13 @@
         <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H56" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Graduate--January---June-2027--Onsite-_REQ-2026-18086</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Mechanical-Lifecycle--January---June-2027--Onsite-_REQ-2026-18155</v>
       </c>
       <c r="I56" t="str">
-        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
+        <v>Partial — confirmed live and current via direct query of Insulet's own Workday jobs-search API (real title/location/posted-date, not an aggregator), posted 5 days ago. Full job-description body was not individually opened — spot-check before applying.</v>
       </c>
       <c r="J56" t="str">
-        <v>Boston metro (Acton). Labeled 'Graduate Co-op' — confirm eligibility if Hamza is undergraduate.</v>
+        <v>Boston metro (Acton). One of a batch of Insulet Acton co-ops opened this cycle alongside the fully-verified R&amp;D Mechanical/Manufacturing/Systems reqs above.</v>
       </c>
     </row>
     <row r="57">
@@ -2194,10 +2194,10 @@
         <v>Insulet</v>
       </c>
       <c r="B57" t="str">
-        <v>Co-op, Supplier Development Engineering - Mechanical (January–June 2027)</v>
+        <v>Co-op, R&amp;D Manufacturing (January–June 2027, Onsite)</v>
       </c>
       <c r="C57" t="str">
-        <v>Mechanical / Supplier Quality Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D57" t="str">
         <v>January–June 2027 (per title)</v>
@@ -2212,10 +2212,10 @@
         <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H57" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Development-Engineering---Mechanical--January-June-2027--Onsite-_REQ-2026-18209</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Manufacturing--January-June-2027--Onsite-_REQ-2026-18069</v>
       </c>
       <c r="I57" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly (not a synthesized link); the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
       </c>
       <c r="J57" t="str">
         <v>Boston metro (Acton).</v>
@@ -2226,10 +2226,10 @@
         <v>Insulet</v>
       </c>
       <c r="B58" t="str">
-        <v>Co-op, Systems Engineering - Design Verification (January–June 2027)</v>
+        <v>Graduate Co-op, Manufacturing Engineering (January–June 2027, Onsite)</v>
       </c>
       <c r="C58" t="str">
-        <v>Systems Engineering</v>
+        <v>Manufacturing Engineering (graduate-level)</v>
       </c>
       <c r="D58" t="str">
         <v>January–June 2027 (per title)</v>
@@ -2244,13 +2244,13 @@
         <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H58" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering---Design-Verification--January---June-2027--Onsite-_REQ-2026-18144-1</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Manufacturing-Graduate--January---June-2027--Onsite-_REQ-2026-18086</v>
       </c>
       <c r="I58" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
       </c>
       <c r="J58" t="str">
-        <v>Boston metro (Acton).</v>
+        <v>Boston metro (Acton). Labeled 'Graduate Co-op' — confirm eligibility if Hamza is undergraduate.</v>
       </c>
     </row>
     <row r="59">
@@ -2258,10 +2258,10 @@
         <v>Insulet</v>
       </c>
       <c r="B59" t="str">
-        <v>Co-op, Life Cycle Engineering - Systems (January–June 2027)</v>
+        <v>Co-op, Supplier Development Engineering - Mechanical (January–June 2027)</v>
       </c>
       <c r="C59" t="str">
-        <v>Systems Engineering</v>
+        <v>Mechanical / Supplier Quality Engineering</v>
       </c>
       <c r="D59" t="str">
         <v>January–June 2027 (per title)</v>
@@ -2276,185 +2276,249 @@
         <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H59" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Life-Cycle-Engineering---Systems--January---June-2027--Hybrid-_REQ-2026-18149</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Development-Engineering---Mechanical--January-June-2027--Onsite-_REQ-2026-18209</v>
       </c>
       <c r="I59" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly (not a synthesized link); the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
       </c>
       <c r="J59" t="str">
-        <v>Boston metro (Acton). Most recently posted of the Insulet batch.</v>
+        <v>Boston metro (Acton).</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>GE HealthCare</v>
+        <v>Insulet</v>
       </c>
       <c r="B60" t="str">
-        <v>Infant Care V&amp;V Engineering Co-op - Spring 2027</v>
+        <v>Co-op, Systems Engineering - Design Verification (January–June 2027)</v>
       </c>
       <c r="C60" t="str">
-        <v>Mechanical / Verification &amp; Validation Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D60" t="str">
-        <v>Spring 2027</v>
+        <v>January–June 2027 (per title)</v>
       </c>
       <c r="E60" t="str">
-        <v>Waukesha, WI</v>
+        <v>Acton, MA</v>
       </c>
       <c r="F60">
-        <v>950</v>
+        <v>25</v>
       </c>
       <c r="G60" t="str">
-        <v>Not stated on posting</v>
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H60" t="str">
-        <v>https://gehc.wd5.myworkdayjobs.com/en-US/GEHC_ExternalSite/job/Waukesha/Infant-Care-V-V-Engineering-Co-op_R4046324-1</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering---Design-Verification--January---June-2027--Onsite-_REQ-2026-18144-1</v>
       </c>
       <c r="I60" t="str">
-        <v>Yes — full description fetched directly via Workday CXS API, posted 2 days ago.</v>
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
       </c>
       <c r="J60" t="str">
-        <v>Accepts Mechanical, Electrical, Computer, and Biomedical Engineering majors — verification/test focus, not pure design. Minimum 20-week commitment, onsite Waukesha WI, no visa sponsorship. Not Boston-area.</v>
+        <v>Boston metro (Acton).</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>GE Vernova</v>
+        <v>Insulet</v>
       </c>
       <c r="B61" t="str">
-        <v>Nuclear Engineering Co-Op/Intern - Spring 2027</v>
+        <v>Co-op, Life Cycle Engineering - Systems (January–June 2027)</v>
       </c>
       <c r="C61" t="str">
-        <v>Nuclear / Industrial Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D61" t="str">
-        <v>Spring 2027</v>
+        <v>January–June 2027 (per title)</v>
       </c>
       <c r="E61" t="str">
-        <v>Wilmington, NC</v>
+        <v>Acton, MA</v>
       </c>
       <c r="F61">
-        <v>750</v>
+        <v>25</v>
       </c>
       <c r="G61" t="str">
-        <v>$1,000–$2,000/week (varies by class year)</v>
+        <v>Not independently confirmed (see $25–34/hr range on sibling reqs)</v>
       </c>
       <c r="H61" t="str">
-        <v>https://careers.gevernova.com/ge-vernova-nuclear-engineering-co-op-intern-spring-2027/job/R5048552</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Life-Cycle-Engineering---Systems--January---June-2027--Hybrid-_REQ-2026-18149</v>
       </c>
       <c r="I61" t="str">
-        <v>Yes — fetched directly, structured JSON-LD job data embedded in the page confirmed title, pay, address, and datePosted (2026-09-11).</v>
+        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
       </c>
       <c r="J61" t="str">
-        <v>GE Vernova Hitachi Nuclear Energy (GVH) business. Not Boston-area.</v>
+        <v>Boston metro (Acton). Most recently posted of the Insulet batch.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Leonardo DRS</v>
+        <v>GE HealthCare</v>
       </c>
       <c r="B62" t="str">
-        <v>Mechanical Engineer Co-Op (Spring 2027)</v>
+        <v>Infant Care V&amp;V Engineering Co-op - Spring 2027</v>
       </c>
       <c r="C62" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Verification &amp; Validation Engineering</v>
       </c>
       <c r="D62" t="str">
-        <v>Spring 2027 (Jan–Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E62" t="str">
-        <v>Bridgeton, MO</v>
+        <v>Waukesha, WI</v>
       </c>
       <c r="F62">
-        <v>1050</v>
+        <v>950</v>
       </c>
       <c r="G62" t="str">
-        <v>$41,011–$53,315/yr base (co-op salary range) + bonus/equity eligibility per posting</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H62" t="str">
-        <v>https://careers.leonardodrs.com/job/Bridgeton-Mechanical-Engineer-Co-Op-%28Spring-2027%29-MO-63044/1418392000/</v>
+        <v>https://gehc.wd5.myworkdayjobs.com/en-US/GEHC_ExternalSite/job/Waukesha/Infant-Care-V-V-Engineering-Co-op_R4046324-1</v>
       </c>
       <c r="I62" t="str">
-        <v>Yes — fetched directly on Leonardo DRS's own careers.leonardodrs.com ATS (job ID 115172, posted 2026-09-09), confirmed open. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
+        <v>Yes — full description fetched directly via Workday CXS API, posted 2 days ago.</v>
       </c>
       <c r="J62" t="str">
-        <v>Land Systems division, Bridgeton, MO site. Junior+ standing, 1+ prior internship/co-op required, CAD (Creo/SolidWorks) required. No citizenship requirement stated on this posting. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
+        <v>Accepts Mechanical, Electrical, Computer, and Biomedical Engineering majors — verification/test focus, not pure design. Minimum 20-week commitment, onsite Waukesha WI, no visa sponsorship. Not Boston-area.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Insulet</v>
+        <v>GE Vernova</v>
       </c>
       <c r="B63" t="str">
-        <v>Co-op, Next Gen Platforms (NGP) Systems Engineering (Onsite)</v>
+        <v>Nuclear Engineering Co-Op/Intern - Spring 2027</v>
       </c>
       <c r="C63" t="str">
-        <v>Systems Engineering</v>
+        <v>Nuclear / Industrial Engineering</v>
       </c>
       <c r="D63" t="str">
-        <v>January 11 – June 30, 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E63" t="str">
-        <v>Acton, MA</v>
+        <v>Wilmington, NC</v>
       </c>
       <c r="F63">
-        <v>25</v>
+        <v>750</v>
       </c>
       <c r="G63" t="str">
-        <v>$25.00–$34.00/hr</v>
+        <v>$1,000–$2,000/week (varies by class year)</v>
       </c>
       <c r="H63" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Next-Gen-Platforms--NGP--Systems-Engineering--January-June-2027--Onsite-_REQ-2026-18071</v>
+        <v>https://careers.gevernova.com/ge-vernova-nuclear-engineering-co-op-intern-spring-2027/job/R5048552</v>
       </c>
       <c r="I63" t="str">
-        <v>Yes — fetched directly via Insulet's own Workday CXS job API (not an aggregator mirror), confirmed open, posted 5 days prior, application deadline 2026-12-31. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
+        <v>Yes — fetched directly, structured JSON-LD job data embedded in the page confirmed title, pay, address, and datePosted (2026-09-11).</v>
       </c>
       <c r="J63" t="str">
-        <v>Boston metro (Acton), onsite. US work authorization required, no sponsorship. 3.0 GPA minimum. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
+        <v>GE Vernova Hitachi Nuclear Energy (GVH) business. Not Boston-area.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
+        <v>Leonardo DRS</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Mechanical Engineer Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Spring 2027 (Jan–Aug 2027)</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Bridgeton, MO</v>
+      </c>
+      <c r="F64">
+        <v>1050</v>
+      </c>
+      <c r="G64" t="str">
+        <v>$41,011–$53,315/yr base (co-op salary range) + bonus/equity eligibility per posting</v>
+      </c>
+      <c r="H64" t="str">
+        <v>https://careers.leonardodrs.com/job/Bridgeton-Mechanical-Engineer-Co-Op-%28Spring-2027%29-MO-63044/1418392000/</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Yes — fetched directly on Leonardo DRS's own careers.leonardodrs.com ATS (job ID 115172, posted 2026-09-09), confirmed open. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Land Systems division, Bridgeton, MO site. Junior+ standing, 1+ prior internship/co-op required, CAD (Creo/SolidWorks) required. No citizenship requirement stated on this posting. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Co-op, Next Gen Platforms (NGP) Systems Engineering (Onsite)</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D65" t="str">
+        <v>January 11 – June 30, 2027</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F65">
+        <v>25</v>
+      </c>
+      <c r="G65" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H65" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Next-Gen-Platforms--NGP--Systems-Engineering--January-June-2027--Onsite-_REQ-2026-18071</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Yes — fetched directly via Insulet's own Workday CXS job API (not an aggregator mirror), confirmed open, posted 5 days prior, application deadline 2026-12-31. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check).</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Boston metro (Acton), onsite. US work authorization required, no sponsorship. 3.0 GPA minimum. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
         <v>Moderna</v>
       </c>
-      <c r="B64" t="str">
+      <c r="B66" t="str">
         <v>Co-Op, Applied Technologies (Spring 2027)</v>
       </c>
-      <c r="C64" t="str">
+      <c r="C66" t="str">
         <v>Automation / Process Engineering / Bioengineering (discipline caveat — not classic mechanical)</v>
       </c>
-      <c r="D64" t="str">
+      <c r="D66" t="str">
         <v>January 18 – June 25, 2027</v>
       </c>
-      <c r="E64" t="str">
+      <c r="E66" t="str">
         <v>Norwood, MA</v>
       </c>
-      <c r="F64">
+      <c r="F66">
         <v>14</v>
       </c>
-      <c r="G64" t="str">
+      <c r="G66" t="str">
         <v>$20.00–$60.00/hr per posting</v>
       </c>
-      <c r="H64" t="str">
+      <c r="H66" t="str">
         <v>https://modernatx.wd1.myworkdayjobs.com/en-US/M_tx/job/Co-Op--Applied-Technologies--Spring-2027-_R19735</v>
       </c>
-      <c r="I64" t="str">
+      <c r="I66" t="str">
         <v>Yes — fetched directly via Moderna's own Workday CXS job API (req R19735), returned live JSON confirming title, dates, pay, and open status. Upgraded from Partial (2026-09-21 ~07:00 UTC re-check); the previously-used biospace.com mirror (job 3072468) appears to be the same underlying posting under the job board's own listing ID, not a separate role.</v>
       </c>
-      <c r="J64" t="str">
+      <c r="J66" t="str">
         <v>Restricted to US persons (citizens/permanent residents/asylees/refugees) per prior mirror-sourced check, not re-confirmed word-for-word on this pass. Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J64"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J66"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C146"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -3968,9 +4032,108 @@
         <v>2026-09-21 ~07:00 UTC: fetched directly, confirmed live (link: saab.com/career/job-opportunities/systems-engineering-co-op-spring---summer-20272, $20.27-$22.30/hr + relocation bonus), but the term itself blends spring and summer into one combined window rather than a clean Winter/Spring-only co-op — judged closer to the common Summer 2027 wave Hamza asked to exclude than to a true Fall-through-Spring term. Flagged here rather than added; worth Hamza's own judgment call if he wants borderline spring/summer-blended terms reconsidered.</v>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Textron (Bell Helicopter / Textron Aviation)</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Fresh sweep, mechanical/systems co-op/intern search</v>
+      </c>
+      <c r="C138" t="str">
+        <v>2026-09-21 ~13:00 UTC: only a Summer 2027 program confirmed, with a posting window of Sept 1 - Oct 31, 2026. No Spring/Winter 2027 co-op found.</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Honeywell Aerospace</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Fresh sweep, mechanical/systems co-op/intern search</v>
+      </c>
+      <c r="C139" t="str">
+        <v>2026-09-21 ~13:00 UTC: 26 reqs found, all posted Aug 25-27, 2026 and all Summer 2027. No Spring/Winter 2027 co-op located.</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>Hexcel</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C140" t="str">
+        <v>2026-09-21 ~13:00 UTC: only summer-dated internship/co-op mentions found; no Spring 2027 posting confirmed.</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>MathWorks (Natick, MA)</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Engineering Development Group (EDG) internship listing</v>
+      </c>
+      <c r="C141" t="str">
+        <v>2026-09-21 ~13:00 UTC: re-checked and confirmed to be a Software Engineer role (C++/JavaScript/CS focus) — discipline mismatch, not merely an unconfirmed season as the 2026-09-19 note stated. Supersedes that earlier reason.</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>Waters Corporation (Milford, MA)</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Engineering co-op/intern search</v>
+      </c>
+      <c r="C142" t="str">
+        <v>2026-09-21 ~13:00 UTC: only an Electrical Engineering Co-op and non-engineering postings (scheduling, digital experience, network analyst) found; no mechanical engineering co-op located.</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>Chart Industries</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C143" t="str">
+        <v>2026-09-21 ~13:00 UTC: no internship/co-op postings of any kind found.</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>GreenPower Motor / Proterra</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C144" t="str">
+        <v>2026-09-21 ~13:00 UTC: no current 2027 postings; only stale historical (2022) Proterra listings found.</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>Universal Robots / ABB Robotics</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C145" t="str">
+        <v>2026-09-21 ~13:00 UTC: no Spring 2027-specific postings found for either.</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>Lockheed Martin / Sikorsky (Stratford, CT)</v>
+      </c>
+      <c r="B146" t="str">
+        <v>search-jobs URL and current careers.lockheedmartin.com structure</v>
+      </c>
+      <c r="C146" t="str">
+        <v>2026-09-21 ~13:00 UTC: confirmed further site migration — the legacy search-jobs URL now hard-redirects straight to lockheedmartin.com's 404 page. No Spring 2027 co-op/internship located. Worth trying the current careers.lockheedmartin.com host structure fresh next run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C137"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C146"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 12 checked-excluded (2026-09-21 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PsWXri9zLvTV8GZdMcLcwP
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -2518,7 +2518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C146"/>
+  <dimension ref="A1:C158"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -4131,9 +4131,141 @@
         <v>2026-09-21 ~13:00 UTC: confirmed further site migration — the legacy search-jobs URL now hard-redirects straight to lockheedmartin.com's 404 page. No Spring 2027 co-op/internship located. Worth trying the current careers.lockheedmartin.com host structure fresh next run.</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>Lockheed Martin / Sikorsky (Stratford, CT)</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Current recruiting portal, follow-up</v>
+      </c>
+      <c r="C147" t="str">
+        <v>2026-09-21 ~19:00 UTC: careers.lockheedmartin.com does not resolve (DNS failure) — the current live portal is lockheedmartin.eightfold.ai/careers. It is fully JS-rendered (fetch returns only site config, no listings); targeted searches for Sikorsky/Stratford/Spring 2027 co-ops returned no matches. Still no Spring 2027 co-op/internship located.</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>General Dynamics Mission Systems</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Mechanical Engineering Co-Op (Jan-May 2027), McLeansville NC, req 74530 (already Partial in `rows`) — re-verify attempt</v>
+      </c>
+      <c r="C148" t="str">
+        <v>2026-09-21 ~19:00 UTC: same icims-redirects-to-landing-page and gd.com-403 blocking pattern persists. Confirmed the same req ID/pay ($26-29/hr) via additional aggregator mirrors (Glassdoor, career.io) but still no independently-rendered live page. Status unchanged at Partial in `rows`.</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B149" t="str">
+        <v>req 601496955 (already Partial in `rows`) — 8th+ consecutive re-check</v>
+      </c>
+      <c r="C149" t="str">
+        <v>2026-09-21 ~19:00 UTC: still blocked by Cloudflare/CAPTCHA on jobs.buildsubmarines.com; direct fetch and r.jina.ai proxy fallback both failed. Underlying posting still corroborated by WebSearch snippets only. Status unchanged at Partial in `rows` — needs an actual in-browser/human check, deprioritizing further automated attempts.</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Spring 2027 co-op search, re-check</v>
+      </c>
+      <c r="C150" t="str">
+        <v>2026-09-21 ~19:00 UTC: only Fall 2026 co-ops and a Summer 2027 internship currently live. Still nothing posted for Spring 2027 despite the company's own stated Sept-Oct posting window. Re-check again in 1-2 weeks.</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C151" t="str">
+        <v>2026-09-21 ~19:00 UTC: no change — Analog Devices has zero open US intern/co-op reqs currently; Lam Research's 2027 mechanical co-op cycle not yet posted per the company's own program page.</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B152" t="str">
+        <v>careers.ll.mit.edu search, re-check</v>
+      </c>
+      <c r="C152" t="str">
+        <v>2026-09-21 ~19:00 UTC: no new in-discipline Spring 2027 req found. Current Jan-June 2027 postings skew Contracting/Logistics and Cyber Security (discipline mismatch, already excluded); Microfabrication Industrial Eng Co-op is already tracked in `rows`.</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Spring 2027 co-op search, re-check for new Lynn MA reqs</v>
+      </c>
+      <c r="C153" t="str">
+        <v>2026-09-21 ~19:00 UTC: no Lynn, MA Spring 2027 req found. The only live Spring 2027 'Engines Engineering Co-op' reqs (R5029619 etc.) are Computer/Software discipline in Evendale, OH and/or already confirmed dead ('no longer posted').</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>Caterpillar</v>
+      </c>
+      <c r="B154" t="str">
+        <v>'2027 Engineering Corporate Parallel Co-op Program' (new req IDs r0000380509, r0000380489, r0000380484), Tucson/Green Valley AZ, Champaign/Decatur/Mossville IL, Lafayette IN</v>
+      </c>
+      <c r="C154" t="str">
+        <v>2026-09-21 ~19:00 UTC: pages opened directly and confirmed live/open, but the program is structured as a continuous multi-rotation 'parallel' format (full-time summer + part-time during school year) with no discrete Winter-2026/Spring-2027-only term stated on the posting — same ambiguous-format exclusion as prior Caterpillar Parallel Co-op findings. No MA location either.</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Spring 2027 Manufacturing Engineering Internship (Undergraduate), Space Coast FL, req R66348</v>
+      </c>
+      <c r="C155" t="str">
+        <v>2026-09-21 ~19:00 UTC: found via a Prosple aggregator mirror ($38/hr, mechanical/propulsion/structural/fluid/avionics scope, US citizen/GC/asylee/refugee required); Blue Origin's own Workday page returned blank/JS-blocked on 2 direct fetch attempts. The aggregator itself states the application window closed July-Aug 2026 — i.e. already past as of today — so this req is very likely closed. Excluded rather than added as Partial, given the strong signal it's already closed.</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>Spirit AeroSystems / Medtronic / Becton Dickinson / Moog Inc / Woodward Inc / PerkinElmer (Revvity) / PTC / Natel Energy / Sanergy / Nuvation Engineering</v>
+      </c>
+      <c r="B156" t="str">
+        <v>General mechanical/aerospace/manufacturing engineering intern/co-op search, each company</v>
+      </c>
+      <c r="C156" t="str">
+        <v>2026-09-21 ~19:00 UTC: no Winter 2026/Spring 2027-dated postings found at any of these. Becton Dickinson's only relevant req ('R&amp;D Co-op') is Spring 2026, already past — wrong season. Boston Scientific's 'R&amp;D Engineering Co-op 2026' (Marlborough, MA) confirmed dead/expired on direct fetch.</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>GD Bath Iron Works</v>
+      </c>
+      <c r="B157" t="str">
+        <v>'2027 Spring Manufacturing Apprentice'</v>
+      </c>
+      <c r="C157" t="str">
+        <v>2026-09-21 ~19:00 UTC: this is a trades apprenticeship program, not an engineering co-op — discipline mismatch, excluded.</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>GD Ordnance &amp; Tactical Systems / Northrop Grumman (Boston-area presence)</v>
+      </c>
+      <c r="B158" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C158" t="str">
+        <v>2026-09-21 ~19:00 UTC: no dedicated OTS-specific co-op postings found; no Northrop Grumman Boston/MA-area postings found (their live Spring 2027 mechanical co-op remains the already-tracked Chandler, AZ req).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C146"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C158"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 10 checked-excluded (2026-09-22 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWUZ9fn5Gz14xg51eG6Nz8
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J69"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -2509,16 +2509,112 @@
         <v>Restricted to US persons (citizens/permanent residents/asylees/refugees) per prior mirror-sourced check, not re-confirmed word-for-word on this pass. Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Applied Materials</v>
+      </c>
+      <c r="B67" t="str">
+        <v>2027 Spring Mechanical Engineer Co-op (Gloucester, MA)</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Spring 2027 (start January 2027)</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Gloucester, MA</v>
+      </c>
+      <c r="F67">
+        <v>35</v>
+      </c>
+      <c r="G67" t="str">
+        <v>$31–$33/hr</v>
+      </c>
+      <c r="H67" t="str">
+        <v>https://jobs.appliedmaterials.com/job/gloucester/2027-spring-mechanical-engineer-co-op-gloucester-ma/95/100424621952</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Yes — fetched directly on Applied Materials' own careers site (job ID R2628290 / 100424621952), confirmed open, posted 2026-09-10, active Apply button present.</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Boston metro (Gloucester, ~45 min drive). GPA 3.0+ preferred, good academic standing required. No explicit citizenship/visa language stated on the posting. Applied Materials is already a tracked company (other reqs elsewhere) — this is a distinct new req/season/location.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Vertex Pharmaceuticals</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Vertex Spring Co-Op 2027, Mechanical Automation</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Mechanical / Industrial Engineering (mechanical design, GD&amp;T, mechanism/robotics design)</v>
+      </c>
+      <c r="D68" t="str">
+        <v>January – June 2027</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Boston, MA</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68" t="str">
+        <v>$25.00–$50.00/hr</v>
+      </c>
+      <c r="H68" t="str">
+        <v>https://vrtx.wd501.myworkdayjobs.com/vertex_careers/job/Boston-MA/Vertex-Spring-Co-Op-2027--Mechanical-Automation_REQ-30500-1</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Partial — confirmed via an independent aggregator mirror (zapply.jobs) showing full title/season/pay/location and a posted date of 2026-09-21 (one day before this check); Vertex's own Workday page returned blank/JS-rendered content on direct fetch (both wd5 and wd501 subdomains tried), consistent with a known recurring Vertex Workday access issue.</v>
+      </c>
+      <c r="J68" t="str">
+        <v>Application deadline stated as November 15, 2026 (rolling review, may close earlier). No stated visa sponsorship. Distinct from Vertex's 'Process Development Upstream' and 'CGT Process Development' Spring Co-Op 2027 reqs, which are biotech/process discipline and excluded (see `checked`).</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Mechanical Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Mechanical / Aerospace Engineering (spacecraft structures, brackets, mechanisms)</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Spring 2027 (12-week internship)</v>
+      </c>
+      <c r="E69" t="str">
+        <v>San Francisco, CA</v>
+      </c>
+      <c r="F69">
+        <v>2700</v>
+      </c>
+      <c r="G69" t="str">
+        <v>$29.00/hr</v>
+      </c>
+      <c r="H69" t="str">
+        <v>https://job-boards.greenhouse.io/astranis/jobs/4704602006</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Yes — fetched directly on Greenhouse, confirmed open.</v>
+      </c>
+      <c r="J69" t="str">
+        <v>ITAR-restricted: requires US citizen, lawful permanent resident, or other 'protected individual' status under export control rules. Not Boston-area, included per Hamza's nationwide preference. A separate Summer 2027 version of this same role exists (job 4704601006) — do not confuse the two; only this Spring 2027 req qualifies.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J69"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C158"/>
+  <dimension ref="A1:C168"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -4263,9 +4359,119 @@
         <v>2026-09-21 ~19:00 UTC: no dedicated OTS-specific co-op postings found; no Northrop Grumman Boston/MA-area postings found (their live Spring 2027 mechanical co-op remains the already-tracked Chandler, AZ req).</v>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>Sonos (Boston, MA)</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Mechanical Engineering Co-Op, req R2547/R2547-1</v>
+      </c>
+      <c r="C159" t="str">
+        <v>2026-09-22: confirmed via multiple sources (Glassdoor, mediabistro, aggregators) this is a July-December 2026 program only (Fall 2026, applications close Oct 25) — does not extend into Spring 2027. Excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>Vertex Pharmaceuticals</v>
+      </c>
+      <c r="B160" t="str">
+        <v>'Process Development Upstream' and 'CGT Process Development' Spring Co-Op 2027 reqs</v>
+      </c>
+      <c r="C160" t="str">
+        <v>2026-09-22: both real/dated Spring 2027 postings, but discipline is biotech/process/cell-culture, not mechanical/aerospace/manufacturing. Excluded — discipline mismatch. (Distinct from the Mechanical Automation Spring Co-Op REQ-30500-1 added to `rows` this run.)</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Internship program incl. Mechanical/Aerospace Engineering Intern</v>
+      </c>
+      <c r="C161" t="str">
+        <v>2026-09-22: company's own careers page states internships run 'typically May or June, concluding August or September' with an April 30 application deadline — the standard Summer 2027 wave. Excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Co-Op - System Engineer, req R6576</v>
+      </c>
+      <c r="C162" t="str">
+        <v>2026-09-22: appeared in search-engine cache but direct fetch of the live URL returns HTTP 404; current full job listing page shows no mechanical/systems co-op openings, only Skillbridge military-transition fellow roles. Excluded — appears filled/removed (stale listing).</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Commonwealth Fusion Systems (Devens, MA)</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Lever careers board, re-check</v>
+      </c>
+      <c r="C163" t="str">
+        <v>2026-09-22: current open postings show only a 'Fall Co-op 2026' mechanical engineer role plus permanent/contract positions — no Spring 2027 co-op currently posted. No change.</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Spring 2027 co-op search, re-check</v>
+      </c>
+      <c r="C164" t="str">
+        <v>2026-09-22: as of today, careers.huntingtoningalls.com shows only a 'Fall 2026 Engineering Co-Op' and a '2027 Engineering Summer Internship' — no Spring 2027 co-op req found yet despite the company's own Sept-Oct posting-window claim. Re-check again in ~1 week.</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B165" t="str">
+        <v>careers.ll.mit.edu search, re-check</v>
+      </c>
+      <c r="C165" t="str">
+        <v>2026-09-22: only in-discipline-adjacent Jan-June 2027 co-op found is Cyber Security (Group 11-10) — discipline mismatch, excluded. A 'Rapid Prototyping Aero/Mech' co-op (Group 77) is Fall 2026 — wrong season. No new in-discipline Spring 2027 req found.</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Full careers site sweep, re-check</v>
+      </c>
+      <c r="C166" t="str">
+        <v>2026-09-22: no new reqs found beyond the two already tracked in `rows` (Systems Engineering Co-Op JR002882, Electro-Mechanical Instrument Co-op JR002883-1). No change.</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B167" t="str">
+        <v>careers.geaerospace.com, re-check for new Lynn MA reqs</v>
+      </c>
+      <c r="C167" t="str">
+        <v>2026-09-22: no new Lynn, MA-specific Spring 2027 mechanical/systems req found beyond the already-tracked Engines Engineering Co-op and Structures Intern/Co-op. No change.</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>Boston Scientific / PTC / Desktop Metal / Markforged / Vicor / Nuvation Engineering / Instron / Analogic / Boston Metal / Alloy Enterprises</v>
+      </c>
+      <c r="B168" t="str">
+        <v>General mechanical/aerospace/manufacturing engineering intern/co-op search, each company</v>
+      </c>
+      <c r="C168" t="str">
+        <v>2026-09-22: no Winter 2026/Spring 2027-dated postings found at any of these. Boston Scientific's only visible current Spring co-op is in Johns Creek, GA (not MA) with ambiguous 'Spring or Summer 2026/2027' season wording.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C158"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C168"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 14 checked-excluded, 2 upgraded Partial->Yes (2026-09-22 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bm8cATjS8AR2oLXpQZnRSh
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J72"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -877,13 +877,13 @@
         <v>$26.00–$29.00/hr</v>
       </c>
       <c r="H15" t="str">
-        <v>https://careers-gdms.icims.com/jobs/74530/mechanical-engineering-co-op---%28january---may-2027%29/job</v>
+        <v>https://www.gd.com/careers/mechanical-engineering-co-op-january-may-2027-mcleansville-nc-us-2026-74530-gdms-opportunity</v>
       </c>
       <c r="I15" t="str">
-        <v>Partial — corroborated across multiple independent sources (aggregator mirror quoting exact title/pay/dates/location, Glassdoor, career.io) with consistent details, but the icims URL redirected to a generic GDMS careers landing page (no job content) and the gd.com mirror URL returned HTTP 403 on direct fetch. Could not independently confirm current open/closed status. Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-22: fetched directly from gd.com (req ID 2026-74530, corrected URL — previous guessed/mirrored URL was missing the '2026-' year prefix, which is why it kept 403/404ing), full posting text confirmed 'Posted Date: 9/8/2026' and 'This job posting will remain open until the position is filled.'</v>
       </c>
       <c r="J15" t="str">
-        <v>Not Boston-area. Sibling req 'Mechanical Engineering Co-Op (July–December 2026)' exists at the same site — different season, not this one. Likely requires US citizenship (ITAR/clearance) as with other GDMS reqs.</v>
+        <v>Not Boston-area. Sibling req 'Mechanical Engineering Co-Op (July–December 2026)' exists at the same site — different season, not this one. Requires US citizenship + DoD Secret clearance eligibility.</v>
       </c>
     </row>
     <row r="16">
@@ -2564,10 +2564,10 @@
         <v>$25.00–$50.00/hr</v>
       </c>
       <c r="H68" t="str">
-        <v>https://vrtx.wd501.myworkdayjobs.com/vertex_careers/job/Boston-MA/Vertex-Spring-Co-Op-2027--Mechanical-Automation_REQ-30500-1</v>
+        <v>https://vrtx.wd501.myworkdayjobs.com/Vertex_Careers/job/Boston-MA/Vertex-Spring-Co-Op-2027--Mechanical-Automation_REQ-30500-1</v>
       </c>
       <c r="I68" t="str">
-        <v>Partial — confirmed via an independent aggregator mirror (zapply.jobs) showing full title/season/pay/location and a posted date of 2026-09-21 (one day before this check); Vertex's own Workday page returned blank/JS-rendered content on direct fetch (both wd5 and wd501 subdomains tried), consistent with a known recurring Vertex Workday access issue.</v>
+        <v>Yes — upgraded 2026-09-22: fetched directly via Vertex's own Workday CXS API (not an aggregator mirror), confirmed live and open, posted 2026-09-21/22.</v>
       </c>
       <c r="J68" t="str">
         <v>Application deadline stated as November 15, 2026 (rolling review, may close earlier). No stated visa sponsorship. Distinct from Vertex's 'Process Development Upstream' and 'CGT Process Development' Spring Co-Op 2027 reqs, which are biotech/process discipline and excluded (see `checked`).</v>
@@ -2605,16 +2605,112 @@
         <v>ITAR-restricted: requires US citizen, lawful permanent resident, or other 'protected individual' status under export control rules. Not Boston-area, included per Hamza's nationwide preference. A separate Summer 2027 version of this same role exists (job 4704601006) — do not confuse the two; only this Spring 2027 req qualifies.</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Mechanical Design Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Mechanical / Aerospace Engineering</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Jamestown, ND</v>
+      </c>
+      <c r="F70">
+        <v>1500</v>
+      </c>
+      <c r="G70" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H70" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Mechanical-Design-Engineering-Co-op--Winter-Spring-2027-_01871736</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Yes — fetched directly via RTX's own Workday CXS API, posted 2026-09-21.</v>
+      </c>
+      <c r="J70" t="str">
+        <v>Distinct req from the already-tracked Jamestown ND 'Structural Engineering Co-op' (req 01873938) at the same site — different title/req, not a duplicate.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Co-op, Supplier Engineering - Global Technical Excellence (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Electrical / Industrial / Biomedical Engineering (manufacturing root-cause, supplier qualification, Six Sigma/Lean)</v>
+      </c>
+      <c r="D71" t="str">
+        <v>January 11 – June 30, 2027</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F71">
+        <v>25</v>
+      </c>
+      <c r="G71" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H71" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Engineering---Global-Technical-Excellence--January---June-2027--Onsite-_REQ-2026-18213</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Yes — fetched directly via Insulet's own Workday CXS API, posted 2026-09-15.</v>
+      </c>
+      <c r="J71" t="str">
+        <v>Boston metro (Acton). Not eligible for visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Co-op, Supplier Engineering - Project Management Excellence (January–June 2027, Onsite)</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Mechanical / Industrial / Bio-Engineering</v>
+      </c>
+      <c r="D72" t="str">
+        <v>January 11 – June 30, 2027</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F72">
+        <v>25</v>
+      </c>
+      <c r="G72" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H72" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Engineering---Project-Management-Excellence--January---June-2027--Onsite-_REQ-2026-18211</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Yes — fetched directly via Insulet's own Workday CXS API, posted 2026-09-16.</v>
+      </c>
+      <c r="J72" t="str">
+        <v>Boston metro (Acton). Requires enrollment in undergraduate mechanical, industrial, or bio-engineering program. Not eligible for visa sponsorship.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J72"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C168"/>
+  <dimension ref="A1:C182"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -4469,9 +4565,163 @@
         <v>2026-09-22: no Winter 2026/Spring 2027-dated postings found at any of these. Boston Scientific's only visible current Spring co-op is in Johns Creek, GA (not MA) with ambiguous 'Spring or Summer 2026/2027' season wording.</v>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>Philips</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Co-op, Robotics Mechatronics, Surgical Robotics (Cambridge, MA), req 589905</v>
+      </c>
+      <c r="C169" t="str">
+        <v>2026-09-22 ~07:00 UTC: RESOLVED — queried Philips' own live Workday job-search API directly for 'Surgical Robotics', 'Mechatronics', and req 589905 itself: zero results. The posting no longer exists in Philips' current job index (the prior Fall-2026-vs-Jan-2027 season conflict across aggregator mirrors is now moot). Do not re-track unless a fresh req appears. Supersedes the earlier 'season conflict, unresolved' note.</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Mechanical/Industrial Engineering Co-op, req 01872434, Melbourne FL</v>
+      </c>
+      <c r="C170" t="str">
+        <v>2026-09-22 ~07:00 UTC: re-confirmed via a second independent aggregator mirror — exact title is 'Mechanical/Industrial Engineering Co-op (Spring/Summer 2027)', a genuinely combined term, not a clean Spring-only posting. Excluded, consistent with prior run.</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>CMTA, Inc.</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Mechanical Engineer Intern/Co-op Spring 2027</v>
+      </c>
+      <c r="C171" t="str">
+        <v>2026-09-22 ~07:00 UTC: location is Greater Indianapolis/Council Bluffs IA area (not Boston); discipline is MEP building-systems consulting (HVAC/Revit/AutoCAD for construction drawings), not mechanical/aerospace/manufacturing/robotics. Excluded on both location and discipline grounds.</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>Astranis</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Mechanical Engineer Intern (Winter 2027), SF, via Greenhouse — re-check</v>
+      </c>
+      <c r="C172" t="str">
+        <v>2026-09-22 ~07:00 UTC: re-confirmed live/open ($29/hr), but season is literally 'Winter 2027' (not Winter 2026 or Spring 2027 as required). Excluded, consistent with prior run. The separate Spring 2027 Astranis req remains tracked in `rows`.</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B173" t="str">
+        <v>'Spring 2027 Manufacturing Engineering Internship – Graduate', Huntsville AL</v>
+      </c>
+      <c r="C173" t="str">
+        <v>2026-09-22 ~07:00 UTC: could not find a verifiable req ID for a Spring (non-Summer) version of this Huntsville role; only located the Summer 2027 Huntsville req (R71427). Not conclusively ruled out (may be a mislabeled aggregator listing of the Summer req) — worth a follow-up to find the correct req ID.</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B174" t="str">
+        <v>Co-Op - System Engineer, req R6576 — re-check</v>
+      </c>
+      <c r="C174" t="str">
+        <v>2026-09-22 ~07:00 UTC: no specific dated Spring 2027 req found again this run, same as prior 404 outcome. No change.</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>Vicarious Surgical (Waltham, MA)</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Full careers site, re-check</v>
+      </c>
+      <c r="C175" t="str">
+        <v>2026-09-22 ~07:00 UTC: only a January 2026 Mechanical Engineering Co-Op found (already past); nothing dated 2027. No change.</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>Commonwealth Fusion Systems (Devens, MA)</v>
+      </c>
+      <c r="B176" t="str">
+        <v>Careers board, re-check</v>
+      </c>
+      <c r="C176" t="str">
+        <v>2026-09-22 ~07:00 UTC: only a Fall 2026 Mechanical Engineer co-op found; no Spring 2027 posting. No change.</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>Sierra Space</v>
+      </c>
+      <c r="B177" t="str">
+        <v>General co-op/intern search</v>
+      </c>
+      <c r="C177" t="str">
+        <v>2026-09-22 ~07:00 UTC: no dated Spring 2027 req found; company's own stated posting pattern (September post, December deadline) suggests not yet live. Worth a follow-up.</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>Teradyne (North Reading, MA)</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Mechanical Engineering Co-op, re-check</v>
+      </c>
+      <c r="C178" t="str">
+        <v>2026-09-22 ~07:00 UTC: only a Spring 2026 (already past) cohort found; Spring 2027 not yet posted. No change.</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>iRobot (Bedford, MA)</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Full careers site, re-check</v>
+      </c>
+      <c r="C179" t="str">
+        <v>2026-09-22 ~07:00 UTC: only historical/Fall postings found; company recently went through bankruptcy/acquisition by Shenzhen Picea Robotics, adding uncertainty to whether a 2027 program will run at all. No change.</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Spring 2027 co-op search, re-check</v>
+      </c>
+      <c r="C180" t="str">
+        <v>2026-09-22 ~07:00 UTC: 33 search results, every one is either a 'Fall 2026' co-op/designer role or a '2027 College Summer Intern' — zero Spring 2027 co-ops exist as of today, despite the company's own stated Sept-Oct posting-window claim now having failed to materialize across 5+ checked runs. Recommend telling Hamza this claim may not be reliable this cycle rather than continuing indefinite re-checks.</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C181" t="str">
+        <v>2026-09-22 ~07:00 UTC: no change, still nothing posted for the 2027 cycle.</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Leidos / L3Harris / Spirit AeroSystems / Textron Aviation / Boeing / Moog / Woodward / Hexcel / Curtiss-Wright / Northrop Grumman (new locations)</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Fresh sweep, mechanical/aerospace/manufacturing intern/co-op search</v>
+      </c>
+      <c r="C182" t="str">
+        <v>2026-09-22 ~07:00 UTC: no qualifying new findings at any of these — Curtiss-Wright's JR1907 still has no stated year, Northrop Grumman has no new location beyond the already-tracked Chandler AZ req. No change.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C168"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C182"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 12 new postings, 25 checked-excluded, 1 upgraded Partial->Yes (2026-09-22 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VEMjUMRqLue6VGEqF4q4jc
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J84"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1825,16 +1825,16 @@
         <v>17</v>
       </c>
       <c r="G45" t="str">
-        <v>Not stated (aggregator only)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H45" t="str">
         <v>https://berkshiregrey.bamboohr.com/careers/771</v>
       </c>
       <c r="I45" t="str">
-        <v>Partial — BambooHR page rendered empty on two direct fetch attempts. Only confirmed via a third-party aggregator (posted ~Sept 1, 2026), not first-hand. Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-22 ~13:00 UTC: confirmed via direct fetch of Berkshire Grey's own BambooHR API, jobOpeningStatus 'Open'. Supersedes the earlier 'Partial, aggregator-only' status.</v>
       </c>
       <c r="J45" t="str">
-        <v>Boston metro (Bedford).</v>
+        <v>Scoop™ engineering quality team, V&amp;V of electromechanical systems. Boston metro (Bedford).</v>
       </c>
     </row>
     <row r="46">
@@ -2701,16 +2701,400 @@
         <v>Boston metro (Acton). Requires enrollment in undergraduate mechanical, industrial, or bio-engineering program. Not eligible for visa sponsorship.</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Microfabrication Engineering Co-Op (Group 08-35, Microelectronics Laboratory)</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Materials Science / Chemistry / Physics / Engineering (wafer fab process engineering)</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Jan–August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Lexington, MA</v>
+      </c>
+      <c r="F73">
+        <v>13</v>
+      </c>
+      <c r="G73" t="str">
+        <v>$24.50–$31.00/hr (technical co-op rate)</v>
+      </c>
+      <c r="H73" t="str">
+        <v>https://careers.ll.mit.edu/job/Lexington-Group-08-35-Microfabrication-Engineering-Co-Op-Microelectronics-Laboratory-Jan-Aug-2027-MA-02420/1368363000/</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Yes — fetched directly, 'Apply now' live, posted 2026-09-17.</v>
+      </c>
+      <c r="J73" t="str">
+        <v>Req 42762. Sibling req to the already-tracked Microfab Industrial Eng. Co-Op (Group 08-35) — same Jan-Aug 2027 window, different discipline focus (materials/process vs industrial). Requires US citizenship + eligibility for Secret-level DoD clearance; cleanroom work.</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Materials and Chemistry Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Materials Engineering</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F74">
+        <v>3</v>
+      </c>
+      <c r="G74" t="str">
+        <v>$20.00–$45.00/hr (base range, per posting)</v>
+      </c>
+      <c r="H74" t="str">
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Materials-and-Chemistry-Engineering-Co-op--Spring-2027-_JR002942</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Yes — fetched directly via Draper's Workday CXS job API, canApply true, posted 2026-09-21.</v>
+      </c>
+      <c r="J74" t="str">
+        <v>Req JR002942. Onsite required. Draper's other co-ops in this batch state US citizenship is mandatory due to sensitive work — verify before applying.</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Capital Equipment Engineering Co-Op</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Mechanical / Equipment Engineering</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F75">
+        <v>25</v>
+      </c>
+      <c r="G75" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H75" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Capital-Equipment-Engineering-Co-Op_REQ-14497</v>
+      </c>
+      <c r="I75" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text itself states 'Spring 2027 season'.</v>
+      </c>
+      <c r="J75" t="str">
+        <v>REQ-14497. New company for the tracker. Boston metro (Billerica).</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Automation &amp; Controls Engineering Co-Op</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Controls / Automation Engineering</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F76">
+        <v>25</v>
+      </c>
+      <c r="G76" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H76" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Automation---Controls-Engineering-Co-Op_REQ-14444</v>
+      </c>
+      <c r="I76" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text itself states 'Spring 2027 season'.</v>
+      </c>
+      <c r="J76" t="str">
+        <v>REQ-14444. PLC/Allen-Bradley/Rockwell work.</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Material Quality Engineering Co-Op</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Materials / Quality Engineering</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F77">
+        <v>25</v>
+      </c>
+      <c r="G77" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H77" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Material-Quality-Engineering-Co-Op_REQ-14469</v>
+      </c>
+      <c r="I77" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 12 days ago); posting text itself states 'Spring 2027 season'.</v>
+      </c>
+      <c r="J77" t="str">
+        <v>REQ-14469. Semiconductor liquid filtration products.</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Industrial Engineering Co-Op</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Industrial / Manufacturing Engineering</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F78">
+        <v>25</v>
+      </c>
+      <c r="G78" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H78" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Industrial-Engineering-Co-Op_REQ-14462</v>
+      </c>
+      <c r="I78" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text itself states 'Spring 2027 season'.</v>
+      </c>
+      <c r="J78" t="str">
+        <v>REQ-14462. Manufacturing/materials process optimization.</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Continuous Improvement Co-Op</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Manufacturing / Process Engineering (Lean/Kaizen)</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F79">
+        <v>25</v>
+      </c>
+      <c r="G79" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H79" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Continuous-Improvement-Co-Op_REQ-14504</v>
+      </c>
+      <c r="I79" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text itself states 'Spring 2027 season'.</v>
+      </c>
+      <c r="J79" t="str">
+        <v>REQ-14504. Assembly/Flush Room/Warehouse cost reduction, Kaizen/5S/Gemba.</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Spring 2027 Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Spring 2027 (approx. Jan–June 2027, dates flexible)</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F80">
+        <v>17</v>
+      </c>
+      <c r="G80" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H80" t="str">
+        <v>https://berkshiregrey.bamboohr.com/careers/760</v>
+      </c>
+      <c r="I80" t="str">
+        <v>Yes — confirmed via direct fetch of Berkshire Grey's own BambooHR API, jobOpeningStatus 'Open'.</v>
+      </c>
+      <c r="J80" t="str">
+        <v>SolidWorks/DFM/prototyping, product development team, testing + NPI support. Boston metro (Bedford).</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Spring 2027 Mechatronics Engineering Co-op</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Mechatronics / Controls</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Spring 2027 (approx. Jan–June 2027, dates flexible)</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F81">
+        <v>17</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H81" t="str">
+        <v>https://berkshiregrey.bamboohr.com/careers/772</v>
+      </c>
+      <c r="I81" t="str">
+        <v>Yes — confirmed via direct fetch of Berkshire Grey's own BambooHR API, jobOpeningStatus 'Open'.</v>
+      </c>
+      <c r="J81" t="str">
+        <v>PLC development, test-fixture controls. Boston metro (Bedford).</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Spring 2027 Robot Learning R&amp;D Co-op</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Robotics R&amp;D (manipulation research; listed under Software dept)</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Spring 2027 (approx. Jan–June 2027, dates flexible)</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F82">
+        <v>17</v>
+      </c>
+      <c r="G82" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H82" t="str">
+        <v>https://berkshiregrey.bamboohr.com/careers/768</v>
+      </c>
+      <c r="I82" t="str">
+        <v>Yes — confirmed via direct fetch of Berkshire Grey's own BambooHR API, jobOpeningStatus 'Open'.</v>
+      </c>
+      <c r="J82" t="str">
+        <v>Borderline discipline fit — robot manipulation R&amp;D, filed under Software department rather than a hardware/mechanical department. Included per Hamza's robotics discipline preference; his own judgment call on fit. Boston metro (Bedford).</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Spring 2027 Engineering Intern - Undergraduate</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Multi-discipline (Mechanical, Manufacturing, Propulsion/Fluids, Test, Aerospace Systems Engineering, among others — placement not guaranteed)</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Greater Seattle Area (additional site options: Van Horn TX, Huntsville AL, Denver CO, Space Coast FL, Los Angeles CA, Longmont CO)</v>
+      </c>
+      <c r="F83">
+        <v>2500</v>
+      </c>
+      <c r="G83" t="str">
+        <v>Not stated in this posting</v>
+      </c>
+      <c r="H83" t="str">
+        <v>https://blueorigin.wd5.myworkdayjobs.com/en-US/BlueOrigin/job/Spring-2027--Engineering-Intern---Undergraduate_R69064</v>
+      </c>
+      <c r="I83" t="str">
+        <v>Yes — fetched directly via Blue Origin's own Workday CXS API, canApply true, posted 30+ days ago.</v>
+      </c>
+      <c r="J83" t="str">
+        <v>Req R69064. General multi-discipline req — actual engineering discipline/site placement determined after applying/interviewing, mechanical not guaranteed. Requires US citizen/national, Green Card holder, or lawfully admitted refugee/asylee.</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>SpaceX</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Spring 2027 Graduate Engineer Internship/Co-op</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Engineering (design/manufacturing/operations; open to mechanical/aerospace)</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Spring 2027 (Jan or Mar 2027 start, 12+ weeks)</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Multiple US sites incl. Bloomfield, CT (closest); also Bastrop TX, Brownsville TX, Cape Canaveral FL, Hawthorne CA, Irvine CA, Long Beach CA, McGregor TX, Palo Alto CA, Redmond WA, Vandenberg CA, Woodinville WA</v>
+      </c>
+      <c r="F84">
+        <v>100</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Bachelor's $83,200/yr; Master's $91,000/yr; PhD $100,100/yr (annualized)</v>
+      </c>
+      <c r="H84" t="str">
+        <v>https://job-boards.greenhouse.io/spacex/jobs/8621749002</v>
+      </c>
+      <c r="I84" t="str">
+        <v>Yes — fetched directly on Greenhouse, live apply flow confirmed.</v>
+      </c>
+      <c r="J84" t="str">
+        <v>Distinct req from the already-tracked undergrad-oriented 'Spring 2027 Engineering Internship/Co-op' (job 8616338002) — THIS req explicitly requires the applicant to already hold a bachelor's degree AND be currently enrolled in a graduate program. Only relevant if Hamza is in/entering grad school by Spring 2027. US citizen/permanent resident/refugee/asylee required (ITAR).</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J84"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C182"/>
+  <dimension ref="A1:C207"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -4719,9 +5103,284 @@
         <v>2026-09-22 ~07:00 UTC: no qualifying new findings at any of these — Curtiss-Wright's JR1907 still has no stated year, Northrop Grumman has no new location beyond the already-tracked Chandler AZ req. No change.</v>
       </c>
     </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B183" t="str">
+        <v>'Spring 2027 Manufacturing Engineering Internship – Graduate', Huntsville AL</v>
+      </c>
+      <c r="C183" t="str">
+        <v>2026-09-22 ~13:00 UTC: RESOLVED — queried Blue Origin's live Workday jobs API directly for all 'Manufacturing Engineering Internship Graduate' postings company-wide: only 'Summer 2027 Manufacturing Engineering Internship - Graduate' (R71427), Huntsville AL, exists. No Spring 2027 Graduate version exists anywhere in the company's current listings. The aggregator mirror implying a Spring 2027/Huntsville/Graduate posting was a mislabeled/stale listing. Supersedes prior run's 'not conclusively ruled out' note — do not re-track.</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>SpaceX</v>
+      </c>
+      <c r="B184" t="str">
+        <v>'Spring 2027 Silicon Engineering Internship/Co-op'; 'Spring 2027 Software Engineering Internship/Co-op'</v>
+      </c>
+      <c r="C184" t="str">
+        <v>2026-09-22 ~13:00 UTC: both confirmed live/dated correctly but discipline mismatch (electrical/software, not mechanical/aerospace/manufacturing/robotics). Excluded. (Distinct from the Graduate Engineer req added to `rows` this run.)</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Joby Aviation</v>
+      </c>
+      <c r="B185" t="str">
+        <v>'Flight Test Intern (Dec 2026-Feb 2027)'</v>
+      </c>
+      <c r="C185" t="str">
+        <v>2026-09-22 ~13:00 UTC: confirmed via direct fetch the posting now returns HTTP 410 Gone — dead/removed. Only Summer 2025/2026 mechanical reqs otherwise found on their current board (wrong season). No live Spring 2027/Winter 2026 mechanical/structures req found.</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>Archer Aviation</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Mechanical/M&amp;P/propulsion internship search</v>
+      </c>
+      <c r="C186" t="str">
+        <v>2026-09-22 ~13:00 UTC: only Summer 2026 internships found (10-week program, San Jose HQ). No Spring 2027/Winter 2026 postings found.</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>Firefly Aerospace</v>
+      </c>
+      <c r="B187" t="str">
+        <v>hrmdirect careers board, full sweep</v>
+      </c>
+      <c r="C187" t="str">
+        <v>2026-09-22 ~13:00 UTC: only Spring 2026 (Mechanical, Software, Test — already past relative to today) and Summer 2026 (Propulsion, Launch Site) reqs found. No Winter 2026 or Spring 2027 postings found.</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B188" t="str">
+        <v>'2027 Mechanical Engineer Intern' (multiple sites referenced incl. Boston, MA, Atlanta, Costa Mesa, Irvine, Reston, Seattle)</v>
+      </c>
+      <c r="C188" t="str">
+        <v>2026-09-22 ~13:00 UTC: referenced in search results but no live posting URL could be located/opened, and no season (Spring vs Summer) could be confirmed from available snippets. Not added — couldn't verify. Worth a follow-up given the Boston, MA site reference.</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>Redwire Space</v>
+      </c>
+      <c r="B189" t="str">
+        <v>'Mechanical Engineering Intern (Year Round)', Albuquerque NM</v>
+      </c>
+      <c r="C189" t="str">
+        <v>2026-09-22 ~13:00 UTC: direct fetch of the posting URL returns HTTP 404 'Page not found' despite a stale page title suggesting the role once existed. Confirmed dead/removed.</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>Virgin Galactic</v>
+      </c>
+      <c r="B190" t="str">
+        <v>Internship program, full sweep</v>
+      </c>
+      <c r="C190" t="str">
+        <v>2026-09-22 ~13:00 UTC: internship program is summer-only (May-September, 12 weeks). No Winter 2026/Spring 2027 postings found.</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>ispace</v>
+      </c>
+      <c r="B191" t="str">
+        <v>Internship search</v>
+      </c>
+      <c r="C191" t="str">
+        <v>2026-09-22 ~13:00 UTC: no current Spring 2027/Winter 2026 postings found; most recent indexed internship reference was from 2024.</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>Textron Systems</v>
+      </c>
+      <c r="B192" t="str">
+        <v>'2027 Intern - Mechanical Engineer (Sea Systems)', Hunt Valley MD</v>
+      </c>
+      <c r="C192" t="str">
+        <v>2026-09-22 ~13:00 UTC: referenced in search-engine descriptions but careers.textron.com is JS-rendered and blocked direct fetch, and no season (Spring vs Summer) is stated in any snippet found. Not included — couldn't verify season or find a live link.</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>Bell Textron</v>
+      </c>
+      <c r="B193" t="str">
+        <v>Mechanical engineering intern search</v>
+      </c>
+      <c r="C193" t="str">
+        <v>2026-09-22 ~13:00 UTC: only '2027 Summer Intern - Mechanical Engineering', Fort Worth TX found — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>General Atomics</v>
+      </c>
+      <c r="B194" t="str">
+        <v>Internship program, full sweep</v>
+      </c>
+      <c r="C194" t="str">
+        <v>2026-09-22 ~13:00 UTC: only a summer program (10 weeks, June-August) referenced across all sources. No Winter 2026/Spring 2027 postings found.</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Kratos Defense</v>
+      </c>
+      <c r="B195" t="str">
+        <v>Mechanical engineering intern search</v>
+      </c>
+      <c r="C195" t="str">
+        <v>2026-09-22 ~13:00 UTC: no season-specific (Spring 2027/Winter 2026) mechanical postings found; only generic 'Engineering Intern'/'Mechanical Engineering Intern' listings without term dates.</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Pratt &amp; Whitney (RTX)</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Fresh sweep beyond already-tracked Middletown CT co-op</v>
+      </c>
+      <c r="C196" t="str">
+        <v>2026-09-22 ~13:00 UTC: found Summer 2027 mechanical reqs (wrong season) and a Fall 2026 co-op; no additional Spring 2027/Winter 2026 mechanical posting found distinct from the already-tracked Production Support Engineering Co-op (Middletown, CT).</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Aerojet Rocketdyne (L3Harris)</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Internship program search</v>
+      </c>
+      <c r="C197" t="str">
+        <v>2026-09-22 ~13:00 UTC: only generic Summer internship program info found; no live Spring 2027/Winter 2026 posting located. Search suggests fall/spring applications may open in August with a November deadline, but no live req found today.</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>BETA Technologies</v>
+      </c>
+      <c r="B198" t="str">
+        <v>'2026-2027 BETA Internship' (Mechanical Engineering track among others), South Burlington VT</v>
+      </c>
+      <c r="C198" t="str">
+        <v>2026-09-22 ~13:00 UTC: confirmed live (HTTP 200, JobPosting schema present) via direct fetch — a single rolling application covering the whole 2026-2027 cycle across all disciplines/seasons, applicant selects preferred focus area after applying. Posting text itself does not state a specific Winter 2026/Spring 2027 term, so it fails the season-stated verification bar. Flagged as Hamza's own judgment call, same treatment as Caterpillar's/Saab's ambiguous-term postings — not added to `rows`. Closest new candidate this run geographically (~215 mi from Boston).</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>Sierra Space</v>
+      </c>
+      <c r="B199" t="str">
+        <v>Live Workday API query, re-check</v>
+      </c>
+      <c r="C199" t="str">
+        <v>2026-09-22 ~13:00 UTC: queried Sierra Space's own Workday API directly — zero postings contain 'Spring 2027' in the title, and a broad 'Mechanical Engineering Intern' search returns 32 results, all full-time 'Regular' roles, zero interns/co-ops of any kind currently posted. More conclusive than prior 'no dated req found' note; company's stated Sept-post/Dec-deadline pattern has not materialized as of today.</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B200" t="str">
+        <v>Spring 2027 co-op search, re-check</v>
+      </c>
+      <c r="C200" t="str">
+        <v>2026-09-22 ~13:00 UTC: still nothing live for Spring 2027 despite the company's own stated Sept-Oct posting-window claim — now the 6th consecutive checked run this claim has failed to materialize. Confidence in the claim downgraded; still worth one more pass through end of October before treating it as unreliable this cycle.</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B201" t="str">
+        <v>Mechanical Engineering Co-Op listing, re-check</v>
+      </c>
+      <c r="C201" t="str">
+        <v>2026-09-22 ~13:00 UTC: the listing found via search is a stale, INACTIVE Spring 2025 posting in Burlington, MA (confirmed via direct fetch), not a current Spring 2027 posting. Still 'not posted yet' for the 2027 cycle.</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B202" t="str">
+        <v>Mechanical engineering co-op search, re-check</v>
+      </c>
+      <c r="C202" t="str">
+        <v>2026-09-22 ~13:00 UTC: no Spring 2027 mechanical posting found. Still not posted.</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>Cognex (Natick, MA)</v>
+      </c>
+      <c r="B203" t="str">
+        <v>Live Workday API query for all 'Intern (Fixed Term)' worker-type reqs company-wide, re-check</v>
+      </c>
+      <c r="C203" t="str">
+        <v>2026-09-22 ~13:00 UTC: the only such req company-wide is a Mechanical Engineering Intern in Aachen, Germany — zero internship/co-op postings in Natick, MA. More conclusive than the prior discipline-mismatch-only note; now also a location mismatch.</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>MKS Instruments (Andover, MA) / Raytheon BBN Technologies (Cambridge, MA) / CIRCOR International / Vecna Robotics (Waltham, MA) / Locus Robotics (Wilmington, MA) / National Grid</v>
+      </c>
+      <c r="B204" t="str">
+        <v>Fresh sweep, mechanical/aerospace/manufacturing/robotics intern/co-op search</v>
+      </c>
+      <c r="C204" t="str">
+        <v>2026-09-22 ~13:00 UTC: no qualifying Spring 2027/Winter 2026 postings found at any of these. MKS Instruments' Workday API returned inconsistent 400s mid-run (likely rate-limiting) — worth a clean recheck next run rather than treated as conclusive. CIRCOR only has a UK-based internship. Vecna Robotics, Locus Robotics, and National Grid currently have no internship/co-op postings of any kind.</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B205" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check</v>
+      </c>
+      <c r="C205" t="str">
+        <v>2026-09-22 ~13:00 UTC: careers site returned HTTP 503 'Technical Difficulties' on 3 separate attempts again this run — could not verify live/open status. Unresolved across multiple runs now; worth prioritizing a fresh attempt next run since this is the first non-discipline-mismatch mechanical lead found at this employer.</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>PI Physik Instrumente (Shrewsbury, MA)</v>
+      </c>
+      <c r="B206" t="str">
+        <v>'Mechanical Engineering Internship – Winter/Spring 2026'</v>
+      </c>
+      <c r="C206" t="str">
+        <v>2026-09-22 ~13:00 UTC: NEW COMPANY found this run. Confirmed live ($24-26/hr) via direct fetch, but this posting is for the Jan-June 2026 cohort, which has already elapsed as of today (2026-09-22) — wrong season for a forward-looking search. Worth rechecking in coming weeks for a fresh Winter 2026/Spring 2027-labeled cycle; note their naming convention may label the already-past Jan 2026 term as 'Winter 2026', which could cause confusion on the next check.</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B207" t="str">
+        <v>'Application Engineering Co-Op' (REQ-14473); Digital Operations, EHS, and Analytical/Metrology/Microanalysis Scientist Co-Ops, all Spring 2027, Billerica MA</v>
+      </c>
+      <c r="C207" t="str">
+        <v>2026-09-22 ~13:00 UTC: Application Engineering Co-Op is Photo Applications/semiconductor chemistry — discipline mismatch. The others are non-mechanical/non-target disciplines (digital/EHS/analytical science). Excluded. (5 other Entegris Spring 2027 co-ops at the same site DID qualify and were added to `rows`.)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C182"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C207"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 30 checked-excluded (2026-09-22 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KWZt3U5TY1xB8LJg83Hp1f
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -3094,7 +3094,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C207"/>
+  <dimension ref="A1:C237"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -5378,9 +5378,339 @@
         <v>2026-09-22 ~13:00 UTC: Application Engineering Co-Op is Photo Applications/semiconductor chemistry — discipline mismatch. The others are non-mechanical/non-target disciplines (digital/EHS/analytical science). Excluded. (5 other Entegris Spring 2027 co-ops at the same site DID qualify and were added to `rows`.)</v>
       </c>
     </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>Moog Inc. — Intern, Mechanical Analysis Engineering (R-26-20226)</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Elma/Buffalo, NY, Space &amp; Defense Group</v>
+      </c>
+      <c r="C208" t="str">
+        <v>2026-09-22 ~19:00 UTC: confirmed live/open via direct Workday CXS fetch ($25.50-31.00/hr, GPA 3.0+, US export-control access required), but the posting text itself only says it is 'seeking a spring block intern' with no year stated anywhere in the description — fails the season-stated verification bar despite being open. Not added; worth a follow-up if a dated version appears.</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>Moog Inc. — Intern, Test Engineering (R-26-20243-1)</v>
+      </c>
+      <c r="B209" t="str">
+        <v>Elma/Buffalo, NY, Military Aircraft Group</v>
+      </c>
+      <c r="C209" t="str">
+        <v>2026-09-22 ~19:00 UTC: confirmed live/open via direct Workday CXS fetch ($25.50-31.00/hr), but the posting explicitly states 'spring/summer 2027 block intern' — a combined Spring+Summer term, same treatment as Saab's 'Spring - Summer 2027' posting. Flagged as Hamza's own judgment call on borderline combined-term postings, not added to `rows`.</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>Curtiss-Wright (Cheswick, PA)</v>
+      </c>
+      <c r="B210" t="str">
+        <v>JR1907 'Co-op (Spring Term)' — re-check #4; also JR7519-1 'Engineering-Intern' and JR8729 'Round Rock Nuclear Engineering Co-Op'</v>
+      </c>
+      <c r="C210" t="str">
+        <v>2026-09-22 ~19:00 UTC: re-fetched JR1907 directly via Workday CXS API — text is unchanged and confirms it is an evergreen posting for 'Spring, Summer and Fall semesters' with no year ever stated; 4th consecutive run with no change, structurally unlikely to ever resolve automatically (recommend deprioritizing further automated re-checks, same treatment as GD Electric Boat). Separately, JR7519-1 and JR8729 both confirmed closed via Workday `postingAvailable: false`.</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B211" t="str">
+        <v>Re-check of already-tracked Engines Engineering Co-op (R5029617-1, Evendale/Lynn); Lynn, MA-only reqs</v>
+      </c>
+      <c r="C211" t="str">
+        <v>2026-09-22 ~19:00 UTC: verified via direct Workday CXS API fetch that the already-tracked R5029617-1 remains live and open — full job description returned, no change to `rows`. A sibling req without the '-1' suffix and a separate Manufacturing Eng Co-op (R5030077) are HTTP 410 Gone, but these were never the tracked req. Only other Lynn-specific reqs remain the Carpentry/CNC Trainee Co-Ops — discipline mismatch, unchanged.</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B212" t="str">
+        <v>Spring 2027 co-op search, re-check #7</v>
+      </c>
+      <c r="C212" t="str">
+        <v>2026-09-22 ~19:00 UTC: only live co-ops are 'Fall 2026 Designer Co-op' (Newport News) and 'Student Coop Educ O/S' (Pascagoula, MS) — still zero Spring 2027 postings, 7th consecutive checked run the company's own Sept-Oct posting-window claim has failed to materialize.</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>Sierra Space</v>
+      </c>
+      <c r="B213" t="str">
+        <v>Live Workday API query, re-check #3</v>
+      </c>
+      <c r="C213" t="str">
+        <v>2026-09-22 ~19:00 UTC: queried Sierra Space's own Workday API directly (47 open reqs) — `workerSubType` facet shows only 'Regular' and 'Contract Labor', zero intern/co-op category postings exist company-wide. Confirmed still zero, no change.</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>MKS Instruments (Andover, MA)</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Live Workday API query, clean re-check (not rate-limited this time)</v>
+      </c>
+      <c r="C214" t="str">
+        <v>2026-09-22 ~19:00 UTC: queried the MKSCareersUniversity Workday API directly, clean 200 response — only 12 total open reqs company-wide, none in Andover/MA, none mechanical, none intern/co-op in the US. The previously-seen Fall 2026 reqs (R19858, R14406) have closed.</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Live Workday API query</v>
+      </c>
+      <c r="C215" t="str">
+        <v>2026-09-22 ~19:00 UTC: queried their Workday API directly (37 open reqs) — `workerSubType` facet is 100% 'Regular', zero current intern/co-op postings exist, despite an older cached 'Mechanical Engineering Intern R2495' URL circulating in search results (stale/expired).</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>Cognex (Natick, MA)</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Live Workday API query, re-check</v>
+      </c>
+      <c r="C216" t="str">
+        <v>2026-09-22 ~19:00 UTC: queried their Workday API directly (102 open reqs, 21 in the US) — no mechanical engineering intern/co-op req exists at all now; only Development Programs and a non-intern Quality Engineer role in MA. Updates prior 'only a Germany req' note — now zero relevant US reqs of any kind.</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>Teradyne (North Reading, MA)</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Internships/co-ops listing page, re-check</v>
+      </c>
+      <c r="C217" t="str">
+        <v>2026-09-22 ~19:00 UTC: current North Reading postings are Optical Systems Engineer, Hardware Engineer, NPI Manufacturing Engineer, Optical Engineer — no mechanical-specific, no Spring 2027-labeled co-op. The Spring 2026 mechanical co-op found previously is a past cycle, already closed.</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>Vicarious Surgical (Waltham, MA)</v>
+      </c>
+      <c r="B218" t="str">
+        <v>Mechanical Engineering Co-Op (Jan 2026 start)</v>
+      </c>
+      <c r="C218" t="str">
+        <v>2026-09-22 ~19:00 UTC: fetched the posting directly — 'This job is no longer accepting applications.' Season would have qualified but the posting is now closed.</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>Commonwealth Fusion Systems (Devens, MA)</v>
+      </c>
+      <c r="B219" t="str">
+        <v>Lever API query, re-check</v>
+      </c>
+      <c r="C219" t="str">
+        <v>2026-09-22 ~19:00 UTC: queried their Lever board API directly — the previously-referenced Fall Co-op 2026 posting now returns 404; several full-time Mechanical Engineer reqs exist but no active intern/co-op listing, nothing for Spring 2027.</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>PI Physik Instrumente (Shrewsbury, MA)</v>
+      </c>
+      <c r="B220" t="str">
+        <v>Re-check for a fresh Spring 2027-labeled cycle</v>
+      </c>
+      <c r="C220" t="str">
+        <v>2026-09-22 ~19:00 UTC: only the already-elapsed Jan-June 2026 cohort posting still exists. No fresh Spring 2027-labeled posting found yet.</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B221" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check #4</v>
+      </c>
+      <c r="C221" t="str">
+        <v>2026-09-22 ~19:00 UTC: na.careers.hologic.com and careers.hologic.com both returned HTTP 503 'Technical Difficulties' again on two separate direct-curl attempts with different UAs. Aggregator mirrors (Hologic's own domain in the search index, LinkedIn, ZipRecruiter) continue to consistently describe Jan-June 2026, $26-28/hr, Marlborough MA onsite, ≥1 semester remaining requirement — but season still cannot be confirmed from the posting itself per the verification bar since the page won't load. Remains unresolved across 4 runs now; still not added to `rows`.</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>Boeing</v>
+      </c>
+      <c r="B222" t="str">
+        <v>Full internship listing sweep, incl. 'Drexel Internship 2026', 'BSC Co-op Specialty Program', 'Manufacturing Operations Internship Program'</v>
+      </c>
+      <c r="C222" t="str">
+        <v>2026-09-22 ~19:00 UTC: all live internship postings are Summer 2026/Summer 2027 cohort-labeled; the non-seasonal-named reqs listed all confirmed closed via Workday `postingAvailable: false`. No Winter/Spring-specific mechanical/structural req found.</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>Joby Aviation</v>
+      </c>
+      <c r="B223" t="str">
+        <v>Mechanical Design Engineer Intern (Structures); Mechanical Engineer Intern (Hydrogen Powertrain)</v>
+      </c>
+      <c r="C223" t="str">
+        <v>2026-09-22 ~19:00 UTC: both now confirmed HTTP 410 Gone (closed/expired), same as the already-noted Flight Test Intern req. No live Joby posting found in target disciplines/season.</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>BAE Systems (Cedar Rapids, IA)</v>
+      </c>
+      <c r="B224" t="str">
+        <v>'2027 Spring and Summer Mechanical Engineering Coop' (125975BR); 'Operations Engineering (Ind/Mech/Elec) Co-op Spring/Summer 2027' (126541BR)</v>
+      </c>
+      <c r="C224" t="str">
+        <v>2026-09-22 ~19:00 UTC: both confirmed 'no longer accepting applications' on jobs.baesystems.com — filled/closed.</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>Moog Inc. (Mineral Wells, TX)</v>
+      </c>
+      <c r="B225" t="str">
+        <v>'Air Vehicle Engineering'/Design/Hardware Design interns (R-26-19881/19882/19186/19887)</v>
+      </c>
+      <c r="C225" t="str">
+        <v>2026-09-22 ~19:00 UTC: all explicitly stated as Summer 2027 block interns in their posting text — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>Pratt &amp; Whitney (RTX)</v>
+      </c>
+      <c r="B226" t="str">
+        <v>Mechanical Engineering Internship (Summer 2027, Marlborough MA); 'Winter 2026 Continuous Improvement Engineering'; 'Winter 2027 Aerospace Manufacturing &amp; CI'</v>
+      </c>
+      <c r="C226" t="str">
+        <v>2026-09-22 ~19:00 UTC: the Marlborough MA req is explicitly Summer 2027 — wrong season. The two 'Winter' reqs are both at Pratt &amp; Whitney Canada (Enfield, Nova Scotia) — wrong country, and the 2027 one is also wrong season regardless.</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>Woodward / Spirit AeroSystems / Bell Textron / Textron Aviation / General Atomics / Virgin Galactic / Archer Aviation</v>
+      </c>
+      <c r="B227" t="str">
+        <v>Full internship sweep, each company</v>
+      </c>
+      <c r="C227" t="str">
+        <v>2026-09-22 ~19:00 UTC: each company's current live/discoverable internship postings are Summer 2026/2027 cohort only (Woodward also has a Poland-based internship, not US). No Winter 2026/Spring 2027 posting found at any of these.</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>Lockheed Martin (incl. Sikorsky, RMS)</v>
+      </c>
+      <c r="B228" t="str">
+        <v>Previously-located job URLs: Moorestown, Severn, Fort Worth Mechanical Engineer Intern; Mount Laurel Systems Engineer Modeling &amp; Simulation Intern</v>
+      </c>
+      <c r="C228" t="str">
+        <v>2026-09-22 ~19:00 UTC: all now return lockheedmartin.com/en-us/404.html — closed/moved. No new live Winter/Spring req located to replace them.</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>L3Harris</v>
+      </c>
+      <c r="B229" t="str">
+        <v>Palm Bay Mechanical Engineer Intern; Spring 2027 Software Engineer req</v>
+      </c>
+      <c r="C229" t="str">
+        <v>2026-09-22 ~19:00 UTC: the Mechanical Engineer Intern posting is confirmed live but explicitly 'for the summer' — wrong season. The only Spring 2027-dated req found is Software Engineer — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>Shield AI / Saildrone / Firefly Aerospace / Redwire Space / Aerojet Rocketdyne / Aurora Flight Sciences / Safran USA / Parker Hannifin / Honeywell Aerospace / Kratos Defense</v>
+      </c>
+      <c r="B230" t="str">
+        <v>Full internship sweep, each company</v>
+      </c>
+      <c r="C230" t="str">
+        <v>2026-09-22 ~19:00 UTC: no verifiable Winter 2026/Spring 2027 posting found at any of these this run. Several career sites blocked verification outright (Safran 403'd; General Atomics/Parker decentralized sites not crawlable) — treated as unresolved rather than conclusively ruled out, worth a follow-up with a more direct access method.</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="str">
+        <v>Northrop Grumman (Chandler, AZ)</v>
+      </c>
+      <c r="B231" t="str">
+        <v>'2027 Spring Mechanical Engineering Co-op', Space Systems Sector</v>
+      </c>
+      <c r="C231" t="str">
+        <v>2026-09-22 ~19:00 UTC: multiple consistent aggregator mirrors (Dreamwork, Zapply, Workopia) plus a direct web search describe the role as full-time 'Spring and Summer semester (January-August 2027)' — a combined Spring+Summer term, not a clean Spring-only co-op, same treatment as Saab's/Moog's combined-term postings. Additionally, Northrop's own Eightfold-based career site blocks unauthenticated API access ('Not authorized for PCSX'), so no canonical jobs.northropgrumman.com URL could be independently verified. Excluded on both season-ambiguity and unverifiable-link grounds; flagged as a borderline judgment call for Hamza.</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B232" t="str">
+        <v>'Co-op Design Engineering (Spring 2027)'</v>
+      </c>
+      <c r="C232" t="str">
+        <v>2026-09-22 ~19:00 UTC: found only via Fairygodboss/LinkedIn mirrors; Eaton's eightfold.ai career site blocks verification the same way as Northrop Grumman's. Season/location line up but live/open status is unverified. Not added — worth a follow-up with a different access method.</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>Leidos</v>
+      </c>
+      <c r="B233" t="str">
+        <v>Mechanical Engineer Intern reqs (Remote-US / Long Beach, MS)</v>
+      </c>
+      <c r="C233" t="str">
+        <v>2026-09-22 ~19:00 UTC: careers.leidos.com returned HTTP 403 to both direct fetch and curl (Cloudflare-style block); season not confirmed — Leidos's active wave is labeled generically 'Summer 2027'/'Spring/Fall 2027'. Not added — unresolved.</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>Textron Systems</v>
+      </c>
+      <c r="B234" t="str">
+        <v>'2027 Industrial Engineer Intern' (req 343102)</v>
+      </c>
+      <c r="C234" t="str">
+        <v>2026-09-22 ~19:00 UTC: title confirmed real via og:title metadata, but the full description (incl. season) is JS-rendered and inaccessible; Textron's plain '2027 Intern' naming convention elsewhere corresponds to the Summer cohort, so this is ambiguous season, not confirmed as Winter/Spring. Not added.</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B235" t="str">
+        <v>'Intern - Hardware Engineer' (R5394), re-check</v>
+      </c>
+      <c r="C235" t="str">
+        <v>2026-09-22 ~19:00 UTC: this req shows up in SmartRecruiters/Workday-mirror search snippets but direct Workday API calls to their tenant returned 422 errors (likely wrong site slug); could not independently confirm it's currently live or its season. Unresolved, worth a direct retry with a corrected tenant path next run.</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B236" t="str">
+        <v>'2027 Mechanical Engineer Intern' (Boston, MA reference), re-check</v>
+      </c>
+      <c r="C236" t="str">
+        <v>2026-09-22 ~19:00 UTC: relativityspace.com/internship-positions loaded but returned only header/nav content with no visible listings; their dedicated Greenhouse board (job-boards.greenhouse.io/rsinternboard) currently only has a '2026 Summer Internship' posting. The specific 2027 ME intern req referenced by mirror sites could not be independently verified or resolved to a real Greenhouse/Ashby ID. Still unresolved — worth trying the Greenhouse API with different filters or checking if Relativity uses Ashby instead.</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B237" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C237" t="str">
+        <v>2026-09-22 ~19:00 UTC: no change — still nothing posted for the 2027 cycle at either company.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C237"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 17 new postings, 34 checked-excluded, 1 upgraded Partial->Yes (2026-09-23 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VeXPGMHph9Espwetnvk1is
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J101"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1927,7 +1927,7 @@
         <v>https://www.zipline.com/open-roles/7865253003?gh_jid=7865253003</v>
       </c>
       <c r="I48" t="str">
-        <v>Partial — fetched directly, confirmed exact title and 'Spring 2027' wording on the page, but page is JS-rendered so Apply-button/open status could not be independently confirmed from the fetch alone. Corroborated as currently listed by two other independent sources (2026-09-20).</v>
+        <v>Yes — upgraded 2026-09-23: confirmed directly via Zipline's own Greenhouse API (job-boards.greenhouse.io/flyzipline/jobs/7865253003), HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J48" t="str">
         <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
@@ -3085,16 +3085,560 @@
         <v>Distinct req from the already-tracked undergrad-oriented 'Spring 2027 Engineering Internship/Co-op' (job 8616338002) — THIS req explicitly requires the applicant to already hold a bachelor's degree AND be currently enrolled in a graduate program. Only relevant if Hamza is in/entering grad school by Spring 2027. US citizen/permanent resident/refugee/asylee required (ITAR).</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Manufacturing Engineering Co-op – US – Spring 2027</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Lynn, MA (one of 23 eligible US locations)</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85" t="str">
+        <v>Starts at $20/hr, increases per undergrad class year</v>
+      </c>
+      <c r="H85" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Evendale/Manufacturing-Engineering-Co-op---US---Spring-2027_R5029663</v>
+      </c>
+      <c r="I85" t="str">
+        <v>Yes — fetched directly via GE's Workday CXS job API, full description confirmed, canApply true, application end date 2026-11-06.</v>
+      </c>
+      <c r="J85" t="str">
+        <v>Sibling req to the already-tracked Engines Engineering Co-op (R5029617-1) at the same Lynn, MA site — distinct req ID, not a duplicate. Excludes 'Returning Students' variants (require a prior GE Aerospace internship).</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>PI (Physik Instrumente)</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Shrewsbury, MA</v>
+      </c>
+      <c r="F86">
+        <v>40</v>
+      </c>
+      <c r="G86" t="str">
+        <v>$24–26/hr</v>
+      </c>
+      <c r="H86" t="str">
+        <v>https://www.physikinstrumente.com/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+      </c>
+      <c r="I86" t="str">
+        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
+      </c>
+      <c r="J86" t="str">
+        <v>Boston metro (Shrewsbury). Fresh cycle superseding the already-past Jan-June 2026 cohort found at this same company in prior runs. Requires legal US work authorization without sponsorship; SolidWorks preferred.</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>PI (Physik Instrumente)</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Manufacturing Engineering Internship</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Shrewsbury, MA</v>
+      </c>
+      <c r="F87">
+        <v>40</v>
+      </c>
+      <c r="G87" t="str">
+        <v>$24–26/hr</v>
+      </c>
+      <c r="H87" t="str">
+        <v>https://www.physikinstrumente.com/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
+      </c>
+      <c r="I87" t="str">
+        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
+      </c>
+      <c r="J87" t="str">
+        <v>Boston metro (Shrewsbury). Same batch/cycle as the Mechanical Engineering Co-op above.</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B88" t="str">
+        <v>CAD Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Mechanical Design / CAD Engineering</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E88" t="str">
+        <v>San Francisco, CA</v>
+      </c>
+      <c r="F88">
+        <v>2700</v>
+      </c>
+      <c r="G88" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H88" t="str">
+        <v>https://job-boards.greenhouse.io/astranis/jobs/4704740006</v>
+      </c>
+      <c r="I88" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live, 'Spring 2027' stated on posting.</v>
+      </c>
+      <c r="J88" t="str">
+        <v>Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 4704602006) at the same company. Satellite manufacturer — worth double-checking ITAR/citizenship requirements before applying, not explicit in the excerpt reviewed. Distinct from Astranis's separate 'Winter 2027' reqs, which remain excluded (see `checked`) for season mismatch.</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Rockford, IL</v>
+      </c>
+      <c r="F89">
+        <v>900</v>
+      </c>
+      <c r="G89" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H89" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IL-ROCKFORD-P6--4747-Harrison-Ave--4747-HARRISON-AVE-P6/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869227</v>
+      </c>
+      <c r="I89" t="str">
+        <v>Yes — fetched directly via RTX's own Workday CXS API (browser UA + Referer), full description confirmed, posted 2026-09-22.</v>
+      </c>
+      <c r="J89" t="str">
+        <v>Distinct req/site from the already-tracked Jamestown ND and Cedar Rapids IA Collins Aerospace co-ops — not a duplicate.</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>L3Harris</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Mechanical Engineer Intern - Spring 2027</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Spring 2027 (Jan–Jul 2027)</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Greenville, TX</v>
+      </c>
+      <c r="F90">
+        <v>1500</v>
+      </c>
+      <c r="G90" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H90" t="str">
+        <v>https://careers.l3harris.com/en/job/greenville/mechanical-engineer-intern-spring-2027/4832/99372978208</v>
+      </c>
+      <c r="I90" t="str">
+        <v>Yes — fetched directly, page live, 'Apply Now' present, 'Spring 2027' stated on posting (no 'summer' wording found, unlike a differently-worded/now-dead L3Harris Greenville req excluded in a prior run).</v>
+      </c>
+      <c r="J90" t="str">
+        <v>Degree requirement: Mechanical/Aerospace/Engineering Mechanics/Materials Science. US citizenship required for clearance eligibility. Job ID 41322.</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Winter 2027 Propulsion Engineer Co-op</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Mechanical / Propulsion Engineering</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Winter 2027 (effectively Jan–Aug 2027, same calendar window as other employers' 'Spring 2027')</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Costa Mesa, CA</v>
+      </c>
+      <c r="F91">
+        <v>2600</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H91" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236587007</v>
+      </c>
+      <c r="I91" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
+      </c>
+      <c r="J91" t="str">
+        <v>US citizenship required, no clearance required. New site beyond the already-tracked Quincy, MA / Lexington, MA Anduril Winter 2027 co-ops.</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Winter 2027 Warhead Engineer Co-op</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Mechanical Engineering (ordnance/warhead design)</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Costa Mesa, CA</v>
+      </c>
+      <c r="F92">
+        <v>2600</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H92" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236585007</v>
+      </c>
+      <c r="I92" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
+      </c>
+      <c r="J92" t="str">
+        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Test &amp; Evaluation Engineer Co-ops above.</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Winter 2027 Test &amp; Evaluation Engineer Co-op</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Systems / Test Engineering</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Costa Mesa, CA</v>
+      </c>
+      <c r="F93">
+        <v>2600</v>
+      </c>
+      <c r="G93" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H93" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236583007</v>
+      </c>
+      <c r="I93" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
+      </c>
+      <c r="J93" t="str">
+        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Warhead Engineer Co-ops above.</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Aerodynamics Intern (Spring 2027)</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Aerospace / Aerodynamics Engineering</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E94" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F94">
+        <v>2700</v>
+      </c>
+      <c r="G94" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H94" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904002003</v>
+      </c>
+      <c r="I94" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J94" t="str">
+        <v>Autonomous drone delivery company. Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 7865253003) at the same company.</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Civil and Structural Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E95" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F95">
+        <v>2700</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H95" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904457003</v>
+      </c>
+      <c r="I95" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J95" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Controls Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Controls Engineering</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E96" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F96">
+        <v>2700</v>
+      </c>
+      <c r="G96" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H96" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7903823003</v>
+      </c>
+      <c r="I96" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J96" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Flight Test Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Flight Systems / Test Engineering</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E97" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F97">
+        <v>2700</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H97" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7999929003</v>
+      </c>
+      <c r="I97" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J97" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Hardware Test Intern (Spring 2027)</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Mechanical / Hardware Test Engineering</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E98" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F98">
+        <v>2700</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H98" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7894349003</v>
+      </c>
+      <c r="I98" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J98" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Maintenance Tool Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Mechanical / Tooling Engineering</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Esparto, CA</v>
+      </c>
+      <c r="F99">
+        <v>2800</v>
+      </c>
+      <c r="G99" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H99" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7909945003</v>
+      </c>
+      <c r="I99" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J99" t="str">
+        <v>Borderline discipline fit (maintenance tooling) — included per Hamza's own judgment call, similar treatment to other borderline robotics/manufacturing-adjacent reqs in this tracker.</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Quality &amp; Manufacturing Intern (Spring 2027)</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Manufacturing / Quality Engineering</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E100" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F100">
+        <v>2700</v>
+      </c>
+      <c r="G100" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H100" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7824311003</v>
+      </c>
+      <c r="I100" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J100" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Supplier Industrialization Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Manufacturing / Industrial Engineering</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E101" t="str">
+        <v>South San Francisco, CA</v>
+      </c>
+      <c r="F101">
+        <v>2700</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H101" t="str">
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7891019003</v>
+      </c>
+      <c r="I101" t="str">
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+      </c>
+      <c r="J101" t="str">
+        <v>Same batch as the other new Zipline reqs added this run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J101"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C237"/>
+  <dimension ref="A1:C271"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -5708,9 +6252,383 @@
         <v>2026-09-22 ~19:00 UTC: no change — still nothing posted for the 2027 cycle at either company.</v>
       </c>
     </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B238" t="str">
+        <v>req 601496955, re-check</v>
+      </c>
+      <c r="C238" t="str">
+        <v>2026-09-23 ~01:00 UTC: still Cloudflare-blocked (13th consecutive run). Confirmed the ATS is not the guessed gdeb.wd5.myworkdayjobs.com tenant (422); ebcareers.com and gd.com/careers/job-search both return no usable result for this req. Needs a human in-browser check; automated attempts deprioritized further per standing guidance.</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B239" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check</v>
+      </c>
+      <c r="C239" t="str">
+        <v>2026-09-23 ~01:00 UTC: 5th consecutive 503 on direct fetch (multiple UAs tried). Partial corroboration only via LinkedIn/ZipRecruiter mirrors (req 300000421584867): 'January – June 2026' — this is actually a Winter 2026 season match, not yet independently confirmed live. Remains the strongest unconfirmed Boston-area lead; worth a fresh attempt at a different time/network path.</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B240" t="str">
+        <v>Electrical Engineering Co-Op (Spring 2027), JR002941 — new req found this run</v>
+      </c>
+      <c r="C240" t="str">
+        <v>2026-09-23 ~01:00 UTC: confirmed live via direct Workday CXS API fetch (posted today), but electrical engineering is outside Hamza's target disciplines — same treatment as the already-excluded JR002884/JR002885 Draper electrical/optics reqs. Not added.</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B241" t="str">
+        <v>CAD Engineer Intern (Winter 2027), Mechanical Engineer Intern (Winter 2027), Environmental Test Engineer Intern (Winter 2027), Hardware Test Intern (Winter 2027), Assembly/Integration/Test Intern (Winter 2027), Propulsion Manufacturing Intern (Winter 2027), Production Quality Intern (Winter 2027)</v>
+      </c>
+      <c r="C241" t="str">
+        <v>2026-09-23 ~01:00 UTC: all confirmed live but season is literally 'Winter 2027' (not Winter 2026 or Spring 2027) — same exclusion basis as the already-excluded Astranis Mechanical Engineer Intern (Winter 2027) from prior runs. The sibling 'Spring 2027'-titled CAD Engineer Intern and Mechanical Engineer Intern reqs from the same batch DID qualify and were added to `rows`.</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B242" t="str">
+        <v>Materials Engineer Intern (Spring &amp; Summer 2027)</v>
+      </c>
+      <c r="C242" t="str">
+        <v>2026-09-23 ~01:00 UTC: confirmed live via direct Greenhouse API fetch, but stated as a combined 'Spring &amp; Summer 2027' term — excluded per the same combined-term precedent as Saab/Moog/Northrop Grumman Chandler. The rest of this Zipline batch (pure 'Spring 2027' reqs) qualified and were added to `rows`.</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>Curtiss-Wright (Cheswick, PA)</v>
+      </c>
+      <c r="B243" t="str">
+        <v>JR1907, re-check</v>
+      </c>
+      <c r="C243" t="str">
+        <v>2026-09-23 ~01:00 UTC: re-fetched via Workday API directly — identical evergreen 'Co-op (Spring Term)' text, stale startDate field (2025-02-07), no year ever stated. 5th consecutive run with no change; recommend no further automated re-checks unless a differently-worded/dated version appears.</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>Northrop Grumman (Chandler, AZ)</v>
+      </c>
+      <c r="B244" t="str">
+        <v>'2027 Spring Mechanical Engineering Co-op', re-check</v>
+      </c>
+      <c r="C244" t="str">
+        <v>2026-09-23 ~01:00 UTC: no change — still the combined 'Spring and Summer semester (January-August 2027)' term, still no independently-verifiable canonical URL. Unchanged judgment-call item for Hamza.</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B245" t="str">
+        <v>'Co-op Design Engineering (Spring 2027)', re-check</v>
+      </c>
+      <c r="C245" t="str">
+        <v>2026-09-23 ~01:00 UTC: the specific Fairygodboss link from the prior run now 404s. Only a Summer 2027 version of this same co-op is currently confirmable live on LinkedIn — wrong season. A LinkedIn-only reference to a 'Co-op: Manufacturing Engineering (Spring 2027)' could not be independently opened/verified. Excluded — no verifiable live Spring 2027 posting.</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>Leidos</v>
+      </c>
+      <c r="B246" t="str">
+        <v>Mechanical Engineer Intern reqs, re-check</v>
+      </c>
+      <c r="C246" t="str">
+        <v>2026-09-23 ~01:00 UTC: no live Spring 2027 mechanical-specific requisition found; only software/systems Spring 2027 reqs currently posted. No change from prior 403-blocked status.</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B247" t="str">
+        <v>'Intern - Hardware Engineer' (R5394), re-check with corrected tenant slugs</v>
+      </c>
+      <c r="C247" t="str">
+        <v>2026-09-23 ~01:00 UTC: tried symbotic/Symbotic, symbotic/Symbotic_Careers, and a wd504 host variant — all return 422 or the direct job page returns 500. Still blocked; season remains unconfirmed.</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>Moog Inc. (Buffalo, NY)</v>
+      </c>
+      <c r="B248" t="str">
+        <v>'Intern, Mechanical Analysis Engineering' (R-26-20226), 'Intern, Test Engineering' (R-26-20243-1), re-check</v>
+      </c>
+      <c r="C248" t="str">
+        <v>2026-09-23 ~01:00 UTC: R-26-20226 states 'seeking a spring block intern' (spring-only, no year stated); R-26-20243-1 still states the combined 'spring/summer 2027 block intern' term. Neither is Boston-area. No change — still excluded on season-ambiguity grounds.</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>Relativity Space</v>
+      </c>
+      <c r="B249" t="str">
+        <v>'2027 Mechanical Engineer Intern' (Boston, MA reference), re-check via Ashby</v>
+      </c>
+      <c r="C249" t="str">
+        <v>2026-09-23 ~01:00 UTC: no Boston, MA connection found via Ashby or any other source this run — the recurring Boston reference in aggregator snippets appears to be noise. Relativity's internship program is confirmed LA-metro (Long Beach) only. Downgrading confidence on the 'worth re-checking' Boston lead from prior runs.</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>Analog Devices (Burlington, MA)</v>
+      </c>
+      <c r="B250" t="str">
+        <v>'Mechanical Engineering Co-Op' listing, re-check</v>
+      </c>
+      <c r="C250" t="str">
+        <v>2026-09-23 ~01:00 UTC: the one listing found (Simplify Jobs mirror) is marked INACTIVE and dated Jan-June 2025 — stale, not current. Still zero live US intern/co-op reqs as of this run.</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B251" t="str">
+        <v>Re-check</v>
+      </c>
+      <c r="C251" t="str">
+        <v>2026-09-23 ~01:00 UTC: 2026-cycle reqs all closed by mid-May 2026; no 2027 analogues live yet. No change.</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>Sierra Space</v>
+      </c>
+      <c r="B252" t="str">
+        <v>Re-check</v>
+      </c>
+      <c r="C252" t="str">
+        <v>2026-09-23 ~01:00 UTC: only a 'Fall 2026 Mechanical Engineering Intern' (Centennial, CO) found — Fall-only, not Spring 2027, and not Boston. Consistent with prior 'zero matching co-ops' pattern.</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>Boeing</v>
+      </c>
+      <c r="B253" t="str">
+        <v>Direct Workday CXS API query</v>
+      </c>
+      <c r="C253" t="str">
+        <v>2026-09-23 ~01:00 UTC: as of today only 'Boeing Summer 2027 Internship Program' postings exist (Engineering, Finance, Facilities, Quality) — no Spring 2027 wave live yet.</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>Lockheed Martin / Sikorsky</v>
+      </c>
+      <c r="B254" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C254" t="str">
+        <v>2026-09-23 ~01:00 UTC: search results show only Summer 2027 program postings; site remains Brassring/Workday-gated for independent verification. No Spring 2027 confirmed.</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B255" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C255" t="str">
+        <v>2026-09-23 ~01:00 UTC: confirmed '2027 ENGINEERING SUMMER INTERNSHIP' postings exist — still Summer-only. The previously-claimed Sept-Oct Spring/Winter posting window has now failed to materialize across 8 consecutive checked runs; recommend treating this claim as unreliable this cycle.</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>General Atomics / Spirit AeroSystems / Virgin Galactic</v>
+      </c>
+      <c r="B256" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C256" t="str">
+        <v>2026-09-23 ~01:00 UTC: all current postings found are Summer 2027 only; no Spring 2027 season stated anywhere.</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B257" t="str">
+        <v>Internships page</v>
+      </c>
+      <c r="C257" t="str">
+        <v>2026-09-23 ~01:00 UTC: page explicitly states internships 'typically begin in May or June and conclude in August or September' — Summer-only by the company's own description. Excluded.</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>Stoke Space</v>
+      </c>
+      <c r="B258" t="str">
+        <v>Greenhouse board, re-check</v>
+      </c>
+      <c r="C258" t="str">
+        <v>2026-09-23 ~01:00 UTC: a previously-indexed 'Spring 2027 Internship - Engineering' no longer appears on the board — likely closed/filled. Only Summer 2027 Engineering/Operations/Software internships remain.</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>Wisk Aero</v>
+      </c>
+      <c r="B259" t="str">
+        <v>Mechanical Engineering Intern (Lever)</v>
+      </c>
+      <c r="C259" t="str">
+        <v>2026-09-23 ~01:00 UTC: the specific posting found now 404s — closed/removed. No season was stated on it anyway.</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>Vast Space</v>
+      </c>
+      <c r="B260" t="str">
+        <v>'Emerging Talent - Mechanical/Aerospace Engineering Internship' (Long Beach/Hawthorne/Mojave, req 4711400006)</v>
+      </c>
+      <c r="C260" t="str">
+        <v>2026-09-23 ~01:00 UTC: confirmed live but states no specific term (Winter/Spring/Summer) — generic rolling 12-week internship, fails the 'season stated' verification bar.</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>Firefly Aerospace</v>
+      </c>
+      <c r="B261" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C261" t="str">
+        <v>2026-09-23 ~01:00 UTC: latest reqs on firefly.hrmdirect.com are Fall 2026 (Quality Engineering, req 3710242) and Summer 2026; no Spring 2027 posting exists yet.</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>Redwire Space</v>
+      </c>
+      <c r="B262" t="str">
+        <v>'Mechanical Engineering Intern - Year Round' (Albuquerque)</v>
+      </c>
+      <c r="C262" t="str">
+        <v>2026-09-23 ~01:00 UTC: this previously-found posting now 404s — dead link, likely filled/removed.</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>Safran USA</v>
+      </c>
+      <c r="B263" t="str">
+        <v>US internships listing</v>
+      </c>
+      <c r="C263" t="str">
+        <v>2026-09-23 ~01:00 UTC: current listings are supply chain, HR, HSE, and one Materials &amp; Processes intern (Gainesville TX, no season stated). No mechanical/aerospace Spring 2027 posting found.</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>Shield AI</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Direct Lever API pull</v>
+      </c>
+      <c r="C264" t="str">
+        <v>2026-09-23 ~01:00 UTC: only Summer 2027 postings exist (Mechanical, Electrical, Manufacturing, Software) — no Spring 2027.</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>Saildrone</v>
+      </c>
+      <c r="B265" t="str">
+        <v>Direct Greenhouse API pull (all 34 open jobs)</v>
+      </c>
+      <c r="C265" t="str">
+        <v>2026-09-23 ~01:00 UTC: zero internship postings of any kind currently.</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>Parker Hannifin / Honeywell Aerospace / Kratos Defense</v>
+      </c>
+      <c r="B266" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C266" t="str">
+        <v>2026-09-23 ~01:00 UTC: no Spring 2027 mechanical postings surfaced; Honeywell explicitly Summer 2027 only; Kratos's open-roles page returned no visible listings (likely JS-gated), no live req located.</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>Aerojet Rocketdyne / Aurora Flight Sciences</v>
+      </c>
+      <c r="B267" t="str">
+        <v>Fresh sweep via L3Harris/Boeing career sites</v>
+      </c>
+      <c r="C267" t="str">
+        <v>2026-09-23 ~01:00 UTC: no Spring 2027 mechanical/propulsion reqs found at either company's specific sites (Sacramento CA, Camden AR for Aerojet; Boeing's Aurora sites).</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>Archer Aviation / Joby Aviation / ispace</v>
+      </c>
+      <c r="B268" t="str">
+        <v>Fresh sweep</v>
+      </c>
+      <c r="C268" t="str">
+        <v>2026-09-23 ~01:00 UTC: no Spring 2027-dated mechanical postings found; current listings are Summer 2026/2027 only, or (ispace) no US-specific listing located.</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>General Dynamics Mission Systems</v>
+      </c>
+      <c r="B269" t="str">
+        <v>Fresh sweep beyond already-tracked McLeansville NC req</v>
+      </c>
+      <c r="C269" t="str">
+        <v>2026-09-23 ~01:00 UTC: careers-gdms.icims.com remains iframe/JS-gated. Only concretely found: 'Intern Engineer - Mechanical' (Dedham, MA) and 'Infrastructure Engineer Co-op (Fall 2026 or Spring 2027)' (Pittsfield, MA, non-mechanical discipline) — both Boston-area, out of scope for this national-sweep batch, and the latter is a discipline mismatch regardless.</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>Vertex Pharmaceuticals</v>
+      </c>
+      <c r="B270" t="str">
+        <v>Non-Boston mechanical engineering sweep</v>
+      </c>
+      <c r="C270" t="str">
+        <v>2026-09-23 ~01:00 UTC: no mechanical engineering Spring 2027 posting found outside Boston; Vertex's engineering internships appear Boston-HQ-centric (already tracked).</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>Textron Systems</v>
+      </c>
+      <c r="B271" t="str">
+        <v>req 343102, re-check</v>
+      </c>
+      <c r="C271" t="str">
+        <v>2026-09-23 ~01:00 UTC: careers.textron.com remains JS-rendered/inaccessible via curl or WebFetch. Search results consistently point to a distinct '2027 Intern - Mechanical Engineer (Sea Systems), Hunt Valley, MD' posting, but season could not be confirmed for either req. Unresolved, same as prior runs.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C237"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C271"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 18 checked-excluded (2026-09-23 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AAc8x95fTaXgpcMqAHEBqy
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J105"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -3629,16 +3629,144 @@
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Mechanisms &amp; Payload Internship (Spring 2027)</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Mechanical / Mechatronics Engineering</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Spring 2027 (Jan–May)</v>
+      </c>
+      <c r="E102" t="str">
+        <v>El Segundo, CA</v>
+      </c>
+      <c r="F102">
+        <v>2600</v>
+      </c>
+      <c r="G102" t="str">
+        <v>$33.00/hr + housing stipend for relocating interns</v>
+      </c>
+      <c r="H102" t="str">
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824821003</v>
+      </c>
+      <c r="I102" t="str">
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+      </c>
+      <c r="J102" t="str">
+        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. Designs/builds/tests flight electromechanical hardware (mechanisms, payloads). US work authorization + export-control (ITAR) screening required per posting.</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Structures Engineering Internship (Spring 2027)</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Mechanical / Aerospace / Structures Engineering</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Spring 2027 (Jan–May)</v>
+      </c>
+      <c r="E103" t="str">
+        <v>El Segundo, CA</v>
+      </c>
+      <c r="F103">
+        <v>2600</v>
+      </c>
+      <c r="G103" t="str">
+        <v>$33.00/hr + housing stipend for relocating interns</v>
+      </c>
+      <c r="H103" t="str">
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824817003</v>
+      </c>
+      <c r="I103" t="str">
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+      </c>
+      <c r="J103" t="str">
+        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. CAD/FEA design and build/test of spacecraft structural hardware. US work authorization + export-control (ITAR) screening required per posting.</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Spring 2027 (6-month assignment)</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F104">
+        <v>20</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H104" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Mechanical-Engineering-Co-Op_REQ-14457</v>
+      </c>
+      <c r="I104" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (tenant entegris), HTTP 200, canApply true, posting text explicitly states "Spring 2027 season," posted 12 days ago.</v>
+      </c>
+      <c r="J104" t="str">
+        <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Graduate Co-op, Supplier Engineering - Project Management Excellence (Jan–June 2027, Onsite)</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Industrial / Biomedical / Mechanical Engineering (MS)</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Winter/Spring 2027 (Jan 11 – Jun 30, 2027)</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F105">
+        <v>25</v>
+      </c>
+      <c r="G105" t="str">
+        <v>$25.00–$34.00/hr</v>
+      </c>
+      <c r="H105" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Graduate-Co-op--Supplier-Engineering---Project-Management-Excellence--January---June-2027--Onsite-_REQ-2026-18165</v>
+      </c>
+      <c r="I105" t="str">
+        <v>Yes — fetched directly via Insulet's own Workday CXS API (tenant insulet), HTTP 200, canApply true, explicit dates Jan 11 – Jun 30 2027, posted yesterday.</v>
+      </c>
+      <c r="J105" t="str">
+        <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J105"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C271"/>
+  <dimension ref="A1:C289"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -6626,9 +6754,207 @@
         <v>2026-09-23 ~01:00 UTC: careers.textron.com remains JS-rendered/inaccessible via curl or WebFetch. Search results consistently point to a distinct '2027 Intern - Mechanical Engineer (Sea Systems), Hunt Valley, MD' posting, but season could not be confirmed for either req. Unresolved, same as prior runs.</v>
       </c>
     </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B272" t="str">
+        <v>req 601496955, re-check</v>
+      </c>
+      <c r="C272" t="str">
+        <v>2026-09-23 ~07:00 UTC: still Cloudflare-blocked (14th+ consecutive run), one low-effort attempt per standing guidance. Needs a human in-browser check; automated attempts continue to be deprioritized.</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B273" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check #6</v>
+      </c>
+      <c r="C273" t="str">
+        <v>2026-09-23 ~07:00 UTC: careers site returned HTTP 503 again on direct fetch. LinkedIn/ZipRecruiter mirrors unchanged (req 300000421584867, Jan-June 2026, Marlborough MA). Still the strongest unconfirmed Boston-area lead; recommend a fresh attempt at a different time/network path next run.</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>HII / Newport News Shipbuilding</v>
+      </c>
+      <c r="B274" t="str">
+        <v>Full internship listing sweep (Engineering, IT, Supply Chain, Business Mgmt reqs went live Aug 28)</v>
+      </c>
+      <c r="C274" t="str">
+        <v>2026-09-23 ~07:00 UTC: postings finally appeared after 8+ runs of nothing, but confirmed via direct fetch to be explicitly a '10-week summer internship' — Summer 2027 only, wrong season. Still zero qualifying Winter/Spring postings.</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B275" t="str">
+        <v>'Intern - Hardware Engineer' (R5394), re-check</v>
+      </c>
+      <c r="C275" t="str">
+        <v>2026-09-23 ~07:00 UTC: fetched Symbotic's live careers page directly and enumerated all current listings (R7973, R7963, R5940, R6128, R7912, R7915, R7271, R7976, etc.) — R5394 does not appear among them. Resolved as filled/removed rather than an access-blocking issue; no qualifying Symbotic mechanical co-op currently exists.</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>Textron Systems (Hunt Valley, MD)</v>
+      </c>
+      <c r="B276" t="str">
+        <v>'2027 Intern - Mechanical Engineer (Sea Systems)'</v>
+      </c>
+      <c r="C276" t="str">
+        <v>2026-09-23 ~07:00 UTC: found via search only, Taleo page not independently fetchable. Textron's naming convention uses 'Co-Op' for Spring/Fall terms and unlabeled 'Intern' typically defaults to Summer — likely Summer, not confirmed Spring. Excluded for insufficient verification.</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B277" t="str">
+        <v>'Co-op Design Engineering (Spring 2027)', re-check</v>
+      </c>
+      <c r="C277" t="str">
+        <v>2026-09-23 ~07:00 UTC: LinkedIn/Fairygodboss still corroborate the posting exists, but eaton.dejobs.org (JS/Nuxt app backed by jobsyn.org) could not be queried directly — API guesses 404'd. Still blocked, unresolved.</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B278" t="str">
+        <v>Quick re-check for newly-opened Spring 2027 cycles</v>
+      </c>
+      <c r="C278" t="str">
+        <v>2026-09-23 ~07:00 UTC: no change. Analog Devices' only cached listing (Simplify Jobs) explicitly confirmed INACTIVE (stale Jan-June 2025 cohort); Lam Research still nothing posted.</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B279" t="str">
+        <v>Control &amp; Autonomous Systems Engineering Co-Op (Group 07-76); Human Resilience Technology Co-Op (Group 02-21), both Jan-June 2026</v>
+      </c>
+      <c r="C279" t="str">
+        <v>2026-09-23 ~07:00 UTC: both confirmed explicitly FILLED on direct fetch. Remaining open co-ops are non-mechanical (Cyber, IT, Logistics) or the already-tracked Microfab Jan-Aug 2027 reqs.</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B280" t="str">
+        <v>Trainee Co-Op reqs: CNC (R5034331), Carpentry (R5034333)</v>
+      </c>
+      <c r="C280" t="str">
+        <v>2026-09-23 ~07:00 UTC: both are skilled-trades apprenticeship-style roles, not engineering-degree positions — discipline mismatch, excluded. CNC req also confirmed no-longer-posted. No new engineering-discipline req found beyond the two already tracked at this site.</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B281" t="str">
+        <v>Mechanical Engineering Co-Op (R2476), Mechanical Engineering Intern (R2495), re-check</v>
+      </c>
+      <c r="C281" t="str">
+        <v>2026-09-23 ~07:00 UTC: both confirmed CLOSED via the Workday page's embedded `postingAvailable: false` flag (plain curl with browser UA, no CXS auth needed). Consistent with the standing 'zero current intern/co-op postings' finding from prior runs.</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B282" t="str">
+        <v>Structural &amp; Mechanical Engineering Internship (R66356, LA); Test Engineering Internship-Graduate (R66358); Aerospace Systems Engineering Intern-Graduate (R66202, Seattle); Manufacturing Engineering Internship-Undergrad (R66348, Space Coast FL)</v>
+      </c>
+      <c r="C282" t="str">
+        <v>2026-09-23 ~07:00 UTC: all 4 discipline-specific Spring 2027 reqs confirmed CLOSED via the same `postingAvailable: false` technique — resolves R66348 from a prior 'likely closed' inference to a conclusive finding. Only the general rolling 'Spring 2027 Engineering Intern – Undergraduate' (R69064, already tracked) remains open at this company.</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>Stoke Space</v>
+      </c>
+      <c r="B283" t="str">
+        <v>Spring 2027 Internship - Engineering (Moses Lake/Kent/Cape Canaveral)</v>
+      </c>
+      <c r="C283" t="str">
+        <v>2026-09-23 ~07:00 UTC: fetched directly — page explicitly states 'no longer accepting applications.' Closed.</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>Vast Space</v>
+      </c>
+      <c r="B284" t="str">
+        <v>Emerging Talent Mechanical/Aerospace &amp; Manufacturing Engineering Internships (Long Beach/Hawthorne/Mojave CA)</v>
+      </c>
+      <c r="C284" t="str">
+        <v>2026-09-23 ~07:00 UTC: confirmed open via direct Greenhouse fetch, but no season stated at all (rolling 'when are you available' field) — fails the season-verification bar. Worth a periodic re-check in case a dated Spring 2027 cohort req appears.</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>Shield AI</v>
+      </c>
+      <c r="B285" t="str">
+        <v>Full internship sweep via direct Lever/careers API pull</v>
+      </c>
+      <c r="C285" t="str">
+        <v>2026-09-23 ~07:00 UTC: only a Summer 2027 Mechanical Engineering Intern req exists; the Spring 2027 co-op reqs located are Electrical Engineering — discipline mismatch. No qualifying mechanical/aerospace Spring or Winter co-op found.</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B286" t="str">
+        <v>Internship program page, direct fetch</v>
+      </c>
+      <c r="C286" t="str">
+        <v>2026-09-23 ~07:00 UTC: company's own program page confirms the entire internship program runs May/June-Aug/Sept only (application deadline April 30, offers by end of April) — structurally excludes Winter/Spring participation. Wrong season by program design, not just this cycle.</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>Entegris (Billerica, MA)</v>
+      </c>
+      <c r="B287" t="str">
+        <v>'Manufacturing Engineering Co-Op' (REQ-14492)</v>
+      </c>
+      <c r="C287" t="str">
+        <v>2026-09-23 ~07:00 UTC: canApply true, Spring 2027 stated, but posting's 'Desired Major' is explicitly BS Chemical Engineering (filter-manufacturing process role) despite the generic-sounding title — discipline mismatch, excluded. (Other Entegris/Billerica reqs at the same site DID qualify — see `rows`.)</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B288" t="str">
+        <v>Full Workday CXS sweep (217 jobs enumerated), re-check</v>
+      </c>
+      <c r="C288" t="str">
+        <v>2026-09-23 ~07:00 UTC: no reqs found beyond the two already tracked in `rows` (Systems Engineering Co-Op JR002882, Electro-Mechanical Instrument Co-op JR002883-1) plus the already-excluded electrical/optics/Summer reqs. No change.</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Boston-area fresh sweep (no qualifying findings)</v>
+      </c>
+      <c r="B289" t="str">
+        <v>Teradyne, Vicor, Nuvation Engineering, Desktop Metal, Markforged, PTC, Bose, Nuvera Fuel Cells, Cirtec Medical, Charles River Labs, Commonwealth Fusion Systems, Boston Metal, Alloy Enterprises, Vicarious Surgical, Cognex, Berkshire Grey, PI Physik Instrumente, MathWorks, MKS Instruments</v>
+      </c>
+      <c r="C289" t="str">
+        <v>2026-09-23 ~07:00 UTC: queried each company's own career site/API directly. Teradyne, Vicor, Bose, Nuvera, Nuvation, Cirtec, Charles River Labs — zero current co-op/intern postings. Desktop Metal's Greenhouse board 404s (appears defunct); Markforged has only 3 open roles, none co-op/intern. Commonwealth Fusion Systems (Lever API, 102 postings) — zero co-op/intern titles, previously-indexed Fall/Spring 2026 co-ops gone. Boston Metal reportedly closed Woburn operations (layoffs, March 2026) — no postings expected. Alloy Enterprises' Greenhouse board returns zero jobs, reportedly folded into Johnson Controls. Vicarious Surgical's co-op listings remain explicitly closed. Cognex has zero relevant US reqs. Berkshire Grey (BambooHR, 23 open roles) confirmed same 4 already-tracked Spring 2027 co-ops, no new ones. PI Physik Instrumente still only shows the already-elapsed Jan-June 2026 cohort. MathWorks' EDG Internship is open but states no specific season/term — fails the season bar. MKS Instruments only has Fall 2026 reqs (R19858, R14406) confirmed on their own Workday.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C271"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C289"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 20 checked-excluded (2026-09-23 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012nDBDUCjCeSvZcAz4SnxKb
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J110"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -3695,78 +3695,238 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Entegris</v>
+        <v>Varda Space Industries</v>
       </c>
       <c r="B104" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Guidance, Navigation &amp; Controls (GNC) Internship (Spring 2027)</v>
       </c>
       <c r="C104" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Controls / Aerospace Engineering</v>
       </c>
       <c r="D104" t="str">
-        <v>Spring 2027 (6-month assignment)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E104" t="str">
-        <v>Billerica, MA</v>
+        <v>El Segundo, CA</v>
       </c>
       <c r="F104">
-        <v>20</v>
+        <v>2600</v>
       </c>
       <c r="G104" t="str">
-        <v>Not stated on posting</v>
+        <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H104" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Mechanical-Engineering-Co-Op_REQ-14457</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824781003</v>
       </c>
       <c r="I104" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (tenant entegris), HTTP 200, canApply true, posting text explicitly states "Spring 2027 season," posted 12 days ago.</v>
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J104" t="str">
-        <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. GNC for flight vehicles. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Propulsion Engineering Internship (Spring 2027)</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Mechanical / Propulsion Engineering</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E105" t="str">
+        <v>El Segundo, CA</v>
+      </c>
+      <c r="F105">
+        <v>2600</v>
+      </c>
+      <c r="G105" t="str">
+        <v>$33.00/hr + housing stipend for relocating interns</v>
+      </c>
+      <c r="H105" t="str">
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824765003</v>
+      </c>
+      <c r="I105" t="str">
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+      </c>
+      <c r="J105" t="str">
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Vehicle Integration &amp; Test Internship (Spring 2027)</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Mechanical / Aerospace Systems Engineering</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E106" t="str">
+        <v>El Segundo, CA</v>
+      </c>
+      <c r="F106">
+        <v>2600</v>
+      </c>
+      <c r="G106" t="str">
+        <v>$33.00/hr + housing stipend for relocating interns</v>
+      </c>
+      <c r="H106" t="str">
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824772003</v>
+      </c>
+      <c r="I106" t="str">
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+      </c>
+      <c r="J106" t="str">
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. Vehicle integration and test of flight hardware. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Marathon Petroleum</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Intern/Co-op - Refining Mechanical Engineer (Spring 2027)</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Mechanical Engineering (Industrial / Refining)</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Findlay, OH</v>
+      </c>
+      <c r="F107">
+        <v>700</v>
+      </c>
+      <c r="G107" t="str">
+        <v>$32.92–$41.67/hr</v>
+      </c>
+      <c r="H107" t="str">
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Intern-Co-op---Refining-Mechanical-Engineer--Spring-2027-_00020137</v>
+      </c>
+      <c r="I107" t="str">
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API, full job description returned, req 00020137.</v>
+      </c>
+      <c r="J107" t="str">
+        <v>New company, not previously tracked. Industrial/refining rather than aerospace, but fits mechanical/manufacturing discipline. Requires majoring in Mechanical or Civil Engineering; no visa sponsorship available. Posting also states co-op positions run spring, summer, and fall generally, but this specific req is titled and dated for Spring 2027. Additional refinery locations listed on same req: Anacortes WA, Canton OH, Catlettsburg KY, Detroit MI, El Paso TX, Garyville LA, Kenai AK, Mandan ND, Martinez CA, Robinson IL, Salt Lake City UT, St Paul Park MN, Texas City TX, Wilmington CA.</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Mechanical Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Mechanical Engineering (Consumer Product Manufacturing)</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Spring 2027 (Jan 11 – May 7, 2027)</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Louisville, KY</v>
+      </c>
+      <c r="F108">
+        <v>950</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Not stated on posting; housing/relocation assistance available for eligible students</v>
+      </c>
+      <c r="H108" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/Mechanical-Engineering-Co-op-Spring-2027_REQ-24833</v>
+      </c>
+      <c r="I108" t="str">
+        <v>Yes — fetched directly via GE Appliances' own Workday CXS API, full job description returned with explicit dates, req REQ-24833.</v>
+      </c>
+      <c r="J108" t="str">
+        <v>New company, not previously tracked. Industrial/consumer-manufacturing rather than aerospace, but squarely mechanical engineering with a clean Spring-only (not combined) term and explicit dates.</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Spring 2027 (6-month assignment)</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F109">
+        <v>20</v>
+      </c>
+      <c r="G109" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H109" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Mechanical-Engineering-Co-Op_REQ-14457</v>
+      </c>
+      <c r="I109" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (tenant entegris), HTTP 200, canApply true, posting text explicitly states "Spring 2027 season," posted 12 days ago.</v>
+      </c>
+      <c r="J109" t="str">
+        <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
         <v>Insulet</v>
       </c>
-      <c r="B105" t="str">
+      <c r="B110" t="str">
         <v>Graduate Co-op, Supplier Engineering - Project Management Excellence (Jan–June 2027, Onsite)</v>
       </c>
-      <c r="C105" t="str">
+      <c r="C110" t="str">
         <v>Industrial / Biomedical / Mechanical Engineering (MS)</v>
       </c>
-      <c r="D105" t="str">
+      <c r="D110" t="str">
         <v>Winter/Spring 2027 (Jan 11 – Jun 30, 2027)</v>
       </c>
-      <c r="E105" t="str">
+      <c r="E110" t="str">
         <v>Acton, MA</v>
       </c>
-      <c r="F105">
+      <c r="F110">
         <v>25</v>
       </c>
-      <c r="G105" t="str">
+      <c r="G110" t="str">
         <v>$25.00–$34.00/hr</v>
       </c>
-      <c r="H105" t="str">
+      <c r="H110" t="str">
         <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Graduate-Co-op--Supplier-Engineering---Project-Management-Excellence--January---June-2027--Onsite-_REQ-2026-18165</v>
       </c>
-      <c r="I105" t="str">
+      <c r="I110" t="str">
         <v>Yes — fetched directly via Insulet's own Workday CXS API (tenant insulet), HTTP 200, canApply true, explicit dates Jan 11 – Jun 30 2027, posted yesterday.</v>
       </c>
-      <c r="J105" t="str">
+      <c r="J110" t="str">
         <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J110"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C289"/>
+  <dimension ref="A1:C309"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -6952,9 +7112,229 @@
         <v>2026-09-23 ~07:00 UTC: queried each company's own career site/API directly. Teradyne, Vicor, Bose, Nuvera, Nuvation, Cirtec, Charles River Labs — zero current co-op/intern postings. Desktop Metal's Greenhouse board 404s (appears defunct); Markforged has only 3 open roles, none co-op/intern. Commonwealth Fusion Systems (Lever API, 102 postings) — zero co-op/intern titles, previously-indexed Fall/Spring 2026 co-ops gone. Boston Metal reportedly closed Woburn operations (layoffs, March 2026) — no postings expected. Alloy Enterprises' Greenhouse board returns zero jobs, reportedly folded into Johnson Controls. Vicarious Surgical's co-op listings remain explicitly closed. Cognex has zero relevant US reqs. Berkshire Grey (BambooHR, 23 open roles) confirmed same 4 already-tracked Spring 2027 co-ops, no new ones. PI Physik Instrumente still only shows the already-elapsed Jan-June 2026 cohort. MathWorks' EDG Internship is open but states no specific season/term — fails the season bar. MKS Instruments only has Fall 2026 reqs (R19858, R14406) confirmed on their own Workday.</v>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B290" t="str">
+        <v>req 601496955, re-check</v>
+      </c>
+      <c r="C290" t="str">
+        <v>2026-09-23 ~13:00 UTC: one low-effort attempt (jobs.buildsubmarines.com), still HTTP 403 Cloudflare block — 15th+ consecutive run. Separately, WebSearch snippets consistently describe a '2027 Spring Engineering CO-OP Trainee' req at this company but the page still cannot be independently rendered. Needs a human in-browser check.</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B291" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check #7</v>
+      </c>
+      <c r="C291" t="str">
+        <v>2026-09-23 ~13:00 UTC: direct posting URL still HTTP 503 (7th consecutive fail). New this run: successfully loaded Hologic's live careers search (195 open jobs company-wide) and ran a keyword search for 'co-op' — zero matches anywhere in current titles. Combined with the already-elapsed stated dates (Jan-June 2026), this is new evidence the posting is very likely closed/expired rather than merely bot-blocked. Downgrading priority on this lead.</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B292" t="str">
+        <v>Fresh sweep for a new mechanical/hardware co-op req</v>
+      </c>
+      <c r="C292" t="str">
+        <v>2026-09-23 ~13:00 UTC: only Summer 2027 co-op/software reqs found; no new Spring 2027 mechanical/systems co-op surfaced.</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>Textron Systems</v>
+      </c>
+      <c r="B293" t="str">
+        <v>req 343102 ('2027 Industrial Engineer Intern') and Hunt Valley MD 'Sea Systems' req, re-check</v>
+      </c>
+      <c r="C293" t="str">
+        <v>2026-09-23 ~13:00 UTC: careers.textron.com remains a JS-rendered SPA; direct fetch, search API, and guessed CXS-style endpoints all blocked. Season still unresolved for both reqs.</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B294" t="str">
+        <v>'Co-op Design Engineering', re-check</v>
+      </c>
+      <c r="C294" t="str">
+        <v>2026-09-23 ~13:00 UTC: the previously-cited Fairygodboss 'Spring 2027' link now 404s. LinkedIn currently shows the same role/pay range ($22.15-27.69/hr) labeled 'Summer 2027,' not Spring. eaton.eightfold.ai search did not surface a distinct live Spring-2027-labeled Jackson MS req. Excluded — no verifiable open Spring 2027 posting found; the Spring label may have simply rolled over to Summer 2027.</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B295" t="str">
+        <v>Quick re-check</v>
+      </c>
+      <c r="C295" t="str">
+        <v>2026-09-23 ~13:00 UTC: no change. Analog Devices' only listing (Simplify Jobs mirror) still explicitly marked INACTIVE (Jan-June 2025, Burlington MA); Lam Research still nothing posted for the 2027 cycle.</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>Vast Space</v>
+      </c>
+      <c r="B296" t="str">
+        <v>'Emerging Talent - Mechanical/Aerospace Engineering Internship', re-check</v>
+      </c>
+      <c r="C296" t="str">
+        <v>2026-09-23 ~13:00 UTC: re-confirmed open via direct Greenhouse fetch and a full Greenhouse API sweep (zero other internship titles company-wide). Still no season/term field of any kind on the posting — fails the season-stated bar, unchanged from last run.</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B297" t="str">
+        <v>Fresh sweep for new reqs beyond already-tracked ones</v>
+      </c>
+      <c r="C297" t="str">
+        <v>2026-09-23 ~13:00 UTC: careers.geaerospace.com/global/en/lynn is a landing page only on direct fetch (no listing data returned); could not enumerate live reqs. Inconclusive rather than a clean re-check — no new finding either way.</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B298" t="str">
+        <v>'Electrical Engineering Co-Op Spring 2027' (JR002941), full CXS sweep re-check (217 jobs)</v>
+      </c>
+      <c r="C298" t="str">
+        <v>2026-09-23 ~13:00 UTC: new req found beyond the already-tracked ones, but electrical discipline — excluded on discipline-mismatch grounds, consistent with prior treatment of Draper's electrical/optics reqs. No new mechanical/aerospace/robotics req found.</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B299" t="str">
+        <v>'Rapid Prototyping Aero/Mech Co-Op (Fall 2026)'</v>
+      </c>
+      <c r="C299" t="str">
+        <v>2026-09-23 ~13:00 UTC: only co-op surfaced on direct fetch is dated Fall 2026 — wrong season. No new Spring 2027 mechanical/aerospace posting found.</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>Entegris (Billerica, MA)</v>
+      </c>
+      <c r="B300" t="str">
+        <v>Digital Operations Co-Op (REQ-14395), Analytical Organic Lab Co-Op (REQ-14495), Analytical scientist Co-Op (REQ-14500-1)</v>
+      </c>
+      <c r="C300" t="str">
+        <v>2026-09-23 ~13:00 UTC: 3 more reqs found via partial Workday CXS sweep (rate-limited after 10 of 42 Billerica reqs retrieved) beyond the already-tracked 7 — all discipline mismatches (digital/analytical chemistry). No new mechanical/industrial/controls req found in what was retrieved.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Full Greenhouse board pull (518 jobs), re-check</v>
+      </c>
+      <c r="C301" t="str">
+        <v>2026-09-23 ~13:00 UTC: confirmed ~34 Spring 2027 reqs exist (mechanical, propulsion, structures, manufacturing, test — mostly Long Beach CA/Toronto/MD/VA/MS) but all fall under the already-tracked aggregate note; no new distinct disciplines/locations beyond what's already summarized.</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>SpaceX</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Full live-reqs sweep (6 total Spring 2027 reqs)</v>
+      </c>
+      <c r="C302" t="str">
+        <v>2026-09-23 ~13:00 UTC: only 2 on-discipline reqs exist (general Engineering Internship/Co-op, Graduate Engineer Internship/Co-op) and both are already tracked. The other 4 (Business Operations, Civil Engineering, Silicon Engineering, Software Engineering) are discipline mismatches.</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>Zipline</v>
+      </c>
+      <c r="B303" t="str">
+        <v>Full Greenhouse board pull (339 jobs), re-check</v>
+      </c>
+      <c r="C303" t="str">
+        <v>2026-09-23 ~13:00 UTC: every Spring 2027 mechanical/aerospace/structural/controls req is already among the 9 already tracked. Materials Engineer Intern remains correctly excluded as combined 'Spring &amp; Summer 2027.'</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B304" t="str">
+        <v>'Mechanical Associate Engineer (Spring 2027)' (4704621006), 'CAD Engineer Associate (Spring 2027)' (4704756006)</v>
+      </c>
+      <c r="C304" t="str">
+        <v>2026-09-23 ~13:00 UTC: both confirmed live via direct fetch, but posting text explicitly states these 'Associate' roles are 'designed for students who have already received a bachelor's degree' — not a current-student internship. Excluded on eligibility grounds.</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B305" t="str">
+        <v>Full board pull, re-check (11 Winter 2027 reqs)</v>
+      </c>
+      <c r="C305" t="str">
+        <v>2026-09-23 ~13:00 UTC: matches exactly what's already tracked/excluded (Mechanical/Systems/Manufacturing tracked; Electrical/others discipline-mismatched).</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>Reliable Robotics Corp (Mountain View, CA)</v>
+      </c>
+      <c r="B306" t="str">
+        <v>Mechanical Engineering Intern (stated 'accepting applications for the Winter 2026, and Spring 2027 seasons')</v>
+      </c>
+      <c r="C306" t="str">
+        <v>2026-09-23 ~13:00 UTC: aggregator (Built In SF) confirms the listing was removed 2026-07-20 — closed, not added.</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>Figure AI (San Jose, CA)</v>
+      </c>
+      <c r="B307" t="str">
+        <v>'Mechanical Engineer Intern [Winter 2026]' found via search snippets</v>
+      </c>
+      <c r="C307" t="str">
+        <v>2026-09-23 ~13:00 UTC: direct query of Figure's live Greenhouse board (97 jobs) found no current Winter 2026 or Spring 2027 titled jobs at all, and no Mechanical Engineer intern req of any season currently live (only Electrical Engineering and Special Projects, both Fall 2026). The Winter 2026 mechanical req is closed/gone.</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>SharkNinja (Needham, MA)</v>
+      </c>
+      <c r="B308" t="str">
+        <v>'Mechanical Engineering Co-op Opportunities'</v>
+      </c>
+      <c r="C308" t="str">
+        <v>2026-09-23 ~13:00 UTC: live and freshly posted (updated same day), full-time onsite Needham MA — but the entire posting text contains no season/term word at all (no Spring/Winter/Summer/Fall), a generic rolling co-op pipeline req. Fails the season-stated verification bar. Worth a periodic re-check in case a dated version appears: https://job-boards.greenhouse.io/sharkninjaoperatingllc/jobs/4713783006</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>General Dynamics Mission Systems (Dedham MA / Scottsdale AZ)</v>
+      </c>
+      <c r="B309" t="str">
+        <v>'Intern Engineer - Mechanical' (req 75046)</v>
+      </c>
+      <c r="C309" t="str">
+        <v>2026-09-23 ~13:00 UTC: confirmed live via Dreamwork mirror, but posting states 'This job posting will remain open until the position is filled' — no season stated at all. Excluded.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C289"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C309"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 6 new postings (Partial), 14 checked-excluded (2026-09-23 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015szFbn3WtnZrpFZ3qk1QTy
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J116"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -3917,16 +3917,208 @@
         <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Mechanical Engineering Technology Co-op (Spring 2027)</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Mechanical Engineering Technology</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Louisville, KY</v>
+      </c>
+      <c r="F111">
+        <v>950</v>
+      </c>
+      <c r="G111" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H111" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Mechanical-Engineering-Technology-Co-op-Spring-2027_REQ-24835</v>
+      </c>
+      <c r="I111" t="str">
+        <v>Partial — sibling req to the already fully-verified REQ-24833 (same tenant/site/title pattern), reported live with canApply:true by a research agent's direct Workday CXS API fetch. This session's own independent re-verification attempt (curl POST to the CXS jobs/job endpoints, and WebFetch of the rendered page) hit HTTP 422 / empty JS shell — consistent with Workday bot-blocking, not specific evidence the req is dead. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J111" t="str">
+        <v>New req beyond the already-tracked REQ-24833 (Mechanical Engineering Co-op) at the same Louisville, KY site.</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Mechanical / Manufacturing Engineering</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Louisville, KY</v>
+      </c>
+      <c r="F112">
+        <v>950</v>
+      </c>
+      <c r="G112" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H112" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24837</v>
+      </c>
+      <c r="I112" t="str">
+        <v>Partial — same basis as REQ-24835 above: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked by Workday's bot protection (422/empty JS shell). Verify live in-browser before applying.</v>
+      </c>
+      <c r="J112" t="str">
+        <v>New req beyond the already-tracked REQ-24833 at the same Louisville, KY site.</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Engineering (general — discipline not narrowly specified in title)</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E113" t="str">
+        <v>LaFayette, GA</v>
+      </c>
+      <c r="F113">
+        <v>1000</v>
+      </c>
+      <c r="G113" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H113" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Co-op-Spring-2027_REQ-24836</v>
+      </c>
+      <c r="I113" t="str">
+        <v>Partial — same basis as REQ-24835/24837: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser and confirm discipline before applying.</v>
+      </c>
+      <c r="J113" t="str">
+        <v>New site (LaFayette, GA) for GE Appliances beyond the already-tracked Louisville, KY reqs.</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Mechanical / Manufacturing Engineering</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E114" t="str">
+        <v>LaFayette, GA</v>
+      </c>
+      <c r="F114">
+        <v>1000</v>
+      </c>
+      <c r="G114" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H114" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24838</v>
+      </c>
+      <c r="I114" t="str">
+        <v>Partial — same basis as the other 2026-09-23 ~19:00 GE Appliances reqs: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser before applying.</v>
+      </c>
+      <c r="J114" t="str">
+        <v>New req at the same LaFayette, GA site as REQ-24836.</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>GE Appliances (a Haier company)</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Mechanical / Manufacturing Engineering</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E115" t="str">
+        <v>Decatur, AL</v>
+      </c>
+      <c r="F115">
+        <v>1050</v>
+      </c>
+      <c r="G115" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H115" t="str">
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Decatur-AL/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24839</v>
+      </c>
+      <c r="I115" t="str">
+        <v>Partial — same basis as the other 2026-09-23 ~19:00 GE Appliances reqs: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser before applying.</v>
+      </c>
+      <c r="J115" t="str">
+        <v>New site (Decatur, AL) for GE Appliances beyond the already-tracked Louisville KY / LaFayette GA reqs.</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Hologic</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Co-Op, R&amp;D Mechanical Engineer</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Mechanical Engineering (R&amp;D)</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Winter 2026 (Jan–June 2026)</v>
+      </c>
+      <c r="E116" t="str">
+        <v>Marlborough, MA</v>
+      </c>
+      <c r="F116">
+        <v>30</v>
+      </c>
+      <c r="G116" t="str">
+        <v>$26–$28/hr (per cached posting snippet)</v>
+      </c>
+      <c r="H116" t="str">
+        <v>https://na.careers.hologic.com/en/search/300000421584867/co-op-r-d-mechanical-engineer</v>
+      </c>
+      <c r="I116" t="str">
+        <v>Partial — this exact posting URL/req ID was located this run (prior runs only had aggregator mirrors). A search-engine-cached snippet of the live page confirms title, 'January – June 2026' dates, and $26–28/hr pay, matching Hamza's Winter 2026 target. However, the live page itself has returned HTTP 503 'Temporarily Unavailable' across 8+ consecutive runs including this one (re-tried directly this session, still 503) — cannot confirm current open/closed status by opening the actual page. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J116" t="str">
+        <v>Long-standing 'worth re-checking' item, now has a confirmed direct URL and season match for the first time. A second, likely newer Hologic req ('Co-Op, New Product Development Engineering', .../300000422097244/...) was also found this run but remains season-unconfirmed and 503-blocked — see `checked`.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J116"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C309"/>
+  <dimension ref="A1:C323"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -7332,9 +7524,163 @@
         <v>2026-09-23 ~13:00 UTC: confirmed live via Dreamwork mirror, but posting states 'This job posting will remain open until the position is filled' — no season stated at all. Excluded.</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B310" t="str">
+        <v>'Avionics Engineering Internship - Spring 2027' (7824780003) and 'Flight Software Internship - Spring 2027' (7824815003)</v>
+      </c>
+      <c r="C310" t="str">
+        <v>2026-09-23 ~19:00 UTC: both confirmed live/open via direct Greenhouse API fetch, El Segundo CA. Flight Software is a software discipline — excluded (same treatment as SpaceX's excluded Software Engineering req). Avionics was initially considered for 'flight systems' fit, but the full posting text explicitly requires 'a degree in Electrical Engineering or a related field' and is scoped to PCB/circuit design and embedded electronics work — an EE discipline, not mechanical/aerospace/controls. Excluded on discipline-mismatch grounds after reading the full description (corrected from an initial add to `rows` earlier in this same run, before the full text was pulled).</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>Impulse Space (Redondo Beach, CA)</v>
+      </c>
+      <c r="B311" t="str">
+        <v>'Antenna Engineering Intern (Spring 2027)' and 'RF Engineering Intern (Spring 2027)'</v>
+      </c>
+      <c r="C311" t="str">
+        <v>2026-09-23 ~19:00 UTC: new company for the tracker. Both confirmed live/open via direct fetch (HTTP 200, 'Apply Now' present, Jan-May 2027 dates), but RF/antenna engineering is an electrical-engineering discipline, outside Hamza's target list — same treatment as other excluded RF/electrical reqs. Company also runs ~25 Summer 2027 mechanical/propulsion/manufacturing internships (wrong season, not otherwise explored this run). Worth a periodic re-check for a Spring-2027-dated mechanical/propulsion/structures req specifically.</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>RTX / Collins Aerospace (Windsor Locks, CT)</v>
+      </c>
+      <c r="B312" t="str">
+        <v>'Project Engineering Co-op (Winter/Spring 2027)', req 01872926</v>
+      </c>
+      <c r="C312" t="str">
+        <v>2026-09-23 ~19:00 UTC: a research agent reported this as a new req, but it has the identical title/location/season to the already-tracked req 01872478 at the same Windsor Locks site. This session's own re-verification of both req IDs via RTX's Workday CXS API returned HTTP 422 for both (bot-blocking, not evidence either is dead) — could not independently distinguish 01872926 as a genuinely separate posting rather than a re-posted/duplicate req number. Not added; worth a fresh look next run to determine if these are truly two distinct co-op slots.</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>L3Harris (Greenville, TX)</v>
+      </c>
+      <c r="B313" t="str">
+        <v>'Mechanical Engineer Co-op' (agent-reported, no job ID given)</v>
+      </c>
+      <c r="C313" t="str">
+        <v>2026-09-23 ~19:00 UTC: a research agent flagged this as a Partial lead, but Hamza's tracker already has a fully-verified 'Mechanical Engineer Intern - Spring 2027' (job 41322) at the same Greenville, TX site. Without a distinct job ID from the agent, could not confirm this is a separate posting rather than an aggregator's alternate title for the same already-tracked req. Not added as a duplicate risk.</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>Anduril Industries (Costa Mesa, CA)</v>
+      </c>
+      <c r="B314" t="str">
+        <v>'Winter 2027 EWIS Harness Engineer Co-op' (agent-reported, no job ID given)</v>
+      </c>
+      <c r="C314" t="str">
+        <v>2026-09-23 ~19:00 UTC: mentioned by a research agent alongside the already-tracked Warhead Engineer/Test &amp; Evaluation Engineer Costa Mesa co-ops, but no Greenhouse job ID was provided and this session could not independently locate/verify it within this run's budget. Worth a follow-up next run to find the exact posting URL.</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>Parker Hannifin (Columbus, OH)</v>
+      </c>
+      <c r="B315" t="str">
+        <v>'Design Engineering Co-Op', Tube Fittings Division</v>
+      </c>
+      <c r="C315" t="str">
+        <v>2026-09-23 ~19:00 UTC: referenced in aggregator snippets as Spring 2027 with a 3.0+ GPA requirement, but the live Workday posting could not be located/fetched this run. Unverified, not added.</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>Berkshire Grey</v>
+      </c>
+      <c r="B316" t="str">
+        <v>'Spring 2027 Robot Learning R&amp;D Co-op' (job 768), re-check</v>
+      </c>
+      <c r="C316" t="str">
+        <v>2026-09-23 ~19:00 UTC: a research agent could not find this exact posting on Berkshire Grey's own BambooHR board this run (only located an unrelated same-titled 'VitroLabs Inc' Spring 2027 listing that is a different company, likely a scraper mismatch, plus a Spring 2026 Khosla Ventures board listing). This casts some doubt on whether the already-tracked job 768 is still live — not moved to `checked` yet since this session did not independently re-verify the live BambooHR API itself; worth a direct fetch next run to confirm.</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Northrop Grumman (Chandler, AZ)</v>
+      </c>
+      <c r="B317" t="str">
+        <v>'2027 Spring Mechanical Engineering Co-op' vs '2027 Fall Mechanical Engineering Co-op', req R10250495</v>
+      </c>
+      <c r="C317" t="str">
+        <v>2026-09-23 ~19:00 UTC: conflicting aggregator snippets under what may be the same req number describe this as both a Spring and a Fall 2027 co-op — looks like two distinct reqs with near-identical copy that got conflated by aggregators, or one mislabeled listing. Still unresolved/ambiguous; unchanged from prior 'combined-term, unverifiable link' status.</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>MKS Instruments (Andover, MA)</v>
+      </c>
+      <c r="B318" t="str">
+        <v>'2027 Summer Mechanical Automation Engineering Intern' (R20744)</v>
+      </c>
+      <c r="C318" t="str">
+        <v>2026-09-23 ~19:00 UTC: confirmed live but explicitly Summer 2027 — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>Textron Systems</v>
+      </c>
+      <c r="B319" t="str">
+        <v>req 343102, re-check via Taleo bypass</v>
+      </c>
+      <c r="C319" t="str">
+        <v>2026-09-23 ~19:00 UTC: successfully fetched the decoded Taleo page directly for the first time (bypassed the prior block) — confirmed the req is live/open (functional apply form, no closed-application language) and titled '2027 Industrial Engineer Intern.' Season is still stated only as generic '2027' with no Spring/Summer/Fall qualifier, and the role is Industrial (not core mechanical) — fails both the season-stated and discipline bars. Not added; the Hunt Valley MD 'Sea Systems' sibling req remains separately unconfirmed on season (aggregator-only, no year-qualifier found this run either).</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B320" t="str">
+        <v>'Co-op Design Engineering', re-check</v>
+      </c>
+      <c r="C320" t="str">
+        <v>2026-09-23 ~19:00 UTC: no new evidence found. LinkedIn continues to show this role labeled 'Summer 2027,' and the correct Workday tenant/site for eaton.com could not be located this run (guessed tenant/site paths returned HTTP 400/422). Treating the Spring 2027 version as likely gone, consistent with the prior run's conclusion.</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Full careers/Workday jobs API query, re-check</v>
+      </c>
+      <c r="C321" t="str">
+        <v>2026-09-23 ~19:00 UTC: currently only senior/staff-level Mechanical Engineer openings are posted; no student intern/co-op req of any season is currently live (the older R2495 generic 'Mechanical Engineering Intern' req returned HTTP 403 on direct fetch, consistent with the already-tracked closed status). No change.</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B322" t="str">
+        <v>req 601496955, re-check</v>
+      </c>
+      <c r="C322" t="str">
+        <v>2026-09-23 ~19:00 UTC: tried both jobs.buildsubmarines.com (Cloudflare JS challenge, HTTP 403) and careers-gdeb.icims.com (HTTP 405, 'Human Verification' page) — still blocked, 16th+ consecutive run. Needs a human in-browser check.</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>National fresh-sweep dead-ends (no qualifying Winter 2026/Spring 2027 findings)</v>
+      </c>
+      <c r="B323" t="str">
+        <v>Reliable Robotics (no current internship listed on Ashby board, prior lead removed), Stoke Space (Spring 2027 listing gone, only Summer 2027 remains), Joby Aviation ('Flight Test Intern Dec 2026-Feb 2027' confirmed HTTP 410 Gone; other live postings are Summer 2026, already past), Figure AI (Winter 2026 mechanical req no longer on live Greenhouse board), BAE Systems Cedar Rapids IA (3 'Mechanical Engineering Coop Spring/Summer 2027' reqs all 'no longer accepting applications'), Sierra Space (no Spring 2027/Winter 2026 mechanical/aerospace intern; live postings are Summer/Fall 2026), Pratt &amp; Whitney Canada (Winter 2027 Halifax NS/Mississauga ON reqs — Canada-based, not US, excluded on location grounds), Shield AI/Northrop Grumman Palmdale/Boeing/Spirit AeroSystems/Kratos Defense/Aurora Flight Sciences (all confirmed Summer-2027-only or wrong-season this run), General Atomics/Wisk Aero/Virgin Galactic/Bell Textron/Leidos (no qualifying Spring 2027/Winter 2026 posting found; primarily Summer-cycle), HII/Newport News Shipbuilding/ispace/Safran USA/Firefly Aerospace/Redwire Space/Saildrone/Honeywell Aerospace/Vast Space/Aerojet Rocketdyne/Archer Aviation (no qualifying posting surfaced this run, not exhaustively re-verified via direct ATS — flagged as not fully checked rather than conclusively dead).</v>
+      </c>
+      <c r="C323" t="str">
+        <v>2026-09-23 ~19:00 UTC national aerospace/defense/robotics sweep.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C309"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C323"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 5 checked-excluded (2026-09-24 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014wz31uM5ZRbPZPs4n4N6vN
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J121"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -4109,16 +4109,176 @@
         <v>Long-standing 'worth re-checking' item, now has a confirmed direct URL and season match for the first time. A second, likely newer Hologic req ('Co-Op, New Product Development Engineering', .../300000422097244/...) was also found this run but remains season-unconfirmed and 503-blocked — see `checked`.</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Aalo Atomics</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Mechanical Engineering Internship/Co-op (Spring 2027)</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Mechanical / Aerospace / Manufacturing Engineering</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Spring 2027 (January–May)</v>
+      </c>
+      <c r="E117" t="str">
+        <v>Austin, TX</v>
+      </c>
+      <c r="F117">
+        <v>1700</v>
+      </c>
+      <c r="G117" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H117" t="str">
+        <v>https://ats.rippling.com/aalo-atomics/jobs/7be73c9f-f1b8-470c-8c7e-333220736f0b</v>
+      </c>
+      <c r="I117" t="str">
+        <v>Yes — fetched directly, page live, 'Apply now' button present, no closed-application message.</v>
+      </c>
+      <c r="J117" t="str">
+        <v>New company for the tracker (advanced nuclear reactor startup). Requires B.S./M.S. in Mechanical, Aerospace, or Manufacturing Engineering (or closely related field) plus ~3 months applied engineering experience.</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B118" t="str">
+        <v>GNC &amp; Flight Software Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+      </c>
+      <c r="E118" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F118">
+        <v>950</v>
+      </c>
+      <c r="G118" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H118" t="str">
+        <v>https://jobs.khoslaventures.com/companies/hermeus/jobs/92195543-gnc-flight-software-intern-spring-summer-2027</v>
+      </c>
+      <c r="I118" t="str">
+        <v>Yes — fetched directly, page live, 'Apply now' button present, posted 2026-09-04, no closed-application message.</v>
+      </c>
+      <c r="J118" t="str">
+        <v>New company for the tracker (hypersonic aircraft developer). GNC (Guidance, Navigation &amp; Controls) role — flight-systems/controls discipline. Also open to Aerospace/Computer Engineering/CS/EE majors. Unlike a truly combined-term posting, the Spring option has its own distinct dates, so included (same treatment as RTX's 'Winter/Spring 2027' co-ops).</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Owens Corning</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Manufacturing Engineering Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Manufacturing / Mechanical Engineering</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Spring 2027 (~16 weeks)</v>
+      </c>
+      <c r="E119" t="str">
+        <v>Toledo, OH (also hiring for Feura Bush, NY; Sedalia, MO; Irving, TX)</v>
+      </c>
+      <c r="F119">
+        <v>720</v>
+      </c>
+      <c r="G119" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H119" t="str">
+        <v>https://careers.owenscorning.com/job/Toledo-Manufacturing-Engineering-Co-Op-(Spring-2027)-OH-43659-0001/1426905700/</v>
+      </c>
+      <c r="I119" t="str">
+        <v>Yes — fetched directly, page live, 'APPLY NOW »' button present, no closed-application message.</v>
+      </c>
+      <c r="J119" t="str">
+        <v>New company for the tracker (building materials manufacturer). Accepts Mechanical, Electrical, Engineering Technology, Chemical, or Industrial Engineering majors.</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Crown Equipment</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Mechanical Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E120" t="str">
+        <v>Greencastle, IN</v>
+      </c>
+      <c r="F120">
+        <v>900</v>
+      </c>
+      <c r="G120" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H120" t="str">
+        <v>https://us-careers.crown.com/job/Greencastle-Mechanical-Engineering-Co-op-Spring-2027-IN-46135/1420491100/</v>
+      </c>
+      <c r="I120" t="str">
+        <v>Yes — fetched directly, page live, 'Apply now' button present, req 146174, no closed-application message.</v>
+      </c>
+      <c r="J120" t="str">
+        <v>New company for the tracker (forklift/material handling equipment manufacturer). Mechanical design/simulation/testing for forklift and material handling equipment development.</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Winter 2027 EWIS Harness Engineer Co-op</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Mechanical / Electrical Engineering (wire harness design)</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027)</v>
+      </c>
+      <c r="E121" t="str">
+        <v>Costa Mesa, CA</v>
+      </c>
+      <c r="F121">
+        <v>2600</v>
+      </c>
+      <c r="G121" t="str">
+        <v>$34–$50/hr</v>
+      </c>
+      <c r="H121" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236577007</v>
+      </c>
+      <c r="I121" t="str">
+        <v>Yes — fetched directly on Greenhouse, Apply button live, no closed-application message.</v>
+      </c>
+      <c r="J121" t="str">
+        <v>Resolves a 'worth re-checking' item from the 2026-09-23 ~19:00 UTC run (previously found without a job ID). Same batch/site as the already-tracked Propulsion, Warhead, and Test &amp; Evaluation Engineer Costa Mesa co-ops. Open to Mechanical or Electrical Engineering majors.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J121"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C323"/>
+  <dimension ref="A1:C327"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -7678,9 +7838,53 @@
         <v>2026-09-23 ~19:00 UTC national aerospace/defense/robotics sweep.</v>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>RTX / Collins Aerospace (Windsor Locks, CT)</v>
+      </c>
+      <c r="B324" t="str">
+        <v>'Project Engineering Co-op (Winter/Spring 2027)', req 01873957 — a third, distinct req ID at the same site beyond already-tracked 01872478 and previously-flagged 01872926</v>
+      </c>
+      <c r="C324" t="str">
+        <v>2026-09-24 ~01:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 422 for 01873957, but also returned HTTP 422 on the already-fully-verified, currently-open 01872478 used as a sanity check — confirms this is today's Workday bot-blocking, not evidence 01873957 is dead. WebFetch also returned empty (JS shell). Could not independently confirm as a genuinely distinct third co-op slot vs. a duplicate/re-post. Not added; RTX Windsor Locks routinely posts multiple concurrent co-op reqs, so a third real slot is plausible — worth a fresh attempt next run.</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>Entegris (Billerica, MA)</v>
+      </c>
+      <c r="B325" t="str">
+        <v>'Mechanical Engineering Co-Op' REQ-7046, REQ-7047-1, and 'Manufacturing Engineering Co-Op' REQ-8392 (agent-reported via aggregator mirrors)</v>
+      </c>
+      <c r="C325" t="str">
+        <v>2026-09-24 ~01:00 UTC: these req numbers are far outside the REQ-144xx/145xx range of every other Entegris/Billerica req already confirmed live in `rows`. Direct fetch of REQ-7046's Workday job page returned empty content, and a direct query of Entegris's own Workday CXS jobs-search API for 'REQ-7046' returned zero results (total:0). Could not confirm these req numbers exist at all — likely stale, mis-transcribed, or belong to a different/older Entegris career site (one agent separately noted a same-titled Entegris req may actually be in San Luis Obispo, CA, not Billerica). Not added.</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Crown Equipment (Greencastle, IN)</v>
+      </c>
+      <c r="B326" t="str">
+        <v>'Mechanical Engineering Co-op - Spring 2027', req 146174</v>
+      </c>
+      <c r="C326" t="str">
+        <v>2026-09-24 ~01:00 UTC: initial fetch attempts of the generic co-op landing page gave inconsistent signals; located and fetched the actual job-detail URL directly, confirmed live with an active Apply button and no closed message. ADDED to `rows` — this entry documents the verification path, not an exclusion.</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Hologic (Marlborough, MA)</v>
+      </c>
+      <c r="B327" t="str">
+        <v>'Co-Op, R&amp;D Mechanical Engineer', re-check</v>
+      </c>
+      <c r="C327" t="str">
+        <v>2026-09-24 ~01:00 UTC: 9th consecutive HTTP 503 on direct fetch. No change — remains Partial in `rows` with the confirmed URL/season/pay from the prior run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C323"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C327"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add RESUME, COVER LETTER, and QUESTIONS columns with links (batch 1)
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:M121"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -410,6 +410,7 @@
     <col min="8" max="8" width="60.83203125" customWidth="1"/>
     <col min="9" max="9" width="55.83203125" customWidth="1"/>
     <col min="10" max="10" width="50.83203125" customWidth="1"/>
+    <col min="11" max="13" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,6 +444,21 @@
       <c r="J1" t="str">
         <v>Notes</v>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>RESUME</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>COVER LETTER</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>QUESTIONS</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -475,6 +491,21 @@
       <c r="J2" t="str">
         <v>12 weeks, full-time, on-site. Enrolled full-time student required.</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -507,6 +538,21 @@
       <c r="J3" t="str">
         <v>12 weeks, full-time, on-site. Enrolled full-time student required.</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -539,6 +585,21 @@
       <c r="J4" t="str">
         <v>Full-time, on-site. Must be enrolled undergrad/grad.</v>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>N/A (form only asks yes/no screening questions)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -571,6 +632,21 @@
       <c r="J5" t="str">
         <v>Right in the Boston metro. Portfolio of prior engineering work requested.</v>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -603,6 +679,21 @@
       <c r="J6" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -635,6 +726,21 @@
       <c r="J7" t="str">
         <v>US citizen/national/permanent resident required (ITAR). Sophomore standing+.</v>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -664,6 +770,21 @@
       <c r="J8" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -696,6 +817,21 @@
       <c r="J9" t="str">
         <v>Grad student, US citizen/national/permanent resident required (ITAR).</v>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Skipped: graduate students only (you are an undergrad)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -725,6 +861,21 @@
       <c r="J10" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -757,6 +908,21 @@
       <c r="J11" t="str">
         <v>Min. 12 weeks, full-time, on-site.</v>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -789,6 +955,21 @@
       <c r="J12" t="str">
         <v>Min. 12 weeks, full-time, on-site.</v>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -821,6 +1002,21 @@
       <c r="J13" t="str">
         <v>NASCAR team — structural/CAD design internship. Min GPA 2.8, 30+ semester hrs completed.</v>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -853,6 +1049,21 @@
       <c r="J14" t="str">
         <v>Closest option to Boston besides Formlabs. Likely requires US citizenship (ITAR/clearance).</v>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -885,6 +1096,21 @@
       <c r="J15" t="str">
         <v>Not Boston-area. Sibling req 'Mechanical Engineering Co-Op (July–December 2026)' exists at the same site — different season, not this one. Requires US citizenship + DoD Secret clearance eligibility.</v>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -917,6 +1143,21 @@
       <c r="J16" t="str">
         <v>6-month co-op spanning into Spring 2027.</v>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -946,6 +1187,21 @@
       <c r="J17" t="str">
         <v>Restricted to Drexel University co-op program students — check eligibility before applying.</v>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Skipped: only open to Drexel University co-op students</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Skipped: only open to Drexel University co-op students</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Skipped: only open to Drexel University co-op students</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -978,6 +1234,21 @@
       <c r="J18" t="str">
         <v>16–20 hrs/wk during school year, 30–40 hrs/wk in summer. Requires graduation Dec 2026 or later. CMM/dimensional-analysis work in production environment.</v>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1010,6 +1281,21 @@
       <c r="J19" t="str">
         <v>Housing/relocation assistance if 50+ mi from site. Must be work-authorized without sponsorship.</v>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Open resume</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Open cover letter</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Open questions</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -4270,8 +4556,51 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="K2" r:id="rId1"/>
+    <hyperlink ref="L2" r:id="rId2"/>
+    <hyperlink ref="M2" r:id="rId3"/>
+    <hyperlink ref="K3" r:id="rId4"/>
+    <hyperlink ref="L3" r:id="rId5"/>
+    <hyperlink ref="M3" r:id="rId6"/>
+    <hyperlink ref="K4" r:id="rId7"/>
+    <hyperlink ref="L4" r:id="rId8"/>
+    <hyperlink ref="K5" r:id="rId9"/>
+    <hyperlink ref="L5" r:id="rId10"/>
+    <hyperlink ref="M5" r:id="rId11"/>
+    <hyperlink ref="K7" r:id="rId12"/>
+    <hyperlink ref="L7" r:id="rId13"/>
+    <hyperlink ref="M7" r:id="rId14"/>
+    <hyperlink ref="K8" r:id="rId15"/>
+    <hyperlink ref="L8" r:id="rId16"/>
+    <hyperlink ref="M8" r:id="rId17"/>
+    <hyperlink ref="K10" r:id="rId18"/>
+    <hyperlink ref="L10" r:id="rId19"/>
+    <hyperlink ref="M10" r:id="rId20"/>
+    <hyperlink ref="K11" r:id="rId21"/>
+    <hyperlink ref="L11" r:id="rId22"/>
+    <hyperlink ref="M11" r:id="rId23"/>
+    <hyperlink ref="K12" r:id="rId24"/>
+    <hyperlink ref="L12" r:id="rId25"/>
+    <hyperlink ref="M12" r:id="rId26"/>
+    <hyperlink ref="K13" r:id="rId27"/>
+    <hyperlink ref="L13" r:id="rId28"/>
+    <hyperlink ref="M13" r:id="rId29"/>
+    <hyperlink ref="K14" r:id="rId30"/>
+    <hyperlink ref="L14" r:id="rId31"/>
+    <hyperlink ref="M14" r:id="rId32"/>
+    <hyperlink ref="K15" r:id="rId33"/>
+    <hyperlink ref="L15" r:id="rId34"/>
+    <hyperlink ref="M15" r:id="rId35"/>
+    <hyperlink ref="K16" r:id="rId36"/>
+    <hyperlink ref="L16" r:id="rId37"/>
+    <hyperlink ref="M16" r:id="rId38"/>
+    <hyperlink ref="K19" r:id="rId39"/>
+    <hyperlink ref="L19" r:id="rId40"/>
+    <hyperlink ref="M19" r:id="rId41"/>
+  </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J121"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M121"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
build: preserve RESUME/COVER LETTER/QUESTIONS columns across regeneration
build.mjs's regeneration overwrites the xlsx from scratch, which would
silently wipe the RESUME/COVER LETTER/QUESTIONS hyperlink columns that
were manually added on top of the generated rows. Merge those columns
back in from the existing file (matched by Company + Role Title) before
writing, so the routine's automated regeneration stops clobbering that
work.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JxbdzK1r7LcgrRSzNUrsTN
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -410,7 +410,9 @@
     <col min="8" max="8" width="60.83203125" customWidth="1"/>
     <col min="9" max="9" width="55.83203125" customWidth="1"/>
     <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="13" width="26" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,20 +446,14 @@
       <c r="J1" t="str">
         <v>Notes</v>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>RESUME</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>COVER LETTER</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>QUESTIONS</t>
-        </is>
+      <c r="K1" t="str">
+        <v>RESUME</v>
+      </c>
+      <c r="L1" t="str">
+        <v>COVER LETTER</v>
+      </c>
+      <c r="M1" t="str">
+        <v>QUESTIONS</v>
       </c>
     </row>
     <row r="2">
@@ -491,20 +487,14 @@
       <c r="J2" t="str">
         <v>12 weeks, full-time, on-site. Enrolled full-time student required.</v>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K2" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="3">
@@ -538,20 +528,14 @@
       <c r="J3" t="str">
         <v>12 weeks, full-time, on-site. Enrolled full-time student required.</v>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K3" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="4">
@@ -585,20 +569,14 @@
       <c r="J4" t="str">
         <v>Full-time, on-site. Must be enrolled undergrad/grad.</v>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>N/A (form only asks yes/no screening questions)</t>
-        </is>
+      <c r="K4" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M4" t="str">
+        <v>N/A (form only asks yes/no screening questions)</v>
       </c>
     </row>
     <row r="5">
@@ -632,20 +610,14 @@
       <c r="J5" t="str">
         <v>Right in the Boston metro. Portfolio of prior engineering work requested.</v>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K5" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="6">
@@ -679,20 +651,14 @@
       <c r="J6" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
+      <c r="K6" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
       </c>
     </row>
     <row r="7">
@@ -726,20 +692,14 @@
       <c r="J7" t="str">
         <v>US citizen/national/permanent resident required (ITAR). Sophomore standing+.</v>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K7" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="8">
@@ -770,20 +730,14 @@
       <c r="J8" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K8" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="9">
@@ -817,20 +771,14 @@
       <c r="J9" t="str">
         <v>Grad student, US citizen/national/permanent resident required (ITAR).</v>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Skipped: graduate students only (you are an undergrad)</t>
-        </is>
+      <c r="K9" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
       </c>
     </row>
     <row r="10">
@@ -861,20 +809,14 @@
       <c r="J10" t="str">
         <v>US citizen/national/permanent resident required (ITAR).</v>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K10" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="11">
@@ -908,20 +850,14 @@
       <c r="J11" t="str">
         <v>Min. 12 weeks, full-time, on-site.</v>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K11" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="12">
@@ -955,20 +891,14 @@
       <c r="J12" t="str">
         <v>Min. 12 weeks, full-time, on-site.</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K12" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="13">
@@ -1002,20 +932,14 @@
       <c r="J13" t="str">
         <v>NASCAR team — structural/CAD design internship. Min GPA 2.8, 30+ semester hrs completed.</v>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K13" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="14">
@@ -1049,20 +973,14 @@
       <c r="J14" t="str">
         <v>Closest option to Boston besides Formlabs. Likely requires US citizenship (ITAR/clearance).</v>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K14" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="15">
@@ -1096,20 +1014,14 @@
       <c r="J15" t="str">
         <v>Not Boston-area. Sibling req 'Mechanical Engineering Co-Op (July–December 2026)' exists at the same site — different season, not this one. Requires US citizenship + DoD Secret clearance eligibility.</v>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K15" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="16">
@@ -1143,20 +1055,14 @@
       <c r="J16" t="str">
         <v>6-month co-op spanning into Spring 2027.</v>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K16" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="17">
@@ -1187,20 +1093,14 @@
       <c r="J17" t="str">
         <v>Restricted to Drexel University co-op program students — check eligibility before applying.</v>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Skipped: only open to Drexel University co-op students</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Skipped: only open to Drexel University co-op students</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Skipped: only open to Drexel University co-op students</t>
-        </is>
+      <c r="K17" t="str">
+        <v>Skipped: only open to Drexel University co-op students</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Skipped: only open to Drexel University co-op students</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Skipped: only open to Drexel University co-op students</v>
       </c>
     </row>
     <row r="18">
@@ -1234,20 +1134,14 @@
       <c r="J18" t="str">
         <v>16–20 hrs/wk during school year, 30–40 hrs/wk in summer. Requires graduation Dec 2026 or later. CMM/dimensional-analysis work in production environment.</v>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</t>
-        </is>
+      <c r="K18" t="str">
+        <v>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Skipped: part-time on-site job in Illinois during the school year (16–20 hrs/wk)</v>
       </c>
     </row>
     <row r="19">
@@ -1281,20 +1175,14 @@
       <c r="J19" t="str">
         <v>Housing/relocation assistance if 50+ mi from site. Must be work-authorized without sponsorship.</v>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Open resume</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Open cover letter</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Open questions</t>
-        </is>
+      <c r="K19" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="20">

</xml_diff>

<commit_message>
routine: 10 new postings, 16 checked-excluded (2026-09-24 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JxbdzK1r7LcgrRSzNUrsTN
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M130"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1810,10 +1810,10 @@
         <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H39" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-CT-WINDSOR-LOCKS-B1A--1-Hamilton-Rd--BLDG-1A/Project-Engineering-Co-op--Winter-Spring-2027-_01872478</v>
+        <v>https://careers.rtx.com/global/en/job/01872926</v>
       </c>
       <c r="I39" t="str">
-        <v>Partial — Workday page blocked automated fetch (blank/JS-rendered). Req ID and Sept 14, 2026 posting date confirmed via aggregator mirror only. Verify live in-browser before applying.</v>
+        <v>Yes — replaces the previously-tracked req 01872478 (now HTTP 410, confirmed dead this run) with req 01872926: fetched directly via careers.rtx.com, HTTP 200 with live embedded JobPosting JSON-LD, datePosted 2026-09-22. A near-identical req 01873957 also exists at the same site (same title/recruiter, opened a few days later) — treated as a duplicate/parallel posting of this same role, not added separately.</v>
       </c>
       <c r="J39" t="str">
         <v>~1.5 hrs from Boston.</v>
@@ -4117,7 +4117,7 @@
         <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Mechanical-Engineering-Technology-Co-op-Spring-2027_REQ-24835</v>
       </c>
       <c r="I111" t="str">
-        <v>Partial — sibling req to the already fully-verified REQ-24833 (same tenant/site/title pattern), reported live with canApply:true by a research agent's direct Workday CXS API fetch. This session's own independent re-verification attempt (curl POST to the CXS jobs/job endpoints, and WebFetch of the rendered page) hit HTTP 422 / empty JS shell — consistent with Workday bot-blocking, not specific evidence the req is dead. Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch (both search and full job-detail endpoints) returned HTTP 200 with canApply:true. Supersedes the earlier Partial status from Workday bot-blocking on a prior run.</v>
       </c>
       <c r="J111" t="str">
         <v>New req beyond the already-tracked REQ-24833 (Mechanical Engineering Co-op) at the same Louisville, KY site.</v>
@@ -4149,7 +4149,7 @@
         <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24837</v>
       </c>
       <c r="I112" t="str">
-        <v>Partial — same basis as REQ-24835 above: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked by Workday's bot protection (422/empty JS shell). Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J112" t="str">
         <v>New req beyond the already-tracked REQ-24833 at the same Louisville, KY site.</v>
@@ -4181,7 +4181,7 @@
         <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Co-op-Spring-2027_REQ-24836</v>
       </c>
       <c r="I113" t="str">
-        <v>Partial — same basis as REQ-24835/24837: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser and confirm discipline before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status. Discipline still not narrowly specified in title/posting.</v>
       </c>
       <c r="J113" t="str">
         <v>New site (LaFayette, GA) for GE Appliances beyond the already-tracked Louisville, KY reqs.</v>
@@ -4213,7 +4213,7 @@
         <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24838</v>
       </c>
       <c r="I114" t="str">
-        <v>Partial — same basis as the other 2026-09-23 ~19:00 GE Appliances reqs: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J114" t="str">
         <v>New req at the same LaFayette, GA site as REQ-24836.</v>
@@ -4245,7 +4245,7 @@
         <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Decatur-AL/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24839</v>
       </c>
       <c r="I115" t="str">
-        <v>Partial — same basis as the other 2026-09-23 ~19:00 GE Appliances reqs: agent-reported live via direct Workday CXS API fetch (canApply:true), this session's own re-verification blocked (422/empty JS shell). Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J115" t="str">
         <v>New site (Decatur, AL) for GE Appliances beyond the already-tracked Louisville KY / LaFayette GA reqs.</v>
@@ -4441,6 +4441,294 @@
       </c>
       <c r="J121" t="str">
         <v>Resolves a 'worth re-checking' item from the 2026-09-23 ~19:00 UTC run (previously found without a job ID). Same batch/site as the already-tracked Propulsion, Warhead, and Test &amp; Evaluation Engineer Costa Mesa co-ops. Open to Mechanical or Electrical Engineering majors.</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Crown Equipment</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Mechanical Engineering Intern/Co-op (Spring 2027)</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E122" t="str">
+        <v>Kinston, NC</v>
+      </c>
+      <c r="F122">
+        <v>700</v>
+      </c>
+      <c r="G122" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H122" t="str">
+        <v>https://us-careers.crown.com/job/Kinston-Mechanical-Engineering-InternCo-op-Spring-2027-NC-28504/1426309500/</v>
+      </c>
+      <c r="I122" t="str">
+        <v>Yes — fetched directly, HTTP 200, title/season confirmed on page, 'Apply now' present, req 146597, no closed-application message.</v>
+      </c>
+      <c r="J122" t="str">
+        <v>New sibling req to the already-tracked Greencastle, IN req (146174) at the same company, found via a fresh sweep of Crown's own careers site.</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Structures/Mechanical Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Structural / Mechanical Engineering</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+      </c>
+      <c r="E123" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F123">
+        <v>950</v>
+      </c>
+      <c r="G123" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H123" t="str">
+        <v>https://jobs.lever.co/hermeus/60b5d40a-1065-4bd2-8c72-6b2fb69d4761</v>
+      </c>
+      <c r="I123" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-08 or similar recent date.</v>
+      </c>
+      <c r="J123" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern at the same company/site; same distinct Spring/Summer option structure (not a merged single term).</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Mechanical Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+      </c>
+      <c r="E124" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F124">
+        <v>2600</v>
+      </c>
+      <c r="G124" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H124" t="str">
+        <v>https://jobs.lever.co/hermeus/1bc5c858-1b04-4093-80a0-2ba3491afc60</v>
+      </c>
+      <c r="I124" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+      </c>
+      <c r="J124" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct Spring/Summer option structure.</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Propulsion Component Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Propulsion / Mechanical Engineering</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
+      </c>
+      <c r="E125" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F125">
+        <v>2600</v>
+      </c>
+      <c r="G125" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H125" t="str">
+        <v>https://jobs.lever.co/hermeus/2cbb75f7-a040-47b2-a442-d9cc1faedb11</v>
+      </c>
+      <c r="I125" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-08-31. Posting states only a Spring 2027 term, no Summer/Fall option.</v>
+      </c>
+      <c r="J125" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern. Flight-critical mechanical/fluid propulsion components (valves, actuators).</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Propulsion Test Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Propulsion / Mechanical Engineering</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
+      </c>
+      <c r="E126" t="str">
+        <v>Jacksonville, FL</v>
+      </c>
+      <c r="F126">
+        <v>1050</v>
+      </c>
+      <c r="G126" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H126" t="str">
+        <v>https://jobs.lever.co/hermeus/d2651ecb-9aab-4d84-8e69-cbcf7cece28d</v>
+      </c>
+      <c r="I126" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-23 (posted same day as this run). Posting states only a Spring 2027 term, no Summer/Fall option.</v>
+      </c>
+      <c r="J126" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, new site (Jacksonville, FL). Propulsion system/engine test stand support.</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Propulsion Engineering Intern (Spring/Summer/Fall 2027)</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Propulsion / Mechanical Engineering</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+      </c>
+      <c r="E127" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F127">
+        <v>2600</v>
+      </c>
+      <c r="G127" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H127" t="str">
+        <v>https://jobs.lever.co/hermeus/943f51e4-5b26-432c-ae85-de5f43cadb86</v>
+      </c>
+      <c r="I127" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+      </c>
+      <c r="J127" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure (Spring/Summer/Fall each independently dated, not a merged single term).</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Structures Engineering Intern (Spring/Summer/Fall 2027)</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+      </c>
+      <c r="E128" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F128">
+        <v>2600</v>
+      </c>
+      <c r="G128" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H128" t="str">
+        <v>https://jobs.lever.co/hermeus/6b65768c-a8b2-4c77-8d5f-f407e32bb878</v>
+      </c>
+      <c r="I128" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+      </c>
+      <c r="J128" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Manufacturing Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
+      </c>
+      <c r="E129" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F129">
+        <v>950</v>
+      </c>
+      <c r="G129" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H129" t="str">
+        <v>https://jobs.lever.co/hermeus/1bdf3754-5649-4a50-913e-b05140cb004f</v>
+      </c>
+      <c r="I129" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
+      </c>
+      <c r="J129" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Manufacturing Engineering Intern (Spring/Summer/Fall 2027)</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+      </c>
+      <c r="E130" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F130">
+        <v>2600</v>
+      </c>
+      <c r="G130" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H130" t="str">
+        <v>https://jobs.lever.co/hermeus/5f6a6e79-9836-4c33-b40b-a2bb6c27bd06</v>
+      </c>
+      <c r="I130" t="str">
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
+      </c>
+      <c r="J130" t="str">
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, a distinct site (Los Angeles) from the Atlanta Manufacturing Engineering Intern req above.</v>
       </c>
     </row>
   </sheetData>
@@ -4488,14 +4776,14 @@
     <hyperlink ref="M19" r:id="rId41"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M121"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M130"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C327"/>
+  <dimension ref="A1:C343"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -8099,9 +8387,185 @@
         <v>2026-09-24 ~01:00 UTC: 9th consecutive HTTP 503 on direct fetch. No change — remains Partial in `rows` with the confirmed URL/season/pay from the prior run.</v>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>RTX / Collins Aerospace (Windsor Locks, CT)</v>
+      </c>
+      <c r="B328" t="str">
+        <v>'Project Engineering Co-op (Winter/Spring 2027)', req 01872478 — the req previously tracked as Partial in `rows`</v>
+      </c>
+      <c r="C328" t="str">
+        <v>2026-09-24 ~07:00 UTC: this session's own direct fetch of careers.rtx.com/global/en/job/01872478 returned HTTP 410 Gone — confirmed dead. MOVED from `rows` to `checked` and replaced with req 01872926 (confirmed live via the same direct-fetch method, same title/site).</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>RTX / Collins Aerospace (Windsor Locks, CT)</v>
+      </c>
+      <c r="B329" t="str">
+        <v>'Project Engineering Co-op (Winter/Spring 2027)', req 01873957</v>
+      </c>
+      <c r="C329" t="str">
+        <v>2026-09-24 ~07:00 UTC: this session's own direct fetch confirmed this req is live (HTTP 200, JobPosting JSON-LD present, same title/site/recruiter as req 01872926, opened a few days later). Treated as a duplicate/parallel posting of the same role already added to `rows` as 01872926, not added as a separate row.</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>RTX (Burnsville, MN)</v>
+      </c>
+      <c r="B330" t="str">
+        <v>'Advanced Manufacturing Engineering Co-Op'</v>
+      </c>
+      <c r="C330" t="str">
+        <v>2026-09-24 ~07:00 UTC: new site found via a research agent; posting states a single combined 'Spring/Summer 2027' term with no separate Spring-only or distinct-dates language (unlike the Hermeus/RTX Windsor Locks postings that explicitly split Spring and Summer into separately-dated options) — fails the season-stated bar as a merged term, same basis as prior combined-term exclusions (Saab, Moog). Not added.</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>GE Aerospace (Evendale, OH)</v>
+      </c>
+      <c r="B331" t="str">
+        <v>'Manufacturing Engineering Co-op – US – Spring 2027' reqs R5030077 and R5029663</v>
+      </c>
+      <c r="C331" t="str">
+        <v>2026-09-24 ~07:00 UTC re-check: R5030077 confirmed HTTP 410 Gone; R5029663 page states 'the job you are looking for is no longer posted.' Consistent with prior runs' findings that these are dead/duplicate-of-tracked. No change.</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>Honda (Lincoln, AL)</v>
+      </c>
+      <c r="B332" t="str">
+        <v>'Engineering Co-op/Intern - Spring 2027'</v>
+      </c>
+      <c r="C332" t="str">
+        <v>2026-09-24 ~07:00 UTC: new company found via national sweep. Fetched directly (careers.honda.com/us/en/job/10993) — page explicitly states 'This position is no longer accepting applications.' Not added.</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B333" t="str">
+        <v>'Spring 2027 Guidance, Navigation &amp; Control (GNC) Internship – Undergraduate', req R66295</v>
+      </c>
+      <c r="C333" t="str">
+        <v>2026-09-24 ~07:00 UTC: new req found via national sweep. Confirmed closed via this session's own direct fetch of the Workday job page embed (postingAvailable: false). Not added.</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B334" t="str">
+        <v>'Spring 2027 Electrical Systems Engineering Internship – Graduate', req R66224</v>
+      </c>
+      <c r="C334" t="str">
+        <v>2026-09-24 ~07:00 UTC: new req found via national sweep. Electrical Engineering discipline, not mechanical/aerospace/manufacturing/robotics/controls — excluded on discipline grounds regardless of open/closed status. Not added.</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>WestRock / Smurfit Westrock</v>
+      </c>
+      <c r="B335" t="str">
+        <v>'Manufacturing Engineering Co-op – Spring 2027, Mills' (Cowpens, SC and other mill locations)</v>
+      </c>
+      <c r="C335" t="str">
+        <v>2026-09-24 ~07:00 UTC: new company found via aggregator listings (LinkedIn, talent.com). Neither a research agent nor this session's own direct fetch of Smurfit Westrock's Avature careers portal could open the live individual posting (404s / portal didn't expose it). Not added — unresolved, worth a fresh attempt with a different access method next run.</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>Fives</v>
+      </c>
+      <c r="B336" t="str">
+        <v>'Manufacturing Engineering Co-Op Spring 2027' (Hebron, KY)</v>
+      </c>
+      <c r="C336" t="str">
+        <v>2026-09-24 ~07:00 UTC: new company found only via a job-board aggregator (Workopia); neither a research agent nor this session's own direct fetch of fivesgroup.com's careers page could locate or open the live posting (404). Not added — unresolved, worth a fresh attempt next run.</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>Textron Systems (Hunt Valley, MD)</v>
+      </c>
+      <c r="B337" t="str">
+        <v>'2027 Intern - Mechanical Engineer (Sea Systems)', re-check</v>
+      </c>
+      <c r="C337" t="str">
+        <v>2026-09-24 ~07:00 UTC: a research agent searched Textron Systems' live 'apply today' board of 280 current openings and did not find this posting — likely closed/filled/removed, though not independently confirmed via direct fetch (JS-rendered site). Season was never confirmed as Spring/Winter-qualified in any prior run either. Not added.</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>Parker Hannifin (Columbus, OH)</v>
+      </c>
+      <c r="B338" t="str">
+        <v>'Design Engineering Co-Op', re-check</v>
+      </c>
+      <c r="C338" t="str">
+        <v>2026-09-24 ~07:00 UTC: jobs.parker.com remained unreachable (DNS/proxy blocked) from this session; only a stale Spring 2026 LinkedIn listing and generic aggregator mentions found. No change — still no live posting located across multiple runs now.</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>Analog Devices / Lam Research</v>
+      </c>
+      <c r="B339" t="str">
+        <v>re-check</v>
+      </c>
+      <c r="C339" t="str">
+        <v>2026-09-24 ~07:00 UTC: no Winter 2026/Spring 2027 postings found at either company. No change — recurring null result across many runs now.</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>Impulse Space (Redondo Beach, CA)</v>
+      </c>
+      <c r="B340" t="str">
+        <v>re-check for a Spring-2027-dated mechanical/propulsion/structures req</v>
+      </c>
+      <c r="C340" t="str">
+        <v>2026-09-24 ~07:00 UTC: all current engineering internship postings (Propulsion, Avionics Mechanical, Opto-Mechanical, Electric Propulsion) are explicitly Summer 2027 only. No Spring 2027 posting found. No change.</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>MKS Instruments (Andover, MA)</v>
+      </c>
+      <c r="B341" t="str">
+        <v>'Mechanical' + 'Spring 2027' search, re-check</v>
+      </c>
+      <c r="C341" t="str">
+        <v>2026-09-24 ~07:00 UTC: this session's own direct query of MKS's own Workday CXS API found zero matching Spring 2027 mechanical postings at Andover — corrects an earlier unsupported aggregator-summary claim of a live MKS mechanical posting. No change.</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B342" t="str">
+        <v>'Co-op: Manufacturing Engineering' and 'Co-op Design Engineering' (Spring 2027), re-check</v>
+      </c>
+      <c r="C342" t="str">
+        <v>2026-09-24 ~07:00 UTC: multiple independent aggregators (LinkedIn, Fairygodboss, Glassdoor, ZipRecruiter) continue to consistently describe both Spring 2027 co-op titles with matching pay ($22.15–$27.69/hr), suggesting the roles may still exist, but the primary source remains blocked (eaton.eightfold.ai API returned 403 'Not authorized', LinkedIn/Fairygodboss mirrors unreachable). Not added — still unresolved, worth a fresh attempt with a different access method.</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>GD Electric Boat (Groton, CT)</v>
+      </c>
+      <c r="B343" t="str">
+        <v>req 601496955, re-check</v>
+      </c>
+      <c r="C343" t="str">
+        <v>2026-09-24 ~07:00 UTC: direct connection to jobs.gd-eb.com was rejected at the network/proxy level before reaching Cloudflare — 18th+ consecutive block. Still needs a human in-browser check.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C327"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C343"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 25 new postings, 5 checked-excluded (2026-09-24 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EmGmwqndnZzf5oJkgFyvjE
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M155"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -4729,6 +4729,806 @@
       </c>
       <c r="J130" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, a distinct site (Los Angeles) from the Atlanta Manufacturing Engineering Intern req above.</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Spring 2027 (~6 months)</v>
+      </c>
+      <c r="E131" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F131">
+        <v>25</v>
+      </c>
+      <c r="G131" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H131" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Manufacturing-Engineering-Co-Op_REQ-14492</v>
+      </c>
+      <c r="I131" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API, HTTP 200, description explicitly states 'Spring 2027 season.'</v>
+      </c>
+      <c r="J131" t="str">
+        <v>New sibling req to the already-tracked Entegris Billerica co-ops (different REQ range than a previously-excluded stale REQ-7046 series). Supports process engineers on the Billerica filter manufacturing line.</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Fives</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E132" t="str">
+        <v>Hebron, KY</v>
+      </c>
+      <c r="F132">
+        <v>900</v>
+      </c>
+      <c r="G132" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H132" t="str">
+        <v>https://career.fivesgroup.com/job/Hebron-Manufacturing-Engineering-Co-Op-Spring-2027-Kent-41048/1362251655/</v>
+      </c>
+      <c r="I132" t="str">
+        <v>Yes — fetched directly on career.fivesgroup.com (Fives's own site, not an aggregator), HTTP 200, 'Apply Now' active, 'Spring 2027' stated in title/body.</v>
+      </c>
+      <c r="J132" t="str">
+        <v>Resolves a block that persisted across multiple prior runs (site previously only found via an aggregator mirror, never opened directly).</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B133" t="str">
+        <v>Manufacturing Engineering Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Winter/Spring 2027 (January–April/June)</v>
+      </c>
+      <c r="E133" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F133">
+        <v>3</v>
+      </c>
+      <c r="G133" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H133" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8161817</v>
+      </c>
+      <c r="I133" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: January - April/June 2027.'</v>
+      </c>
+      <c r="J133" t="str">
+        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Hardware R&amp;D Engineering Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Mechanical/Hardware Engineering</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Winter/Spring 2027 (January–April)</v>
+      </c>
+      <c r="E134" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F134">
+        <v>3</v>
+      </c>
+      <c r="G134" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H134" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172226</v>
+      </c>
+      <c r="I134" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
+      </c>
+      <c r="J134" t="str">
+        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B135" t="str">
+        <v>Materials Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Materials Engineering</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Winter/Spring 2027 (January–April)</v>
+      </c>
+      <c r="E135" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F135">
+        <v>3</v>
+      </c>
+      <c r="G135" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H135" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199092</v>
+      </c>
+      <c r="I135" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
+      </c>
+      <c r="J135" t="str">
+        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Mission Systems Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
+      </c>
+      <c r="E136" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F136">
+        <v>950</v>
+      </c>
+      <c r="G136" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H136" t="str">
+        <v>https://jobs.lever.co/hermeus/9229aa88-f54d-4ecd-85ee-b31f53b4207d</v>
+      </c>
+      <c r="I136" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring (Jan–Apr) vs Summer (May–Aug) dated slots.</v>
+      </c>
+      <c r="J136" t="str">
+        <v>Mix of hardware and software systems-integration work; included under Hamza's aerospace/systems discipline.</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Flight Operations &amp; Airworthiness Engineering Intern (Spring/Summer/Fall 2027)</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Flight Systems</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+      </c>
+      <c r="E137" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F137">
+        <v>950</v>
+      </c>
+      <c r="G137" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H137" t="str">
+        <v>https://jobs.lever.co/hermeus/944918b0-17ca-46ec-9413-5acd7086addf</v>
+      </c>
+      <c r="I137" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring/Summer/Fall 2027 dated slots.</v>
+      </c>
+      <c r="J137" t="str">
+        <v>New discipline not previously tracked at Hermeus; on experimental high-performance aircraft flight test/airworthiness.</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Additive Manufacturing Intern, Spring 2027</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F138">
+        <v>2600</v>
+      </c>
+      <c r="G138" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H138" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7983576003</v>
+      </c>
+      <c r="I138" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J138" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Combustion Devices Intern, Spring 2027</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Propulsion Engineering</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F139">
+        <v>2600</v>
+      </c>
+      <c r="G139" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H139" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986744003</v>
+      </c>
+      <c r="I139" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J139" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Fluid Component Intern, Spring 2027</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E140" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F140">
+        <v>2600</v>
+      </c>
+      <c r="G140" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H140" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990367003</v>
+      </c>
+      <c r="I140" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J140" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Fluid Systems Intern, Spring 2027</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F141">
+        <v>2600</v>
+      </c>
+      <c r="G141" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H141" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986788003</v>
+      </c>
+      <c r="I141" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J141" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Integration &amp; Test Intern, Spring 2027</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F142">
+        <v>2600</v>
+      </c>
+      <c r="G142" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H142" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987252003</v>
+      </c>
+      <c r="I142" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J142" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Manufacturing Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F143">
+        <v>2600</v>
+      </c>
+      <c r="G143" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H143" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7984943003</v>
+      </c>
+      <c r="I143" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J143" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026; sibling reqs also open at Middle River, MD and Wallops Island, VA (see below).</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Manufacturing Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C144" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E144" t="str">
+        <v>Middle River, MD</v>
+      </c>
+      <c r="F144">
+        <v>400</v>
+      </c>
+      <c r="G144" t="str">
+        <v>$25/hr</v>
+      </c>
+      <c r="H144" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987020003</v>
+      </c>
+      <c r="I144" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J144" t="str">
+        <v>Sibling req to the Long Beach, CA and Wallops Island, VA Manufacturing Engineering Intern postings.</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Manufacturing Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E145" t="str">
+        <v>Wallops Island, VA</v>
+      </c>
+      <c r="F145">
+        <v>450</v>
+      </c>
+      <c r="G145" t="str">
+        <v>$25/hr</v>
+      </c>
+      <c r="H145" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996617003</v>
+      </c>
+      <c r="I145" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J145" t="str">
+        <v>Sibling req to the Long Beach, CA and Middle River, MD Manufacturing Engineering Intern postings.</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Mechanical Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E146" t="str">
+        <v>Silver Spring, MD</v>
+      </c>
+      <c r="F146">
+        <v>440</v>
+      </c>
+      <c r="G146" t="str">
+        <v>$25/hr</v>
+      </c>
+      <c r="H146" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7989995003</v>
+      </c>
+      <c r="I146" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J146" t="str">
+        <v>Distinct site from the already-tracked Long Beach, CA Mechanical Engineering Intern req.</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Propulsion Analyst Intern, Spring 2027</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Propulsion Engineering</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E147" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F147">
+        <v>2600</v>
+      </c>
+      <c r="G147" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H147" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986824003</v>
+      </c>
+      <c r="I147" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J147" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Propulsion Design Intern, Spring 2027</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Propulsion Engineering</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E148" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F148">
+        <v>2600</v>
+      </c>
+      <c r="G148" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H148" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987110003</v>
+      </c>
+      <c r="I148" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J148" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Propulsion Intern, Spring 2027</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Propulsion Engineering</v>
+      </c>
+      <c r="D149" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E149" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F149">
+        <v>2600</v>
+      </c>
+      <c r="G149" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H149" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986790003</v>
+      </c>
+      <c r="I149" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J149" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Structural Analysis Intern, Spring 2027</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E150" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F150">
+        <v>2600</v>
+      </c>
+      <c r="G150" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H150" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986685003</v>
+      </c>
+      <c r="I150" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J150" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Test Engineering Intern - Manufacturing, Spring 2027</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E151" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F151">
+        <v>2600</v>
+      </c>
+      <c r="G151" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H151" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987042003</v>
+      </c>
+      <c r="I151" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J151" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Test Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D152" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E152" t="str">
+        <v>Stennis Space Center, MS</v>
+      </c>
+      <c r="F152">
+        <v>1500</v>
+      </c>
+      <c r="G152" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H152" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990352003</v>
+      </c>
+      <c r="I152" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season confirmed in body; pay range not found in content.</v>
+      </c>
+      <c r="J152" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Thermal Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E153" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F153">
+        <v>2600</v>
+      </c>
+      <c r="G153" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H153" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8000951003</v>
+      </c>
+      <c r="I153" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J153" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Turbomachinery Intern, Spring 2027</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Propulsion Engineering</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E154" t="str">
+        <v>Long Beach, CA</v>
+      </c>
+      <c r="F154">
+        <v>2600</v>
+      </c>
+      <c r="G154" t="str">
+        <v>$28/hr</v>
+      </c>
+      <c r="H154" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987210003</v>
+      </c>
+      <c r="I154" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J154" t="str">
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B155" t="str">
+        <v>R&amp;D Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Materials Engineering</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E155" t="str">
+        <v>Albuquerque, NM</v>
+      </c>
+      <c r="F155">
+        <v>2200</v>
+      </c>
+      <c r="G155" t="str">
+        <v>$20/hr</v>
+      </c>
+      <c r="H155" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996578003</v>
+      </c>
+      <c r="I155" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+      </c>
+      <c r="J155" t="str">
+        <v>Materials/manufacturing-process R&amp;D on phase-change materials for solar arrays (constellation programs).</v>
       </c>
     </row>
   </sheetData>
@@ -4776,14 +5576,14 @@
     <hyperlink ref="M19" r:id="rId41"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M130"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M155"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C343"/>
+  <dimension ref="A1:C348"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -8425,10 +9225,10 @@
         <v>GE Aerospace (Evendale, OH)</v>
       </c>
       <c r="B331" t="str">
-        <v>'Manufacturing Engineering Co-op – US – Spring 2027' reqs R5030077 and R5029663</v>
+        <v>'Manufacturing Engineering Co-op – US – Spring 2027' req R5030077 (a distinct req from the already-tracked R5029663)</v>
       </c>
       <c r="C331" t="str">
-        <v>2026-09-24 ~07:00 UTC re-check: R5030077 confirmed HTTP 410 Gone; R5029663 page states 'the job you are looking for is no longer posted.' Consistent with prior runs' findings that these are dead/duplicate-of-tracked. No change.</v>
+        <v>2026-09-24 ~07:00 UTC re-check: R5030077 confirmed HTTP 410 Gone. CORRECTION (2026-09-24 ~13:00 UTC): the same 07:00 UTC entry incorrectly also claimed req R5029663 was dead ('no longer posted') — this was an error. R5029663 is the already-tracked live `rows` entry; this session's own direct Workday CXS API query just now returned canApply: true, posted: true, with 30+ days left to apply, and the description also lists Lynn, MA among many eligible sites. R5029663 remains correctly live in `rows`, unchanged.</v>
       </c>
     </row>
     <row r="332">
@@ -8563,9 +9363,64 @@
         <v>2026-09-24 ~07:00 UTC: direct connection to jobs.gd-eb.com was rejected at the network/proxy level before reaching Cloudflare — 18th+ consecutive block. Still needs a human in-browser check.</v>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B344" t="str">
+        <v>Industrial Design Intern (Winter/Spring 2027), Somerville MA</v>
+      </c>
+      <c r="C344" t="str">
+        <v>2026-09-24 ~13:00 UTC: confirmed live via direct Greenhouse API fetch (season/location correct), but discipline is product/industrial design, not industrial engineering or Hamza's other target disciplines — excluded on discipline grounds.</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B345" t="str">
+        <v>Mechanical Engineer Intern (Winter 2027), San Francisco CA, job 4704600006</v>
+      </c>
+      <c r="C345" t="str">
+        <v>2026-09-24 ~13:00 UTC: confirmed live and open via direct Greenhouse fetch, but season is stated as 'Winter 2027' specifically — not Winter 2026 or Spring 2027 as required. Excluded on season grounds (the already-tracked sibling req 4704602006 is the correct Spring 2027 posting).</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B346" t="str">
+        <v>Full Greenhouse API sweep of all 35 current 'Spring 2027' titled reqs</v>
+      </c>
+      <c r="C346" t="str">
+        <v>2026-09-24 ~13:00 UTC: this session queried Rocket Lab's own Greenhouse jobs API directly for every open 'Spring 2027' req company-wide. 18 matching Hamza's target disciplines were added to `rows` (see Manufacturing/Mechanical/Propulsion/Structural/Thermal/Systems/Materials Intern entries). The remaining 17 were excluded on discipline grounds (all confirmed live, just off-target): Business Development Intern, Electrical Engineering Intern (Toronto, CAN — also non-US), Mechanical Engineering Intern (Toronto, CAN — non-US location), Flight Software Intern (software, not hardware), Indirect Procurement Intern, Logistics Intern, People &amp; Culture Intern, Security Analyst Intern (x4: Long Beach CA, Albuquerque NM, Wallops Island VA, Middle River MD), Supply Chain Intern (x4: Middle River MD, Tucson AZ, Silver Spring MD, Long Beach CA).</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>Entegris (Billerica, MA)</v>
+      </c>
+      <c r="B347" t="str">
+        <v>Full re-sweep of current Billerica reqs beyond the 6 already tracked</v>
+      </c>
+      <c r="C347" t="str">
+        <v>2026-09-24 ~13:00 UTC: this session's own direct Workday CXS API query of REQ-14457/14492/14497/14444/14469/14462/14504 confirmed all are live Spring 2027 postings; REQ-14492 (Manufacturing Engineering Co-Op) was the one not yet tracked — ADDED to `rows`. The other 5 were already tracked from prior runs. No further untracked Billerica reqs found.</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>Textron Systems (Hunt Valley, MD)</v>
+      </c>
+      <c r="B348" t="str">
+        <v>'2027 Intern - Mechanical Engineer (Sea Systems)', final re-check</v>
+      </c>
+      <c r="C348" t="str">
+        <v>2026-09-24 ~13:00 UTC: a research agent swept Textron Systems' full live 'apply today' board (280 current openings) — this posting is not among them. Combined with the season never having been confirmed as Spring/Winter in any prior run, treating this as resolved/closed; dropping from the active watch list unless a fresh sibling req surfaces.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C343"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C348"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 8 new postings, 6 checked-excluded (2026-09-24 19:00 UTC)
Also upgrades GD Electric Boat's 19-run-blocked Partial entry to a
fully-verified working link.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XdpriwEAWAGpDzLDcq4V5y
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M155"/>
+  <dimension ref="A1:M163"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -1510,10 +1510,10 @@
         <v>2027 Spring Engineering CO-OP Trainee</v>
       </c>
       <c r="C30" t="str">
-        <v>Mechanical / Structural / Aerospace-Aeronautical / Systems / Naval Architecture / Industrial / Electromechanical / Robotics Engineering (multi-discipline req)</v>
+        <v>Mechanical / Structural / Aerospace-Aeronautical / Marine-Ocean / Systems / Nuclear / Naval Architecture / Electromechanical / Robotics / Industrial Engineering (multi-discipline req; students placed into orgs incl. Platform Systems, Ship Signatures, Fluid Systems, Propulsion Plant Structures/Fluid Systems, Hull &amp; External Structures, Solid Mechanics)</v>
       </c>
       <c r="D30" t="str">
-        <v>Spring of 2027 (per listing summary)</v>
+        <v>Spring 2027 academic semester, full-time 4-6 month co-op for academic credit (posting explicitly states 'not a summer internship')</v>
       </c>
       <c r="E30" t="str">
         <v>Groton, CT (co-ops also placed in New London/North Stonington CT, North Kingstown/Newport RI)</v>
@@ -1525,13 +1525,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H30" t="str">
-        <v>https://jobs.buildsubmarines.com/job/601496955</v>
+        <v>https://www.gd.com/careers/2027-spring-engineering-co-op-trainee-groton-ct-us-2026-20763-eb-opportunity (apply via https://www.click2apply.net/5JaLBlcYpVYVJC1xkCgV8a)</v>
       </c>
       <c r="I30" t="str">
-        <v>Partial — found via GD Electric Boat's own dedicated recruiting site (jobs.buildsubmarines.com) with a specific req ID, mirroring the pattern of GD's known 2026 cycle req. The page itself is behind a Cloudflare bot-check wall — blocked on WebFetch, curl w/ browser UA, and a reader-proxy fetch, all returning a security-verification/CAPTCHA screen. Could not independently confirm live/open status or the exact discipline breakdown. Verify live in-browser before applying.</v>
+        <v>Yes — upgraded 2026-09-24 ~19:00 UTC: independently fetched directly via curl with a browser user-agent (HTTP 200, no Cloudflare block on this gd.com-hosted mirror, unlike the buildsubmarines.com portal). Full job description confirmed: req 2026-20763, Spring 2027 academic semester, US citizenship required, disciplines and eligibility all verbatim-confirmed from the live page text.</v>
       </c>
       <c r="J30" t="str">
-        <v>Was flagged 'worth re-checking' in the prior run; upgraded from 'no verifiable link' to 'specific req ID found, still blocked'.</v>
+        <v>This is the same role/title as the long-blocked jobs.buildsubmarines.com req 601496955 (still Cloudflare-blocked as of this run, 20+ consecutive fails) — likely the identical opportunity mirrored on GD's own corporate site under a different req numbering scheme (2026-20763). Using this working link going forward. US citizenship required; no remote option; not a summer internship.</v>
       </c>
     </row>
     <row r="31">
@@ -5529,6 +5529,262 @@
       </c>
       <c r="J155" t="str">
         <v>Materials/manufacturing-process R&amp;D on phase-change materials for solar arrays (constellation programs).</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Manufacturing Engineer Co-Op</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D156" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E156" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F156">
+        <v>17</v>
+      </c>
+      <c r="G156" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H156" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Manufacturing-Engineer-Co-Op_REQ-14484</v>
+      </c>
+      <c r="I156" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J156" t="str">
+        <v>REQ-14484. New Entegris site for the tracker (Bedford, in addition to the 7 already-tracked Billerica reqs).</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Design and Process Engineering Co-Op</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Mechanical / Process Engineering</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E157" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F157">
+        <v>17</v>
+      </c>
+      <c r="G157" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H157" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Design-and-Process-Engineering-Co-Op_REQ-14491</v>
+      </c>
+      <c r="I157" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J157" t="str">
+        <v>REQ-14491. Bedford, MA sibling req.</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Industrial Engineering Co-Op</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Industrial Engineering</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E158" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F158">
+        <v>17</v>
+      </c>
+      <c r="G158" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H158" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14465</v>
+      </c>
+      <c r="I158" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J158" t="str">
+        <v>REQ-14465. Bedford, MA sibling req; a second, distinct Industrial Engineering Co-Op req (REQ-14452) was also found open at the same site — see next row.</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Industrial Engineering Co-Op</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Industrial Engineering</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E159" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F159">
+        <v>17</v>
+      </c>
+      <c r="G159" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H159" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14452</v>
+      </c>
+      <c r="I159" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J159" t="str">
+        <v>REQ-14452. Distinct req from the identically-titled REQ-14465 above (same site/title, separate req IDs) — both independently confirmed open, not a duplicate.</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Process Engineering Co-Op</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Process / Manufacturing Engineering</v>
+      </c>
+      <c r="D160" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E160" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F160">
+        <v>17</v>
+      </c>
+      <c r="G160" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H160" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Process-Engineering-Co-Op_REQ-14458</v>
+      </c>
+      <c r="I160" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J160" t="str">
+        <v>REQ-14458. Bedford, MA sibling req.</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Reliability Engineer Co-Op</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Reliability / Mechanical Engineering</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Spring 2027 season (6-month assignment)</v>
+      </c>
+      <c r="E161" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F161">
+        <v>17</v>
+      </c>
+      <c r="G161" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H161" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Reliability-Engineer-Co-Op_REQ-14399</v>
+      </c>
+      <c r="I161" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+      </c>
+      <c r="J161" t="str">
+        <v>REQ-14399. Bedford, MA sibling req.</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>MetOx International</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Mechanical Engineering Co-Op/Intern</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Spring/Summer 2027 (Internship: part-time Spring 2027 + full-time Summer 2027) or Co-Op: full-time January-August 2027</v>
+      </c>
+      <c r="E162" t="str">
+        <v>Houston, TX</v>
+      </c>
+      <c r="F162">
+        <v>1600</v>
+      </c>
+      <c r="G162" t="str">
+        <v>Not stated on posting (non-local co-op candidates eligible for a monthly stipend)</v>
+      </c>
+      <c r="H162" t="str">
+        <v>https://job-boards.greenhouse.io/metoxinternationalinc/jobs/5405775008</v>
+      </c>
+      <c r="I162" t="str">
+        <v>Yes — fetched directly via Greenhouse (HTTP 200), full description confirms title, season options, and an active Apply button.</v>
+      </c>
+      <c r="J162" t="str">
+        <v>New company for the tracker — superconducting-technology energy startup. SolidWorks/FEA/CFD-focused mechanical design role, Balance-of-Plant systems. Co-Op option begins January 2027 (Spring start), included per the same 'distinct dated Spring option within a combined-term posting' treatment as Hermeus.</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>Sanofi</v>
+      </c>
+      <c r="B163" t="str">
+        <v>2027 Spring Co-op Opportunities (incl. Engineering &amp; Maintenance / HSE / Reliability tracks)</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Mechanical / Industrial / Reliability / Process Engineering (umbrella posting, multiple functional tracks)</v>
+      </c>
+      <c r="D163" t="str">
+        <v>Spring 2027, starting January 2027, 6-month duration</v>
+      </c>
+      <c r="E163" t="str">
+        <v>Swiftwater, PA</v>
+      </c>
+      <c r="F163">
+        <v>270</v>
+      </c>
+      <c r="G163" t="str">
+        <v>$32-$35/hour</v>
+      </c>
+      <c r="H163" t="str">
+        <v>https://jobs.sanofi.com/en/job/swiftwater/2027-spring-co-op-opportunities-swiftwater-pa/2649/41259827904</v>
+      </c>
+      <c r="I163" t="str">
+        <v>Yes — fetched directly via jobs.sanofi.com (Sanofi's own site, not an aggregator), confirmed live with an active 'Apply Now' button, pay and dates confirmed in body.</v>
+      </c>
+      <c r="J163" t="str">
+        <v>Umbrella-style posting, same pattern as the already-tracked Sanofi/Genzyme Framingham row — multiple near-identical parallel req IDs found on job-board mirrors (biospace.com job 3075194 'Engineering &amp; Maintenance' track at $35/hr, plus others at 3075170/3062903/3069311) likely representing different functional tracks of the same 2027 Spring Co-op program. Requires permanent US work authorization without sponsorship. Distinct from the already-tracked Sanofi (Genzyme) Framingham, MA row.</v>
       </c>
     </row>
   </sheetData>
@@ -5576,14 +5832,14 @@
     <hyperlink ref="M19" r:id="rId41"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M155"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M163"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C348"/>
+  <dimension ref="A1:C354"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -9418,9 +9674,75 @@
         <v>2026-09-24 ~13:00 UTC: a research agent swept Textron Systems' full live 'apply today' board (280 current openings) — this posting is not among them. Combined with the season never having been confirmed as Spring/Winter in any prior run, treating this as resolved/closed; dropping from the active watch list unless a fresh sibling req surfaces.</v>
       </c>
     </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Entegris (Bedford, MA)</v>
+      </c>
+      <c r="B349" t="str">
+        <v>'Mechanical Engineering Co-Op', REQ-14401</v>
+      </c>
+      <c r="C349" t="str">
+        <v>2026-09-24 ~19:00 UTC: this session's own direct Workday CXS API fetch confirms this req is live (canApply true), but the posting text is internally contradictory on season — it states the assignment is 'for the Fall 2026 season' in one place, but the eligibility section separately says 'beginning in January through June' (a Spring-dated window). Given this direct conflict and no way to resolve which is authoritative, excluding rather than guessing which season actually applies — worth a fresh look next run to see if the posting has been corrected. (The 6 other new Bedford, MA Spring-2027-stated Entegris co-ops found this run had no such contradiction and were added to `rows`.)</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>iRobot (Bedford, MA)</v>
+      </c>
+      <c r="B350" t="str">
+        <v>'Mechanical Engineering Intern - Innovation (Spring/Summer)', req R4085</v>
+      </c>
+      <c r="C350" t="str">
+        <v>2026-09-24 ~19:00 UTC: located a specific req number for the first time (via web search of iRobot's own Workday tenant, irobot.wd503.myworkdayjobs.com) at Bedford, MA — a Boston-area, on-target-discipline lead. However, this session's own direct Workday CXS API fetch and WebFetch both returned blocked/empty responses (403 permission denied), so neither the live/open status nor whether 'Spring' is a distinct, separately-dated option (vs. a merged Spring/Summer term, which would fail the season bar per prior treatment of combined-term postings) could be confirmed. Not added — worth a fresh direct-fetch attempt next run now that the exact req/URL is on record.</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>GE Vernova</v>
+      </c>
+      <c r="B351" t="str">
+        <v>'Power Conversion &amp; Storage Engineering Intern/Co-Op - Spring 2027', Findlay Township, PA</v>
+      </c>
+      <c r="C351" t="str">
+        <v>2026-09-24 ~19:00 UTC: this session confirmed the Summer 2027 sibling req (R5050017) is genuinely live on careers.gevernova.com, and multiple independent aggregators (Dreamwork, Workopia, Zapply) consistently describe an identically-detailed Spring 2027 version ($21-$34/hr, Jan-Apr, Findlay Township PA) — but extensive direct searching could not turn up the actual req ID or a working careers.gevernova.com URL for the Spring variant specifically (site search is JS-rendered, direct URL guesses 404'd). Not added without a verifiable direct link — worth another attempt next run, ideally via a research agent with different tooling.</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>WestRock / Smurfit Westrock (Cowpens, SC)</v>
+      </c>
+      <c r="B352" t="str">
+        <v>'Manufacturing Engineering Co-op - Spring 2027, Mills', re-check</v>
+      </c>
+      <c r="C352" t="str">
+        <v>2026-09-24 ~19:00 UTC: the specific LinkedIn posting cited by aggregators (job ID 4413763900) now redirects to a generic LinkedIn job-search page rather than showing the posting itself — the same signature multiple prior runs have seen on other companies' listings that turned out to be expired/removed. Smurfit Westrock's own Avature portal remains a non-scrapable JS shell. Still not independently confirmed either way; leaning toward likely closed/removed but not certain enough to declare dead. No change to active-watch status, deprioritizing further automated attempts.</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B353" t="str">
+        <v>'Co-op Design Engineering' / 'Co-op: Manufacturing Engineering' (Spring 2027), re-check</v>
+      </c>
+      <c r="C353" t="str">
+        <v>2026-09-24 ~19:00 UTC: eaton.eightfold.ai and eaton.dejobs.org both still return JS-shell/blocked responses; the specific Fairygodboss and LinkedIn URLs used in the prior run's aggregator evidence now 404 or redirect to generic search pages. No independently verifiable live posting found this run either. No change — still unresolved across many consecutive runs.</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>Parker Hannifin (Columbus, OH)</v>
+      </c>
+      <c r="B354" t="str">
+        <v>'Design Engineering Co-Op', re-check</v>
+      </c>
+      <c r="C354" t="str">
+        <v>2026-09-24 ~19:00 UTC: jobs.parker.com still returns a DNS resolution failure (getaddrinfo ENOTFOUND) and www.parker.com/us/en/careers.html returns HTTP 403 from this session. No change — still unreachable across many consecutive runs.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C348"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C354"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 9 new postings, 4 checked-excluded (2026-09-25 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AEfHQuetD1VuzoGuAvpCsP
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M163"/>
+  <dimension ref="A1:M172"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -5785,6 +5785,294 @@
       </c>
       <c r="J163" t="str">
         <v>Umbrella-style posting, same pattern as the already-tracked Sanofi/Genzyme Framingham row — multiple near-identical parallel req IDs found on job-board mirrors (biospace.com job 3075194 'Engineering &amp; Maintenance' track at $35/hr, plus others at 3075170/3062903/3069311) likely representing different functional tracks of the same 2027 Spring Co-op program. Requires permanent US work authorization without sponsorship. Distinct from the already-tracked Sanofi (Genzyme) Framingham, MA row.</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>Marathon Petroleum</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Intern/Co-op - Midstream Logistics and Storage Mechanical/Civil/Electrical Engineering (Spring 2027)</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Mechanical / Civil / Electrical Engineering</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E164" t="str">
+        <v>Findlay, OH (+ Indianapolis, IN; La Palma, CA; Salt Lake City, UT)</v>
+      </c>
+      <c r="F164">
+        <v>700</v>
+      </c>
+      <c r="G164" t="str">
+        <v>$33.54-$42.45/hour</v>
+      </c>
+      <c r="H164" t="str">
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Findlay-Ohio/Intern-Co-op---Midstream-Logistics-and-Storage-Mechanical-Civil-Electrical-Engineering--Spring-2027-_00024207</v>
+      </c>
+      <c r="I164" t="str">
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024207, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
+      </c>
+      <c r="J164" t="str">
+        <v>New sibling req beyond the already-tracked Refining Mechanical Engineer (Spring 2027) req 00020137 at the same Findlay, OH site — this one covers the Logistics &amp; Storage organization (pipelines/marine transport).</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>Marathon Petroleum</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Intern/Co-op - Midstream Natural Gas and NGL Services Chemical/Mechanical/Civil/Petroleum/Electrical Engineering (Spring 2027)</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Mechanical / Chemical / Civil / Petroleum / Electrical Engineering</v>
+      </c>
+      <c r="D165" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E165" t="str">
+        <v>Canonsburg, PA (+ 12 other locations incl. Denver CO, Houston TX, Midland TX, Oklahoma City OK, Tulsa OK)</v>
+      </c>
+      <c r="F165">
+        <v>430</v>
+      </c>
+      <c r="G165" t="str">
+        <v>$33.54-$43.23/hour</v>
+      </c>
+      <c r="H165" t="str">
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Canonsburg-Pennsylvania/Intern-Co-op---Midstream-Natural-Gas-and-NGL-Services-Chemical-Mechanical-Civil-Petroleum-Electrical-Engineering--Spring-2027-_00024213</v>
+      </c>
+      <c r="I165" t="str">
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024213, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
+      </c>
+      <c r="J165" t="str">
+        <v>New sibling req beyond the already-tracked Marathon Petroleum entries — covers Natural Gas &amp; NGL Services (pipeline integrity, compressor/pump stations, automation/controls).</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>Rendezvous Robotics</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Mechanical Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Spring 2027 (12-15 weeks)</v>
+      </c>
+      <c r="E166" t="str">
+        <v>Golden, CO</v>
+      </c>
+      <c r="F166">
+        <v>1780</v>
+      </c>
+      <c r="G166" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H166" t="str">
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4329123009</v>
+      </c>
+      <c r="I166" t="str">
+        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
+      </c>
+      <c r="J166" t="str">
+        <v>New company for the tracker — small spacecraft-assembly startup (electromagnetic self-assembling tiles). First published 2026-07-22; still listed live on the board as of this run despite being ~2 months old.</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>Rendezvous Robotics</v>
+      </c>
+      <c r="B167" t="str">
+        <v>GNC Intern (Spring 2027)</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
+      </c>
+      <c r="D167" t="str">
+        <v>Spring 2027 (12-15 weeks)</v>
+      </c>
+      <c r="E167" t="str">
+        <v>Golden, CO</v>
+      </c>
+      <c r="F167">
+        <v>1780</v>
+      </c>
+      <c r="G167" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H167" t="str">
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332465009</v>
+      </c>
+      <c r="I167" t="str">
+        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
+      </c>
+      <c r="J167" t="str">
+        <v>Dynamics/controls of a reconfigurable spacecraft assembled from electromagnetically-docked tiles; open to aerospace/mechanical/electrical/physics majors with coursework in dynamics and controls — squarely a controls/flight-systems role, same treatment as the already-tracked Hermeus GNC intern.</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>Rendezvous Robotics</v>
+      </c>
+      <c r="B168" t="str">
+        <v>Manufacturing and Test Engineering Intern (Spring 2027)</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D168" t="str">
+        <v>Spring 2027 (per Greenhouse job title; the body text itself only states 'Golden, CO | Full-Time | 12-15 Weeks' with no season restated)</v>
+      </c>
+      <c r="E168" t="str">
+        <v>Golden, CO</v>
+      </c>
+      <c r="F168">
+        <v>1780</v>
+      </c>
+      <c r="G168" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H168" t="str">
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332082009</v>
+      </c>
+      <c r="I168" t="str">
+        <v>Partial — fetched directly via Greenhouse's own public API (HTTP 200 JSON); the official posting title is 'Manufacturing and Test Engineering Intern (Spring 2027)' but, unlike its 3 sibling Rendezvous Robotics postings, the job description body never restates 'Spring 2027' anywhere — season confirmation rests on the title alone.</v>
+      </c>
+      <c r="J168" t="str">
+        <v>Open to Mechanical/Electrical/Industrial Engineering majors; testbed development, manufacturing support, and hardware verification for spacecraft tiles.</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>Vast Space</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Emerging Talent - Mechanical/Aerospace Engineering Internship</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Mechanical / Aerospace Engineering</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
+      </c>
+      <c r="E169" t="str">
+        <v>Long Beach, CA (also hiring for Hawthorne, CA and Mojave, CA)</v>
+      </c>
+      <c r="F169">
+        <v>2600</v>
+      </c>
+      <c r="G169" t="str">
+        <v>$35-$42/hour</v>
+      </c>
+      <c r="H169" t="str">
+        <v>https://job-boards.greenhouse.io/vast/jobs/4711400006</v>
+      </c>
+      <c r="I169" t="str">
+        <v>Yes — fetched directly on Greenhouse; the application form's 'When are you available for an internship?' field is a dropdown containing 'Spring 2027' as its own distinct option (plus 'Summer: May 18 - Aug 6, 2027' / 'May 25 - Aug 13' / 'June 8 - Aug 27' / 'June 22 - Sept 10' and 'Fall 2027') — confirmed via the page's raw JSON, not just rendered text.</v>
+      </c>
+      <c r="J169" t="str">
+        <v>Previously excluded in 3 prior runs (2026-09-23) because the posting had no season/term field at all — this session's direct re-fetch found the application form now includes a genuine dated Spring 2027 option, same 'distinct dated Spring slot within a combined-term posting' treatment as Hermeus. ITAR: US person status required.</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>Vast Space</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Emerging Talent - Manufacturing Engineering Internship</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D170" t="str">
+        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
+      </c>
+      <c r="E170" t="str">
+        <v>Long Beach, CA (also hiring for Hawthorne, CA)</v>
+      </c>
+      <c r="F170">
+        <v>2600</v>
+      </c>
+      <c r="G170" t="str">
+        <v>$35-$42/hour</v>
+      </c>
+      <c r="H170" t="str">
+        <v>https://job-boards.greenhouse.io/vast/jobs/4711403006</v>
+      </c>
+      <c r="I170" t="str">
+        <v>Yes — fetched directly on Greenhouse; same 'When are you available for an internship?' dropdown with a distinct 'Spring 2027' option confirmed via the page's raw JSON, alongside the same 4 dated Summer 2027 ranges and Fall 2027.</v>
+      </c>
+      <c r="J170" t="str">
+        <v>Sibling req to the Mechanical/Aerospace Engineering Internship above, same site/pay/season structure.</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>Moog Inc.</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Intern, Design Engineering</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Mechanical / Aerospace Engineering (Air Vehicle Engineering)</v>
+      </c>
+      <c r="D171" t="str">
+        <v>Spring 2027 block intern</v>
+      </c>
+      <c r="E171" t="str">
+        <v>Mineral Wells, TX</v>
+      </c>
+      <c r="F171">
+        <v>1750</v>
+      </c>
+      <c r="G171" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H171" t="str">
+        <v>https://moog.wd5.myworkdayjobs.com/en-US/MOOG_External_Career_Site/job/Mineral-Wells-TX/Intern--Design-Engineering_R-26-19186</v>
+      </c>
+      <c r="I171" t="str">
+        <v>Yes — fetched directly via Moog's own Workday CXS API (HTTP 200 JSON), req R-26-19186, canApply true, posted 21 days ago, body states 'seeking a spring 2027 block intern' verbatim.</v>
+      </c>
+      <c r="J171" t="str">
+        <v>Corrects an earlier (2026-09-22) `checked` entry that had lumped this req in with 3 Summer-2027 Mineral Wells siblings (R-26-19881/19882/19887, which remain correctly excluded) — this session's fresh direct fetch shows R-26-19186 now/actually states Spring 2027, a different season from those siblings.</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Application Engineering Co-Op</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Applications / Process Engineering (Photo Applications)</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Spring 2027 season</v>
+      </c>
+      <c r="E172" t="str">
+        <v>Billerica, MA</v>
+      </c>
+      <c r="F172">
+        <v>17</v>
+      </c>
+      <c r="G172" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H172" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Application-Engineering-Co-Op_REQ-14473</v>
+      </c>
+      <c r="I172" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14473, canApply true, posted 15 days ago, body states 'Spring 2027' twice ('Spring 2027 to join our team' / 'Photo Applications team for the Spring 2027 season').</v>
+      </c>
+      <c r="J172" t="str">
+        <v>New sibling req beyond the 13 already-tracked Entegris Billerica/Bedford reqs, found via this session's own Entegris jobs-search API sweep (not from either research agent, who both mis-transcribed nearby req numbers — see ROUTINE-LOG for the correction).</v>
       </c>
     </row>
   </sheetData>
@@ -5832,14 +6120,14 @@
     <hyperlink ref="M19" r:id="rId41"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M163"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M172"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C354"/>
+  <dimension ref="A1:C358"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -8315,10 +8603,10 @@
         <v>Moog Inc. (Mineral Wells, TX)</v>
       </c>
       <c r="B225" t="str">
-        <v>'Air Vehicle Engineering'/Design/Hardware Design interns (R-26-19881/19882/19186/19887)</v>
+        <v>'Air Vehicle Engineering'/Design/Hardware Design interns (R-26-19881/19882/19887)</v>
       </c>
       <c r="C225" t="str">
-        <v>2026-09-22 ~19:00 UTC: all explicitly stated as Summer 2027 block interns in their posting text — wrong season, excluded.</v>
+        <v>2026-09-22 ~19:00 UTC: all explicitly stated as Summer 2027 block interns in their posting text — wrong season, excluded. CORRECTED 2026-09-25 ~01:00 UTC: this entry originally also listed sibling req R-26-19186 as Summer 2027, but this session's own direct Workday CXS re-fetch of R-26-19186 today shows it now explicitly states 'seeking a spring 2027 block intern' — a different season than its siblings. Removed from this exclusion group and added to `rows` as a verified Spring 2027 finding; R-26-19881/19882/19887 remain correctly excluded here as Summer 2027.</v>
       </c>
     </row>
     <row r="226">
@@ -9099,7 +9387,7 @@
         <v>'Emerging Talent - Mechanical/Aerospace Engineering Internship', re-check</v>
       </c>
       <c r="C296" t="str">
-        <v>2026-09-23 ~13:00 UTC: re-confirmed open via direct Greenhouse fetch and a full Greenhouse API sweep (zero other internship titles company-wide). Still no season/term field of any kind on the posting — fails the season-stated bar, unchanged from last run.</v>
+        <v>2026-09-23 ~13:00 UTC: re-confirmed open via direct Greenhouse fetch and a full Greenhouse API sweep (zero other internship titles company-wide). Still no season/term field of any kind on the posting — fails the season-stated bar, unchanged from last run. SUPERSEDED 2026-09-25 ~01:00 UTC: this session's own direct fetch of both the Mechanical/Aerospace and Manufacturing Engineering postings today found the application form's 'When are you available for an internship?' dropdown now includes a distinct 'Spring 2027' option alongside four dated Summer 2027 ranges and 'Fall 2027' — a genuine posting update since the last re-check, not present before. Both postings now pass the season-stated bar and were moved to `rows`.</v>
       </c>
     </row>
     <row r="297">
@@ -9740,9 +10028,53 @@
         <v>2026-09-24 ~19:00 UTC: jobs.parker.com still returns a DNS resolution failure (getaddrinfo ENOTFOUND) and www.parker.com/us/en/careers.html returns HTTP 403 from this session. No change — still unreachable across many consecutive runs.</v>
       </c>
     </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>Rendezvous Robotics</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Avionics Engineering Intern (Spring 2027), Golden CO, job 4329118009</v>
+      </c>
+      <c r="C355" t="str">
+        <v>2026-09-25 ~01:00 UTC: confirmed live via direct Greenhouse API fetch (title/season match), but the posting requires 'a degree in Electrical Engineering, Computer Engineering, or a related field' and is scoped to PCB design/power electronics/battery management — an EE discipline, not mechanical/aerospace/controls. Same treatment as the earlier Varda Space 'Avionics Engineering Internship' exclusion. Its 3 siblings (Mechanical Engineering, GNC, Manufacturing and Test Engineering Interns) do fit target disciplines and were added to `rows`.</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Moog Inc.</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Intern, Actuation Engineering (R-26-19536, Torrance CA); Intern, Engineering (R-26-19391, Buffalo/East Aurora NY)</v>
+      </c>
+      <c r="C356" t="str">
+        <v>2026-09-25 ~01:00 UTC: both confirmed live via direct Workday CXS API fetch (canApply true), and both explicitly say 'seeking a spring block intern' — but neither posting states a year anywhere in the description, unlike the now-confirmed R-26-19186 (Spring 2027) or the confirmed-Summer-2027 siblings. Cannot determine whether these are Spring 2026 or Spring 2027 cohorts; excluded pending a year being added to the posting. Worth a fresh look next run in case Moog updates the text.</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>Rocket Lab / Anduril Industries / ASM International / Owens Corning / Crown Equipment / Hermeus</v>
+      </c>
+      <c r="B357" t="str">
+        <v>Cross-check of every 'new' finding both research agents reported this run against the current `build.mjs`</v>
+      </c>
+      <c r="C357" t="str">
+        <v>2026-09-25 ~01:00 UTC: this session independently verified every reported 'new' req at these 6 companies and found all of them already tracked — Rocket Lab's reported 20-req Spring 2027 list matches the already-tracked 20 exactly (no new reqs beyond that wave); Anduril's reported 7-req 'Winter 2027' co-op cluster (Mechanical/Manufacturing/Propulsion/Systems/Test &amp; Evaluation/Warhead/EWIS Harness) matches the already-tracked 7 Anduril reqs exactly, same Greenhouse job IDs; ASM's Phoenix AZ Manufacturing Engineering Intern (job 4830098101), Owens Corning's Toledo OH Manufacturing Engineering Co-Op (req 70284, URL job id 1426905700), Crown Equipment's Greencastle IN Mechanical Engineering Co-op (URL job id 1420491100, req 146174), and Hermeus's Atlanta GA Structures/Mechanical Engineering Intern (Lever id 60b5d40a-1065-4bd2-8c72-6b2fb69d4761) are each byte-for-byte the same posting already in `rows`. None re-added.</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B358" t="str">
+        <v>'REQ-8386' (Capital Equipment Engineering Co-Op, Billerica MA), 'REQ-8392' (Manufacturing Engineering Co-Op), 'REQ-7124' (Materials Engineering Co-Op) as reported by a research agent</v>
+      </c>
+      <c r="C358" t="str">
+        <v>2026-09-25 ~01:00 UTC: none of these 3 req numbers exist — this session's own Entegris jobs-search API returned zero results for each. Cross-referencing by title/location instead found the real req numbers: Capital Equipment Engineering Co-Op at Billerica, MA is actually REQ-14497 (already tracked in `rows`); Manufacturing Engineering Co-Op at Billerica, MA is actually REQ-14492 (already tracked); Materials Engineering Co-Op is at Chaska, MN (REQ-14451), not a Massachusetts site at all — wrong location, not added. Same pattern as a prior run's 'REQ-7046' mis-transcription. This same search sweep did surface one genuinely new req — Application Engineering Co-Op, Billerica MA (REQ-14473) — added to `rows`.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C354"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C358"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
applications batch 1: relink rows 20-39, add Collins docs, fix duplicate-row link carryover
- Relink 17 rows (20, 22-27, 29-38) to existing batch 1/2 documents whose K/L/M links were lost
- Row 26 duplicates row 5 (same Formlabs posting), linked to the earlier files
- Skip row 21 (NASA Pathways, deadline passed) and row 28 (Eaton, must live near Syracuse, no relocation help)
- New resume, cover letter, and questions for row 39 (Collins Aerospace Project Engineering Co-op)
- build.mjs: match carried-over K/L/M on Company + Role + Application Link so sibling reqs
  with the same title (e.g. Rocket Lab in two cities) no longer share documents

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -1216,6 +1216,15 @@
       <c r="J20" t="str">
         <v>Housing/relocation assistance if 50+ mi from site. Must be work-authorized without sponsorship.</v>
       </c>
+      <c r="K20" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1245,6 +1254,15 @@
       <c r="J21" t="str">
         <v>US citizenship required. Cumulative GPA 2.9+ required. Spring 2027 window opens on USAJOBS in fall 2026.</v>
       </c>
+      <c r="K21" t="str">
+        <v>Skipped: application deadline was Sept 14, 2026 and has passed</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Skipped: application deadline was Sept 14, 2026 and has passed</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Skipped: application deadline was Sept 14, 2026 and has passed</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1277,6 +1295,15 @@
       <c r="J22" t="str">
         <v>Requires US citizenship + eligibility for Secret-level DoD clearance. Sibling req 'Microfabrication Engineering Co-Op' (same Jan–Aug 2027 window, Group 08-35) also exists but wasn't separately fetched.</v>
       </c>
+      <c r="K22" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1309,6 +1336,15 @@
       <c r="J23" t="str">
         <v>GAD division placement. Pay $20.00-$45.00/hr per posting.</v>
       </c>
+      <c r="K23" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1341,6 +1377,15 @@
       <c r="J24" t="str">
         <v>US Citizenship required — Draper cannot sponsor/hire H1B or Student Visa holders; dual citizens not eligible. CAD (Creo/SolidWorks), FEA (ANSYS/COMSOL) skills mentioned. Pay $20.00-$45.00/hr per posting.</v>
       </c>
+      <c r="K24" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -1373,6 +1418,15 @@
       <c r="J25" t="str">
         <v>Requires graduation between Dec 2026–Aug 2027. Prior req IDs for this role (e.g. 3088739, the 2026-cycle version) are confirmed dead (404).</v>
       </c>
+      <c r="K25" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1405,6 +1459,15 @@
       <c r="J26" t="str">
         <v>Boston metro. Portfolio of prior engineering work required — application not considered without one.</v>
       </c>
+      <c r="K26" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1437,6 +1500,15 @@
       <c r="J27" t="str">
         <v>Boston metro. Portfolio of prior engineering work required.</v>
       </c>
+      <c r="K27" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1469,6 +1541,15 @@
       <c r="J28" t="str">
         <v>Min GPA 2.8. No visa sponsorship (no CPT/OPT/H-1B support). Must live within ~50 mi of Syracuse, NY — no relocation assistance.</v>
       </c>
+      <c r="K28" t="str">
+        <v>Skipped: must live within about 50 miles of Syracuse, NY and there is no relocation help</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Skipped: must live within about 50 miles of Syracuse, NY and there is no relocation help</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Skipped: must live within about 50 miles of Syracuse, NY and there is no relocation help</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1501,6 +1582,15 @@
       <c r="J29" t="str">
         <v>Small modular-construction/robotics-manufacturing startup, Boston metro (Andover/Billerica). Shop-based role — CAD, welding, machining, fixturing.</v>
       </c>
+      <c r="K29" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1533,6 +1623,15 @@
       <c r="J30" t="str">
         <v>This is the same role/title as the long-blocked jobs.buildsubmarines.com req 601496955 (still Cloudflare-blocked as of this run, 20+ consecutive fails) — likely the identical opportunity mirrored on GD's own corporate site under a different req numbering scheme (2026-20763). Using this working link going forward. US citizenship required; no remote option; not a summer internship.</v>
       </c>
+      <c r="K30" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M30" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1565,6 +1664,15 @@
       <c r="J31" t="str">
         <v>Boston metro (Quincy). Corrects an earlier 'checked' entry for Anduril that only found Summer 2027 postings — this Winter 2027 cohort is a separate, later-posted cycle.</v>
       </c>
+      <c r="K31" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M31" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1597,6 +1705,15 @@
       <c r="J32" t="str">
         <v>Boston metro (Quincy). Same cohort/site as the Mechanical Engineer Co-op above.</v>
       </c>
+      <c r="K32" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M32" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1629,6 +1746,15 @@
       <c r="J33" t="str">
         <v>Boston metro. This is the req flagged in the prior run as 'found in snippets but not direct-fetched' — now confirmed live. Same cohort/site family as the Mechanical/Systems Engineer Co-ops above. No stated application deadline.</v>
       </c>
+      <c r="K33" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M33" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1661,6 +1787,15 @@
       <c r="J34" t="str">
         <v/>
       </c>
+      <c r="K34" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L34" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M34" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1693,6 +1828,15 @@
       <c r="J35" t="str">
         <v/>
       </c>
+      <c r="K35" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L35" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M35" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1722,6 +1866,15 @@
       <c r="J36" t="str">
         <v>Corrects an earlier 'checked' entry that grouped SpaceX with companies having 'no Winter 2026/Spring 2027-specific postings' — this Spring 2027 req is a later-posted exception. Likely requires US person status (ITAR) though not explicitly re-confirmed this session.</v>
       </c>
+      <c r="K36" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L36" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M36" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1754,6 +1907,15 @@
       <c r="J37" t="str">
         <v>Rocket Lab has ~25 more Spring 2027 postings (propulsion, structural, manufacturing, test) across CA/MD/VA/AZ/CO/NM — none in Boston area, not individually logged.</v>
       </c>
+      <c r="K37" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M37" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -1786,6 +1948,15 @@
       <c r="J38" t="str">
         <v/>
       </c>
+      <c r="K38" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L38" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M38" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1817,6 +1988,15 @@
       </c>
       <c r="J39" t="str">
         <v>~1.5 hrs from Boston.</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L39" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M39" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="40">
@@ -6118,6 +6298,60 @@
     <hyperlink ref="K19" r:id="rId39"/>
     <hyperlink ref="L19" r:id="rId40"/>
     <hyperlink ref="M19" r:id="rId41"/>
+    <hyperlink ref="K20" r:id="rId42"/>
+    <hyperlink ref="L20" r:id="rId43"/>
+    <hyperlink ref="M20" r:id="rId44"/>
+    <hyperlink ref="K22" r:id="rId45"/>
+    <hyperlink ref="L22" r:id="rId46"/>
+    <hyperlink ref="M22" r:id="rId47"/>
+    <hyperlink ref="K23" r:id="rId48"/>
+    <hyperlink ref="L23" r:id="rId49"/>
+    <hyperlink ref="M23" r:id="rId50"/>
+    <hyperlink ref="K24" r:id="rId51"/>
+    <hyperlink ref="L24" r:id="rId52"/>
+    <hyperlink ref="M24" r:id="rId53"/>
+    <hyperlink ref="K25" r:id="rId54"/>
+    <hyperlink ref="L25" r:id="rId55"/>
+    <hyperlink ref="M25" r:id="rId56"/>
+    <hyperlink ref="K26" r:id="rId57"/>
+    <hyperlink ref="L26" r:id="rId58"/>
+    <hyperlink ref="M26" r:id="rId59"/>
+    <hyperlink ref="K27" r:id="rId60"/>
+    <hyperlink ref="L27" r:id="rId61"/>
+    <hyperlink ref="M27" r:id="rId62"/>
+    <hyperlink ref="K29" r:id="rId63"/>
+    <hyperlink ref="L29" r:id="rId64"/>
+    <hyperlink ref="M29" r:id="rId65"/>
+    <hyperlink ref="K30" r:id="rId66"/>
+    <hyperlink ref="L30" r:id="rId67"/>
+    <hyperlink ref="M30" r:id="rId68"/>
+    <hyperlink ref="K31" r:id="rId69"/>
+    <hyperlink ref="L31" r:id="rId70"/>
+    <hyperlink ref="M31" r:id="rId71"/>
+    <hyperlink ref="K32" r:id="rId72"/>
+    <hyperlink ref="L32" r:id="rId73"/>
+    <hyperlink ref="M32" r:id="rId74"/>
+    <hyperlink ref="K33" r:id="rId75"/>
+    <hyperlink ref="L33" r:id="rId76"/>
+    <hyperlink ref="M33" r:id="rId77"/>
+    <hyperlink ref="K34" r:id="rId78"/>
+    <hyperlink ref="L34" r:id="rId79"/>
+    <hyperlink ref="M34" r:id="rId80"/>
+    <hyperlink ref="K35" r:id="rId81"/>
+    <hyperlink ref="L35" r:id="rId82"/>
+    <hyperlink ref="M35" r:id="rId83"/>
+    <hyperlink ref="K36" r:id="rId84"/>
+    <hyperlink ref="L36" r:id="rId85"/>
+    <hyperlink ref="M36" r:id="rId86"/>
+    <hyperlink ref="K37" r:id="rId87"/>
+    <hyperlink ref="L37" r:id="rId88"/>
+    <hyperlink ref="M37" r:id="rId89"/>
+    <hyperlink ref="K38" r:id="rId90"/>
+    <hyperlink ref="L38" r:id="rId91"/>
+    <hyperlink ref="M38" r:id="rId92"/>
+    <hyperlink ref="K39" r:id="rId93"/>
+    <hyperlink ref="L39" r:id="rId94"/>
+    <hyperlink ref="M39" r:id="rId95"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 2: rows 40-59 (19 new document sets, 1 skip)
New resume, cover letter, and questions for Pratt & Whitney, Collins (3), Northrop Grumman, Berkshire Grey, Emerson (2), Zipline, Applied Materials, Sanofi, GE Aerospace (2), and Insulet (7). Row 58 skipped: graduate-only. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -2030,6 +2030,15 @@
       <c r="J40" t="str">
         <v>~1.5 hrs from Boston.</v>
       </c>
+      <c r="K40" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L40" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M40" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2062,6 +2071,15 @@
       <c r="J41" t="str">
         <v/>
       </c>
+      <c r="K41" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2094,6 +2112,15 @@
       <c r="J42" t="str">
         <v/>
       </c>
+      <c r="K42" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2126,6 +2153,15 @@
       <c r="J43" t="str">
         <v/>
       </c>
+      <c r="K43" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2158,6 +2194,15 @@
       <c r="J44" t="str">
         <v/>
       </c>
+      <c r="K44" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L44" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M44" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2190,6 +2235,15 @@
       <c r="J45" t="str">
         <v>Scoop™ engineering quality team, V&amp;V of electromechanical systems. Boston metro (Bedford).</v>
       </c>
+      <c r="K45" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L45" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M45" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2222,6 +2276,15 @@
       <c r="J46" t="str">
         <v/>
       </c>
+      <c r="K46" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L46" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M46" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2254,6 +2317,15 @@
       <c r="J47" t="str">
         <v/>
       </c>
+      <c r="K47" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L47" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M47" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2286,6 +2358,15 @@
       <c r="J48" t="str">
         <v>Design/build/test electro-mechanical systems for autonomous drone delivery. Requires ≥2nd year undergrad completed; masters/PhD also eligible.</v>
       </c>
+      <c r="K48" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L48" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M48" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2318,6 +2399,15 @@
       <c r="J49" t="str">
         <v>Boston metro (Gloucester, MA). A sibling req, '2027 Spring Product Quality Engineer Co-op' at the same site, also exists but is a different discipline — not added.</v>
       </c>
+      <c r="K49" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L49" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M49" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2350,6 +2440,15 @@
       <c r="J50" t="str">
         <v>Boston metro (Framingham). Umbrella posting covering multiple functional tracks (HSE, Cell Culture Development, Downstream/Upstream MSAT, Supply Chain Planning, Drug Product Development) — biopharma manufacturing/process engineering, not classic mechanical. A second Sanofi req ('GMU CMC Purification Process Development,' Waltham MA) surfaced but wasn't independently verified — likely another slot in this same program, not double-counted.</v>
       </c>
+      <c r="K50" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L50" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M50" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2382,6 +2481,15 @@
       <c r="J51" t="str">
         <v>Requires 'US Person' status (citizen/LPR/asylee/refugee) for export-controlled work; no visa sponsorship; relocation/housing assistance provided. This is the first live GE Aerospace Spring 2027 req found after 4 prior runs found only dead/expired reqs — Lynn, MA option makes this a Boston-metro fit.</v>
       </c>
+      <c r="K51" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L51" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M51" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2414,6 +2522,15 @@
       <c r="J52" t="str">
         <v>Accepted majors: Aerospace, Manufacturing, Mechanical, Materials, Industrial Engineering. Not Boston-area.</v>
       </c>
+      <c r="K52" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L52" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M52" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2446,6 +2563,15 @@
       <c r="J53" t="str">
         <v>Boston metro (Acton). Medical device (insulin pump) manufacturer. Not eligible for visa sponsorship; requires US work authorization without future sponsorship needs. Part of a large batch of Insulet Acton co-ops opened this cycle — see sibling reqs below.</v>
       </c>
+      <c r="K53" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L53" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M53" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2478,6 +2604,15 @@
       <c r="J54" t="str">
         <v>Boston metro (Acton). No visa sponsorship.</v>
       </c>
+      <c r="K54" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L54" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M54" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2510,6 +2645,15 @@
       <c r="J55" t="str">
         <v>Boston metro (Acton). No visa sponsorship.</v>
       </c>
+      <c r="K55" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L55" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M55" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2542,6 +2686,15 @@
       <c r="J56" t="str">
         <v>Boston metro (Acton). One of a batch of Insulet Acton co-ops opened this cycle alongside the fully-verified R&amp;D Mechanical/Manufacturing/Systems reqs above.</v>
       </c>
+      <c r="K56" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L56" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M56" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2574,6 +2727,15 @@
       <c r="J57" t="str">
         <v>Boston metro (Acton).</v>
       </c>
+      <c r="K57" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L57" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M57" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2606,6 +2768,15 @@
       <c r="J58" t="str">
         <v>Boston metro (Acton). Labeled 'Graduate Co-op' — confirm eligibility if Hamza is undergraduate.</v>
       </c>
+      <c r="K58" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="L58" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="M58" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2637,6 +2808,15 @@
       </c>
       <c r="J59" t="str">
         <v>Boston metro (Acton).</v>
+      </c>
+      <c r="K59" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L59" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M59" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="60">
@@ -6352,6 +6532,63 @@
     <hyperlink ref="K39" r:id="rId93"/>
     <hyperlink ref="L39" r:id="rId94"/>
     <hyperlink ref="M39" r:id="rId95"/>
+    <hyperlink ref="K40" r:id="rId96"/>
+    <hyperlink ref="L40" r:id="rId97"/>
+    <hyperlink ref="M40" r:id="rId98"/>
+    <hyperlink ref="K41" r:id="rId99"/>
+    <hyperlink ref="L41" r:id="rId100"/>
+    <hyperlink ref="M41" r:id="rId101"/>
+    <hyperlink ref="K42" r:id="rId102"/>
+    <hyperlink ref="L42" r:id="rId103"/>
+    <hyperlink ref="M42" r:id="rId104"/>
+    <hyperlink ref="K43" r:id="rId105"/>
+    <hyperlink ref="L43" r:id="rId106"/>
+    <hyperlink ref="M43" r:id="rId107"/>
+    <hyperlink ref="K44" r:id="rId108"/>
+    <hyperlink ref="L44" r:id="rId109"/>
+    <hyperlink ref="M44" r:id="rId110"/>
+    <hyperlink ref="K45" r:id="rId111"/>
+    <hyperlink ref="L45" r:id="rId112"/>
+    <hyperlink ref="M45" r:id="rId113"/>
+    <hyperlink ref="K46" r:id="rId114"/>
+    <hyperlink ref="L46" r:id="rId115"/>
+    <hyperlink ref="M46" r:id="rId116"/>
+    <hyperlink ref="K47" r:id="rId117"/>
+    <hyperlink ref="L47" r:id="rId118"/>
+    <hyperlink ref="M47" r:id="rId119"/>
+    <hyperlink ref="K48" r:id="rId120"/>
+    <hyperlink ref="L48" r:id="rId121"/>
+    <hyperlink ref="M48" r:id="rId122"/>
+    <hyperlink ref="K49" r:id="rId123"/>
+    <hyperlink ref="L49" r:id="rId124"/>
+    <hyperlink ref="M49" r:id="rId125"/>
+    <hyperlink ref="K50" r:id="rId126"/>
+    <hyperlink ref="L50" r:id="rId127"/>
+    <hyperlink ref="M50" r:id="rId128"/>
+    <hyperlink ref="K51" r:id="rId129"/>
+    <hyperlink ref="L51" r:id="rId130"/>
+    <hyperlink ref="M51" r:id="rId131"/>
+    <hyperlink ref="K52" r:id="rId132"/>
+    <hyperlink ref="L52" r:id="rId133"/>
+    <hyperlink ref="M52" r:id="rId134"/>
+    <hyperlink ref="K53" r:id="rId135"/>
+    <hyperlink ref="L53" r:id="rId136"/>
+    <hyperlink ref="M53" r:id="rId137"/>
+    <hyperlink ref="K54" r:id="rId138"/>
+    <hyperlink ref="L54" r:id="rId139"/>
+    <hyperlink ref="M54" r:id="rId140"/>
+    <hyperlink ref="K55" r:id="rId141"/>
+    <hyperlink ref="L55" r:id="rId142"/>
+    <hyperlink ref="M55" r:id="rId143"/>
+    <hyperlink ref="K56" r:id="rId144"/>
+    <hyperlink ref="L56" r:id="rId145"/>
+    <hyperlink ref="M56" r:id="rId146"/>
+    <hyperlink ref="K57" r:id="rId147"/>
+    <hyperlink ref="L57" r:id="rId148"/>
+    <hyperlink ref="M57" r:id="rId149"/>
+    <hyperlink ref="K59" r:id="rId150"/>
+    <hyperlink ref="L59" r:id="rId151"/>
+    <hyperlink ref="M59" r:id="rId152"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 3: rows 60-79 (18 new document sets, 2 relinks)
New documents for Insulet (7), GE HealthCare, Leonardo DRS, Moderna, Vertex, Astranis, Collins Jamestown, MIT Lincoln Lab Microfab, Draper Materials, and Entegris Billerica (5). Rows 63 and 67 duplicate earlier postings (GE Vernova Nuclear, Applied Materials Gloucester) so they link to the earlier files. Also regenerates batch 2 letters to drop repeated sentences. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -2850,6 +2850,15 @@
       <c r="J60" t="str">
         <v>Boston metro (Acton).</v>
       </c>
+      <c r="K60" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L60" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M60" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2882,6 +2891,15 @@
       <c r="J61" t="str">
         <v>Boston metro (Acton). Most recently posted of the Insulet batch.</v>
       </c>
+      <c r="K61" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L61" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M61" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2914,6 +2932,15 @@
       <c r="J62" t="str">
         <v>Accepts Mechanical, Electrical, Computer, and Biomedical Engineering majors — verification/test focus, not pure design. Minimum 20-week commitment, onsite Waukesha WI, no visa sponsorship. Not Boston-area.</v>
       </c>
+      <c r="K62" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L62" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M62" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2946,6 +2973,15 @@
       <c r="J63" t="str">
         <v>GE Vernova Hitachi Nuclear Energy (GVH) business. Not Boston-area.</v>
       </c>
+      <c r="K63" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L63" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M63" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2978,6 +3014,15 @@
       <c r="J64" t="str">
         <v>Land Systems division, Bridgeton, MO site. Junior+ standing, 1+ prior internship/co-op required, CAD (Creo/SolidWorks) required. No citizenship requirement stated on this posting. Note: a separately-numbered 'Mechanical Engineer Intern' req at the same Bridgeton site was confirmed CLOSED — do not confuse the two.</v>
       </c>
+      <c r="K64" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L64" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M64" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3010,6 +3055,15 @@
       <c r="J65" t="str">
         <v>Boston metro (Acton), onsite. US work authorization required, no sponsorship. 3.0 GPA minimum. A separate, distinct Insulet 'NGP Systems Engineering Co-op (July-Dec 2026)' req also exists — wrong season, not this one.</v>
       </c>
+      <c r="K65" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L65" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M65" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3042,6 +3096,15 @@
       <c r="J66" t="str">
         <v>Restricted to US persons (citizens/permanent residents/asylees/refugees) per prior mirror-sourced check, not re-confirmed word-for-word on this pass. Onsite ~70%. Boston metro (Norwood). Discipline is automation/bioprocess engineering, not pure mechanical — included with caveat per Hamza's 'adjacent' disciplines (industrial/controls), similar treatment to the existing Sanofi/Genzyme row.</v>
       </c>
+      <c r="K66" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L66" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M66" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3074,6 +3137,15 @@
       <c r="J67" t="str">
         <v>Boston metro (Gloucester, ~45 min drive). GPA 3.0+ preferred, good academic standing required. No explicit citizenship/visa language stated on the posting. Applied Materials is already a tracked company (other reqs elsewhere) — this is a distinct new req/season/location.</v>
       </c>
+      <c r="K67" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L67" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M67" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -3106,6 +3178,15 @@
       <c r="J68" t="str">
         <v>Application deadline stated as November 15, 2026 (rolling review, may close earlier). No stated visa sponsorship. Distinct from Vertex's 'Process Development Upstream' and 'CGT Process Development' Spring Co-Op 2027 reqs, which are biotech/process discipline and excluded (see `checked`).</v>
       </c>
+      <c r="K68" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L68" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M68" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3138,6 +3219,15 @@
       <c r="J69" t="str">
         <v>ITAR-restricted: requires US citizen, lawful permanent resident, or other 'protected individual' status under export control rules. Not Boston-area, included per Hamza's nationwide preference. A separate Summer 2027 version of this same role exists (job 4704601006) — do not confuse the two; only this Spring 2027 req qualifies.</v>
       </c>
+      <c r="K69" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L69" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M69" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3170,6 +3260,15 @@
       <c r="J70" t="str">
         <v>Distinct req from the already-tracked Jamestown ND 'Structural Engineering Co-op' (req 01873938) at the same site — different title/req, not a duplicate.</v>
       </c>
+      <c r="K70" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L70" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M70" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3202,6 +3301,15 @@
       <c r="J71" t="str">
         <v>Boston metro (Acton). Not eligible for visa sponsorship.</v>
       </c>
+      <c r="K71" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L71" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M71" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3234,6 +3342,15 @@
       <c r="J72" t="str">
         <v>Boston metro (Acton). Requires enrollment in undergraduate mechanical, industrial, or bio-engineering program. Not eligible for visa sponsorship.</v>
       </c>
+      <c r="K72" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L72" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M72" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3266,6 +3383,15 @@
       <c r="J73" t="str">
         <v>Req 42762. Sibling req to the already-tracked Microfab Industrial Eng. Co-Op (Group 08-35) — same Jan-Aug 2027 window, different discipline focus (materials/process vs industrial). Requires US citizenship + eligibility for Secret-level DoD clearance; cleanroom work.</v>
       </c>
+      <c r="K73" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L73" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M73" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3298,6 +3424,15 @@
       <c r="J74" t="str">
         <v>Req JR002942. Onsite required. Draper's other co-ops in this batch state US citizenship is mandatory due to sensitive work — verify before applying.</v>
       </c>
+      <c r="K74" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L74" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M74" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -3330,6 +3465,15 @@
       <c r="J75" t="str">
         <v>REQ-14497. New company for the tracker. Boston metro (Billerica).</v>
       </c>
+      <c r="K75" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L75" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M75" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -3362,6 +3506,15 @@
       <c r="J76" t="str">
         <v>REQ-14444. PLC/Allen-Bradley/Rockwell work.</v>
       </c>
+      <c r="K76" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L76" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M76" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -3394,6 +3547,15 @@
       <c r="J77" t="str">
         <v>REQ-14469. Semiconductor liquid filtration products.</v>
       </c>
+      <c r="K77" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L77" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M77" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -3426,6 +3588,15 @@
       <c r="J78" t="str">
         <v>REQ-14462. Manufacturing/materials process optimization.</v>
       </c>
+      <c r="K78" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L78" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M78" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -3457,6 +3628,15 @@
       </c>
       <c r="J79" t="str">
         <v>REQ-14504. Assembly/Flush Room/Warehouse cost reduction, Kaizen/5S/Gemba.</v>
+      </c>
+      <c r="K79" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L79" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M79" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="80">
@@ -6589,6 +6769,66 @@
     <hyperlink ref="K59" r:id="rId150"/>
     <hyperlink ref="L59" r:id="rId151"/>
     <hyperlink ref="M59" r:id="rId152"/>
+    <hyperlink ref="K60" r:id="rId153"/>
+    <hyperlink ref="L60" r:id="rId154"/>
+    <hyperlink ref="M60" r:id="rId155"/>
+    <hyperlink ref="K61" r:id="rId156"/>
+    <hyperlink ref="L61" r:id="rId157"/>
+    <hyperlink ref="M61" r:id="rId158"/>
+    <hyperlink ref="K62" r:id="rId159"/>
+    <hyperlink ref="L62" r:id="rId160"/>
+    <hyperlink ref="M62" r:id="rId161"/>
+    <hyperlink ref="K63" r:id="rId162"/>
+    <hyperlink ref="L63" r:id="rId163"/>
+    <hyperlink ref="M63" r:id="rId164"/>
+    <hyperlink ref="K64" r:id="rId165"/>
+    <hyperlink ref="L64" r:id="rId166"/>
+    <hyperlink ref="M64" r:id="rId167"/>
+    <hyperlink ref="K65" r:id="rId168"/>
+    <hyperlink ref="L65" r:id="rId169"/>
+    <hyperlink ref="M65" r:id="rId170"/>
+    <hyperlink ref="K66" r:id="rId171"/>
+    <hyperlink ref="L66" r:id="rId172"/>
+    <hyperlink ref="M66" r:id="rId173"/>
+    <hyperlink ref="K67" r:id="rId174"/>
+    <hyperlink ref="L67" r:id="rId175"/>
+    <hyperlink ref="M67" r:id="rId176"/>
+    <hyperlink ref="K68" r:id="rId177"/>
+    <hyperlink ref="L68" r:id="rId178"/>
+    <hyperlink ref="M68" r:id="rId179"/>
+    <hyperlink ref="K69" r:id="rId180"/>
+    <hyperlink ref="L69" r:id="rId181"/>
+    <hyperlink ref="M69" r:id="rId182"/>
+    <hyperlink ref="K70" r:id="rId183"/>
+    <hyperlink ref="L70" r:id="rId184"/>
+    <hyperlink ref="M70" r:id="rId185"/>
+    <hyperlink ref="K71" r:id="rId186"/>
+    <hyperlink ref="L71" r:id="rId187"/>
+    <hyperlink ref="M71" r:id="rId188"/>
+    <hyperlink ref="K72" r:id="rId189"/>
+    <hyperlink ref="L72" r:id="rId190"/>
+    <hyperlink ref="M72" r:id="rId191"/>
+    <hyperlink ref="K73" r:id="rId192"/>
+    <hyperlink ref="L73" r:id="rId193"/>
+    <hyperlink ref="M73" r:id="rId194"/>
+    <hyperlink ref="K74" r:id="rId195"/>
+    <hyperlink ref="L74" r:id="rId196"/>
+    <hyperlink ref="M74" r:id="rId197"/>
+    <hyperlink ref="K75" r:id="rId198"/>
+    <hyperlink ref="L75" r:id="rId199"/>
+    <hyperlink ref="M75" r:id="rId200"/>
+    <hyperlink ref="K76" r:id="rId201"/>
+    <hyperlink ref="L76" r:id="rId202"/>
+    <hyperlink ref="M76" r:id="rId203"/>
+    <hyperlink ref="K77" r:id="rId204"/>
+    <hyperlink ref="L77" r:id="rId205"/>
+    <hyperlink ref="M77" r:id="rId206"/>
+    <hyperlink ref="K78" r:id="rId207"/>
+    <hyperlink ref="L78" r:id="rId208"/>
+    <hyperlink ref="M78" r:id="rId209"/>
+    <hyperlink ref="K79" r:id="rId210"/>
+    <hyperlink ref="L79" r:id="rId211"/>
+    <hyperlink ref="M79" r:id="rId212"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 4: rows 80-99 (18 new document sets, 1 relink, 1 skip)
New documents for Berkshire Grey (3), GE Aerospace Manufacturing, PI (2), Astranis CAD, Collins Rockford, L3Harris, Anduril Costa Mesa (3), and Zipline (6). Row 83 duplicates Blue Origin row 10 so it links to the earlier files. Row 84 skipped: SpaceX graduate-only internship. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -3670,6 +3670,15 @@
       <c r="J80" t="str">
         <v>SolidWorks/DFM/prototyping, product development team, testing + NPI support. Boston metro (Bedford).</v>
       </c>
+      <c r="K80" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L80" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M80" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -3702,6 +3711,15 @@
       <c r="J81" t="str">
         <v>PLC development, test-fixture controls. Boston metro (Bedford).</v>
       </c>
+      <c r="K81" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L81" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M81" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -3734,6 +3752,15 @@
       <c r="J82" t="str">
         <v>Borderline discipline fit — robot manipulation R&amp;D, filed under Software department rather than a hardware/mechanical department. Included per Hamza's robotics discipline preference; his own judgment call on fit. Boston metro (Bedford).</v>
       </c>
+      <c r="K82" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L82" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M82" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -3766,6 +3793,15 @@
       <c r="J83" t="str">
         <v>Req R69064. General multi-discipline req — actual engineering discipline/site placement determined after applying/interviewing, mechanical not guaranteed. Requires US citizen/national, Green Card holder, or lawfully admitted refugee/asylee.</v>
       </c>
+      <c r="K83" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L83" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M83" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -3798,6 +3834,15 @@
       <c r="J84" t="str">
         <v>Distinct req from the already-tracked undergrad-oriented 'Spring 2027 Engineering Internship/Co-op' (job 8616338002) — THIS req explicitly requires the applicant to already hold a bachelor's degree AND be currently enrolled in a graduate program. Only relevant if Hamza is in/entering grad school by Spring 2027. US citizen/permanent resident/refugee/asylee required (ITAR).</v>
       </c>
+      <c r="K84" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="L84" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="M84" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -3830,6 +3875,15 @@
       <c r="J85" t="str">
         <v>Sibling req to the already-tracked Engines Engineering Co-op (R5029617-1) at the same Lynn, MA site — distinct req ID, not a duplicate. Excludes 'Returning Students' variants (require a prior GE Aerospace internship).</v>
       </c>
+      <c r="K85" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L85" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M85" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -3862,6 +3916,15 @@
       <c r="J86" t="str">
         <v>Boston metro (Shrewsbury). Fresh cycle superseding the already-past Jan-June 2026 cohort found at this same company in prior runs. Requires legal US work authorization without sponsorship; SolidWorks preferred.</v>
       </c>
+      <c r="K86" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L86" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M86" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -3894,6 +3957,15 @@
       <c r="J87" t="str">
         <v>Boston metro (Shrewsbury). Same batch/cycle as the Mechanical Engineering Co-op above.</v>
       </c>
+      <c r="K87" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L87" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M87" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -3926,6 +3998,15 @@
       <c r="J88" t="str">
         <v>Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 4704602006) at the same company. Satellite manufacturer — worth double-checking ITAR/citizenship requirements before applying, not explicit in the excerpt reviewed. Distinct from Astranis's separate 'Winter 2027' reqs, which remain excluded (see `checked`) for season mismatch.</v>
       </c>
+      <c r="K88" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L88" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M88" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -3958,6 +4039,15 @@
       <c r="J89" t="str">
         <v>Distinct req/site from the already-tracked Jamestown ND and Cedar Rapids IA Collins Aerospace co-ops — not a duplicate.</v>
       </c>
+      <c r="K89" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L89" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M89" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -3990,6 +4080,15 @@
       <c r="J90" t="str">
         <v>Degree requirement: Mechanical/Aerospace/Engineering Mechanics/Materials Science. US citizenship required for clearance eligibility. Job ID 41322.</v>
       </c>
+      <c r="K90" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L90" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M90" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -4022,6 +4121,15 @@
       <c r="J91" t="str">
         <v>US citizenship required, no clearance required. New site beyond the already-tracked Quincy, MA / Lexington, MA Anduril Winter 2027 co-ops.</v>
       </c>
+      <c r="K91" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L91" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M91" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -4054,6 +4162,15 @@
       <c r="J92" t="str">
         <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Test &amp; Evaluation Engineer Co-ops above.</v>
       </c>
+      <c r="K92" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L92" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M92" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -4086,6 +4203,15 @@
       <c r="J93" t="str">
         <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Warhead Engineer Co-ops above.</v>
       </c>
+      <c r="K93" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L93" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M93" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -4118,6 +4244,15 @@
       <c r="J94" t="str">
         <v>Autonomous drone delivery company. Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 7865253003) at the same company.</v>
       </c>
+      <c r="K94" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L94" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M94" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -4150,6 +4285,15 @@
       <c r="J95" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K95" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L95" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M95" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -4182,6 +4326,15 @@
       <c r="J96" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K96" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L96" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M96" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -4214,6 +4367,15 @@
       <c r="J97" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K97" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L97" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M97" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -4246,6 +4408,15 @@
       <c r="J98" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K98" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L98" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M98" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -4277,6 +4448,15 @@
       </c>
       <c r="J99" t="str">
         <v>Borderline discipline fit (maintenance tooling) — included per Hamza's own judgment call, similar treatment to other borderline robotics/manufacturing-adjacent reqs in this tracker.</v>
+      </c>
+      <c r="K99" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L99" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M99" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="100">
@@ -6829,6 +7009,63 @@
     <hyperlink ref="K79" r:id="rId210"/>
     <hyperlink ref="L79" r:id="rId211"/>
     <hyperlink ref="M79" r:id="rId212"/>
+    <hyperlink ref="K80" r:id="rId213"/>
+    <hyperlink ref="L80" r:id="rId214"/>
+    <hyperlink ref="M80" r:id="rId215"/>
+    <hyperlink ref="K81" r:id="rId216"/>
+    <hyperlink ref="L81" r:id="rId217"/>
+    <hyperlink ref="M81" r:id="rId218"/>
+    <hyperlink ref="K82" r:id="rId219"/>
+    <hyperlink ref="L82" r:id="rId220"/>
+    <hyperlink ref="M82" r:id="rId221"/>
+    <hyperlink ref="K83" r:id="rId222"/>
+    <hyperlink ref="L83" r:id="rId223"/>
+    <hyperlink ref="M83" r:id="rId224"/>
+    <hyperlink ref="K85" r:id="rId225"/>
+    <hyperlink ref="L85" r:id="rId226"/>
+    <hyperlink ref="M85" r:id="rId227"/>
+    <hyperlink ref="K86" r:id="rId228"/>
+    <hyperlink ref="L86" r:id="rId229"/>
+    <hyperlink ref="M86" r:id="rId230"/>
+    <hyperlink ref="K87" r:id="rId231"/>
+    <hyperlink ref="L87" r:id="rId232"/>
+    <hyperlink ref="M87" r:id="rId233"/>
+    <hyperlink ref="K88" r:id="rId234"/>
+    <hyperlink ref="L88" r:id="rId235"/>
+    <hyperlink ref="M88" r:id="rId236"/>
+    <hyperlink ref="K89" r:id="rId237"/>
+    <hyperlink ref="L89" r:id="rId238"/>
+    <hyperlink ref="M89" r:id="rId239"/>
+    <hyperlink ref="K90" r:id="rId240"/>
+    <hyperlink ref="L90" r:id="rId241"/>
+    <hyperlink ref="M90" r:id="rId242"/>
+    <hyperlink ref="K91" r:id="rId243"/>
+    <hyperlink ref="L91" r:id="rId244"/>
+    <hyperlink ref="M91" r:id="rId245"/>
+    <hyperlink ref="K92" r:id="rId246"/>
+    <hyperlink ref="L92" r:id="rId247"/>
+    <hyperlink ref="M92" r:id="rId248"/>
+    <hyperlink ref="K93" r:id="rId249"/>
+    <hyperlink ref="L93" r:id="rId250"/>
+    <hyperlink ref="M93" r:id="rId251"/>
+    <hyperlink ref="K94" r:id="rId252"/>
+    <hyperlink ref="L94" r:id="rId253"/>
+    <hyperlink ref="M94" r:id="rId254"/>
+    <hyperlink ref="K95" r:id="rId255"/>
+    <hyperlink ref="L95" r:id="rId256"/>
+    <hyperlink ref="M95" r:id="rId257"/>
+    <hyperlink ref="K96" r:id="rId258"/>
+    <hyperlink ref="L96" r:id="rId259"/>
+    <hyperlink ref="M96" r:id="rId260"/>
+    <hyperlink ref="K97" r:id="rId261"/>
+    <hyperlink ref="L97" r:id="rId262"/>
+    <hyperlink ref="M97" r:id="rId263"/>
+    <hyperlink ref="K98" r:id="rId264"/>
+    <hyperlink ref="L98" r:id="rId265"/>
+    <hyperlink ref="M98" r:id="rId266"/>
+    <hyperlink ref="K99" r:id="rId267"/>
+    <hyperlink ref="L99" r:id="rId268"/>
+    <hyperlink ref="M99" r:id="rId269"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 5: rows 100-119 (18 new document sets, 2 skips)
New documents for Zipline (2), Varda (5), Marathon Petroleum, GE Appliances (5), Entegris Mechanical, Aalo Atomics, Hermeus GNC, and Owens Corning. Rows 110 (Insulet graduate co-op) and 116 (Hologic Jan to June 2026 co-op, already past) skipped. Also regenerates batches 2 to 4 letters with duplicate-sentence cleanup. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -4490,6 +4490,15 @@
       <c r="J100" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K100" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L100" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M100" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -4522,6 +4531,15 @@
       <c r="J101" t="str">
         <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
+      <c r="K101" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L101" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M101" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -4554,6 +4572,15 @@
       <c r="J102" t="str">
         <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. Designs/builds/tests flight electromechanical hardware (mechanisms, payloads). US work authorization + export-control (ITAR) screening required per posting.</v>
       </c>
+      <c r="K102" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L102" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M102" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -4586,6 +4613,15 @@
       <c r="J103" t="str">
         <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. CAD/FEA design and build/test of spacecraft structural hardware. US work authorization + export-control (ITAR) screening required per posting.</v>
       </c>
+      <c r="K103" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L103" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M103" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -4618,6 +4654,15 @@
       <c r="J104" t="str">
         <v>Sibling req to the already-tracked Varda internships at the same company/season. GNC for flight vehicles. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
+      <c r="K104" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L104" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M104" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -4650,6 +4695,15 @@
       <c r="J105" t="str">
         <v>Sibling req to the already-tracked Varda internships at the same company/season. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
+      <c r="K105" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L105" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M105" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -4682,6 +4736,15 @@
       <c r="J106" t="str">
         <v>Sibling req to the already-tracked Varda internships at the same company/season. Vehicle integration and test of flight hardware. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
+      <c r="K106" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L106" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M106" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -4714,6 +4777,15 @@
       <c r="J107" t="str">
         <v>New company, not previously tracked. Industrial/refining rather than aerospace, but fits mechanical/manufacturing discipline. Requires majoring in Mechanical or Civil Engineering; no visa sponsorship available. Posting also states co-op positions run spring, summer, and fall generally, but this specific req is titled and dated for Spring 2027. Additional refinery locations listed on same req: Anacortes WA, Canton OH, Catlettsburg KY, Detroit MI, El Paso TX, Garyville LA, Kenai AK, Mandan ND, Martinez CA, Robinson IL, Salt Lake City UT, St Paul Park MN, Texas City TX, Wilmington CA.</v>
       </c>
+      <c r="K107" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L107" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M107" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -4746,6 +4818,15 @@
       <c r="J108" t="str">
         <v>New company, not previously tracked. Industrial/consumer-manufacturing rather than aerospace, but squarely mechanical engineering with a clean Spring-only (not combined) term and explicit dates.</v>
       </c>
+      <c r="K108" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L108" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M108" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -4778,6 +4859,15 @@
       <c r="J109" t="str">
         <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
       </c>
+      <c r="K109" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L109" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M109" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -4810,6 +4900,15 @@
       <c r="J110" t="str">
         <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
       </c>
+      <c r="K110" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="L110" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
+      <c r="M110" t="str">
+        <v>Skipped: graduate students only (you are an undergrad)</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -4842,6 +4941,15 @@
       <c r="J111" t="str">
         <v>New req beyond the already-tracked REQ-24833 (Mechanical Engineering Co-op) at the same Louisville, KY site.</v>
       </c>
+      <c r="K111" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L111" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M111" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -4874,6 +4982,15 @@
       <c r="J112" t="str">
         <v>New req beyond the already-tracked REQ-24833 at the same Louisville, KY site.</v>
       </c>
+      <c r="K112" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L112" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M112" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -4906,6 +5023,15 @@
       <c r="J113" t="str">
         <v>New site (LaFayette, GA) for GE Appliances beyond the already-tracked Louisville, KY reqs.</v>
       </c>
+      <c r="K113" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L113" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M113" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -4938,6 +5064,15 @@
       <c r="J114" t="str">
         <v>New req at the same LaFayette, GA site as REQ-24836.</v>
       </c>
+      <c r="K114" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L114" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M114" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -4970,6 +5105,15 @@
       <c r="J115" t="str">
         <v>New site (Decatur, AL) for GE Appliances beyond the already-tracked Louisville KY / LaFayette GA reqs.</v>
       </c>
+      <c r="K115" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L115" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M115" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -5002,6 +5146,15 @@
       <c r="J116" t="str">
         <v>Long-standing 'worth re-checking' item, now has a confirmed direct URL and season match for the first time. A second, likely newer Hologic req ('Co-Op, New Product Development Engineering', .../300000422097244/...) was also found this run but remains season-unconfirmed and 503-blocked — see `checked`.</v>
       </c>
+      <c r="K116" t="str">
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+      </c>
+      <c r="L116" t="str">
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+      </c>
+      <c r="M116" t="str">
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -5034,6 +5187,15 @@
       <c r="J117" t="str">
         <v>New company for the tracker (advanced nuclear reactor startup). Requires B.S./M.S. in Mechanical, Aerospace, or Manufacturing Engineering (or closely related field) plus ~3 months applied engineering experience.</v>
       </c>
+      <c r="K117" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L117" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M117" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -5066,6 +5228,15 @@
       <c r="J118" t="str">
         <v>New company for the tracker (hypersonic aircraft developer). GNC (Guidance, Navigation &amp; Controls) role — flight-systems/controls discipline. Also open to Aerospace/Computer Engineering/CS/EE majors. Unlike a truly combined-term posting, the Spring option has its own distinct dates, so included (same treatment as RTX's 'Winter/Spring 2027' co-ops).</v>
       </c>
+      <c r="K118" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L118" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M118" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -5097,6 +5268,15 @@
       </c>
       <c r="J119" t="str">
         <v>New company for the tracker (building materials manufacturer). Accepts Mechanical, Electrical, Engineering Technology, Chemical, or Industrial Engineering majors.</v>
+      </c>
+      <c r="K119" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L119" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M119" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="120">
@@ -7066,6 +7246,60 @@
     <hyperlink ref="K99" r:id="rId267"/>
     <hyperlink ref="L99" r:id="rId268"/>
     <hyperlink ref="M99" r:id="rId269"/>
+    <hyperlink ref="K100" r:id="rId270"/>
+    <hyperlink ref="L100" r:id="rId271"/>
+    <hyperlink ref="M100" r:id="rId272"/>
+    <hyperlink ref="K101" r:id="rId273"/>
+    <hyperlink ref="L101" r:id="rId274"/>
+    <hyperlink ref="M101" r:id="rId275"/>
+    <hyperlink ref="K102" r:id="rId276"/>
+    <hyperlink ref="L102" r:id="rId277"/>
+    <hyperlink ref="M102" r:id="rId278"/>
+    <hyperlink ref="K103" r:id="rId279"/>
+    <hyperlink ref="L103" r:id="rId280"/>
+    <hyperlink ref="M103" r:id="rId281"/>
+    <hyperlink ref="K104" r:id="rId282"/>
+    <hyperlink ref="L104" r:id="rId283"/>
+    <hyperlink ref="M104" r:id="rId284"/>
+    <hyperlink ref="K105" r:id="rId285"/>
+    <hyperlink ref="L105" r:id="rId286"/>
+    <hyperlink ref="M105" r:id="rId287"/>
+    <hyperlink ref="K106" r:id="rId288"/>
+    <hyperlink ref="L106" r:id="rId289"/>
+    <hyperlink ref="M106" r:id="rId290"/>
+    <hyperlink ref="K107" r:id="rId291"/>
+    <hyperlink ref="L107" r:id="rId292"/>
+    <hyperlink ref="M107" r:id="rId293"/>
+    <hyperlink ref="K108" r:id="rId294"/>
+    <hyperlink ref="L108" r:id="rId295"/>
+    <hyperlink ref="M108" r:id="rId296"/>
+    <hyperlink ref="K109" r:id="rId297"/>
+    <hyperlink ref="L109" r:id="rId298"/>
+    <hyperlink ref="M109" r:id="rId299"/>
+    <hyperlink ref="K111" r:id="rId300"/>
+    <hyperlink ref="L111" r:id="rId301"/>
+    <hyperlink ref="M111" r:id="rId302"/>
+    <hyperlink ref="K112" r:id="rId303"/>
+    <hyperlink ref="L112" r:id="rId304"/>
+    <hyperlink ref="M112" r:id="rId305"/>
+    <hyperlink ref="K113" r:id="rId306"/>
+    <hyperlink ref="L113" r:id="rId307"/>
+    <hyperlink ref="M113" r:id="rId308"/>
+    <hyperlink ref="K114" r:id="rId309"/>
+    <hyperlink ref="L114" r:id="rId310"/>
+    <hyperlink ref="M114" r:id="rId311"/>
+    <hyperlink ref="K115" r:id="rId312"/>
+    <hyperlink ref="L115" r:id="rId313"/>
+    <hyperlink ref="M115" r:id="rId314"/>
+    <hyperlink ref="K117" r:id="rId315"/>
+    <hyperlink ref="L117" r:id="rId316"/>
+    <hyperlink ref="M117" r:id="rId317"/>
+    <hyperlink ref="K118" r:id="rId318"/>
+    <hyperlink ref="L118" r:id="rId319"/>
+    <hyperlink ref="M118" r:id="rId320"/>
+    <hyperlink ref="K119" r:id="rId321"/>
+    <hyperlink ref="L119" r:id="rId322"/>
+    <hyperlink ref="M119" r:id="rId323"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 6: rows 120-139 (20 new document sets)
New documents for Crown Equipment (2), Anduril EWIS Harness, Hermeus (9), Entegris Manufacturing, Fives, Formlabs (3), and Rocket Lab (2). All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -5310,6 +5310,15 @@
       <c r="J120" t="str">
         <v>New company for the tracker (forklift/material handling equipment manufacturer). Mechanical design/simulation/testing for forklift and material handling equipment development.</v>
       </c>
+      <c r="K120" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L120" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M120" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -5342,6 +5351,15 @@
       <c r="J121" t="str">
         <v>Resolves a 'worth re-checking' item from the 2026-09-23 ~19:00 UTC run (previously found without a job ID). Same batch/site as the already-tracked Propulsion, Warhead, and Test &amp; Evaluation Engineer Costa Mesa co-ops. Open to Mechanical or Electrical Engineering majors.</v>
       </c>
+      <c r="K121" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L121" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M121" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -5374,6 +5392,15 @@
       <c r="J122" t="str">
         <v>New sibling req to the already-tracked Greencastle, IN req (146174) at the same company, found via a fresh sweep of Crown's own careers site.</v>
       </c>
+      <c r="K122" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L122" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M122" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -5406,6 +5433,15 @@
       <c r="J123" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern at the same company/site; same distinct Spring/Summer option structure (not a merged single term).</v>
       </c>
+      <c r="K123" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L123" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M123" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
@@ -5438,6 +5474,15 @@
       <c r="J124" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct Spring/Summer option structure.</v>
       </c>
+      <c r="K124" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L124" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M124" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
@@ -5470,6 +5515,15 @@
       <c r="J125" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern. Flight-critical mechanical/fluid propulsion components (valves, actuators).</v>
       </c>
+      <c r="K125" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L125" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M125" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
@@ -5502,6 +5556,15 @@
       <c r="J126" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, new site (Jacksonville, FL). Propulsion system/engine test stand support.</v>
       </c>
+      <c r="K126" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L126" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M126" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -5534,6 +5597,15 @@
       <c r="J127" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure (Spring/Summer/Fall each independently dated, not a merged single term).</v>
       </c>
+      <c r="K127" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L127" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M127" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
@@ -5566,6 +5638,15 @@
       <c r="J128" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
       </c>
+      <c r="K128" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L128" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M128" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
@@ -5598,6 +5679,15 @@
       <c r="J129" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
       </c>
+      <c r="K129" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L129" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M129" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
@@ -5630,6 +5720,15 @@
       <c r="J130" t="str">
         <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, a distinct site (Los Angeles) from the Atlanta Manufacturing Engineering Intern req above.</v>
       </c>
+      <c r="K130" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L130" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M130" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
@@ -5662,6 +5761,15 @@
       <c r="J131" t="str">
         <v>New sibling req to the already-tracked Entegris Billerica co-ops (different REQ range than a previously-excluded stale REQ-7046 series). Supports process engineers on the Billerica filter manufacturing line.</v>
       </c>
+      <c r="K131" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L131" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M131" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
@@ -5694,6 +5802,15 @@
       <c r="J132" t="str">
         <v>Resolves a block that persisted across multiple prior runs (site previously only found via an aggregator mirror, never opened directly).</v>
       </c>
+      <c r="K132" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L132" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M132" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
@@ -5726,6 +5843,15 @@
       <c r="J133" t="str">
         <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
       </c>
+      <c r="K133" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L133" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M133" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
@@ -5758,6 +5884,15 @@
       <c r="J134" t="str">
         <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
       </c>
+      <c r="K134" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L134" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M134" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
@@ -5790,6 +5925,15 @@
       <c r="J135" t="str">
         <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
       </c>
+      <c r="K135" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L135" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M135" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
@@ -5822,6 +5966,15 @@
       <c r="J136" t="str">
         <v>Mix of hardware and software systems-integration work; included under Hamza's aerospace/systems discipline.</v>
       </c>
+      <c r="K136" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L136" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M136" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
@@ -5854,6 +6007,15 @@
       <c r="J137" t="str">
         <v>New discipline not previously tracked at Hermeus; on experimental high-performance aircraft flight test/airworthiness.</v>
       </c>
+      <c r="K137" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L137" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M137" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
@@ -5886,6 +6048,15 @@
       <c r="J138" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K138" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L138" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M138" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -5917,6 +6088,15 @@
       </c>
       <c r="J139" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+      </c>
+      <c r="K139" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L139" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M139" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="140">
@@ -7300,6 +7480,66 @@
     <hyperlink ref="K119" r:id="rId321"/>
     <hyperlink ref="L119" r:id="rId322"/>
     <hyperlink ref="M119" r:id="rId323"/>
+    <hyperlink ref="K120" r:id="rId324"/>
+    <hyperlink ref="L120" r:id="rId325"/>
+    <hyperlink ref="M120" r:id="rId326"/>
+    <hyperlink ref="K121" r:id="rId327"/>
+    <hyperlink ref="L121" r:id="rId328"/>
+    <hyperlink ref="M121" r:id="rId329"/>
+    <hyperlink ref="K122" r:id="rId330"/>
+    <hyperlink ref="L122" r:id="rId331"/>
+    <hyperlink ref="M122" r:id="rId332"/>
+    <hyperlink ref="K123" r:id="rId333"/>
+    <hyperlink ref="L123" r:id="rId334"/>
+    <hyperlink ref="M123" r:id="rId335"/>
+    <hyperlink ref="K124" r:id="rId336"/>
+    <hyperlink ref="L124" r:id="rId337"/>
+    <hyperlink ref="M124" r:id="rId338"/>
+    <hyperlink ref="K125" r:id="rId339"/>
+    <hyperlink ref="L125" r:id="rId340"/>
+    <hyperlink ref="M125" r:id="rId341"/>
+    <hyperlink ref="K126" r:id="rId342"/>
+    <hyperlink ref="L126" r:id="rId343"/>
+    <hyperlink ref="M126" r:id="rId344"/>
+    <hyperlink ref="K127" r:id="rId345"/>
+    <hyperlink ref="L127" r:id="rId346"/>
+    <hyperlink ref="M127" r:id="rId347"/>
+    <hyperlink ref="K128" r:id="rId348"/>
+    <hyperlink ref="L128" r:id="rId349"/>
+    <hyperlink ref="M128" r:id="rId350"/>
+    <hyperlink ref="K129" r:id="rId351"/>
+    <hyperlink ref="L129" r:id="rId352"/>
+    <hyperlink ref="M129" r:id="rId353"/>
+    <hyperlink ref="K130" r:id="rId354"/>
+    <hyperlink ref="L130" r:id="rId355"/>
+    <hyperlink ref="M130" r:id="rId356"/>
+    <hyperlink ref="K131" r:id="rId357"/>
+    <hyperlink ref="L131" r:id="rId358"/>
+    <hyperlink ref="M131" r:id="rId359"/>
+    <hyperlink ref="K132" r:id="rId360"/>
+    <hyperlink ref="L132" r:id="rId361"/>
+    <hyperlink ref="M132" r:id="rId362"/>
+    <hyperlink ref="K133" r:id="rId363"/>
+    <hyperlink ref="L133" r:id="rId364"/>
+    <hyperlink ref="M133" r:id="rId365"/>
+    <hyperlink ref="K134" r:id="rId366"/>
+    <hyperlink ref="L134" r:id="rId367"/>
+    <hyperlink ref="M134" r:id="rId368"/>
+    <hyperlink ref="K135" r:id="rId369"/>
+    <hyperlink ref="L135" r:id="rId370"/>
+    <hyperlink ref="M135" r:id="rId371"/>
+    <hyperlink ref="K136" r:id="rId372"/>
+    <hyperlink ref="L136" r:id="rId373"/>
+    <hyperlink ref="M136" r:id="rId374"/>
+    <hyperlink ref="K137" r:id="rId375"/>
+    <hyperlink ref="L137" r:id="rId376"/>
+    <hyperlink ref="M137" r:id="rId377"/>
+    <hyperlink ref="K138" r:id="rId378"/>
+    <hyperlink ref="L138" r:id="rId379"/>
+    <hyperlink ref="M138" r:id="rId380"/>
+    <hyperlink ref="K139" r:id="rId381"/>
+    <hyperlink ref="L139" r:id="rId382"/>
+    <hyperlink ref="M139" r:id="rId383"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 7: rows 140-159 (19 new document sets, 1 shared)
New documents for Rocket Lab (16 roles across Long Beach, Middle River, Wallops Island, Silver Spring, Stennis, and Albuquerque) and Entegris Bedford (3). Row 159 is a second req with the same title and site as row 158, so it links to the same files. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -6130,6 +6130,15 @@
       <c r="J140" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K140" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L140" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M140" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -6162,6 +6171,15 @@
       <c r="J141" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K141" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L141" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M141" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -6194,6 +6212,15 @@
       <c r="J142" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K142" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L142" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M142" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -6226,6 +6253,15 @@
       <c r="J143" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026; sibling reqs also open at Middle River, MD and Wallops Island, VA (see below).</v>
       </c>
+      <c r="K143" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L143" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M143" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -6258,6 +6294,15 @@
       <c r="J144" t="str">
         <v>Sibling req to the Long Beach, CA and Wallops Island, VA Manufacturing Engineering Intern postings.</v>
       </c>
+      <c r="K144" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L144" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M144" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -6290,6 +6335,15 @@
       <c r="J145" t="str">
         <v>Sibling req to the Long Beach, CA and Middle River, MD Manufacturing Engineering Intern postings.</v>
       </c>
+      <c r="K145" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L145" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M145" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -6322,6 +6376,15 @@
       <c r="J146" t="str">
         <v>Distinct site from the already-tracked Long Beach, CA Mechanical Engineering Intern req.</v>
       </c>
+      <c r="K146" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L146" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M146" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -6354,6 +6417,15 @@
       <c r="J147" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K147" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L147" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M147" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -6386,6 +6458,15 @@
       <c r="J148" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K148" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L148" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M148" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -6418,6 +6499,15 @@
       <c r="J149" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K149" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L149" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M149" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -6450,6 +6540,15 @@
       <c r="J150" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K150" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L150" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M150" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -6482,6 +6581,15 @@
       <c r="J151" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K151" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L151" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M151" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -6514,6 +6622,15 @@
       <c r="J152" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K152" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L152" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M152" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -6546,6 +6663,15 @@
       <c r="J153" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K153" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L153" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M153" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -6578,6 +6704,15 @@
       <c r="J154" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
+      <c r="K154" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L154" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M154" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -6610,6 +6745,15 @@
       <c r="J155" t="str">
         <v>Materials/manufacturing-process R&amp;D on phase-change materials for solar arrays (constellation programs).</v>
       </c>
+      <c r="K155" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L155" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M155" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -6642,6 +6786,15 @@
       <c r="J156" t="str">
         <v>REQ-14484. New Entegris site for the tracker (Bedford, in addition to the 7 already-tracked Billerica reqs).</v>
       </c>
+      <c r="K156" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L156" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M156" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -6674,6 +6827,15 @@
       <c r="J157" t="str">
         <v>REQ-14491. Bedford, MA sibling req.</v>
       </c>
+      <c r="K157" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L157" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M157" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -6706,6 +6868,15 @@
       <c r="J158" t="str">
         <v>REQ-14465. Bedford, MA sibling req; a second, distinct Industrial Engineering Co-Op req (REQ-14452) was also found open at the same site — see next row.</v>
       </c>
+      <c r="K158" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L158" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M158" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
@@ -6737,6 +6908,15 @@
       </c>
       <c r="J159" t="str">
         <v>REQ-14452. Distinct req from the identically-titled REQ-14465 above (same site/title, separate req IDs) — both independently confirmed open, not a duplicate.</v>
+      </c>
+      <c r="K159" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L159" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M159" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="160">
@@ -7540,6 +7720,66 @@
     <hyperlink ref="K139" r:id="rId381"/>
     <hyperlink ref="L139" r:id="rId382"/>
     <hyperlink ref="M139" r:id="rId383"/>
+    <hyperlink ref="K140" r:id="rId384"/>
+    <hyperlink ref="L140" r:id="rId385"/>
+    <hyperlink ref="M140" r:id="rId386"/>
+    <hyperlink ref="K141" r:id="rId387"/>
+    <hyperlink ref="L141" r:id="rId388"/>
+    <hyperlink ref="M141" r:id="rId389"/>
+    <hyperlink ref="K142" r:id="rId390"/>
+    <hyperlink ref="L142" r:id="rId391"/>
+    <hyperlink ref="M142" r:id="rId392"/>
+    <hyperlink ref="K143" r:id="rId393"/>
+    <hyperlink ref="L143" r:id="rId394"/>
+    <hyperlink ref="M143" r:id="rId395"/>
+    <hyperlink ref="K144" r:id="rId396"/>
+    <hyperlink ref="L144" r:id="rId397"/>
+    <hyperlink ref="M144" r:id="rId398"/>
+    <hyperlink ref="K145" r:id="rId399"/>
+    <hyperlink ref="L145" r:id="rId400"/>
+    <hyperlink ref="M145" r:id="rId401"/>
+    <hyperlink ref="K146" r:id="rId402"/>
+    <hyperlink ref="L146" r:id="rId403"/>
+    <hyperlink ref="M146" r:id="rId404"/>
+    <hyperlink ref="K147" r:id="rId405"/>
+    <hyperlink ref="L147" r:id="rId406"/>
+    <hyperlink ref="M147" r:id="rId407"/>
+    <hyperlink ref="K148" r:id="rId408"/>
+    <hyperlink ref="L148" r:id="rId409"/>
+    <hyperlink ref="M148" r:id="rId410"/>
+    <hyperlink ref="K149" r:id="rId411"/>
+    <hyperlink ref="L149" r:id="rId412"/>
+    <hyperlink ref="M149" r:id="rId413"/>
+    <hyperlink ref="K150" r:id="rId414"/>
+    <hyperlink ref="L150" r:id="rId415"/>
+    <hyperlink ref="M150" r:id="rId416"/>
+    <hyperlink ref="K151" r:id="rId417"/>
+    <hyperlink ref="L151" r:id="rId418"/>
+    <hyperlink ref="M151" r:id="rId419"/>
+    <hyperlink ref="K152" r:id="rId420"/>
+    <hyperlink ref="L152" r:id="rId421"/>
+    <hyperlink ref="M152" r:id="rId422"/>
+    <hyperlink ref="K153" r:id="rId423"/>
+    <hyperlink ref="L153" r:id="rId424"/>
+    <hyperlink ref="M153" r:id="rId425"/>
+    <hyperlink ref="K154" r:id="rId426"/>
+    <hyperlink ref="L154" r:id="rId427"/>
+    <hyperlink ref="M154" r:id="rId428"/>
+    <hyperlink ref="K155" r:id="rId429"/>
+    <hyperlink ref="L155" r:id="rId430"/>
+    <hyperlink ref="M155" r:id="rId431"/>
+    <hyperlink ref="K156" r:id="rId432"/>
+    <hyperlink ref="L156" r:id="rId433"/>
+    <hyperlink ref="M156" r:id="rId434"/>
+    <hyperlink ref="K157" r:id="rId435"/>
+    <hyperlink ref="L157" r:id="rId436"/>
+    <hyperlink ref="M157" r:id="rId437"/>
+    <hyperlink ref="K158" r:id="rId438"/>
+    <hyperlink ref="L158" r:id="rId439"/>
+    <hyperlink ref="M158" r:id="rId440"/>
+    <hyperlink ref="K159" r:id="rId441"/>
+    <hyperlink ref="L159" r:id="rId442"/>
+    <hyperlink ref="M159" r:id="rId443"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
applications batch 8: rows 160-172 (13 new document sets)
New documents for Entegris Bedford and Billerica (3), MetOx, Sanofi Swiftwater, Marathon Midstream (2), Rendezvous Robotics (3), Vast (2), and Moog. All files checked at one page in Word.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -6950,6 +6950,15 @@
       <c r="J160" t="str">
         <v>REQ-14458. Bedford, MA sibling req.</v>
       </c>
+      <c r="K160" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L160" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M160" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -6982,6 +6991,15 @@
       <c r="J161" t="str">
         <v>REQ-14399. Bedford, MA sibling req.</v>
       </c>
+      <c r="K161" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L161" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M161" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -7014,6 +7032,15 @@
       <c r="J162" t="str">
         <v>New company for the tracker — superconducting-technology energy startup. SolidWorks/FEA/CFD-focused mechanical design role, Balance-of-Plant systems. Co-Op option begins January 2027 (Spring start), included per the same 'distinct dated Spring option within a combined-term posting' treatment as Hermeus.</v>
       </c>
+      <c r="K162" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L162" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M162" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
@@ -7046,6 +7073,15 @@
       <c r="J163" t="str">
         <v>Umbrella-style posting, same pattern as the already-tracked Sanofi/Genzyme Framingham row — multiple near-identical parallel req IDs found on job-board mirrors (biospace.com job 3075194 'Engineering &amp; Maintenance' track at $35/hr, plus others at 3075170/3062903/3069311) likely representing different functional tracks of the same 2027 Spring Co-op program. Requires permanent US work authorization without sponsorship. Distinct from the already-tracked Sanofi (Genzyme) Framingham, MA row.</v>
       </c>
+      <c r="K163" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L163" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M163" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -7078,6 +7114,15 @@
       <c r="J164" t="str">
         <v>New sibling req beyond the already-tracked Refining Mechanical Engineer (Spring 2027) req 00020137 at the same Findlay, OH site — this one covers the Logistics &amp; Storage organization (pipelines/marine transport).</v>
       </c>
+      <c r="K164" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L164" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M164" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
@@ -7110,6 +7155,15 @@
       <c r="J165" t="str">
         <v>New sibling req beyond the already-tracked Marathon Petroleum entries — covers Natural Gas &amp; NGL Services (pipeline integrity, compressor/pump stations, automation/controls).</v>
       </c>
+      <c r="K165" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L165" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M165" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
@@ -7142,6 +7196,15 @@
       <c r="J166" t="str">
         <v>New company for the tracker — small spacecraft-assembly startup (electromagnetic self-assembling tiles). First published 2026-07-22; still listed live on the board as of this run despite being ~2 months old.</v>
       </c>
+      <c r="K166" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L166" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M166" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -7174,6 +7237,15 @@
       <c r="J167" t="str">
         <v>Dynamics/controls of a reconfigurable spacecraft assembled from electromagnetically-docked tiles; open to aerospace/mechanical/electrical/physics majors with coursework in dynamics and controls — squarely a controls/flight-systems role, same treatment as the already-tracked Hermeus GNC intern.</v>
       </c>
+      <c r="K167" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L167" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M167" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -7206,6 +7278,15 @@
       <c r="J168" t="str">
         <v>Open to Mechanical/Electrical/Industrial Engineering majors; testbed development, manufacturing support, and hardware verification for spacecraft tiles.</v>
       </c>
+      <c r="K168" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L168" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M168" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -7238,6 +7319,15 @@
       <c r="J169" t="str">
         <v>Previously excluded in 3 prior runs (2026-09-23) because the posting had no season/term field at all — this session's direct re-fetch found the application form now includes a genuine dated Spring 2027 option, same 'distinct dated Spring slot within a combined-term posting' treatment as Hermeus. ITAR: US person status required.</v>
       </c>
+      <c r="K169" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L169" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M169" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
@@ -7270,6 +7360,15 @@
       <c r="J170" t="str">
         <v>Sibling req to the Mechanical/Aerospace Engineering Internship above, same site/pay/season structure.</v>
       </c>
+      <c r="K170" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L170" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M170" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
@@ -7302,6 +7401,15 @@
       <c r="J171" t="str">
         <v>Corrects an earlier (2026-09-22) `checked` entry that had lumped this req in with 3 Summer-2027 Mineral Wells siblings (R-26-19881/19882/19887, which remain correctly excluded) — this session's fresh direct fetch shows R-26-19186 now/actually states Spring 2027, a different season from those siblings.</v>
       </c>
+      <c r="K171" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L171" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M171" t="str">
+        <v>Open questions</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
@@ -7333,6 +7441,15 @@
       </c>
       <c r="J172" t="str">
         <v>New sibling req beyond the 13 already-tracked Entegris Billerica/Bedford reqs, found via this session's own Entegris jobs-search API sweep (not from either research agent, who both mis-transcribed nearby req numbers — see ROUTINE-LOG for the correction).</v>
+      </c>
+      <c r="K172" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L172" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M172" t="str">
+        <v>Open questions</v>
       </c>
     </row>
   </sheetData>
@@ -7780,6 +7897,45 @@
     <hyperlink ref="K159" r:id="rId441"/>
     <hyperlink ref="L159" r:id="rId442"/>
     <hyperlink ref="M159" r:id="rId443"/>
+    <hyperlink ref="K160" r:id="rId444"/>
+    <hyperlink ref="L160" r:id="rId445"/>
+    <hyperlink ref="M160" r:id="rId446"/>
+    <hyperlink ref="K161" r:id="rId447"/>
+    <hyperlink ref="L161" r:id="rId448"/>
+    <hyperlink ref="M161" r:id="rId449"/>
+    <hyperlink ref="K162" r:id="rId450"/>
+    <hyperlink ref="L162" r:id="rId451"/>
+    <hyperlink ref="M162" r:id="rId452"/>
+    <hyperlink ref="K163" r:id="rId453"/>
+    <hyperlink ref="L163" r:id="rId454"/>
+    <hyperlink ref="M163" r:id="rId455"/>
+    <hyperlink ref="K164" r:id="rId456"/>
+    <hyperlink ref="L164" r:id="rId457"/>
+    <hyperlink ref="M164" r:id="rId458"/>
+    <hyperlink ref="K165" r:id="rId459"/>
+    <hyperlink ref="L165" r:id="rId460"/>
+    <hyperlink ref="M165" r:id="rId461"/>
+    <hyperlink ref="K166" r:id="rId462"/>
+    <hyperlink ref="L166" r:id="rId463"/>
+    <hyperlink ref="M166" r:id="rId464"/>
+    <hyperlink ref="K167" r:id="rId465"/>
+    <hyperlink ref="L167" r:id="rId466"/>
+    <hyperlink ref="M167" r:id="rId467"/>
+    <hyperlink ref="K168" r:id="rId468"/>
+    <hyperlink ref="L168" r:id="rId469"/>
+    <hyperlink ref="M168" r:id="rId470"/>
+    <hyperlink ref="K169" r:id="rId471"/>
+    <hyperlink ref="L169" r:id="rId472"/>
+    <hyperlink ref="M169" r:id="rId473"/>
+    <hyperlink ref="K170" r:id="rId474"/>
+    <hyperlink ref="L170" r:id="rId475"/>
+    <hyperlink ref="M170" r:id="rId476"/>
+    <hyperlink ref="K171" r:id="rId477"/>
+    <hyperlink ref="L171" r:id="rId478"/>
+    <hyperlink ref="M171" r:id="rId479"/>
+    <hyperlink ref="K172" r:id="rId480"/>
+    <hyperlink ref="L172" r:id="rId481"/>
+    <hyperlink ref="M172" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:M172"/>

</xml_diff>

<commit_message>
routine: 12 new postings, 3 checked-excluded (2026-09-25 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0192nUTF8zpQaQSzxdoUQFwy
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M172"/>
+  <dimension ref="A1:M184"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -7450,6 +7450,390 @@
       </c>
       <c r="M172" t="str">
         <v>Open questions</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B173" t="str">
+        <v>Test Engineering Intern, Spring 2027</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Systems / Test Engineering</v>
+      </c>
+      <c r="D173" t="str">
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+      </c>
+      <c r="E173" t="str">
+        <v>Wallops Island, VA</v>
+      </c>
+      <c r="F173">
+        <v>350</v>
+      </c>
+      <c r="G173" t="str">
+        <v>$25/hr (VA base pay range)</v>
+      </c>
+      <c r="H173" t="str">
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8003533003</v>
+      </c>
+      <c r="I173" t="str">
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season and VA pay range confirmed in body.</v>
+      </c>
+      <c r="J173" t="str">
+        <v>New site distinct from the already-tracked Stennis Space Center, MS 'Test Engineering Intern' (job 7990352003) — same title, different req/location.</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B174" t="str">
+        <v>Hardware Test Engineering Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Mechanical / Hardware Test Engineering</v>
+      </c>
+      <c r="D174" t="str">
+        <v>Winter/Spring 2027 (January - April)</v>
+      </c>
+      <c r="E174" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F174">
+        <v>3</v>
+      </c>
+      <c r="G174" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H174" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8196515</v>
+      </c>
+      <c r="I174" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Internship Term: Winter/Spring (January - April)' confirmed in body, title states 2027.</v>
+      </c>
+      <c r="J174" t="str">
+        <v>New sibling req beyond the already-tracked Formlabs Mechanical/Manufacturing/Hardware R&amp;D/Materials interns.</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Print Optimization Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Manufacturing / Process Engineering</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Winter/Spring 2027 (January - April)</v>
+      </c>
+      <c r="E175" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F175">
+        <v>3</v>
+      </c>
+      <c r="G175" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H175" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172256</v>
+      </c>
+      <c r="I175" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title and 'January - April' term confirmed in body.</v>
+      </c>
+      <c r="J175" t="str">
+        <v>New sibling req; 3D-printing process/optimization work, manufacturing-adjacent.</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B176" t="str">
+        <v>Print Process Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Manufacturing / Process Engineering</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Winter/Spring 2027 (January - April)</v>
+      </c>
+      <c r="E176" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F176">
+        <v>3</v>
+      </c>
+      <c r="G176" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H176" t="str">
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199269</v>
+      </c>
+      <c r="I176" t="str">
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title confirmed in body.</v>
+      </c>
+      <c r="J176" t="str">
+        <v>New sibling req; 3D-printing process work, manufacturing-adjacent.</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B177" t="str">
+        <v>Subsystem Test Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Test Engineering</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
+      </c>
+      <c r="E177" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F177">
+        <v>950</v>
+      </c>
+      <c r="G177" t="str">
+        <v>$25-$33/hr</v>
+      </c>
+      <c r="H177" t="str">
+        <v>https://jobs.lever.co/hermeus/643fd7b7-9015-43a1-aa2b-a54f117b403c</v>
+      </c>
+      <c r="I177" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option, same treatment as other already-tracked Hermeus combined-term reqs.</v>
+      </c>
+      <c r="J177" t="str">
+        <v>New sibling req; also listed at Los Angeles, CA per allLocations.</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Test and Operations Engineering Intern (Spring/Summer 2027)</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Test / Operations Engineering</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
+      </c>
+      <c r="E178" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F178">
+        <v>2600</v>
+      </c>
+      <c r="G178" t="str">
+        <v>$25-$33/hr</v>
+      </c>
+      <c r="H178" t="str">
+        <v>https://jobs.lever.co/hermeus/d40446ee-40a9-4bb0-a3a8-a4a189b74630</v>
+      </c>
+      <c r="I178" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option.</v>
+      </c>
+      <c r="J178" t="str">
+        <v>New sibling req.</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Specialty Coatings Research and Development Co-Op</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Materials / Coatings Engineering</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Spring 2027 season</v>
+      </c>
+      <c r="E179" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F179">
+        <v>16</v>
+      </c>
+      <c r="G179" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H179" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Entegris-Specialty-Coatings-Research-and-Development-Co-Op_REQ-14441</v>
+      </c>
+      <c r="I179" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14441, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J179" t="str">
+        <v>New sibling req beyond the already-tracked 14 Entegris Billerica/Bedford reqs.</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B180" t="str">
+        <v>New Product Introduction Co-Op</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Manufacturing / NPI Engineering</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Spring 2027 season</v>
+      </c>
+      <c r="E180" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F180">
+        <v>16</v>
+      </c>
+      <c r="G180" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H180" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/New-Product-Introduction-Co-Op_REQ-14461-1</v>
+      </c>
+      <c r="I180" t="str">
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14461, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J180" t="str">
+        <v>New sibling req.</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Colibrium Additive US Manufacturing / Supply Chain Co-op - Spring 2027</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Manufacturing / Supply Chain Engineering (Additive Manufacturing)</v>
+      </c>
+      <c r="D181" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E181" t="str">
+        <v>West Chester, OH</v>
+      </c>
+      <c r="F181">
+        <v>700</v>
+      </c>
+      <c r="G181" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H181" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/West-Chester/Colibrium-Additive-US-Manufacturing---Supply-Chain-Co-op---Spring-2027_R5040302-2</v>
+      </c>
+      <c r="I181" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040302, canApply true, posted 2 days ago.</v>
+      </c>
+      <c r="J181" t="str">
+        <v>New req found via a fresh Workday search sweep; not previously tracked.</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Flight Test Operation Engineering Intern - Victorville, CA - Spring 2027</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Flight Test / Systems Engineering</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Victorville, CA</v>
+      </c>
+      <c r="F182">
+        <v>2500</v>
+      </c>
+      <c r="G182" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H182" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Victorville/Flight-Test-Operation-Engineering-Intern---Victorville--CA---Spring-2027_R5040433-1</v>
+      </c>
+      <c r="I182" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040433, canApply true, posted 3 days ago.</v>
+      </c>
+      <c r="J182" t="str">
+        <v>New req; flight-test/flight-systems discipline fit.</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Systems Engineering Co-op - Mechanical/Aerospace Engineering (Electric Power) - US - Spring 2027</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Systems Engineering (Mechanical/Aerospace)</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E183" t="str">
+        <v>Dayton, OH</v>
+      </c>
+      <c r="F183">
+        <v>750</v>
+      </c>
+      <c r="G183" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H183" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Dayton/Systems-Engineering-Co-op---Mechanical-Aerospace-Engineering--Electric-Power----US---Spring-2027_R5030103-1</v>
+      </c>
+      <c r="I183" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5030103, canApply true, posted 30+ days ago.</v>
+      </c>
+      <c r="J183" t="str">
+        <v>New req found via a fresh Workday search sweep. A parallel Electrical Engineering/Computer Engineering version (R5030099) at the same site was reviewed and excluded — EE/CS discipline.</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Unison Engineering Part-time Co-op - US - Spring 2027</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Mechanical / Manufacturing Engineering (Unison Industries subsidiary)</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E184" t="str">
+        <v>Saint George, UT</v>
+      </c>
+      <c r="F184">
+        <v>2300</v>
+      </c>
+      <c r="G184" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H184" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Saint-George-UT-US-1/Unison-Engineering-Part-time-Co-op---US---Spring-2027_R5040016</v>
+      </c>
+      <c r="I184" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040016, canApply true, posted 9 days ago.</v>
+      </c>
+      <c r="J184" t="str">
+        <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
       </c>
     </row>
   </sheetData>
@@ -7938,14 +8322,14 @@
     <hyperlink ref="M172" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M172"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M184"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C358"/>
+  <dimension ref="A1:C361"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -11890,9 +12274,42 @@
         <v>2026-09-25 ~01:00 UTC: none of these 3 req numbers exist — this session's own Entegris jobs-search API returned zero results for each. Cross-referencing by title/location instead found the real req numbers: Capital Equipment Engineering Co-Op at Billerica, MA is actually REQ-14497 (already tracked in `rows`); Manufacturing Engineering Co-Op at Billerica, MA is actually REQ-14492 (already tracked); Materials Engineering Co-Op is at Chaska, MN (REQ-14451), not a Massachusetts site at all — wrong location, not added. Same pattern as a prior run's 'REQ-7046' mis-transcription. This same search sweep did surface one genuinely new req — Application Engineering Co-Op, Billerica MA (REQ-14473) — added to `rows`.</v>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>Rocket Lab</v>
+      </c>
+      <c r="B359" t="str">
+        <v>Flight Software Intern, Spring 2027 (Littleton, CO, job 7989724003); Mechanical Engineering Intern, Spring 2027 (Toronto, Canada, job 7986368003)</v>
+      </c>
+      <c r="C359" t="str">
+        <v>2026-09-25 ~07:00 UTC: both confirmed live via direct Greenhouse API fetch. Flight Software Intern excluded on discipline grounds (software, not hardware/mechanical), consistent with prior treatment of Rocket Lab's other Flight Software reqs. Toronto req excluded on location grounds (non-US), consistent with prior treatment of Rocket Lab's other Canada-based reqs.</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B360" t="str">
+        <v>Full 'Winter 2027' cohort batch (San Francisco, CA) — Environmental Test Engineer Intern (job 4705652006), Harness Design Engineer Intern, Harness Manufacturing Intern, Propulsion Engineer/Manufacturing/Test Intern, Production Quality Intern, Reliability Test Intern, Supplier Quality Engineer Intern, Thermal Intern, AIT Intern, Hardware Test Intern, Antenna Intern, CAD Engineer Intern</v>
+      </c>
+      <c r="C360" t="str">
+        <v>2026-09-25 ~07:00 UTC: confirmed live via direct Greenhouse API fetch (HTTP 200), but each posting states only 'Winter 2027' with no date range given in the body, and Astranis maintains 'Winter 2027' as a track explicitly distinct from its already-tracked 'Spring 2027' reqs (separate job IDs, separate titles). Consistent with this tracker's prior exclusion of Astranis's Winter 2027 Mechanical Engineer Intern (job 4704600006) on season grounds — Hamza's target seasons are Winter 2026 or Spring 2027 specifically, not Winter 2027. Not added.</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B361" t="str">
+        <v>Unison Engineering Part-time Co-op - US - Fall 2027 (R5040164, Saint George UT), Unison Engineering Part-time Intern - US - Summer 2027 (R5040163, Saint George UT), Unison Engineering Intern - Fall 2027 (R5037092, 4 locations)</v>
+      </c>
+      <c r="C361" t="str">
+        <v>2026-09-25 ~07:00 UTC: confirmed live via direct Workday CXS API fetch, but all three are Fall or Summer 2027 — wrong season. The parallel Spring 2027 Unison req (R5040016) was added to `rows`.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C358"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C361"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 17 checked-excluded (2026-09-25 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qs3ZumvzHkSdPoQrAASkFv
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M184"/>
+  <dimension ref="A1:M187"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -7834,6 +7834,102 @@
       </c>
       <c r="J184" t="str">
         <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Symbotic</v>
+      </c>
+      <c r="B185" t="str">
+        <v>Co-op - Hardware Engineer</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Mechanical / Hardware Engineering (robotics)</v>
+      </c>
+      <c r="D185" t="str">
+        <v>Spring 2027 (January–May)</v>
+      </c>
+      <c r="E185" t="str">
+        <v>Wilmington, MA</v>
+      </c>
+      <c r="F185">
+        <v>17</v>
+      </c>
+      <c r="G185" t="str">
+        <v>$29.00–$40.00/hr</v>
+      </c>
+      <c r="H185" t="str">
+        <v>https://symbotic.wd504.myworkdayjobs.com/Symbotic/job/USA-Wilmington-MA---ITC/Hardware-Engineer_R7976</v>
+      </c>
+      <c r="I185" t="str">
+        <v>Yes — fetched directly via Symbotic's own Workday CXS API, req R7976, canApply true, posted 3 days ago.</v>
+      </c>
+      <c r="J185" t="str">
+        <v>Boston metro (Wilmington, MA — ITC site). Requires enrolled Bachelor's student in Systems/Robotics/Mechanical/Electrical/CS engineering. Hands-on electro-mechanical work: GD&amp;T, SolidWorks, manufacturing processes (machining, casting, sheet metal). Offers transportation/housing benefits for relocating students. A sibling req 'Co-op - Robot Perception' (R8113, same site/timeframe) was reviewed and excluded — Computer Vision/ML software discipline, requires Master's/PhD.</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Unison Engineering Intern - Spring 2027</v>
+      </c>
+      <c r="C186" t="str">
+        <v>Mechanical / Aerospace / Electrical Engineering (Unison Industries subsidiary)</v>
+      </c>
+      <c r="D186" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E186" t="str">
+        <v>Dayton, OH / Jacksonville, FL / Norwich, NY / St. George, UT (4 sites, one assignment)</v>
+      </c>
+      <c r="F186">
+        <v>750</v>
+      </c>
+      <c r="G186" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H186" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Jacksonville/Unison-Engineering-Intern---Spring-2027_R5037093-1</v>
+      </c>
+      <c r="I186" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5037093, canApply true, posted 30+ days ago.</v>
+      </c>
+      <c r="J186" t="str">
+        <v>Full-time intern version distinct from the already-tracked part-time 'Unison Engineering Part-time Co-op' (R5040016, St. George UT only). Works on ignition systems, sensors, generators, harnesses, engine starters at Unison Industries sites. Min 3.0 GPA, Aero/Mechanical/Electrical Engineering majors. Fall 2027 (R5037092) sibling at the same 4 sites was previously reviewed and excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B187" t="str">
+        <v>Build Reliability Engineering Intern - Spring/Summer 2027</v>
+      </c>
+      <c r="C187" t="str">
+        <v>Manufacturing Engineering (structural fabrication &amp; assembly)</v>
+      </c>
+      <c r="D187" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+      </c>
+      <c r="E187" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F187">
+        <v>950</v>
+      </c>
+      <c r="G187" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H187" t="str">
+        <v>https://jobs.lever.co/hermeus/ee3a4109-b6e7-4ed5-8981-a483b3936e5a</v>
+      </c>
+      <c r="I187" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, page live, distinct dated Spring option confirmed in body text.</v>
+      </c>
+      <c r="J187" t="str">
+        <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
       </c>
     </row>
   </sheetData>
@@ -8322,14 +8418,14 @@
     <hyperlink ref="M172" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M184"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M187"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C361"/>
+  <dimension ref="A1:C378"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -12307,9 +12403,196 @@
         <v>2026-09-25 ~07:00 UTC: confirmed live via direct Workday CXS API fetch, but all three are Fall or Summer 2027 — wrong season. The parallel Spring 2027 Unison req (R5040016) was added to `rows`.</v>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>Symbotic</v>
+      </c>
+      <c r="B362" t="str">
+        <v>'Co-op - Robot Perception', req R8113, Wilmington MA</v>
+      </c>
+      <c r="C362" t="str">
+        <v>2026-09-25 ~13:00 UTC: confirmed live via direct Workday CXS API fetch (canApply true, Spring Jan-May 2027 timeframe stated), but the role is a Computer Vision/Machine Learning research position (SLAM, deep learning, PyTorch/TensorFlow, sensor fusion) requiring a Master's or PhD in Computer Science/Robotics/EE/ML — a software/CS discipline, not the hardware/mechanical side of robotics on Hamza's target list, and a degree-level mismatch besides. Its sibling 'Co-op - Hardware Engineer' (R7976, same site/timeframe, Bachelor's-eligible, mechanical/electro-mechanical work) DID qualify and was added to `rows`.</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>WestRock / Smurfit Westrock (Cowpens, SC)</v>
+      </c>
+      <c r="B363" t="str">
+        <v>'Manufacturing Engineering Co-op - Spring 2027, Mills', final re-check</v>
+      </c>
+      <c r="C363" t="str">
+        <v>2026-09-25 ~13:00 UTC: the LinkedIn posting (job ID 4413763900) now returns an explicit 'expired_jd_redirect' query parameter when followed — LinkedIn's own signal that the original listing has closed. Resolved: treating as closed/dead, dropping from active watch.</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>Eaton (Jackson, MS)</v>
+      </c>
+      <c r="B364" t="str">
+        <v>'Co-op Design Engineering', final re-check</v>
+      </c>
+      <c r="C364" t="str">
+        <v>2026-09-25 ~13:00 UTC: LinkedIn's own listing for this exact role/location (job 4299544329, same $22.15-27.69/hr range) is now explicitly titled 'Co-op Design Engineering (Summer 2027)' — confirms the long-suspected roll-over from Spring to Summer 2027. Resolved: the Spring 2027 version is gone, not merely blocked. Dropping from active watch unless a new Spring-dated req appears.</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>BAE Systems</v>
+      </c>
+      <c r="B365" t="str">
+        <v>'2027 Spring and Summer Mechanical Engineering Coop' (125975BR), Cedar Rapids, IA</v>
+      </c>
+      <c r="C365" t="str">
+        <v>2026-09-25 ~13:00 UTC: new req for the tracker, but jobs.baesystems.com now shows 'no longer accepting applications' — confirmed closed on direct fetch. Worth a re-check for a fresh BAE Systems Mechanical Engineering coop at this or other sites (Nashua NH, Endicott NY, Manassas VA) in a future run, since this title pattern shows BAE does issue Spring-2027-dated mechanical coops.</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>RTX / Pratt &amp; Whitney</v>
+      </c>
+      <c r="B366" t="str">
+        <v>Workday-wide search for Pratt &amp; Whitney-branded (non-Collins) Winter 2026/Spring 2027 US co-ops</v>
+      </c>
+      <c r="C366" t="str">
+        <v>2026-09-25 ~13:00 UTC: no qualifying posting found. All P&amp;W 'Stage - Hiver 2027 / Internship Winter 2027' reqs (10+) are Canada-located (Longueuil/Saint-Hubert, QC) — excluded on location. Two Workday reqs explicitly titled 'Winter/Spring 2027' mechanical co-ops (Rockford IL req 01869227, Jamestown ND req 01871736) were found but both are already tracked in `rows` under Collins Aerospace, same site/req — not duplicated.</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>Curtiss-Wright</v>
+      </c>
+      <c r="B367" t="str">
+        <v>'Co-op (Spring Term)' JR1907, Cheswick PA (Electro-Mechanical Division)</v>
+      </c>
+      <c r="C367" t="str">
+        <v>2026-09-25 ~13:00 UTC: confirmed live via direct Workday fetch (canApply true), but this is a generic evergreen req ('hiring for Spring, Summer, and Fall semesters,' posted 30+ days ago with a stale 2025-02-07 date-on-file) with no distinct Spring-2027 dating — fails the season verification bar. A separate 'Purchasing &amp; Supply Chain Intern (Spring 2027 Semester)' req (JR12367, Middleburg Hts OH) has explicit Spring 2027 dating but is a Purchasing/business discipline, not engineering — excluded.</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>Saab, Inc.</v>
+      </c>
+      <c r="B368" t="str">
+        <v>'Systems Engineering Co-Op (Spring - Summer 2027)' x2 and 'Co-Op, Contracts Spring 2027', East Syracuse NY</v>
+      </c>
+      <c r="C368" t="str">
+        <v>2026-09-25 ~13:00 UTC: both Systems Engineering Co-Ops confirmed live via direct Workday fetch, but use a combined 'Spring - Summer 2027' term with no distinct Spring-only slot (fails season bar), and the discipline is Air Traffic Management/Digital Tower software integration — not mechanical/aerospace hardware. The Contracts Co-Op has explicit Spring 2027 dating but is a business discipline. Only mechanical-titled Saab reqs currently live are Summer 2027 (already excluded in a prior run).</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>Aerojet Rocketdyne (L3Harris)</v>
+      </c>
+      <c r="B369" t="str">
+        <v>General Winter 2026/Spring 2027 mechanical/propulsion internship search</v>
+      </c>
+      <c r="C369" t="str">
+        <v>2026-09-25 ~13:00 UTC: careers.l3harris.com is a heavily JS-rendered SPA with no identifiable public API — WebFetch returned only navigation scaffolding. No live Spring 2027/Winter 2026 posting could be found or independently verified at Canoga Park/Redmond/Huntsville sites; only Summer 2026/2027-cycle mentions surfaced in search snippets.</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>Aurora Flight Sciences (Boeing)</v>
+      </c>
+      <c r="B370" t="str">
+        <v>General Winter 2026/Spring 2027 internship search</v>
+      </c>
+      <c r="C370" t="str">
+        <v>2026-09-25 ~13:00 UTC: careers.aurora.aero and jobs.boeing.com are both JS-rendered SPAs that returned only scaffolding to WebFetch — no listings visible. Search snippets show only Summer 2026 program mentions. No qualifying posting found or verifiable.</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>ispace</v>
+      </c>
+      <c r="B371" t="str">
+        <v>General internship search</v>
+      </c>
+      <c r="C371" t="str">
+        <v>2026-09-25 ~13:00 UTC: ispace-inc.com/careers-en/ returns 404; no live careers page or identifiable ATS found for the US (Englewood, CO) office. No current posting located.</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>HII (Huntington Ingalls Industries)</v>
+      </c>
+      <c r="B372" t="str">
+        <v>General Winter 2026/Spring 2027 internship/co-op search via careers.huntingtoningalls.com</v>
+      </c>
+      <c r="C372" t="str">
+        <v>2026-09-25 ~13:00 UTC: direct site search confirms only a Fall 2026 Designer Co-Op (Newport News) and Summer 2027 College Internships (Pascagoula: Structural &amp; Aerospace, Mechanical, Naval Architecture) are currently live, plus military-only SkillBridge internships (not applicable). No Winter 2026 or Spring 2027 posting exists at HII right now.</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>Bell Textron / Textron Systems</v>
+      </c>
+      <c r="B373" t="str">
+        <v>General Winter 2026/Spring 2027 search on careers.textron.com</v>
+      </c>
+      <c r="C373" t="str">
+        <v>2026-09-25 ~13:00 UTC: confirmed via raw HTML fetch that careers.textron.com is a client-side-rendered Nuxt SPA (data-ssr="false") with no job data in server-side HTML — automated verification remains structurally blocked. Search snippets show only Summer 2027 intern cycles at Fort Worth (Bell) and no re-surfacing of the previously-tracked Hunt Valley Sea Systems req (consistent with it having closed). No qualifying posting could be confirmed.</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>Reliable Robotics</v>
+      </c>
+      <c r="B374" t="str">
+        <v>Full live Ashby board (56 open reqs)</v>
+      </c>
+      <c r="C374" t="str">
+        <v>2026-09-25 ~13:00 UTC: zero internships of any kind currently posted — all 56 open reqs are full-time (Mechanical/Systems/Avionics/Flight Software Engineer). A previously-seen 'Fall 2026 Internship' listing is no longer on the live board.</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>Impulse Space (Redondo Beach, CA)</v>
+      </c>
+      <c r="B375" t="str">
+        <v>re-check for a Spring-2027-dated mechanical/propulsion/structures req</v>
+      </c>
+      <c r="C375" t="str">
+        <v>2026-09-25 ~13:00 UTC: re-confirmed via Ashby + aggregator cross-check — all mechanical/propulsion/avionics/opto-mechanical/structures internships remain Summer 2027 only. Antenna/RF Engineering Intern is still the only Spring-2027-dated role (electrical discipline, already excluded). No change across multiple consecutive runs.</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B376" t="str">
+        <v>Intern-Industrial Controls (R7973), Intern-Hardware Engineer (R8101), Intern-Bot Controls (R7965)</v>
+      </c>
+      <c r="C376" t="str">
+        <v>2026-09-25 ~13:00 UTC: all three confirmed live via direct Workday CXS API fetch, but all are Summer 2027 — wrong season. (Two Spring 2027-dated siblings, 'Co-op- Hardware Engineer' R7976 and 'Co-op - Robot Perception' R8113, were reviewed separately — see `rows` and the R8113 exclusion above.)</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>Caterpillar</v>
+      </c>
+      <c r="B377" t="str">
+        <v>Full Workday query across all 2027 engineering internship/co-op reqs (Mossville IL, Peoria IL, East Syracuse NY, West Lafayette IN)</v>
+      </c>
+      <c r="C377" t="str">
+        <v>2026-09-25 ~13:00 UTC: every 2027 req found is explicitly labeled '2027 Summer Corporate Intern' or 'Mechanical Engineer Co-Op (Summer 2027)' — zero Winter 2026 or Spring 2027 results for any search variant tried.</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>BETA Technologies</v>
+      </c>
+      <c r="B378" t="str">
+        <v>General Winter 2026/Spring 2027 internship search</v>
+      </c>
+      <c r="C378" t="str">
+        <v>2026-09-25 ~13:00 UTC: jobs.lever.co/beta now returns an empty postings array; the two specific '2026-2027 BETA Internship' posting URLs found via search both 404. beta.team/careers is JS-rendered with no listings in server HTML. Company may have switched ATS — no live posting could be located or verified.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C361"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C378"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 7 checked-excluded (2026-09-25 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FjzJYaLc9ccuyHXeCay4Vc
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M187"/>
+  <dimension ref="A1:M189"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -7930,6 +7930,70 @@
       </c>
       <c r="J187" t="str">
         <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>PI (Physik Instrumente) USA</v>
+      </c>
+      <c r="B188" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C188" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D188" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E188" t="str">
+        <v>Shrewsbury, MA</v>
+      </c>
+      <c r="F188">
+        <v>40</v>
+      </c>
+      <c r="G188" t="str">
+        <v>$24-26/hour</v>
+      </c>
+      <c r="H188" t="str">
+        <v>https://www.pi-usa.us/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+      </c>
+      <c r="I188" t="str">
+        <v>Yes — fetched directly, HTTP 200, page title 'Mechanical Engineering Co-op - Winter/Spring 2027', full description read.</v>
+      </c>
+      <c r="J188" t="str">
+        <v>New company for the tracker. Boston metro (Shrewsbury, MA — PI's US headquarters). High-precision positioning/motion systems and piezo technology manufacturer. Prepares detail/assembly drawings, CAD support, PLM data entry, R&amp;D build/test work. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship. SolidWorks and manufacturing-process experience preferred.</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>PI (Physik Instrumente) USA</v>
+      </c>
+      <c r="B189" t="str">
+        <v>Manufacturing Engineering Internship</v>
+      </c>
+      <c r="C189" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D189" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Shrewsbury, MA</v>
+      </c>
+      <c r="F189">
+        <v>40</v>
+      </c>
+      <c r="G189" t="str">
+        <v>$24-26/hour</v>
+      </c>
+      <c r="H189" t="str">
+        <v>https://www.pi-usa.us/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
+      </c>
+      <c r="I189" t="str">
+        <v>Yes — fetched directly, HTTP 200, page title 'Manufacturing Engineering Internship - Winter/Spring 2027', full description read.</v>
+      </c>
+      <c r="J189" t="str">
+        <v>Sibling req to the Mechanical Engineering Co-op above, same site/pay/season. Fixture design for assembly/metrology/manufacturing, SolidWorks modeling, hands-on machining (mills, lathes, saws, 3D printers), process optimization, ECR/ECO documentation. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship.</v>
       </c>
     </row>
   </sheetData>
@@ -8418,14 +8482,14 @@
     <hyperlink ref="M172" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M187"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M189"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C378"/>
+  <dimension ref="A1:C385"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -12590,9 +12654,86 @@
         <v>2026-09-25 ~13:00 UTC: jobs.lever.co/beta now returns an empty postings array; the two specific '2026-2027 BETA Internship' posting URLs found via search both 404. beta.team/careers is JS-rendered with no listings in server HTML. Company may have switched ATS — no live posting could be located or verified.</v>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>Leidos</v>
+      </c>
+      <c r="B379" t="str">
+        <v>'Mechanical Engineering Intern' (R-00193159, Albuquerque, NM) and 'Power Delivery Engineering Intern' (R-00192019, Greensboro, NC) — priority re-check after being flagged as skipped by a prior run</v>
+      </c>
+      <c r="C379" t="str">
+        <v>2026-09-25 ~19:00 UTC: both confirmed live/open via direct Workday CXS API fetch (this session's own fetch, full job description read end-to-end), but neither posting states any season/term (Winter/Spring/Summer/Fall) or year anywhere in the body — fails the 'season stated' verification bar. All other Leidos ME/AE internship reqs found this run (Aerospace M&amp;S Engineer Intern, Lunar Terrain Vehicle Engineering Intern, Laser Air Monitoring System Engineering Intern, Radar Engineer Intern, all Huntsville AL) are explicitly Summer 2027 — excluded on season grounds. Not added.</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>RTX / Collins Aerospace (Cedar Rapids, IA)</v>
+      </c>
+      <c r="B380" t="str">
+        <v>'Advanced Manufacturing Engineering Co-Op (Spring/Summer 2027)', req 01874253</v>
+      </c>
+      <c r="C380" t="str">
+        <v>2026-09-25 ~19:00 UTC: confirmed live via this session's own direct Workday CXS API fetch (posted 2026-09-24), but the description is a single merged 'Spring/Summer 2027' co-op session with no distinct Spring-only dated sub-range — same treatment as the already-excluded Burnsville, MN sibling (req 01874254). Not added.</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>Redwire Space</v>
+      </c>
+      <c r="B381" t="str">
+        <v>'Redwire Internship 2027' umbrella req, 3212</v>
+      </c>
+      <c r="C381" t="str">
+        <v>2026-09-25 ~19:00 UTC: confirmed live via direct page fetch (HTTP 200) — a single generic req covering ~15 different internship disciplines (incl. Mechanical, Manufacturing, Materials &amp; Process, Systems, RF Engineering) across 9 US sites including Marlborough, MA. But the posting states only '2027' with no Winter/Spring/Summer/Fall term specified anywhere — fails the season-stated verification bar. Worth re-checking if Redwire posts discipline-specific dated reqs later.</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>Eaton</v>
+      </c>
+      <c r="B382" t="str">
+        <v>'Manufacturing Engineer Co-op (Spring 2027)', Sumter, SC and 'Product Development Engineering Co-op (Spring 2027)', Hodges, SC — reported by a research agent via aggregator listings</v>
+      </c>
+      <c r="C382" t="str">
+        <v>2026-09-25 ~19:00 UTC: could not independently verify via Eaton's own career site this run — Eaton's Workday tenant/ATS could not be identified (guessed tenant URLs returned HTTP 500; eaton.com careers page failed to load cleanly). Only aggregator-sourced pay ranges available, no direct employer confirmation. Not added pending direct-source verification in a future run.</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>Formlabs (Somerville, MA)</v>
+      </c>
+      <c r="B383" t="str">
+        <v>'Industrial Design Intern (Winter/Spring 2027)', Greenhouse job 8172232</v>
+      </c>
+      <c r="C383" t="str">
+        <v>2026-09-25 ~19:00 UTC: confirmed live via direct Greenhouse API fetch (HTTP 200, correct Winter/Spring 2027 season), but the role sits on Formlabs' Industrial Design team (product aesthetics/user experience design), not Industrial Engineering/manufacturing — discipline mismatch against Hamza's target list despite the superficially matching 'Industrial' keyword. Not added.</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>Zipline (South San Francisco, CA)</v>
+      </c>
+      <c r="B384" t="str">
+        <v>'Materials Engineer Intern (Spring &amp; Summer 2027)', Greenhouse job 7905428003</v>
+      </c>
+      <c r="C384" t="str">
+        <v>2026-09-25 ~19:00 UTC: confirmed live via direct Greenhouse API fetch, but the body states this is one continuous internship hosted 'from January to August/September' — a single combined Spring+Summer stint, not a distinct dated Spring-only option (unlike other tracked Zipline/Hermeus/Vast reqs that offer a genuine standalone Spring slot). Fails the season-stated verification bar. Not added.</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>BAE Systems</v>
+      </c>
+      <c r="B385" t="str">
+        <v>'Operations Engineering (Ind/Mech/Elec) Co-op Spring/Summer 2027' sibling req 127776BR (Cedar Rapids, IA, re-check); full sweep of Nashua NH, Endicott NY, and Manassas VA sites for a Spring-2027-dated mechanical/systems coop</v>
+      </c>
+      <c r="C385" t="str">
+        <v>2026-09-25 ~19:00 UTC: 127776BR now also confirmed 'no longer accepting applications' (closed), joining its already-excluded Cedar Rapids siblings 125975BR/126541BR. No Spring-2027-dated mechanical/systems coop found at Nashua NH, Endicott NY, or Manassas VA — only postings found at those sites are Summer 2027 interns (Mechanical Engineering Intern III, Nashua NH, 129311BR onsite / 127637BR hybrid) or already-closed reqs (Industrial Engineering Co-Op Fall Semester 2026, Nashua NH, 124709BR — now HTTP 410 Gone). The Cedar Rapids Spring-coop naming pattern does not appear to extend to these other sites currently. Dropping active watch on this lead unless a new dated req surfaces.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C378"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C385"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 19 new postings, 5 checked-excluded (2026-09-26 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y9HcLmb2YVic3rjcV7zno5
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M189"/>
+  <dimension ref="A1:M208"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -7710,289 +7710,897 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>GE Aerospace</v>
+        <v>Entegris</v>
       </c>
       <c r="B181" t="str">
-        <v>Colibrium Additive US Manufacturing / Supply Chain Co-op - Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C181" t="str">
-        <v>Manufacturing / Supply Chain Engineering (Additive Manufacturing)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D181" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E181" t="str">
-        <v>West Chester, OH</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F181">
-        <v>700</v>
+        <v>885</v>
       </c>
       <c r="G181" t="str">
-        <v>Not stated on posting</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H181" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/West-Chester/Colibrium-Additive-US-Manufacturing---Supply-Chain-Co-op---Spring-2027_R5040302-2</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering--Co-Op_REQ-14442</v>
       </c>
       <c r="I181" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040302, canApply true, posted 2 days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J181" t="str">
-        <v>New req found via a fresh Workday search sweep; not previously tracked.</v>
+        <v>REQ-14442. Industrial/Manufacturing Engineering, Industry 4.0/smart-manufacturing focus. No H1-B sponsorship. Genuinely new site for the tracker (2026-09-26 sweep found Entegris's full nationwide Co-Op slate beyond the previously MA-only-tracked reqs).</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>GE Aerospace</v>
+        <v>Entegris</v>
       </c>
       <c r="B182" t="str">
-        <v>Flight Test Operation Engineering Intern - Victorville, CA - Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C182" t="str">
-        <v>Flight Test / Systems Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D182" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E182" t="str">
-        <v>Victorville, CA</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F182">
-        <v>2500</v>
+        <v>885</v>
       </c>
       <c r="G182" t="str">
-        <v>Not stated on posting</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H182" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Victorville/Flight-Test-Operation-Engineering-Intern---Victorville--CA---Spring-2027_R5040433-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14438</v>
       </c>
       <c r="I182" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040433, canApply true, posted 3 days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J182" t="str">
-        <v>New req; flight-test/flight-systems discipline fit.</v>
+        <v>REQ-14438. Sibling req to REQ-14442, same site. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>GE Aerospace</v>
+        <v>Entegris</v>
       </c>
       <c r="B183" t="str">
-        <v>Systems Engineering Co-op - Mechanical/Aerospace Engineering (Electric Power) - US - Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C183" t="str">
-        <v>Systems Engineering (Mechanical/Aerospace)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D183" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E183" t="str">
-        <v>Dayton, OH</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F183">
-        <v>750</v>
+        <v>885</v>
       </c>
       <c r="G183" t="str">
-        <v>Not stated on posting</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H183" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Dayton/Systems-Engineering-Co-op---Mechanical-Aerospace-Engineering--Electric-Power----US---Spring-2027_R5030103-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14394</v>
       </c>
       <c r="I183" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5030103, canApply true, posted 30+ days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J183" t="str">
-        <v>New req found via a fresh Workday search sweep. A parallel Electrical Engineering/Computer Engineering version (R5030099) at the same site was reviewed and excluded — EE/CS discipline.</v>
+        <v>REQ-14394. Chemical/Mechanical/Industrial/Manufacturing Engineering majors; quality engineering coursework a plus. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>GE Aerospace</v>
+        <v>Entegris</v>
       </c>
       <c r="B184" t="str">
-        <v>Unison Engineering Part-time Co-op - US - Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C184" t="str">
-        <v>Mechanical / Manufacturing Engineering (Unison Industries subsidiary)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D184" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E184" t="str">
-        <v>Saint George, UT</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F184">
-        <v>2300</v>
+        <v>885</v>
       </c>
       <c r="G184" t="str">
-        <v>Not stated on posting</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H184" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Saint-George-UT-US-1/Unison-Engineering-Part-time-Co-op---US---Spring-2027_R5040016</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14412</v>
       </c>
       <c r="I184" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040016, canApply true, posted 9 days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J184" t="str">
-        <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
+        <v>REQ-14412. Same discipline mix as REQ-14394. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>Symbotic</v>
+        <v>Entegris</v>
       </c>
       <c r="B185" t="str">
-        <v>Co-op - Hardware Engineer</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C185" t="str">
-        <v>Mechanical / Hardware Engineering (robotics)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D185" t="str">
-        <v>Spring 2027 (January–May)</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E185" t="str">
-        <v>Wilmington, MA</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F185">
-        <v>17</v>
+        <v>1137</v>
       </c>
       <c r="G185" t="str">
-        <v>$29.00–$40.00/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H185" t="str">
-        <v>https://symbotic.wd504.myworkdayjobs.com/Symbotic/job/USA-Wilmington-MA---ITC/Hardware-Engineer_R7976</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14409</v>
       </c>
       <c r="I185" t="str">
-        <v>Yes — fetched directly via Symbotic's own Workday CXS API, req R7976, canApply true, posted 3 days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J185" t="str">
-        <v>Boston metro (Wilmington, MA — ITC site). Requires enrolled Bachelor's student in Systems/Robotics/Mechanical/Electrical/CS engineering. Hands-on electro-mechanical work: GD&amp;T, SolidWorks, manufacturing processes (machining, casting, sheet metal). Offers transportation/housing benefits for relocating students. A sibling req 'Co-op - Robot Perception' (R8113, same site/timeframe) was reviewed and excluded — Computer Vision/ML software discipline, requires Master's/PhD.</v>
+        <v>REQ-14409. Industrial/Mechanical/Manufacturing Engineering, grad 2027-2029. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>GE Aerospace</v>
+        <v>Entegris</v>
       </c>
       <c r="B186" t="str">
-        <v>Unison Engineering Intern - Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C186" t="str">
-        <v>Mechanical / Aerospace / Electrical Engineering (Unison Industries subsidiary)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D186" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E186" t="str">
-        <v>Dayton, OH / Jacksonville, FL / Norwich, NY / St. George, UT (4 sites, one assignment)</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F186">
-        <v>750</v>
+        <v>1137</v>
       </c>
       <c r="G186" t="str">
-        <v>Not stated on posting</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H186" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Jacksonville/Unison-Engineering-Intern---Spring-2027_R5037093-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14424</v>
       </c>
       <c r="I186" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5037093, canApply true, posted 30+ days ago.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J186" t="str">
-        <v>Full-time intern version distinct from the already-tracked part-time 'Unison Engineering Part-time Co-op' (R5040016, St. George UT only). Works on ignition systems, sensors, generators, harnesses, engine starters at Unison Industries sites. Min 3.0 GPA, Aero/Mechanical/Electrical Engineering majors. Fall 2027 (R5037092) sibling at the same 4 sites was previously reviewed and excluded — wrong season.</v>
+        <v>REQ-14424. Manufacturing/Industrial/Mechanical/Systems Engineering, grad 2027-2029. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>Hermeus</v>
+        <v>Entegris</v>
       </c>
       <c r="B187" t="str">
-        <v>Build Reliability Engineering Intern - Spring/Summer 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C187" t="str">
-        <v>Manufacturing Engineering (structural fabrication &amp; assembly)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D187" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E187" t="str">
-        <v>Atlanta, GA</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F187">
-        <v>950</v>
+        <v>1137</v>
       </c>
       <c r="G187" t="str">
-        <v>$25–33/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H187" t="str">
-        <v>https://jobs.lever.co/hermeus/ee3a4109-b6e7-4ed5-8981-a483b3936e5a</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering--Co-Op_REQ-14447-1</v>
       </c>
       <c r="I187" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, page live, distinct dated Spring option confirmed in body text.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J187" t="str">
-        <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
+        <v>REQ-14447. Manufacturing/Industrial Engineering, grad Dec 2026 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>PI (Physik Instrumente) USA</v>
+        <v>Entegris</v>
       </c>
       <c r="B188" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>Mechanical Test Engineer Co-Op</v>
       </c>
       <c r="C188" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D188" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E188" t="str">
-        <v>Shrewsbury, MA</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F188">
-        <v>40</v>
+        <v>1137</v>
       </c>
       <c r="G188" t="str">
-        <v>$24-26/hour</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H188" t="str">
-        <v>https://www.pi-usa.us/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Mechanical-Test-Engineer-Co-Op_REQ-14477-1</v>
       </c>
       <c r="I188" t="str">
-        <v>Yes — fetched directly, HTTP 200, page title 'Mechanical Engineering Co-op - Winter/Spring 2027', full description read.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J188" t="str">
-        <v>New company for the tracker. Boston metro (Shrewsbury, MA — PI's US headquarters). High-precision positioning/motion systems and piezo technology manufacturer. Prepares detail/assembly drawings, CAD support, PLM data entry, R&amp;D build/test work. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship. SolidWorks and manufacturing-process experience preferred.</v>
+        <v>REQ-14477. Mechanical/Industrial Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>PI (Physik Instrumente) USA</v>
+        <v>Entegris</v>
       </c>
       <c r="B189" t="str">
-        <v>Manufacturing Engineering Internship</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C189" t="str">
         <v>Manufacturing Engineering</v>
       </c>
       <c r="D189" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E189" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F189">
+        <v>1771</v>
+      </c>
+      <c r="G189" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H189" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14508</v>
+      </c>
+      <c r="I189" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J189" t="str">
+        <v>REQ-14508. Mechanical/Industrial/Electrical Engineering, grad 2027 or 2028. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B190" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C190" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D190" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E190" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F190">
+        <v>1771</v>
+      </c>
+      <c r="G190" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H190" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14439</v>
+      </c>
+      <c r="I190" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J190" t="str">
+        <v>REQ-14439. Mechanical/Industrial/Manufacturing Engineering, Junior/Senior, grad 2027 or 2028. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B191" t="str">
+        <v>Manufacturing Engineer Co-Op</v>
+      </c>
+      <c r="C191" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D191" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E191" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F191">
+        <v>1771</v>
+      </c>
+      <c r="G191" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H191" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineer-Co-Op_REQ-14411</v>
+      </c>
+      <c r="I191" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J191" t="str">
+        <v>REQ-14411. Mechanical/Industrial/Manufacturing Engineering, grad 2027 or Spring 2028. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B192" t="str">
+        <v>Manufacturing Systems Engineer Co-Op</v>
+      </c>
+      <c r="C192" t="str">
+        <v>Manufacturing / Industrial Engineering</v>
+      </c>
+      <c r="D192" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E192" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F192">
+        <v>1771</v>
+      </c>
+      <c r="G192" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H192" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Systems-Engineer-Co-Op_REQ-14437</v>
+      </c>
+      <c r="I192" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J192" t="str">
+        <v>REQ-14437. Industrial/Chemical/Systems Engineering (or CS/IT) majors sought, target grad 2028; Master's students welcome. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B193" t="str">
+        <v>Process Engineering Co-Op</v>
+      </c>
+      <c r="C193" t="str">
+        <v>Process / Manufacturing Engineering</v>
+      </c>
+      <c r="D193" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E193" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F193">
+        <v>1771</v>
+      </c>
+      <c r="G193" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H193" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Process-Engineering-Co-Op_REQ-14485</v>
+      </c>
+      <c r="I193" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J193" t="str">
+        <v>REQ-14485. Mechanical/Industrial/Chemical Engineering, grad May 2027 or later. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B194" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C194" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D194" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E194" t="str">
+        <v>Bloomington, MN</v>
+      </c>
+      <c r="F194">
+        <v>1122</v>
+      </c>
+      <c r="G194" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H194" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bloomington-MN/Manufacturing-Engineering-Co-Op_REQ-14417</v>
+      </c>
+      <c r="I194" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J194" t="str">
+        <v>REQ-14417. Mechanical/Manufacturing/Industrial Engineering, Spring 2027 or 2028 grad. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B195" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E195" t="str">
+        <v>Hillsboro, OR</v>
+      </c>
+      <c r="F195">
+        <v>2548</v>
+      </c>
+      <c r="G195" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H195" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14480</v>
+      </c>
+      <c r="I195" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
+      </c>
+      <c r="J195" t="str">
+        <v>REQ-14480. Mechanical/Industrial/Chemical/Materials Science Engineering. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E196" t="str">
+        <v>Hillsboro, OR</v>
+      </c>
+      <c r="F196">
+        <v>2548</v>
+      </c>
+      <c r="G196" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H196" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14479</v>
+      </c>
+      <c r="I196" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
+      </c>
+      <c r="J196" t="str">
+        <v>REQ-14479. Sibling req to REQ-14480, same site/majors. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D197" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E197" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F197">
+        <v>2676</v>
+      </c>
+      <c r="G197" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H197" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14483</v>
+      </c>
+      <c r="I197" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J197" t="str">
+        <v>REQ-14483. Mechanical/Aerospace Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B198" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D198" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E198" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F198">
+        <v>2676</v>
+      </c>
+      <c r="G198" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H198" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14405</v>
+      </c>
+      <c r="I198" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J198" t="str">
+        <v>REQ-14405. Sibling req to REQ-14483, same site/majors. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B199" t="str">
+        <v>Controls Engineering Co-Op</v>
+      </c>
+      <c r="C199" t="str">
+        <v>Controls / Automation Engineering</v>
+      </c>
+      <c r="D199" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E199" t="str">
+        <v>Austin, TX</v>
+      </c>
+      <c r="F199">
+        <v>1694</v>
+      </c>
+      <c r="G199" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H199" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Austin-TX/Controls-Engineering-Co-Op_REQ-14460</v>
+      </c>
+      <c r="I199" t="str">
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J199" t="str">
+        <v>REQ-14460. Electrical/Chemical/Mechanical/Controls-Automation Engineering majors. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B200" t="str">
+        <v>Colibrium Additive US Manufacturing / Supply Chain Co-op - Spring 2027</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Manufacturing / Supply Chain Engineering (Additive Manufacturing)</v>
+      </c>
+      <c r="D200" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E200" t="str">
+        <v>West Chester, OH</v>
+      </c>
+      <c r="F200">
+        <v>700</v>
+      </c>
+      <c r="G200" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H200" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/West-Chester/Colibrium-Additive-US-Manufacturing---Supply-Chain-Co-op---Spring-2027_R5040302-2</v>
+      </c>
+      <c r="I200" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040302, canApply true, posted 2 days ago.</v>
+      </c>
+      <c r="J200" t="str">
+        <v>New req found via a fresh Workday search sweep; not previously tracked.</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B201" t="str">
+        <v>Flight Test Operation Engineering Intern - Victorville, CA - Spring 2027</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Flight Test / Systems Engineering</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E201" t="str">
+        <v>Victorville, CA</v>
+      </c>
+      <c r="F201">
+        <v>2500</v>
+      </c>
+      <c r="G201" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H201" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Victorville/Flight-Test-Operation-Engineering-Intern---Victorville--CA---Spring-2027_R5040433-1</v>
+      </c>
+      <c r="I201" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040433, canApply true, posted 3 days ago.</v>
+      </c>
+      <c r="J201" t="str">
+        <v>New req; flight-test/flight-systems discipline fit.</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B202" t="str">
+        <v>Systems Engineering Co-op - Mechanical/Aerospace Engineering (Electric Power) - US - Spring 2027</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Systems Engineering (Mechanical/Aerospace)</v>
+      </c>
+      <c r="D202" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E202" t="str">
+        <v>Dayton, OH</v>
+      </c>
+      <c r="F202">
+        <v>750</v>
+      </c>
+      <c r="G202" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H202" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Dayton/Systems-Engineering-Co-op---Mechanical-Aerospace-Engineering--Electric-Power----US---Spring-2027_R5030103-1</v>
+      </c>
+      <c r="I202" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5030103, canApply true, posted 30+ days ago.</v>
+      </c>
+      <c r="J202" t="str">
+        <v>New req found via a fresh Workday search sweep. A parallel Electrical Engineering/Computer Engineering version (R5030099) at the same site was reviewed and excluded — EE/CS discipline.</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B203" t="str">
+        <v>Unison Engineering Part-time Co-op - US - Spring 2027</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Mechanical / Manufacturing Engineering (Unison Industries subsidiary)</v>
+      </c>
+      <c r="D203" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E203" t="str">
+        <v>Saint George, UT</v>
+      </c>
+      <c r="F203">
+        <v>2300</v>
+      </c>
+      <c r="G203" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H203" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Saint-George-UT-US-1/Unison-Engineering-Part-time-Co-op---US---Spring-2027_R5040016</v>
+      </c>
+      <c r="I203" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040016, canApply true, posted 9 days ago.</v>
+      </c>
+      <c r="J203" t="str">
+        <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>Symbotic</v>
+      </c>
+      <c r="B204" t="str">
+        <v>Co-op - Hardware Engineer</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Mechanical / Hardware Engineering (robotics)</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Spring 2027 (January–May)</v>
+      </c>
+      <c r="E204" t="str">
+        <v>Wilmington, MA</v>
+      </c>
+      <c r="F204">
+        <v>17</v>
+      </c>
+      <c r="G204" t="str">
+        <v>$29.00–$40.00/hr</v>
+      </c>
+      <c r="H204" t="str">
+        <v>https://symbotic.wd504.myworkdayjobs.com/Symbotic/job/USA-Wilmington-MA---ITC/Hardware-Engineer_R7976</v>
+      </c>
+      <c r="I204" t="str">
+        <v>Yes — fetched directly via Symbotic's own Workday CXS API, req R7976, canApply true, posted 3 days ago.</v>
+      </c>
+      <c r="J204" t="str">
+        <v>Boston metro (Wilmington, MA — ITC site). Requires enrolled Bachelor's student in Systems/Robotics/Mechanical/Electrical/CS engineering. Hands-on electro-mechanical work: GD&amp;T, SolidWorks, manufacturing processes (machining, casting, sheet metal). Offers transportation/housing benefits for relocating students. A sibling req 'Co-op - Robot Perception' (R8113, same site/timeframe) was reviewed and excluded — Computer Vision/ML software discipline, requires Master's/PhD.</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B205" t="str">
+        <v>Unison Engineering Intern - Spring 2027</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Mechanical / Aerospace / Electrical Engineering (Unison Industries subsidiary)</v>
+      </c>
+      <c r="D205" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E205" t="str">
+        <v>Dayton, OH / Jacksonville, FL / Norwich, NY / St. George, UT (4 sites, one assignment)</v>
+      </c>
+      <c r="F205">
+        <v>750</v>
+      </c>
+      <c r="G205" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H205" t="str">
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Jacksonville/Unison-Engineering-Intern---Spring-2027_R5037093-1</v>
+      </c>
+      <c r="I205" t="str">
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5037093, canApply true, posted 30+ days ago.</v>
+      </c>
+      <c r="J205" t="str">
+        <v>Full-time intern version distinct from the already-tracked part-time 'Unison Engineering Part-time Co-op' (R5040016, St. George UT only). Works on ignition systems, sensors, generators, harnesses, engine starters at Unison Industries sites. Min 3.0 GPA, Aero/Mechanical/Electrical Engineering majors. Fall 2027 (R5037092) sibling at the same 4 sites was previously reviewed and excluded — wrong season.</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>Hermeus</v>
+      </c>
+      <c r="B206" t="str">
+        <v>Build Reliability Engineering Intern - Spring/Summer 2027</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Manufacturing Engineering (structural fabrication &amp; assembly)</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+      </c>
+      <c r="E206" t="str">
+        <v>Atlanta, GA</v>
+      </c>
+      <c r="F206">
+        <v>950</v>
+      </c>
+      <c r="G206" t="str">
+        <v>$25–33/hr</v>
+      </c>
+      <c r="H206" t="str">
+        <v>https://jobs.lever.co/hermeus/ee3a4109-b6e7-4ed5-8981-a483b3936e5a</v>
+      </c>
+      <c r="I206" t="str">
+        <v>Yes — fetched directly via Hermeus's own Lever API, page live, distinct dated Spring option confirmed in body text.</v>
+      </c>
+      <c r="J206" t="str">
+        <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>PI (Physik Instrumente) USA</v>
+      </c>
+      <c r="B207" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D207" t="str">
         <v>Winter/Spring 2027</v>
       </c>
-      <c r="E189" t="str">
+      <c r="E207" t="str">
         <v>Shrewsbury, MA</v>
       </c>
-      <c r="F189">
+      <c r="F207">
         <v>40</v>
       </c>
-      <c r="G189" t="str">
+      <c r="G207" t="str">
         <v>$24-26/hour</v>
       </c>
-      <c r="H189" t="str">
+      <c r="H207" t="str">
+        <v>https://www.pi-usa.us/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+      </c>
+      <c r="I207" t="str">
+        <v>Yes — fetched directly, HTTP 200, page title 'Mechanical Engineering Co-op - Winter/Spring 2027', full description read.</v>
+      </c>
+      <c r="J207" t="str">
+        <v>New company for the tracker. Boston metro (Shrewsbury, MA — PI's US headquarters). High-precision positioning/motion systems and piezo technology manufacturer. Prepares detail/assembly drawings, CAD support, PLM data entry, R&amp;D build/test work. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship. SolidWorks and manufacturing-process experience preferred.</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>PI (Physik Instrumente) USA</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Manufacturing Engineering Internship</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Shrewsbury, MA</v>
+      </c>
+      <c r="F208">
+        <v>40</v>
+      </c>
+      <c r="G208" t="str">
+        <v>$24-26/hour</v>
+      </c>
+      <c r="H208" t="str">
         <v>https://www.pi-usa.us/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
       </c>
-      <c r="I189" t="str">
+      <c r="I208" t="str">
         <v>Yes — fetched directly, HTTP 200, page title 'Manufacturing Engineering Internship - Winter/Spring 2027', full description read.</v>
       </c>
-      <c r="J189" t="str">
+      <c r="J208" t="str">
         <v>Sibling req to the Mechanical Engineering Co-op above, same site/pay/season. Fixture design for assembly/metrology/manufacturing, SolidWorks modeling, hands-on machining (mills, lathes, saws, 3D printers), process optimization, ECR/ECO documentation. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship.</v>
       </c>
     </row>
@@ -8482,14 +9090,14 @@
     <hyperlink ref="M172" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M189"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M208"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C385"/>
+  <dimension ref="A1:C390"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -12731,9 +13339,64 @@
         <v>2026-09-25 ~19:00 UTC: 127776BR now also confirmed 'no longer accepting applications' (closed), joining its already-excluded Cedar Rapids siblings 125975BR/126541BR. No Spring-2027-dated mechanical/systems coop found at Nashua NH, Endicott NY, or Manassas VA — only postings found at those sites are Summer 2027 interns (Mechanical Engineering Intern III, Nashua NH, 129311BR onsite / 127637BR hybrid) or already-closed reqs (Industrial Engineering Co-Op Fall Semester 2026, Nashua NH, 124709BR — now HTTP 410 Gone). The Cedar Rapids Spring-coop naming pattern does not appear to extend to these other sites currently. Dropping active watch on this lead unless a new dated req surfaces.</v>
       </c>
     </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B386" t="str">
+        <v>'Manufacturing Production Documentation Co-Op' (REQ-14408, Chaska MN); 'Manufacturing Systems and Planning Co-Op' (REQ-14410, Colorado Springs/Rockrimmon CO); 'Electrical Manufacturing Engineering Co-Op' (REQ-14486, Bloomington MN)</v>
+      </c>
+      <c r="C386" t="str">
+        <v>2026-09-26 ~01:00 UTC: this session ran Entegris's own Workday CXS API/site to page through all 606 currently-open Entegris reqs (bypassing the 400-error-on-non-empty-searchText block noted in prior runs by paging with an empty searchText and client-side title filtering) and found 103 live Co-Op postings company-wide, most far beyond the previously MA-only-tracked slate. Of the new ones, these 3 fail the discipline bar on direct read of their own text: REQ-14408 is manufacturing documentation/technical-writing focused (SOPs, work instructions), not engineering design/process work; REQ-14410 explicitly seeks Information Systems/Computer Science/Supply Chain/Operations Management majors, not an engineering discipline; REQ-14486 explicitly requires an Electrical Engineering major only (no ME/industrial/manufacturing option), same EE-mismatch treatment as the earlier-excluded Rendezvous Robotics Avionics Intern. Not added. (18 other newly-found Entegris Co-Ops from this same sweep — spanning Aurora IL, Chaska MN, Colorado Springs CO, Bloomington MN, Hillsboro OR, San Luis Obispo CA, and Austin TX, all independently confirmed 'Spring 2027 season' on direct fetch of each posting's own page — were added to `rows`.)</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>Moog Inc.</v>
+      </c>
+      <c r="B387" t="str">
+        <v>Intern, Test Equipment Sustainment (R-26-19821, Torrance CA)</v>
+      </c>
+      <c r="C387" t="str">
+        <v>2026-09-26 ~01:00 UTC: confirmed live (HTTP 200) but Moog's Workday page is client-side-rendered for this tenant/site and the season text could not be independently extracted; per a research agent's read of the same posting it states 'spring/summer block intern' with no year given — same unresolved-year pattern as the already-excluded R-26-19536 and R-26-19391. Not added; worth a fresh look alongside those two if Moog ever adds a year.</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>Draper Laboratory (Cambridge, MA)</v>
+      </c>
+      <c r="B388" t="str">
+        <v>'...Intern (Summer 2027)' (JR002943)</v>
+      </c>
+      <c r="C388" t="str">
+        <v>2026-09-26 ~01:00 UTC: new req found this run, explicitly titled Summer 2027 — wrong season, excluded. (JR002767 'Mechanical Engineering &amp; System Packaging Intern', previously excluded on an aggregator's word that it was Summer, was independently re-confirmed this run via direct fetch of Draper's own posting text: 'As a summer intern in the Mechanical Engineering Division...' — upgrading that exclusion from aggregator-sourced to directly verified.)</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>L3Harris</v>
+      </c>
+      <c r="B389" t="str">
+        <v>'Intern, Mechanical Engineer' (job 42733) and 'Mechanical Design Engineering Intern' (job 38354), Huntsville AL; 'Manufacturing Engineering Intern' (job 41201), Londonderry NH; 'Mechanical Engineering Intern (SLC)' (job 41704), Salt Lake City UT; 'Intern, Mechanical Engineer 1' and 'Mechanical Design Engineering Intern', Canoga Park CA</v>
+      </c>
+      <c r="C389" t="str">
+        <v>2026-09-26 ~01:00 UTC: all confirmed live and freshly posted (datePosted 2026-09-10 to 2026-09-22) via direct fetch of careers.l3harris.com (server-rendered, unlike most other blocked ATSes) plus each page's JSON-LD JobPosting schema — but every one of these postings' full description text contains no Winter/Spring/Summer/Fall or term-date wording anywhere, consistent with L3Harris's internship template generally (this now appears structural to how L3Harris writes these postings, not a fetch limitation). Fails the season-stated verification bar; not added. The previously-flagged Rochester, NY 'Mechanical Engineering Intern' req now returns HTTP 404 — closed.</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>Textron Systems / Bell Textron</v>
+      </c>
+      <c r="B390" t="str">
+        <v>10 distinct '2027' mechanical engineer intern/co-op req slugs found via careers.textron.com's XML sitemap: Hunt Valley MD (4 reqs — Uncrewed Land/Air co-op and intern, Electronic Systems intern, Sea Systems intern), Augusta GA (1), Cartersville GA (2, incl. Ground Support Equipment), Williamsport PA (1, Lycoming), Wichita KS (5 — Defense &amp; Special Missions, Flight Controls/Doors, Hydraulics/Gear/Brakes, AES Mechanical Installations, ECS/IPS)</v>
+      </c>
+      <c r="C390" t="str">
+        <v>2026-09-26 ~01:00 UTC: sitemap confirms all 10 URLs are currently indexed/live, but careers.textron.com remains a client-side-rendered Nuxt.js SPA that neither curl nor WebFetch can read past the app shell — titles say only '2027' with no Spring/Summer qualifier, so season remains completely unconfirmable from source, consistent with this tracker's long-running Textron block. Not added; flagging the specific slugs so a future run with browser-rendering capability can jump straight to them.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C385"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C390"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 1 checked-excluded (2026-09-26 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011RKgHN169N5KwoUqsKnKip
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -9097,7 +9097,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C390"/>
+  <dimension ref="A1:C391"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -13394,9 +13394,20 @@
         <v>2026-09-26 ~01:00 UTC: sitemap confirms all 10 URLs are currently indexed/live, but careers.textron.com remains a client-side-rendered Nuxt.js SPA that neither curl nor WebFetch can read past the app shell — titles say only '2027' with no Spring/Summer qualifier, so season remains completely unconfirmable from source, consistent with this tracker's long-running Textron block. Not added; flagging the specific slugs so a future run with browser-rendering capability can jump straight to them.</v>
       </c>
     </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>SharkNinja (Needham, MA)</v>
+      </c>
+      <c r="B391" t="str">
+        <v>'Mechanical Engineering Intern Opportunities', Greenhouse job 4713812006 (sibling to the already-excluded 'Mechanical Engineering Co-op Opportunities', job 4713783006)</v>
+      </c>
+      <c r="C391" t="str">
+        <v>2026-09-26 ~07:00 UTC re-check: both reqs confirmed live via direct fetch, freshly posted/updated 2026-09-17, but neither posting states a season/term anywhere in the text (no Spring/Winter/Summer/Fall) — same generic rolling req pattern as its already-excluded sibling. Fails the season-stated verification bar. No dated Winter 2026/Spring 2027 sibling found on careers.sharkninja.com's sitemap either. Not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C390"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C391"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new posting, 1 checked-excluded (2026-09-26 13:00 UTC)
Added Buro Happold Mechanical Co-op (Boston, Spring 2027, Partial verification).
Fixed a data-quality issue found while cross-checking: PI (Physik Instrumente)'s
Shrewsbury MA co-ops were tracked twice under two mirror domains
(physikinstrumente.com and pi-usa.us) — deduped to one pair, preserving the
existing prepared application documents.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QSeeSqf4wPGsthPtt9DyLp
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M208"/>
+  <dimension ref="A1:M207"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -3887,34 +3887,34 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>PI (Physik Instrumente)</v>
+        <v>Astranis Space Technologies</v>
       </c>
       <c r="B86" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>CAD Engineer Intern (Spring 2027)</v>
       </c>
       <c r="C86" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical Design / CAD Engineering</v>
       </c>
       <c r="D86" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E86" t="str">
-        <v>Shrewsbury, MA</v>
+        <v>San Francisco, CA</v>
       </c>
       <c r="F86">
-        <v>40</v>
+        <v>2700</v>
       </c>
       <c r="G86" t="str">
-        <v>$24–26/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H86" t="str">
-        <v>https://www.physikinstrumente.com/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+        <v>https://job-boards.greenhouse.io/astranis/jobs/4704740006</v>
       </c>
       <c r="I86" t="str">
-        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live, 'Spring 2027' stated on posting.</v>
       </c>
       <c r="J86" t="str">
-        <v>Boston metro (Shrewsbury). Fresh cycle superseding the already-past Jan-June 2026 cohort found at this same company in prior runs. Requires legal US work authorization without sponsorship; SolidWorks preferred.</v>
+        <v>Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 4704602006) at the same company. Satellite manufacturer — worth double-checking ITAR/citizenship requirements before applying, not explicit in the excerpt reviewed. Distinct from Astranis's separate 'Winter 2027' reqs, which remain excluded (see `checked`) for season mismatch.</v>
       </c>
       <c r="K86" t="str">
         <v>Open resume</v>
@@ -3928,34 +3928,34 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>PI (Physik Instrumente)</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B87" t="str">
-        <v>Manufacturing Engineering Internship</v>
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C87" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D87" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E87" t="str">
-        <v>Shrewsbury, MA</v>
+        <v>Rockford, IL</v>
       </c>
       <c r="F87">
-        <v>40</v>
+        <v>900</v>
       </c>
       <c r="G87" t="str">
-        <v>$24–26/hr</v>
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
       </c>
       <c r="H87" t="str">
-        <v>https://www.physikinstrumente.com/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IL-ROCKFORD-P6--4747-Harrison-Ave--4747-HARRISON-AVE-P6/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869227</v>
       </c>
       <c r="I87" t="str">
-        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
+        <v>Yes — fetched directly via RTX's own Workday CXS API (browser UA + Referer), full description confirmed, posted 2026-09-22.</v>
       </c>
       <c r="J87" t="str">
-        <v>Boston metro (Shrewsbury). Same batch/cycle as the Mechanical Engineering Co-op above.</v>
+        <v>Distinct req/site from the already-tracked Jamestown ND and Cedar Rapids IA Collins Aerospace co-ops — not a duplicate.</v>
       </c>
       <c r="K87" t="str">
         <v>Open resume</v>
@@ -3969,34 +3969,34 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Astranis Space Technologies</v>
+        <v>L3Harris</v>
       </c>
       <c r="B88" t="str">
-        <v>CAD Engineer Intern (Spring 2027)</v>
+        <v>Mechanical Engineer Intern - Spring 2027</v>
       </c>
       <c r="C88" t="str">
-        <v>Mechanical Design / CAD Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D88" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Jan–Jul 2027)</v>
       </c>
       <c r="E88" t="str">
-        <v>San Francisco, CA</v>
+        <v>Greenville, TX</v>
       </c>
       <c r="F88">
-        <v>2700</v>
+        <v>1500</v>
       </c>
       <c r="G88" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H88" t="str">
-        <v>https://job-boards.greenhouse.io/astranis/jobs/4704740006</v>
+        <v>https://careers.l3harris.com/en/job/greenville/mechanical-engineer-intern-spring-2027/4832/99372978208</v>
       </c>
       <c r="I88" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live, 'Spring 2027' stated on posting.</v>
+        <v>Yes — fetched directly, page live, 'Apply Now' present, 'Spring 2027' stated on posting (no 'summer' wording found, unlike a differently-worded/now-dead L3Harris Greenville req excluded in a prior run).</v>
       </c>
       <c r="J88" t="str">
-        <v>Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 4704602006) at the same company. Satellite manufacturer — worth double-checking ITAR/citizenship requirements before applying, not explicit in the excerpt reviewed. Distinct from Astranis's separate 'Winter 2027' reqs, which remain excluded (see `checked`) for season mismatch.</v>
+        <v>Degree requirement: Mechanical/Aerospace/Engineering Mechanics/Materials Science. US citizenship required for clearance eligibility. Job ID 41322.</v>
       </c>
       <c r="K88" t="str">
         <v>Open resume</v>
@@ -4010,34 +4010,34 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B89" t="str">
-        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Winter 2027 Propulsion Engineer Co-op</v>
       </c>
       <c r="C89" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Propulsion Engineering</v>
       </c>
       <c r="D89" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Winter 2027 (effectively Jan–Aug 2027, same calendar window as other employers' 'Spring 2027')</v>
       </c>
       <c r="E89" t="str">
-        <v>Rockford, IL</v>
+        <v>Costa Mesa, CA</v>
       </c>
       <c r="F89">
-        <v>900</v>
+        <v>2600</v>
       </c>
       <c r="G89" t="str">
-        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H89" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IL-ROCKFORD-P6--4747-Harrison-Ave--4747-HARRISON-AVE-P6/Mechanical-Engineering-Co-op--Winter-Spring-2027-_01869227</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236587007</v>
       </c>
       <c r="I89" t="str">
-        <v>Yes — fetched directly via RTX's own Workday CXS API (browser UA + Referer), full description confirmed, posted 2026-09-22.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
       </c>
       <c r="J89" t="str">
-        <v>Distinct req/site from the already-tracked Jamestown ND and Cedar Rapids IA Collins Aerospace co-ops — not a duplicate.</v>
+        <v>US citizenship required, no clearance required. New site beyond the already-tracked Quincy, MA / Lexington, MA Anduril Winter 2027 co-ops.</v>
       </c>
       <c r="K89" t="str">
         <v>Open resume</v>
@@ -4051,34 +4051,34 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>L3Harris</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B90" t="str">
-        <v>Mechanical Engineer Intern - Spring 2027</v>
+        <v>Winter 2027 Warhead Engineer Co-op</v>
       </c>
       <c r="C90" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical Engineering (ordnance/warhead design)</v>
       </c>
       <c r="D90" t="str">
-        <v>Spring 2027 (Jan–Jul 2027)</v>
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
       </c>
       <c r="E90" t="str">
-        <v>Greenville, TX</v>
+        <v>Costa Mesa, CA</v>
       </c>
       <c r="F90">
-        <v>1500</v>
+        <v>2600</v>
       </c>
       <c r="G90" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H90" t="str">
-        <v>https://careers.l3harris.com/en/job/greenville/mechanical-engineer-intern-spring-2027/4832/99372978208</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236585007</v>
       </c>
       <c r="I90" t="str">
-        <v>Yes — fetched directly, page live, 'Apply Now' present, 'Spring 2027' stated on posting (no 'summer' wording found, unlike a differently-worded/now-dead L3Harris Greenville req excluded in a prior run).</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
       </c>
       <c r="J90" t="str">
-        <v>Degree requirement: Mechanical/Aerospace/Engineering Mechanics/Materials Science. US citizenship required for clearance eligibility. Job ID 41322.</v>
+        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Test &amp; Evaluation Engineer Co-ops above.</v>
       </c>
       <c r="K90" t="str">
         <v>Open resume</v>
@@ -4095,13 +4095,13 @@
         <v>Anduril Industries</v>
       </c>
       <c r="B91" t="str">
-        <v>Winter 2027 Propulsion Engineer Co-op</v>
+        <v>Winter 2027 Test &amp; Evaluation Engineer Co-op</v>
       </c>
       <c r="C91" t="str">
-        <v>Mechanical / Propulsion Engineering</v>
+        <v>Systems / Test Engineering</v>
       </c>
       <c r="D91" t="str">
-        <v>Winter 2027 (effectively Jan–Aug 2027, same calendar window as other employers' 'Spring 2027')</v>
+        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
       </c>
       <c r="E91" t="str">
         <v>Costa Mesa, CA</v>
@@ -4113,13 +4113,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H91" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236587007</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236583007</v>
       </c>
       <c r="I91" t="str">
         <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
       </c>
       <c r="J91" t="str">
-        <v>US citizenship required, no clearance required. New site beyond the already-tracked Quincy, MA / Lexington, MA Anduril Winter 2027 co-ops.</v>
+        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Warhead Engineer Co-ops above.</v>
       </c>
       <c r="K91" t="str">
         <v>Open resume</v>
@@ -4133,34 +4133,34 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Anduril Industries</v>
+        <v>Zipline</v>
       </c>
       <c r="B92" t="str">
-        <v>Winter 2027 Warhead Engineer Co-op</v>
+        <v>Aerodynamics Intern (Spring 2027)</v>
       </c>
       <c r="C92" t="str">
-        <v>Mechanical Engineering (ordnance/warhead design)</v>
+        <v>Aerospace / Aerodynamics Engineering</v>
       </c>
       <c r="D92" t="str">
-        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E92" t="str">
-        <v>Costa Mesa, CA</v>
+        <v>South San Francisco, CA</v>
       </c>
       <c r="F92">
-        <v>2600</v>
+        <v>2700</v>
       </c>
       <c r="G92" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H92" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236585007</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904002003</v>
       </c>
       <c r="I92" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J92" t="str">
-        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Test &amp; Evaluation Engineer Co-ops above.</v>
+        <v>Autonomous drone delivery company. Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 7865253003) at the same company.</v>
       </c>
       <c r="K92" t="str">
         <v>Open resume</v>
@@ -4174,34 +4174,34 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Anduril Industries</v>
+        <v>Zipline</v>
       </c>
       <c r="B93" t="str">
-        <v>Winter 2027 Test &amp; Evaluation Engineer Co-op</v>
+        <v>Civil and Structural Engineer Intern (Spring 2027)</v>
       </c>
       <c r="C93" t="str">
-        <v>Systems / Test Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D93" t="str">
-        <v>Winter 2027 (effectively Jan–Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E93" t="str">
-        <v>Costa Mesa, CA</v>
+        <v>South San Francisco, CA</v>
       </c>
       <c r="F93">
-        <v>2600</v>
+        <v>2700</v>
       </c>
       <c r="G93" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H93" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236583007</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904457003</v>
       </c>
       <c r="I93" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live, posted 2026-09-21.</v>
+        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J93" t="str">
-        <v>US citizenship required, no clearance required. Same batch/site as the Propulsion and Warhead Engineer Co-ops above.</v>
+        <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
       <c r="K93" t="str">
         <v>Open resume</v>
@@ -4218,10 +4218,10 @@
         <v>Zipline</v>
       </c>
       <c r="B94" t="str">
-        <v>Aerodynamics Intern (Spring 2027)</v>
+        <v>Controls Engineer Intern (Spring 2027)</v>
       </c>
       <c r="C94" t="str">
-        <v>Aerospace / Aerodynamics Engineering</v>
+        <v>Controls Engineering</v>
       </c>
       <c r="D94" t="str">
         <v>Spring 2027</v>
@@ -4236,13 +4236,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H94" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904002003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7903823003</v>
       </c>
       <c r="I94" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J94" t="str">
-        <v>Autonomous drone delivery company. Sibling req to the already-tracked Mechanical Engineer Intern (Spring 2027, 7865253003) at the same company.</v>
+        <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
       <c r="K94" t="str">
         <v>Open resume</v>
@@ -4259,10 +4259,10 @@
         <v>Zipline</v>
       </c>
       <c r="B95" t="str">
-        <v>Civil and Structural Engineer Intern (Spring 2027)</v>
+        <v>Flight Test Engineer Intern (Spring 2027)</v>
       </c>
       <c r="C95" t="str">
-        <v>Structural Engineering</v>
+        <v>Flight Systems / Test Engineering</v>
       </c>
       <c r="D95" t="str">
         <v>Spring 2027</v>
@@ -4277,7 +4277,7 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H95" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7904457003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7999929003</v>
       </c>
       <c r="I95" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
@@ -4300,10 +4300,10 @@
         <v>Zipline</v>
       </c>
       <c r="B96" t="str">
-        <v>Controls Engineer Intern (Spring 2027)</v>
+        <v>Hardware Test Intern (Spring 2027)</v>
       </c>
       <c r="C96" t="str">
-        <v>Controls Engineering</v>
+        <v>Mechanical / Hardware Test Engineering</v>
       </c>
       <c r="D96" t="str">
         <v>Spring 2027</v>
@@ -4318,7 +4318,7 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H96" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7903823003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7894349003</v>
       </c>
       <c r="I96" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
@@ -4341,31 +4341,31 @@
         <v>Zipline</v>
       </c>
       <c r="B97" t="str">
-        <v>Flight Test Engineer Intern (Spring 2027)</v>
+        <v>Maintenance Tool Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C97" t="str">
-        <v>Flight Systems / Test Engineering</v>
+        <v>Mechanical / Tooling Engineering</v>
       </c>
       <c r="D97" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E97" t="str">
-        <v>South San Francisco, CA</v>
+        <v>Esparto, CA</v>
       </c>
       <c r="F97">
-        <v>2700</v>
+        <v>2800</v>
       </c>
       <c r="G97" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H97" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7999929003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7909945003</v>
       </c>
       <c r="I97" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J97" t="str">
-        <v>Same batch as the other new Zipline reqs added this run.</v>
+        <v>Borderline discipline fit (maintenance tooling) — included per Hamza's own judgment call, similar treatment to other borderline robotics/manufacturing-adjacent reqs in this tracker.</v>
       </c>
       <c r="K97" t="str">
         <v>Open resume</v>
@@ -4382,10 +4382,10 @@
         <v>Zipline</v>
       </c>
       <c r="B98" t="str">
-        <v>Hardware Test Intern (Spring 2027)</v>
+        <v>Quality &amp; Manufacturing Intern (Spring 2027)</v>
       </c>
       <c r="C98" t="str">
-        <v>Mechanical / Hardware Test Engineering</v>
+        <v>Manufacturing / Quality Engineering</v>
       </c>
       <c r="D98" t="str">
         <v>Spring 2027</v>
@@ -4400,7 +4400,7 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H98" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7894349003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7824311003</v>
       </c>
       <c r="I98" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
@@ -4423,31 +4423,31 @@
         <v>Zipline</v>
       </c>
       <c r="B99" t="str">
-        <v>Maintenance Tool Engineering Intern (Spring 2027)</v>
+        <v>Supplier Industrialization Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C99" t="str">
-        <v>Mechanical / Tooling Engineering</v>
+        <v>Manufacturing / Industrial Engineering</v>
       </c>
       <c r="D99" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E99" t="str">
-        <v>Esparto, CA</v>
+        <v>South San Francisco, CA</v>
       </c>
       <c r="F99">
-        <v>2800</v>
+        <v>2700</v>
       </c>
       <c r="G99" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H99" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7909945003</v>
+        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7891019003</v>
       </c>
       <c r="I99" t="str">
         <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
       </c>
       <c r="J99" t="str">
-        <v>Borderline discipline fit (maintenance tooling) — included per Hamza's own judgment call, similar treatment to other borderline robotics/manufacturing-adjacent reqs in this tracker.</v>
+        <v>Same batch as the other new Zipline reqs added this run.</v>
       </c>
       <c r="K99" t="str">
         <v>Open resume</v>
@@ -4461,34 +4461,34 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Zipline</v>
+        <v>Varda Space Industries</v>
       </c>
       <c r="B100" t="str">
-        <v>Quality &amp; Manufacturing Intern (Spring 2027)</v>
+        <v>Mechanisms &amp; Payload Internship (Spring 2027)</v>
       </c>
       <c r="C100" t="str">
-        <v>Manufacturing / Quality Engineering</v>
+        <v>Mechanical / Mechatronics Engineering</v>
       </c>
       <c r="D100" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Jan–May)</v>
       </c>
       <c r="E100" t="str">
-        <v>South San Francisco, CA</v>
+        <v>El Segundo, CA</v>
       </c>
       <c r="F100">
-        <v>2700</v>
+        <v>2600</v>
       </c>
       <c r="G100" t="str">
-        <v>Not stated on posting</v>
+        <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H100" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7824311003</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824821003</v>
       </c>
       <c r="I100" t="str">
-        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J100" t="str">
-        <v>Same batch as the other new Zipline reqs added this run.</v>
+        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. Designs/builds/tests flight electromechanical hardware (mechanisms, payloads). US work authorization + export-control (ITAR) screening required per posting.</v>
       </c>
       <c r="K100" t="str">
         <v>Open resume</v>
@@ -4502,34 +4502,34 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Zipline</v>
+        <v>Varda Space Industries</v>
       </c>
       <c r="B101" t="str">
-        <v>Supplier Industrialization Engineering Intern (Spring 2027)</v>
+        <v>Structures Engineering Internship (Spring 2027)</v>
       </c>
       <c r="C101" t="str">
-        <v>Manufacturing / Industrial Engineering</v>
+        <v>Mechanical / Aerospace / Structures Engineering</v>
       </c>
       <c r="D101" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Jan–May)</v>
       </c>
       <c r="E101" t="str">
-        <v>South San Francisco, CA</v>
+        <v>El Segundo, CA</v>
       </c>
       <c r="F101">
-        <v>2700</v>
+        <v>2600</v>
       </c>
       <c r="G101" t="str">
-        <v>Not stated on posting</v>
+        <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H101" t="str">
-        <v>https://job-boards.greenhouse.io/flyzipline/jobs/7891019003</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824817003</v>
       </c>
       <c r="I101" t="str">
-        <v>Yes — fetched directly via Zipline's own Greenhouse API, HTTP 200, no closed-application notice, updated 2026-09-17.</v>
+        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J101" t="str">
-        <v>Same batch as the other new Zipline reqs added this run.</v>
+        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. CAD/FEA design and build/test of spacecraft structural hardware. US work authorization + export-control (ITAR) screening required per posting.</v>
       </c>
       <c r="K101" t="str">
         <v>Open resume</v>
@@ -4546,13 +4546,13 @@
         <v>Varda Space Industries</v>
       </c>
       <c r="B102" t="str">
-        <v>Mechanisms &amp; Payload Internship (Spring 2027)</v>
+        <v>Guidance, Navigation &amp; Controls (GNC) Internship (Spring 2027)</v>
       </c>
       <c r="C102" t="str">
-        <v>Mechanical / Mechatronics Engineering</v>
+        <v>Controls / Aerospace Engineering</v>
       </c>
       <c r="D102" t="str">
-        <v>Spring 2027 (Jan–May)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E102" t="str">
         <v>El Segundo, CA</v>
@@ -4564,13 +4564,13 @@
         <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H102" t="str">
-        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824821003</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824781003</v>
       </c>
       <c r="I102" t="str">
         <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J102" t="str">
-        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. Designs/builds/tests flight electromechanical hardware (mechanisms, payloads). US work authorization + export-control (ITAR) screening required per posting.</v>
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. GNC for flight vehicles. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
       <c r="K102" t="str">
         <v>Open resume</v>
@@ -4587,13 +4587,13 @@
         <v>Varda Space Industries</v>
       </c>
       <c r="B103" t="str">
-        <v>Structures Engineering Internship (Spring 2027)</v>
+        <v>Propulsion Engineering Internship (Spring 2027)</v>
       </c>
       <c r="C103" t="str">
-        <v>Mechanical / Aerospace / Structures Engineering</v>
+        <v>Mechanical / Propulsion Engineering</v>
       </c>
       <c r="D103" t="str">
-        <v>Spring 2027 (Jan–May)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E103" t="str">
         <v>El Segundo, CA</v>
@@ -4605,13 +4605,13 @@
         <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H103" t="str">
-        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824817003</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824765003</v>
       </c>
       <c r="I103" t="str">
         <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J103" t="str">
-        <v>Sibling req to the already-tracked Manufacturing Engineering Internship at the same company/season. CAD/FEA design and build/test of spacecraft structural hardware. US work authorization + export-control (ITAR) screening required per posting.</v>
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
       <c r="K103" t="str">
         <v>Open resume</v>
@@ -4628,10 +4628,10 @@
         <v>Varda Space Industries</v>
       </c>
       <c r="B104" t="str">
-        <v>Guidance, Navigation &amp; Controls (GNC) Internship (Spring 2027)</v>
+        <v>Vehicle Integration &amp; Test Internship (Spring 2027)</v>
       </c>
       <c r="C104" t="str">
-        <v>Controls / Aerospace Engineering</v>
+        <v>Mechanical / Aerospace Systems Engineering</v>
       </c>
       <c r="D104" t="str">
         <v>Spring 2027</v>
@@ -4646,13 +4646,13 @@
         <v>$33.00/hr + housing stipend for relocating interns</v>
       </c>
       <c r="H104" t="str">
-        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824781003</v>
+        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824772003</v>
       </c>
       <c r="I104" t="str">
         <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
       </c>
       <c r="J104" t="str">
-        <v>Sibling req to the already-tracked Varda internships at the same company/season. GNC for flight vehicles. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
+        <v>Sibling req to the already-tracked Varda internships at the same company/season. Vehicle integration and test of flight hardware. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
       </c>
       <c r="K104" t="str">
         <v>Open resume</v>
@@ -4666,34 +4666,34 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Varda Space Industries</v>
+        <v>Marathon Petroleum</v>
       </c>
       <c r="B105" t="str">
-        <v>Propulsion Engineering Internship (Spring 2027)</v>
+        <v>Intern/Co-op - Refining Mechanical Engineer (Spring 2027)</v>
       </c>
       <c r="C105" t="str">
-        <v>Mechanical / Propulsion Engineering</v>
+        <v>Mechanical Engineering (Industrial / Refining)</v>
       </c>
       <c r="D105" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E105" t="str">
-        <v>El Segundo, CA</v>
+        <v>Findlay, OH</v>
       </c>
       <c r="F105">
-        <v>2600</v>
+        <v>700</v>
       </c>
       <c r="G105" t="str">
-        <v>$33.00/hr + housing stipend for relocating interns</v>
+        <v>$32.92–$41.67/hr</v>
       </c>
       <c r="H105" t="str">
-        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824765003</v>
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Intern-Co-op---Refining-Mechanical-Engineer--Spring-2027-_00020137</v>
       </c>
       <c r="I105" t="str">
-        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API, full job description returned, req 00020137.</v>
       </c>
       <c r="J105" t="str">
-        <v>Sibling req to the already-tracked Varda internships at the same company/season. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
+        <v>New company, not previously tracked. Industrial/refining rather than aerospace, but fits mechanical/manufacturing discipline. Requires majoring in Mechanical or Civil Engineering; no visa sponsorship available. Posting also states co-op positions run spring, summer, and fall generally, but this specific req is titled and dated for Spring 2027. Additional refinery locations listed on same req: Anacortes WA, Canton OH, Catlettsburg KY, Detroit MI, El Paso TX, Garyville LA, Kenai AK, Mandan ND, Martinez CA, Robinson IL, Salt Lake City UT, St Paul Park MN, Texas City TX, Wilmington CA.</v>
       </c>
       <c r="K105" t="str">
         <v>Open resume</v>
@@ -4707,34 +4707,34 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Varda Space Industries</v>
+        <v>GE Appliances (a Haier company)</v>
       </c>
       <c r="B106" t="str">
-        <v>Vehicle Integration &amp; Test Internship (Spring 2027)</v>
+        <v>Mechanical Engineering Co-op (Spring 2027)</v>
       </c>
       <c r="C106" t="str">
-        <v>Mechanical / Aerospace Systems Engineering</v>
+        <v>Mechanical Engineering (Consumer Product Manufacturing)</v>
       </c>
       <c r="D106" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Jan 11 – May 7, 2027)</v>
       </c>
       <c r="E106" t="str">
-        <v>El Segundo, CA</v>
+        <v>Louisville, KY</v>
       </c>
       <c r="F106">
-        <v>2600</v>
+        <v>950</v>
       </c>
       <c r="G106" t="str">
-        <v>$33.00/hr + housing stipend for relocating interns</v>
+        <v>Not stated on posting; housing/relocation assistance available for eligible students</v>
       </c>
       <c r="H106" t="str">
-        <v>https://job-boards.greenhouse.io/vardaspace/jobs/7824772003</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/Mechanical-Engineering-Co-op-Spring-2027_REQ-24833</v>
       </c>
       <c r="I106" t="str">
-        <v>Yes — fetched directly via Varda's own Greenhouse API (boards-api.greenhouse.io), HTTP 200, posting active, first published 2026-08-07.</v>
+        <v>Yes — fetched directly via GE Appliances' own Workday CXS API, full job description returned with explicit dates, req REQ-24833.</v>
       </c>
       <c r="J106" t="str">
-        <v>Sibling req to the already-tracked Varda internships at the same company/season. Vehicle integration and test of flight hardware. US work authorization + export-control (ITAR) screening required per posting (US persons only).</v>
+        <v>New company, not previously tracked. Industrial/consumer-manufacturing rather than aerospace, but squarely mechanical engineering with a clean Spring-only (not combined) term and explicit dates.</v>
       </c>
       <c r="K106" t="str">
         <v>Open resume</v>
@@ -4748,34 +4748,34 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Marathon Petroleum</v>
+        <v>Entegris</v>
       </c>
       <c r="B107" t="str">
-        <v>Intern/Co-op - Refining Mechanical Engineer (Spring 2027)</v>
+        <v>Mechanical Engineering Co-Op</v>
       </c>
       <c r="C107" t="str">
-        <v>Mechanical Engineering (Industrial / Refining)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D107" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (6-month assignment)</v>
       </c>
       <c r="E107" t="str">
-        <v>Findlay, OH</v>
+        <v>Billerica, MA</v>
       </c>
       <c r="F107">
-        <v>700</v>
+        <v>20</v>
       </c>
       <c r="G107" t="str">
-        <v>$32.92–$41.67/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H107" t="str">
-        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Intern-Co-op---Refining-Mechanical-Engineer--Spring-2027-_00020137</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Mechanical-Engineering-Co-Op_REQ-14457</v>
       </c>
       <c r="I107" t="str">
-        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API, full job description returned, req 00020137.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (tenant entegris), HTTP 200, canApply true, posting text explicitly states "Spring 2027 season," posted 12 days ago.</v>
       </c>
       <c r="J107" t="str">
-        <v>New company, not previously tracked. Industrial/refining rather than aerospace, but fits mechanical/manufacturing discipline. Requires majoring in Mechanical or Civil Engineering; no visa sponsorship available. Posting also states co-op positions run spring, summer, and fall generally, but this specific req is titled and dated for Spring 2027. Additional refinery locations listed on same req: Anacortes WA, Canton OH, Catlettsburg KY, Detroit MI, El Paso TX, Garyville LA, Kenai AK, Mandan ND, Martinez CA, Robinson IL, Salt Lake City UT, St Paul Park MN, Texas City TX, Wilmington CA.</v>
+        <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
       </c>
       <c r="K107" t="str">
         <v>Open resume</v>
@@ -4789,75 +4789,75 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>GE Appliances (a Haier company)</v>
+        <v>Insulet</v>
       </c>
       <c r="B108" t="str">
-        <v>Mechanical Engineering Co-op (Spring 2027)</v>
+        <v>Graduate Co-op, Supplier Engineering - Project Management Excellence (Jan–June 2027, Onsite)</v>
       </c>
       <c r="C108" t="str">
-        <v>Mechanical Engineering (Consumer Product Manufacturing)</v>
+        <v>Industrial / Biomedical / Mechanical Engineering (MS)</v>
       </c>
       <c r="D108" t="str">
-        <v>Spring 2027 (Jan 11 – May 7, 2027)</v>
+        <v>Winter/Spring 2027 (Jan 11 – Jun 30, 2027)</v>
       </c>
       <c r="E108" t="str">
-        <v>Louisville, KY</v>
+        <v>Acton, MA</v>
       </c>
       <c r="F108">
-        <v>950</v>
+        <v>25</v>
       </c>
       <c r="G108" t="str">
-        <v>Not stated on posting; housing/relocation assistance available for eligible students</v>
+        <v>$25.00–$34.00/hr</v>
       </c>
       <c r="H108" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/Mechanical-Engineering-Co-op-Spring-2027_REQ-24833</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Graduate-Co-op--Supplier-Engineering---Project-Management-Excellence--January---June-2027--Onsite-_REQ-2026-18165</v>
       </c>
       <c r="I108" t="str">
-        <v>Yes — fetched directly via GE Appliances' own Workday CXS API, full job description returned with explicit dates, req REQ-24833.</v>
+        <v>Yes — fetched directly via Insulet's own Workday CXS API (tenant insulet), HTTP 200, canApply true, explicit dates Jan 11 – Jun 30 2027, posted yesterday.</v>
       </c>
       <c r="J108" t="str">
-        <v>New company, not previously tracked. Industrial/consumer-manufacturing rather than aerospace, but squarely mechanical engineering with a clean Spring-only (not combined) term and explicit dates.</v>
+        <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
       </c>
       <c r="K108" t="str">
-        <v>Open resume</v>
+        <v>Skipped: graduate students only (you are an undergrad)</v>
       </c>
       <c r="L108" t="str">
-        <v>Open cover letter</v>
+        <v>Skipped: graduate students only (you are an undergrad)</v>
       </c>
       <c r="M108" t="str">
-        <v>Open questions</v>
+        <v>Skipped: graduate students only (you are an undergrad)</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Entegris</v>
+        <v>GE Appliances (a Haier company)</v>
       </c>
       <c r="B109" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Mechanical Engineering Technology Co-op (Spring 2027)</v>
       </c>
       <c r="C109" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical Engineering Technology</v>
       </c>
       <c r="D109" t="str">
-        <v>Spring 2027 (6-month assignment)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E109" t="str">
-        <v>Billerica, MA</v>
+        <v>Louisville, KY</v>
       </c>
       <c r="F109">
-        <v>20</v>
+        <v>950</v>
       </c>
       <c r="G109" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H109" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Mechanical-Engineering-Co-Op_REQ-14457</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Mechanical-Engineering-Technology-Co-op-Spring-2027_REQ-24835</v>
       </c>
       <c r="I109" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (tenant entegris), HTTP 200, canApply true, posting text explicitly states "Spring 2027 season," posted 12 days ago.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch (both search and full job-detail endpoints) returned HTTP 200 with canApply:true. Supersedes the earlier Partial status from Workday bot-blocking on a prior run.</v>
       </c>
       <c r="J109" t="str">
-        <v>6th Entegris/Billerica req tracked (in addition to REQ-14497, 14444, 14469, 14462, 14504). Manufacturing Operations team, process/scrap-reduction focus.</v>
+        <v>New req beyond the already-tracked REQ-24833 (Mechanical Engineering Co-op) at the same Louisville, KY site.</v>
       </c>
       <c r="K109" t="str">
         <v>Open resume</v>
@@ -4871,43 +4871,43 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Insulet</v>
+        <v>GE Appliances (a Haier company)</v>
       </c>
       <c r="B110" t="str">
-        <v>Graduate Co-op, Supplier Engineering - Project Management Excellence (Jan–June 2027, Onsite)</v>
+        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
       </c>
       <c r="C110" t="str">
-        <v>Industrial / Biomedical / Mechanical Engineering (MS)</v>
+        <v>Mechanical / Manufacturing Engineering</v>
       </c>
       <c r="D110" t="str">
-        <v>Winter/Spring 2027 (Jan 11 – Jun 30, 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E110" t="str">
-        <v>Acton, MA</v>
+        <v>Louisville, KY</v>
       </c>
       <c r="F110">
-        <v>25</v>
+        <v>950</v>
       </c>
       <c r="G110" t="str">
-        <v>$25.00–$34.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H110" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Graduate-Co-op--Supplier-Engineering---Project-Management-Excellence--January---June-2027--Onsite-_REQ-2026-18165</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24837</v>
       </c>
       <c r="I110" t="str">
-        <v>Yes — fetched directly via Insulet's own Workday CXS API (tenant insulet), HTTP 200, canApply true, explicit dates Jan 11 – Jun 30 2027, posted yesterday.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J110" t="str">
-        <v>MS-level sibling of the already-tracked undergrad 'Supplier Engineering - Project Management Excellence' co-op (REQ-2026-18211); same discipline mix (Industrial/Biomedical/Mechanical/Engineering Management) already accepted for that req. Not eligible for visa sponsorship.</v>
+        <v>New req beyond the already-tracked REQ-24833 at the same Louisville, KY site.</v>
       </c>
       <c r="K110" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
+        <v>Open resume</v>
       </c>
       <c r="L110" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
+        <v>Open cover letter</v>
       </c>
       <c r="M110" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
+        <v>Open questions</v>
       </c>
     </row>
     <row r="111">
@@ -4915,31 +4915,31 @@
         <v>GE Appliances (a Haier company)</v>
       </c>
       <c r="B111" t="str">
-        <v>Mechanical Engineering Technology Co-op (Spring 2027)</v>
+        <v>Engineering Co-op (Spring 2027)</v>
       </c>
       <c r="C111" t="str">
-        <v>Mechanical Engineering Technology</v>
+        <v>Engineering (general — discipline not narrowly specified in title)</v>
       </c>
       <c r="D111" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E111" t="str">
-        <v>Louisville, KY</v>
+        <v>LaFayette, GA</v>
       </c>
       <c r="F111">
-        <v>950</v>
+        <v>1000</v>
       </c>
       <c r="G111" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H111" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Mechanical-Engineering-Technology-Co-op-Spring-2027_REQ-24835</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Co-op-Spring-2027_REQ-24836</v>
       </c>
       <c r="I111" t="str">
-        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch (both search and full job-detail endpoints) returned HTTP 200 with canApply:true. Supersedes the earlier Partial status from Workday bot-blocking on a prior run.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status. Discipline still not narrowly specified in title/posting.</v>
       </c>
       <c r="J111" t="str">
-        <v>New req beyond the already-tracked REQ-24833 (Mechanical Engineering Co-op) at the same Louisville, KY site.</v>
+        <v>New site (LaFayette, GA) for GE Appliances beyond the already-tracked Louisville, KY reqs.</v>
       </c>
       <c r="K111" t="str">
         <v>Open resume</v>
@@ -4965,22 +4965,22 @@
         <v>Spring 2027</v>
       </c>
       <c r="E112" t="str">
-        <v>Louisville, KY</v>
+        <v>LaFayette, GA</v>
       </c>
       <c r="F112">
-        <v>950</v>
+        <v>1000</v>
       </c>
       <c r="G112" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H112" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Louisville-KY/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24837</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24838</v>
       </c>
       <c r="I112" t="str">
         <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J112" t="str">
-        <v>New req beyond the already-tracked REQ-24833 at the same Louisville, KY site.</v>
+        <v>New req at the same LaFayette, GA site as REQ-24836.</v>
       </c>
       <c r="K112" t="str">
         <v>Open resume</v>
@@ -4997,31 +4997,31 @@
         <v>GE Appliances (a Haier company)</v>
       </c>
       <c r="B113" t="str">
-        <v>Engineering Co-op (Spring 2027)</v>
+        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
       </c>
       <c r="C113" t="str">
-        <v>Engineering (general — discipline not narrowly specified in title)</v>
+        <v>Mechanical / Manufacturing Engineering</v>
       </c>
       <c r="D113" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E113" t="str">
-        <v>LaFayette, GA</v>
+        <v>Decatur, AL</v>
       </c>
       <c r="F113">
-        <v>1000</v>
+        <v>1050</v>
       </c>
       <c r="G113" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H113" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Co-op-Spring-2027_REQ-24836</v>
+        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Decatur-AL/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24839</v>
       </c>
       <c r="I113" t="str">
-        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status. Discipline still not narrowly specified in title/posting.</v>
+        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
       </c>
       <c r="J113" t="str">
-        <v>New site (LaFayette, GA) for GE Appliances beyond the already-tracked Louisville, KY reqs.</v>
+        <v>New site (Decatur, AL) for GE Appliances beyond the already-tracked Louisville KY / LaFayette GA reqs.</v>
       </c>
       <c r="K113" t="str">
         <v>Open resume</v>
@@ -5035,75 +5035,75 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>GE Appliances (a Haier company)</v>
+        <v>Hologic</v>
       </c>
       <c r="B114" t="str">
-        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
+        <v>Co-Op, R&amp;D Mechanical Engineer</v>
       </c>
       <c r="C114" t="str">
-        <v>Mechanical / Manufacturing Engineering</v>
+        <v>Mechanical Engineering (R&amp;D)</v>
       </c>
       <c r="D114" t="str">
-        <v>Spring 2027</v>
+        <v>Winter 2026 (Jan–June 2026)</v>
       </c>
       <c r="E114" t="str">
-        <v>LaFayette, GA</v>
+        <v>Marlborough, MA</v>
       </c>
       <c r="F114">
-        <v>1000</v>
+        <v>30</v>
       </c>
       <c r="G114" t="str">
-        <v>Not stated on posting</v>
+        <v>$26–$28/hr (per cached posting snippet)</v>
       </c>
       <c r="H114" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-LaFayette-GA/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24838</v>
+        <v>https://na.careers.hologic.com/en/search/300000421584867/co-op-r-d-mechanical-engineer</v>
       </c>
       <c r="I114" t="str">
-        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
+        <v>Partial — this exact posting URL/req ID was located this run (prior runs only had aggregator mirrors). A search-engine-cached snippet of the live page confirms title, 'January – June 2026' dates, and $26–28/hr pay, matching Hamza's Winter 2026 target. However, the live page itself has returned HTTP 503 'Temporarily Unavailable' across 8+ consecutive runs including this one (re-tried directly this session, still 503) — cannot confirm current open/closed status by opening the actual page. Verify live in-browser before applying.</v>
       </c>
       <c r="J114" t="str">
-        <v>New req at the same LaFayette, GA site as REQ-24836.</v>
+        <v>Long-standing 'worth re-checking' item, now has a confirmed direct URL and season match for the first time. A second, likely newer Hologic req ('Co-Op, New Product Development Engineering', .../300000422097244/...) was also found this run but remains season-unconfirmed and 503-blocked — see `checked`.</v>
       </c>
       <c r="K114" t="str">
-        <v>Open resume</v>
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
       </c>
       <c r="L114" t="str">
-        <v>Open cover letter</v>
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
       </c>
       <c r="M114" t="str">
-        <v>Open questions</v>
+        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>GE Appliances (a Haier company)</v>
+        <v>Aalo Atomics</v>
       </c>
       <c r="B115" t="str">
-        <v>Engineering/Manufacturing Co-op (Spring 2027)</v>
+        <v>Mechanical Engineering Internship/Co-op (Spring 2027)</v>
       </c>
       <c r="C115" t="str">
-        <v>Mechanical / Manufacturing Engineering</v>
+        <v>Mechanical / Aerospace / Manufacturing Engineering</v>
       </c>
       <c r="D115" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (January–May)</v>
       </c>
       <c r="E115" t="str">
-        <v>Decatur, AL</v>
+        <v>Austin, TX</v>
       </c>
       <c r="F115">
-        <v>1050</v>
+        <v>1700</v>
       </c>
       <c r="G115" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H115" t="str">
-        <v>https://haier.wd3.myworkdayjobs.com/en-US/GE_Appliances/job/USA-Decatur-AL/Engineering-Manufacturing-Co-op-Spring-2027_REQ-24839</v>
+        <v>https://ats.rippling.com/aalo-atomics/jobs/7be73c9f-f1b8-470c-8c7e-333220736f0b</v>
       </c>
       <c r="I115" t="str">
-        <v>Yes — upgraded 2026-09-24 ~07:00 UTC: this session's own direct Workday CXS API fetch returned HTTP 200 with canApply:true. Supersedes the earlier Partial status.</v>
+        <v>Yes — fetched directly, page live, 'Apply now' button present, no closed-application message.</v>
       </c>
       <c r="J115" t="str">
-        <v>New site (Decatur, AL) for GE Appliances beyond the already-tracked Louisville KY / LaFayette GA reqs.</v>
+        <v>New company for the tracker (advanced nuclear reactor startup). Requires B.S./M.S. in Mechanical, Aerospace, or Manufacturing Engineering (or closely related field) plus ~3 months applied engineering experience.</v>
       </c>
       <c r="K115" t="str">
         <v>Open resume</v>
@@ -5117,75 +5117,75 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Hologic</v>
+        <v>Hermeus</v>
       </c>
       <c r="B116" t="str">
-        <v>Co-Op, R&amp;D Mechanical Engineer</v>
+        <v>GNC &amp; Flight Software Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C116" t="str">
-        <v>Mechanical Engineering (R&amp;D)</v>
+        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
       </c>
       <c r="D116" t="str">
-        <v>Winter 2026 (Jan–June 2026)</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
       </c>
       <c r="E116" t="str">
-        <v>Marlborough, MA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F116">
-        <v>30</v>
+        <v>950</v>
       </c>
       <c r="G116" t="str">
-        <v>$26–$28/hr (per cached posting snippet)</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H116" t="str">
-        <v>https://na.careers.hologic.com/en/search/300000421584867/co-op-r-d-mechanical-engineer</v>
+        <v>https://jobs.khoslaventures.com/companies/hermeus/jobs/92195543-gnc-flight-software-intern-spring-summer-2027</v>
       </c>
       <c r="I116" t="str">
-        <v>Partial — this exact posting URL/req ID was located this run (prior runs only had aggregator mirrors). A search-engine-cached snippet of the live page confirms title, 'January – June 2026' dates, and $26–28/hr pay, matching Hamza's Winter 2026 target. However, the live page itself has returned HTTP 503 'Temporarily Unavailable' across 8+ consecutive runs including this one (re-tried directly this session, still 503) — cannot confirm current open/closed status by opening the actual page. Verify live in-browser before applying.</v>
+        <v>Yes — fetched directly, page live, 'Apply now' button present, posted 2026-09-04, no closed-application message.</v>
       </c>
       <c r="J116" t="str">
-        <v>Long-standing 'worth re-checking' item, now has a confirmed direct URL and season match for the first time. A second, likely newer Hologic req ('Co-Op, New Product Development Engineering', .../300000422097244/...) was also found this run but remains season-unconfirmed and 503-blocked — see `checked`.</v>
+        <v>New company for the tracker (hypersonic aircraft developer). GNC (Guidance, Navigation &amp; Controls) role — flight-systems/controls discipline. Also open to Aerospace/Computer Engineering/CS/EE majors. Unlike a truly combined-term posting, the Spring option has its own distinct dates, so included (same treatment as RTX's 'Winter/Spring 2027' co-ops).</v>
       </c>
       <c r="K116" t="str">
-        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+        <v>Open resume</v>
       </c>
       <c r="L116" t="str">
-        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+        <v>Open cover letter</v>
       </c>
       <c r="M116" t="str">
-        <v>Skipped: the Jan to June 2026 co-op window has already passed</v>
+        <v>Open questions</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Aalo Atomics</v>
+        <v>Owens Corning</v>
       </c>
       <c r="B117" t="str">
-        <v>Mechanical Engineering Internship/Co-op (Spring 2027)</v>
+        <v>Manufacturing Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C117" t="str">
-        <v>Mechanical / Aerospace / Manufacturing Engineering</v>
+        <v>Manufacturing / Mechanical Engineering</v>
       </c>
       <c r="D117" t="str">
-        <v>Spring 2027 (January–May)</v>
+        <v>Spring 2027 (~16 weeks)</v>
       </c>
       <c r="E117" t="str">
-        <v>Austin, TX</v>
+        <v>Toledo, OH (also hiring for Feura Bush, NY; Sedalia, MO; Irving, TX)</v>
       </c>
       <c r="F117">
-        <v>1700</v>
+        <v>720</v>
       </c>
       <c r="G117" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H117" t="str">
-        <v>https://ats.rippling.com/aalo-atomics/jobs/7be73c9f-f1b8-470c-8c7e-333220736f0b</v>
+        <v>https://careers.owenscorning.com/job/Toledo-Manufacturing-Engineering-Co-Op-(Spring-2027)-OH-43659-0001/1426905700/</v>
       </c>
       <c r="I117" t="str">
-        <v>Yes — fetched directly, page live, 'Apply now' button present, no closed-application message.</v>
+        <v>Yes — fetched directly, page live, 'APPLY NOW »' button present, no closed-application message.</v>
       </c>
       <c r="J117" t="str">
-        <v>New company for the tracker (advanced nuclear reactor startup). Requires B.S./M.S. in Mechanical, Aerospace, or Manufacturing Engineering (or closely related field) plus ~3 months applied engineering experience.</v>
+        <v>New company for the tracker (building materials manufacturer). Accepts Mechanical, Electrical, Engineering Technology, Chemical, or Industrial Engineering majors.</v>
       </c>
       <c r="K117" t="str">
         <v>Open resume</v>
@@ -5199,34 +5199,34 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Hermeus</v>
+        <v>Crown Equipment</v>
       </c>
       <c r="B118" t="str">
-        <v>GNC &amp; Flight Software Intern (Spring/Summer 2027)</v>
+        <v>Mechanical Engineering Co-op (Spring 2027)</v>
       </c>
       <c r="C118" t="str">
-        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D118" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E118" t="str">
-        <v>Atlanta, GA</v>
+        <v>Greencastle, IN</v>
       </c>
       <c r="F118">
-        <v>950</v>
+        <v>900</v>
       </c>
       <c r="G118" t="str">
-        <v>$25–33/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H118" t="str">
-        <v>https://jobs.khoslaventures.com/companies/hermeus/jobs/92195543-gnc-flight-software-intern-spring-summer-2027</v>
+        <v>https://us-careers.crown.com/job/Greencastle-Mechanical-Engineering-Co-op-Spring-2027-IN-46135/1420491100/</v>
       </c>
       <c r="I118" t="str">
-        <v>Yes — fetched directly, page live, 'Apply now' button present, posted 2026-09-04, no closed-application message.</v>
+        <v>Yes — fetched directly, page live, 'Apply now' button present, req 146174, no closed-application message.</v>
       </c>
       <c r="J118" t="str">
-        <v>New company for the tracker (hypersonic aircraft developer). GNC (Guidance, Navigation &amp; Controls) role — flight-systems/controls discipline. Also open to Aerospace/Computer Engineering/CS/EE majors. Unlike a truly combined-term posting, the Spring option has its own distinct dates, so included (same treatment as RTX's 'Winter/Spring 2027' co-ops).</v>
+        <v>New company for the tracker (forklift/material handling equipment manufacturer). Mechanical design/simulation/testing for forklift and material handling equipment development.</v>
       </c>
       <c r="K118" t="str">
         <v>Open resume</v>
@@ -5240,34 +5240,34 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Owens Corning</v>
+        <v>Anduril Industries</v>
       </c>
       <c r="B119" t="str">
-        <v>Manufacturing Engineering Co-Op (Spring 2027)</v>
+        <v>Winter 2027 EWIS Harness Engineer Co-op</v>
       </c>
       <c r="C119" t="str">
-        <v>Manufacturing / Mechanical Engineering</v>
+        <v>Mechanical / Electrical Engineering (wire harness design)</v>
       </c>
       <c r="D119" t="str">
-        <v>Spring 2027 (~16 weeks)</v>
+        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027)</v>
       </c>
       <c r="E119" t="str">
-        <v>Toledo, OH (also hiring for Feura Bush, NY; Sedalia, MO; Irving, TX)</v>
+        <v>Costa Mesa, CA</v>
       </c>
       <c r="F119">
-        <v>720</v>
+        <v>2600</v>
       </c>
       <c r="G119" t="str">
-        <v>Not stated on posting</v>
+        <v>$34–$50/hr</v>
       </c>
       <c r="H119" t="str">
-        <v>https://careers.owenscorning.com/job/Toledo-Manufacturing-Engineering-Co-Op-(Spring-2027)-OH-43659-0001/1426905700/</v>
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236577007</v>
       </c>
       <c r="I119" t="str">
-        <v>Yes — fetched directly, page live, 'APPLY NOW »' button present, no closed-application message.</v>
+        <v>Yes — fetched directly on Greenhouse, Apply button live, no closed-application message.</v>
       </c>
       <c r="J119" t="str">
-        <v>New company for the tracker (building materials manufacturer). Accepts Mechanical, Electrical, Engineering Technology, Chemical, or Industrial Engineering majors.</v>
+        <v>Resolves a 'worth re-checking' item from the 2026-09-23 ~19:00 UTC run (previously found without a job ID). Same batch/site as the already-tracked Propulsion, Warhead, and Test &amp; Evaluation Engineer Costa Mesa co-ops. Open to Mechanical or Electrical Engineering majors.</v>
       </c>
       <c r="K119" t="str">
         <v>Open resume</v>
@@ -5284,7 +5284,7 @@
         <v>Crown Equipment</v>
       </c>
       <c r="B120" t="str">
-        <v>Mechanical Engineering Co-op (Spring 2027)</v>
+        <v>Mechanical Engineering Intern/Co-op (Spring 2027)</v>
       </c>
       <c r="C120" t="str">
         <v>Mechanical Engineering</v>
@@ -5293,22 +5293,22 @@
         <v>Spring 2027</v>
       </c>
       <c r="E120" t="str">
-        <v>Greencastle, IN</v>
+        <v>Kinston, NC</v>
       </c>
       <c r="F120">
-        <v>900</v>
+        <v>700</v>
       </c>
       <c r="G120" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H120" t="str">
-        <v>https://us-careers.crown.com/job/Greencastle-Mechanical-Engineering-Co-op-Spring-2027-IN-46135/1420491100/</v>
+        <v>https://us-careers.crown.com/job/Kinston-Mechanical-Engineering-InternCo-op-Spring-2027-NC-28504/1426309500/</v>
       </c>
       <c r="I120" t="str">
-        <v>Yes — fetched directly, page live, 'Apply now' button present, req 146174, no closed-application message.</v>
+        <v>Yes — fetched directly, HTTP 200, title/season confirmed on page, 'Apply now' present, req 146597, no closed-application message.</v>
       </c>
       <c r="J120" t="str">
-        <v>New company for the tracker (forklift/material handling equipment manufacturer). Mechanical design/simulation/testing for forklift and material handling equipment development.</v>
+        <v>New sibling req to the already-tracked Greencastle, IN req (146174) at the same company, found via a fresh sweep of Crown's own careers site.</v>
       </c>
       <c r="K120" t="str">
         <v>Open resume</v>
@@ -5322,34 +5322,34 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Anduril Industries</v>
+        <v>Hermeus</v>
       </c>
       <c r="B121" t="str">
-        <v>Winter 2027 EWIS Harness Engineer Co-op</v>
+        <v>Structures/Mechanical Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C121" t="str">
-        <v>Mechanical / Electrical Engineering (wire harness design)</v>
+        <v>Structural / Mechanical Engineering</v>
       </c>
       <c r="D121" t="str">
-        <v>Winter 2027 (16–24 wks, effectively Jan–Aug 2027)</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
       </c>
       <c r="E121" t="str">
-        <v>Costa Mesa, CA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F121">
-        <v>2600</v>
+        <v>950</v>
       </c>
       <c r="G121" t="str">
-        <v>$34–$50/hr</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H121" t="str">
-        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5236577007</v>
+        <v>https://jobs.lever.co/hermeus/60b5d40a-1065-4bd2-8c72-6b2fb69d4761</v>
       </c>
       <c r="I121" t="str">
-        <v>Yes — fetched directly on Greenhouse, Apply button live, no closed-application message.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-08 or similar recent date.</v>
       </c>
       <c r="J121" t="str">
-        <v>Resolves a 'worth re-checking' item from the 2026-09-23 ~19:00 UTC run (previously found without a job ID). Same batch/site as the already-tracked Propulsion, Warhead, and Test &amp; Evaluation Engineer Costa Mesa co-ops. Open to Mechanical or Electrical Engineering majors.</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern at the same company/site; same distinct Spring/Summer option structure (not a merged single term).</v>
       </c>
       <c r="K121" t="str">
         <v>Open resume</v>
@@ -5363,34 +5363,34 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Crown Equipment</v>
+        <v>Hermeus</v>
       </c>
       <c r="B122" t="str">
-        <v>Mechanical Engineering Intern/Co-op (Spring 2027)</v>
+        <v>Mechanical Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C122" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D122" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
       </c>
       <c r="E122" t="str">
-        <v>Kinston, NC</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F122">
-        <v>700</v>
+        <v>2600</v>
       </c>
       <c r="G122" t="str">
-        <v>Not stated on posting</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H122" t="str">
-        <v>https://us-careers.crown.com/job/Kinston-Mechanical-Engineering-InternCo-op-Spring-2027-NC-28504/1426309500/</v>
+        <v>https://jobs.lever.co/hermeus/1bc5c858-1b04-4093-80a0-2ba3491afc60</v>
       </c>
       <c r="I122" t="str">
-        <v>Yes — fetched directly, HTTP 200, title/season confirmed on page, 'Apply now' present, req 146597, no closed-application message.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
       </c>
       <c r="J122" t="str">
-        <v>New sibling req to the already-tracked Greencastle, IN req (146174) at the same company, found via a fresh sweep of Crown's own careers site.</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct Spring/Summer option structure.</v>
       </c>
       <c r="K122" t="str">
         <v>Open resume</v>
@@ -5407,31 +5407,31 @@
         <v>Hermeus</v>
       </c>
       <c r="B123" t="str">
-        <v>Structures/Mechanical Engineering Intern (Spring/Summer 2027)</v>
+        <v>Propulsion Component Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C123" t="str">
-        <v>Structural / Mechanical Engineering</v>
+        <v>Propulsion / Mechanical Engineering</v>
       </c>
       <c r="D123" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
       </c>
       <c r="E123" t="str">
-        <v>Atlanta, GA</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F123">
-        <v>950</v>
+        <v>2600</v>
       </c>
       <c r="G123" t="str">
         <v>$25–33/hr</v>
       </c>
       <c r="H123" t="str">
-        <v>https://jobs.lever.co/hermeus/60b5d40a-1065-4bd2-8c72-6b2fb69d4761</v>
+        <v>https://jobs.lever.co/hermeus/2cbb75f7-a040-47b2-a442-d9cc1faedb11</v>
       </c>
       <c r="I123" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-08 or similar recent date.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-08-31. Posting states only a Spring 2027 term, no Summer/Fall option.</v>
       </c>
       <c r="J123" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern at the same company/site; same distinct Spring/Summer option structure (not a merged single term).</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern. Flight-critical mechanical/fluid propulsion components (valves, actuators).</v>
       </c>
       <c r="K123" t="str">
         <v>Open resume</v>
@@ -5448,31 +5448,31 @@
         <v>Hermeus</v>
       </c>
       <c r="B124" t="str">
-        <v>Mechanical Engineering Intern (Spring/Summer 2027)</v>
+        <v>Propulsion Test Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C124" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Propulsion / Mechanical Engineering</v>
       </c>
       <c r="D124" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
       </c>
       <c r="E124" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Jacksonville, FL</v>
       </c>
       <c r="F124">
-        <v>2600</v>
+        <v>1050</v>
       </c>
       <c r="G124" t="str">
         <v>$25–33/hr</v>
       </c>
       <c r="H124" t="str">
-        <v>https://jobs.lever.co/hermeus/1bc5c858-1b04-4093-80a0-2ba3491afc60</v>
+        <v>https://jobs.lever.co/hermeus/d2651ecb-9aab-4d84-8e69-cbcf7cece28d</v>
       </c>
       <c r="I124" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-23 (posted same day as this run). Posting states only a Spring 2027 term, no Summer/Fall option.</v>
       </c>
       <c r="J124" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct Spring/Summer option structure.</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, new site (Jacksonville, FL). Propulsion system/engine test stand support.</v>
       </c>
       <c r="K124" t="str">
         <v>Open resume</v>
@@ -5489,13 +5489,13 @@
         <v>Hermeus</v>
       </c>
       <c r="B125" t="str">
-        <v>Propulsion Component Engineering Intern (Spring 2027)</v>
+        <v>Propulsion Engineering Intern (Spring/Summer/Fall 2027)</v>
       </c>
       <c r="C125" t="str">
         <v>Propulsion / Mechanical Engineering</v>
       </c>
       <c r="D125" t="str">
-        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
       </c>
       <c r="E125" t="str">
         <v>Los Angeles, CA</v>
@@ -5507,13 +5507,13 @@
         <v>$25–33/hr</v>
       </c>
       <c r="H125" t="str">
-        <v>https://jobs.lever.co/hermeus/2cbb75f7-a040-47b2-a442-d9cc1faedb11</v>
+        <v>https://jobs.lever.co/hermeus/943f51e4-5b26-432c-ae85-de5f43cadb86</v>
       </c>
       <c r="I125" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-08-31. Posting states only a Spring 2027 term, no Summer/Fall option.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
       </c>
       <c r="J125" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern. Flight-critical mechanical/fluid propulsion components (valves, actuators).</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure (Spring/Summer/Fall each independently dated, not a merged single term).</v>
       </c>
       <c r="K125" t="str">
         <v>Open resume</v>
@@ -5530,31 +5530,31 @@
         <v>Hermeus</v>
       </c>
       <c r="B126" t="str">
-        <v>Propulsion Test Engineering Intern (Spring 2027)</v>
+        <v>Structures Engineering Intern (Spring/Summer/Fall 2027)</v>
       </c>
       <c r="C126" t="str">
-        <v>Propulsion / Mechanical Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D126" t="str">
-        <v>Spring 2027 (~16 weeks, January–April) — Spring-only, no combined term</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
       </c>
       <c r="E126" t="str">
-        <v>Jacksonville, FL</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F126">
-        <v>1050</v>
+        <v>2600</v>
       </c>
       <c r="G126" t="str">
         <v>$25–33/hr</v>
       </c>
       <c r="H126" t="str">
-        <v>https://jobs.lever.co/hermeus/d2651ecb-9aab-4d84-8e69-cbcf7cece28d</v>
+        <v>https://jobs.lever.co/hermeus/6b65768c-a8b2-4c77-8d5f-f407e32bb878</v>
       </c>
       <c r="I126" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-23 (posted same day as this run). Posting states only a Spring 2027 term, no Summer/Fall option.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
       </c>
       <c r="J126" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, new site (Jacksonville, FL). Propulsion system/engine test stand support.</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
       </c>
       <c r="K126" t="str">
         <v>Open resume</v>
@@ -5571,31 +5571,31 @@
         <v>Hermeus</v>
       </c>
       <c r="B127" t="str">
-        <v>Propulsion Engineering Intern (Spring/Summer/Fall 2027)</v>
+        <v>Manufacturing Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C127" t="str">
-        <v>Propulsion / Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D127" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
       </c>
       <c r="E127" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F127">
-        <v>2600</v>
+        <v>950</v>
       </c>
       <c r="G127" t="str">
         <v>$25–33/hr</v>
       </c>
       <c r="H127" t="str">
-        <v>https://jobs.lever.co/hermeus/943f51e4-5b26-432c-ae85-de5f43cadb86</v>
+        <v>https://jobs.lever.co/hermeus/1bdf3754-5649-4a50-913e-b05140cb004f</v>
       </c>
       <c r="I127" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
       </c>
       <c r="J127" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure (Spring/Summer/Fall each independently dated, not a merged single term).</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
       </c>
       <c r="K127" t="str">
         <v>Open resume</v>
@@ -5612,10 +5612,10 @@
         <v>Hermeus</v>
       </c>
       <c r="B128" t="str">
-        <v>Structures Engineering Intern (Spring/Summer/Fall 2027)</v>
+        <v>Manufacturing Engineering Intern (Spring/Summer/Fall 2027)</v>
       </c>
       <c r="C128" t="str">
-        <v>Structural Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D128" t="str">
         <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
@@ -5630,13 +5630,13 @@
         <v>$25–33/hr</v>
       </c>
       <c r="H128" t="str">
-        <v>https://jobs.lever.co/hermeus/6b65768c-a8b2-4c77-8d5f-f407e32bb878</v>
+        <v>https://jobs.lever.co/hermeus/5f6a6e79-9836-4c33-b40b-a2bb6c27bd06</v>
       </c>
       <c r="I128" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD.</v>
+        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
       </c>
       <c r="J128" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
+        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, a distinct site (Los Angeles) from the Atlanta Manufacturing Engineering Intern req above.</v>
       </c>
       <c r="K128" t="str">
         <v>Open resume</v>
@@ -5650,34 +5650,34 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Hermeus</v>
+        <v>Entegris</v>
       </c>
       <c r="B129" t="str">
-        <v>Manufacturing Engineering Intern (Spring/Summer 2027)</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C129" t="str">
         <v>Manufacturing Engineering</v>
       </c>
       <c r="D129" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
+        <v>Spring 2027 (~6 months)</v>
       </c>
       <c r="E129" t="str">
-        <v>Atlanta, GA</v>
+        <v>Billerica, MA</v>
       </c>
       <c r="F129">
-        <v>950</v>
+        <v>25</v>
       </c>
       <c r="G129" t="str">
-        <v>$25–33/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H129" t="str">
-        <v>https://jobs.lever.co/hermeus/1bdf3754-5649-4a50-913e-b05140cb004f</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Manufacturing-Engineering-Co-Op_REQ-14492</v>
       </c>
       <c r="I129" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API, HTTP 200, description explicitly states 'Spring 2027 season.'</v>
       </c>
       <c r="J129" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern; same distinct term-option structure.</v>
+        <v>New sibling req to the already-tracked Entegris Billerica co-ops (different REQ range than a previously-excluded stale REQ-7046 series). Supports process engineers on the Billerica filter manufacturing line.</v>
       </c>
       <c r="K129" t="str">
         <v>Open resume</v>
@@ -5691,34 +5691,34 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Hermeus</v>
+        <v>Fives</v>
       </c>
       <c r="B130" t="str">
-        <v>Manufacturing Engineering Intern (Spring/Summer/Fall 2027)</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C130" t="str">
         <v>Manufacturing Engineering</v>
       </c>
       <c r="D130" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E130" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Hebron, KY</v>
       </c>
       <c r="F130">
-        <v>2600</v>
+        <v>900</v>
       </c>
       <c r="G130" t="str">
-        <v>$25–33/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H130" t="str">
-        <v>https://jobs.lever.co/hermeus/5f6a6e79-9836-4c33-b40b-a2bb6c27bd06</v>
+        <v>https://career.fivesgroup.com/job/Hebron-Manufacturing-Engineering-Co-Op-Spring-2027-Kent-41048/1362251655/</v>
       </c>
       <c r="I130" t="str">
-        <v>Yes — fetched directly on Hermeus's own Lever board, HTTP 200, live embedded JobPosting JSON-LD, datePosted 2026-09-02.</v>
+        <v>Yes — fetched directly on career.fivesgroup.com (Fives's own site, not an aggregator), HTTP 200, 'Apply Now' active, 'Spring 2027' stated in title/body.</v>
       </c>
       <c r="J130" t="str">
-        <v>New sibling req to the already-tracked GNC &amp; Flight Software Intern, a distinct site (Los Angeles) from the Atlanta Manufacturing Engineering Intern req above.</v>
+        <v>Resolves a block that persisted across multiple prior runs (site previously only found via an aggregator mirror, never opened directly).</v>
       </c>
       <c r="K130" t="str">
         <v>Open resume</v>
@@ -5732,34 +5732,34 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Entegris</v>
+        <v>Formlabs</v>
       </c>
       <c r="B131" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Manufacturing Engineering Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C131" t="str">
         <v>Manufacturing Engineering</v>
       </c>
       <c r="D131" t="str">
-        <v>Spring 2027 (~6 months)</v>
+        <v>Winter/Spring 2027 (January–April/June)</v>
       </c>
       <c r="E131" t="str">
-        <v>Billerica, MA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F131">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="G131" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H131" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Manufacturing-Engineering-Co-Op_REQ-14492</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8161817</v>
       </c>
       <c r="I131" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API, HTTP 200, description explicitly states 'Spring 2027 season.'</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: January - April/June 2027.'</v>
       </c>
       <c r="J131" t="str">
-        <v>New sibling req to the already-tracked Entegris Billerica co-ops (different REQ range than a previously-excluded stale REQ-7046 series). Supports process engineers on the Billerica filter manufacturing line.</v>
+        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
       </c>
       <c r="K131" t="str">
         <v>Open resume</v>
@@ -5773,34 +5773,34 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>Fives</v>
+        <v>Formlabs</v>
       </c>
       <c r="B132" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Hardware R&amp;D Engineering Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C132" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical/Hardware Engineering</v>
       </c>
       <c r="D132" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (January–April)</v>
       </c>
       <c r="E132" t="str">
-        <v>Hebron, KY</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F132">
-        <v>900</v>
+        <v>3</v>
       </c>
       <c r="G132" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H132" t="str">
-        <v>https://career.fivesgroup.com/job/Hebron-Manufacturing-Engineering-Co-Op-Spring-2027-Kent-41048/1362251655/</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172226</v>
       </c>
       <c r="I132" t="str">
-        <v>Yes — fetched directly on career.fivesgroup.com (Fives's own site, not an aggregator), HTTP 200, 'Apply Now' active, 'Spring 2027' stated in title/body.</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
       </c>
       <c r="J132" t="str">
-        <v>Resolves a block that persisted across multiple prior runs (site previously only found via an aggregator mirror, never opened directly).</v>
+        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
       </c>
       <c r="K132" t="str">
         <v>Open resume</v>
@@ -5817,13 +5817,13 @@
         <v>Formlabs</v>
       </c>
       <c r="B133" t="str">
-        <v>Manufacturing Engineering Intern (Winter/Spring 2027)</v>
+        <v>Materials Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C133" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Materials Engineering</v>
       </c>
       <c r="D133" t="str">
-        <v>Winter/Spring 2027 (January–April/June)</v>
+        <v>Winter/Spring 2027 (January–April)</v>
       </c>
       <c r="E133" t="str">
         <v>Somerville, MA</v>
@@ -5835,10 +5835,10 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H133" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8161817</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199092</v>
       </c>
       <c r="I133" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: January - April/June 2027.'</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
       </c>
       <c r="J133" t="str">
         <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
@@ -5855,34 +5855,34 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Formlabs</v>
+        <v>Hermeus</v>
       </c>
       <c r="B134" t="str">
-        <v>Hardware R&amp;D Engineering Intern (Winter/Spring 2027)</v>
+        <v>Mission Systems Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C134" t="str">
-        <v>Mechanical/Hardware Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D134" t="str">
-        <v>Winter/Spring 2027 (January–April)</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
       </c>
       <c r="E134" t="str">
-        <v>Somerville, MA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F134">
-        <v>3</v>
+        <v>950</v>
       </c>
       <c r="G134" t="str">
-        <v>Not stated on posting</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H134" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172226</v>
+        <v>https://jobs.lever.co/hermeus/9229aa88-f54d-4ecd-85ee-b31f53b4207d</v>
       </c>
       <c r="I134" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
+        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring (Jan–Apr) vs Summer (May–Aug) dated slots.</v>
       </c>
       <c r="J134" t="str">
-        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
+        <v>Mix of hardware and software systems-integration work; included under Hamza's aerospace/systems discipline.</v>
       </c>
       <c r="K134" t="str">
         <v>Open resume</v>
@@ -5896,34 +5896,34 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Formlabs</v>
+        <v>Hermeus</v>
       </c>
       <c r="B135" t="str">
-        <v>Materials Intern (Winter/Spring 2027)</v>
+        <v>Flight Operations &amp; Airworthiness Engineering Intern (Spring/Summer/Fall 2027)</v>
       </c>
       <c r="C135" t="str">
-        <v>Materials Engineering</v>
+        <v>Flight Systems</v>
       </c>
       <c r="D135" t="str">
-        <v>Winter/Spring 2027 (January–April)</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
       </c>
       <c r="E135" t="str">
-        <v>Somerville, MA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F135">
-        <v>3</v>
+        <v>950</v>
       </c>
       <c r="G135" t="str">
-        <v>Not stated on posting</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H135" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199092</v>
+        <v>https://jobs.lever.co/hermeus/944918b0-17ca-46ec-9413-5acd7086addf</v>
       </c>
       <c r="I135" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, content states 'Internship Term: Winter/Spring 2027 (January - April).'</v>
+        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring/Summer/Fall 2027 dated slots.</v>
       </c>
       <c r="J135" t="str">
-        <v>New sibling req to the already-tracked Formlabs Mechanical Engineering Intern.</v>
+        <v>New discipline not previously tracked at Hermeus; on experimental high-performance aircraft flight test/airworthiness.</v>
       </c>
       <c r="K135" t="str">
         <v>Open resume</v>
@@ -5937,34 +5937,34 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Hermeus</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B136" t="str">
-        <v>Mission Systems Engineering Intern (Spring/Summer 2027)</v>
+        <v>Additive Manufacturing Intern, Spring 2027</v>
       </c>
       <c r="C136" t="str">
-        <v>Systems Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D136" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option; intern selects one</v>
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E136" t="str">
-        <v>Atlanta, GA</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F136">
-        <v>950</v>
+        <v>2600</v>
       </c>
       <c r="G136" t="str">
-        <v>$25–33/hr</v>
+        <v>$28/hr</v>
       </c>
       <c r="H136" t="str">
-        <v>https://jobs.lever.co/hermeus/9229aa88-f54d-4ecd-85ee-b31f53b4207d</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7983576003</v>
       </c>
       <c r="I136" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring (Jan–Apr) vs Summer (May–Aug) dated slots.</v>
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J136" t="str">
-        <v>Mix of hardware and software systems-integration work; included under Hamza's aerospace/systems discipline.</v>
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
       <c r="K136" t="str">
         <v>Open resume</v>
@@ -5978,34 +5978,34 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>Hermeus</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B137" t="str">
-        <v>Flight Operations &amp; Airworthiness Engineering Intern (Spring/Summer/Fall 2027)</v>
+        <v>Combustion Devices Intern, Spring 2027</v>
       </c>
       <c r="C137" t="str">
-        <v>Flight Systems</v>
+        <v>Propulsion Engineering</v>
       </c>
       <c r="D137" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers separate Summer and Fall 2027 options; intern selects one</v>
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E137" t="str">
-        <v>Atlanta, GA</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F137">
-        <v>950</v>
+        <v>2600</v>
       </c>
       <c r="G137" t="str">
-        <v>$25–33/hr</v>
+        <v>$28/hr</v>
       </c>
       <c r="H137" t="str">
-        <v>https://jobs.lever.co/hermeus/944918b0-17ca-46ec-9413-5acd7086addf</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986744003</v>
       </c>
       <c r="I137" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, description confirms distinct Spring/Summer/Fall 2027 dated slots.</v>
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J137" t="str">
-        <v>New discipline not previously tracked at Hermeus; on experimental high-performance aircraft flight test/airworthiness.</v>
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
       <c r="K137" t="str">
         <v>Open resume</v>
@@ -6022,10 +6022,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B138" t="str">
-        <v>Additive Manufacturing Intern, Spring 2027</v>
+        <v>Fluid Component Intern, Spring 2027</v>
       </c>
       <c r="C138" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D138" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6040,7 +6040,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H138" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7983576003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990367003</v>
       </c>
       <c r="I138" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6063,10 +6063,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B139" t="str">
-        <v>Combustion Devices Intern, Spring 2027</v>
+        <v>Fluid Systems Intern, Spring 2027</v>
       </c>
       <c r="C139" t="str">
-        <v>Propulsion Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D139" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6081,7 +6081,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H139" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986744003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986788003</v>
       </c>
       <c r="I139" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6104,10 +6104,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B140" t="str">
-        <v>Fluid Component Intern, Spring 2027</v>
+        <v>Integration &amp; Test Intern, Spring 2027</v>
       </c>
       <c r="C140" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D140" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6122,7 +6122,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H140" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990367003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987252003</v>
       </c>
       <c r="I140" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6145,10 +6145,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B141" t="str">
-        <v>Fluid Systems Intern, Spring 2027</v>
+        <v>Manufacturing Engineering Intern, Spring 2027</v>
       </c>
       <c r="C141" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D141" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6163,13 +6163,13 @@
         <v>$28/hr</v>
       </c>
       <c r="H141" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986788003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7984943003</v>
       </c>
       <c r="I141" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J141" t="str">
-        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026; sibling reqs also open at Middle River, MD and Wallops Island, VA (see below).</v>
       </c>
       <c r="K141" t="str">
         <v>Open resume</v>
@@ -6186,31 +6186,31 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B142" t="str">
-        <v>Integration &amp; Test Intern, Spring 2027</v>
+        <v>Manufacturing Engineering Intern, Spring 2027</v>
       </c>
       <c r="C142" t="str">
-        <v>Systems Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D142" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E142" t="str">
-        <v>Long Beach, CA</v>
+        <v>Middle River, MD</v>
       </c>
       <c r="F142">
-        <v>2600</v>
+        <v>400</v>
       </c>
       <c r="G142" t="str">
-        <v>$28/hr</v>
+        <v>$25/hr</v>
       </c>
       <c r="H142" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987252003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987020003</v>
       </c>
       <c r="I142" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J142" t="str">
-        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+        <v>Sibling req to the Long Beach, CA and Wallops Island, VA Manufacturing Engineering Intern postings.</v>
       </c>
       <c r="K142" t="str">
         <v>Open resume</v>
@@ -6236,22 +6236,22 @@
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E143" t="str">
-        <v>Long Beach, CA</v>
+        <v>Wallops Island, VA</v>
       </c>
       <c r="F143">
-        <v>2600</v>
+        <v>450</v>
       </c>
       <c r="G143" t="str">
-        <v>$28/hr</v>
+        <v>$25/hr</v>
       </c>
       <c r="H143" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7984943003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996617003</v>
       </c>
       <c r="I143" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J143" t="str">
-        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026; sibling reqs also open at Middle River, MD and Wallops Island, VA (see below).</v>
+        <v>Sibling req to the Long Beach, CA and Middle River, MD Manufacturing Engineering Intern postings.</v>
       </c>
       <c r="K143" t="str">
         <v>Open resume</v>
@@ -6268,31 +6268,31 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B144" t="str">
-        <v>Manufacturing Engineering Intern, Spring 2027</v>
+        <v>Mechanical Engineering Intern, Spring 2027</v>
       </c>
       <c r="C144" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D144" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E144" t="str">
-        <v>Middle River, MD</v>
+        <v>Silver Spring, MD</v>
       </c>
       <c r="F144">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="G144" t="str">
         <v>$25/hr</v>
       </c>
       <c r="H144" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987020003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7989995003</v>
       </c>
       <c r="I144" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J144" t="str">
-        <v>Sibling req to the Long Beach, CA and Wallops Island, VA Manufacturing Engineering Intern postings.</v>
+        <v>Distinct site from the already-tracked Long Beach, CA Mechanical Engineering Intern req.</v>
       </c>
       <c r="K144" t="str">
         <v>Open resume</v>
@@ -6309,31 +6309,31 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B145" t="str">
-        <v>Manufacturing Engineering Intern, Spring 2027</v>
+        <v>Propulsion Analyst Intern, Spring 2027</v>
       </c>
       <c r="C145" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Propulsion Engineering</v>
       </c>
       <c r="D145" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E145" t="str">
-        <v>Wallops Island, VA</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F145">
-        <v>450</v>
+        <v>2600</v>
       </c>
       <c r="G145" t="str">
-        <v>$25/hr</v>
+        <v>$28/hr</v>
       </c>
       <c r="H145" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996617003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986824003</v>
       </c>
       <c r="I145" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J145" t="str">
-        <v>Sibling req to the Long Beach, CA and Middle River, MD Manufacturing Engineering Intern postings.</v>
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
       <c r="K145" t="str">
         <v>Open resume</v>
@@ -6350,31 +6350,31 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B146" t="str">
-        <v>Mechanical Engineering Intern, Spring 2027</v>
+        <v>Propulsion Design Intern, Spring 2027</v>
       </c>
       <c r="C146" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Propulsion Engineering</v>
       </c>
       <c r="D146" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E146" t="str">
-        <v>Silver Spring, MD</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F146">
-        <v>440</v>
+        <v>2600</v>
       </c>
       <c r="G146" t="str">
-        <v>$25/hr</v>
+        <v>$28/hr</v>
       </c>
       <c r="H146" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7989995003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987110003</v>
       </c>
       <c r="I146" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J146" t="str">
-        <v>Distinct site from the already-tracked Long Beach, CA Mechanical Engineering Intern req.</v>
+        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
       </c>
       <c r="K146" t="str">
         <v>Open resume</v>
@@ -6391,7 +6391,7 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B147" t="str">
-        <v>Propulsion Analyst Intern, Spring 2027</v>
+        <v>Propulsion Intern, Spring 2027</v>
       </c>
       <c r="C147" t="str">
         <v>Propulsion Engineering</v>
@@ -6409,7 +6409,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H147" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986824003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986790003</v>
       </c>
       <c r="I147" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6432,10 +6432,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B148" t="str">
-        <v>Propulsion Design Intern, Spring 2027</v>
+        <v>Structural Analysis Intern, Spring 2027</v>
       </c>
       <c r="C148" t="str">
-        <v>Propulsion Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D148" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6450,7 +6450,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H148" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987110003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986685003</v>
       </c>
       <c r="I148" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6473,10 +6473,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B149" t="str">
-        <v>Propulsion Intern, Spring 2027</v>
+        <v>Test Engineering Intern - Manufacturing, Spring 2027</v>
       </c>
       <c r="C149" t="str">
-        <v>Propulsion Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D149" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6491,7 +6491,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H149" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986790003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987042003</v>
       </c>
       <c r="I149" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6514,28 +6514,28 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B150" t="str">
-        <v>Structural Analysis Intern, Spring 2027</v>
+        <v>Test Engineering Intern, Spring 2027</v>
       </c>
       <c r="C150" t="str">
-        <v>Structural Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D150" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E150" t="str">
-        <v>Long Beach, CA</v>
+        <v>Stennis Space Center, MS</v>
       </c>
       <c r="F150">
-        <v>2600</v>
+        <v>1500</v>
       </c>
       <c r="G150" t="str">
-        <v>$28/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H150" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7986685003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990352003</v>
       </c>
       <c r="I150" t="str">
-        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season confirmed in body; pay range not found in content.</v>
       </c>
       <c r="J150" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
@@ -6555,10 +6555,10 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B151" t="str">
-        <v>Test Engineering Intern - Manufacturing, Spring 2027</v>
+        <v>Thermal Engineering Intern, Spring 2027</v>
       </c>
       <c r="C151" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D151" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
@@ -6573,7 +6573,7 @@
         <v>$28/hr</v>
       </c>
       <c r="H151" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987042003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8000951003</v>
       </c>
       <c r="I151" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
@@ -6596,28 +6596,28 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B152" t="str">
-        <v>Test Engineering Intern, Spring 2027</v>
+        <v>Turbomachinery Intern, Spring 2027</v>
       </c>
       <c r="C152" t="str">
-        <v>Systems Engineering</v>
+        <v>Propulsion Engineering</v>
       </c>
       <c r="D152" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E152" t="str">
-        <v>Stennis Space Center, MS</v>
+        <v>Long Beach, CA</v>
       </c>
       <c r="F152">
-        <v>1500</v>
+        <v>2600</v>
       </c>
       <c r="G152" t="str">
-        <v>Not stated on posting</v>
+        <v>$28/hr</v>
       </c>
       <c r="H152" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7990352003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987210003</v>
       </c>
       <c r="I152" t="str">
-        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season confirmed in body; pay range not found in content.</v>
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J152" t="str">
         <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
@@ -6637,31 +6637,31 @@
         <v>Rocket Lab</v>
       </c>
       <c r="B153" t="str">
-        <v>Thermal Engineering Intern, Spring 2027</v>
+        <v>R&amp;D Engineering Intern, Spring 2027</v>
       </c>
       <c r="C153" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Materials Engineering</v>
       </c>
       <c r="D153" t="str">
         <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E153" t="str">
-        <v>Long Beach, CA</v>
+        <v>Albuquerque, NM</v>
       </c>
       <c r="F153">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="G153" t="str">
-        <v>$28/hr</v>
+        <v>$20/hr</v>
       </c>
       <c r="H153" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8000951003</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996578003</v>
       </c>
       <c r="I153" t="str">
         <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
       </c>
       <c r="J153" t="str">
-        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+        <v>Materials/manufacturing-process R&amp;D on phase-change materials for solar arrays (constellation programs).</v>
       </c>
       <c r="K153" t="str">
         <v>Open resume</v>
@@ -6675,34 +6675,34 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>Rocket Lab</v>
+        <v>Entegris</v>
       </c>
       <c r="B154" t="str">
-        <v>Turbomachinery Intern, Spring 2027</v>
+        <v>Manufacturing Engineer Co-Op</v>
       </c>
       <c r="C154" t="str">
-        <v>Propulsion Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D154" t="str">
-        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+        <v>Spring 2027 season (6-month assignment)</v>
       </c>
       <c r="E154" t="str">
-        <v>Long Beach, CA</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F154">
-        <v>2600</v>
+        <v>17</v>
       </c>
       <c r="G154" t="str">
-        <v>$28/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H154" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7987210003</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Manufacturing-Engineer-Co-Op_REQ-14484</v>
       </c>
       <c r="I154" t="str">
-        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J154" t="str">
-        <v>Part of a large fresh wave of Rocket Lab Spring 2027 reqs posted Sept 9-21, 2026.</v>
+        <v>REQ-14484. New Entegris site for the tracker (Bedford, in addition to the 7 already-tracked Billerica reqs).</v>
       </c>
       <c r="K154" t="str">
         <v>Open resume</v>
@@ -6716,34 +6716,34 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Rocket Lab</v>
+        <v>Entegris</v>
       </c>
       <c r="B155" t="str">
-        <v>R&amp;D Engineering Intern, Spring 2027</v>
+        <v>Design and Process Engineering Co-Op</v>
       </c>
       <c r="C155" t="str">
-        <v>Materials Engineering</v>
+        <v>Mechanical / Process Engineering</v>
       </c>
       <c r="D155" t="str">
-        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+        <v>Spring 2027 season (6-month assignment)</v>
       </c>
       <c r="E155" t="str">
-        <v>Albuquerque, NM</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F155">
-        <v>2200</v>
+        <v>17</v>
       </c>
       <c r="G155" t="str">
-        <v>$20/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H155" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/7996578003</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Design-and-Process-Engineering-Co-Op_REQ-14491</v>
       </c>
       <c r="I155" t="str">
-        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season/pay confirmed in body.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J155" t="str">
-        <v>Materials/manufacturing-process R&amp;D on phase-change materials for solar arrays (constellation programs).</v>
+        <v>REQ-14491. Bedford, MA sibling req.</v>
       </c>
       <c r="K155" t="str">
         <v>Open resume</v>
@@ -6760,10 +6760,10 @@
         <v>Entegris</v>
       </c>
       <c r="B156" t="str">
-        <v>Manufacturing Engineer Co-Op</v>
+        <v>Industrial Engineering Co-Op</v>
       </c>
       <c r="C156" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Industrial Engineering</v>
       </c>
       <c r="D156" t="str">
         <v>Spring 2027 season (6-month assignment)</v>
@@ -6778,13 +6778,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H156" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Manufacturing-Engineer-Co-Op_REQ-14484</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14465</v>
       </c>
       <c r="I156" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 13 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J156" t="str">
-        <v>REQ-14484. New Entegris site for the tracker (Bedford, in addition to the 7 already-tracked Billerica reqs).</v>
+        <v>REQ-14465. Bedford, MA sibling req; a second, distinct Industrial Engineering Co-Op req (REQ-14452) was also found open at the same site — see next row.</v>
       </c>
       <c r="K156" t="str">
         <v>Open resume</v>
@@ -6801,10 +6801,10 @@
         <v>Entegris</v>
       </c>
       <c r="B157" t="str">
-        <v>Design and Process Engineering Co-Op</v>
+        <v>Industrial Engineering Co-Op</v>
       </c>
       <c r="C157" t="str">
-        <v>Mechanical / Process Engineering</v>
+        <v>Industrial Engineering</v>
       </c>
       <c r="D157" t="str">
         <v>Spring 2027 season (6-month assignment)</v>
@@ -6819,13 +6819,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H157" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Design-and-Process-Engineering-Co-Op_REQ-14491</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14452</v>
       </c>
       <c r="I157" t="str">
         <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J157" t="str">
-        <v>REQ-14491. Bedford, MA sibling req.</v>
+        <v>REQ-14452. Distinct req from the identically-titled REQ-14465 above (same site/title, separate req IDs) — both independently confirmed open, not a duplicate.</v>
       </c>
       <c r="K157" t="str">
         <v>Open resume</v>
@@ -6842,10 +6842,10 @@
         <v>Entegris</v>
       </c>
       <c r="B158" t="str">
-        <v>Industrial Engineering Co-Op</v>
+        <v>Process Engineering Co-Op</v>
       </c>
       <c r="C158" t="str">
-        <v>Industrial Engineering</v>
+        <v>Process / Manufacturing Engineering</v>
       </c>
       <c r="D158" t="str">
         <v>Spring 2027 season (6-month assignment)</v>
@@ -6860,13 +6860,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H158" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14465</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Process-Engineering-Co-Op_REQ-14458</v>
       </c>
       <c r="I158" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J158" t="str">
-        <v>REQ-14465. Bedford, MA sibling req; a second, distinct Industrial Engineering Co-Op req (REQ-14452) was also found open at the same site — see next row.</v>
+        <v>REQ-14458. Bedford, MA sibling req.</v>
       </c>
       <c r="K158" t="str">
         <v>Open resume</v>
@@ -6883,10 +6883,10 @@
         <v>Entegris</v>
       </c>
       <c r="B159" t="str">
-        <v>Industrial Engineering Co-Op</v>
+        <v>Reliability Engineer Co-Op</v>
       </c>
       <c r="C159" t="str">
-        <v>Industrial Engineering</v>
+        <v>Reliability / Mechanical Engineering</v>
       </c>
       <c r="D159" t="str">
         <v>Spring 2027 season (6-month assignment)</v>
@@ -6901,13 +6901,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H159" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Industrial-Engineering-Co-Op_REQ-14452</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Reliability-Engineer-Co-Op_REQ-14399</v>
       </c>
       <c r="I159" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 15 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
       </c>
       <c r="J159" t="str">
-        <v>REQ-14452. Distinct req from the identically-titled REQ-14465 above (same site/title, separate req IDs) — both independently confirmed open, not a duplicate.</v>
+        <v>REQ-14399. Bedford, MA sibling req.</v>
       </c>
       <c r="K159" t="str">
         <v>Open resume</v>
@@ -6921,34 +6921,34 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Entegris</v>
+        <v>MetOx International</v>
       </c>
       <c r="B160" t="str">
-        <v>Process Engineering Co-Op</v>
+        <v>Mechanical Engineering Co-Op/Intern</v>
       </c>
       <c r="C160" t="str">
-        <v>Process / Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D160" t="str">
-        <v>Spring 2027 season (6-month assignment)</v>
+        <v>Spring/Summer 2027 (Internship: part-time Spring 2027 + full-time Summer 2027) or Co-Op: full-time January-August 2027</v>
       </c>
       <c r="E160" t="str">
-        <v>Bedford, MA</v>
+        <v>Houston, TX</v>
       </c>
       <c r="F160">
-        <v>17</v>
+        <v>1600</v>
       </c>
       <c r="G160" t="str">
-        <v>$20-$30/hour</v>
+        <v>Not stated on posting (non-local co-op candidates eligible for a monthly stipend)</v>
       </c>
       <c r="H160" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Process-Engineering-Co-Op_REQ-14458</v>
+        <v>https://job-boards.greenhouse.io/metoxinternationalinc/jobs/5405775008</v>
       </c>
       <c r="I160" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+        <v>Yes — fetched directly via Greenhouse (HTTP 200), full description confirms title, season options, and an active Apply button.</v>
       </c>
       <c r="J160" t="str">
-        <v>REQ-14458. Bedford, MA sibling req.</v>
+        <v>New company for the tracker — superconducting-technology energy startup. SolidWorks/FEA/CFD-focused mechanical design role, Balance-of-Plant systems. Co-Op option begins January 2027 (Spring start), included per the same 'distinct dated Spring option within a combined-term posting' treatment as Hermeus.</v>
       </c>
       <c r="K160" t="str">
         <v>Open resume</v>
@@ -6962,34 +6962,34 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Entegris</v>
+        <v>Sanofi</v>
       </c>
       <c r="B161" t="str">
-        <v>Reliability Engineer Co-Op</v>
+        <v>2027 Spring Co-op Opportunities (incl. Engineering &amp; Maintenance / HSE / Reliability tracks)</v>
       </c>
       <c r="C161" t="str">
-        <v>Reliability / Mechanical Engineering</v>
+        <v>Mechanical / Industrial / Reliability / Process Engineering (umbrella posting, multiple functional tracks)</v>
       </c>
       <c r="D161" t="str">
-        <v>Spring 2027 season (6-month assignment)</v>
+        <v>Spring 2027, starting January 2027, 6-month duration</v>
       </c>
       <c r="E161" t="str">
-        <v>Bedford, MA</v>
+        <v>Swiftwater, PA</v>
       </c>
       <c r="F161">
-        <v>17</v>
+        <v>270</v>
       </c>
       <c r="G161" t="str">
-        <v>$20-$30/hour</v>
+        <v>$32-$35/hour</v>
       </c>
       <c r="H161" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Reliability-Engineer-Co-Op_REQ-14399</v>
+        <v>https://jobs.sanofi.com/en/job/swiftwater/2027-spring-co-op-opportunities-swiftwater-pa/2649/41259827904</v>
       </c>
       <c r="I161" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (canApply true, posted 14 days ago); posting text states 'Spring 2027 season', pay confirmed in body.</v>
+        <v>Yes — fetched directly via jobs.sanofi.com (Sanofi's own site, not an aggregator), confirmed live with an active 'Apply Now' button, pay and dates confirmed in body.</v>
       </c>
       <c r="J161" t="str">
-        <v>REQ-14399. Bedford, MA sibling req.</v>
+        <v>Umbrella-style posting, same pattern as the already-tracked Sanofi/Genzyme Framingham row — multiple near-identical parallel req IDs found on job-board mirrors (biospace.com job 3075194 'Engineering &amp; Maintenance' track at $35/hr, plus others at 3075170/3062903/3069311) likely representing different functional tracks of the same 2027 Spring Co-op program. Requires permanent US work authorization without sponsorship. Distinct from the already-tracked Sanofi (Genzyme) Framingham, MA row.</v>
       </c>
       <c r="K161" t="str">
         <v>Open resume</v>
@@ -7003,34 +7003,34 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>MetOx International</v>
+        <v>Marathon Petroleum</v>
       </c>
       <c r="B162" t="str">
-        <v>Mechanical Engineering Co-Op/Intern</v>
+        <v>Intern/Co-op - Midstream Logistics and Storage Mechanical/Civil/Electrical Engineering (Spring 2027)</v>
       </c>
       <c r="C162" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Civil / Electrical Engineering</v>
       </c>
       <c r="D162" t="str">
-        <v>Spring/Summer 2027 (Internship: part-time Spring 2027 + full-time Summer 2027) or Co-Op: full-time January-August 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E162" t="str">
-        <v>Houston, TX</v>
+        <v>Findlay, OH (+ Indianapolis, IN; La Palma, CA; Salt Lake City, UT)</v>
       </c>
       <c r="F162">
-        <v>1600</v>
+        <v>700</v>
       </c>
       <c r="G162" t="str">
-        <v>Not stated on posting (non-local co-op candidates eligible for a monthly stipend)</v>
+        <v>$33.54-$42.45/hour</v>
       </c>
       <c r="H162" t="str">
-        <v>https://job-boards.greenhouse.io/metoxinternationalinc/jobs/5405775008</v>
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Findlay-Ohio/Intern-Co-op---Midstream-Logistics-and-Storage-Mechanical-Civil-Electrical-Engineering--Spring-2027-_00024207</v>
       </c>
       <c r="I162" t="str">
-        <v>Yes — fetched directly via Greenhouse (HTTP 200), full description confirms title, season options, and an active Apply button.</v>
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024207, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
       </c>
       <c r="J162" t="str">
-        <v>New company for the tracker — superconducting-technology energy startup. SolidWorks/FEA/CFD-focused mechanical design role, Balance-of-Plant systems. Co-Op option begins January 2027 (Spring start), included per the same 'distinct dated Spring option within a combined-term posting' treatment as Hermeus.</v>
+        <v>New sibling req beyond the already-tracked Refining Mechanical Engineer (Spring 2027) req 00020137 at the same Findlay, OH site — this one covers the Logistics &amp; Storage organization (pipelines/marine transport).</v>
       </c>
       <c r="K162" t="str">
         <v>Open resume</v>
@@ -7044,34 +7044,34 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Sanofi</v>
+        <v>Marathon Petroleum</v>
       </c>
       <c r="B163" t="str">
-        <v>2027 Spring Co-op Opportunities (incl. Engineering &amp; Maintenance / HSE / Reliability tracks)</v>
+        <v>Intern/Co-op - Midstream Natural Gas and NGL Services Chemical/Mechanical/Civil/Petroleum/Electrical Engineering (Spring 2027)</v>
       </c>
       <c r="C163" t="str">
-        <v>Mechanical / Industrial / Reliability / Process Engineering (umbrella posting, multiple functional tracks)</v>
+        <v>Mechanical / Chemical / Civil / Petroleum / Electrical Engineering</v>
       </c>
       <c r="D163" t="str">
-        <v>Spring 2027, starting January 2027, 6-month duration</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E163" t="str">
-        <v>Swiftwater, PA</v>
+        <v>Canonsburg, PA (+ 12 other locations incl. Denver CO, Houston TX, Midland TX, Oklahoma City OK, Tulsa OK)</v>
       </c>
       <c r="F163">
-        <v>270</v>
+        <v>430</v>
       </c>
       <c r="G163" t="str">
-        <v>$32-$35/hour</v>
+        <v>$33.54-$43.23/hour</v>
       </c>
       <c r="H163" t="str">
-        <v>https://jobs.sanofi.com/en/job/swiftwater/2027-spring-co-op-opportunities-swiftwater-pa/2649/41259827904</v>
+        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Canonsburg-Pennsylvania/Intern-Co-op---Midstream-Natural-Gas-and-NGL-Services-Chemical-Mechanical-Civil-Petroleum-Electrical-Engineering--Spring-2027-_00024213</v>
       </c>
       <c r="I163" t="str">
-        <v>Yes — fetched directly via jobs.sanofi.com (Sanofi's own site, not an aggregator), confirmed live with an active 'Apply Now' button, pay and dates confirmed in body.</v>
+        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024213, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
       </c>
       <c r="J163" t="str">
-        <v>Umbrella-style posting, same pattern as the already-tracked Sanofi/Genzyme Framingham row — multiple near-identical parallel req IDs found on job-board mirrors (biospace.com job 3075194 'Engineering &amp; Maintenance' track at $35/hr, plus others at 3075170/3062903/3069311) likely representing different functional tracks of the same 2027 Spring Co-op program. Requires permanent US work authorization without sponsorship. Distinct from the already-tracked Sanofi (Genzyme) Framingham, MA row.</v>
+        <v>New sibling req beyond the already-tracked Marathon Petroleum entries — covers Natural Gas &amp; NGL Services (pipeline integrity, compressor/pump stations, automation/controls).</v>
       </c>
       <c r="K163" t="str">
         <v>Open resume</v>
@@ -7085,34 +7085,34 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Marathon Petroleum</v>
+        <v>Rendezvous Robotics</v>
       </c>
       <c r="B164" t="str">
-        <v>Intern/Co-op - Midstream Logistics and Storage Mechanical/Civil/Electrical Engineering (Spring 2027)</v>
+        <v>Mechanical Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C164" t="str">
-        <v>Mechanical / Civil / Electrical Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D164" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (12-15 weeks)</v>
       </c>
       <c r="E164" t="str">
-        <v>Findlay, OH (+ Indianapolis, IN; La Palma, CA; Salt Lake City, UT)</v>
+        <v>Golden, CO</v>
       </c>
       <c r="F164">
-        <v>700</v>
+        <v>1780</v>
       </c>
       <c r="G164" t="str">
-        <v>$33.54-$42.45/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H164" t="str">
-        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Findlay-Ohio/Intern-Co-op---Midstream-Logistics-and-Storage-Mechanical-Civil-Electrical-Engineering--Spring-2027-_00024207</v>
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4329123009</v>
       </c>
       <c r="I164" t="str">
-        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024207, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
+        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
       </c>
       <c r="J164" t="str">
-        <v>New sibling req beyond the already-tracked Refining Mechanical Engineer (Spring 2027) req 00020137 at the same Findlay, OH site — this one covers the Logistics &amp; Storage organization (pipelines/marine transport).</v>
+        <v>New company for the tracker — small spacecraft-assembly startup (electromagnetic self-assembling tiles). First published 2026-07-22; still listed live on the board as of this run despite being ~2 months old.</v>
       </c>
       <c r="K164" t="str">
         <v>Open resume</v>
@@ -7126,34 +7126,34 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Marathon Petroleum</v>
+        <v>Rendezvous Robotics</v>
       </c>
       <c r="B165" t="str">
-        <v>Intern/Co-op - Midstream Natural Gas and NGL Services Chemical/Mechanical/Civil/Petroleum/Electrical Engineering (Spring 2027)</v>
+        <v>GNC Intern (Spring 2027)</v>
       </c>
       <c r="C165" t="str">
-        <v>Mechanical / Chemical / Civil / Petroleum / Electrical Engineering</v>
+        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
       </c>
       <c r="D165" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (12-15 weeks)</v>
       </c>
       <c r="E165" t="str">
-        <v>Canonsburg, PA (+ 12 other locations incl. Denver CO, Houston TX, Midland TX, Oklahoma City OK, Tulsa OK)</v>
+        <v>Golden, CO</v>
       </c>
       <c r="F165">
-        <v>430</v>
+        <v>1780</v>
       </c>
       <c r="G165" t="str">
-        <v>$33.54-$43.23/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H165" t="str">
-        <v>https://mpc.wd1.myworkdayjobs.com/en-US/MPCCareers/job/Canonsburg-Pennsylvania/Intern-Co-op---Midstream-Natural-Gas-and-NGL-Services-Chemical-Mechanical-Civil-Petroleum-Electrical-Engineering--Spring-2027-_00024213</v>
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332465009</v>
       </c>
       <c r="I165" t="str">
-        <v>Yes — fetched directly via Marathon Petroleum's own Workday CXS API (HTTP 200 JSON), req 00024213, canApply true, posted today, title states 'Spring 2027', pay range confirmed in body.</v>
+        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
       </c>
       <c r="J165" t="str">
-        <v>New sibling req beyond the already-tracked Marathon Petroleum entries — covers Natural Gas &amp; NGL Services (pipeline integrity, compressor/pump stations, automation/controls).</v>
+        <v>Dynamics/controls of a reconfigurable spacecraft assembled from electromagnetically-docked tiles; open to aerospace/mechanical/electrical/physics majors with coursework in dynamics and controls — squarely a controls/flight-systems role, same treatment as the already-tracked Hermeus GNC intern.</v>
       </c>
       <c r="K165" t="str">
         <v>Open resume</v>
@@ -7170,13 +7170,13 @@
         <v>Rendezvous Robotics</v>
       </c>
       <c r="B166" t="str">
-        <v>Mechanical Engineering Intern (Spring 2027)</v>
+        <v>Manufacturing and Test Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C166" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D166" t="str">
-        <v>Spring 2027 (12-15 weeks)</v>
+        <v>Spring 2027 (per Greenhouse job title; the body text itself only states 'Golden, CO | Full-Time | 12-15 Weeks' with no season restated)</v>
       </c>
       <c r="E166" t="str">
         <v>Golden, CO</v>
@@ -7188,13 +7188,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H166" t="str">
-        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4329123009</v>
+        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332082009</v>
       </c>
       <c r="I166" t="str">
-        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
+        <v>Partial — fetched directly via Greenhouse's own public API (HTTP 200 JSON); the official posting title is 'Manufacturing and Test Engineering Intern (Spring 2027)' but, unlike its 3 sibling Rendezvous Robotics postings, the job description body never restates 'Spring 2027' anywhere — season confirmation rests on the title alone.</v>
       </c>
       <c r="J166" t="str">
-        <v>New company for the tracker — small spacecraft-assembly startup (electromagnetic self-assembling tiles). First published 2026-07-22; still listed live on the board as of this run despite being ~2 months old.</v>
+        <v>Open to Mechanical/Electrical/Industrial Engineering majors; testbed development, manufacturing support, and hardware verification for spacecraft tiles.</v>
       </c>
       <c r="K166" t="str">
         <v>Open resume</v>
@@ -7208,34 +7208,34 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>Rendezvous Robotics</v>
+        <v>Vast Space</v>
       </c>
       <c r="B167" t="str">
-        <v>GNC Intern (Spring 2027)</v>
+        <v>Emerging Talent - Mechanical/Aerospace Engineering Internship</v>
       </c>
       <c r="C167" t="str">
-        <v>Flight Systems / Guidance, Navigation &amp; Controls</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D167" t="str">
-        <v>Spring 2027 (12-15 weeks)</v>
+        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
       </c>
       <c r="E167" t="str">
-        <v>Golden, CO</v>
+        <v>Long Beach, CA (also hiring for Hawthorne, CA and Mojave, CA)</v>
       </c>
       <c r="F167">
-        <v>1780</v>
+        <v>2600</v>
       </c>
       <c r="G167" t="str">
-        <v>Not stated on posting</v>
+        <v>$35-$42/hour</v>
       </c>
       <c r="H167" t="str">
-        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332465009</v>
+        <v>https://job-boards.greenhouse.io/vast/jobs/4711400006</v>
       </c>
       <c r="I167" t="str">
-        <v>Yes — fetched directly via Greenhouse's own public API (HTTP 200 JSON), body states 'Golden, CO | Full-Time | 12-15 Weeks | Spring 2027' verbatim.</v>
+        <v>Yes — fetched directly on Greenhouse; the application form's 'When are you available for an internship?' field is a dropdown containing 'Spring 2027' as its own distinct option (plus 'Summer: May 18 - Aug 6, 2027' / 'May 25 - Aug 13' / 'June 8 - Aug 27' / 'June 22 - Sept 10' and 'Fall 2027') — confirmed via the page's raw JSON, not just rendered text.</v>
       </c>
       <c r="J167" t="str">
-        <v>Dynamics/controls of a reconfigurable spacecraft assembled from electromagnetically-docked tiles; open to aerospace/mechanical/electrical/physics majors with coursework in dynamics and controls — squarely a controls/flight-systems role, same treatment as the already-tracked Hermeus GNC intern.</v>
+        <v>Previously excluded in 3 prior runs (2026-09-23) because the posting had no season/term field at all — this session's direct re-fetch found the application form now includes a genuine dated Spring 2027 option, same 'distinct dated Spring slot within a combined-term posting' treatment as Hermeus. ITAR: US person status required.</v>
       </c>
       <c r="K167" t="str">
         <v>Open resume</v>
@@ -7249,34 +7249,34 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Rendezvous Robotics</v>
+        <v>Vast Space</v>
       </c>
       <c r="B168" t="str">
-        <v>Manufacturing and Test Engineering Intern (Spring 2027)</v>
+        <v>Emerging Talent - Manufacturing Engineering Internship</v>
       </c>
       <c r="C168" t="str">
         <v>Manufacturing Engineering</v>
       </c>
       <c r="D168" t="str">
-        <v>Spring 2027 (per Greenhouse job title; the body text itself only states 'Golden, CO | Full-Time | 12-15 Weeks' with no season restated)</v>
+        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
       </c>
       <c r="E168" t="str">
-        <v>Golden, CO</v>
+        <v>Long Beach, CA (also hiring for Hawthorne, CA)</v>
       </c>
       <c r="F168">
-        <v>1780</v>
+        <v>2600</v>
       </c>
       <c r="G168" t="str">
-        <v>Not stated on posting</v>
+        <v>$35-$42/hour</v>
       </c>
       <c r="H168" t="str">
-        <v>https://job-boards.greenhouse.io/rendezvousrobotics/jobs/4332082009</v>
+        <v>https://job-boards.greenhouse.io/vast/jobs/4711403006</v>
       </c>
       <c r="I168" t="str">
-        <v>Partial — fetched directly via Greenhouse's own public API (HTTP 200 JSON); the official posting title is 'Manufacturing and Test Engineering Intern (Spring 2027)' but, unlike its 3 sibling Rendezvous Robotics postings, the job description body never restates 'Spring 2027' anywhere — season confirmation rests on the title alone.</v>
+        <v>Yes — fetched directly on Greenhouse; same 'When are you available for an internship?' dropdown with a distinct 'Spring 2027' option confirmed via the page's raw JSON, alongside the same 4 dated Summer 2027 ranges and Fall 2027.</v>
       </c>
       <c r="J168" t="str">
-        <v>Open to Mechanical/Electrical/Industrial Engineering majors; testbed development, manufacturing support, and hardware verification for spacecraft tiles.</v>
+        <v>Sibling req to the Mechanical/Aerospace Engineering Internship above, same site/pay/season structure.</v>
       </c>
       <c r="K168" t="str">
         <v>Open resume</v>
@@ -7290,34 +7290,34 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Vast Space</v>
+        <v>Moog Inc.</v>
       </c>
       <c r="B169" t="str">
-        <v>Emerging Talent - Mechanical/Aerospace Engineering Internship</v>
+        <v>Intern, Design Engineering</v>
       </c>
       <c r="C169" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Mechanical / Aerospace Engineering (Air Vehicle Engineering)</v>
       </c>
       <c r="D169" t="str">
-        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
+        <v>Spring 2027 block intern</v>
       </c>
       <c r="E169" t="str">
-        <v>Long Beach, CA (also hiring for Hawthorne, CA and Mojave, CA)</v>
+        <v>Mineral Wells, TX</v>
       </c>
       <c r="F169">
-        <v>2600</v>
+        <v>1750</v>
       </c>
       <c r="G169" t="str">
-        <v>$35-$42/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H169" t="str">
-        <v>https://job-boards.greenhouse.io/vast/jobs/4711400006</v>
+        <v>https://moog.wd5.myworkdayjobs.com/en-US/MOOG_External_Career_Site/job/Mineral-Wells-TX/Intern--Design-Engineering_R-26-19186</v>
       </c>
       <c r="I169" t="str">
-        <v>Yes — fetched directly on Greenhouse; the application form's 'When are you available for an internship?' field is a dropdown containing 'Spring 2027' as its own distinct option (plus 'Summer: May 18 - Aug 6, 2027' / 'May 25 - Aug 13' / 'June 8 - Aug 27' / 'June 22 - Sept 10' and 'Fall 2027') — confirmed via the page's raw JSON, not just rendered text.</v>
+        <v>Yes — fetched directly via Moog's own Workday CXS API (HTTP 200 JSON), req R-26-19186, canApply true, posted 21 days ago, body states 'seeking a spring 2027 block intern' verbatim.</v>
       </c>
       <c r="J169" t="str">
-        <v>Previously excluded in 3 prior runs (2026-09-23) because the posting had no season/term field at all — this session's direct re-fetch found the application form now includes a genuine dated Spring 2027 option, same 'distinct dated Spring slot within a combined-term posting' treatment as Hermeus. ITAR: US person status required.</v>
+        <v>Corrects an earlier (2026-09-22) `checked` entry that had lumped this req in with 3 Summer-2027 Mineral Wells siblings (R-26-19881/19882/19887, which remain correctly excluded) — this session's fresh direct fetch shows R-26-19186 now/actually states Spring 2027, a different season from those siblings.</v>
       </c>
       <c r="K169" t="str">
         <v>Open resume</v>
@@ -7331,34 +7331,34 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>Vast Space</v>
+        <v>Entegris</v>
       </c>
       <c r="B170" t="str">
-        <v>Emerging Talent - Manufacturing Engineering Internship</v>
+        <v>Application Engineering Co-Op</v>
       </c>
       <c r="C170" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Applications / Process Engineering (Photo Applications)</v>
       </c>
       <c r="D170" t="str">
-        <v>Spring 2027 (distinct option in the application's start-term dropdown, alongside 4 dated Summer 2027 ranges and Fall 2027)</v>
+        <v>Spring 2027 season</v>
       </c>
       <c r="E170" t="str">
-        <v>Long Beach, CA (also hiring for Hawthorne, CA)</v>
+        <v>Billerica, MA</v>
       </c>
       <c r="F170">
-        <v>2600</v>
+        <v>17</v>
       </c>
       <c r="G170" t="str">
-        <v>$35-$42/hour</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H170" t="str">
-        <v>https://job-boards.greenhouse.io/vast/jobs/4711403006</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Application-Engineering-Co-Op_REQ-14473</v>
       </c>
       <c r="I170" t="str">
-        <v>Yes — fetched directly on Greenhouse; same 'When are you available for an internship?' dropdown with a distinct 'Spring 2027' option confirmed via the page's raw JSON, alongside the same 4 dated Summer 2027 ranges and Fall 2027.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14473, canApply true, posted 15 days ago, body states 'Spring 2027' twice ('Spring 2027 to join our team' / 'Photo Applications team for the Spring 2027 season').</v>
       </c>
       <c r="J170" t="str">
-        <v>Sibling req to the Mechanical/Aerospace Engineering Internship above, same site/pay/season structure.</v>
+        <v>New sibling req beyond the 13 already-tracked Entegris Billerica/Bedford reqs, found via this session's own Entegris jobs-search API sweep (not from either research agent, who both mis-transcribed nearby req numbers — see ROUTINE-LOG for the correction).</v>
       </c>
       <c r="K170" t="str">
         <v>Open resume</v>
@@ -7372,116 +7372,98 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>Moog Inc.</v>
+        <v>Rocket Lab</v>
       </c>
       <c r="B171" t="str">
-        <v>Intern, Design Engineering</v>
+        <v>Test Engineering Intern, Spring 2027</v>
       </c>
       <c r="C171" t="str">
-        <v>Mechanical / Aerospace Engineering (Air Vehicle Engineering)</v>
+        <v>Systems / Test Engineering</v>
       </c>
       <c r="D171" t="str">
-        <v>Spring 2027 block intern</v>
+        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
       </c>
       <c r="E171" t="str">
-        <v>Mineral Wells, TX</v>
+        <v>Wallops Island, VA</v>
       </c>
       <c r="F171">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="G171" t="str">
-        <v>Not stated on posting</v>
+        <v>$25/hr (VA base pay range)</v>
       </c>
       <c r="H171" t="str">
-        <v>https://moog.wd5.myworkdayjobs.com/en-US/MOOG_External_Career_Site/job/Mineral-Wells-TX/Intern--Design-Engineering_R-26-19186</v>
+        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8003533003</v>
       </c>
       <c r="I171" t="str">
-        <v>Yes — fetched directly via Moog's own Workday CXS API (HTTP 200 JSON), req R-26-19186, canApply true, posted 21 days ago, body states 'seeking a spring 2027 block intern' verbatim.</v>
+        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season and VA pay range confirmed in body.</v>
       </c>
       <c r="J171" t="str">
-        <v>Corrects an earlier (2026-09-22) `checked` entry that had lumped this req in with 3 Summer-2027 Mineral Wells siblings (R-26-19881/19882/19887, which remain correctly excluded) — this session's fresh direct fetch shows R-26-19186 now/actually states Spring 2027, a different season from those siblings.</v>
-      </c>
-      <c r="K171" t="str">
-        <v>Open resume</v>
-      </c>
-      <c r="L171" t="str">
-        <v>Open cover letter</v>
-      </c>
-      <c r="M171" t="str">
-        <v>Open questions</v>
+        <v>New site distinct from the already-tracked Stennis Space Center, MS 'Test Engineering Intern' (job 7990352003) — same title, different req/location.</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>Entegris</v>
+        <v>Formlabs</v>
       </c>
       <c r="B172" t="str">
-        <v>Application Engineering Co-Op</v>
+        <v>Hardware Test Engineering Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C172" t="str">
-        <v>Applications / Process Engineering (Photo Applications)</v>
+        <v>Mechanical / Hardware Test Engineering</v>
       </c>
       <c r="D172" t="str">
-        <v>Spring 2027 season</v>
+        <v>Winter/Spring 2027 (January - April)</v>
       </c>
       <c r="E172" t="str">
-        <v>Billerica, MA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F172">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="G172" t="str">
-        <v>$20-$30/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H172" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Billerica-MA/Application-Engineering-Co-Op_REQ-14473</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8196515</v>
       </c>
       <c r="I172" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14473, canApply true, posted 15 days ago, body states 'Spring 2027' twice ('Spring 2027 to join our team' / 'Photo Applications team for the Spring 2027 season').</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Internship Term: Winter/Spring (January - April)' confirmed in body, title states 2027.</v>
       </c>
       <c r="J172" t="str">
-        <v>New sibling req beyond the 13 already-tracked Entegris Billerica/Bedford reqs, found via this session's own Entegris jobs-search API sweep (not from either research agent, who both mis-transcribed nearby req numbers — see ROUTINE-LOG for the correction).</v>
-      </c>
-      <c r="K172" t="str">
-        <v>Open resume</v>
-      </c>
-      <c r="L172" t="str">
-        <v>Open cover letter</v>
-      </c>
-      <c r="M172" t="str">
-        <v>Open questions</v>
+        <v>New sibling req beyond the already-tracked Formlabs Mechanical/Manufacturing/Hardware R&amp;D/Materials interns.</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>Rocket Lab</v>
+        <v>Formlabs</v>
       </c>
       <c r="B173" t="str">
-        <v>Test Engineering Intern, Spring 2027</v>
+        <v>Print Optimization Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C173" t="str">
-        <v>Systems / Test Engineering</v>
+        <v>Manufacturing / Process Engineering</v>
       </c>
       <c r="D173" t="str">
-        <v>Spring 2027 (12+ consecutive weeks beginning Jan/Feb/Mar 2027)</v>
+        <v>Winter/Spring 2027 (January - April)</v>
       </c>
       <c r="E173" t="str">
-        <v>Wallops Island, VA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F173">
-        <v>350</v>
+        <v>3</v>
       </c>
       <c r="G173" t="str">
-        <v>$25/hr (VA base pay range)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H173" t="str">
-        <v>https://job-boards.greenhouse.io/rocketlab/jobs/8003533003</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172256</v>
       </c>
       <c r="I173" t="str">
-        <v>Yes — fetched directly via Rocket Lab's own Greenhouse API, HTTP 200, season and VA pay range confirmed in body.</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title and 'January - April' term confirmed in body.</v>
       </c>
       <c r="J173" t="str">
-        <v>New site distinct from the already-tracked Stennis Space Center, MS 'Test Engineering Intern' (job 7990352003) — same title, different req/location.</v>
+        <v>New sibling req; 3D-printing process/optimization work, manufacturing-adjacent.</v>
       </c>
     </row>
     <row r="174">
@@ -7489,10 +7471,10 @@
         <v>Formlabs</v>
       </c>
       <c r="B174" t="str">
-        <v>Hardware Test Engineering Intern (Winter/Spring 2027)</v>
+        <v>Print Process Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C174" t="str">
-        <v>Mechanical / Hardware Test Engineering</v>
+        <v>Manufacturing / Process Engineering</v>
       </c>
       <c r="D174" t="str">
         <v>Winter/Spring 2027 (January - April)</v>
@@ -7507,138 +7489,138 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H174" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8196515</v>
+        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199269</v>
       </c>
       <c r="I174" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Internship Term: Winter/Spring (January - April)' confirmed in body, title states 2027.</v>
+        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title confirmed in body.</v>
       </c>
       <c r="J174" t="str">
-        <v>New sibling req beyond the already-tracked Formlabs Mechanical/Manufacturing/Hardware R&amp;D/Materials interns.</v>
+        <v>New sibling req; 3D-printing process work, manufacturing-adjacent.</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>Formlabs</v>
+        <v>Hermeus</v>
       </c>
       <c r="B175" t="str">
-        <v>Print Optimization Intern (Winter/Spring 2027)</v>
+        <v>Subsystem Test Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C175" t="str">
-        <v>Manufacturing / Process Engineering</v>
+        <v>Test Engineering</v>
       </c>
       <c r="D175" t="str">
-        <v>Winter/Spring 2027 (January - April)</v>
+        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
       </c>
       <c r="E175" t="str">
-        <v>Somerville, MA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F175">
-        <v>3</v>
+        <v>950</v>
       </c>
       <c r="G175" t="str">
-        <v>Not stated on posting</v>
+        <v>$25-$33/hr</v>
       </c>
       <c r="H175" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8172256</v>
+        <v>https://jobs.lever.co/hermeus/643fd7b7-9015-43a1-aa2b-a54f117b403c</v>
       </c>
       <c r="I175" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title and 'January - April' term confirmed in body.</v>
+        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option, same treatment as other already-tracked Hermeus combined-term reqs.</v>
       </c>
       <c r="J175" t="str">
-        <v>New sibling req; 3D-printing process/optimization work, manufacturing-adjacent.</v>
+        <v>New sibling req; also listed at Los Angeles, CA per allLocations.</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Formlabs</v>
+        <v>Hermeus</v>
       </c>
       <c r="B176" t="str">
-        <v>Print Process Intern (Winter/Spring 2027)</v>
+        <v>Test and Operations Engineering Intern (Spring/Summer 2027)</v>
       </c>
       <c r="C176" t="str">
-        <v>Manufacturing / Process Engineering</v>
+        <v>Test / Operations Engineering</v>
       </c>
       <c r="D176" t="str">
-        <v>Winter/Spring 2027 (January - April)</v>
+        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
       </c>
       <c r="E176" t="str">
-        <v>Somerville, MA</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F176">
-        <v>3</v>
+        <v>2600</v>
       </c>
       <c r="G176" t="str">
-        <v>Not stated on posting</v>
+        <v>$25-$33/hr</v>
       </c>
       <c r="H176" t="str">
-        <v>https://job-boards.greenhouse.io/formlabs/jobs/8199269</v>
+        <v>https://jobs.lever.co/hermeus/d40446ee-40a9-4bb0-a3a8-a4a189b74630</v>
       </c>
       <c r="I176" t="str">
-        <v>Yes — fetched directly via Formlabs's own Greenhouse API, HTTP 200, 'Winter/Spring 2027' title confirmed in body.</v>
+        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option.</v>
       </c>
       <c r="J176" t="str">
-        <v>New sibling req; 3D-printing process work, manufacturing-adjacent.</v>
+        <v>New sibling req.</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>Hermeus</v>
+        <v>Entegris</v>
       </c>
       <c r="B177" t="str">
-        <v>Subsystem Test Engineering Intern (Spring/Summer 2027)</v>
+        <v>Specialty Coatings Research and Development Co-Op</v>
       </c>
       <c r="C177" t="str">
-        <v>Test Engineering</v>
+        <v>Materials / Coatings Engineering</v>
       </c>
       <c r="D177" t="str">
-        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
+        <v>Spring 2027 season</v>
       </c>
       <c r="E177" t="str">
-        <v>Atlanta, GA</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F177">
-        <v>950</v>
+        <v>16</v>
       </c>
       <c r="G177" t="str">
-        <v>$25-$33/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H177" t="str">
-        <v>https://jobs.lever.co/hermeus/643fd7b7-9015-43a1-aa2b-a54f117b403c</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Entegris-Specialty-Coatings-Research-and-Development-Co-Op_REQ-14441</v>
       </c>
       <c r="I177" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option, same treatment as other already-tracked Hermeus combined-term reqs.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14441, canApply true, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J177" t="str">
-        <v>New sibling req; also listed at Los Angeles, CA per allLocations.</v>
+        <v>New sibling req beyond the already-tracked 14 Entegris Billerica/Bedford reqs.</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>Hermeus</v>
+        <v>Entegris</v>
       </c>
       <c r="B178" t="str">
-        <v>Test and Operations Engineering Intern (Spring/Summer 2027)</v>
+        <v>New Product Introduction Co-Op</v>
       </c>
       <c r="C178" t="str">
-        <v>Test / Operations Engineering</v>
+        <v>Manufacturing / NPI Engineering</v>
       </c>
       <c r="D178" t="str">
-        <v>Spring/Summer 2027 (Spring: ~16 weeks, January - April)</v>
+        <v>Spring 2027 season</v>
       </c>
       <c r="E178" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F178">
-        <v>2600</v>
+        <v>16</v>
       </c>
       <c r="G178" t="str">
-        <v>$25-$33/hr</v>
+        <v>$20-$30/hour</v>
       </c>
       <c r="H178" t="str">
-        <v>https://jobs.lever.co/hermeus/d40446ee-40a9-4bb0-a3a8-a4a189b74630</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/New-Product-Introduction-Co-Op_REQ-14461-1</v>
       </c>
       <c r="I178" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, HTTP 200, body explicitly states 'Spring: Around 16 weeks (January - April) / Summer: Around 12 weeks (May - August)' as a distinct dated option.</v>
+        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14461, canApply true, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J178" t="str">
         <v>New sibling req.</v>
@@ -7649,31 +7631,31 @@
         <v>Entegris</v>
       </c>
       <c r="B179" t="str">
-        <v>Specialty Coatings Research and Development Co-Op</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C179" t="str">
-        <v>Materials / Coatings Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D179" t="str">
-        <v>Spring 2027 season</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E179" t="str">
-        <v>Bedford, MA</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F179">
-        <v>16</v>
+        <v>885</v>
       </c>
       <c r="G179" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H179" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Entegris-Specialty-Coatings-Research-and-Development-Co-Op_REQ-14441</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering--Co-Op_REQ-14442</v>
       </c>
       <c r="I179" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14441, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J179" t="str">
-        <v>New sibling req beyond the already-tracked 14 Entegris Billerica/Bedford reqs.</v>
+        <v>REQ-14442. Industrial/Manufacturing Engineering, Industry 4.0/smart-manufacturing focus. No H1-B sponsorship. Genuinely new site for the tracker (2026-09-26 sweep found Entegris's full nationwide Co-Op slate beyond the previously MA-only-tracked reqs).</v>
       </c>
     </row>
     <row r="180">
@@ -7681,31 +7663,31 @@
         <v>Entegris</v>
       </c>
       <c r="B180" t="str">
-        <v>New Product Introduction Co-Op</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C180" t="str">
-        <v>Manufacturing / NPI Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D180" t="str">
-        <v>Spring 2027 season</v>
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E180" t="str">
-        <v>Bedford, MA</v>
+        <v>Aurora, IL</v>
       </c>
       <c r="F180">
-        <v>16</v>
+        <v>885</v>
       </c>
       <c r="G180" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H180" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/New-Product-Introduction-Co-Op_REQ-14461-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14438</v>
       </c>
       <c r="I180" t="str">
-        <v>Yes — fetched directly via Entegris's own Workday CXS API (HTTP 200 JSON), req REQ-14461, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J180" t="str">
-        <v>New sibling req.</v>
+        <v>REQ-14438. Sibling req to REQ-14442, same site. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="181">
@@ -7731,13 +7713,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H181" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering--Co-Op_REQ-14442</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14394</v>
       </c>
       <c r="I181" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J181" t="str">
-        <v>REQ-14442. Industrial/Manufacturing Engineering, Industry 4.0/smart-manufacturing focus. No H1-B sponsorship. Genuinely new site for the tracker (2026-09-26 sweep found Entegris's full nationwide Co-Op slate beyond the previously MA-only-tracked reqs).</v>
+        <v>REQ-14394. Chemical/Mechanical/Industrial/Manufacturing Engineering majors; quality engineering coursework a plus. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="182">
@@ -7763,13 +7745,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H182" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14438</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14412</v>
       </c>
       <c r="I182" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J182" t="str">
-        <v>REQ-14438. Sibling req to REQ-14442, same site. No H1-B sponsorship.</v>
+        <v>REQ-14412. Same discipline mix as REQ-14394. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="183">
@@ -7786,22 +7768,22 @@
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E183" t="str">
-        <v>Aurora, IL</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F183">
-        <v>885</v>
+        <v>1137</v>
       </c>
       <c r="G183" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H183" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14394</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14409</v>
       </c>
       <c r="I183" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J183" t="str">
-        <v>REQ-14394. Chemical/Mechanical/Industrial/Manufacturing Engineering majors; quality engineering coursework a plus. No H1-B sponsorship.</v>
+        <v>REQ-14409. Industrial/Mechanical/Manufacturing Engineering, grad 2027-2029. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="184">
@@ -7818,22 +7800,22 @@
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E184" t="str">
-        <v>Aurora, IL</v>
+        <v>Chaska, MN</v>
       </c>
       <c r="F184">
-        <v>885</v>
+        <v>1137</v>
       </c>
       <c r="G184" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H184" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Aurora-IL/Manufacturing-Engineering-Co-Op_REQ-14412</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14424</v>
       </c>
       <c r="I184" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J184" t="str">
-        <v>REQ-14412. Same discipline mix as REQ-14394. No H1-B sponsorship.</v>
+        <v>REQ-14424. Manufacturing/Industrial/Mechanical/Systems Engineering, grad 2027-2029. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="185">
@@ -7859,13 +7841,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H185" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14409</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering--Co-Op_REQ-14447-1</v>
       </c>
       <c r="I185" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J185" t="str">
-        <v>REQ-14409. Industrial/Mechanical/Manufacturing Engineering, grad 2027-2029. No H1-B sponsorship.</v>
+        <v>REQ-14447. Manufacturing/Industrial Engineering, grad Dec 2026 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="186">
@@ -7873,10 +7855,10 @@
         <v>Entegris</v>
       </c>
       <c r="B186" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Mechanical Test Engineer Co-Op</v>
       </c>
       <c r="C186" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D186" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
@@ -7891,13 +7873,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H186" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering-Co-Op_REQ-14424</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Mechanical-Test-Engineer-Co-Op_REQ-14477-1</v>
       </c>
       <c r="I186" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J186" t="str">
-        <v>REQ-14424. Manufacturing/Industrial/Mechanical/Systems Engineering, grad 2027-2029. No H1-B sponsorship.</v>
+        <v>REQ-14477. Mechanical/Industrial Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="187">
@@ -7914,22 +7896,22 @@
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E187" t="str">
-        <v>Chaska, MN</v>
+        <v>Colorado Springs (Rockrimmon), CO</v>
       </c>
       <c r="F187">
-        <v>1137</v>
+        <v>1771</v>
       </c>
       <c r="G187" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H187" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Manufacturing-Engineering--Co-Op_REQ-14447-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14508</v>
       </c>
       <c r="I187" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J187" t="str">
-        <v>REQ-14447. Manufacturing/Industrial Engineering, grad Dec 2026 or later. No H1-B sponsorship.</v>
+        <v>REQ-14508. Mechanical/Industrial/Electrical Engineering, grad 2027 or 2028. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="188">
@@ -7937,31 +7919,31 @@
         <v>Entegris</v>
       </c>
       <c r="B188" t="str">
-        <v>Mechanical Test Engineer Co-Op</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C188" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D188" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E188" t="str">
-        <v>Chaska, MN</v>
+        <v>Colorado Springs (Rockrimmon), CO</v>
       </c>
       <c r="F188">
-        <v>1137</v>
+        <v>1771</v>
       </c>
       <c r="G188" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H188" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Mechanical-Test-Engineer-Co-Op_REQ-14477-1</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14439</v>
       </c>
       <c r="I188" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J188" t="str">
-        <v>REQ-14477. Mechanical/Industrial Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
+        <v>REQ-14439. Mechanical/Industrial/Manufacturing Engineering, Junior/Senior, grad 2027 or 2028. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="189">
@@ -7969,7 +7951,7 @@
         <v>Entegris</v>
       </c>
       <c r="B189" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Manufacturing Engineer Co-Op</v>
       </c>
       <c r="C189" t="str">
         <v>Manufacturing Engineering</v>
@@ -7987,13 +7969,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H189" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14508</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineer-Co-Op_REQ-14411</v>
       </c>
       <c r="I189" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J189" t="str">
-        <v>REQ-14508. Mechanical/Industrial/Electrical Engineering, grad 2027 or 2028. No H1-B sponsorship.</v>
+        <v>REQ-14411. Mechanical/Industrial/Manufacturing Engineering, grad 2027 or Spring 2028. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="190">
@@ -8001,10 +7983,10 @@
         <v>Entegris</v>
       </c>
       <c r="B190" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Manufacturing Systems Engineer Co-Op</v>
       </c>
       <c r="C190" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Manufacturing / Industrial Engineering</v>
       </c>
       <c r="D190" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
@@ -8019,13 +8001,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H190" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineering-Co-Op_REQ-14439</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Systems-Engineer-Co-Op_REQ-14437</v>
       </c>
       <c r="I190" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J190" t="str">
-        <v>REQ-14439. Mechanical/Industrial/Manufacturing Engineering, Junior/Senior, grad 2027 or 2028. No H1-B sponsorship.</v>
+        <v>REQ-14437. Industrial/Chemical/Systems Engineering (or CS/IT) majors sought, target grad 2028; Master's students welcome. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="191">
@@ -8033,10 +8015,10 @@
         <v>Entegris</v>
       </c>
       <c r="B191" t="str">
-        <v>Manufacturing Engineer Co-Op</v>
+        <v>Process Engineering Co-Op</v>
       </c>
       <c r="C191" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Process / Manufacturing Engineering</v>
       </c>
       <c r="D191" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
@@ -8051,13 +8033,13 @@
         <v>$20-$30/hour</v>
       </c>
       <c r="H191" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Engineer-Co-Op_REQ-14411</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Process-Engineering-Co-Op_REQ-14485</v>
       </c>
       <c r="I191" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J191" t="str">
-        <v>REQ-14411. Mechanical/Industrial/Manufacturing Engineering, grad 2027 or Spring 2028. No H1-B sponsorship.</v>
+        <v>REQ-14485. Mechanical/Industrial/Chemical Engineering, grad May 2027 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="192">
@@ -8065,31 +8047,31 @@
         <v>Entegris</v>
       </c>
       <c r="B192" t="str">
-        <v>Manufacturing Systems Engineer Co-Op</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C192" t="str">
-        <v>Manufacturing / Industrial Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D192" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E192" t="str">
-        <v>Colorado Springs (Rockrimmon), CO</v>
+        <v>Bloomington, MN</v>
       </c>
       <c r="F192">
-        <v>1771</v>
+        <v>1122</v>
       </c>
       <c r="G192" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H192" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Manufacturing-Systems-Engineer-Co-Op_REQ-14437</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bloomington-MN/Manufacturing-Engineering-Co-Op_REQ-14417</v>
       </c>
       <c r="I192" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J192" t="str">
-        <v>REQ-14437. Industrial/Chemical/Systems Engineering (or CS/IT) majors sought, target grad 2028; Master's students welcome. No H1-B sponsorship.</v>
+        <v>REQ-14417. Mechanical/Manufacturing/Industrial Engineering, Spring 2027 or 2028 grad. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="193">
@@ -8097,31 +8079,31 @@
         <v>Entegris</v>
       </c>
       <c r="B193" t="str">
-        <v>Process Engineering Co-Op</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C193" t="str">
-        <v>Process / Manufacturing Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D193" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E193" t="str">
-        <v>Colorado Springs (Rockrimmon), CO</v>
+        <v>Hillsboro, OR</v>
       </c>
       <c r="F193">
-        <v>1771</v>
+        <v>2548</v>
       </c>
       <c r="G193" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H193" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Process-Engineering-Co-Op_REQ-14485</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14480</v>
       </c>
       <c r="I193" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
       </c>
       <c r="J193" t="str">
-        <v>REQ-14485. Mechanical/Industrial/Chemical Engineering, grad May 2027 or later. No H1-B sponsorship.</v>
+        <v>REQ-14480. Mechanical/Industrial/Chemical/Materials Science Engineering. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="194">
@@ -8138,22 +8120,22 @@
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E194" t="str">
-        <v>Bloomington, MN</v>
+        <v>Hillsboro, OR</v>
       </c>
       <c r="F194">
-        <v>1122</v>
+        <v>2548</v>
       </c>
       <c r="G194" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H194" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bloomington-MN/Manufacturing-Engineering-Co-Op_REQ-14417</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14479</v>
       </c>
       <c r="I194" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
       </c>
       <c r="J194" t="str">
-        <v>REQ-14417. Mechanical/Manufacturing/Industrial Engineering, Spring 2027 or 2028 grad. No H1-B sponsorship.</v>
+        <v>REQ-14479. Sibling req to REQ-14480, same site/majors. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="195">
@@ -8161,31 +8143,31 @@
         <v>Entegris</v>
       </c>
       <c r="B195" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Mechanical Engineering Co-Op</v>
       </c>
       <c r="C195" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D195" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E195" t="str">
-        <v>Hillsboro, OR</v>
+        <v>San Luis Obispo, CA</v>
       </c>
       <c r="F195">
-        <v>2548</v>
+        <v>2676</v>
       </c>
       <c r="G195" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H195" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14480</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14483</v>
       </c>
       <c r="I195" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J195" t="str">
-        <v>REQ-14480. Mechanical/Industrial/Chemical/Materials Science Engineering. No H1-B sponsorship.</v>
+        <v>REQ-14483. Mechanical/Aerospace Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="196">
@@ -8193,31 +8175,31 @@
         <v>Entegris</v>
       </c>
       <c r="B196" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Mechanical Engineering Co-Op</v>
       </c>
       <c r="C196" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D196" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E196" t="str">
-        <v>Hillsboro, OR</v>
+        <v>San Luis Obispo, CA</v>
       </c>
       <c r="F196">
-        <v>2548</v>
+        <v>2676</v>
       </c>
       <c r="G196" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H196" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Manufacturing-Engineering-Co-Op_REQ-14479</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14405</v>
       </c>
       <c r="I196" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'; GPA 3.0+ mentioned.</v>
+        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J196" t="str">
-        <v>REQ-14479. Sibling req to REQ-14480, same site/majors. No H1-B sponsorship.</v>
+        <v>REQ-14405. Sibling req to REQ-14483, same site/majors. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="197">
@@ -8225,95 +8207,95 @@
         <v>Entegris</v>
       </c>
       <c r="B197" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Controls Engineering Co-Op</v>
       </c>
       <c r="C197" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Controls / Automation Engineering</v>
       </c>
       <c r="D197" t="str">
         <v>Spring 2027 season (6-month assignment, begins January)</v>
       </c>
       <c r="E197" t="str">
-        <v>San Luis Obispo, CA</v>
+        <v>Austin, TX</v>
       </c>
       <c r="F197">
-        <v>2676</v>
+        <v>1694</v>
       </c>
       <c r="G197" t="str">
         <v>$20-$30/hour</v>
       </c>
       <c r="H197" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14483</v>
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Austin-TX/Controls-Engineering-Co-Op_REQ-14460</v>
       </c>
       <c r="I197" t="str">
         <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
       </c>
       <c r="J197" t="str">
-        <v>REQ-14483. Mechanical/Aerospace Engineering, grad Spring 2027 or later. No H1-B sponsorship.</v>
+        <v>REQ-14460. Electrical/Chemical/Mechanical/Controls-Automation Engineering majors. No H1-B sponsorship.</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Entegris</v>
+        <v>GE Aerospace</v>
       </c>
       <c r="B198" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Colibrium Additive US Manufacturing / Supply Chain Co-op - Spring 2027</v>
       </c>
       <c r="C198" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing / Supply Chain Engineering (Additive Manufacturing)</v>
       </c>
       <c r="D198" t="str">
-        <v>Spring 2027 season (6-month assignment, begins January)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E198" t="str">
-        <v>San Luis Obispo, CA</v>
+        <v>West Chester, OH</v>
       </c>
       <c r="F198">
-        <v>2676</v>
+        <v>700</v>
       </c>
       <c r="G198" t="str">
-        <v>$20-$30/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H198" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Mechanical-Engineering-Co-Op_REQ-14405</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/West-Chester/Colibrium-Additive-US-Manufacturing---Supply-Chain-Co-op---Spring-2027_R5040302-2</v>
       </c>
       <c r="I198" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040302, canApply true, posted 2 days ago.</v>
       </c>
       <c r="J198" t="str">
-        <v>REQ-14405. Sibling req to REQ-14483, same site/majors. No H1-B sponsorship.</v>
+        <v>New req found via a fresh Workday search sweep; not previously tracked.</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Entegris</v>
+        <v>GE Aerospace</v>
       </c>
       <c r="B199" t="str">
-        <v>Controls Engineering Co-Op</v>
+        <v>Flight Test Operation Engineering Intern - Victorville, CA - Spring 2027</v>
       </c>
       <c r="C199" t="str">
-        <v>Controls / Automation Engineering</v>
+        <v>Flight Test / Systems Engineering</v>
       </c>
       <c r="D199" t="str">
-        <v>Spring 2027 season (6-month assignment, begins January)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E199" t="str">
-        <v>Austin, TX</v>
+        <v>Victorville, CA</v>
       </c>
       <c r="F199">
-        <v>1694</v>
+        <v>2500</v>
       </c>
       <c r="G199" t="str">
-        <v>$20-$30/hour</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H199" t="str">
-        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Austin-TX/Controls-Engineering-Co-Op_REQ-14460</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Victorville/Flight-Test-Operation-Engineering-Intern---Victorville--CA---Spring-2027_R5040433-1</v>
       </c>
       <c r="I199" t="str">
-        <v>Yes — fetched directly, page live, body states 'join our team for the Spring 2027 season.'</v>
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040433, canApply true, posted 3 days ago.</v>
       </c>
       <c r="J199" t="str">
-        <v>REQ-14460. Electrical/Chemical/Mechanical/Controls-Automation Engineering majors. No H1-B sponsorship.</v>
+        <v>New req; flight-test/flight-systems discipline fit.</v>
       </c>
     </row>
     <row r="200">
@@ -8321,31 +8303,31 @@
         <v>GE Aerospace</v>
       </c>
       <c r="B200" t="str">
-        <v>Colibrium Additive US Manufacturing / Supply Chain Co-op - Spring 2027</v>
+        <v>Systems Engineering Co-op - Mechanical/Aerospace Engineering (Electric Power) - US - Spring 2027</v>
       </c>
       <c r="C200" t="str">
-        <v>Manufacturing / Supply Chain Engineering (Additive Manufacturing)</v>
+        <v>Systems Engineering (Mechanical/Aerospace)</v>
       </c>
       <c r="D200" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E200" t="str">
-        <v>West Chester, OH</v>
+        <v>Dayton, OH</v>
       </c>
       <c r="F200">
-        <v>700</v>
+        <v>750</v>
       </c>
       <c r="G200" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H200" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/West-Chester/Colibrium-Additive-US-Manufacturing---Supply-Chain-Co-op---Spring-2027_R5040302-2</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Dayton/Systems-Engineering-Co-op---Mechanical-Aerospace-Engineering--Electric-Power----US---Spring-2027_R5030103-1</v>
       </c>
       <c r="I200" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040302, canApply true, posted 2 days ago.</v>
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5030103, canApply true, posted 30+ days ago.</v>
       </c>
       <c r="J200" t="str">
-        <v>New req found via a fresh Workday search sweep; not previously tracked.</v>
+        <v>New req found via a fresh Workday search sweep. A parallel Electrical Engineering/Computer Engineering version (R5030099) at the same site was reviewed and excluded — EE/CS discipline.</v>
       </c>
     </row>
     <row r="201">
@@ -8353,63 +8335,63 @@
         <v>GE Aerospace</v>
       </c>
       <c r="B201" t="str">
-        <v>Flight Test Operation Engineering Intern - Victorville, CA - Spring 2027</v>
+        <v>Unison Engineering Part-time Co-op - US - Spring 2027</v>
       </c>
       <c r="C201" t="str">
-        <v>Flight Test / Systems Engineering</v>
+        <v>Mechanical / Manufacturing Engineering (Unison Industries subsidiary)</v>
       </c>
       <c r="D201" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E201" t="str">
-        <v>Victorville, CA</v>
+        <v>Saint George, UT</v>
       </c>
       <c r="F201">
-        <v>2500</v>
+        <v>2300</v>
       </c>
       <c r="G201" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H201" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Victorville/Flight-Test-Operation-Engineering-Intern---Victorville--CA---Spring-2027_R5040433-1</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Saint-George-UT-US-1/Unison-Engineering-Part-time-Co-op---US---Spring-2027_R5040016</v>
       </c>
       <c r="I201" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040433, canApply true, posted 3 days ago.</v>
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040016, canApply true, posted 9 days ago.</v>
       </c>
       <c r="J201" t="str">
-        <v>New req; flight-test/flight-systems discipline fit.</v>
+        <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>GE Aerospace</v>
+        <v>Symbotic</v>
       </c>
       <c r="B202" t="str">
-        <v>Systems Engineering Co-op - Mechanical/Aerospace Engineering (Electric Power) - US - Spring 2027</v>
+        <v>Co-op - Hardware Engineer</v>
       </c>
       <c r="C202" t="str">
-        <v>Systems Engineering (Mechanical/Aerospace)</v>
+        <v>Mechanical / Hardware Engineering (robotics)</v>
       </c>
       <c r="D202" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (January–May)</v>
       </c>
       <c r="E202" t="str">
-        <v>Dayton, OH</v>
+        <v>Wilmington, MA</v>
       </c>
       <c r="F202">
-        <v>750</v>
+        <v>17</v>
       </c>
       <c r="G202" t="str">
-        <v>Not stated on posting</v>
+        <v>$29.00–$40.00/hr</v>
       </c>
       <c r="H202" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Dayton/Systems-Engineering-Co-op---Mechanical-Aerospace-Engineering--Electric-Power----US---Spring-2027_R5030103-1</v>
+        <v>https://symbotic.wd504.myworkdayjobs.com/Symbotic/job/USA-Wilmington-MA---ITC/Hardware-Engineer_R7976</v>
       </c>
       <c r="I202" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5030103, canApply true, posted 30+ days ago.</v>
+        <v>Yes — fetched directly via Symbotic's own Workday CXS API, req R7976, canApply true, posted 3 days ago.</v>
       </c>
       <c r="J202" t="str">
-        <v>New req found via a fresh Workday search sweep. A parallel Electrical Engineering/Computer Engineering version (R5030099) at the same site was reviewed and excluded — EE/CS discipline.</v>
+        <v>Boston metro (Wilmington, MA — ITC site). Requires enrolled Bachelor's student in Systems/Robotics/Mechanical/Electrical/CS engineering. Hands-on electro-mechanical work: GD&amp;T, SolidWorks, manufacturing processes (machining, casting, sheet metal). Offers transportation/housing benefits for relocating students. A sibling req 'Co-op - Robot Perception' (R8113, same site/timeframe) was reviewed and excluded — Computer Vision/ML software discipline, requires Master's/PhD.</v>
       </c>
     </row>
     <row r="203">
@@ -8417,191 +8399,177 @@
         <v>GE Aerospace</v>
       </c>
       <c r="B203" t="str">
-        <v>Unison Engineering Part-time Co-op - US - Spring 2027</v>
+        <v>Unison Engineering Intern - Spring 2027</v>
       </c>
       <c r="C203" t="str">
-        <v>Mechanical / Manufacturing Engineering (Unison Industries subsidiary)</v>
+        <v>Mechanical / Aerospace / Electrical Engineering (Unison Industries subsidiary)</v>
       </c>
       <c r="D203" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E203" t="str">
-        <v>Saint George, UT</v>
+        <v>Dayton, OH / Jacksonville, FL / Norwich, NY / St. George, UT (4 sites, one assignment)</v>
       </c>
       <c r="F203">
-        <v>2300</v>
+        <v>750</v>
       </c>
       <c r="G203" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H203" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Saint-George-UT-US-1/Unison-Engineering-Part-time-Co-op---US---Spring-2027_R5040016</v>
+        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Jacksonville/Unison-Engineering-Intern---Spring-2027_R5037093-1</v>
       </c>
       <c r="I203" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5040016, canApply true, posted 9 days ago.</v>
+        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5037093, canApply true, posted 30+ days ago.</v>
       </c>
       <c r="J203" t="str">
-        <v>Posting explicitly states 'this internship role is for local Utah university students' — no relocation/housing assistance provided. Included per verification bar, but likely a poor fit unless Hamza is local to St. George, UT. Fall 2027 (R5040164) and Summer 2027 (R5040163) sibling reqs at the same site were reviewed and excluded — wrong season.</v>
+        <v>Full-time intern version distinct from the already-tracked part-time 'Unison Engineering Part-time Co-op' (R5040016, St. George UT only). Works on ignition systems, sensors, generators, harnesses, engine starters at Unison Industries sites. Min 3.0 GPA, Aero/Mechanical/Electrical Engineering majors. Fall 2027 (R5037092) sibling at the same 4 sites was previously reviewed and excluded — wrong season.</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Symbotic</v>
+        <v>Hermeus</v>
       </c>
       <c r="B204" t="str">
-        <v>Co-op - Hardware Engineer</v>
+        <v>Build Reliability Engineering Intern - Spring/Summer 2027</v>
       </c>
       <c r="C204" t="str">
-        <v>Mechanical / Hardware Engineering (robotics)</v>
+        <v>Manufacturing Engineering (structural fabrication &amp; assembly)</v>
       </c>
       <c r="D204" t="str">
-        <v>Spring 2027 (January–May)</v>
+        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
       </c>
       <c r="E204" t="str">
-        <v>Wilmington, MA</v>
+        <v>Atlanta, GA</v>
       </c>
       <c r="F204">
-        <v>17</v>
+        <v>950</v>
       </c>
       <c r="G204" t="str">
-        <v>$29.00–$40.00/hr</v>
+        <v>$25–33/hr</v>
       </c>
       <c r="H204" t="str">
-        <v>https://symbotic.wd504.myworkdayjobs.com/Symbotic/job/USA-Wilmington-MA---ITC/Hardware-Engineer_R7976</v>
+        <v>https://jobs.lever.co/hermeus/ee3a4109-b6e7-4ed5-8981-a483b3936e5a</v>
       </c>
       <c r="I204" t="str">
-        <v>Yes — fetched directly via Symbotic's own Workday CXS API, req R7976, canApply true, posted 3 days ago.</v>
+        <v>Yes — fetched directly via Hermeus's own Lever API, page live, distinct dated Spring option confirmed in body text.</v>
       </c>
       <c r="J204" t="str">
-        <v>Boston metro (Wilmington, MA — ITC site). Requires enrolled Bachelor's student in Systems/Robotics/Mechanical/Electrical/CS engineering. Hands-on electro-mechanical work: GD&amp;T, SolidWorks, manufacturing processes (machining, casting, sheet metal). Offers transportation/housing benefits for relocating students. A sibling req 'Co-op - Robot Perception' (R8113, same site/timeframe) was reviewed and excluded — Computer Vision/ML software discipline, requires Master's/PhD.</v>
+        <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>GE Aerospace</v>
+        <v>PI (Physik Instrumente)</v>
       </c>
       <c r="B205" t="str">
-        <v>Unison Engineering Intern - Spring 2027</v>
+        <v>Mechanical Engineering Co-op</v>
       </c>
       <c r="C205" t="str">
-        <v>Mechanical / Aerospace / Electrical Engineering (Unison Industries subsidiary)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D205" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E205" t="str">
-        <v>Dayton, OH / Jacksonville, FL / Norwich, NY / St. George, UT (4 sites, one assignment)</v>
+        <v>Shrewsbury, MA</v>
       </c>
       <c r="F205">
-        <v>750</v>
+        <v>40</v>
       </c>
       <c r="G205" t="str">
-        <v>Not stated on posting</v>
+        <v>$24–26/hr</v>
       </c>
       <c r="H205" t="str">
-        <v>https://geaerospace.wd5.myworkdayjobs.com/GE_ExternalSite/job/Jacksonville/Unison-Engineering-Intern---Spring-2027_R5037093-1</v>
+        <v>https://www.physikinstrumente.com/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
       </c>
       <c r="I205" t="str">
-        <v>Yes — fetched directly via GE Aerospace's own Workday CXS API, req R5037093, canApply true, posted 30+ days ago.</v>
+        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
       </c>
       <c r="J205" t="str">
-        <v>Full-time intern version distinct from the already-tracked part-time 'Unison Engineering Part-time Co-op' (R5040016, St. George UT only). Works on ignition systems, sensors, generators, harnesses, engine starters at Unison Industries sites. Min 3.0 GPA, Aero/Mechanical/Electrical Engineering majors. Fall 2027 (R5037092) sibling at the same 4 sites was previously reviewed and excluded — wrong season.</v>
+        <v>Boston metro (Shrewsbury). Fresh cycle superseding the already-past Jan-June 2026 cohort found at this same company in prior runs. Requires legal US work authorization without sponsorship; SolidWorks preferred. Mirrored identically (same ADP apply-link ID) at pi-usa.us/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027 — same posting, use either link.</v>
+      </c>
+      <c r="K205" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L205" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M205" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>Hermeus</v>
+        <v>PI (Physik Instrumente)</v>
       </c>
       <c r="B206" t="str">
-        <v>Build Reliability Engineering Intern - Spring/Summer 2027</v>
+        <v>Manufacturing Engineering Internship</v>
       </c>
       <c r="C206" t="str">
-        <v>Manufacturing Engineering (structural fabrication &amp; assembly)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D206" t="str">
-        <v>Spring 2027 option (~16 weeks, January–April) — posting also offers a separate Summer 2027 option (~12 weeks, May–August); intern selects one</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E206" t="str">
-        <v>Atlanta, GA</v>
+        <v>Shrewsbury, MA</v>
       </c>
       <c r="F206">
-        <v>950</v>
+        <v>40</v>
       </c>
       <c r="G206" t="str">
-        <v>$25–33/hr</v>
+        <v>$24–26/hr</v>
       </c>
       <c r="H206" t="str">
-        <v>https://jobs.lever.co/hermeus/ee3a4109-b6e7-4ed5-8981-a483b3936e5a</v>
+        <v>https://www.physikinstrumente.com/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
       </c>
       <c r="I206" t="str">
-        <v>Yes — fetched directly via Hermeus's own Lever API, page live, distinct dated Spring option confirmed in body text.</v>
+        <v>Yes — fetched directly, page live, 'Winter/Spring 2027' stated on posting.</v>
       </c>
       <c r="J206" t="str">
-        <v>New sibling req beyond already-tracked Hermeus postings. Hands-on factory-floor work: sheet metal, welded assemblies, tooling, manufacturing process improvement for aircraft structures. Open to 3rd/4th-year undergrads or Master's/PhD students in Mechanical/Aerospace/Materials Science Engineering. GPA 3.0+. US person required (export control). Same 'distinct dated Spring option within a combined-term posting' treatment as other tracked Hermeus reqs.</v>
+        <v>Boston metro (Shrewsbury). Same batch/cycle as the Mechanical Engineering Co-op above. Mirrored identically (same ADP apply-link ID) at pi-usa.us/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027 — same posting, use either link.</v>
+      </c>
+      <c r="K206" t="str">
+        <v>Open resume</v>
+      </c>
+      <c r="L206" t="str">
+        <v>Open cover letter</v>
+      </c>
+      <c r="M206" t="str">
+        <v>Open questions</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>PI (Physik Instrumente) USA</v>
+        <v>Buro Happold</v>
       </c>
       <c r="B207" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>Mechanical Co-op</v>
       </c>
       <c r="C207" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical Engineering (HVAC/Building Systems)</v>
       </c>
       <c r="D207" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E207" t="str">
-        <v>Shrewsbury, MA</v>
+        <v>Boston, MA</v>
       </c>
       <c r="F207">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="G207" t="str">
-        <v>$24-26/hour</v>
+        <v>$24.00–$34.00/hr</v>
       </c>
       <c r="H207" t="str">
-        <v>https://www.pi-usa.us/en/about/careers/job/mechanical-engineering-co-op-winterspring-2027</v>
+        <v>https://vacancies.burohappold.com/</v>
       </c>
       <c r="I207" t="str">
-        <v>Yes — fetched directly, HTTP 200, page title 'Mechanical Engineering Co-op - Winter/Spring 2027', full description read.</v>
+        <v>Partial — could not independently open the primary posting on vacancies.burohappold.com (site paginates ~23 pages of results with no working keyword/location filter observed, and the specific job-detail URL/ID could not be located). Title, location, term, and pay ($24-34/hr) are corroborated consistently across two independent secondary sources (a Workopia mirror and search-engine snippets), and Buro Happold's Boston office is confirmed to run a recurring seasonal co-op program (verified sibling postings for Spring/Fall 2025 and 2026 exist on their own site at sequential job IDs). Could not confirm live/open status or an application-deadline field directly.</v>
       </c>
       <c r="J207" t="str">
-        <v>New company for the tracker. Boston metro (Shrewsbury, MA — PI's US headquarters). High-precision positioning/motion systems and piezo technology manufacturer. Prepares detail/assembly drawings, CAD support, PLM data entry, R&amp;D build/test work. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship. SolidWorks and manufacturing-process experience preferred.</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="str">
-        <v>PI (Physik Instrumente) USA</v>
-      </c>
-      <c r="B208" t="str">
-        <v>Manufacturing Engineering Internship</v>
-      </c>
-      <c r="C208" t="str">
-        <v>Manufacturing Engineering</v>
-      </c>
-      <c r="D208" t="str">
-        <v>Winter/Spring 2027</v>
-      </c>
-      <c r="E208" t="str">
-        <v>Shrewsbury, MA</v>
-      </c>
-      <c r="F208">
-        <v>40</v>
-      </c>
-      <c r="G208" t="str">
-        <v>$24-26/hour</v>
-      </c>
-      <c r="H208" t="str">
-        <v>https://www.pi-usa.us/en/about/careers/job/manufacturing-engineering-internship-winterspring-2027</v>
-      </c>
-      <c r="I208" t="str">
-        <v>Yes — fetched directly, HTTP 200, page title 'Manufacturing Engineering Internship - Winter/Spring 2027', full description read.</v>
-      </c>
-      <c r="J208" t="str">
-        <v>Sibling req to the Mechanical Engineering Co-op above, same site/pay/season. Fixture design for assembly/metrology/manufacturing, SolidWorks modeling, hands-on machining (mills, lathes, saws, 3D printers), process optimization, ECR/ECO documentation. Must be currently enrolled full-time; legally authorized to work in the US without sponsorship.</v>
+        <v>Building-services engineering firm (structural/MEP consultancy) — HVAC/mechanical building-systems co-op, not aerospace/manufacturing, but fits Hamza's 'adjacent — structural' category and is in Boston itself. Requires Bachelor's in Mechanical or Architectural Engineering, HVAC/thermo/fluids coursework, BIM software familiarity. Needs a follow-up attempt to find the live job-detail URL on vacancies.burohappold.com directly (try searching/filtering by 'Mechanical' + 'Boston' rather than guessing job IDs).</v>
       </c>
     </row>
   </sheetData>
@@ -8899,12 +8867,12 @@
     <hyperlink ref="K107" r:id="rId291"/>
     <hyperlink ref="L107" r:id="rId292"/>
     <hyperlink ref="M107" r:id="rId293"/>
-    <hyperlink ref="K108" r:id="rId294"/>
-    <hyperlink ref="L108" r:id="rId295"/>
-    <hyperlink ref="M108" r:id="rId296"/>
-    <hyperlink ref="K109" r:id="rId297"/>
-    <hyperlink ref="L109" r:id="rId298"/>
-    <hyperlink ref="M109" r:id="rId299"/>
+    <hyperlink ref="K109" r:id="rId294"/>
+    <hyperlink ref="L109" r:id="rId295"/>
+    <hyperlink ref="M109" r:id="rId296"/>
+    <hyperlink ref="K110" r:id="rId297"/>
+    <hyperlink ref="L110" r:id="rId298"/>
+    <hyperlink ref="M110" r:id="rId299"/>
     <hyperlink ref="K111" r:id="rId300"/>
     <hyperlink ref="L111" r:id="rId301"/>
     <hyperlink ref="M111" r:id="rId302"/>
@@ -8914,12 +8882,12 @@
     <hyperlink ref="K113" r:id="rId306"/>
     <hyperlink ref="L113" r:id="rId307"/>
     <hyperlink ref="M113" r:id="rId308"/>
-    <hyperlink ref="K114" r:id="rId309"/>
-    <hyperlink ref="L114" r:id="rId310"/>
-    <hyperlink ref="M114" r:id="rId311"/>
-    <hyperlink ref="K115" r:id="rId312"/>
-    <hyperlink ref="L115" r:id="rId313"/>
-    <hyperlink ref="M115" r:id="rId314"/>
+    <hyperlink ref="K115" r:id="rId309"/>
+    <hyperlink ref="L115" r:id="rId310"/>
+    <hyperlink ref="M115" r:id="rId311"/>
+    <hyperlink ref="K116" r:id="rId312"/>
+    <hyperlink ref="L116" r:id="rId313"/>
+    <hyperlink ref="M116" r:id="rId314"/>
     <hyperlink ref="K117" r:id="rId315"/>
     <hyperlink ref="L117" r:id="rId316"/>
     <hyperlink ref="M117" r:id="rId317"/>
@@ -9082,22 +9050,22 @@
     <hyperlink ref="K170" r:id="rId474"/>
     <hyperlink ref="L170" r:id="rId475"/>
     <hyperlink ref="M170" r:id="rId476"/>
-    <hyperlink ref="K171" r:id="rId477"/>
-    <hyperlink ref="L171" r:id="rId478"/>
-    <hyperlink ref="M171" r:id="rId479"/>
-    <hyperlink ref="K172" r:id="rId480"/>
-    <hyperlink ref="L172" r:id="rId481"/>
-    <hyperlink ref="M172" r:id="rId482"/>
+    <hyperlink ref="K205" r:id="rId477"/>
+    <hyperlink ref="L205" r:id="rId478"/>
+    <hyperlink ref="M205" r:id="rId479"/>
+    <hyperlink ref="K206" r:id="rId480"/>
+    <hyperlink ref="L206" r:id="rId481"/>
+    <hyperlink ref="M206" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M208"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M207"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C391"/>
+  <dimension ref="A1:C392"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -13405,9 +13373,20 @@
         <v>2026-09-26 ~07:00 UTC re-check: both reqs confirmed live via direct fetch, freshly posted/updated 2026-09-17, but neither posting states a season/term anywhere in the text (no Spring/Winter/Summer/Fall) — same generic rolling req pattern as its already-excluded sibling. Fails the season-stated verification bar. No dated Winter 2026/Spring 2027 sibling found on careers.sharkninja.com's sitemap either. Not added.</v>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>PI (Physik Instrumente) USA — pi-usa.us-domain duplicate</v>
+      </c>
+      <c r="B392" t="str">
+        <v>'Mechanical Engineering Co-op' and 'Manufacturing Engineering Internship' (Winter/Spring 2027, Shrewsbury MA) as posted on pi-usa.us</v>
+      </c>
+      <c r="C392" t="str">
+        <v>2026-09-26 ~13:00 UTC: while cross-checking this run's findings, this session noticed the tracker carried these same two Shrewsbury, MA co-ops as 4 separate `rows` entries — once under physikinstrumente.com (Company: 'PI (Physik Instrumente)') and again under pi-usa.us (Company: 'PI (Physik Instrumente) USA'). Direct curl of both domains' identical URL paths confirmed byte-identical apply-link IDs (ADP 'applyonline/click?jp=67557317' on both pages) and the same legal entity ('PI (Physik Instrumente), LP') — these are the same two job postings mirrored across the company's global (.com) and US-subsidiary (pi-usa.us) websites, not 4 distinct openings. Removed the pi-usa.us-domain duplicate pair from `rows`, keeping the original physikinstrumente.com pair (which already has Hamza's prepared resume/cover-letter/questions documents linked in `applications/` under the 'PI (Physik Instrumente)' company name — switching to the pi-usa.us name would have orphaned that existing work). The physikinstrumente.com rows' notes now mention the pi-usa.us mirror URL as an equally-valid alternate apply link. Net effect: 2 fewer rows in the spreadsheet, no loss of a real opportunity, existing application documents preserved.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C392"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new/upgraded postings, 4 checked-excluded (2026-09-26 19:00 UTC)
Installed Playwright + headless Chromium to render JS-blocked ATSes
(Eaton eightfold.ai, Buro Happold, Textron Nuxt SPA) that plain
curl/WebFetch could not read past the app shell across many prior runs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FiKh5CC4vZrTEap4EVFedf
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M207"/>
+  <dimension ref="A1:M209"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -8563,13 +8563,77 @@
         <v>$24.00–$34.00/hr</v>
       </c>
       <c r="H207" t="str">
-        <v>https://vacancies.burohappold.com/</v>
+        <v>https://vacancies.burohappold.com/jobs/job/Mechanical-Coop-Boston-Spring-2027/2462</v>
       </c>
       <c r="I207" t="str">
-        <v>Partial — could not independently open the primary posting on vacancies.burohappold.com (site paginates ~23 pages of results with no working keyword/location filter observed, and the specific job-detail URL/ID could not be located). Title, location, term, and pay ($24-34/hr) are corroborated consistently across two independent secondary sources (a Workopia mirror and search-engine snippets), and Buro Happold's Boston office is confirmed to run a recurring seasonal co-op program (verified sibling postings for Spring/Fall 2025 and 2026 exist on their own site at sequential job IDs). Could not confirm live/open status or an application-deadline field directly.</v>
+        <v>Yes — 2026-09-26 ~19:00 UTC: upgraded from Partial. Independently fetched via a headless-browser render of vacancies.burohappold.com's own keyword search (its ATS is JS-rendered; a plain fetch only returns pagination scaffolding, but rendering it directly resolved the exact job-detail URL/ID for the first time). Full posting text confirmed live, title/location/term/pay all match.</v>
       </c>
       <c r="J207" t="str">
-        <v>Building-services engineering firm (structural/MEP consultancy) — HVAC/mechanical building-systems co-op, not aerospace/manufacturing, but fits Hamza's 'adjacent — structural' category and is in Boston itself. Requires Bachelor's in Mechanical or Architectural Engineering, HVAC/thermo/fluids coursework, BIM software familiarity. Needs a follow-up attempt to find the live job-detail URL on vacancies.burohappold.com directly (try searching/filtering by 'Mechanical' + 'Boston' rather than guessing job IDs).</v>
+        <v>Building-services engineering firm (structural/MEP consultancy) — HVAC/mechanical building-systems co-op, not aerospace/manufacturing, but fits Hamza's 'adjacent — structural' category and is in Boston itself. Requires Bachelor's in Mechanical or Architectural Engineering, HVAC/thermo/fluids coursework, BIM software familiarity.</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>Eaton</v>
+      </c>
+      <c r="B208" t="str">
+        <v>Manufacturing Engineer Co-op - Spring 2027</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E208" t="str">
+        <v>Sumter, SC</v>
+      </c>
+      <c r="F208">
+        <v>900</v>
+      </c>
+      <c r="G208" t="str">
+        <v>$22.15–27.69/hr (by class year)</v>
+      </c>
+      <c r="H208" t="str">
+        <v>https://eaton.eightfold.ai/careers/job/687239184994</v>
+      </c>
+      <c r="I208" t="str">
+        <v>Yes — 2026-09-26 ~19:00 UTC: independently fetched via a headless-browser render of Eaton's own eightfold.ai ATS (a pure client-rendered SPA that plain curl/WebFetch cannot read past the app shell — resolved this run with a real browser render). Job Req ID 73120, full description read directly, 'Spring 2027 Start Date' stated explicitly with class-year pay tiers.</v>
+      </c>
+      <c r="J208" t="str">
+        <v>Commercial products &amp; assemblies (CPA) engineering team. Requires enrollment in Mechanical, Electrical, Industrial, or Manufacturing Engineering bachelor's/master's program, min. 1 prior internship/co-op, 2.8+ GPA. No visa sponsorship (no CPT/OPT/STEM OPT/H-1B support). Relocation assistance provided for candidates outside 50mi of Sumter, SC. Resolves a multi-run 'Eaton ATS unreadable' blocker.</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>Eaton</v>
+      </c>
+      <c r="B209" t="str">
+        <v>Product Development Engineering Co-op - Spring 2027</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Mechanical Engineering (Product Development / R&amp;D)</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E209" t="str">
+        <v>Hodges, SC</v>
+      </c>
+      <c r="F209">
+        <v>950</v>
+      </c>
+      <c r="G209" t="str">
+        <v>$22.15–27.69/hr (by class year)</v>
+      </c>
+      <c r="H209" t="str">
+        <v>https://eaton.eightfold.ai/careers/job/687239184785</v>
+      </c>
+      <c r="I209" t="str">
+        <v>Yes — 2026-09-26 ~19:00 UTC: independently fetched via a headless-browser render of Eaton's own eightfold.ai ATS (same method as the Sumter, SC sibling above). Job Req ID 73116, full description read directly, 'Spring 2027 Start Date' stated explicitly with class-year pay tiers.</v>
+      </c>
+      <c r="J209" t="str">
+        <v>Busway product line (Pow-R-Way III / Powerwave 2) — CAD solid modeling, design simulation, DFMA, product testing/validation. Same eligibility/GPA/no-sponsorship terms as the Sumter, SC sibling.</v>
       </c>
     </row>
   </sheetData>
@@ -9058,14 +9122,14 @@
     <hyperlink ref="M206" r:id="rId482"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M207"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M209"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C392"/>
+  <dimension ref="A1:C395"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -13384,9 +13448,42 @@
         <v>2026-09-26 ~13:00 UTC: while cross-checking this run's findings, this session noticed the tracker carried these same two Shrewsbury, MA co-ops as 4 separate `rows` entries — once under physikinstrumente.com (Company: 'PI (Physik Instrumente)') and again under pi-usa.us (Company: 'PI (Physik Instrumente) USA'). Direct curl of both domains' identical URL paths confirmed byte-identical apply-link IDs (ADP 'applyonline/click?jp=67557317' on both pages) and the same legal entity ('PI (Physik Instrumente), LP') — these are the same two job postings mirrored across the company's global (.com) and US-subsidiary (pi-usa.us) websites, not 4 distinct openings. Removed the pi-usa.us-domain duplicate pair from `rows`, keeping the original physikinstrumente.com pair (which already has Hamza's prepared resume/cover-letter/questions documents linked in `applications/` under the 'PI (Physik Instrumente)' company name — switching to the pi-usa.us name would have orphaned that existing work). The physikinstrumente.com rows' notes now mention the pi-usa.us mirror URL as an equally-valid alternate apply link. Net effect: 2 fewer rows in the spreadsheet, no loss of a real opportunity, existing application documents preserved.</v>
       </c>
     </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>Eaton</v>
+      </c>
+      <c r="B393" t="str">
+        <v>'Mechanical Engineer Internship / Co-op', Moon Township, PA (Job Req IDs 71539 and 71556, ES AMER ARS division and Energy Transition Team)</v>
+      </c>
+      <c r="C393" t="str">
+        <v>2026-09-26 ~19:00 UTC: RESOLVED — this session installed a headless Chromium (Playwright, already available in this sandbox's image at /opt/pw-browsers) to render Eaton's eightfold.ai ATS directly for the first time, closing out a blocker that spanned 3+ prior runs (guessed tenant URLs 500'd, plain curl/WebFetch only saw the app shell). Both Moon Township, PA reqs are confirmed live, but each explicitly states 'This position can either be a rotational co-op assignment, or a Summer 2027 internship' — no distinct Spring-2027-dated slot, fails the season bar. The company's genuinely Spring-2027-dated siblings (Manufacturing Engineer Co-op, Sumter SC, req 73120; Product Development Engineering Co-op, Hodges SC, req 73116) WERE independently confirmed via this same method and added to `rows` — see above. This also resolves the 2026-09-25 ~19:00 UTC entry below, which could not identify Eaton's ATS at all; it is eaton.eightfold.ai, and it is readable with a real browser render, not curl.</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>Buro Happold</v>
+      </c>
+      <c r="B394" t="str">
+        <v>'Plumbing &amp; Fire Protection Co-op - Boston - Spring 2027', job 2463 (sibling to the Mechanical Co-op, job 2462, upgraded to `rows` this run)</v>
+      </c>
+      <c r="C394" t="str">
+        <v>2026-09-26 ~19:00 UTC: confirmed live via the same headless-browser render that resolved the Mechanical Co-op sibling (same site, term, and $24-34/hr pay), but Plumbing &amp; Fire Protection engineering is not on Hamza's target discipline list (mechanical/aerospace/manufacturing/robotics/adjacent-structural) — discipline mismatch. Not added.</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>Textron Systems / Bell Textron</v>
+      </c>
+      <c r="B395" t="str">
+        <v>Full re-fetch via headless-browser render (not curl/WebFetch) of every live '2027' mechanical/manufacturing/systems intern-or-co-op req on careers.textron.com's current sitemap: 6 at Hunt Valley, MD (co-op mechanical engineer, co-op systems engineer, intern mechanical engineer ×2, intern manufacturing engineer, intern mechanical engineer/sea systems), 3 at Williamsport, PA/Lycoming (intern mechanical engineering, intern manufacturing engineer, intern systems engineer), 2 at Cartersville, GA (manufacturing engineer intern, mechanical engineer intern/ground support equipment), and 3 at Slidell/New Orleans, LA (intern manufacturing engineer ×2, intern integration test engineer/marine)</v>
+      </c>
+      <c r="C395" t="str">
+        <v>2026-09-26 ~19:00 UTC: RESOLVED, definitively — careers.textron.com's Nuxt SPA had blocked curl/WebFetch across 3+ prior runs; this session rendered it directly with a real headless Chromium (Playwright) instead, and every one of these 14 postings' full body text was read successfully. None state Winter/Spring/Summer/Fall anywhere — instead each gives only a generic application-window deadline (e.g. 'Applications... accepted through October 31, 2026'). This confirms, for the first time from directly-read full text rather than an inferred title pattern, that Textron's internship/co-op postings structurally omit season — not a fetch limitation, a template choice. Not added. Recommend downgrading Textron from 'needs a browser-rendering attempt' to an occasional light-touch title-only check, since even full rendering cannot pass the season bar here. (Note: the specific req slugs/IDs surfaced by the 2026-09-26 ~01:00 UTC run — Wichita KS, Augusta GA engineering reqs — are no longer present on today's sitemap; Textron's live req list rotates fairly quickly, so slug lists should not be treated as stable across runs.)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C392"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C395"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 3 checked-excluded (2026-09-27 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GWPKdgaQkpEM659wuYdiiU
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -9084,7 +9084,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C403"/>
+  <dimension ref="A1:C406"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -13518,9 +13518,39 @@
         <v>2026-09-27 ~01:00 UTC re-check: both confirmed live, 12-week/40hr rotational assignment, $25-43/hr, applications due Dec 30 2026 — but the posting still never states Spring vs. Summer anywhere in its own text. No FAQ/program page found confirming a Spring start; a Summer 2027 start is at least as plausible given the program's typical cadence. Still excluded pending a dated version. No change.</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B404" t="str">
+        <v>'Applications Engineering Internship - Spring 2027' (req 7824822003, El Segundo, CA)</v>
+      </c>
+      <c r="C404" t="str">
+        <v>2026-09-27 ~07:00 UTC: flagged as a new sibling req beyond Varda's already-tracked batch by this run's national-sweep agent (not previously seen — job ID absent from `build.mjs`). This session independently fetched the posting directly via Varda's own Greenhouse API and read the full description: despite the 'Applications Engineer' title sitting inside an aerospace company, the role itself is enterprise-IT/software — building integrations between ERP/PLM/HRIS platforms, data pipelines, dashboards, and internal tooling. Not a mechanical/aerospace/manufacturing/robotics/structural/controls discipline. Excluded on discipline-mismatch grounds, same treatment as the already-excluded Rendezvous Robotics and Varda 'Avionics Engineering' EE-discipline reqs.</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>National sweep, 2026-09-27 ~07:00 UTC — mostly-already-tracked batch</v>
+      </c>
+      <c r="B405" t="str">
+        <v>Two parallel research agents' fresh Boston-area and national sweeps this run, each briefed with the current known-blocker list and headless-browser method. Nearly every specific req/URL either reported (Blue Origin R71445/Summer-only LA lead, Moog R-26-20226/R-26-20243, GE Vernova R5049161, Zipline's full 7-req Spring 2027 batch, Rendezvous Robotics' 4 Golden-CO reqs, Varda's Structures/Propulsion/Mechanisms/Manufacturing/Vehicle-Integration reqs, Astranis's Spring 2027 Mechanical/CAD batch, Hermeus's 11-req Lever batch, Draper JR002883-1, GE Aerospace R5029617-1, Vertex REQ-30500-1, Insulet's REQ-2026-18007/18061, GD Electric Boat 2026-20763, Formlabs 8130829, Amazon Robotics 10535282/10536817, Entegris Billerica REQ-14457 and San Luis Obispo REQ-14405/14483/Chaska REQ-14477-1, Aalo Atomics, Owens Corning, Crown Equipment, Marathon Petroleum req 00020137, GE Appliances LaFayette GA/Decatur AL reqs) was independently cross-checked by this session against `build.mjs` and found already tracked byte-for-byte (same job IDs/req numbers/URLs) — a strong sign, after 8+ days of near-daily sweeps, that mainstream Boston-area and aerospace/defense employer coverage is essentially saturated. The only genuinely new lead surfaced (Varda's Applications Engineering Internship) failed the discipline bar — see the dedicated entry above. Apptronik, Figure AI (Winter 2026 mechanical req confirmed gone from live Greenhouse board), Reliable Robotics, Agility Robotics, BETA Technologies' ambiguous '2026-2027' program, Karman Space &amp; Defense (ADP-hosted board, not yet queried), Curtiss-Wright, and Anduril/Shield AI/Joby/Archer/Wisk (all Summer-2027-only) remain unresolved-or-excluded dead ends, unchanged from prior runs. No new `rows` entries this run.</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>Boston-area fresh sweep, 2026-09-27 ~07:00 UTC — nothing qualifying found</v>
+      </c>
+      <c r="B406" t="str">
+        <v>PTC (software-only, no hardware discipline — permanent rule-out), MathWorks (software-centric, nothing mechanical for Spring 2027), Teradyne (zero live co-op-keyword reqs company-wide), Vicor (no dedicated intern/co-op title), Cognex (only Aachen, Germany mechanical-intern matches, none US), MKS Instruments (only 3 open reqs company-wide, none Andover/mechanical/Spring-2027), Charles River Laboratories/Boston Metal/Nuvation Engineering/Nuvera Fuel Cells/Cirtec Medical (no postings surfaced for any), PI (Physik Instrumente)/pi-usa.us (current live Shrewsbury MA posting is now dated 'Fall 2026' — wrong season, no Spring 2027 posting yet), Symbotic (only Software/ML/Perception/Robotics/Systems Co-ops live; the one plausible 'Hardware Engineer' req 404/500'd — likely stale), Boston Dynamics (previously-tracked reqs R2476/R2495 now both return Workday 'page does not exist' — confirms the 2026-09-26 finding that these are gone, re-verified independently this run), iRobot (only Spring/Summer combined or Fall combined windows, no clean Winter-2026/Spring-2027-only posting), Commonwealth Fusion Systems (Fall 2026 and Spring/Summer 2026 co-ops only, nothing for Spring 2027), Hologic (na.careers.hologic.com still intermittently 503ing — could not confirm any live posting; consistent with the 2026-09-26 ~01:00 UTC recommendation to deprioritize), Bose (LinkedIn-sourced titles only, season unconfirmed, not independently opened this run — still needs direct follow-up), Analog Devices/Lam Research/Parker Hannifin (still nothing posted for the 2027 cycle), SharkNinja (still Spring 2026/Fall 2026/Summer 2027 only, no Spring 2027 yet), Waters Corporation (iCIMS AWS WAF CAPTCHA still blocks both plain fetch and headless-browser rendering — genuinely unverifiable), MIT Lincoln Laboratory (only generic Summer 2026 SRP postings found, no targeted Spring 2027 req identified this pass), Entegris Aurora IL/Colorado Springs CO/Bloomington MN/Hillsboro OR/Austin TX (a non-exhaustive keyword search found no live mechanical co-op reqs at these sites right now; not a confirmed absence, the Workday facet-filter crawl was incomplete).</v>
+      </c>
+      <c r="C406" t="str">
+        <v>2026-09-27 ~07:00 UTC Boston-area sweep — see the national-sweep entry above for the Varda Applications Engineering exclusion and the saturated-coverage cross-check.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C406"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 15 new postings (14 Entegris + 1 Blue Origin), 7 checked-excluded, 5 Insulet upgrades (2026-09-27 13:00 UTC)
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M209"/>
+  <dimension ref="A1:M223"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -625,16 +625,16 @@
         <v>Blue Origin</v>
       </c>
       <c r="B6" t="str">
-        <v>Spring 2027 Structural &amp; Mechanical Systems Engineering Internship – Graduate</v>
+        <v>Mechanical Engineering Co-Op (Fixed Term)</v>
       </c>
       <c r="C6" t="str">
-        <v>Structural / Mechanical Systems Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D6" t="str">
-        <v>Spring 2027 (~15 wks)</v>
+        <v>~5-month co-op, January–June 2027</v>
       </c>
       <c r="E6" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Altadena, CA (Honeybee Robotics, a Blue Origin company)</v>
       </c>
       <c r="F6">
         <v>2600</v>
@@ -643,22 +643,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H6" t="str">
-        <v>https://www.ziprecruiter.com/c/Blue-Origin/Job/Spring-2027-Structural-&amp;-Mechanical-Systems-Engineering-Internship-Graduate/-in-Los-Angeles,CA?jid=67aec7854122d860</v>
+        <v>https://blueorigin.wd5.myworkdayjobs.com/BlueOrigin/job/Los-Angeles-CA/Mechanical-Engineering-Co-Op--Fixed-Term-_R71542</v>
       </c>
       <c r="I6" t="str">
-        <v>Partial — this is a ZipRecruiter mirror of the Blue Origin listing (couldn't locate the direct Workday URL). Confirm on blueorigin.com/careers before applying.</v>
+        <v>Yes — fetched directly via Blue Origin's own Workday CXS API (req R71542), canApply true, body states 'This is a ~5 month co-op from January to June 2027' at the Honeybee Robotics (Altadena, CA) site.</v>
       </c>
       <c r="J6" t="str">
-        <v>Grad student, US citizen/national/permanent resident required (ITAR).</v>
-      </c>
-      <c r="K6" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
-      </c>
-      <c r="L6" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
-      </c>
-      <c r="M6" t="str">
-        <v>Skipped: graduate students only (you are an undergrad)</v>
+        <v>REQ R71542. US citizen/national/permanent resident (Green Card) or asylee/refugee required (ITAR/export control). 2026-09-27 ~13:00 UTC: replaces the prior ZipRecruiter-sourced 'Structural &amp; Mechanical Systems Engineering Internship – Graduate' lead, which this run independently confirmed is dead (its only current live sibling with that exact title is Summer 2027, req R71445) — see `checked`.</v>
       </c>
     </row>
     <row r="7">
@@ -2561,7 +2552,7 @@
         <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Mechanical-Lifecycle--January---June-2027--Onsite-_REQ-2026-18155</v>
       </c>
       <c r="I53" t="str">
-        <v>Partial — confirmed live and current via direct query of Insulet's own Workday jobs-search API (real title/location/posted-date, not an aggregator), posted 5 days ago. Full job-description body was not individually opened — spot-check before applying.</v>
+        <v>Yes — 2026-09-27 ~13:00 UTC: upgraded from Partial via direct fetch of Insulet's Workday CXS job JSON (canApply true, body states 'Position Dates: January 11th, 2027 - June 30th, 2027').</v>
       </c>
       <c r="J53" t="str">
         <v>Boston metro (Acton). One of a batch of Insulet Acton co-ops opened this cycle alongside the fully-verified R&amp;D Mechanical/Manufacturing/Systems reqs above.</v>
@@ -2602,7 +2593,7 @@
         <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--R-D-Manufacturing--January-June-2027--Onsite-_REQ-2026-18069</v>
       </c>
       <c r="I54" t="str">
-        <v>Partial — confirmed live via direct Workday jobs-search API query, posted 5 days ago. Full description not individually opened — spot-check before applying.</v>
+        <v>Yes — 2026-09-27 ~13:00 UTC: upgraded from Partial via direct fetch of Insulet's Workday CXS job JSON (canApply true, body states 'Position Dates: January 11, 2027 – June 30, 2027').</v>
       </c>
       <c r="J54" t="str">
         <v>Boston metro (Acton).</v>
@@ -2684,7 +2675,7 @@
         <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Supplier-Development-Engineering---Mechanical--January-June-2027--Onsite-_REQ-2026-18209</v>
       </c>
       <c r="I56" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly (not a synthesized link); the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Yes — 2026-09-27 ~13:00 UTC: upgraded from Partial via direct fetch of Insulet's Workday CXS job JSON (canApply true, body states 'Position Dates: January 11, 2027 – June 30, 2027').</v>
       </c>
       <c r="J56" t="str">
         <v>Boston metro (Acton).</v>
@@ -2725,7 +2716,7 @@
         <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Systems-Engineering---Design-Verification--January---June-2027--Onsite-_REQ-2026-18144-1</v>
       </c>
       <c r="I57" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Yes — 2026-09-27 ~13:00 UTC: upgraded from Partial via direct fetch of Insulet's Workday CXS job JSON (canApply true, body states 'Position Dates: January 11, 2027 – June 30, 2027').</v>
       </c>
       <c r="J57" t="str">
         <v>Boston metro (Acton).</v>
@@ -2766,7 +2757,7 @@
         <v>https://insulet.wd5.myworkdayjobs.com/insuletcareers/job/Acton-Massachusetts/Co-op--Life-Cycle-Engineering---Systems--January---June-2027--Hybrid-_REQ-2026-18149</v>
       </c>
       <c r="I58" t="str">
-        <v>Partial — title/season/pay/location confirmed via a Dreamwork aggregator mirror that quotes Insulet's own Workday application URL directly; the live Workday page itself is JS-rendered and returned blank on direct fetch. Spot-check before applying.</v>
+        <v>Yes — 2026-09-27 ~13:00 UTC: upgraded from Partial via direct fetch of Insulet's Workday CXS job JSON (canApply true, body states 'Position Dates: January 11, 2027 – June 30, 2027').</v>
       </c>
       <c r="J58" t="str">
         <v>Boston metro (Acton). Most recently posted of the Insulet batch.</v>
@@ -8598,6 +8589,454 @@
       </c>
       <c r="J209" t="str">
         <v>3-6+ month internship/co-op durations, multiple locations. Same graduation-window/eligibility pattern as Amazon Robotics' other tracked req. Boston-area (~22 mi).</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B210" t="str">
+        <v>Science &amp; Engineering Co-op</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Mechanical / Chemical Engineering</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E210" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F210">
+        <v>17</v>
+      </c>
+      <c r="G210" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H210" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Bedford-MA/Science---Engineering-Co-op_REQ-14396</v>
+      </c>
+      <c r="I210" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J210" t="str">
+        <v>REQ-14396. Bachelor's in mechanical or chemical engineering preferred. No H1-B sponsorship (standard Entegris co-op policy).</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B211" t="str">
+        <v>Continuous Improvement Engineer Co-Op</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Industrial / Manufacturing / Mechanical Engineering</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E211" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F211">
+        <v>2676</v>
+      </c>
+      <c r="G211" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H211" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Continuous-Improvement-Engineer-Co-Op_REQ-14398</v>
+      </c>
+      <c r="I211" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J211" t="str">
+        <v>REQ-14398. Industrial, Manufacturing, or Mechanical Engineering, desired grad year 2028 or sooner. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B212" t="str">
+        <v>Maintenance Engineering Technician Co-Op</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E212" t="str">
+        <v>Hillsboro, OR</v>
+      </c>
+      <c r="F212">
+        <v>2548</v>
+      </c>
+      <c r="G212" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H212" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Maintenance-Engineering-Technician-Co-Op_REQ-14400</v>
+      </c>
+      <c r="I212" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J212" t="str">
+        <v>REQ-14400. Desired major: Mechanical Engineering, 2027 grad. 'Technician' in title despite ME major requirement. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B213" t="str">
+        <v>Product Development Engineering Co-Op</v>
+      </c>
+      <c r="C213" t="str">
+        <v>STEM (general) — works on Chemical Mechanical Planarization pad manufacturing/process development</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E213" t="str">
+        <v>Hillsboro, OR</v>
+      </c>
+      <c r="F213">
+        <v>2548</v>
+      </c>
+      <c r="G213" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H213" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Hillsboro-OR/Product-Development-Engineering-Co-Op_REQ-14418</v>
+      </c>
+      <c r="I213" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J213" t="str">
+        <v>REQ-14418. Desired major stated only as 'rising junior or senior working towards a Bachelor of Science in a STEM field' — broader than a named ME/manufacturing major, but the role itself is manufacturing-process-development work (CMP pad manufacturing). Included per manufacturing discipline fit; Hamza's own call given the open-ended major line. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B214" t="str">
+        <v>NPI Engineering Co-Op</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Industrial / Mechanical Engineering</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E214" t="str">
+        <v>Chaska, MN</v>
+      </c>
+      <c r="F214">
+        <v>1137</v>
+      </c>
+      <c r="G214" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H214" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/NPI-Engineering-Co-Op_REQ-14426</v>
+      </c>
+      <c r="I214" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for a six-month Spring 2027 assignment.'</v>
+      </c>
+      <c r="J214" t="str">
+        <v>REQ-14426. Industrial or Mechanical Engineering, 2027/2028 grad. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Designer/Drafter Co-Op</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E215" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F215">
+        <v>2676</v>
+      </c>
+      <c r="G215" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H215" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Designer-Drafter-Co-Op_REQ-14428-1</v>
+      </c>
+      <c r="I215" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J215" t="str">
+        <v>REQ-14428. Mechanical Engineer, graduating Spring 2027 or later. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Product Design Co-Op</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Spring 2027 season (fulltime assignment, begins January)</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F216">
+        <v>1771</v>
+      </c>
+      <c r="G216" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H216" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Product-Design-Co-Op_REQ-14435</v>
+      </c>
+      <c r="I216" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J216" t="str">
+        <v>REQ-14435. Desired major: Mechanical Engineering. Must have completed junior year. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Materials Engineering Co-Op</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Materials / Chemical / Polymer Engineering</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Chaska, MN</v>
+      </c>
+      <c r="F217">
+        <v>1137</v>
+      </c>
+      <c r="G217" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H217" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Materials-Engineering-Co-Op_REQ-14451</v>
+      </c>
+      <c r="I217" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J217" t="str">
+        <v>REQ-14451. Materials/Chemical/Polymer Engineering, target grad Dec 2027 or May 2028. Polymer/materials development for semiconductor purity solutions — fits Hamza's 'materials' adjacent-discipline preference. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B218" t="str">
+        <v>Continuous Improvement Co-Op</v>
+      </c>
+      <c r="C218" t="str">
+        <v>Mechanical / Electrical / Manufacturing / Industrial Engineering</v>
+      </c>
+      <c r="D218" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E218" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F218">
+        <v>1771</v>
+      </c>
+      <c r="G218" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H218" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Continuous-Improvement-Co-Op_REQ-14455</v>
+      </c>
+      <c r="I218" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J218" t="str">
+        <v>REQ-14455. Mechanical/Electrical/Manufacturing/Industrial Engineering or Operations Management/Supply Chain. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B219" t="str">
+        <v>Continuous Improvement Engineer Co-Op</v>
+      </c>
+      <c r="C219" t="str">
+        <v>Industrial / Manufacturing / Mechanical / Electrical Engineering</v>
+      </c>
+      <c r="D219" t="str">
+        <v>Spring 2027 season (fulltime assignment, begins January)</v>
+      </c>
+      <c r="E219" t="str">
+        <v>Chaska, MN</v>
+      </c>
+      <c r="F219">
+        <v>1137</v>
+      </c>
+      <c r="G219" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H219" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Chaska-MN/Continuous-Improvement-Engineer-Co-Op_REQ-14478</v>
+      </c>
+      <c r="I219" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J219" t="str">
+        <v>REQ-14478. Industrial/Manufacturing/Mechanical/Electrical Engineering, Operations Management, Supply Chain Management, Engineering Management, Business Analytics, or related. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B220" t="str">
+        <v>NPI Engineering Co-Op</v>
+      </c>
+      <c r="C220" t="str">
+        <v>Mechanical / Industrial / Manufacturing Engineering</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Spring 2027 season (fulltime assignment, begins January)</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F220">
+        <v>1771</v>
+      </c>
+      <c r="G220" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H220" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/NPI-Engineering-Co-Op_REQ-14488</v>
+      </c>
+      <c r="I220" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J220" t="str">
+        <v>REQ-14488. Mechanical/Industrial/Manufacturing Engineering, Engineering Technology, Plastics Engineering Technology, Quality Engineering, or Project Management. Grad Spring 2027 or later. No H1-B sponsorship. Distinct site label ('Rockrimmon') from the plain 'Colorado Springs, CO' sibling reqs — same physical Entegris site per this tracker's established convention.</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B221" t="str">
+        <v>Research and Development Co-Op</v>
+      </c>
+      <c r="C221" t="str">
+        <v>Chemistry / Chemical / Mechanical / Industrial Engineering</v>
+      </c>
+      <c r="D221" t="str">
+        <v>Spring 2027 season (6-month assignment, begins January)</v>
+      </c>
+      <c r="E221" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F221">
+        <v>2676</v>
+      </c>
+      <c r="G221" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H221" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Research-and-Development-Co-Op_REQ-14490</v>
+      </c>
+      <c r="I221" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J221" t="str">
+        <v>REQ-14490. Chemistry, Chemical Engineering, Mechanical Engineering, Industrial Engineering, or related science/engineering field. Grad Spring 2027 or later. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B222" t="str">
+        <v>Product Engineering Co-Op</v>
+      </c>
+      <c r="C222" t="str">
+        <v>Mechanical / Aerospace / Chemical Engineering</v>
+      </c>
+      <c r="D222" t="str">
+        <v>Spring 2027 season (begins January)</v>
+      </c>
+      <c r="E222" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F222">
+        <v>1771</v>
+      </c>
+      <c r="G222" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H222" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Colorado-Springs-CO/Product-Engineering-Co-Op_REQ-14503</v>
+      </c>
+      <c r="I222" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J222" t="str">
+        <v>REQ-14503. Mechanical Engineering, Aerospace Engineering, Chemical Engineering, or similar. Undergrad, grad date May 2027 or later. CAD-based product development (reticle handling products). No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B223" t="str">
+        <v>Quality Engineering Co-Op</v>
+      </c>
+      <c r="C223" t="str">
+        <v>Mechanical / Industrial / Chemical / Manufacturing / Materials / Aerospace / Systems Engineering</v>
+      </c>
+      <c r="D223" t="str">
+        <v>Spring 2027 season (begins January)</v>
+      </c>
+      <c r="E223" t="str">
+        <v>Colorado Springs (Rockrimmon), CO</v>
+      </c>
+      <c r="F223">
+        <v>1771</v>
+      </c>
+      <c r="G223" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H223" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Rockrimmon-Colorado-Springs-CO/Quality-Engineering-Co-Op_REQ-14468</v>
+      </c>
+      <c r="I223" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J223" t="str">
+        <v>REQ-14468. Body explicitly welcomes 'a variety of engineering backgrounds, including: Mechanical Engineering, Industrial Engineering, Chemical Engineering, Manufacturing Engineering, Materials Engineering, Plastics Engineering, Aerospace Engineering, Systems Engineering.' No H1-B sponsorship.</v>
       </c>
     </row>
   </sheetData>
@@ -9077,14 +9516,14 @@
     <hyperlink ref="M202" r:id="rId473"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M209"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M223"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C406"/>
+  <dimension ref="A1:C413"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -13548,9 +13987,86 @@
         <v>2026-09-27 ~07:00 UTC Boston-area sweep — see the national-sweep entry above for the Varda Applications Engineering exclusion and the saturated-coverage cross-check.</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B407" t="str">
+        <v>'Lab Automation &amp; AI Engineering Co-Op' (REQ-14498, Billerica, MA)</v>
+      </c>
+      <c r="C407" t="str">
+        <v>2026-09-27 ~13:00 UTC: found during this run's full Workday facet-crawl of Entegris's 8 tracked sites (part of the same batch that surfaced 13 new Spring 2027 co-ops added to `rows` this run). Confirmed live/canApply, Spring 2027 season, but desired major is Chemical Engineering or Chemistry only — no ME/manufacturing/industrial option. Discipline mismatch, not added.</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>Entegris — Electrical Manufacturing Engineering Co-Op (REQ-14486, Bloomington, MN)</v>
+      </c>
+      <c r="B408" t="str">
+        <v>Re-check of an already-excluded req after a conflicting agent claim</v>
+      </c>
+      <c r="C408" t="str">
+        <v>2026-09-27 ~13:00 UTC: this run's national-sweep agent claimed a fresh fetch showed the desired-major line now reading 'electrical engineering, Mechanical Engineering, Manufacturing Engineering, or a related technical field' (i.e. no longer EE-only) and flagged it for possible re-inclusion. This session independently re-fetched the same req directly via Entegris's Workday CXS API and read the full body text: it states only 'Electrical Engineering, graduating Spring 2027 or later' — no Mechanical/Manufacturing wording anywhere. The agent's claim does not match the live posting (apparent misread, same pattern as a prior run's Moog R-26-20226 false-positive). Exclusion CONFIRMED, unchanged — still EE-only, discipline mismatch. Not added.</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>Alloy Enterprises (Burlington, MA)</v>
+      </c>
+      <c r="B409" t="str">
+        <v>'Co-Op, Thermal Test Engineer, Fall 2026 (July-December)'</v>
+      </c>
+      <c r="C409" t="str">
+        <v>2026-09-27 ~13:00 UTC: correction to a prior run's assumption that this company was defunct/absorbed into Johnson Controls — it is alive with a live Ashby board (jobs.ashbyhq.com/alloyenterprises), 5 open roles, confirmed via direct fetch ($23-$50/hr range stated). This specific Thermal Test Engineer co-op is confirmed live but explicitly Fall 2026, not Winter 2026/Spring 2027 — wrong season. No Spring 2027 co-op currently posted. Not added; worth a periodic re-check now that the company/ATS is confirmed active.</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>PI (Physik Instrumente) / PI USA — Fall 2026 sibling posting</v>
+      </c>
+      <c r="B410" t="str">
+        <v>'Mechanical Engineering Internship – Fall 2026' and 'Supply Chain Internship – Fall 2026' (Shrewsbury, MA)</v>
+      </c>
+      <c r="C410" t="str">
+        <v>2026-09-27 ~13:00 UTC: confirmed via search that a distinct Fall-2026-titled sibling posting existed at this company (different URL slug/content from the two tracked Winter/Spring 2027 rows) — resolves the 2026-09-27 ~07:00 UTC entry's ambiguous 'current live posting is now dated Fall 2026' note, which was a mix-up with this separate req, not a change to the tracked rows. Direct re-fetch this run of both tracked Winter/Spring 2027 URLs confirms they are unchanged (HTTP 200, 'Winter/Spring 2027' still stated). This Fall 2026 sibling itself now 404s on both physikinstrumente.com and pi-usa.us and no longer appears on PI's live jobs listing — appears expired, and would be wrong-season regardless. Not added; no change to the tracked rows.</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B411" t="str">
+        <v>'Spring 2027 Structural &amp; Mechanical Systems Engineering Internship – Graduate', Los Angeles, CA (ZipRecruiter-mirror-only lead, previously tracked in `rows` as Partial)</v>
+      </c>
+      <c r="C411" t="str">
+        <v>2026-09-27 ~13:00 UTC: RESOLVED, dead. This session independently paged Blue Origin's own Workday CXS API filtered to Los Angeles + the Intern/Co-op job category (10 current postings) and confirmed no live req exists with this exact Spring-2027 title — only a Summer 2027 sibling with the identical title (req R71445) is currently posted. The ZipRecruiter-sourced lead is stale/dead (likely referencing an expired req or conflated with the live Summer 2027 one). MOVED from `rows` to `checked` (net -1 row from this cause); replaced in `rows` by a genuinely new Spring 2027 Blue Origin/Honeybee Robotics Mechanical Engineering Co-Op (req R71542, same Los Angeles-area facet search) found in the same query — see `rows`.</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B412" t="str">
+        <v>'Electronics/Electrical Systems Engineer Co-Op (Fixed Term)' (req R71548, Los Angeles/Altadena, CA — Honeybee Robotics)</v>
+      </c>
+      <c r="C412" t="str">
+        <v>2026-09-27 ~13:00 UTC: found via the same Los Angeles + Intern/Co-op facet search that surfaced the new Mechanical Engineering Co-Op (req R71542, added to `rows`). Confirmed live, same Spring 2027 (Jan-June) term and site, but Electrical/Electronics discipline — not on Hamza's target list. Not added.</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>National-sweep dead ends, 2026-09-27 ~13:00 UTC</v>
+      </c>
+      <c r="B413" t="str">
+        <v>Figure AI (Greenhouse board: zero Mechanical Engineer Intern postings, only Fall 2026 EE Intern/Special Projects Intern — the previously-circulated 'Winter 2026 Mechanical' lead is stale/closed), Archer Aviation (Greenhouse board `archer56`: zero intern-titled postings; the specific job ID 7574255003 found via search now 404s — closed), Stoke Space (Greenhouse board: only Summer 2027 Engineering/Ops/Software internships currently live; the Spring 2027 lead shown by aggregators is not on the employer's own board — appears closed, and wrong season regardless), Reliable Robotics (real ATS identified as Ashby, board slug `reliable-robotics`; zero intern-titled postings, only full-time Sr./Mechanical/Manufacturing Engineer roles — the aggregator-sourced 'Winter 2026/Spring 2027 Mechanical Engineering Intern' language could not be confirmed live), Textron Aviation (Wichita KS 'Engineering Mechanical Systems' 2027 internship reqs are Textron's standard Summer cycle, 10-week late-May–Aug — wrong season; careers.textron.com remains an unreadable Nuxt SPA past the app shell), Spirit AeroSystems (only Summer 2027 internship tracks found at Wichita KS — no Spring 2027 co-op located), Karman Space &amp; Defense (ADP WorkforceNow SPA, could not independently verify; aggregator-only 'Mechanical Aerospace Engineering Intern' lead, season/dates unconfirmed from source — inconclusive), BETA Technologies (Lever board now returns an empty postings array and prior posting URLs 404 — may have switched ATS, unchanged from the 2026-09-25 note), Firefly Aerospace/Redwire Space/Sierra Space/Impulse Space/Shield AI/Joby Aviation/Agility Robotics/Apptronik/General Atomics/HII/Curtiss-Wright (quick-check only per instructions — every mechanical/aerospace intern posting located was Summer 2026/2027, Fall 2026, or season-unstated; no Winter 2026/Spring 2027-dated posting found for any this round, not exhaustively re-swept).</v>
+      </c>
+      <c r="C413" t="str">
+        <v>See individual notes above; all either confirmed closed/wrong-season on the employer's own source, or genuinely unverifiable and flagged as inconclusive rather than silently dropped or upgraded.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C406"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C413"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 7 checked-excluded (2026-09-27 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016CY3NBhCYmd9Tkb4Ai6B9h
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M223"/>
+  <dimension ref="A1:M227"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9037,6 +9037,134 @@
       </c>
       <c r="J223" t="str">
         <v>REQ-14468. Body explicitly welcomes 'a variety of engineering backgrounds, including: Mechanical Engineering, Industrial Engineering, Chemical Engineering, Manufacturing Engineering, Materials Engineering, Plastics Engineering, Aerospace Engineering, Systems Engineering.' No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B224" t="str">
+        <v>Research and Development Engineer/Scientist Co-Op</v>
+      </c>
+      <c r="C224" t="str">
+        <v>Materials Engineering / R&amp;D</v>
+      </c>
+      <c r="D224" t="str">
+        <v>Spring 2027 season (6 months, begins January)</v>
+      </c>
+      <c r="E224" t="str">
+        <v>Danbury, CT</v>
+      </c>
+      <c r="F224">
+        <v>140</v>
+      </c>
+      <c r="G224" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H224" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Danbury-CT/Research-and-Development-Engineer-Scientist-Co-Op_REQ-14430</v>
+      </c>
+      <c r="I224" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J224" t="str">
+        <v>REQ-14430. 2026-09-27 sweep. Desired majors: Chemistry, Physics, Chemical Engineer, Mechanical Engineer, Materials Engineer. Builds/automates lab equipment for gas packaging/delivery and dry-etch product development. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B225" t="str">
+        <v>Quality Engineer Co-Op</v>
+      </c>
+      <c r="C225" t="str">
+        <v>Mechanical / Industrial / Manufacturing / Materials Engineering (Quality)</v>
+      </c>
+      <c r="D225" t="str">
+        <v>Spring 2027 season (6 months, begins January)</v>
+      </c>
+      <c r="E225" t="str">
+        <v>San Luis Obispo, CA</v>
+      </c>
+      <c r="F225">
+        <v>2676</v>
+      </c>
+      <c r="G225" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H225" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/San-Luis-Obispo-CA/Quality-Engineer-Co-Op_REQ-14434</v>
+      </c>
+      <c r="I225" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J225" t="str">
+        <v>REQ-14434. 2026-09-27 sweep. Desired majors: Mechanical/Industrial/Manufacturing/Chemical/Materials Engineering. MRB/CAPA, quality data analysis, process improvement on the production floor. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B226" t="str">
+        <v>Analytical Quality Engineering Co-Op</v>
+      </c>
+      <c r="C226" t="str">
+        <v>Industrial / Systems / Materials Engineering (Quality)</v>
+      </c>
+      <c r="D226" t="str">
+        <v>Spring 2027 season (6 months, January–June)</v>
+      </c>
+      <c r="E226" t="str">
+        <v>Round Rock, TX</v>
+      </c>
+      <c r="F226">
+        <v>1681</v>
+      </c>
+      <c r="G226" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H226" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Round-Rock-TX/Analytical-Quality-Engineering-Co-Op_REQ-14464</v>
+      </c>
+      <c r="I226" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J226" t="str">
+        <v>REQ-14464. 2026-09-27 sweep. Desired majors: Chemical/Industrial/Systems/Quality Engineering, Chemistry, Materials Science. Lab-documentation standardization/KPI-tracking project, MS Analytical Quality team. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B227" t="str">
+        <v>R&amp;D Co-Op</v>
+      </c>
+      <c r="C227" t="str">
+        <v>Materials Engineering</v>
+      </c>
+      <c r="D227" t="str">
+        <v>Spring 2027 season (6 months, begins January)</v>
+      </c>
+      <c r="E227" t="str">
+        <v>Franklin, MA</v>
+      </c>
+      <c r="F227">
+        <v>26</v>
+      </c>
+      <c r="G227" t="str">
+        <v>$20-$30/hour</v>
+      </c>
+      <c r="H227" t="str">
+        <v>https://entegris.wd1.myworkdayjobs.com/EntegrisCareers/job/Franklin-MA/R-D-Co-Op_REQ-14446</v>
+      </c>
+      <c r="I227" t="str">
+        <v>Yes — fetched directly via Workday CXS API, canApply true, body states 'join our team for the Spring 2027 season.'</v>
+      </c>
+      <c r="J227" t="str">
+        <v>REQ-14446. 2026-09-27 sweep. Desired majors: Chemical Engineering, Materials Science/Engineering. Characterization/testing of adsorbent materials for filtration/purification. No H1-B sponsorship.</v>
       </c>
     </row>
   </sheetData>
@@ -9516,14 +9644,14 @@
     <hyperlink ref="M202" r:id="rId473"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M223"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M227"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C413"/>
+  <dimension ref="A1:C420"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -14064,9 +14192,86 @@
         <v>See individual notes above; all either confirmed closed/wrong-season on the employer's own source, or genuinely unverifiable and flagged as inconclusive rather than silently dropped or upgraded.</v>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>Entegris</v>
+      </c>
+      <c r="B414" t="str">
+        <v>'Electrical Engineer Co-Op' (REQ-14436, San Luis Obispo, CA)</v>
+      </c>
+      <c r="C414" t="str">
+        <v>2026-09-27 ~19:00 UTC: found during this run's full 29-page Workday CXS re-sweep of all company-wide Co-Op-titled reqs (searchText paging, offset 0-560). Confirmed live/canApply, Spring 2027 season, but body explicitly seeks Electrical Engineering only (SolidWorks Electrical/DraftSight drawings) — same EE-only mismatch treatment as REQ-14486/R71548. Not added.</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>Entegris — science/analyst-titled Co-Ops, 2026-09-27 ~19:00 UTC</v>
+      </c>
+      <c r="B415" t="str">
+        <v>'R&amp;D Analytical Chemist Co-Op' (REQ-14471, Danbury CT), 'Microanalysis Scientist Co-Op' (REQ-14476, Billerica MA), 'Research Associate Co-Op - ICPS' (REQ-14482, Aurora IL), 'Nanoparticle Research Associate Co-Op' (REQ-14493, Aurora IL), 'Metrology Scientist Co-Op' (REQ-14501, Billerica MA)</v>
+      </c>
+      <c r="C415" t="str">
+        <v>2026-09-27 ~19:00 UTC: all found in the same full company-wide sweep, all confirmed live/canApply/Spring 2027 season, but each is a chemistry/lab-scientist role (analytical chemistry, microanalysis, nanoparticle research, metrology) rather than an engineering discipline on Hamza's list — same treatment as the earlier-excluded REQ-14498 (Chemical Eng/Chemistry-only Lab Automation &amp; AI Engineering Co-Op). Not added.</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>Entegris — non-engineering Co-Ops, 2026-09-27 ~19:00 UTC</v>
+      </c>
+      <c r="B416" t="str">
+        <v>38 additional new Co-Op-titled reqs surfaced by this run's full company-wide sweep, spanning HR (REQ-14404), Marketing (REQ-14406), Business Process Architect (REQ-14407), IT Portfolio/Project Management (REQ-14414), Sustainability (REQ-14415), Operations Technical Training Platforms (REQ-14416), Production Scheduler (REQ-14419), Environmental Health &amp; Safety (REQ-14420, 14448, 14449, 14489), Analytical Lab (REQ-14422), general Quality (REQ-14425), Facility Technician (REQ-14427), Enterprise Transformation Program Coordination (REQ-14433), general Operations (REQ-14453), Enterprise Solution Architecture Analyst (REQ-14445), Product Associate (REQ-14443), Procurement Solutions Process Development (REQ-14456), Technical Training (REQ-14459, 14467), IT Program Management (REQ-14463), Cybersecurity Engineer (REQ-14472), Internal Audit (REQ-14475), Customer Service (REQ-14481), Portfolio Analytics Analyst (REQ-14499), Operational Excellence (REQ-14502), Cyber Threat Analyst (REQ-14505), Innovation Training/Application (REQ-14506, 14507), AI Continuous Improvement (REQ-14509), and Sales Strategy/Pricing &amp; Commercial Analytics (REQ-14510, 14511).</v>
+      </c>
+      <c r="C416" t="str">
+        <v>All confirmed live/Spring-2027-season on direct fetch but are HR, IT, business, finance, sales, EHS, or training functions — none is a mechanical/aerospace/manufacturing/robotics/materials/structural/controls engineering discipline. Not added (not individually detailed further; titles alone establish the mismatch).</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>Blue Origin</v>
+      </c>
+      <c r="B417" t="str">
+        <v>Re-check of the LA/Altadena Honeybee Robotics facet, plus tracked req R71542</v>
+      </c>
+      <c r="C417" t="str">
+        <v>2026-09-27 ~19:00 UTC: the previously-used 'Contingent, Temporary, &amp; Intern' jobFamilyGroup facet id now consistently 400s on Blue Origin's Workday CXS API (server-side, reproduced 3x with a fresh id lookup each time) — likely a new block on that specific facet. Worked around by paging full-text 'Co-Op'/'Intern' search (200+ results, offsets 0-180) and filtering for Los Angeles/Altadena: only turned up the already-excluded R71548 (Electrical, unchanged) and confirmed via direct job-page fetch that the already-tracked R71542 (Mechanical Engineering Co-Op, Honeybee Robotics) is still canApply true, posted 18 days ago. No new LA-area Spring 2027 mechanical/aerospace req found. No change to `rows` or `checked`.</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B418" t="str">
+        <v>Full company-wide re-sweep via Workday CXS ('Co-op'/'Intern' full-text search, ~305 unique postings enumerated across US/UK/global sites)</v>
+      </c>
+      <c r="C418" t="str">
+        <v>2026-09-27 ~19:00 UTC: explicitly prioritized per this run's instructions. Every Spring-2027-dated Co-op/Intern title found (Colibrium Additive US Mfg/Supply Chain R5040302, Digital Technology Co-op R5029741, Engines Engineering Co-op R5029617/R5029619, Flight Test Operation Engineering Intern R5040433, SaaS Data Science Co-op R5040450, US Communications Co-op R5039320, Unison Engineering Intern R5037093, Unison Engineering Part-time Co-op R5040016) is either already tracked in `rows` under the same base req number, or a non-target discipline (Digital Technology, Data Science, Communications). No new mechanical/aerospace/manufacturing/systems Spring 2027 req found; GE Aerospace's US Spring-2027 slate appears saturated at the 8 reqs already tracked.</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B419" t="str">
+        <v>Full re-sweep via Workday CXS ('Co-op'/'Co-Op' search, 100 postings enumerated)</v>
+      </c>
+      <c r="C419" t="str">
+        <v>2026-09-27 ~19:00 UTC: no reqs found beyond the two already tracked in `rows` (Systems Engineering Co-Op JR002882, Electro-Mechanical Instrument Co-op JR002883-1, Materials and Chemistry Engineering Co-op JR002942) plus the already-excluded Electrical Engineering Co-Op (JR002941), Sensor Electrical Engineering Co-op (JR002885), Optics-Physics Sensor Engineering Co-op (JR002884, EE/optics discipline mismatch — re-confirmed unchanged, not upgraded), and Mechanical Engineering &amp; System Packaging Intern (JR002943, Summer 2027 — wrong season). Consistent with prior runs' saturation finding; no change.</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B420" t="str">
+        <v>careers.ll.mit.edu re-check (site search is a JS-rendered SuccessFactors/SmashFly page that does not filter by URL keyword on static fetch — worked around via targeted web search instead) plus direct re-fetch of both tracked microfab req URLs</v>
+      </c>
+      <c r="C420" t="str">
+        <v>2026-09-27 ~19:00 UTC: explicitly prioritized per this run's instructions. No new Winter 2026/Spring 2027 mechanical/aerospace/structural/systems co-op found beyond the two already-tracked Microelectronics Laboratory (Group 08-35) microfab co-ops (Jan-Aug 2027) — both re-confirmed HTTP 200/still live. The only other Winter/Spring-adjacent postings surfaced by search (Group 7-74 'Machine Learning for Aerospace Engineering' Jan-Jun 2026, Group 07-74 'Structural &amp; Thermal-Fluids Engineering' Summer 2026) are already in the past relative to today's date (2026-09-27) and are not current live postings. Site remains hard to fully re-sweep programmatically (no working keyword-filtered API found); worth trying a headless-browser method in a future run if one becomes available.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C413"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C420"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 7 checked-excluded (2026-09-28 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkuZe7N6RHR3Ur9Retqvmi
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M227"/>
+  <dimension ref="A1:M230"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9165,6 +9165,102 @@
       </c>
       <c r="J227" t="str">
         <v>REQ-14446. 2026-09-27 sweep. Desired majors: Chemical Engineering, Materials Science/Engineering. Characterization/testing of adsorbent materials for filtration/purification. No H1-B sponsorship.</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="str">
+        <v>RTX / Collins Aerospace</v>
+      </c>
+      <c r="B228" t="str">
+        <v>Mechanical Design Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C228" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D228" t="str">
+        <v>Winter/Spring 2027 (runs January through July/August, including the Spring semester)</v>
+      </c>
+      <c r="E228" t="str">
+        <v>Rockford, IL</v>
+      </c>
+      <c r="F228">
+        <v>900</v>
+      </c>
+      <c r="G228" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H228" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IL-ROCKFORD-P6--4747-Harrison-Ave--4747-HARRISON-AVE-P6/Mechanical-Design-Engineering-Co-op--Winter-Spring-2027-_01873225</v>
+      </c>
+      <c r="I228" t="str">
+        <v>Yes — fetched directly via RTX's own Workday CXS API, canApply true, posted 2026-09-27 (today at discovery). Body explicitly states the co-op 'will run January- July/August (including the Spring semester; it is expected students will take a semester off from coursework...).'</v>
+      </c>
+      <c r="J228" t="str">
+        <v>Req 01873225. New company for the tracker. U.S. citizenship strictly required ('only U.S. citizens are authorized to access information under this program/contract'), no security clearance required. A sibling 'Summer/Fall 2027' req exists at the same site — excluded, wrong season.</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="str">
+        <v>Applied Materials</v>
+      </c>
+      <c r="B229" t="str">
+        <v>2027 Spring Product Quality Engineer Co-op - Bachelor's</v>
+      </c>
+      <c r="C229" t="str">
+        <v>Mechanical / Industrial Engineering (Quality)</v>
+      </c>
+      <c r="D229" t="str">
+        <v>Spring 2027 (co-op begins Jan. 2027, training starts early-mid Dec 2026; ~6 months on-site)</v>
+      </c>
+      <c r="E229" t="str">
+        <v>Gloucester, MA</v>
+      </c>
+      <c r="F229">
+        <v>26</v>
+      </c>
+      <c r="G229" t="str">
+        <v>$31-$33/hour</v>
+      </c>
+      <c r="H229" t="str">
+        <v>https://careers.appliedmaterials.com/careers/job/790318404669</v>
+      </c>
+      <c r="I229" t="str">
+        <v>Yes — fetched directly (JobPosting JSON-LD on the live page), datePosted 2026-09-09, validThrough 2027-03-08.</v>
+      </c>
+      <c r="J229" t="str">
+        <v>Req R2628290 (VSU BU Implant). Bachelor's student in mechanical or industrial engineering, good academic standing. Supports quality group: defective-material processing, supplier visits, cross-functional problem solving.</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="str">
+        <v>Applied Materials</v>
+      </c>
+      <c r="B230" t="str">
+        <v>2026-2027 Process Engineer Co-op - Doctorate</v>
+      </c>
+      <c r="C230" t="str">
+        <v>Mechanical Engineering / Materials Science (semiconductor process R&amp;D)</v>
+      </c>
+      <c r="D230" t="str">
+        <v>Fall 2026 through Spring 2027 (multiple start dates Sept-Nov 2026, 6-9 month co-op term)</v>
+      </c>
+      <c r="E230" t="str">
+        <v>Gloucester, MA</v>
+      </c>
+      <c r="F230">
+        <v>26</v>
+      </c>
+      <c r="G230" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H230" t="str">
+        <v>https://careers.appliedmaterials.com/careers/job/790317811290</v>
+      </c>
+      <c r="I230" t="str">
+        <v>Yes — fetched directly (JobPosting JSON-LD on the live page), datePosted 2026-08-14.</v>
+      </c>
+      <c r="J230" t="str">
+        <v>Req R2626230. PhD-ONLY role — requires currently pursuing a PhD in Electrical/Chemical/Mechanical Engineering, Materials Science, Chemistry, or Physics; verify this matches Hamza's own class standing before applying. Thin-film characterization/patterning R&amp;D for next-gen semiconductor nodes; cleanroom protocols.</v>
       </c>
     </row>
   </sheetData>
@@ -9644,14 +9740,14 @@
     <hyperlink ref="M202" r:id="rId473"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M227"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M230"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C420"/>
+  <dimension ref="A1:C427"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -14269,9 +14365,86 @@
         <v>2026-09-27 ~19:00 UTC: explicitly prioritized per this run's instructions. No new Winter 2026/Spring 2027 mechanical/aerospace/structural/systems co-op found beyond the two already-tracked Microelectronics Laboratory (Group 08-35) microfab co-ops (Jan-Aug 2027) — both re-confirmed HTTP 200/still live. The only other Winter/Spring-adjacent postings surfaced by search (Group 7-74 'Machine Learning for Aerospace Engineering' Jan-Jun 2026, Group 07-74 'Structural &amp; Thermal-Fluids Engineering' Summer 2026) are already in the past relative to today's date (2026-09-27) and are not current live postings. Site remains hard to fully re-sweep programmatically (no working keyword-filtered API found); worth trying a headless-browser method in a future run if one becomes available.</v>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B421" t="str">
+        <v>Healthcare Mechanical Engineering Co-op (Spring), R266691 — new req, posted 2 days before this run</v>
+      </c>
+      <c r="C421" t="str">
+        <v>2026-09-28 ~01:00 UTC: this session independently fetched the req directly via ADI's own Workday CXS API (canApply true). The posting is internally contradictory on season, same failure pattern as the already-excluded Entegris REQ-14401: the role-description opening explicitly states 'This is a full-time, in-person co-op opportunity running from June through December,' but the Qualifications section separately states 'Available to work full-time, on-site from January through June.' Given the direct conflict and no way to resolve which window is authoritative, excluding rather than guessing — worth a fresh look if the posting is corrected.</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>Caterpillar</v>
+      </c>
+      <c r="B422" t="str">
+        <v>'2027 Engineering Corporate Parallel Co-op Program', req R0000380509 (7 locations incl. Mossville IL, Tucson/Green Valley AZ, Champaign/Decatur IL, Lafayette IN)</v>
+      </c>
+      <c r="C422" t="str">
+        <v>2026-09-28 ~01:00 UTC: confirmed live via direct Workday CXS API fetch (canApply true, $25-43/hr, GPA 3.0+, mechanical/simulation/controls-development work — strong discipline fit). Excluded on season grounds: the posting explicitly describes 'continuous employment... full-time in-person during the summer and then part-time throughout the school year' on an annual/ongoing basis, not a discrete Winter 2026 or Spring 2027 block — fails the season-specific bar. Worth noting for Hamza's own judgment if he'd consider a year-round parallel program despite the season mismatch.</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>Parker Hannifin</v>
+      </c>
+      <c r="B423" t="str">
+        <v>Official careers portal (parkercareers.ttcportals.com, parker.com)</v>
+      </c>
+      <c r="C423" t="str">
+        <v>2026-09-28 ~01:00 UTC: portal returned HTTP 403 Forbidden on direct fetch — could not access or verify directly. Aggregator-only mentions found (not independently confirmed): a '2027 Manufacturing Engineering Co-Op' in Manitowoc, WI (aggregator describes Jan-Aug 2027 and May-Dec 2027 rotations) and a 'Material Science Co-op' in Columbus, OH explicitly titled Spring 2026 (wrong/past season). Neither added — no verified req ID, URL, or season text from the actual posting.</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B424" t="str">
+        <v>careers.lamresearch.com / opportunities.lamresearch.com (Eightfold ATS)</v>
+      </c>
+      <c r="C424" t="str">
+        <v>2026-09-28 ~01:00 UTC: site is JS-rendered and its API returned 'Not authorized' on direct query. Web search confirms Lam's 2026 mechanical/materials/process co-op cycle (Fremont, CA / Tualatin, OR) closed by mid-May 2026 and no 2027 requisitions have posted yet. Nothing to add; worth a re-check in a few weeks when the 2027 cycle typically opens.</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>Waters Corporation (Milford, MA)</v>
+      </c>
+      <c r="B425" t="str">
+        <v>jobs.waters.com / uscareers-waters.icims.com, re-check</v>
+      </c>
+      <c r="C425" t="str">
+        <v>2026-09-28 ~01:00 UTC: this run's block presented differently than before (DNS-level failure / ENOTFOUND on both curl-via-proxy and WebFetch, rather than the previously-documented AWS WAF CAPTCHA) — still fully inaccessible either way. Aggregator-only, unverified mentions found: a 'Research Electrical Engineering Co-Op' (Milford, MA, discipline mismatch besides being unverifiable) and a vague reference to a Liquid Chromatography Operations Engineering co-op — neither has a confirmed season, req ID, or working application URL. Genuinely unverifiable with current tooling; unchanged from prior runs.</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>ABB / ABB Robotics</v>
+      </c>
+      <c r="B426" t="str">
+        <v>careers.abb (general search)</v>
+      </c>
+      <c r="C426" t="str">
+        <v>2026-09-28 ~01:00 UTC: careers.abb is JS-rendered; direct fetch returned only generic program blurbs, no live listings enumerable. An aggregator mentions an 'Application Engineering Intern — Spring 2027' in Lombard, IL, but the actual posting could not be fetched or verified — not added.</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>National + Boston-area sweep, 2026-09-28 ~01:00 UTC — saturation reconfirmed</v>
+      </c>
+      <c r="B427" t="str">
+        <v>Two parallel research agents (Boston-area + national) briefed with the current known-blocker/saturation state and this run's priorities (Entegris full company-wide sweep, GE Aerospace, Draper, MIT Lincoln Laboratory, Blue Origin, Moog, Lam Research, Parker Hannifin, Caterpillar, Rendezvous Robotics/Hermeus/Varda/Rocket Lab, plus a light untried-company pass).</v>
+      </c>
+      <c r="C427" t="str">
+        <v>Every specific req/URL either agent reported was independently cross-checked by this session against `build.mjs` (by REQ ID/job ID) before any edit. Entegris: a full 54-req company-wide Workday sweep (San Luis Obispo, Bedford, Billerica, Franklin, Chaska, Aurora, Hillsboro, Colorado Springs, Austin, Bloomington MA/CT/TX/MN/IL/OR/CO sites) found every single engineering-discipline req already tracked in `rows` or `checked`, byte-for-byte by REQ ID — the board has not produced a genuinely new req since the 2026-09-27 ~19:00 UTC sweep. Draper (6 reqs), GE Aerospace (Lynn-specific + national Spring 2027 slate), and MIT Lincoln Laboratory (both microfab co-ops) were each independently re-swept and found fully saturated at their already-tracked reqs — no changes. Blue Origin (R71542/R71548), Moog (R-26-20226/R-26-20243 — re-confirmed same ambiguous/combined-term wording as prior runs, no change), Rocket Lab (~20-req Spring 2027 wave), Varda (7 El Segundo reqs), Hermeus (11-req Lever batch), Rendezvous Robotics (4 Golden CO reqs), and Anduril (8-req Winter 2027 Quincy/Lexington/Costa Mesa batch, including the EWIS Harness Engineer Co-op resolved in a prior run) were all confirmed already tracked with matching job IDs — no new items. Genuinely new finds from this run (RTX/Collins Rockford IL, 2 new Applied Materials Gloucester MA reqs) were added to `rows` above; Analog Devices, Caterpillar, Parker Hannifin, Lam Research, Waters, and ABB findings were added to `checked` above. SharkNinja (still Fall 2026 only, no Spring 2027 yet), KLA, Woodward, Textron/Textron eAviation (JS-blocked, no verifiable dated posting), and Relativity Space (Greenhouse board returned 0 jobs, likely migrated ATS — unexamined) turned up nothing actionable this run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C420"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C427"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new posting, 12 checked-excluded (2026-09-28 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VaHeC1Tn881WpZgV12syCM
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M232"/>
+  <dimension ref="A1:M233"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9316,6 +9316,38 @@
       </c>
       <c r="J232" t="str">
         <v>Req R26_04216. New company for the tracker. No discipline restriction stated beyond general engineering; posting text did not specify eligibility/citizenship requirements — confirm directly with employer before applying.</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B233" t="str">
+        <v>Application Engineer Co-op (Spring 2027)</v>
+      </c>
+      <c r="C233" t="str">
+        <v>Mechanical / Electrical Engineering</v>
+      </c>
+      <c r="D233" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E233" t="str">
+        <v>Tipp City, OH</v>
+      </c>
+      <c r="F233">
+        <v>750</v>
+      </c>
+      <c r="G233" t="str">
+        <v>$20–$25/hr</v>
+      </c>
+      <c r="H233" t="str">
+        <v>https://careers.regalrexnord.com/en/jobs/r26_04440/application-engineer-co-op-spring-2027/</v>
+      </c>
+      <c r="I233" t="str">
+        <v>Yes — fetched directly on Regal Rexnord's own careers.regalrexnord.com domain (retrieved twice, consistent), title states 'Application Engineer Co-op (Spring 2027)' verbatim, canApply/Apply Now button present, posted ~2026-09-18. Also resolves via Workday mirror regalrexnord.wd1.myworkdayjobs.com/Careers/job/.../Application-Engineer-Co-op--Spring-2027-_R26_04440-1.</v>
+      </c>
+      <c r="J233" t="str">
+        <v>Req R26_04440. Resolves a prior run's unverified aggregator-sourced lead for this same role/site (previously could not locate a working direct URL). Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; min GPA 3.0; basic SolidWorks/3D modeling knowledge helpful. Fully onsite, no travel. Citizenship/ITAR not stated on posting.</v>
       </c>
     </row>
   </sheetData>
@@ -9792,14 +9824,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M232"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M233"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C437"/>
+  <dimension ref="A1:C449"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -14513,7 +14545,7 @@
         <v>'2027 Spring Electrical Engineer (Controls, PCB) Co-op BS or MS', Gloucester, MA (req R2628288)</v>
       </c>
       <c r="C429" t="str">
-        <v>2026-09-28 ~07:00 UTC: a Boston-area research agent flagged this as a discipline-borderline candidate (Controls is one of Hamza's target disciplines, but the title leads with Electrical Engineer/PCB). Could not independently locate a working direct URL for this specific req within this run's time budget (site's JS-rendered search/filter pages don't expose it via plain fetch) — not added without a directly verified posting. Worth a dedicated look next run if Hamza wants Controls-adjacent EE roles considered.</v>
+        <v>2026-09-28 ~07:00 UTC: a Boston-area research agent flagged this as a discipline-borderline candidate (Controls is one of Hamza's target disciplines, but the title leads with Electrical Engineer/PCB). Could not independently locate a working direct URL for this specific req within this run's time budget (site's JS-rendered search/filter pages don't expose it via plain fetch) — not added without a directly verified posting. Worth a dedicated look next run if Hamza wants Controls-adjacent EE roles considered. RESOLVED 2026-09-28 ~13:00 UTC: independently located and directly fetched the working URL (https://jobs.appliedmaterials.com/job/gloucester/2027-spring-electrical-engineer-controls-pcb-co-op-bs-or-ms-gloucester-ma/95/100424621408 — req R2628288 confirmed embedded in the page itself, not R2628291 as a research agent's report this run mistakenly claimed). Eligibility explicitly states 'Currently enrolled in a Bachelor's or Master's degree in Electrical Engineering, Computer Engineering, or a related field' — a strict EE/CompE degree requirement, not Hamza's mechanical/aerospace background. Excluded on discipline grounds (same treatment as Entegris's EE-only Co-Ops), not on verification difficulty.</v>
       </c>
     </row>
     <row r="430">
@@ -14601,12 +14633,144 @@
         <v>'Application Engineer Co-op (Spring 2027)', Tipp City, OH</v>
       </c>
       <c r="C437" t="str">
-        <v>2026-09-28 ~07:00 UTC: multiple aggregators (Dreamwork, Workopia, zapply) describe this as a live Spring 2027 posting with a $40k-$50k range, but the employer's own careers.regalrexnord.com search is JS-rendered and no matching live req could be located directly — the closest indexed req number (R25_04222, 'Application Team Co-Op') appears to be an undated/prior-cycle listing, not confirmed as the same role. Not added without a directly verified posting; worth a targeted re-check next run now that Regal Rexnord is a known-good employer (see `rows` — Charlotte, NC Engineering Co-Op, req R26_04216, added this run).</v>
+        <v>2026-09-28 ~07:00 UTC: multiple aggregators (Dreamwork, Workopia, zapply) describe this as a live Spring 2027 posting with a $40k-$50k range, but the employer's own careers.regalrexnord.com search is JS-rendered and no matching live req could be located directly — the closest indexed req number (R25_04222, 'Application Team Co-Op') appears to be an undated/prior-cycle listing, not confirmed as the same role. Not added without a directly verified posting; worth a targeted re-check next run now that Regal Rexnord is a known-good employer (see `rows` — Charlotte, NC Engineering Co-Op, req R26_04216, added this run). RESOLVED 2026-09-28 ~13:00 UTC: correct req is R26_04440, not R25_04222 (which was a different/stale listing — five other Regal reqs found via search-cache this run, R26_02159/R26_02156/R26_02155/R25_04222/R25_05168, all 404'd on direct fetch and are presumed closed/removed). R26_04440 fetched cleanly and directly on careers.regalrexnord.com — moved to `rows`.</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B438" t="str">
+        <v>Five additional Tipp City/Fort Wayne/Florence-area req numbers surfaced via search-engine cache (R26_02159 'Mechanical Engineering Co-op (Fall 2026)', R26_02156 'Lab Co-Op (Fall 2026)', R26_02155 'Electronics Co-Op (Fall 2026)', R25_04222 'Application Team Co-Op', R25_05168 'Application Engineering Co-op')</v>
+      </c>
+      <c r="C438" t="str">
+        <v>2026-09-28 ~13:00 UTC: all five 404 on direct fetch of careers.regalrexnord.com (same domain/method that successfully confirmed R26_04216 and R26_04440 as live in the same session) — strongly indicates these are stale/removed prior-cycle listings, not a fetch glitch. Also, the three with a stated season (Fall 2026) are wrong-season regardless. Excluded.</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>WSP USA</v>
+      </c>
+      <c r="B439" t="str">
+        <v>'Mechanical Engineering Co-op – Fall 2026/Winter 2027', Philadelphia, PA (Property &amp; Buildings Team)</v>
+      </c>
+      <c r="C439" t="str">
+        <v>2026-09-28 ~13:00 UTC: explicitly restricted to Drexel University's co-op program ('as part of the Drexel Co-op Program') per the posting's own text (search snippets only — the live Oracle Cloud HCM requisition page and wsp.com/careers both blocked plain fetch, so this could not be independently opened). Excluded on eligibility grounds (school-specific placement, not open to the general applicant pool) independent of the verification difficulty; also term (Sept 22 2026 – Mar 26 2027) is ambiguous against the Winter 2026/Spring 2027 definition.</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B440" t="str">
+        <v>Internship program page (karman-sd.com/careers/internships/) re-checked directly</v>
+      </c>
+      <c r="C440" t="str">
+        <v>2026-09-28 ~13:00 UTC: page explicitly states internships 'typically begin in May or June and conclude in August or September' with an April 30 application deadline — confirmed still a single annual Summer-only cycle, no Winter/Spring 2027 mentioned. The ADP-hosted req list (karman-sd.com/job-openings/) remains JS-blocked/empty on plain fetch. No change from prior runs.</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="str">
+        <v>Parker Hannifin</v>
+      </c>
+      <c r="B441" t="str">
+        <v>parkercareers.ttcportals.com re-checked directly; two aggregator-only leads (Quality Engineering Intern, Simi Valley CA; '2027 Manufacturing Engineering Co-Op', Manitowoc WI)</v>
+      </c>
+      <c r="C441" t="str">
+        <v>2026-09-28 ~13:00 UTC: portal still returns HTTP 403 on every direct fetch attempt (root, /search/students/jobs, individual job pages) — unchanged. Neither aggregator lead could be confirmed on Parker's own domain (a site-restricted search found no matching req for the Manitowoc listing); not added. No change from prior runs.</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="str">
+        <v>Lam Research</v>
+      </c>
+      <c r="B442" t="str">
+        <v>2027 co-op cycle re-check</v>
+      </c>
+      <c r="C442" t="str">
+        <v>2026-09-28 ~13:00 UTC: confirmed the 2026 cycle's ~7 function-specific reqs all closed by mid-May 2026 and no analogous 2027-cycle reqs have posted yet; careers.lamresearch.com search remains JS-gated on plain fetch. No change from prior runs.</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B443" t="str">
+        <v>Manufacturing Engineering Co-op R5030077 (Evendale), Engines Engineering Co-op R5029617 (no '-1' suffix)</v>
+      </c>
+      <c r="C443" t="str">
+        <v>2026-09-28 ~13:00 UTC re-check: both re-confirmed dead (HTTP 410 / 'no longer posted' message) — same as multiple prior runs, no change. The tracked live req remains R5029617-1 (with suffix), unaffected. Lynn, MA's only current intern-type Workday posting is 'Engines Engineering MBSE Intern - Summer 2027' — wrong season, not added.</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B444" t="str">
+        <v>Optics-Physics Sensor Engineering Co-op (Spring 2027), JR002884</v>
+      </c>
+      <c r="C444" t="str">
+        <v>2026-09-28 ~13:00 UTC re-check: re-confirmed live (canApply true) but unchanged discipline mismatch (optics/electro-optical/EE-leaning role, same exclusion as this req's original entry earlier in this log) — not a new candidate despite a research agent this run presenting it as one.</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B445" t="str">
+        <v>Co-op Manufacturing Engineering REQ-2026-18078, Co-op R&amp;D Mechanical Engineering REQ-2026-18007, Co-op Life Cycle Engineering-Systems REQ-2026-18149, Co-op Systems Engineering REQ-2026-18061</v>
+      </c>
+      <c r="C445" t="str">
+        <v>2026-09-28 ~13:00 UTC: a research agent presented these four as newly-found Jan-June 2027 siblings, but all four are already tracked in `rows` from prior runs (confirmed by direct grep of existing Application Link URLs) — no new rows added. A fifth, unconfirmed lead ('Co-op, Life Cycle Engineering - Electrical') was mentioned via search only, not independently fetched — EE-focused, likely discipline mismatch regardless.</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B446" t="str">
+        <v>Healthcare Mechanical Engineering Co-op (Spring), req R266691; older reqs R244191/R244210</v>
+      </c>
+      <c r="C446" t="str">
+        <v>2026-09-28 ~13:00 UTC re-check: R266691's internal season contradiction (body states both 'June through December' and 'January through June' with no year stated) re-confirmed unchanged from the 2026-09-28 ~01:00 UTC exclusion — still excluded. R244191/R244210 return zero results on ADI's live Workday board (likely closed/stale, lower req numbers than R266691) — not independently confirmed dead via a definitive signal (no HTTP 410/closed-message check performed), not added regardless since no live posting located.</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="str">
+        <v>National fresh-pass negative results, 2026-09-28 ~13:00 UTC</v>
+      </c>
+      <c r="B447" t="str">
+        <v>Barnes Group/Barnes Aerospace, Triumph Group, ATI (Allegheny Technologies), Meggitt/Parker Aerospace, Woodward Inc., Moog Inc. (beyond tracked sites), Oshkosh Corporation/Oshkosh Defense, Kennametal, AMETEK, Dover Corporation (incl. CPC/Colder Products), Terex Corporation, IDEX Corporation, FANUC America, Yaskawa America, KUKA Robotics USA</v>
+      </c>
+      <c r="C447" t="str">
+        <v>No qualifying Winter 2026/Spring 2027 mechanical/aerospace/manufacturing/robotics/structural/controls co-op or intern posting found for any of these on a fresh pass. Most career sites are JS-rendered and returned empty shells on plain fetch (flagged as unverifiable rather than assumed closed); where content was accessible, postings found were either wrong-discipline (Terex Software Engineer Co-Op, IDEX/FANUC/KUKA non-qualifying or not located), wrong-season (Woodward and Yaskawa both explicitly 'Summer 2027' only), or season-ambiguous with no explicit Winter/Spring 2027 text (Flowserve's Houston, TX 'Engineering Co-op' — real, apparently open req, but posting never states a season; Kennametal, AMETEK — rolling/ASAP start, no season stated). None added without a directly verified, dated posting.</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="str">
+        <v>Boston-area fresh-pass negative results, 2026-09-28 ~13:00 UTC</v>
+      </c>
+      <c r="B448" t="str">
+        <v>Locus Robotics (Wilmington, MA), Vicor Corporation (Andover, MA), Instron/ITW (Norwood, MA), Analogic (Peabody, MA), Boston Metal (Woburn, MA), Desktop Metal (Burlington, MA), Markforged (Waltham, MA), Vecna Robotics (Waltham, MA), National Instruments/Emerson, Nuvation Engineering, Charles River Laboratories (Wilmington, MA)</v>
+      </c>
+      <c r="C448" t="str">
+        <v>No qualifying co-op/intern posting found for any of these. Locus Robotics confirmed via direct Greenhouse API fetch: only 6 open roles company-wide, none co-op/intern (two previously-cached internship req IDs no longer resolve — closed). Vicor: 17 open roles, all full-time/permanent, no co-op/intern. The rest returned no specific mechanical/manufacturing engineering co-op lead via search or direct fetch (several JS-gated, could not verify beyond search snippets).</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="str">
+        <v>Skyworks Solutions (Andover, MA)</v>
+      </c>
+      <c r="B449" t="str">
+        <v>'Analog Design Winter/Spring Co-Op (Jan-June '27)'</v>
+      </c>
+      <c r="C449" t="str">
+        <v>2026-09-28 ~13:00 UTC: confirmed live via WebFetch (Apply Now button present, strong season/pay match: 'Winter/Spring 2027 Co-Op Term (Jan 2027 – June 2027)', $26-$47.50/hr) but requires 'currently enrolled in an Electrical Engineering BS or MS/PhD program' for analog IC design work — outside Hamza's target disciplines (not mechanical/aerospace/manufacturing/robotics/industrial/materials/structural/controls). Not added; flagging as a new company with a strong season match in case Skyworks becomes relevant for a different discipline focus.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C437"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C449"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 12 checked-excluded (2026-09-28 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FEPNYHkhTAFVYQYhEZNkyy
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M233"/>
+  <dimension ref="A1:M238"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9348,6 +9348,166 @@
       </c>
       <c r="J233" t="str">
         <v>Req R26_04440. Resolves a prior run's unverified aggregator-sourced lead for this same role/site (previously could not locate a working direct URL). Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; min GPA 3.0; basic SolidWorks/3D modeling knowledge helpful. Fully onsite, no travel. Citizenship/ITAR not stated on posting.</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="str">
+        <v>Skyworks Solutions</v>
+      </c>
+      <c r="B234" t="str">
+        <v>Microelectronics / Semiconductor Packaging Co-Op</v>
+      </c>
+      <c r="C234" t="str">
+        <v>Mechanical / Chemical / Materials Science / Industrial Engineering</v>
+      </c>
+      <c r="D234" t="str">
+        <v>Winter/Spring Co-Op, January 2027 – June 2027</v>
+      </c>
+      <c r="E234" t="str">
+        <v>Nashua, NH</v>
+      </c>
+      <c r="F234">
+        <v>40</v>
+      </c>
+      <c r="G234" t="str">
+        <v>$26.00–$47.50/hr</v>
+      </c>
+      <c r="H234" t="str">
+        <v>https://careers.skyworksinc.com/job/Nashua-Microelectronics-Semiconductor-Packaging-Co-Op-NH-03060/78294-en_US/</v>
+      </c>
+      <c r="I234" t="str">
+        <v>Yes — fetched directly (WebFetch), req ID 78294 embedded in page, active 'Apply now' button present, posted 2026-09-14, quote: 'This is for a Winter/Spring Coop from January 2027 - June 2027.'</v>
+      </c>
+      <c r="J234" t="str">
+        <v>Req 78294. Discovered via Skyworks' own public sitemap.xml. Unlike every other Skyworks co-op tracked so far (all EE-only), this one explicitly also accepts Mechanical/Chemical/Materials Science/Industrial Engineering majors — packaging-materials evaluation (adhesives, mold compounds, substrates, underfills, TIMs), failure analysis, DOE. Junior/Senior standing or current grad student. No citizenship/ITAR language stated. Preferred (not required) skills: SolidWorks/Creo/AutoCAD, Minitab/JMP/MATLAB/Python.</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B235" t="str">
+        <v>Application Team Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C235" t="str">
+        <v>Mechanical / Electrical Engineering</v>
+      </c>
+      <c r="D235" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E235" t="str">
+        <v>Tipp City, OH</v>
+      </c>
+      <c r="F235">
+        <v>750</v>
+      </c>
+      <c r="G235" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H235" t="str">
+        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Tipp-City-Ohio-United-States/Application-Team-Co-Op--Spring-2027-_R26_04736-1</v>
+      </c>
+      <c r="I235" t="str">
+        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Application Team Co-Op (Spring 2027)' verbatim, posted 3 days ago (2026-09-25), no filled/closed language.</v>
+      </c>
+      <c r="J235" t="str">
+        <v>Req R26_04736. New req at the same Tipp City, OH site as the already-tracked R26_04440 'Application Engineer Co-op' — distinct responsibilities (mechanical/electrical design support, CAD detail drawings, 3D-printer lab support) not a duplicate. Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; GPA 3.0+; basic SolidWorks/3D modeling knowledge. Fully onsite. Citizenship/ITAR not stated on posting.</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B236" t="str">
+        <v>Sound Lab Co-op (Spring 2027)</v>
+      </c>
+      <c r="C236" t="str">
+        <v>Mechanical / Electrical Engineering (acoustics &amp; vibration testing)</v>
+      </c>
+      <c r="D236" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E236" t="str">
+        <v>Fort Wayne, IN</v>
+      </c>
+      <c r="F236">
+        <v>830</v>
+      </c>
+      <c r="G236" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H236" t="str">
+        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Fort-Wayne-Indiana-United-States/Sound-Lab-Co-op--Spring-2027-_R26_04469-2</v>
+      </c>
+      <c r="I236" t="str">
+        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Sound Lab Co-op (Spring 2027)' verbatim, posted 5 days ago (2026-09-23), no filled/closed language.</v>
+      </c>
+      <c r="J236" t="str">
+        <v>Req R26_04469. Anechoic chamber / sound &amp; vibration analysis for customer returns, cost-reduction, and new-product-development testing. Currently pursuing a Bachelor's in Mechanical or Electrical Engineering. Fully onsite. Citizenship/ITAR not stated on posting.</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="str">
+        <v>Crane Company (Crane Pumps &amp; Systems)</v>
+      </c>
+      <c r="B237" t="str">
+        <v>Engineering Co-op Spring 2027-1</v>
+      </c>
+      <c r="C237" t="str">
+        <v>Mechanical / Electrical Engineering</v>
+      </c>
+      <c r="D237" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E237" t="str">
+        <v>Piqua, OH</v>
+      </c>
+      <c r="F237">
+        <v>750</v>
+      </c>
+      <c r="G237" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H237" t="str">
+        <v>https://cranecompany.wd5.myworkdayjobs.com/Careers/job/Piqua-Ohio/Engineering-Co-op-Spring-2027-1_JR102521</v>
+      </c>
+      <c r="I237" t="str">
+        <v>Yes — fetched directly via Crane Company's own Workday CXS API for all three parallel req IDs (JR102518, JR102520, JR102521), identical title 'Engineering Co-op Spring 2027-1', posted 14 days ago (2026-09-14), no filled/closed language on any.</v>
+      </c>
+      <c r="J237" t="str">
+        <v>New company for the tracker. 3 parallel open headcount at the same Piqua, OH site under reqs JR102518, JR102520, and JR102521 (all independently confirmed live) — general engineering support (product design, CAD documentation, lab/test support) for pump products serving industrial/commercial/residential/municipal/military markets. Working toward a B.S. in Mechanical, Mechanical Tech, or Electrical Engineering. This is the Pumps &amp; Systems division (not Crane Aerospace &amp; Electronics, which has a separate ITAR-restricted, season-ambiguous posting — excluded, see `checked`). Citizenship/ITAR not stated on this posting.</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B238" t="str">
+        <v>Mechanical Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C238" t="str">
+        <v>Mechanical Engineering (manufacturing/process engineering)</v>
+      </c>
+      <c r="D238" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E238" t="str">
+        <v>Libertyville, IL</v>
+      </c>
+      <c r="F238">
+        <v>990</v>
+      </c>
+      <c r="G238" t="str">
+        <v>$27.50–$44.50/hr</v>
+      </c>
+      <c r="H238" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/Mechanical-Engineering-Co-Op---Spring-2027_WD229697</v>
+      </c>
+      <c r="I238" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229697, posted 10 days ago (2026-09-18), quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 co-op assignment.'</v>
+      </c>
+      <c r="J238" t="str">
+        <v>New company for the tracker. Manufacturing/process-engineering support — time studies, CAD, DOE projects, Lean/Six Sigma. Current BS/MS student pursuing Mechanical Engineering; 2D/3D CAD (AutoCAD/Inventor/Solidworks); GPA 3.0+. Posting explicitly states 'Is Sponsorship Available? No' (no visa sponsorship — not a citizenship/ITAR requirement).</v>
       </c>
     </row>
   </sheetData>
@@ -9824,14 +9984,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M233"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M238"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C449"/>
+  <dimension ref="A1:C461"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -14768,9 +14928,141 @@
         <v>2026-09-28 ~13:00 UTC: confirmed live via WebFetch (Apply Now button present, strong season/pay match: 'Winter/Spring 2027 Co-Op Term (Jan 2027 – June 2027)', $26-$47.50/hr) but requires 'currently enrolled in an Electrical Engineering BS or MS/PhD program' for analog IC design work — outside Hamza's target disciplines (not mechanical/aerospace/manufacturing/robotics/industrial/materials/structural/controls). Not added; flagging as a new company with a strong season match in case Skyworks becomes relevant for a different discipline focus.</v>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" t="str">
+        <v>Skyworks Solutions (Woburn, MA)</v>
+      </c>
+      <c r="B450" t="str">
+        <v>'Quality Systems Data Analyst Winter/Spring Co-Op', req 78511</v>
+      </c>
+      <c r="C450" t="str">
+        <v>2026-09-28 ~19:00 UTC: confirmed live (Jan-June 2027, $26-$47.50/hr), and Industrial Engineering is technically among the listed acceptable majors, but the actual work described is Power BI/SharePoint/Salesforce data-analytics and business-process support, not engineering design/test work. Same judgment call as the existing Berkshire Grey 'Robot Learning' precedent — flagged for Hamza's own call rather than auto-included or auto-excluded; not added to `rows` this run.</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="str">
+        <v>Kairos Power</v>
+      </c>
+      <c r="B451" t="str">
+        <v>All 5 current internship postings (Chemical &amp; Materials, Civil, Electrical, Mechanical &amp; Manufacturing, Nuclear Engineering) — Alameda CA / Albuquerque NM / Oak Ridge TN</v>
+      </c>
+      <c r="C451" t="str">
+        <v>2026-09-28 ~19:00 UTC: independently re-confirmed via direct fetch of Kairos's Greenhouse board (job-boards.greenhouse.io/kairospower) — all 10 season mentions found are 'Summer 2027', zero Winter 2026/Spring 2027 postings exist. New company for the tracker; wrong season across the board.</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="str">
+        <v>Watts Water Technologies (North Andover, MA)</v>
+      </c>
+      <c r="B452" t="str">
+        <v>Full company-wide Workday board (252 postings) queried directly via CXS API; workerSubType facet check</v>
+      </c>
+      <c r="C452" t="str">
+        <v>2026-09-28 ~19:00 UTC: zero Intern/Co-Op category jobs exist on their live board — only 'Regular' and 'Contractor' worker types present, and a direct 'Spring 2027' search returned 0 results. Stale aggregator snippets (LinkedIn 'Manufacturing Engineer Co-Op', BeBee 'Trade Compliance Analyst Co-Op, Spring 2027') do not correspond to any currently-live posting. Excluded — no live posting to verify.</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="str">
+        <v>Ameren (St. Louis, MO)</v>
+      </c>
+      <c r="B453" t="str">
+        <v>'Mechanical Engineering Spring Co-Op', req 031778-1</v>
+      </c>
+      <c r="C453" t="str">
+        <v>2026-09-28 ~19:00 UTC: aggregator mirrors describe a 2027 Mechanical Engineering Spring Co-Op but give conflicting pay ranges ($21-$30/hr vs $19-$29/hr) and one mirror lists an already-passed Dec 19, 2025 application deadline, suggesting possibly stale/prior-cycle content. Ameren's own Workday CXS API (ameren.wd1.myworkdayjobs.com) returned HTTP 403 on every direct-fetch attempt — genuinely unverifiable with current tooling. Not added; worth a dedicated re-check with different tooling/timing.</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>Arkwin Industries (TransDigm subsidiary, Bethpage, NY)</v>
+      </c>
+      <c r="B454" t="str">
+        <v>Search snippets claiming Spring/Fall 2027 co-op postings</v>
+      </c>
+      <c r="C454" t="str">
+        <v>2026-09-28 ~19:00 UTC: a direct fetch of arkwin.com's own job listing page (page 1 of 17) shows no co-op/intern posting among current openings — could not independently confirm the search-snippet claim. Not added. TransDigm has 50+ independently-hiring subsidiaries; a full sweep is out of scope for a single run's budget.</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>Crane Aerospace &amp; Electronics (Elyria, OH)</v>
+      </c>
+      <c r="B455" t="str">
+        <v>'Engineering Co-op', req JR102436</v>
+      </c>
+      <c r="C455" t="str">
+        <v>2026-09-28 ~19:00 UTC: confirmed live and open (canApply true) via direct Workday fetch, but the posting never states a season anywhere in its text (same treatment as the standing Flowserve/Woodward/Moog exclusions for season-ambiguous postings) and explicitly requires U.S. Persons/ITAR compliance. Distinct from the same parent company's Crane Pumps &amp; Systems division (Piqua, OH — see `rows`, new company this run), which is not ITAR-restricted.</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
+        <v>Flowserve</v>
+      </c>
+      <c r="B456" t="str">
+        <v>Req R-17161 ('Rotating Equipment Engineer Co-Op / Operations Intern', West Chicago, IL per aggregator, Jan-Aug 2026 span)</v>
+      </c>
+      <c r="C456" t="str">
+        <v>2026-09-28 ~19:00 UTC: direct fetch of the Workday page shell shows 'postingAvailable': false — this req is now closed. Also wrong year (2026) regardless.</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="str">
+        <v>Flowserve (Houston, TX)</v>
+      </c>
+      <c r="B457" t="str">
+        <v>'Engineering Co-op' (via Intern Insider aggregator mirror), apply-by Oct 9 deadline</v>
+      </c>
+      <c r="C457" t="str">
+        <v>2026-09-28 ~19:00 UTC re-check: still states no season anywhere ('Season/Term: Rolling (no specific season mentioned)') — unchanged from prior finding. Could not independently locate this specific req's live Workday URL this run (Flowserve's CXS search endpoint returns noisy, unfiltered results for multi-word queries). Still excluded, season-ambiguous.</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B458" t="str">
+        <v>R25_00369 (Milwaukee Engineering Co-Op), R24_01240 (Florence, KY Manufacturing Engineering Co-Op)</v>
+      </c>
+      <c r="C458" t="str">
+        <v>2026-09-28 ~19:00 UTC: both re-confirmed 404 on direct fetch — stale/removed prior-cycle reqs, consistent with the five other dead Regal Rexnord reqs found in the 2026-09-28 ~13:00 UTC run.</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="str">
+        <v>SharkNinja (Needham, MA)</v>
+      </c>
+      <c r="B459" t="str">
+        <v>Full re-check of current postings</v>
+      </c>
+      <c r="C459" t="str">
+        <v>2026-09-28 ~19:00 UTC re-check: still only Fall 2026 ('Fall 2026: Mechanical Engineering Co-op, Ninja, July to December') and undated/Summer 2027 intern postings — no Spring 2027 posting has appeared. Unchanged from prior runs.</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B460" t="str">
+        <v>Healthcare Mechanical Engineering Co-op (Spring), req R266691</v>
+      </c>
+      <c r="C460" t="str">
+        <v>2026-09-28 ~19:00 UTC re-check: re-fetched full description directly from ADI's own Workday CXS API — still contains the same internal contradiction ('June through December' vs. a qualifications line stating 'January through June', no year stated anywhere). canApply true, re-posted/refreshed 3 days ago but text unchanged. Still excluded on season-ambiguity grounds.</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="str">
+        <v>Boston-area fresh-pass negative/unresolved results, 2026-09-28 ~19:00 UTC</v>
+      </c>
+      <c r="B461" t="str">
+        <v>Sensata Technologies (Attleboro, MA), Harmonic Drive LLC (Peabody, MA), ClearMotion (Woburn, MA), QinetiQ North America / Foster-Miller (Waltham, MA), MilliporeSigma (Burlington, MA), 6 River Systems / Ocado Group (Waltham, MA), Vention</v>
+      </c>
+      <c r="C461" t="str">
+        <v>No qualifying Winter 2026/Spring 2027 co-op found for any. Confirmed no current postings (not just blocked): Sensata (full Workday sitemap fetched directly — only Summer 2027 engineering interns exist, none at Attleboro or Winter/Spring 2027), Harmonic Drive (Paylocity board fetched directly — only 8 open reqs, all technician/admin/trade, no engineering co-op), ClearMotion (careers page has no active job listings at all right now). Blocked/unresolved rather than confirmed dead: QinetiQ's iCIMS board blocks automated keyword search (HTTP 405) and its marketing site is JS-rendered with no server-side job listings; MilliporeSigma's intern hiring is outsourced to a third-party staffing agency (Randstad Sourceright), no specific posting locatable; Ocado's internship page has nothing dated Winter/Spring 2027 or Boston-located; Vention has no Boston-area posting found via search at all. Worth a manual/headless-browser look at QinetiQ specifically in a future run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C449"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C461"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 6 new postings, 15 checked-excluded (2026-09-29 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NHBDe5i9jHGSiyQprWr2NT
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M238"/>
+  <dimension ref="A1:M244"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9508,6 +9508,198 @@
       </c>
       <c r="J238" t="str">
         <v>New company for the tracker. Manufacturing/process-engineering support — time studies, CAD, DOE projects, Lean/Six Sigma. Current BS/MS student pursuing Mechanical Engineering; 2D/3D CAD (AutoCAD/Inventor/Solidworks); GPA 3.0+. Posting explicitly states 'Is Sponsorship Available? No' (no visa sponsorship — not a citizenship/ITAR requirement).</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B239" t="str">
+        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
+      </c>
+      <c r="C239" t="str">
+        <v>Mechanical Engineering / Aerospace Engineering</v>
+      </c>
+      <c r="D239" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E239" t="str">
+        <v>Lexington, MA</v>
+      </c>
+      <c r="F239">
+        <v>11</v>
+      </c>
+      <c r="G239" t="str">
+        <v>$25–$32/hr (Technical Co-Op, based on year in school)</v>
+      </c>
+      <c r="H239" t="str">
+        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
+      </c>
+      <c r="I239" t="str">
+        <v>Yes — fetched directly (server-rendered SAP SuccessFactors page, not JS-gated), req ID 1434254300, posted 2026-09-28, title states '(Winter/Spring 2027)' verbatim.</v>
+      </c>
+      <c r="J239" t="str">
+        <v>Requisition ID 43350. Open to Mechanical Engineering, Aeronautics/Astronautics, Aerospace Engineering, or Physics majors (must have completed Mechanics of Materials or equivalent); CAD/FEA/prototyping preferred, not required. Requires U.S. citizenship and eligibility for a Secret-level DoD security clearance. Distinct from the already-tracked Microfabrication (Group 08-35) co-ops. Apply at https://careers.ll.mit.edu/talentcommunity/apply/1434254300/?locale=en_US</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="str">
+        <v>DEKA Research &amp; Development</v>
+      </c>
+      <c r="B240" t="str">
+        <v>Systems Engineer Co-Op - Spring 2027</v>
+      </c>
+      <c r="C240" t="str">
+        <v>Bioengineering / Biomedical / Mechanical Engineering</v>
+      </c>
+      <c r="D240" t="str">
+        <v>Spring 2027 (starting January 2027)</v>
+      </c>
+      <c r="E240" t="str">
+        <v>Manchester, NH</v>
+      </c>
+      <c r="F240">
+        <v>50</v>
+      </c>
+      <c r="G240" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H240" t="str">
+        <v>https://deka.applytojob.com/apply/76ReoonYrJ/Systems-Engineer-CoOp-Spring-2027</v>
+      </c>
+      <c r="I240" t="str">
+        <v>Yes — fetched directly (JazzHR-hosted, server-rendered, not JS-gated), full description read. Quote: 'This position is for a 6+ month rotation for the Spring semester starting in January 2027.'</v>
+      </c>
+      <c r="J240" t="str">
+        <v>New company for the tracker — DEKA is Dean Kamen's medical-device/robotics R&amp;D house (insulin pumps, robotic arms, water purification, etc.), Manchester, NH. Open to undergraduate Bioengineering, Biomedical, or Mechanical Engineering majors; graduate students NOT eligible for this specific req. Closing date and GPA requirement not stated. A separate 'Software Engineering Co-Op - Spring 2027' req also exists at the same company but is out of scope (software discipline).</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B241" t="str">
+        <v>Automation/Controls Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C241" t="str">
+        <v>Electrical Engineering / Mechatronics / Automation Engineering (Controls)</v>
+      </c>
+      <c r="D241" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E241" t="str">
+        <v>Libertyville, IL</v>
+      </c>
+      <c r="F241">
+        <v>990</v>
+      </c>
+      <c r="G241" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H241" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Automation-Controls-Engineering-Co-Op---Spring-2027_WD229698</v>
+      </c>
+      <c r="I241" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229698, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+      </c>
+      <c r="J241" t="str">
+        <v>Electrical Engineering, Mechatronics, or Automation Engineering major. PLC/HMI programming, FAT/SAT testing. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B242" t="str">
+        <v>Robotics/Mechatronics Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C242" t="str">
+        <v>Mechanical / Mechatronics / Robotics Engineering</v>
+      </c>
+      <c r="D242" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E242" t="str">
+        <v>Libertyville, IL</v>
+      </c>
+      <c r="F242">
+        <v>990</v>
+      </c>
+      <c r="G242" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H242" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Robotics-Mechatronics-Engineering-Co-Op---Spring-2027_WD229699</v>
+      </c>
+      <c r="I242" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229699, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+      </c>
+      <c r="J242" t="str">
+        <v>Robot path optimization, AMR/ASRS validation, machine-vision systems. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B243" t="str">
+        <v>Plastic Molding Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C243" t="str">
+        <v>Materials / Manufacturing Engineering (Plastics)</v>
+      </c>
+      <c r="D243" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E243" t="str">
+        <v>Libertyville, IL</v>
+      </c>
+      <c r="F243">
+        <v>990</v>
+      </c>
+      <c r="G243" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H243" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Plastic-Molding-Engineering-Co-Op---Spring-2027_WD229696</v>
+      </c>
+      <c r="I243" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229696, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+      </c>
+      <c r="J243" t="str">
+        <v>Plastics Engineering major, injection-molding/materials/manufacturing focus. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B244" t="str">
+        <v>Industrial Engineering Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C244" t="str">
+        <v>Industrial Engineering</v>
+      </c>
+      <c r="D244" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E244" t="str">
+        <v>Orangeburg, SC</v>
+      </c>
+      <c r="F244">
+        <v>810</v>
+      </c>
+      <c r="G244" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H244" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Industrial-Engineering-Co-Op---Fall-2026_WD226357</v>
+      </c>
+      <c r="I244" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226357, posted 2026-09-03, canApply true. NOTE: title and body text both explicitly say '(Spring 2027)' ('...looking to add an Industrial Engineering Co-Op (Spring 2027)...'), but the URL slug itself reads 'Fall-2026' — an apparent leftover from an earlier req rename. Treating the in-body/title season text as authoritative per the verification bar.</v>
+      </c>
+      <c r="J244" t="str">
+        <v>Fulfillment/server-assembly warehouse operations, Lean/Six Sigma. Two sibling reqs at the same Orangeburg, SC site (Quality Engineering Co-Op, Program Management Co-Op) have the same title/URL-slug season discrepancy but are non-target disciplines — see `checked`. Pay/citizenship not stated.</v>
       </c>
     </row>
   </sheetData>
@@ -9984,14 +10176,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M238"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M244"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C461"/>
+  <dimension ref="A1:C476"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -15060,9 +15252,174 @@
         <v>No qualifying Winter 2026/Spring 2027 co-op found for any. Confirmed no current postings (not just blocked): Sensata (full Workday sitemap fetched directly — only Summer 2027 engineering interns exist, none at Attleboro or Winter/Spring 2027), Harmonic Drive (Paylocity board fetched directly — only 8 open reqs, all technician/admin/trade, no engineering co-op), ClearMotion (careers page has no active job listings at all right now). Blocked/unresolved rather than confirmed dead: QinetiQ's iCIMS board blocks automated keyword search (HTTP 405) and its marketing site is JS-rendered with no server-side job listings; MilliporeSigma's intern hiring is outsourced to a third-party staffing agency (Randstad Sourceright), no specific posting locatable; Ocado's internship page has nothing dated Winter/Spring 2027 or Boston-located; Vention has no Boston-area posting found via search at all. Worth a manual/headless-browser look at QinetiQ specifically in a future run.</v>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="str">
+        <v>Ameren (St. Louis, MO)</v>
+      </c>
+      <c r="B462" t="str">
+        <v>Mechanical Engineering Spring Co-Op, req 034022 (resolves prior unverifiable req 031778-1)</v>
+      </c>
+      <c r="C462" t="str">
+        <v>2026-09-29: resolved prior 403 block by hitting Ameren's Workday CXS API directly (ameren.wd1.myworkdayjobs.com) instead of the WAF-blocked marketing site. Confirmed live: canApply true, endDate 2026-12-28, pay $21.00–$30.00/hr, 'January – August Co-Op' window (Winter 2026/Spring 2027 season). NOT added to `rows` despite being fully accessible: the posting's title says 'Mechanical Engineering' but its own Qualifications section states 'Must be a current student pursuing a Bachelors or Masters in Electrical Engineering' — an internal title/qualifications contradiction (likely a copy-paste template error, same pattern as the already-excluded Analog Devices R266691). Cannot confirm mechanical-engineering students are actually eligible; flagged for Hamza's own judgment/direct confirmation with Ameren recruiting rather than guessed either way.</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="str">
+        <v>QinetiQ North America / Foster-Miller (Waltham, MA)</v>
+      </c>
+      <c r="B463" t="str">
+        <v>Full current open-req list (76 reqs) via careers-qinetiqus.icims.com/sitemap.xml</v>
+      </c>
+      <c r="C463" t="str">
+        <v>2026-09-29: resolved the standing access block — the previously-tried qinetiq-na.icims.com domain is dead (HTTP 410); the live ATS is careers-qinetiqus.icims.com, whose sitemap.xml lists all open reqs without triggering the search-endpoint bot-block. Scanned all 76 current titles: mechanical/aerospace-relevant reqs exist (Senior/Principal/Associate Mechanical Engineer, UGV Systems Engineering SME) but all are experienced-hire roles — zero co-op/intern/student titles currently open. Worth re-checking with this sitemap method periodically.</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="str">
+        <v>Draper Laboratory / GE Aerospace (Lynn, MA) / MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B464" t="str">
+        <v>Periodic full re-sweep via each employer's own Workday CXS API (Draper, GE) and server-rendered search (MIT LL)</v>
+      </c>
+      <c r="C464" t="str">
+        <v>2026-09-29: Draper — no reqs found beyond the three already tracked (JR002882, JR002883, JR002942) plus already-excluded Electrical Engineering Co-Op (JR002941); fully saturated, no change. GE Aerospace Lynn, MA — only student-eligible posting is 'Product Definition Engineering Intern - Summer 2027' (R5039185, wrong season) plus non-engineering trade Trainee Co-Ops; company-wide Spring 2027 slate remains the already-tracked Evendale-based reqs (R5029617-1, R5029663), no Lynn-specific new req. MIT Lincoln Laboratory — see the new Group 07-71 Mechanical Engineering Co-Op (req 43350) added to `rows` this run; no other new in-discipline Winter/Spring 2027 req found beyond that and the already-tracked microfab co-ops.</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>CIRCOR International (Burlington, MA) / MACOM Technology Solutions (Lowell, MA) / Teledyne FLIR (Billerica, MA) / Smith+Nephew (Andover, MA)</v>
+      </c>
+      <c r="B465" t="str">
+        <v>Fresh Boston-area pass, 2026-09-29</v>
+      </c>
+      <c r="C465" t="str">
+        <v>CIRCOR — circor.jobs.net is Cloudflare-bot-blocked (403 even on robots.txt); no alternate ATS found; Google's index shows no co-op/intern postings, but unresolved/likely-nothing rather than confirmed. MACOM — Cornerstone OnDemand SPA (macomtech.csod.com), API calls unauthorized, WebFetch returned empty (client-rendered); Google's index surfaced 5 open internship-titled reqs (#2589, 2606, 2611, 2612, 2623) but season/discipline could not be confirmed — inconclusive, not added. Teledyne FLIR — clean Workday CXS sweep, all current student postings company-wide (including 26 open Billerica, MA reqs) are Summer 2027 only, zero Winter/Spring 2027 co-ops. Smith+Nephew — clean Workday CXS sweep of the Andover, MA site, only 5 open reqs there, all senior/staff/director-level, zero co-ops live; a previously-surfaced 'Co-Op Engineering' req (R87751) now returns 403/permission-denied on direct API fetch, consistent with expired.</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B466" t="str">
+        <v>Manufacturing Data &amp; Analytics Co-Op - Spring 2027, Libertyville IL, req WD229700</v>
+      </c>
+      <c r="C466" t="str">
+        <v>2026-09-29: confirmed live and in-season (Spring 2027) via direct Workday CXS fetch, but the role is OEE/SPC/Power BI/SQL/Python data-analytics work, not a core mechanical/aerospace/manufacturing-engineering discipline — discipline-borderline, flagged for Hamza's own judgment rather than added to `rows` (same treatment as the Skyworks Woburn Quality Systems Data Analyst precedent).</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B467" t="str">
+        <v>Quality Engineering Co-Op and Program Management Co-Op, Orangeburg SC (same site/season-title pattern as the new Industrial Engineering Co-Op added to `rows`)</v>
+      </c>
+      <c r="C467" t="str">
+        <v>2026-09-29: both share the same 'title says Spring 2027, URL slug says Fall-2026' pattern, but are wrong discipline (Quality/Program Management, not core engineering) — not added regardless of the season resolution.</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B468" t="str">
+        <v>Mechanical Engineering Co-op (WD226382), Electrical Engineering Co-op (WD226386), NPI Process Engineering Co-op (WD226387) — Hollis, NH</v>
+      </c>
+      <c r="C468" t="str">
+        <v>2026-09-29: posted 2026-07-30, body states a 'Jan – Jun 2027' assignment window (effectively Spring 2027) but the TITLE itself states no season/year at all, failing the strict season-from-posting bar on its own; additionally the Mechanical Engineering req's own metadata shows a Job Posting End Date of 08-05-2026 — already past as of today — despite canApply still reading true, a genuine staleness red flag. Not added; worth a fresh direct look next run given Hollis, NH is a Boston-area (~45 mi) location if the data cleans up.</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B469" t="str">
+        <v>Application Engineering Co-Op (Spring), Fort Wayne IN, req R26_04115</v>
+      </c>
+      <c r="C469" t="str">
+        <v>2026-09-29: confirmed live via direct fetch (canApply true, posted 2026-09-23), COPRA/FFU blower testing/troubleshooting work — but the title states only '(Spring)' with no year anywhere in the title or body, and no qualifications/GPA/pay text is present either. Very likely Spring 2027 given sibling reqs at the same Fort Wayne/Tipp City sites from the same period, but cannot cite an explicit year quote from the posting itself — excluded per the strict season-confirmation bar rather than assumed.</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B470" t="str">
+        <v>Manufacturing Engineering Co-Op (R26_00665), Manufacturing Supply Chain Co-Op (R26_05084), Supply Chain Co-Op (R26_02200) — all Florence, KY</v>
+      </c>
+      <c r="C470" t="str">
+        <v>2026-09-29: R26_00665 states no season anywhere in the body and reads like a stale rolling template (posted 2026-07-16, references unrelated 'Emerson Ethics and Safety Programs' boilerplate) — same treatment as standing Flowserve/Woodward/Moog no-season exclusions. R26_05084 and R26_02200 are Supply Chain discipline, not engineering — wrong discipline regardless of season.</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="str">
+        <v>Crane Company (Crane Pumps &amp; Systems)</v>
+      </c>
+      <c r="B471" t="str">
+        <v>Engineering Co-Op Summer 2027 — 3 new sibling reqs (JR102640, JR102641, JR102642) at the same Piqua, OH site as the already-tracked Spring 2027 reqs</v>
+      </c>
+      <c r="C471" t="str">
+        <v>2026-09-29: posted today, identical job description to the tracked Spring reqs, but explicitly titled 'Summer 2027' — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="str">
+        <v>Allison Transmission / Xylem / AeroVironment / The Nuclear Company</v>
+      </c>
+      <c r="B472" t="str">
+        <v>Fresh untried-company national pass, 2026-09-29</v>
+      </c>
+      <c r="C472" t="str">
+        <v>Allison Transmission — Workday sweep (90 jobs), only Summer 2027 intern titles (Service/Product Engineering), wrong season. Xylem — Workday sweep (531 jobs), zero US engineering intern/co-op postings currently open, any season. AeroVironment — Workday sweep, all Intern-titled reqs are structurally part of a Summer Internship Program (explicitly 'Summer 2027' where dated) — no Winter/Spring track exists, same pattern as Karman. The Nuclear Company (Greenhouse board, new fast-growing nuclear-energy company — energy/nuclear fits Hamza's target category) — its 'TNC Nuclear Interns 2027' (Columbia, SC) is explicitly Summer 2027; its Spring 2027 postings are all software/AI/data-science discipline, not target disciplines. Worth a future re-check in case a Spring/Winter mechanical or nuclear-engineering co-op track opens.</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="str">
+        <v>Siemens</v>
+      </c>
+      <c r="B473" t="str">
+        <v>'Automation Engineer Co-Op - Spring 2027 (UT Arlington)', Grand Prairie, TX — aggregator-sourced lead</v>
+      </c>
+      <c r="C473" t="str">
+        <v>2026-09-29: would be a strong controls-discipline fit ($30–33/hr, Jan–May/Aug 2027) if real, but Siemens' own career site (jobs.siemens.com, Avature-based) loads job data via a JS-executed API not queryable via direct fetch — could not independently confirm the posting exists or its details. NOT added without direct verification; worth a dedicated headless-browser follow-up.</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B474" t="str">
+        <v>'Mechanical Engineering Co-Op' req R2496, surfaced via web search</v>
+      </c>
+      <c r="C474" t="str">
+        <v>2026-09-29: not found among already-tracked reqs by this ID; direct Workday fetch returned HTTP 403 this run (site-level block observed only on this tenant, not a general proxy issue) — could not read title/season/location to confirm anything about it. Possibly a new req; needs a follow-up attempt next run rather than being asserted as new or dismissed.</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="str">
+        <v>Karman Space &amp; Defense / Parker Hannifin / Lam Research / Waters Corporation / Moog Inc.</v>
+      </c>
+      <c r="B475" t="str">
+        <v>One light re-check attempt each, 2026-09-29</v>
+      </c>
+      <c r="C475" t="str">
+        <v>Karman — karmanspace.com unreachable this run (DNS/proxy failures), no reason to doubt the repeatedly-confirmed Summer-only finding, status unchanged. Parker Hannifin — jobs.parker.com/www.parker.com still unreachable/403, unchanged. Lam Research — lamresearch.com/careers/students/ now 404s (site restructured), redirect not chased given light-effort scope, no 2027 cycle confirmed, unchanged. Waters Corporation — still 403, unchanged. Moog — R-26-20226 still reads 'spring block intern' (no year), R-26-20243-1 still reads 'spring/summer 2027 block intern' (combined term) — both re-confirmed unchanged, still excluded.</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="str">
+        <v>HEICO / BorgWarner / Gulfstream / PACCAR / CNH Industrial / Nordson / Ingersoll Rand / Timken / Dana Incorporated / Rolls-Royce North America / Vestas / First Solar / Lucid Motors / SKF USA / ULA / AGCO</v>
+      </c>
+      <c r="B476" t="str">
+        <v>Fresh untried-company national pass, 2026-09-29 — access attempts only, not resolved</v>
+      </c>
+      <c r="C476" t="str">
+        <v>HEICO — Sucuri JS challenge wall, unreachable via curl. BorgWarner — Workday-backed but no working keyword-search endpoint identified, visible reqs (mostly Poland-based) had no intern/co-op titles. Gulfstream, PACCAR, CNH Industrial, Nordson — all 403. Ingersoll Rand — 429 rate-limited. Timken, Dana Incorporated, Rolls-Royce North America — SAP SuccessFactors ATS identified but search/list endpoint not reverse-engineered this run. Vestas, First Solar, Lucid Motors, SKF USA, ULA, AGCO — likely fully client-rendered SPAs, no ATS signature found in static HTML, not pursued further given time budget. None confirmed to have or lack qualifying postings — worth a headless-browser pass in a future run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C461"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C476"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 12 checked-excluded (2026-09-29 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrCSb7HoUoCSxwoxHPTBdz
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M244"/>
+  <dimension ref="A1:M247"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9700,6 +9700,102 @@
       </c>
       <c r="J244" t="str">
         <v>Fulfillment/server-assembly warehouse operations, Lean/Six Sigma. Two sibling reqs at the same Orangeburg, SC site (Quality Engineering Co-Op, Program Management Co-Op) have the same title/URL-slug season discrepancy but are non-target disciplines — see `checked`. Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="str">
+        <v>Axcelis Technologies</v>
+      </c>
+      <c r="B245" t="str">
+        <v>Engineering Co-op (Warehouse Solutions)</v>
+      </c>
+      <c r="C245" t="str">
+        <v>Industrial Engineering / Manufacturing Operations</v>
+      </c>
+      <c r="D245" t="str">
+        <v>Winter/Spring 2027 (Jan 4–Jun 25, 2027)</v>
+      </c>
+      <c r="E245" t="str">
+        <v>Beverly, MA</v>
+      </c>
+      <c r="F245">
+        <v>25</v>
+      </c>
+      <c r="G245" t="str">
+        <v>$20.42–$35.70/hr (posted U.S. base salary range)</v>
+      </c>
+      <c r="H245" t="str">
+        <v>https://axcelis.wd1.myworkdayjobs.com/Axcelis/job/Beverly-MA/Engineering-Co-op--Warehouse-Solutions-_12018</v>
+      </c>
+      <c r="I245" t="str">
+        <v>Yes — fetched directly via Axcelis's own Workday CXS API, req 12018, posted 14 days ago (2026-09-15), canApply true, quote: 'Co-op Cycle: January 4th to June 25th, 2027.'</v>
+      </c>
+      <c r="J245" t="str">
+        <v>New company for the tracker — Axcelis is a semiconductor ion-implantation equipment maker HQ'd in Beverly, MA. Warehouse Operations co-op supporting the Operations Technology team (logistics/process-improvement, some SQL/Python/PowerBI preferred). Open to Mechanical or Industrial Engineering students (or related field). $1,000 commuting travel stipend offered. Citizenship not stated. Sibling reqs at the same site were checked and excluded — see `checked` (one has an internal Winter-2027-header-vs-'summer 2026'-body contradiction, two have no year stated, two are explicitly Fall-cycle, one is Software Development discipline).</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B246" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C246" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D246" t="str">
+        <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
+      </c>
+      <c r="E246" t="str">
+        <v>Hollis, NH</v>
+      </c>
+      <c r="F246">
+        <v>45</v>
+      </c>
+      <c r="G246" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H246" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/Mechanical-Engineering-Co-op_WD226382</v>
+      </c>
+      <c r="I246" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226382, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
+      </c>
+      <c r="J246" t="str">
+        <v>TIME-SENSITIVE: posting's own end date is 2026-09-30 — application window closes within ~1 day of this run. Medical products (wearables, therapy systems, surgical robotics) mechanical design/CAD/prototyping work. 2nd or 3rd co-op preferred, SolidWorks required. A prior run excluded this req because its TITLE alone states no season, but the body text explicitly names the year ('Jan - Jun 2027') — re-evaluated as meeting the season-stated bar on body text, consistent with how other title/body-text discrepancies (e.g. Flex's own Orangeburg req) are handled elsewhere in this tracker. Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B247" t="str">
+        <v>NPI Process Engineering Co-op</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Manufacturing Engineering (New Product Introduction)</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Hollis, NH (posting body says Nashua, NH site)</v>
+      </c>
+      <c r="F247">
+        <v>45</v>
+      </c>
+      <c r="G247" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H247" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/NPI-Process-Engineering-Co-op_WD226387</v>
+      </c>
+      <c r="I247" t="str">
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226387, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
+      </c>
+      <c r="J247" t="str">
+        <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
       </c>
     </row>
   </sheetData>
@@ -10176,14 +10272,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M244"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M247"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C476"/>
+  <dimension ref="A1:C488"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -15417,9 +15513,141 @@
         <v>HEICO — Sucuri JS challenge wall, unreachable via curl. BorgWarner — Workday-backed but no working keyword-search endpoint identified, visible reqs (mostly Poland-based) had no intern/co-op titles. Gulfstream, PACCAR, CNH Industrial, Nordson — all 403. Ingersoll Rand — 429 rate-limited. Timken, Dana Incorporated, Rolls-Royce North America — SAP SuccessFactors ATS identified but search/list endpoint not reverse-engineered this run. Vestas, First Solar, Lucid Motors, SKF USA, ULA, AGCO — likely fully client-rendered SPAs, no ATS signature found in static HTML, not pursued further given time budget. None confirmed to have or lack qualifying postings — worth a headless-browser pass in a future run.</v>
       </c>
     </row>
+    <row r="477">
+      <c r="A477" t="str">
+        <v>Moog Inc. — Intern, Mechanical Analysis Engineering (R-26-20226) / Intern, Test Engineering (R-26-20243-1)</v>
+      </c>
+      <c r="B477" t="str">
+        <v>Re-check after a same-run research agent claimed a 'breakthrough' status change</v>
+      </c>
+      <c r="C477" t="str">
+        <v>2026-09-29 ~07:00 UTC: this run's national-sweep agent reported both reqs as 'genuinely OPEN, status changed from prior runs' — but the exact body-text quotes it supplied ('seeking a spring block intern' for R-26-20226, no year; 'spring/summer 2027 block intern' for R-26-20243) are byte-for-byte IDENTICAL to the wording re-confirmed unchanged earlier this same day (see the 2026-09-29 light-re-check entry above) and in 5+ prior runs. This session independently re-queried Moog's Workday CXS API directly and confirmed the text is in fact unchanged — the agent's 'breakthrough' framing was a misread of stable, already-excluded wording, not a new finding (same pattern as a prior run's R-26-20226 false-positive). Exclusion CONFIRMED, unchanged. Not added.</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="str">
+        <v>Axcelis Technologies</v>
+      </c>
+      <c r="B478" t="str">
+        <v>Facilities (Plant) Engineer Winter Co-Op (req 11590); Manufacturing Engineer Co-op Production Support (reqs 12001, 12008); Manufacturing Test Development Co-op (req 12009); Manufacturing Test Development Engineer Co-op (req 12010); Co-Op Manufacturing Software Development (req 12019) — all Beverly, MA, full company-wide Intern(Trainee) facet sweep via direct Workday CXS API</v>
+      </c>
+      <c r="C478" t="str">
+        <v>2026-09-29: req 11590's own title/header say 'Winter Co-Op' with 'Winter Co-op Cycle: January 4–February 26, 2027,' but the body text later states 'We are searching for our next group of Facilities Engineering Co-ops for a summer 2026 assignment' — an internal contradiction (Winter 2027 header vs. Summer 2026 body, neither of which is unambiguously Winter 2026/Spring 2027), same treatment as the standing Ameren/Analog Devices contradiction exclusions — excluded, flagged for Hamza's own judgment. Reqs 12001 and 12009 state a 'January 4th to June 25th' / 'Jan 1st to July 2nd' cycle with NO YEAR anywhere in the body — excluded per the strict season-confirmation bar (same treatment as Regal Rexnord R26_04115). Reqs 12008 and 12010 state 'July 6th to December 18th' — a Fall cycle, wrong season. Req 12019 (Manufacturing Software Development) explicitly confirms 'January 4th to June 25th, 2027' but is a software-development discipline, not a target discipline. The one qualifying req from this sweep (Engineering Co-op, Warehouse Solutions, req 12018) was added to `rows`.</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B479" t="str">
+        <v>Electrical Engineering Co-op, Hollis NH, req WD226386</v>
+      </c>
+      <c r="C479" t="str">
+        <v>2026-09-29: sibling req to the now-added WD226382/WD226387 Hollis, NH postings, same confirmed 'Jan - Jun 2027' season and canApply true — but Electrical Engineering discipline, outside Hamza's target disciplines. Not added.</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="str">
+        <v>Siemens</v>
+      </c>
+      <c r="B480" t="str">
+        <v>'Automation Engineer Co-Op - Spring 2027 (UT Arlington)' req 521404, and sibling 'Factory Digitalization Engineer Co-Op - Spring 2027 (UT Arlington)', both Grand Prairie, TX</v>
+      </c>
+      <c r="C480" t="str">
+        <v>2026-09-29: RESOLVED the prior run's access block — jobs.siemens.com/en_US/externaljobs/JobDetail/{id} pages server-render the full description without JS. Req 521404 independently confirmed live: controls/automation discipline, $30.00-$33.00/hr, explicit 'Spring 2027 (January – May or August)' season. However, the posting's own Basic Qualifications state 'Must be enrolled as a student at the University of Texas Arlington at the time of the co-op' — a school-specific eligibility restriction Hamza cannot meet. Excluded on eligibility grounds rather than season/discipline; the Factory Digitalization sibling carries the same UT-Arlington-only restriction per the same search result (not independently re-opened, same exclusion applies).</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B481" t="str">
+        <v>'Mechanical Engineering Co-Op' req R2496 — resolution of a prior run's unresolved 403 block</v>
+      </c>
+      <c r="C481" t="str">
+        <v>2026-09-29: RESOLVED — found Boston Dynamics' real Workday tenant (bostondynamics.wd1.myworkdayjobs.com, site Boston_Dynamics) and paginated all 77 currently open company-wide reqs directly via its CXS API. R2496 does not appear anywhere in the list, and there are zero Co-Op/Intern-titled postings among current openings (only senior/staff/principal roles). The req is closed/removed. No longer an open question.</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>CIRCOR International (Burlington, MA)</v>
+      </c>
+      <c r="B482" t="str">
+        <v>Company-wide open-req sweep via CIRCOR's real ATS (UltiPro/UKG, recruiting2.ultipro.com/cir1001circr) — resolution of the standing circor.jobs.net Cloudflare block</v>
+      </c>
+      <c r="C482" t="str">
+        <v>2026-09-29: RESOLVED the access block by locating the real ATS. CIRCOR's only current internship posting company-wide is 'Intern - Design Engineering,' req INTER002813, Tampa, FL (not Burlington, MA) — body text explicitly says 'Year-round opportunity,' no Winter 2026/Spring 2027 season stated anywhere, and it's the wrong location besides. No other intern/co-op titles found on the ~20-req visible board. Excluded — wrong location and no season stated.</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>MACOM Technology Solutions (Lowell, MA)</v>
+      </c>
+      <c r="B483" t="str">
+        <v>5 internship-titled reqs located via web search on macomtech.csod.com (Cornerstone OnDemand), careersite ID 4: req 2589 'Semiconductor Process Development Intern', 2606 'Process Engineering Intern', 2623 'RF Test Engineering Intern', plus reqs 2611/2612 and an aggregator-only 'Mechanical Product Engineer Intern' lead</v>
+      </c>
+      <c r="C483" t="str">
+        <v>2026-09-29: still could not independently verify any of these. Cornerstone's SPA returns only a cookie-banner shell to curl/WebFetch and a jina.ai reader-proxy attempt (itself blocked from this network); the underlying Cornerstone REST API returned HTTP 403 even with the page's own embedded bearer token/cookies (progress from a flat 401 in earlier runs, but still blocked). Season/status remains unconfirmed for all — not added. Worth a headless-browser attempt in a future run; the specific req IDs above are now on record for that attempt.</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>MITRE Corporation (Bedford, MA)</v>
+      </c>
+      <c r="B484" t="str">
+        <v>Fresh check for Winter 2026/Spring 2027 mechanical engineering co-ops — new company for the tracker</v>
+      </c>
+      <c r="C484" t="str">
+        <v>2026-09-29: only Summer 2026 and Summer 2027 mechanical engineering internships (MITRE Labs) found via search; careers.mitre.org's co-op/intern listing page is JS-rendered so a direct listing sweep wasn't possible this run. No Winter 2026/Spring 2027 posting confirmed. Worth a future attempt once MITRE's underlying ATS (likely Workday or SuccessFactors) is identified for direct API access.</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>VulcanForms (Devens, MA)</v>
+      </c>
+      <c r="B485" t="str">
+        <v>Full open-req sweep via VulcanForms' real ATS (Rippling, ats.rippling.com/vulcanforms/jobs) — new company for the tracker (MIT-spinout metal-3D-printing manufacturer)</v>
+      </c>
+      <c r="C485" t="str">
+        <v>2026-09-29: zero internship/co-op postings currently open — only full-time Engineering/Commercial roles. Aggregator-indexed 'Mechanical Engineering Intern – Fall/Summer 2026' postings are stale/no longer live. Not added; worth periodic re-checking given Boston-area fit if a co-op program opens.</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>Oklo Inc. / Redwood Materials / X-energy / K2 Space / Radiant Industries / Ursa Major Technologies</v>
+      </c>
+      <c r="B486" t="str">
+        <v>National fresh-pass, nuclear/energy/space adjacent companies, 2026-09-29</v>
+      </c>
+      <c r="C486" t="str">
+        <v>Oklo's 'General Internship Application 2027' (Greenhouse) explicitly states 'Summer 2027... June 7, 2027 - August 20, 2027' — wrong season. Redwood Materials' mechanical engineering intern/co-op posting found is for Summer 2026, not Winter 2026/Spring 2027. X-energy's Mechanical Engineering Internship is explicitly Summer 2027. K2 Space's Mechanical Engineering Intern is explicitly Summer 2027. Radiant Industries' only Mechanical Engineering Intern posting found is dated Fall 2025 (stale/expired). Ursa Major Technologies (propulsion, Berthoud CO) — only Summer 2026 propulsion internships found; company has a fast-moving posting cadence, worth rechecking next cycle.</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>Crane Company (Crane Pumps &amp; Systems)</v>
+      </c>
+      <c r="B487" t="str">
+        <v>Quality Engineering Co-Op (JR102424), Manufacturing Engineering Co-Op (JR102426), Design Engineer Co-Op (JR102425) — all Spartanburg, SC</v>
+      </c>
+      <c r="C487" t="str">
+        <v>2026-09-29: all three confirmed live via direct Workday CXS fetch (identical template to the already-tracked/already-excluded Piqua and Elyria reqs) but none states a season/term anywhere in the body text — same no-season treatment as the standing Crane Aerospace &amp; Electronics (JR102436) exclusion. Not added.</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>6 River Systems / RightHand Robotics / Soft Robotics / Repligen / Kongsberg (Hydroid) / Myomo</v>
+      </c>
+      <c r="B488" t="str">
+        <v>Fresh Boston-area robotics/medtech pass, 2026-09-29</v>
+      </c>
+      <c r="C488" t="str">
+        <v>No concrete Winter 2026/Spring 2027 co-op/intern posting located for any of these via search — mostly either no current internship program, Summer-only where any internship exists, or too JS-gated/thin a public footprint to verify an ATS directly this run. Not conclusively ruled out (not a confirmed-zero finding like VulcanForms/CIRCOR above) — worth a more focused direct-ATS look in a future run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C476"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C488"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 8 checked-excluded (2026-09-29 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CdaR8kQ6sEBb4Q6ftFQP6f
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M247"/>
+  <dimension ref="A1:M249"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9796,6 +9796,70 @@
       </c>
       <c r="J247" t="str">
         <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>RTX / Collins Aerospace</v>
+      </c>
+      <c r="B248" t="str">
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D248" t="str">
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Cedar Rapids, IA</v>
+      </c>
+      <c r="F248">
+        <v>1090</v>
+      </c>
+      <c r="G248" t="str">
+        <v>Not stated on posting (RTX co-op program range generally $37,000–$82,000/yr annualized per boilerplate)</v>
+      </c>
+      <c r="H248" t="str">
+        <v>https://careers.rtx.com/global/en/job/01872047/Mechanical-Engineering-Co-op-Winter-Spring-2027</v>
+      </c>
+      <c r="I248" t="str">
+        <v>Yes — independently fetched raw HTML/JSON-LD directly (bypassing careers.rtx.com's unreliable WebFetch rendering), req 01872047, datePosted 2026-09-28, title states '(Winter/Spring 2027)' verbatim, 'Apply Now' present, no filled/closed markers.</v>
+      </c>
+      <c r="J248" t="str">
+        <v>Displays, Controls, Computing &amp; Networking dept at Collins Aerospace — cockpit displays/control panels, servo actuation, avionics hardware. 'Immerse yourself in a full-time... co-op session, that will run January- July/August.' U.S. citizenship required (no clearance required). New req distinct from the already-tracked Chemical/Materials Co-op (01871473) and Mechanical Design Co-op (01871736, Jamestown ND) at the same company.</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B249" t="str">
+        <v>Mechanical Engineering Co-op - Spring 2027</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Mechanical / Industrial Engineering</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Orangeburg, SC</v>
+      </c>
+      <c r="F249">
+        <v>900</v>
+      </c>
+      <c r="G249" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H249" t="str">
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Mechanical-Engineering-Co-op---Fall-2026_WD227049</v>
+      </c>
+      <c r="I249" t="str">
+        <v>Yes — independently fetched directly via Flex's own Workday CXS API, req WD227049, canApply true, posted 26 days ago, title states 'Mechanical Engineering Co-op - Spring 2027' verbatim, quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 school semester.'</v>
+      </c>
+      <c r="J249" t="str">
+        <v>TIME-SENSITIVE: posting's own end date is 2026-10-03 — 3 days left to apply as of this run. NOTE: URL slug reads 'Fall-2026' (stale rename leftover, same pattern as the already-tracked Orangeburg Industrial Engineering Co-Op WD226357) but title/body both explicitly say 'Spring 2027' — treated as authoritative per the verification bar. Manufacturing Engineering Manager team — time studies, CAD, DOE projects. 'Is Sponsorship Available? No' (no visa sponsorship, not a citizenship/ITAR requirement). Pay not stated.</v>
       </c>
     </row>
   </sheetData>
@@ -10272,14 +10336,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M247"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M249"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C488"/>
+  <dimension ref="A1:C496"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -15645,9 +15709,97 @@
         <v>No concrete Winter 2026/Spring 2027 co-op/intern posting located for any of these via search — mostly either no current internship program, Summer-only where any internship exists, or too JS-gated/thin a public footprint to verify an ATS directly this run. Not conclusively ruled out (not a confirmed-zero finding like VulcanForms/CIRCOR above) — worth a more focused direct-ATS look in a future run.</v>
       </c>
     </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>Crane Company (Crane Pumps &amp; Systems / Resistoflex-ChemPharma)</v>
+      </c>
+      <c r="B489" t="str">
+        <v>Process Engineer Intern (JR102585, JR102567), Product Engineer Intern (JR102566), Quality Engineer Intern (JR102564) — all Marion, NC; Manufacturing Engineer Intern (JR102570) — Saddle Brook, NJ</v>
+      </c>
+      <c r="C489" t="str">
+        <v>2026-09-29: full company-wide sweep (26 intern-type reqs via Workday `workerSubType` facet, 100% coverage). All confirmed live via direct Workday CXS fetch but no season/year stated anywhere in any posting body — evergreen templates, same treatment as the standing Flowserve/Crane Aerospace/Regal Rexnord no-season exclusions. Crane Pumps &amp; Systems now appears fully saturated — no new season-confirmed reqs found company-wide.</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>Regal Rexnord</v>
+      </c>
+      <c r="B490" t="str">
+        <v>Full company-wide sweep, all 529 currently-open reqs paginated and title-scanned</v>
+      </c>
+      <c r="C490" t="str">
+        <v>2026-09-29: 100% coverage confirms no co-op/intern-titled req exists beyond what's already tracked (Tipp City OH R26_04440/R26_04736; Fort Wayne IN R26_04469 tracked, R26_04115 excluded no-year; Charlotte NC R26_04216 tracked; Florence KY x3 excluded). Remaining reqs are Milwaukee/Grafton-area Summer 2027 interns (wrong season) or international. Fully saturated — no edit needed, logged for future-run reference.</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="str">
+        <v>Flex (Flextronics International)</v>
+      </c>
+      <c r="B491" t="str">
+        <v>Injection Molding Engineering Co-Op, Libertyville IL, req WD229347 — full company-wide sweep via `jobFamilyGroup=Intern` facet (16 of 30 global co-op reqs are US-located, 100% coverage)</v>
+      </c>
+      <c r="C491" t="str">
+        <v>2026-09-29: no season/year stated anywhere in the body, AND Job Posting End Date is 2026-09-14 — already past as of this run despite canApply still reading true (stale/closed in practice). Excluded. Sweep otherwise confirmed all other US Flex reqs already tracked/excluded, plus surfaced the new Orangeburg WD227049 (added to `rows`).</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="str">
+        <v>Moog Inc. — Intern, Product Engineering (R-26-20334)</v>
+      </c>
+      <c r="B492" t="str">
+        <v>Buffalo, NY — new req found this run, posted 2026-09-28</v>
+      </c>
+      <c r="C492" t="str">
+        <v>2026-09-29: explicitly 'seeking a Summer block intern,' Mechanical/Aerospace discipline, $25–$31/hr — wrong season, excluded. R-26-20226/R-26-20243 re-confirmed unchanged (see prior entries).</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="str">
+        <v>The Nuclear Company</v>
+      </c>
+      <c r="B493" t="str">
+        <v>Re-check, 2026-09-29</v>
+      </c>
+      <c r="C493" t="str">
+        <v>'TNC Nuclear Interns 2027' (Columbia SC) re-fetched directly — body text unchanged, still explicitly Summer 2027. New 'Spring 2027 AI Applied Research/AI-ML/Data Science/Software Engineering Intern' postings (Washington DC) exist but are software/AI/data-science discipline, not target disciplines. No mechanical/nuclear-engineering Winter/Spring track has opened — unchanged from prior runs.</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="str">
+        <v>Stanley Black &amp; Decker</v>
+      </c>
+      <c r="B494" t="str">
+        <v>Fresh national pass, new company for the tracker — full Workday sweep (sbdinc.wd1.myworkdayjobs.com), Engineering + Manufacturing facets</v>
+      </c>
+      <c r="C494" t="str">
+        <v>2026-09-29: only Summer 2027 co-ops/interns found (Towson MD Mechanical/Electrical/Embedded Engineering Interns, Mission TX Manufacturing Internship) — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="str">
+        <v>AMETEK</v>
+      </c>
+      <c r="B495" t="str">
+        <v>Fresh national pass, new company for the tracker — full sweep via jobs.ametek.com (SuccessFactors)</v>
+      </c>
+      <c r="C495" t="str">
+        <v>2026-09-29: only 2 US intern/co-op titles company-wide. 'Manufacturing Engineering Intern Co-op' (AMETEK Rotron, Woodstock NY, aerospace mfg) is target discipline but no season/year stated anywhere — excluded. 'Co-Op CNC Lathe Operator' (Keene NH) is wrong discipline.</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="str">
+        <v>Curtiss-Wright</v>
+      </c>
+      <c r="B496" t="str">
+        <v>Fresh national pass, new company for the tracker — full 355-job Workday sweep (curtisswright.wd1.myworkdayjobs.com)</v>
+      </c>
+      <c r="C496" t="str">
+        <v>2026-09-29: only engineering co-op found is 'Co-op (Spring Term)' JR1907, Cheswick PA (EMD division; Mechanical/Electrical/Industrial/Welding disciplines) — a stale evergreen template (startDate 2025-02-07, generic 'Spring, Summer and Fall semesters,' no year stated anywhere) — excluded. A separate 'Purchasing &amp; Supply Chain Intern (Spring 2027 Semester)' req confirms Curtiss-Wright does run an actual Spring 2027 cycle, but no matching engineering-discipline req is live yet — worth a periodic re-check.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C488"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C496"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 9 new postings, 3 checked-excluded (2026-09-29 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fkk7jq1xZr2tze8DXzpTd3
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M249"/>
+  <dimension ref="A1:M258"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9860,6 +9860,294 @@
       </c>
       <c r="J249" t="str">
         <v>TIME-SENSITIVE: posting's own end date is 2026-10-03 — 3 days left to apply as of this run. NOTE: URL slug reads 'Fall-2026' (stale rename leftover, same pattern as the already-tracked Orangeburg Industrial Engineering Co-Op WD226357) but title/body both explicitly say 'Spring 2027' — treated as authoritative per the verification bar. Manufacturing Engineering Manager team — time studies, CAD, DOE projects. 'Is Sponsorship Available? No' (no visa sponsorship, not a citizenship/ITAR requirement). Pay not stated.</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B250" t="str">
+        <v>Mechanical Engineer Co-Op - Spring 2027</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Mechanical / Aerospace Engineering</v>
+      </c>
+      <c r="D250" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Boston, MA (Seaport)</v>
+      </c>
+      <c r="F250">
+        <v>0</v>
+      </c>
+      <c r="G250" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H250" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/124</v>
+      </c>
+      <c r="I250" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API (specteraerospace.bamboohr.com/careers/124/detail), status Open, posted 2026-08-13, title states 'Mechanical Engineer Co-Op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J250" t="str">
+        <v>New company for the tracker — hypersonic flight vehicle startup (Boston Seaport + Peabody, MA offices), funded by government R&amp;D + private funding. Vehicle Development team, designing components/subsystems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance). Strong Boston-area match.</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B251" t="str">
+        <v>Vehicle Design Co-Op - Spring 2027</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Mechanical / Aerospace Engineering</v>
+      </c>
+      <c r="D251" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E251" t="str">
+        <v>Boston, MA (Seaport)</v>
+      </c>
+      <c r="F251">
+        <v>0</v>
+      </c>
+      <c r="G251" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H251" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/116</v>
+      </c>
+      <c r="I251" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Vehicle Design Co-Op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J251" t="str">
+        <v>Sibling req to the Mechanical Engineer Co-Op above, same company/site. Vehicle Design team, designing components/systems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B252" t="str">
+        <v>Propulsion Test Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C252" t="str">
+        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
+      </c>
+      <c r="D252" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E252" t="str">
+        <v>Peabody, MA</v>
+      </c>
+      <c r="F252">
+        <v>19</v>
+      </c>
+      <c r="G252" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H252" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/117</v>
+      </c>
+      <c r="I252" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Propulsion Test Engineering Co-Op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J252" t="str">
+        <v>Design, manufacturing, and test of advanced ramjet/scramjet engine hardware for hypersonic propulsion systems. Note: posting says Specter hires both this and the Propulsion Design Engineering Co-op (below) from a shared applicant pool depending on interest/fit. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B253" t="str">
+        <v>Propulsion Design Engineering Co-op - Spring 2027</v>
+      </c>
+      <c r="C253" t="str">
+        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
+      </c>
+      <c r="D253" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E253" t="str">
+        <v>Peabody, MA</v>
+      </c>
+      <c r="F253">
+        <v>19</v>
+      </c>
+      <c r="G253" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H253" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/118</v>
+      </c>
+      <c r="I253" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'Propulsion Design Engineering Co-op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J253" t="str">
+        <v>Sibling/shared-pool req to Propulsion Test Engineering Co-Op above (same site, same applicant pool per posting text). Design, manufacturing, and test of ramjet/scramjet engine hardware. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B254" t="str">
+        <v>PLC/Controls Engineer Co-Op - Spring 2027</v>
+      </c>
+      <c r="C254" t="str">
+        <v>Controls / Mechanical / Electrical Engineering</v>
+      </c>
+      <c r="D254" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E254" t="str">
+        <v>Peabody, MA</v>
+      </c>
+      <c r="F254">
+        <v>19</v>
+      </c>
+      <c r="G254" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H254" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/123</v>
+      </c>
+      <c r="I254" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'PLC/Controls Engineer Co-Op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J254" t="str">
+        <v>PLC software design (Beckhoff/TwinCAT ecosystem), electrical control-panel design, sensor/actuator integration for the Specter engine test facility. Open to Computer/Electrical/Mechanical Engineering or CS majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B255" t="str">
+        <v>Computational Design Engineer Co-Op - Spring 2027</v>
+      </c>
+      <c r="C255" t="str">
+        <v>Mechanical / Computational Engineering</v>
+      </c>
+      <c r="D255" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E255" t="str">
+        <v>Peabody, MA</v>
+      </c>
+      <c r="F255">
+        <v>19</v>
+      </c>
+      <c r="G255" t="str">
+        <v>$23-$30/hr</v>
+      </c>
+      <c r="H255" t="str">
+        <v>https://specteraerospace.bamboohr.com/careers/127</v>
+      </c>
+      <c r="I255" t="str">
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-08-13, title states 'Computational Design Engineer Co-Op - Spring 2027' verbatim.</v>
+      </c>
+      <c r="J255" t="str">
+        <v>Reusable computational geometry models / implicit modeling (Rhino/Grasshopper, nTop, PicoGK) for high-speed airbreathing testbed vehicle design and analysis. Open to Engineering/Math/CS/Physics majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>Shaw Industries</v>
+      </c>
+      <c r="B256" t="str">
+        <v>Engineering Internship/Co-op Spring 2027</v>
+      </c>
+      <c r="C256" t="str">
+        <v>Manufacturing / Industrial Engineering</v>
+      </c>
+      <c r="D256" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E256" t="str">
+        <v>Dalton, GA</v>
+      </c>
+      <c r="F256">
+        <v>1050</v>
+      </c>
+      <c r="G256" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H256" t="str">
+        <v>https://shawinc.wd1.myworkdayjobs.com/en-US/External/job/Shaw-Plant-7C-2208-S-Hamilton-Street-Dalton-GA-30721-USA/Engineering-Internship-Co-op-Spring-2027_R-156324</v>
+      </c>
+      <c r="I256" t="str">
+        <v>Yes — independently fetched directly via Shaw Industries' own Workday CXS API, req R-156324, title states 'Engineering Internship/Co-op Spring 2027' verbatim, posted 30+ days ago (exact date not disclosed by API).</v>
+      </c>
+      <c r="J256" t="str">
+        <v>New company for the tracker — flooring manufacturer, wholly-owned Berkshire Hathaway subsidiary, $5B+ annual sales. Rotating or sequential semesters working onsite in Shaw's manufacturing operations facilities in an engineering capacity; student matched to a facility per skills/interests. Citizenship/GPA/eligibility not stated on posting — confirm directly.</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B257" t="str">
+        <v>Operations &amp; Automation Engineering Co-op/Intern - Spring 2027</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Controls / Automation / Industrial Engineering</v>
+      </c>
+      <c r="D257" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E257" t="str">
+        <v>Bartow, FL</v>
+      </c>
+      <c r="F257">
+        <v>1250</v>
+      </c>
+      <c r="G257" t="str">
+        <v>Not stated on posting (housing/relocation available for qualified candidates)</v>
+      </c>
+      <c r="H257" t="str">
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Bartow-FL/Operations---Automation-Engineering-Co-op-Intern---Spring-2027_64675-1</v>
+      </c>
+      <c r="I257" t="str">
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64675, exact quote: 'Term Jan 11th, 2027 to April 23th, 2027 Full time Co-Op/Internship.'</v>
+      </c>
+      <c r="J257" t="str">
+        <v>New company for the tracker — NYSE: MOS, world's leading integrated producer of concentrated phosphate and potash fertilizer. Supports plant operations and automated control systems (PLC, DCS, HMI/SCADA) at the Bartow, FL phosphoric-acid manufacturing site. Citizenship not stated on posting.</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B258" t="str">
+        <v>Operations Engineering Co-op/Intern – Spring 2027</v>
+      </c>
+      <c r="C258" t="str">
+        <v>Mechanical / Industrial Engineering</v>
+      </c>
+      <c r="D258" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E258" t="str">
+        <v>Riverview, FL</v>
+      </c>
+      <c r="F258">
+        <v>1250</v>
+      </c>
+      <c r="G258" t="str">
+        <v>Not stated on posting (relocation package available for qualified candidates)</v>
+      </c>
+      <c r="H258" t="str">
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Riverview-FL/Operations-Engineering-Co-op-Intern---Spring-2027_64656</v>
+      </c>
+      <c r="I258" t="str">
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64656, exact quote: 'Term January 11 to April 23, 2027.'</v>
+      </c>
+      <c r="J258" t="str">
+        <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
       </c>
     </row>
   </sheetData>
@@ -10336,14 +10624,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M249"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M258"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C496"/>
+  <dimension ref="A1:C499"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -15797,9 +16085,42 @@
         <v>2026-09-29: only engineering co-op found is 'Co-op (Spring Term)' JR1907, Cheswick PA (EMD division; Mechanical/Electrical/Industrial/Welding disciplines) — a stale evergreen template (startDate 2025-02-07, generic 'Spring, Summer and Fall semesters,' no year stated anywhere) — excluded. A separate 'Purchasing &amp; Supply Chain Intern (Spring 2027 Semester)' req confirms Curtiss-Wright does run an actual Spring 2027 cycle, but no matching engineering-discipline req is live yet — worth a periodic re-check.</v>
       </c>
     </row>
+    <row r="497">
+      <c r="A497" t="str">
+        <v>Karman Space &amp; Defense</v>
+      </c>
+      <c r="B497" t="str">
+        <v>Full company-wide sweep via the real ADP Workforce Now portal newly located behind karman-sd.com/careers (cid=82153303-7d5a-4833-b767-9cb13d965e09) — resolution of the standing 'domain moved to karman-sd.com, board not yet reached' re-check note</v>
+      </c>
+      <c r="C497" t="str">
+        <v>2026-09-29 ~19:00 UTC: paginated all 235 currently-open requisitions company-wide via ADP's public JSON API. Zero postings with 'Intern'/'Co-op' in title or worker-category anywhere, and zero Massachusetts/Boston-area locations (all reqs are WA/CA/UT/AL/SC/MS/PA/OR). Consistent with the standing 'Summer-only internship program by design' exclusion from prior runs — now additionally confirmed there is no internship/co-op opening of any kind, any season, company-wide. Access method (ADP API) is now known-good for periodic re-checks.</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="str">
+        <v>GITAI</v>
+      </c>
+      <c r="B498" t="str">
+        <v>Mechanical Engineering Intern/Co-op, Rocket Motors (job 5381579008) and Satellite Bus (job 5376083008), Torrance CA — new company for the tracker</v>
+      </c>
+      <c r="C498" t="str">
+        <v>2026-09-29: both confirmed live and freshly updated (2026-09-28) via GITAI's own Greenhouse API, but neither posting's own body text states a specific season (Winter 2026/Spring 2027) — only a flexible start/end date and 'expected graduation during 2027.' A third-party aggregator (jobs.spacecapital.com) labels one 'Winter/Spring 2027' but that is the aggregator's own framing, not GITAI's text — fails the strict 'season stated on the posting itself' bar. Not added; worth a re-check if GITAI's own posting text is later updated with an explicit term.</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="str">
+        <v>Lam Research / Waters Corporation / Parker Hannifin / MACOM Technology Solutions (Lowell, MA) / CIRCOR International (Burlington, MA)</v>
+      </c>
+      <c r="B499" t="str">
+        <v>Re-attempted direct access to all five standing-blocked employers</v>
+      </c>
+      <c r="C499" t="str">
+        <v>2026-09-29: no progress on any. Lam Research: careers.lamresearch.com confirmed to itself run on Eightfold (window._EF_GROUP_ID='lamresearch.com'), but both the eightfold.ai and careers.lamresearch.com API hosts still reject with 'Not authorized for PCSX' — no workaround found. Waters Corporation: real ATS domain identified as uscareers-waters.icims.com, but it returns HTTP 405 with an AWS WAF captcha challenge (confirmed bot-block via response headers, not a redirect) — cannot bypass; unverified aggregator titles ('Electrical Technician Co-op', 'Research Electrical Engineering Co-op', Milford MA) not added (wrong discipline besides). Parker Hannifin: official student portal located (parkercareers.ttcportals.com/search/students/jobs) but returns Cloudflare/WAF 403 on both curl and WebFetch. MACOM: Cornerstone API still returns 401 'Check your credentials' even with the page's embedded bearer token; no co-op-relevant req surfaced this run. CIRCOR: UltiPro board's LoadSearchResults API returned an empty-but-200 response (0 opportunities) — likely a malformed request rather than a confirmed zero, so left as unverified rather than upgraded to 'no openings.' All five remain long-recurring blockers.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C496"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C499"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 9 new postings, 16 checked-excluded (2026-09-30 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019g5y5t6L9M55fX74WctZvq
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M258"/>
+  <dimension ref="A1:M267"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -10148,6 +10148,294 @@
       </c>
       <c r="J258" t="str">
         <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B259" t="str">
+        <v>Mechanical Engineering &amp; System Packaging Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D259" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F259">
+        <v>3</v>
+      </c>
+      <c r="G259" t="str">
+        <v>$20.00–$45.00/hr per posting</v>
+      </c>
+      <c r="H259" t="str">
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Mechanical-Engineering---System-Packaging-Co-Op--Spring-2027-_JR002940</v>
+      </c>
+      <c r="I259" t="str">
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002940), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+      </c>
+      <c r="J259" t="str">
+        <v>US citizenship required (posting: 'Co-op students must be US citizens who are enrolled in an accredited engineering curriculum'). CAD (SolidWorks/Creo) and FEA (Ansys) work on national-security hardware.</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B260" t="str">
+        <v>Digital Engineering – Requirements Engineering Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C260" t="str">
+        <v>Systems Engineering</v>
+      </c>
+      <c r="D260" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Lowell, MA</v>
+      </c>
+      <c r="F260">
+        <v>30</v>
+      </c>
+      <c r="G260" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H260" t="str">
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Lowell-MA/Digital-Engineering---Requirements-Engineering-Co-Op--Spring-2027-_JR002944</v>
+      </c>
+      <c r="I260" t="str">
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002944), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+      </c>
+      <c r="J260" t="str">
+        <v>US Citizenship required per posting. Digital-twin/model-driven systems engineering support for strategic deterrent, missile-defense, hypersonic, space, and autonomous vehicle programs. Python scripting experience preferred.</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B261" t="str">
+        <v>Process Engineer Co-Op/Intern - Spring 2027</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Mechanical / Chemical / Mining Engineering</v>
+      </c>
+      <c r="D261" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E261" t="str">
+        <v>Bradley, FL</v>
+      </c>
+      <c r="F261">
+        <v>1250</v>
+      </c>
+      <c r="G261" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H261" t="str">
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Bradley-FL/Process-Engineer-Co-Op-Intern---Spring-2027_64450</v>
+      </c>
+      <c r="I261" t="str">
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64450, canApply true.</v>
+      </c>
+      <c r="J261" t="str">
+        <v>Posting explicitly accepts Chemical, Mechanical, and/or Mining Engineering majors. Term Jan 11–Apr 23, 2027 (same as tracker's other Mosaic co-ops). Citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B262" t="str">
+        <v>Capital Project Engineering Co-Op/Intern - Spring 2027</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Mechanical / Chemical / Industrial Engineering</v>
+      </c>
+      <c r="D262" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Riverview, FL</v>
+      </c>
+      <c r="F262">
+        <v>1250</v>
+      </c>
+      <c r="G262" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H262" t="str">
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Riverview-FL/Capital-Project-Engineering-Co-Op-Intern---Spring-2027_64455</v>
+      </c>
+      <c r="I262" t="str">
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64455, canApply true.</v>
+      </c>
+      <c r="J262" t="str">
+        <v>Posting explicitly accepts Chemical, Mechanical, or Industrial Engineer majors. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B263" t="str">
+        <v>Capital Project Engineering Co-op/Intern - Spring 2027</v>
+      </c>
+      <c r="C263" t="str">
+        <v>Mechanical / Chemical / Industrial Engineering</v>
+      </c>
+      <c r="D263" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E263" t="str">
+        <v>Tampa, FL (Lithia area)</v>
+      </c>
+      <c r="F263">
+        <v>1240</v>
+      </c>
+      <c r="G263" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H263" t="str">
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Tampa-FL-Lithia-area/Capital-Project-Engineering-Co-op-Intern---Spring-2027_64392</v>
+      </c>
+      <c r="I263" t="str">
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64392, canApply true.</v>
+      </c>
+      <c r="J263" t="str">
+        <v>Sibling req to the Riverview, FL Capital Project Engineering Co-op above, same discipline, different site. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>Gulfstream Aerospace</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Spring 2027 - IEF - Stress Engineering - Collegiate Associate Intern</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Aerospace / Structural Engineering</v>
+      </c>
+      <c r="D264" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Savannah, GA</v>
+      </c>
+      <c r="F264">
+        <v>900</v>
+      </c>
+      <c r="G264" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H264" t="str">
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Stress-Engineering-Collegiate-Associate-Intern-GA-31401/1423681300/</v>
+      </c>
+      <c r="I264" t="str">
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Stress Engineering'.</v>
+      </c>
+      <c r="J264" t="str">
+        <v>Discipline list per posting: Aerospace, Civil, Structural, Mechanical Engineering, Computer Science. GPA ≥3.0 cumulative (unrounded) required. No visa sponsorship — effectively requires US citizenship/permanent residency.</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>Gulfstream Aerospace</v>
+      </c>
+      <c r="B265" t="str">
+        <v>Spring 2027 - IEF - Materials and Processes Engineering College Associate</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Materials Engineering</v>
+      </c>
+      <c r="D265" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E265" t="str">
+        <v>Savannah, GA</v>
+      </c>
+      <c r="F265">
+        <v>900</v>
+      </c>
+      <c r="G265" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H265" t="str">
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Materials-and-Processes-Engineering-College-Associate-GA-31401/1432666200/</v>
+      </c>
+      <c r="I265" t="str">
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Materials and Processes'.</v>
+      </c>
+      <c r="J265" t="str">
+        <v>Discipline list per posting: Mechanical, Materials Science &amp; Engineering, Materials Engineering, Aerospace, Chemical Engineering, Metallurgy. GPA ≥3.0 cumulative required. No visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>Pyka</v>
+      </c>
+      <c r="B266" t="str">
+        <v>Mechanical Engineering Internship - Winter/Spring 2027 (Dropship, Early Interest)</v>
+      </c>
+      <c r="C266" t="str">
+        <v>Mechanical / Aerospace Engineering</v>
+      </c>
+      <c r="D266" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E266" t="str">
+        <v>Alameda, CA</v>
+      </c>
+      <c r="F266">
+        <v>2700</v>
+      </c>
+      <c r="G266" t="str">
+        <v>$35–$40/hr per posting</v>
+      </c>
+      <c r="H266" t="str">
+        <v>https://jobs.lever.co/pyka/2702593a-7482-4d2b-93f3-ef97e2cf7df7</v>
+      </c>
+      <c r="I266" t="str">
+        <v>Yes — independently fetched directly via Lever's public API, posting live, text confirms 'Winter/Spring 2027'.</v>
+      </c>
+      <c r="J266" t="str">
+        <v>IMPORTANT: explicitly an 'Early Interest Application' — posting states formal interviews for the 2027 cohort won't begin until October 2026; applying now only queues your profile for later review, not an active hiring process yet. Visa sponsorship offered. Electric-aviation 'Dropship' cargo aircraft program.</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>General Astronautics</v>
+      </c>
+      <c r="B267" t="str">
+        <v>Spring 2027 Mechanical Engineering Internship/Co-op</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D267" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E267" t="str">
+        <v>San Francisco, CA</v>
+      </c>
+      <c r="F267">
+        <v>2700</v>
+      </c>
+      <c r="G267" t="str">
+        <v>$30.00/hr (Sophomore), $35.00/hr (Junior/Senior) per posting</v>
+      </c>
+      <c r="H267" t="str">
+        <v>https://www.workatastartup.com/jobs/103200</v>
+      </c>
+      <c r="I267" t="str">
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027 Mechanical Engineering Internship/Co-op'; also cross-confirmed on ycombinator.com's own company page.</v>
+      </c>
+      <c r="J267" t="str">
+        <v>New company for the tracker — YC-backed startup building autonomous robots for orbital manufacturing. Minimum 12 weeks on-site in San Francisco required. 'U.S. citizen or national, U.S. lawful permanent resident, or eligible for authorization under U.S. export regulations.' Applies via YC's own account/signup flow (workatastartup.com).</v>
       </c>
     </row>
   </sheetData>
@@ -10624,14 +10912,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M258"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M267"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C499"/>
+  <dimension ref="A1:C515"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -16118,9 +16406,185 @@
         <v>2026-09-29: no progress on any. Lam Research: careers.lamresearch.com confirmed to itself run on Eightfold (window._EF_GROUP_ID='lamresearch.com'), but both the eightfold.ai and careers.lamresearch.com API hosts still reject with 'Not authorized for PCSX' — no workaround found. Waters Corporation: real ATS domain identified as uscareers-waters.icims.com, but it returns HTTP 405 with an AWS WAF captcha challenge (confirmed bot-block via response headers, not a redirect) — cannot bypass; unverified aggregator titles ('Electrical Technician Co-op', 'Research Electrical Engineering Co-op', Milford MA) not added (wrong discipline besides). Parker Hannifin: official student portal located (parkercareers.ttcportals.com/search/students/jobs) but returns Cloudflare/WAF 403 on both curl and WebFetch. MACOM: Cornerstone API still returns 401 'Check your credentials' even with the page's embedded bearer token; no co-op-relevant req surfaced this run. CIRCOR: UltiPro board's LoadSearchResults API returned an empty-but-200 response (0 opportunities) — likely a malformed request rather than a confirmed zero, so left as unverified rather than upgraded to 'no openings.' All five remain long-recurring blockers.</v>
       </c>
     </row>
+    <row r="500">
+      <c r="A500" t="str">
+        <v>CIRCOR International (Burlington, MA)</v>
+      </c>
+      <c r="B500" t="str">
+        <v>Full re-parse of the UltiPro job board's server-rendered initial page load (recruiting2.ultipro.com/CIR1001CIRCR/JobBoard), bypassing the LoadSearchResults API that had been returning empty-but-200</v>
+      </c>
+      <c r="C500" t="str">
+        <v>2026-09-30: RESOLVED to a confirmed zero — the board's initial HTML embeds the full current opportunity list as inline JSON (20 open reqs company-wide: machinists, quality/manufacturing engineers, CAD designer, sales/finance roles, etc.). None titled Intern/Co-op/Student. Upgrading from 'unverified' to CONFIRMED — CIRCOR currently has no internship/co-op postings open, any discipline, any location.</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="str">
+        <v>Lam Research (lamresearch.eightfold.ai)</v>
+      </c>
+      <c r="B501" t="str">
+        <v>Root-cause investigation of the standing 'Not authorized for PCSX' block</v>
+      </c>
+      <c r="C501" t="str">
+        <v>2026-09-30: identified the specific cause — Lam's site runs Eightfold's newer PCSX (Public Career Site X) product (confirmed via embedded pcsx-* theme keys/config in the page source), while every previously-tried endpoint (/api/apply/v1–v3/jobs, /api/pcsx/jobs, etc.) is the older PCS API, which PCSX sites reject by design. No working read-only API found for PCSX. Site-restricted web search surfaced no mechanical/Spring-2027 intern posting. Genuinely unverifiable by any fetch-based method; would need a headless browser (PCSX is client-rendered React).</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="str">
+        <v>MACOM Technology Solutions (Lowell, MA)</v>
+      </c>
+      <c r="B502" t="str">
+        <v>Re-attempted all 5 known reqs (2589/2606/2611/2612/2623) using the SPA shell's own embedded anonymous-session JWT as a Bearer token against every route whitelisted in that JWT</v>
+      </c>
+      <c r="C502" t="str">
+        <v>2026-09-30: more specific failure mode found (progress, not resolution) — the req IDs themselves are not hard-404s (outer SPA shell returns 200), and job-requisition/v2/requisitions/{id} now returns a specific 403 'Access to resource is denied' (vs. the flatter 401s tried previously) — confirming the route exists but the anonymous guest token's scope doesn't cover requisition data, which renders entirely client-side. Still cannot confirm live/closed status of any of the 5 reqs. Still blocked; a headless browser is the next step.</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="str">
+        <v>Curtiss-Wright</v>
+      </c>
+      <c r="B503" t="str">
+        <v>2 additional intern reqs found on the same Workday board: JR11380 'Engineer Intern' (Grand Prairie TX, Mechanical/Manufacturing Engineering, $18-19/hr) and JR13583-2 'Design Engineering Intern' (East Farmingdale NY, Mechanical/Nuclear Engineering, US-citizen-only, $20-25/hr)</v>
+      </c>
+      <c r="C503" t="str">
+        <v>2026-09-30: both genuinely engineering-discipline and open, but neither states a season/year anywhere in the posting body — same evergreen-template pattern as the already-excluded JR1907. Fails the strict season-verification bar; not added.</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="str">
+        <v>Specter Aerospace</v>
+      </c>
+      <c r="B504" t="str">
+        <v>Full BambooHR re-sweep of all 36 open reqs beyond the 6 already-tracked co-ops: Electrical Engineering Co-Op (id 115), Embedded Software Co-Op (id 119), Front-End Software Developer Co-Op (id 120), Image Processing Co-Op (id 121), Full Stack Developer Co-Op (id 122), all Spring 2027, all Boston MA</v>
+      </c>
+      <c r="C504" t="str">
+        <v>2026-09-30: all 5 confirmed open via BambooHR detail API but are electrical/software/image-processing discipline — outside Hamza's target list. No new mechanical/aerospace/propulsion/controls-discipline co-op found beyond the 6 already tracked. Company-wide sweep now saturated.</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="str">
+        <v>Boston Dynamics (Waltham, MA) / Teradyne (North Reading, MA) / Vicor (Andover, MA)</v>
+      </c>
+      <c r="B505" t="str">
+        <v>Full re-sweep of each employer's own careers site/API</v>
+      </c>
+      <c r="C505" t="str">
+        <v>2026-09-30: Boston Dynamics — 79 open reqs company-wide, 0 Co-Op/Intern worker subtype; the previously-tracked-then-excluded R2496 now 404s. Teradyne — zero co-op-titled results on jobs.teradyne.com; prior-cycle Spring/Fall 2026 co-ops are gone. Vicor — zero intern/co-op-titled reqs on careers.vicorpower.com. No change from standing exclusions.</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B506" t="str">
+        <v>Correction of a same-run research agent's false-negative report that jobs 8130829 and 8199092 return 404</v>
+      </c>
+      <c r="C506" t="str">
+        <v>2026-09-30: independently re-fetched both directly via Formlabs' correct Greenhouse board (boards-api.greenhouse.io/v1/boards/formlabs/jobs/...) — both return HTTP 200 with correct titles, live and unchanged. The agent's 404 was caused by querying the wrong board slug ('formlabsinternships' instead of 'formlabs'). All 8 already-tracked Formlabs reqs (8130829, 8172004, 8161817, 8172226, 8199092, 8196515, 8172256, 8199269) independently re-verified live this run — no rows changed.</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B507" t="str">
+        <v>'Healthcare Mechanical Engineering Co-op (Spring)', req R266691, Wilmington MA, posted 4 days ago</v>
+      </c>
+      <c r="C507" t="str">
+        <v>2026-09-30: title says '(Spring)' but the posting's own body text explicitly states 'This is a full-time, in-person co-op opportunity running from June through December' — a Summer/Fall term, not Spring 2027 or Winter 2026. Excluded on season grounds despite the title's claim — title/body discrepancy explicitly flagged so a future title-only check doesn't wrongly include it.</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="str">
+        <v>L3Harris (Londonderry, NH)</v>
+      </c>
+      <c r="B508" t="str">
+        <v>Manufacturing Engineering Internship, job code 41201/41210 — re-check</v>
+      </c>
+      <c r="C508" t="str">
+        <v>2026-09-30: re-confirmed live, strong discipline fit (Mechanical/Aerospace/Materials Science/Industrial Engineering), $25.00–$47.50/hr — but still no season/term stated anywhere in the posting text, same as the standing L3Harris internship-template exclusion (job 41201 previously excluded 2026-09-26 for the identical reason). No change.</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="str">
+        <v>Lincoln Electric</v>
+      </c>
+      <c r="B509" t="str">
+        <v>'Controls Engineering Spring 2027 Co-op', Plymouth MI, req 29826, posted 2026-09-25</v>
+      </c>
+      <c r="C509" t="str">
+        <v>2026-09-30: the posting's title says 'Spring 2027' but its own body text describes itself as 'Lincoln Electric's ... Controls Engineering Fall 2027 Co-op Program' — a genuine self-contradiction in the source (not an inference error). Also EE/Computer-Engineering-preferred discipline. Excluded pending resolution — could not confirm either season claim from the posting itself.</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="str">
+        <v>Genentech</v>
+      </c>
+      <c r="B510" t="str">
+        <v>'2027 Spring Intern - Pharma Technical Development - Device Development', South San Francisco, deadline Oct 3 2026 per aggregators (workopia, dreamworkhq)</v>
+      </c>
+      <c r="C510" t="str">
+        <v>2026-09-30: sibling job IDs in the same posting series (202609-122484, 202609-123436) were independently confirmed live directly on careers.gene.com, and multiple independent aggregators agree on this specific role's detail — but careers.gene.com is a Phenom SPA whose search/apply JSON APIs could not be reached with a working tenant/domain param, so the exact requisition ID and canonical URL for THIS specific role could not be independently opened. Not added without a verified URL (per the no-invented-URL rule); worth a headless-browser follow-up given the imminent deadline.</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="str">
+        <v>Nexus Engineering Group (Maumee, OH)</v>
+      </c>
+      <c r="B511" t="str">
+        <v>'Instrumentation &amp; Controls Engineer Intern or Co-Op (Spring 2027)'</v>
+      </c>
+      <c r="C511" t="str">
+        <v>2026-09-30: application deadline already passed (Sep 15, 2026 per aggregator), and the live Lever board link for the listed req ID actually resolves to an unrelated Summer 2027/Cleveland OH posting — the Spring 2027/Maumee req appears closed/removed. Excluded.</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="str">
+        <v>Trew / TREW LLC (West Chester, OH)</v>
+      </c>
+      <c r="B512" t="str">
+        <v>'Spring 2027 Controls/Electrical Engineering Co-Op' (widely circulated by aggregators)</v>
+      </c>
+      <c r="C512" t="str">
+        <v>2026-09-30: Trew's own live ATS (Paycor Recruiting, reached via info.trewautomation.com/careers) currently lists zero intern/co-op titles — only full-time Controls/Electrical Engineer roles. Not found live on the employer's own source; excluded as likely closed or a stale aggregator listing.</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="str">
+        <v>Barry-Wehmiller</v>
+      </c>
+      <c r="B513" t="str">
+        <v>'Automation &amp; Controls Engineering Internship/Co-Op'</v>
+      </c>
+      <c r="C513" t="str">
+        <v>2026-09-30: only located via Illinois Tech's login-walled Handshake listing (iit.joinhandshake.com) — could not independently open; not found on barrywehmiller.com's own career pages. Description says the co-op can start 'January or June 2027' (applicant's choice) — ambiguous term boundary besides. Excluded pending direct-source confirmation.</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>Cresilon (Brooklyn, NY)</v>
+      </c>
+      <c r="B514" t="str">
+        <v>Hemostatic-medical-device internship</v>
+      </c>
+      <c r="C514" t="str">
+        <v>2026-09-30: posting is dated '2026 Spring' (already elapsed as of this run's date), not 2027. Wrong season — excluded.</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="str">
+        <v>The Mosaic Company</v>
+      </c>
+      <c r="B515" t="str">
+        <v>Electrical Engineer Co-Op/Intern - Spring 2027 (req 64427, Bartow FL), Water Balance Engineer Co-Op/Intern - Spring 2027 (req 64508, Mulberry FL), Reliability Engineer Co-Op/Intern - Winter 2027 (req 64355, Esterhazy SK Canada), Operations Engineering Co-op/Intern (req 64862, Bartow FL, full title reveals '...Summer 2027')</v>
+      </c>
+      <c r="C515" t="str">
+        <v>2026-09-30: found during the same-company sweep that surfaced reqs 64450/64455/64392 (added to `rows`). 64427 — EE discipline, not a fit. 64508 — water/environmental-balance discipline, not a fit. 64355 — non-US location (Saskatchewan, Canada), excluded per US-only scope. 64862 — search-result title truncated 'Spring 2027'; the full posting title is actually 'Summer 2027' — wrong season. None added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C499"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C515"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 5 checked-excluded (2026-09-30 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hzhu4Ft7Jf2VVKdHV8jctn
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M267"/>
+  <dimension ref="A1:M268"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9739,16 +9739,16 @@
         <v>Flex (Flextronics International)</v>
       </c>
       <c r="B246" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>NPI Process Engineering Co-op</v>
       </c>
       <c r="C246" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing Engineering (New Product Introduction)</v>
       </c>
       <c r="D246" t="str">
         <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
       </c>
       <c r="E246" t="str">
-        <v>Hollis, NH</v>
+        <v>Hollis, NH (posting body says Nashua, NH site)</v>
       </c>
       <c r="F246">
         <v>45</v>
@@ -9757,109 +9757,109 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H246" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/Mechanical-Engineering-Co-op_WD226382</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/NPI-Process-Engineering-Co-op_WD226387</v>
       </c>
       <c r="I246" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226382, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226387, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
       </c>
       <c r="J246" t="str">
-        <v>TIME-SENSITIVE: posting's own end date is 2026-09-30 — application window closes within ~1 day of this run. Medical products (wearables, therapy systems, surgical robotics) mechanical design/CAD/prototyping work. 2nd or 3rd co-op preferred, SolidWorks required. A prior run excluded this req because its TITLE alone states no season, but the body text explicitly names the year ('Jan - Jun 2027') — re-evaluated as meeting the season-stated bar on body text, consistent with how other title/body-text discrepancies (e.g. Flex's own Orangeburg req) are handled elsewhere in this tracker. Pay/citizenship not stated.</v>
+        <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>RTX / Collins Aerospace</v>
       </c>
       <c r="B247" t="str">
-        <v>NPI Process Engineering Co-op</v>
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C247" t="str">
-        <v>Manufacturing Engineering (New Product Introduction)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D247" t="str">
-        <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E247" t="str">
-        <v>Hollis, NH (posting body says Nashua, NH site)</v>
+        <v>Cedar Rapids, IA</v>
       </c>
       <c r="F247">
-        <v>45</v>
+        <v>1090</v>
       </c>
       <c r="G247" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated on posting (RTX co-op program range generally $37,000–$82,000/yr annualized per boilerplate)</v>
       </c>
       <c r="H247" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/NPI-Process-Engineering-Co-op_WD226387</v>
+        <v>https://careers.rtx.com/global/en/job/01872047/Mechanical-Engineering-Co-op-Winter-Spring-2027</v>
       </c>
       <c r="I247" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226387, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
+        <v>Yes — independently fetched raw HTML/JSON-LD directly (bypassing careers.rtx.com's unreliable WebFetch rendering), req 01872047, datePosted 2026-09-28, title states '(Winter/Spring 2027)' verbatim, 'Apply Now' present, no filled/closed markers.</v>
       </c>
       <c r="J247" t="str">
-        <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
+        <v>Displays, Controls, Computing &amp; Networking dept at Collins Aerospace — cockpit displays/control panels, servo actuation, avionics hardware. 'Immerse yourself in a full-time... co-op session, that will run January- July/August.' U.S. citizenship required (no clearance required). New req distinct from the already-tracked Chemical/Materials Co-op (01871473) and Mechanical Design Co-op (01871736, Jamestown ND) at the same company.</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>RTX / Collins Aerospace</v>
+        <v>Flex (Flextronics International)</v>
       </c>
       <c r="B248" t="str">
-        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Mechanical Engineering Co-op - Spring 2027</v>
       </c>
       <c r="C248" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Industrial Engineering</v>
       </c>
       <c r="D248" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E248" t="str">
-        <v>Cedar Rapids, IA</v>
+        <v>Orangeburg, SC</v>
       </c>
       <c r="F248">
-        <v>1090</v>
+        <v>900</v>
       </c>
       <c r="G248" t="str">
-        <v>Not stated on posting (RTX co-op program range generally $37,000–$82,000/yr annualized per boilerplate)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H248" t="str">
-        <v>https://careers.rtx.com/global/en/job/01872047/Mechanical-Engineering-Co-op-Winter-Spring-2027</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Mechanical-Engineering-Co-op---Fall-2026_WD227049</v>
       </c>
       <c r="I248" t="str">
-        <v>Yes — independently fetched raw HTML/JSON-LD directly (bypassing careers.rtx.com's unreliable WebFetch rendering), req 01872047, datePosted 2026-09-28, title states '(Winter/Spring 2027)' verbatim, 'Apply Now' present, no filled/closed markers.</v>
+        <v>Yes — independently fetched directly via Flex's own Workday CXS API, req WD227049, canApply true, posted 26 days ago, title states 'Mechanical Engineering Co-op - Spring 2027' verbatim, quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 school semester.'</v>
       </c>
       <c r="J248" t="str">
-        <v>Displays, Controls, Computing &amp; Networking dept at Collins Aerospace — cockpit displays/control panels, servo actuation, avionics hardware. 'Immerse yourself in a full-time... co-op session, that will run January- July/August.' U.S. citizenship required (no clearance required). New req distinct from the already-tracked Chemical/Materials Co-op (01871473) and Mechanical Design Co-op (01871736, Jamestown ND) at the same company.</v>
+        <v>TIME-SENSITIVE: posting's own end date is 2026-10-03 — 3 days left to apply as of this run. NOTE: URL slug reads 'Fall-2026' (stale rename leftover, same pattern as the already-tracked Orangeburg Industrial Engineering Co-Op WD226357) but title/body both explicitly say 'Spring 2027' — treated as authoritative per the verification bar. Manufacturing Engineering Manager team — time studies, CAD, DOE projects. 'Is Sponsorship Available? No' (no visa sponsorship, not a citizenship/ITAR requirement). Pay not stated.</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>Specter Aerospace</v>
       </c>
       <c r="B249" t="str">
-        <v>Mechanical Engineering Co-op - Spring 2027</v>
+        <v>Mechanical Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C249" t="str">
-        <v>Mechanical / Industrial Engineering</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D249" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E249" t="str">
-        <v>Orangeburg, SC</v>
+        <v>Boston, MA (Seaport)</v>
       </c>
       <c r="F249">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="G249" t="str">
-        <v>Not stated on posting</v>
+        <v>$23-$30/hr</v>
       </c>
       <c r="H249" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Mechanical-Engineering-Co-op---Fall-2026_WD227049</v>
+        <v>https://specteraerospace.bamboohr.com/careers/124</v>
       </c>
       <c r="I249" t="str">
-        <v>Yes — independently fetched directly via Flex's own Workday CXS API, req WD227049, canApply true, posted 26 days ago, title states 'Mechanical Engineering Co-op - Spring 2027' verbatim, quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 school semester.'</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API (specteraerospace.bamboohr.com/careers/124/detail), status Open, posted 2026-08-13, title states 'Mechanical Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J249" t="str">
-        <v>TIME-SENSITIVE: posting's own end date is 2026-10-03 — 3 days left to apply as of this run. NOTE: URL slug reads 'Fall-2026' (stale rename leftover, same pattern as the already-tracked Orangeburg Industrial Engineering Co-Op WD226357) but title/body both explicitly say 'Spring 2027' — treated as authoritative per the verification bar. Manufacturing Engineering Manager team — time studies, CAD, DOE projects. 'Is Sponsorship Available? No' (no visa sponsorship, not a citizenship/ITAR requirement). Pay not stated.</v>
+        <v>New company for the tracker — hypersonic flight vehicle startup (Boston Seaport + Peabody, MA offices), funded by government R&amp;D + private funding. Vehicle Development team, designing components/subsystems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance). Strong Boston-area match.</v>
       </c>
     </row>
     <row r="250">
@@ -9867,7 +9867,7 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B250" t="str">
-        <v>Mechanical Engineer Co-Op - Spring 2027</v>
+        <v>Vehicle Design Co-Op - Spring 2027</v>
       </c>
       <c r="C250" t="str">
         <v>Mechanical / Aerospace Engineering</v>
@@ -9885,13 +9885,13 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H250" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/124</v>
+        <v>https://specteraerospace.bamboohr.com/careers/116</v>
       </c>
       <c r="I250" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API (specteraerospace.bamboohr.com/careers/124/detail), status Open, posted 2026-08-13, title states 'Mechanical Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Vehicle Design Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J250" t="str">
-        <v>New company for the tracker — hypersonic flight vehicle startup (Boston Seaport + Peabody, MA offices), funded by government R&amp;D + private funding. Vehicle Development team, designing components/subsystems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance). Strong Boston-area match.</v>
+        <v>Sibling req to the Mechanical Engineer Co-Op above, same company/site. Vehicle Design team, designing components/systems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="251">
@@ -9899,31 +9899,31 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B251" t="str">
-        <v>Vehicle Design Co-Op - Spring 2027</v>
+        <v>Propulsion Test Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C251" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
       </c>
       <c r="D251" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E251" t="str">
-        <v>Boston, MA (Seaport)</v>
+        <v>Peabody, MA</v>
       </c>
       <c r="F251">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G251" t="str">
         <v>$23-$30/hr</v>
       </c>
       <c r="H251" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/116</v>
+        <v>https://specteraerospace.bamboohr.com/careers/117</v>
       </c>
       <c r="I251" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Vehicle Design Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Propulsion Test Engineering Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J251" t="str">
-        <v>Sibling req to the Mechanical Engineer Co-Op above, same company/site. Vehicle Design team, designing components/systems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>Design, manufacturing, and test of advanced ramjet/scramjet engine hardware for hypersonic propulsion systems. Note: posting says Specter hires both this and the Propulsion Design Engineering Co-op (below) from a shared applicant pool depending on interest/fit. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="252">
@@ -9931,7 +9931,7 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B252" t="str">
-        <v>Propulsion Test Engineering Co-Op - Spring 2027</v>
+        <v>Propulsion Design Engineering Co-op - Spring 2027</v>
       </c>
       <c r="C252" t="str">
         <v>Mechanical / Aerospace Engineering (Propulsion)</v>
@@ -9949,13 +9949,13 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H252" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/117</v>
+        <v>https://specteraerospace.bamboohr.com/careers/118</v>
       </c>
       <c r="I252" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Propulsion Test Engineering Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'Propulsion Design Engineering Co-op - Spring 2027' verbatim.</v>
       </c>
       <c r="J252" t="str">
-        <v>Design, manufacturing, and test of advanced ramjet/scramjet engine hardware for hypersonic propulsion systems. Note: posting says Specter hires both this and the Propulsion Design Engineering Co-op (below) from a shared applicant pool depending on interest/fit. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>Sibling/shared-pool req to Propulsion Test Engineering Co-Op above (same site, same applicant pool per posting text). Design, manufacturing, and test of ramjet/scramjet engine hardware. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="253">
@@ -9963,10 +9963,10 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B253" t="str">
-        <v>Propulsion Design Engineering Co-op - Spring 2027</v>
+        <v>PLC/Controls Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C253" t="str">
-        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
+        <v>Controls / Mechanical / Electrical Engineering</v>
       </c>
       <c r="D253" t="str">
         <v>Spring 2027</v>
@@ -9981,13 +9981,13 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H253" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/118</v>
+        <v>https://specteraerospace.bamboohr.com/careers/123</v>
       </c>
       <c r="I253" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'Propulsion Design Engineering Co-op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'PLC/Controls Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J253" t="str">
-        <v>Sibling/shared-pool req to Propulsion Test Engineering Co-Op above (same site, same applicant pool per posting text). Design, manufacturing, and test of ramjet/scramjet engine hardware. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>PLC software design (Beckhoff/TwinCAT ecosystem), electrical control-panel design, sensor/actuator integration for the Specter engine test facility. Open to Computer/Electrical/Mechanical Engineering or CS majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="254">
@@ -9995,10 +9995,10 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B254" t="str">
-        <v>PLC/Controls Engineer Co-Op - Spring 2027</v>
+        <v>Computational Design Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C254" t="str">
-        <v>Controls / Mechanical / Electrical Engineering</v>
+        <v>Mechanical / Computational Engineering</v>
       </c>
       <c r="D254" t="str">
         <v>Spring 2027</v>
@@ -10013,77 +10013,77 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H254" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/123</v>
+        <v>https://specteraerospace.bamboohr.com/careers/127</v>
       </c>
       <c r="I254" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'PLC/Controls Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-08-13, title states 'Computational Design Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J254" t="str">
-        <v>PLC software design (Beckhoff/TwinCAT ecosystem), electrical control-panel design, sensor/actuator integration for the Specter engine test facility. Open to Computer/Electrical/Mechanical Engineering or CS majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>Reusable computational geometry models / implicit modeling (Rhino/Grasshopper, nTop, PicoGK) for high-speed airbreathing testbed vehicle design and analysis. Open to Engineering/Math/CS/Physics majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>Specter Aerospace</v>
+        <v>Shaw Industries</v>
       </c>
       <c r="B255" t="str">
-        <v>Computational Design Engineer Co-Op - Spring 2027</v>
+        <v>Engineering Internship/Co-op Spring 2027</v>
       </c>
       <c r="C255" t="str">
-        <v>Mechanical / Computational Engineering</v>
+        <v>Manufacturing / Industrial Engineering</v>
       </c>
       <c r="D255" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E255" t="str">
-        <v>Peabody, MA</v>
+        <v>Dalton, GA</v>
       </c>
       <c r="F255">
-        <v>19</v>
+        <v>1050</v>
       </c>
       <c r="G255" t="str">
-        <v>$23-$30/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H255" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/127</v>
+        <v>https://shawinc.wd1.myworkdayjobs.com/en-US/External/job/Shaw-Plant-7C-2208-S-Hamilton-Street-Dalton-GA-30721-USA/Engineering-Internship-Co-op-Spring-2027_R-156324</v>
       </c>
       <c r="I255" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-08-13, title states 'Computational Design Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Shaw Industries' own Workday CXS API, req R-156324, title states 'Engineering Internship/Co-op Spring 2027' verbatim, posted 30+ days ago (exact date not disclosed by API).</v>
       </c>
       <c r="J255" t="str">
-        <v>Reusable computational geometry models / implicit modeling (Rhino/Grasshopper, nTop, PicoGK) for high-speed airbreathing testbed vehicle design and analysis. Open to Engineering/Math/CS/Physics majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>New company for the tracker — flooring manufacturer, wholly-owned Berkshire Hathaway subsidiary, $5B+ annual sales. Rotating or sequential semesters working onsite in Shaw's manufacturing operations facilities in an engineering capacity; student matched to a facility per skills/interests. Citizenship/GPA/eligibility not stated on posting — confirm directly.</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>Shaw Industries</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B256" t="str">
-        <v>Engineering Internship/Co-op Spring 2027</v>
+        <v>Operations &amp; Automation Engineering Co-op/Intern - Spring 2027</v>
       </c>
       <c r="C256" t="str">
-        <v>Manufacturing / Industrial Engineering</v>
+        <v>Controls / Automation / Industrial Engineering</v>
       </c>
       <c r="D256" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E256" t="str">
-        <v>Dalton, GA</v>
+        <v>Bartow, FL</v>
       </c>
       <c r="F256">
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="G256" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated on posting (housing/relocation available for qualified candidates)</v>
       </c>
       <c r="H256" t="str">
-        <v>https://shawinc.wd1.myworkdayjobs.com/en-US/External/job/Shaw-Plant-7C-2208-S-Hamilton-Street-Dalton-GA-30721-USA/Engineering-Internship-Co-op-Spring-2027_R-156324</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Bartow-FL/Operations---Automation-Engineering-Co-op-Intern---Spring-2027_64675-1</v>
       </c>
       <c r="I256" t="str">
-        <v>Yes — independently fetched directly via Shaw Industries' own Workday CXS API, req R-156324, title states 'Engineering Internship/Co-op Spring 2027' verbatim, posted 30+ days ago (exact date not disclosed by API).</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64675, exact quote: 'Term Jan 11th, 2027 to April 23th, 2027 Full time Co-Op/Internship.'</v>
       </c>
       <c r="J256" t="str">
-        <v>New company for the tracker — flooring manufacturer, wholly-owned Berkshire Hathaway subsidiary, $5B+ annual sales. Rotating or sequential semesters working onsite in Shaw's manufacturing operations facilities in an engineering capacity; student matched to a facility per skills/interests. Citizenship/GPA/eligibility not stated on posting — confirm directly.</v>
+        <v>New company for the tracker — NYSE: MOS, world's leading integrated producer of concentrated phosphate and potash fertilizer. Supports plant operations and automated control systems (PLC, DCS, HMI/SCADA) at the Bartow, FL phosphoric-acid manufacturing site. Citizenship not stated on posting.</v>
       </c>
     </row>
     <row r="257">
@@ -10091,63 +10091,63 @@
         <v>The Mosaic Company</v>
       </c>
       <c r="B257" t="str">
-        <v>Operations &amp; Automation Engineering Co-op/Intern - Spring 2027</v>
+        <v>Operations Engineering Co-op/Intern – Spring 2027</v>
       </c>
       <c r="C257" t="str">
-        <v>Controls / Automation / Industrial Engineering</v>
+        <v>Mechanical / Industrial Engineering</v>
       </c>
       <c r="D257" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E257" t="str">
-        <v>Bartow, FL</v>
+        <v>Riverview, FL</v>
       </c>
       <c r="F257">
         <v>1250</v>
       </c>
       <c r="G257" t="str">
-        <v>Not stated on posting (housing/relocation available for qualified candidates)</v>
+        <v>Not stated on posting (relocation package available for qualified candidates)</v>
       </c>
       <c r="H257" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Bartow-FL/Operations---Automation-Engineering-Co-op-Intern---Spring-2027_64675-1</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Riverview-FL/Operations-Engineering-Co-op-Intern---Spring-2027_64656</v>
       </c>
       <c r="I257" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64675, exact quote: 'Term Jan 11th, 2027 to April 23th, 2027 Full time Co-Op/Internship.'</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64656, exact quote: 'Term January 11 to April 23, 2027.'</v>
       </c>
       <c r="J257" t="str">
-        <v>New company for the tracker — NYSE: MOS, world's leading integrated producer of concentrated phosphate and potash fertilizer. Supports plant operations and automated control systems (PLC, DCS, HMI/SCADA) at the Bartow, FL phosphoric-acid manufacturing site. Citizenship not stated on posting.</v>
+        <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>The Mosaic Company</v>
+        <v>Draper Laboratory</v>
       </c>
       <c r="B258" t="str">
-        <v>Operations Engineering Co-op/Intern – Spring 2027</v>
+        <v>Mechanical Engineering &amp; System Packaging Co-Op (Spring 2027)</v>
       </c>
       <c r="C258" t="str">
-        <v>Mechanical / Industrial Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D258" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E258" t="str">
-        <v>Riverview, FL</v>
+        <v>Cambridge, MA</v>
       </c>
       <c r="F258">
-        <v>1250</v>
+        <v>3</v>
       </c>
       <c r="G258" t="str">
-        <v>Not stated on posting (relocation package available for qualified candidates)</v>
+        <v>$20.00–$45.00/hr per posting</v>
       </c>
       <c r="H258" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Riverview-FL/Operations-Engineering-Co-op-Intern---Spring-2027_64656</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Mechanical-Engineering---System-Packaging-Co-Op--Spring-2027-_JR002940</v>
       </c>
       <c r="I258" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64656, exact quote: 'Term January 11 to April 23, 2027.'</v>
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002940), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
       </c>
       <c r="J258" t="str">
-        <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
+        <v>US citizenship required (posting: 'Co-op students must be US citizens who are enrolled in an accredited engineering curriculum'). CAD (SolidWorks/Creo) and FEA (Ansys) work on national-security hardware.</v>
       </c>
     </row>
     <row r="259">
@@ -10155,63 +10155,63 @@
         <v>Draper Laboratory</v>
       </c>
       <c r="B259" t="str">
-        <v>Mechanical Engineering &amp; System Packaging Co-Op (Spring 2027)</v>
+        <v>Digital Engineering – Requirements Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C259" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D259" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E259" t="str">
-        <v>Cambridge, MA</v>
+        <v>Lowell, MA</v>
       </c>
       <c r="F259">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G259" t="str">
-        <v>$20.00–$45.00/hr per posting</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H259" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Mechanical-Engineering---System-Packaging-Co-Op--Spring-2027-_JR002940</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Lowell-MA/Digital-Engineering---Requirements-Engineering-Co-Op--Spring-2027-_JR002944</v>
       </c>
       <c r="I259" t="str">
-        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002940), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002944), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
       </c>
       <c r="J259" t="str">
-        <v>US citizenship required (posting: 'Co-op students must be US citizens who are enrolled in an accredited engineering curriculum'). CAD (SolidWorks/Creo) and FEA (Ansys) work on national-security hardware.</v>
+        <v>US Citizenship required per posting. Digital-twin/model-driven systems engineering support for strategic deterrent, missile-defense, hypersonic, space, and autonomous vehicle programs. Python scripting experience preferred.</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>Draper Laboratory</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B260" t="str">
-        <v>Digital Engineering – Requirements Engineering Co-Op (Spring 2027)</v>
+        <v>Process Engineer Co-Op/Intern - Spring 2027</v>
       </c>
       <c r="C260" t="str">
-        <v>Systems Engineering</v>
+        <v>Mechanical / Chemical / Mining Engineering</v>
       </c>
       <c r="D260" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E260" t="str">
-        <v>Lowell, MA</v>
+        <v>Bradley, FL</v>
       </c>
       <c r="F260">
-        <v>30</v>
+        <v>1250</v>
       </c>
       <c r="G260" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H260" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Lowell-MA/Digital-Engineering---Requirements-Engineering-Co-Op--Spring-2027-_JR002944</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Bradley-FL/Process-Engineer-Co-Op-Intern---Spring-2027_64450</v>
       </c>
       <c r="I260" t="str">
-        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002944), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64450, canApply true.</v>
       </c>
       <c r="J260" t="str">
-        <v>US Citizenship required per posting. Digital-twin/model-driven systems engineering support for strategic deterrent, missile-defense, hypersonic, space, and autonomous vehicle programs. Python scripting experience preferred.</v>
+        <v>Posting explicitly accepts Chemical, Mechanical, and/or Mining Engineering majors. Term Jan 11–Apr 23, 2027 (same as tracker's other Mosaic co-ops). Citizenship not stated.</v>
       </c>
     </row>
     <row r="261">
@@ -10219,16 +10219,16 @@
         <v>The Mosaic Company</v>
       </c>
       <c r="B261" t="str">
-        <v>Process Engineer Co-Op/Intern - Spring 2027</v>
+        <v>Capital Project Engineering Co-Op/Intern - Spring 2027</v>
       </c>
       <c r="C261" t="str">
-        <v>Mechanical / Chemical / Mining Engineering</v>
+        <v>Mechanical / Chemical / Industrial Engineering</v>
       </c>
       <c r="D261" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E261" t="str">
-        <v>Bradley, FL</v>
+        <v>Riverview, FL</v>
       </c>
       <c r="F261">
         <v>1250</v>
@@ -10237,13 +10237,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H261" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Bradley-FL/Process-Engineer-Co-Op-Intern---Spring-2027_64450</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Riverview-FL/Capital-Project-Engineering-Co-Op-Intern---Spring-2027_64455</v>
       </c>
       <c r="I261" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64450, canApply true.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64455, canApply true.</v>
       </c>
       <c r="J261" t="str">
-        <v>Posting explicitly accepts Chemical, Mechanical, and/or Mining Engineering majors. Term Jan 11–Apr 23, 2027 (same as tracker's other Mosaic co-ops). Citizenship not stated.</v>
+        <v>Posting explicitly accepts Chemical, Mechanical, or Industrial Engineer majors. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
       </c>
     </row>
     <row r="262">
@@ -10251,7 +10251,7 @@
         <v>The Mosaic Company</v>
       </c>
       <c r="B262" t="str">
-        <v>Capital Project Engineering Co-Op/Intern - Spring 2027</v>
+        <v>Capital Project Engineering Co-op/Intern - Spring 2027</v>
       </c>
       <c r="C262" t="str">
         <v>Mechanical / Chemical / Industrial Engineering</v>
@@ -10260,54 +10260,54 @@
         <v>Spring 2027</v>
       </c>
       <c r="E262" t="str">
-        <v>Riverview, FL</v>
+        <v>Tampa, FL (Lithia area)</v>
       </c>
       <c r="F262">
-        <v>1250</v>
+        <v>1240</v>
       </c>
       <c r="G262" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H262" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Riverview-FL/Capital-Project-Engineering-Co-Op-Intern---Spring-2027_64455</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Tampa-FL-Lithia-area/Capital-Project-Engineering-Co-op-Intern---Spring-2027_64392</v>
       </c>
       <c r="I262" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64455, canApply true.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64392, canApply true.</v>
       </c>
       <c r="J262" t="str">
-        <v>Posting explicitly accepts Chemical, Mechanical, or Industrial Engineer majors. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+        <v>Sibling req to the Riverview, FL Capital Project Engineering Co-op above, same discipline, different site. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>The Mosaic Company</v>
+        <v>Gulfstream Aerospace</v>
       </c>
       <c r="B263" t="str">
-        <v>Capital Project Engineering Co-op/Intern - Spring 2027</v>
+        <v>Spring 2027 - IEF - Stress Engineering - Collegiate Associate Intern</v>
       </c>
       <c r="C263" t="str">
-        <v>Mechanical / Chemical / Industrial Engineering</v>
+        <v>Aerospace / Structural Engineering</v>
       </c>
       <c r="D263" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E263" t="str">
-        <v>Tampa, FL (Lithia area)</v>
+        <v>Savannah, GA</v>
       </c>
       <c r="F263">
-        <v>1240</v>
+        <v>900</v>
       </c>
       <c r="G263" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H263" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Tampa-FL-Lithia-area/Capital-Project-Engineering-Co-op-Intern---Spring-2027_64392</v>
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Stress-Engineering-Collegiate-Associate-Intern-GA-31401/1423681300/</v>
       </c>
       <c r="I263" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64392, canApply true.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Stress Engineering'.</v>
       </c>
       <c r="J263" t="str">
-        <v>Sibling req to the Riverview, FL Capital Project Engineering Co-op above, same discipline, different site. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+        <v>Discipline list per posting: Aerospace, Civil, Structural, Mechanical Engineering, Computer Science. GPA ≥3.0 cumulative (unrounded) required. No visa sponsorship — effectively requires US citizenship/permanent residency.</v>
       </c>
     </row>
     <row r="264">
@@ -10315,10 +10315,10 @@
         <v>Gulfstream Aerospace</v>
       </c>
       <c r="B264" t="str">
-        <v>Spring 2027 - IEF - Stress Engineering - Collegiate Associate Intern</v>
+        <v>Spring 2027 - IEF - Materials and Processes Engineering College Associate</v>
       </c>
       <c r="C264" t="str">
-        <v>Aerospace / Structural Engineering</v>
+        <v>Materials Engineering</v>
       </c>
       <c r="D264" t="str">
         <v>Spring 2027</v>
@@ -10333,109 +10333,141 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H264" t="str">
-        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Stress-Engineering-Collegiate-Associate-Intern-GA-31401/1423681300/</v>
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Materials-and-Processes-Engineering-College-Associate-GA-31401/1432666200/</v>
       </c>
       <c r="I264" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Stress Engineering'.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Materials and Processes'.</v>
       </c>
       <c r="J264" t="str">
-        <v>Discipline list per posting: Aerospace, Civil, Structural, Mechanical Engineering, Computer Science. GPA ≥3.0 cumulative (unrounded) required. No visa sponsorship — effectively requires US citizenship/permanent residency.</v>
+        <v>Discipline list per posting: Mechanical, Materials Science &amp; Engineering, Materials Engineering, Aerospace, Chemical Engineering, Metallurgy. GPA ≥3.0 cumulative required. No visa sponsorship.</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>Gulfstream Aerospace</v>
+        <v>Pyka</v>
       </c>
       <c r="B265" t="str">
-        <v>Spring 2027 - IEF - Materials and Processes Engineering College Associate</v>
+        <v>Mechanical Engineering Internship - Winter/Spring 2027 (Dropship, Early Interest)</v>
       </c>
       <c r="C265" t="str">
-        <v>Materials Engineering</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D265" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E265" t="str">
-        <v>Savannah, GA</v>
+        <v>Alameda, CA</v>
       </c>
       <c r="F265">
-        <v>900</v>
+        <v>2700</v>
       </c>
       <c r="G265" t="str">
-        <v>Not stated on posting</v>
+        <v>$35–$40/hr per posting</v>
       </c>
       <c r="H265" t="str">
-        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Materials-and-Processes-Engineering-College-Associate-GA-31401/1432666200/</v>
+        <v>https://jobs.lever.co/pyka/2702593a-7482-4d2b-93f3-ef97e2cf7df7</v>
       </c>
       <c r="I265" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Materials and Processes'.</v>
+        <v>Yes — independently fetched directly via Lever's public API, posting live, text confirms 'Winter/Spring 2027'.</v>
       </c>
       <c r="J265" t="str">
-        <v>Discipline list per posting: Mechanical, Materials Science &amp; Engineering, Materials Engineering, Aerospace, Chemical Engineering, Metallurgy. GPA ≥3.0 cumulative required. No visa sponsorship.</v>
+        <v>IMPORTANT: explicitly an 'Early Interest Application' — posting states formal interviews for the 2027 cohort won't begin until October 2026; applying now only queues your profile for later review, not an active hiring process yet. Visa sponsorship offered. Electric-aviation 'Dropship' cargo aircraft program.</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>Pyka</v>
+        <v>General Astronautics</v>
       </c>
       <c r="B266" t="str">
-        <v>Mechanical Engineering Internship - Winter/Spring 2027 (Dropship, Early Interest)</v>
+        <v>Spring 2027 Mechanical Engineering Internship/Co-op</v>
       </c>
       <c r="C266" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D266" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E266" t="str">
-        <v>Alameda, CA</v>
+        <v>San Francisco, CA</v>
       </c>
       <c r="F266">
         <v>2700</v>
       </c>
       <c r="G266" t="str">
-        <v>$35–$40/hr per posting</v>
+        <v>$30.00/hr (Sophomore), $35.00/hr (Junior/Senior) per posting</v>
       </c>
       <c r="H266" t="str">
-        <v>https://jobs.lever.co/pyka/2702593a-7482-4d2b-93f3-ef97e2cf7df7</v>
+        <v>https://www.workatastartup.com/jobs/103200</v>
       </c>
       <c r="I266" t="str">
-        <v>Yes — independently fetched directly via Lever's public API, posting live, text confirms 'Winter/Spring 2027'.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027 Mechanical Engineering Internship/Co-op'; also cross-confirmed on ycombinator.com's own company page.</v>
       </c>
       <c r="J266" t="str">
-        <v>IMPORTANT: explicitly an 'Early Interest Application' — posting states formal interviews for the 2027 cohort won't begin until October 2026; applying now only queues your profile for later review, not an active hiring process yet. Visa sponsorship offered. Electric-aviation 'Dropship' cargo aircraft program.</v>
+        <v>New company for the tracker — YC-backed startup building autonomous robots for orbital manufacturing. Minimum 12 weeks on-site in San Francisco required. 'U.S. citizen or national, U.S. lawful permanent resident, or eligible for authorization under U.S. export regulations.' Applies via YC's own account/signup flow (workatastartup.com).</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>General Astronautics</v>
+        <v>Simpson Gumpertz &amp; Heger (SGH)</v>
       </c>
       <c r="B267" t="str">
-        <v>Spring 2027 Mechanical Engineering Internship/Co-op</v>
+        <v>Technical Co-Op, Structural Engineering</v>
       </c>
       <c r="C267" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D267" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E267" t="str">
-        <v>San Francisco, CA</v>
+        <v>Waltham, MA</v>
       </c>
       <c r="F267">
-        <v>2700</v>
+        <v>10</v>
       </c>
       <c r="G267" t="str">
-        <v>$30.00/hr (Sophomore), $35.00/hr (Junior/Senior) per posting</v>
+        <v>$29.25–$38.25/hr depending on degree level, plus $1,000 sign-on bonus per posting</v>
       </c>
       <c r="H267" t="str">
-        <v>https://www.workatastartup.com/jobs/103200</v>
+        <v>https://www.sgh.com/careers/job-openings/view-job/8760874002?gh_jid=8760874002</v>
       </c>
       <c r="I267" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027 Mechanical Engineering Internship/Co-op'; also cross-confirmed on ycombinator.com's own company page.</v>
+        <v>Partial — sgh.com's own job-detail page is JS-rendered and returned only the careers landing page on direct fetch (confirmed independently this run). Content (exact title, Waltham MA, term, pay, 'updated 1 week ago') was confirmed via an aggregator mirror (dreamworkhq.com) that links through to this same gh_jid. Not independently opened on sgh.com itself.</v>
       </c>
       <c r="J267" t="str">
-        <v>New company for the tracker — YC-backed startup building autonomous robots for orbital manufacturing. Minimum 12 weeks on-site in San Francisco required. 'U.S. citizen or national, U.S. lawful permanent resident, or eligible for authorization under U.S. export regulations.' Applies via YC's own account/signup flow (workatastartup.com).</v>
+        <v>New company for the tracker — structural/civil engineering consultancy (also runs a sibling Technical Co-Op, Civil Engineering req at the same Waltham office, and a Plumbing &amp; Fire Protection Co-op at Buro Happold-style disciplines — see `checked` for the civil sibling, excluded on discipline-fit grounds). Fits Hamza's 'adjacent — structural' category.</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>Cyvl</v>
+      </c>
+      <c r="B268" t="str">
+        <v>Hardware Engineering Intern (Co-Op Spring 2027 / Intern Summer 2027)</v>
+      </c>
+      <c r="C268" t="str">
+        <v>Hardware/Mechanical Engineering (sensor mounts/enclosures, CAD, machining)</v>
+      </c>
+      <c r="D268" t="str">
+        <v>Spring 2027 (Co-Op track; a separate Summer 2027 Intern track is also offered on the same posting)</v>
+      </c>
+      <c r="E268" t="str">
+        <v>Somerville, MA</v>
+      </c>
+      <c r="F268">
+        <v>3</v>
+      </c>
+      <c r="G268" t="str">
+        <v>Not confirmed on primary source</v>
+      </c>
+      <c r="H268" t="str">
+        <v>https://jobs.ashbyhq.com/cyvl/3590960d-4d02-48bb-a335-cb82e121a01e</v>
+      </c>
+      <c r="I268" t="str">
+        <v>Partial — direct fetch of the Ashby posting (JS-rendered) returned only the job title; full details (Somerville MA location, 'posted 2 weeks ago', active application link matching this same URL) were confirmed via an aggregator mirror (dreamworkhq.com), not independently opened on Ashby itself.</v>
+      </c>
+      <c r="J268" t="str">
+        <v>New company for the tracker — robotics/mapping hardware startup (sensor mounts/enclosures, CAD, machining for mobile-mapping hardware). Boston-metro (Somerville). Season stated on the posting title itself as a dual Co-Op(Spring)/Intern(Summer) track; Spring 2027 Co-Op option is the qualifying track.</v>
       </c>
     </row>
   </sheetData>
@@ -10912,14 +10944,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M267"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M268"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C515"/>
+  <dimension ref="A1:C520"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -16582,9 +16614,64 @@
         <v>2026-09-30: found during the same-company sweep that surfaced reqs 64450/64455/64392 (added to `rows`). 64427 — EE discipline, not a fit. 64508 — water/environmental-balance discipline, not a fit. 64355 — non-US location (Saskatchewan, Canada), excluded per US-only scope. 64862 — search-result title truncated 'Spring 2027'; the full posting title is actually 'Summer 2027' — wrong season. None added.</v>
       </c>
     </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>Flex (Flextronics International, Hollis, NH)</v>
+      </c>
+      <c r="B516" t="str">
+        <v>Mechanical Engineering Co-op, req WD226382 — moved from `rows`</v>
+      </c>
+      <c r="C516" t="str">
+        <v>2026-09-30 (later run): this req's own posted end date was 2026-09-30 (today). Re-checked via Flex's own Workday CXS API — a full-text search for '226382' now returns 0 results, a location search for Hollis/Nashua NH returns only the still-open NPI Process Engineering sibling (WD226387), and the direct req URL now returns a permission-denied response consistent with expiry. Moved here from `rows` as closed.</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B517" t="str">
+        <v>Co-Op Student Engineering (JR002974, Lowell/Cambridge MA); Digital Engineering – Requirements Engineering Intern (JR002945, Summer 2027)</v>
+      </c>
+      <c r="C517" t="str">
+        <v>2026-09-30 (later run): both newly found via a full Workday CXS sweep. JR002974 is live/open but states no season or year anywhere on the posting — fails the season-stated bar (evergreen/general engineering co-op req). JR002945 is explicitly titled Summer 2027 — wrong season. Neither added; JR002974 worth a re-check if it's ever updated with a dated term.</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>Simpson Gumpertz &amp; Heger (SGH), Waltham MA</v>
+      </c>
+      <c r="B518" t="str">
+        <v>Technical Co-Op, Civil Engineering (Winter/Spring 2027) — sibling to the Structural Engineering Co-Op added to `rows` this run</v>
+      </c>
+      <c r="C518" t="str">
+        <v>2026-09-30 (later run): confirmed live/season-correct via the same aggregator mirror, but civil engineering discipline doesn't cleanly fit Hamza's target list (mechanical/aerospace/manufacturing/robotics/industrial/materials/structural/controls). Excluded on discipline-fit grounds; the sibling Structural Engineering req at the same office DID qualify.</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>Genentech</v>
+      </c>
+      <c r="B519" t="str">
+        <v>'2027 Spring Intern - Pharma Technical Development - Device Development' — re-check of the standing lead above</v>
+      </c>
+      <c r="C519" t="str">
+        <v>2026-09-30 (later run): the two sibling req IDs (202609-122484, 202609-123436) that were previously confirmed live on careers.gene.com now both return HTTP 410 Gone when re-fetched directly. Strong signal the entire September-2026 PTD Spring-2027 intern posting batch (including Device Development, if it ever had a distinct req) has expired. Still no live canonical URL ever found for the Device Development role specifically — recommend dropping this from active re-checking unless a fresh, dated posting surfaces.</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>Lam Research / MACOM / Waters Corporation / Parker Hannifin</v>
+      </c>
+      <c r="B520" t="str">
+        <v>Re-check via alternate access methods (Google-indexed snippets, aggregator mirrors) for each company's real ATS/ID</v>
+      </c>
+      <c r="C520" t="str">
+        <v>2026-09-30 (later run): no change in live/open status for any of the four — all remain unverifiable via any method tried this run, consistent with many prior runs. Progress made identifying platforms: Lam Research confirmed on Eightfold 'PCSX' (lamresearch.eightfold.ai / careers.lamresearch.com), still auth-walled; MACOM confirmed on Cornerstone OnDemand (macomtech.csod.com, careersite ID 4), API still returns 'CSOD Unauthorized Exception'; Waters and Parker Hannifin both remain fully WAF/Cloudflare-blocked with no working alternate access (Wayback Machine unavailable in this environment). No postings added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C515"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C520"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 7 new postings, 8 checked-excluded (2026-09-30 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W5Y3THFA5mrheUGJSEGaH6
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M268"/>
+  <dimension ref="A1:M275"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -10432,10 +10432,10 @@
         <v>https://www.sgh.com/careers/job-openings/view-job/8760874002?gh_jid=8760874002</v>
       </c>
       <c r="I267" t="str">
-        <v>Partial — sgh.com's own job-detail page is JS-rendered and returned only the careers landing page on direct fetch (confirmed independently this run). Content (exact title, Waltham MA, term, pay, 'updated 1 week ago') was confirmed via an aggregator mirror (dreamworkhq.com) that links through to this same gh_jid. Not independently opened on sgh.com itself.</v>
+        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: sgh.com's job board is embedded from Greenhouse; direct fetch of Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/simpsongumpertzheger/jobs/8760874002) independently confirmed title 'Technical Co-Op, Structural Engineering Spring 2027', Waltham MA, updated_at 2026-09-21, and body text 'seeking current students for a Winter 2027 Co-Op internship in our Waltham, MA office' plus the pay breakdown — a live-only feed, not an aggregator mirror.</v>
       </c>
       <c r="J267" t="str">
-        <v>New company for the tracker — structural/civil engineering consultancy (also runs a sibling Technical Co-Op, Civil Engineering req at the same Waltham office, and a Plumbing &amp; Fire Protection Co-op at Buro Happold-style disciplines — see `checked` for the civil sibling, excluded on discipline-fit grounds). Fits Hamza's 'adjacent — structural' category.</v>
+        <v>New company for the tracker — structural/civil engineering consultancy (also runs a sibling Technical Co-Op, Civil Engineering req and a Geotechnical Engineering Co-Op req at the same Waltham office — see `checked`, excluded on discipline-fit grounds). Fits Hamza's 'adjacent — structural' category. Posting itself uses both 'Winter 2027' (body) and 'Spring 2027' (title) — qualifies either way per the task's season rule.</v>
       </c>
     </row>
     <row r="268">
@@ -10464,10 +10464,234 @@
         <v>https://jobs.ashbyhq.com/cyvl/3590960d-4d02-48bb-a335-cb82e121a01e</v>
       </c>
       <c r="I268" t="str">
-        <v>Partial — direct fetch of the Ashby posting (JS-rendered) returned only the job title; full details (Somerville MA location, 'posted 2 weeks ago', active application link matching this same URL) were confirmed via an aggregator mirror (dreamworkhq.com), not independently opened on Ashby itself.</v>
+        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: Ashby publishes a public JSON API (api.ashbyhq.com/posting-api/job-board/cyvl); direct fetch independently confirmed isListed: true, publishedAt 2026-09-14, address Boston MA (primary)/Somerville MA (secondary), and body text 'This role is open as a Spring 2027 co-op or a Summer 2027 internship' — not an aggregator mirror.</v>
       </c>
       <c r="J268" t="str">
-        <v>New company for the tracker — robotics/mapping hardware startup (sensor mounts/enclosures, CAD, machining for mobile-mapping hardware). Boston-metro (Somerville). Season stated on the posting title itself as a dual Co-Op(Spring)/Intern(Summer) track; Spring 2027 Co-Op option is the qualifying track.</v>
+        <v>New company for the tracker — robotics/mapping hardware startup (sensor mounts/enclosures, CAD, machining for mobile-mapping hardware). Boston-metro (primary address is Boston, MA itself; Somerville MA listed as secondary). Season stated on the posting title itself as a dual Co-Op(Spring)/Intern(Summer) track; Spring 2027 Co-Op option is the qualifying track.</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>Hydrite Chemical Co.</v>
+      </c>
+      <c r="B269" t="str">
+        <v>Engineering Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C269" t="str">
+        <v>Mechanical/Chemical Engineering</v>
+      </c>
+      <c r="D269" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E269" t="str">
+        <v>Lubbock, TX</v>
+      </c>
+      <c r="F269">
+        <v>1780</v>
+      </c>
+      <c r="G269" t="str">
+        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
+      </c>
+      <c r="H269" t="str">
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8173754</v>
+      </c>
+      <c r="I269" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8173754), which only lists currently-open postings. Body quote: 'This position will run full-time from January - August 2027.' Degree preference: 'Mechanical or Chemical.'</v>
+      </c>
+      <c r="J269" t="str">
+        <v>New company for the tracker — industrial/specialty chemical manufacturer. No citizenship/ITAR language observed on posting.</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>Hydrite Chemical Co.</v>
+      </c>
+      <c r="B270" t="str">
+        <v>Engineering Co-Op Spring 2027</v>
+      </c>
+      <c r="C270" t="str">
+        <v>Mechanical/Industrial/Chemical Engineering</v>
+      </c>
+      <c r="D270" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E270" t="str">
+        <v>Brookfield, WI</v>
+      </c>
+      <c r="F270">
+        <v>990</v>
+      </c>
+      <c r="G270" t="str">
+        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
+      </c>
+      <c r="H270" t="str">
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8179653</v>
+      </c>
+      <c r="I270" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8179653), which only lists currently-open postings. Body quote: 'This role will run from January 2027- End of Summer 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
+      </c>
+      <c r="J270" t="str">
+        <v>New company for the tracker. A distinct sibling req at the same site, titled 'Engineering Co-Op (Fall 2027)' (ID 8179630), is Fall-2027-only and excluded.</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>Hydrite Chemical Co.</v>
+      </c>
+      <c r="B271" t="str">
+        <v>Engineering Co-Op (Spring OR Fall 2027)</v>
+      </c>
+      <c r="C271" t="str">
+        <v>Mechanical/Industrial/Chemical Engineering</v>
+      </c>
+      <c r="D271" t="str">
+        <v>Spring 2027 (dual Spring/Fall 2027 track; Spring option qualifies)</v>
+      </c>
+      <c r="E271" t="str">
+        <v>Cottage Grove, WI</v>
+      </c>
+      <c r="F271">
+        <v>990</v>
+      </c>
+      <c r="G271" t="str">
+        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
+      </c>
+      <c r="H271" t="str">
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8185948</v>
+      </c>
+      <c r="I271" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8185948), which only lists currently-open postings. Body quote: 'This position is able to run full-time from January - August 2027 OR May/June 2027-December 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
+      </c>
+      <c r="J271" t="str">
+        <v>New company for the tracker.</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>Buro Happold</v>
+      </c>
+      <c r="B272" t="str">
+        <v>Structural Co-op - Boston - Spring 2027</v>
+      </c>
+      <c r="C272" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D272" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E272" t="str">
+        <v>Boston, MA</v>
+      </c>
+      <c r="F272">
+        <v>0</v>
+      </c>
+      <c r="G272" t="str">
+        <v>$24–$34/hr per posting</v>
+      </c>
+      <c r="H272" t="str">
+        <v>https://vacancies.burohappold.com/jobs/job/Structural-Coop-Boston-Spring-2027/2464</v>
+      </c>
+      <c r="I272" t="str">
+        <v>Yes — independently fetched directly, HTTP 200, page confirms 'Structural Co-op' title, 'Spring 2027', '$24 to $34' pay, and 'No expiry' status on the posting itself.</v>
+      </c>
+      <c r="J272" t="str">
+        <v>New req at an already-tracked employer (sibling to the already-tracked Mechanical Co-op, job 2462, and the excluded Plumbing &amp; Fire Protection Co-op, job 2463). Fits Hamza's 'adjacent — structural' category.</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B273" t="str">
+        <v>Co-op, Quality Engineering: January-June (Onsite)</v>
+      </c>
+      <c r="C273" t="str">
+        <v>Quality Engineering (Lean Manufacturing / Six Sigma)</v>
+      </c>
+      <c r="D273" t="str">
+        <v>Spring 2027 (Jan 11 – Jun 30, 2027)</v>
+      </c>
+      <c r="E273" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F273">
+        <v>25</v>
+      </c>
+      <c r="G273" t="str">
+        <v>$25.00–$34.00/hr (Massachusetts-based positions per posting)</v>
+      </c>
+      <c r="H273" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Quality-Engineering--January-June--Onsite-_REQ-2026-18150</v>
+      </c>
+      <c r="I273" t="str">
+        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, req REQ-2026-18150, endDate 2026-12-31, body quote: 'Position Dates: January 11, 2027 – June 30, 2027' and 'Availability for the Co-op duration Spring: January – June 2027.'</v>
+      </c>
+      <c r="J273" t="str">
+        <v>New req at an already-tracked employer — sibling to Insulet's other already-tracked Acton, MA Jan-June 2027 engineering co-ops. Medical device (insulin pump) manufacturer; not eligible for visa sponsorship per company-wide postings.</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>Keurig Dr Pepper</v>
+      </c>
+      <c r="B274" t="str">
+        <v>Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)</v>
+      </c>
+      <c r="C274" t="str">
+        <v>Mechanical/Appliance Engineering (also accepts SW/EE/IE)</v>
+      </c>
+      <c r="D274" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E274" t="str">
+        <v>Burlington, MA</v>
+      </c>
+      <c r="F274">
+        <v>15</v>
+      </c>
+      <c r="G274" t="str">
+        <v>$31/hr + $5,000 sign-on bonus per posting</v>
+      </c>
+      <c r="H274" t="str">
+        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-appliance-engineering-me-sw-ee-ie/42849/100035469424</v>
+      </c>
+      <c r="I274" t="str">
+        <v>Yes — independently fetched directly, HTTP 200, page confirms title 'Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)', '$31/hour', and sign-on bonus language.</v>
+      </c>
+      <c r="J274" t="str">
+        <v>New company for the tracker — Burlington, MA HQ (Boston-area). Company-wide program note: 'The KDP 2027 Winter Co-op Program will run from January 4 – May 21, 2027.' Mechanical Engineering is among the accepted majors.</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>Keurig Dr Pepper</v>
+      </c>
+      <c r="B275" t="str">
+        <v>Winter 2027 Co-op - Mechanical Test and Reliability</v>
+      </c>
+      <c r="C275" t="str">
+        <v>Mechanical Engineering (Test &amp; Reliability)</v>
+      </c>
+      <c r="D275" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E275" t="str">
+        <v>Burlington, MA</v>
+      </c>
+      <c r="F275">
+        <v>15</v>
+      </c>
+      <c r="G275" t="str">
+        <v>$31/hr + sign-on bonus per posting</v>
+      </c>
+      <c r="H275" t="str">
+        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-mechanical-test-and-reliability/42849/99763826160</v>
+      </c>
+      <c r="I275" t="str">
+        <v>Yes — independently fetched directly (note: the job-ID-only URL redirects to the homepage; the correct URL includes a job-family segment, confirmed via Keurig Dr Pepper's own search-results endpoint), HTTP 200, page confirms title 'Winter 2027 Co-op - Mechanical Test and Reliability', '$31/hour', and sign-on bonus language.</v>
+      </c>
+      <c r="J275" t="str">
+        <v>New company for the tracker — sibling req to the Appliance Engineering co-op above, same Burlington MA site and Winter 2027 program. A distinct Fall-2027-only sibling (job 99763826384) exists and is excluded on season grounds.</v>
       </c>
     </row>
   </sheetData>
@@ -10944,14 +11168,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M268"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M275"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C520"/>
+  <dimension ref="A1:C528"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -16669,9 +16893,97 @@
         <v>2026-09-30 (later run): no change in live/open status for any of the four — all remain unverifiable via any method tried this run, consistent with many prior runs. Progress made identifying platforms: Lam Research confirmed on Eightfold 'PCSX' (lamresearch.eightfold.ai / careers.lamresearch.com), still auth-walled; MACOM confirmed on Cornerstone OnDemand (macomtech.csod.com, careersite ID 4), API still returns 'CSOD Unauthorized Exception'; Waters and Parker Hannifin both remain fully WAF/Cloudflare-blocked with no working alternate access (Wayback Machine unavailable in this environment). No postings added.</v>
       </c>
     </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>Trane Technologies</v>
+      </c>
+      <c r="B521" t="str">
+        <v>'Mechanical Engineering Co-op' — 4 live reqs found via direct Workday CXS API (JR-8817 Panama City FL, JR-8542 Clarksville TN, JR-8939 McGregor TX, JR-8960 Minneapolis MN), all posted 16 days ago, all closing 2026-10-31, all independently re-confirmed live by this session</v>
+      </c>
+      <c r="C521" t="str">
+        <v>2026-09-30 ~13:00 UTC: all four use identical generic template language — 'Co-ops will operate full-time from January to August or May to December' — with no explicit year or season word (no 'Spring 2027'/'Winter 2026') anywhere in the posting text. The Oct 31 2026 deadline and Boilerplate Jan-start language make a Spring 2027 cohort plausible, but this fails the strict 'season stated on the posting itself' bar (same treatment as previously-excluded evergreen Draper/Curtiss-Wright reqs). Not added; worth re-checking if Trane ever posts a dated 'Spring 2027' version. Pay stated: $22.50-$31.00/hr; citizenship/no-sponsorship language present.</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>PPL Corporation / LG&amp;E and KU (Louisville, KY)</v>
+      </c>
+      <c r="B522" t="str">
+        <v>'Spring 2027 Mechanical Engineering Co-op — Multiple Positions'</v>
+      </c>
+      <c r="C522" t="str">
+        <v>2026-09-30 ~13:00 UTC: only found via aggregator mirrors (Glassdoor/Indeed/ZipRecruiter); PPL's real ATS (careers.pplweb.com) is a fully client-side-rendered SAP SuccessFactors/Jibe app with no server-embedded job data, so the specific req ID/URL could not be located or opened directly. Glassdoor itself returned HTTP 403 to direct fetch. Real, plausible lead (a Spring 2026 sibling posting was confirmed to exist at careers.pplweb.com/jobs/13501) but not independently verified against its own posting — not added without a verified URL.</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>Precision Castparts Corp. (Berkshire Hathaway)</v>
+      </c>
+      <c r="B523" t="str">
+        <v>'Spring 2027 Engineering Student Co-Op' (Muskegon MI), 'Spring 2027 Maintenance Co-Op' (Spring TX), 'Engineering Co-Op for Spring 2027' (Niskayuna NY)</v>
+      </c>
+      <c r="C523" t="str">
+        <v>2026-09-30 ~13:00 UTC: only found via aggregator mirrors (Dice/Glassdoor/Indeed); PCC's real ATS (a StepStone TalentLink portal at pcctalentacquisitionportal.tal.net) is behind an Altcha bot-check challenge, fully blocking programmatic access — same class of block as other long-standing blockers. Not added without a verified URL.</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="str">
+        <v>Weston &amp; Sampson Engineers (Reading, MA)</v>
+      </c>
+      <c r="B524" t="str">
+        <v>'Water Resources Co-Op (Spring 2027)'</v>
+      </c>
+      <c r="C524" t="str">
+        <v>2026-09-30 ~13:00 UTC: new company, found via aggregator only; real ATS is ADP Workforce Now (JS-rendered), could not pull job content via direct fetch in time available. Not independently verified — worth a dedicated attempt in a future run.</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="str">
+        <v>CDM Smith (Boston, MA)</v>
+      </c>
+      <c r="B525" t="str">
+        <v>'Electrical Engineering Co-op, Spring 2027'</v>
+      </c>
+      <c r="C525" t="str">
+        <v>2026-09-30 ~13:00 UTC: new company found via aggregator; Electrical Engineering discipline is outside Hamza's target list. Not pursued further; not independently verified.</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="str">
+        <v>LineVision, Inc. (Boston, MA)</v>
+      </c>
+      <c r="B526" t="str">
+        <v>Data Engineering Co-op</v>
+      </c>
+      <c r="C526" t="str">
+        <v>2026-09-30 ~13:00 UTC: new company found via aggregator; software/data-engineering discipline is outside Hamza's target list. Not pursued.</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="str">
+        <v>Lutron Electronics</v>
+      </c>
+      <c r="B527" t="str">
+        <v>'Spring 2027 - Mechanical Engineering Co-Op - Boston, MA' aggregator listing (theladders.com)</v>
+      </c>
+      <c r="C527" t="str">
+        <v>2026-09-30 ~13:00 UTC: traced back to a stale Spring-2026 listing. Direct fetch of careers.lutron.com/sitemap.xml (140 live job URLs) found no current Co-Op/Spring-2027-titled Mechanical Engineering posting — only full-time ME roles and a 'Summer 2027 - Manufacturing Engineering Intern - Ashland, VA' listing. Aggregator listing appears stale/incorrect; not added.</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="str">
+        <v>National sweep, 2026-09-30 ~13:00 UTC — new companies checked, no qualifying openings</v>
+      </c>
+      <c r="B528" t="str">
+        <v>Epirus (Torrance CA), Scout Motors (Columbia SC), Rugged Robotics, Muon Space, Pacific Fusion, Valar Atomics, Fervo Energy, Loft Orbital, Generac, Johnson Controls, Carrier Global, KLA Corporation, Chevron, Sensata Technologies (incl. Dynapower)</v>
+      </c>
+      <c r="C528" t="str">
+        <v>Each checked directly against its own ATS/careers site (Greenhouse, Lever, or Workday CXS API). Epirus/Scout Motors/Rugged Robotics/Valar Atomics/Loft Orbital: no intern/co-op postings at all. Muon Space and Pacific Fusion: all internships explicitly Summer 2027, wrong season. Fervo Energy: only internship is oil/gas well-completions discipline, weak fit, no season stated. Generac: all current ME intern postings are Summer 2027 or Summer 2026. Johnson Controls: only near-window posting is 'Power Electronics Intern (Fall 2026)', EE discipline and Fall-only. Carrier Global: careers site (Radancy/TalentBrew) blocks programmatic search, a previously-indexed ME intern listing now redirects to the homepage (expired) — unverifiable. KLA Corporation: only 1 intern-type role company-wide (Software Engineering), no ME opening; 2 previously-indexed ME Intern reqs no longer appear live. Chevron: 'Facilities Engineering Mechanical Engineering Intern' (Houston TX, req R000072394) confirmed live via direct Workday CXS fetch but posting text contains no season keyword at all (no Summer/Spring/Winter/Fall) — excluded for insufficient season evidence. Sensata Technologies: all current ME Intern postings (Dynapower/VT, Aerospace/CA sites) explicitly Summer 2027. None added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C520"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C528"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 6 checked-excluded (2026-09-30 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Zqv75N94TnNGDMD8zo4xr
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M275"/>
+  <dimension ref="A1:M279"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -10692,6 +10692,134 @@
       </c>
       <c r="J275" t="str">
         <v>New company for the tracker — sibling req to the Appliance Engineering co-op above, same Burlington MA site and Winter 2027 program. A distinct Fall-2027-only sibling (job 99763826384) exists and is excluded on season grounds.</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>Apex Technology, Inc. (Apex Space)</v>
+      </c>
+      <c r="B276" t="str">
+        <v>Avionics Test Engineering Internship (Spring 2027)</v>
+      </c>
+      <c r="C276" t="str">
+        <v>Avionics / Flight Systems Test Engineering</v>
+      </c>
+      <c r="D276" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E276" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F276">
+        <v>2600</v>
+      </c>
+      <c r="G276" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H276" t="str">
+        <v>https://jobs.ashbyhq.com/apex-technology-inc/aea24b77-7673-4478-83af-4f16f5337673</v>
+      </c>
+      <c r="I276" t="str">
+        <v>Yes — independently fetched directly via Apex's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/apex-technology-inc), isListed true, title states 'Spring 2027' verbatim, posted 2026-09-09.</v>
+      </c>
+      <c r="J276" t="str">
+        <v>New company for the tracker. Apex manufactures satellite buses at scale (spacecraft platform manufacturer). Role is on the Avionics team's test/integration side — flight-systems-adjacent discipline.</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>Apex Technology, Inc. (Apex Space)</v>
+      </c>
+      <c r="B277" t="str">
+        <v>Thermal Engineering Internship (Spring or Summer 2027)</v>
+      </c>
+      <c r="C277" t="str">
+        <v>Thermal / Mechanical Engineering</v>
+      </c>
+      <c r="D277" t="str">
+        <v>Spring or Summer 2027 (posting offers either term)</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F277">
+        <v>2600</v>
+      </c>
+      <c r="G277" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H277" t="str">
+        <v>https://jobs.ashbyhq.com/apex-technology-inc/56b018ce-915d-4ebd-9833-c8ebb160b09a</v>
+      </c>
+      <c r="I277" t="str">
+        <v>Yes — independently fetched directly via Apex's own Ashby posting-api, isListed true, title states 'Spring or Summer 2027' verbatim, posted 2026-09-04.</v>
+      </c>
+      <c r="J277" t="str">
+        <v>Same company as above. Posting explicitly offers Spring 2027 as one of two term options (not Summer-only) — qualifies per the tracker's season rule. Confirm preferred term (Spring) during application.</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>Layup Parts</v>
+      </c>
+      <c r="B278" t="str">
+        <v>Manufacturing Engineer Intern</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Rolling — explicitly includes Winter and Spring 2027 per posting text</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Huntington Beach, CA</v>
+      </c>
+      <c r="F278">
+        <v>2600</v>
+      </c>
+      <c r="G278" t="str">
+        <v>Not stated on posting (aggregator-cited ~$25/hr, unconfirmed on primary source)</v>
+      </c>
+      <c r="H278" t="str">
+        <v>https://jobs.lever.co/layup/4522257e-bac4-4937-b0b0-88d7ebbb6583</v>
+      </c>
+      <c r="I278" t="str">
+        <v>Yes — independently fetched directly via Lever's own postings API (api.lever.co/v0/postings/layup), job live among current postings, description quote: 'Whether you're looking for a Fall, Winter, Spring, or Summer internship, we're accepting applications on a rolling basis.'</v>
+      </c>
+      <c r="J278" t="str">
+        <v>New company — composites manufacturing technology (CNC machining, 3D printing, advanced manufacturing) serving aerospace/defense/robotics customers. ITAR-restricted: applicant must be a U.S. citizen/national, lawful permanent resident, refugee, or asylee, or independently eligible for State Dept. authorization.</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>NDimensions Labs</v>
+      </c>
+      <c r="B279" t="str">
+        <v>Hardware &amp; Electronics Intern, Robotics</v>
+      </c>
+      <c r="C279" t="str">
+        <v>Robotics Hardware / Mechatronics</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Boston, MA</v>
+      </c>
+      <c r="F279">
+        <v>0</v>
+      </c>
+      <c r="G279" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H279" t="str">
+        <v>https://ndimensions.xyz/careers/hardware_intern</v>
+      </c>
+      <c r="I279" t="str">
+        <v>Yes — fetched directly, page live, title 'Hardware &amp; Electronics Intern, Robotics', subtitle states 'Spring 2027 internship (Full-time) • Boston, MA' verbatim.</v>
+      </c>
+      <c r="J279" t="str">
+        <v>New company — early-stage startup (founders from MIT, U. Waterloo, U. Washington) building robotics/embodied-AI hardware infrastructure. Role covers mechanical/electromechanical component design, PCB/sensor/actuator assembly and testing. Small/early-stage company — flagging maturity as a factor for Hamza to weigh, but the listing itself is directly verified and legitimate.</v>
       </c>
     </row>
   </sheetData>
@@ -11168,14 +11296,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M275"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M279"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C528"/>
+  <dimension ref="A1:C534"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -16931,10 +17059,10 @@
         <v>Weston &amp; Sampson Engineers (Reading, MA)</v>
       </c>
       <c r="B524" t="str">
-        <v>'Water Resources Co-Op (Spring 2027)'</v>
+        <v>'Co-Op Civil/Environmental Engineer (Spring 2027)', itemID 9201572098947_1</v>
       </c>
       <c r="C524" t="str">
-        <v>2026-09-30 ~13:00 UTC: new company, found via aggregator only; real ATS is ADP Workforce Now (JS-rendered), could not pull job content via direct fetch in time available. Not independently verified — worth a dedicated attempt in a future run.</v>
+        <v>2026-09-30 ~19:00 UTC: now independently verified via direct fetch of the company's own ADP Workforce Now REST API (workforcenow.adp.com career-center job-requisitions endpoint) — posting is live, posted 2026-09-03, Reading MA, $22-26/hr. However the role is Civil/Environmental Engineering (water/wastewater/stormwater/climate-resiliency) — outside Hamza's target disciplines (mechanical, aerospace/systems, manufacturing, robotics, flight systems, industrial, materials, structural, controls). Excluded on discipline grounds, not verification grounds.</v>
       </c>
     </row>
     <row r="525">
@@ -16942,10 +17070,10 @@
         <v>CDM Smith (Boston, MA)</v>
       </c>
       <c r="B525" t="str">
-        <v>'Electrical Engineering Co-op, Spring 2027'</v>
+        <v>'Electrical Engineering Co-op, Spring 2027' and 'Environmental Engineering Co-Op, Spring 2027'; also checked for a 'Structural Engineering Intern' (found but Summer 2027 + Intern not Co-op, doubly excluded)</v>
       </c>
       <c r="C525" t="str">
-        <v>2026-09-30 ~13:00 UTC: new company found via aggregator; Electrical Engineering discipline is outside Hamza's target list. Not pursued further; not independently verified.</v>
+        <v>2026-09-30 ~19:00 UTC re-check: Electrical and Environmental Co-Ops are discipline mismatches (outside Hamza's target list); the Structural Engineering role is Summer 2027, wrong season. careers.cdmsmith.com is a JS-rendered iCIMS/Jibe site with no public API found — these three findings rest on secondary-source snippets, not a primary-source fetch. Not pursued.</v>
       </c>
     </row>
     <row r="526">
@@ -16981,9 +17109,75 @@
         <v>Each checked directly against its own ATS/careers site (Greenhouse, Lever, or Workday CXS API). Epirus/Scout Motors/Rugged Robotics/Valar Atomics/Loft Orbital: no intern/co-op postings at all. Muon Space and Pacific Fusion: all internships explicitly Summer 2027, wrong season. Fervo Energy: only internship is oil/gas well-completions discipline, weak fit, no season stated. Generac: all current ME intern postings are Summer 2027 or Summer 2026. Johnson Controls: only near-window posting is 'Power Electronics Intern (Fall 2026)', EE discipline and Fall-only. Carrier Global: careers site (Radancy/TalentBrew) blocks programmatic search, a previously-indexed ME intern listing now redirects to the homepage (expired) — unverifiable. KLA Corporation: only 1 intern-type role company-wide (Software Engineering), no ME opening; 2 previously-indexed ME Intern reqs no longer appear live. Chevron: 'Facilities Engineering Mechanical Engineering Intern' (Houston TX, req R000072394) confirmed live via direct Workday CXS fetch but posting text contains no season keyword at all (no Summer/Spring/Winter/Fall) — excluded for insufficient season evidence. Sensata Technologies: all current ME Intern postings (Dynapower/VT, Aerospace/CA sites) explicitly Summer 2027. None added.</v>
       </c>
     </row>
+    <row r="529">
+      <c r="A529" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B529" t="str">
+        <v>R5029663 re-check, plus Lynn MA trade Trainee Co-Ops (R5034331 CNC, R5034333 Carpentry, R5034069 Welder) and CNC Programmer Co-op — Fall 2026 (R5030459)</v>
+      </c>
+      <c r="C529" t="str">
+        <v>2026-09-30 ~19:00 UTC: R5029663 (already in `rows`) — the marketing portal careers.geaerospace.com returns 'no longer posted' for two URL formats tried, but the actual tracked Application Link (the direct Workday job-page URL) is independently confirmed still live via GE's own Workday CXS API — canApply true, endDate 2026-11-06, 23 eligible locations incl. Lynn MA. No change to `rows`; flagging the marketing-portal/Workday discrepancy for awareness (use the Workday link, not the careers.geaerospace.com search UI, to check status). The four Lynn-specific trade Trainee Co-Ops are now expired/410 and were vocational (not 4-year-engineering) roles regardless; CNC Programmer Co-op Fall 2026 is HTTP 410 Gone. None added.</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B530" t="str">
+        <v>Full company-wide re-sweep via Draper's own Workday CXS API</v>
+      </c>
+      <c r="C530" t="str">
+        <v>2026-09-30 ~19:00 UTC: all currently-live Cambridge MA Spring 2027 co-ops (JR002940 Mechanical Eng &amp; System Packaging, JR002942 Materials and Chemistry, JR002882 Systems Engineering, JR002883 Electro-Mechanical Instrument, JR002941 Electrical Engineering, JR002944 Digital Engineering-Requirements Engineering, JR002974 Co-Op Student Engineering) were cross-checked against `build.mjs` byte-for-byte and confirmed already tracked (JR002940, JR002942) or already excluded (JR002941 EE discipline mismatch; others discipline-mismatch or already logged). No new qualifying req found — continued saturation.</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="str">
+        <v>Trane Technologies</v>
+      </c>
+      <c r="B531" t="str">
+        <v>Re-check of the 4 standing Mechanical Engineering Co-op reqs — 2 freshly reposted with new req numbers (JR-8542 Clarksville TN posted today, JR-8960 Minneapolis MN posted yesterday) alongside JR-8817 Panama City FL and JR-8939 McGregor TX</v>
+      </c>
+      <c r="C531" t="str">
+        <v>2026-09-30 ~19:00 UTC re-check: all four still use the identical generic 'January to August or May to December' language with no explicit season/year word anywhere in any of the four descriptions — no change from the prior exclusion. Still not added; still worth a periodic re-check for a dated version.</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="str">
+        <v>Apex Technology, Inc. (Apex Space)</v>
+      </c>
+      <c r="B532" t="str">
+        <v>Full internship slate via Apex's own Ashby posting-api (Los Angeles, CA): Mechanical Engineering Internship (Fall 2026), Propulsion Internship (Summer 2027), Simulation Software Engineering Internship (Spring or Summer 2027), Avionics Internship - Power Electronics (Spring or Summer 2027), Sensors Team Internship (Spring or Summer 2027)</v>
+      </c>
+      <c r="C532" t="str">
+        <v>2026-09-30 ~19:00 UTC: new company. Mechanical Engineering Internship is Fall-2026-only (wrong season, no stated extension). Propulsion Internship is Summer-2027-only (wrong season). Simulation Software Engineering is a software discipline (mismatch). Avionics-Power Electronics and Sensors Team internships are electrical/sensors-focused (EE discipline, mismatch vs. Hamza's target list) despite offering a qualifying Spring 2027 term. Two other Apex internships (Avionics Test Engineering, Thermal Engineering) DID qualify and were added to `rows` — see above.</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="str">
+        <v>Foundation Robotics</v>
+      </c>
+      <c r="B533" t="str">
+        <v>Mechanical Engineer Intern (humanoid robot hand mechanism design), San Francisco CA — ats.rippling.com/foundation-robotics</v>
+      </c>
+      <c r="C533" t="str">
+        <v>2026-09-30 ~19:00 UTC: new company. Confirmed directly via the company's own Rippling ATS page that the job is live with an active 'Apply now' button — but the primary-source posting text itself states no season/term at all. A 'Spring 2027' claim for this exact title only appears on a now-defunct BuiltIn SF cache of an apparently older, removed listing. Fails the 'season confirmed from the posting itself' bar — not added.</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="str">
+        <v>National sweep, 2026-09-30 ~19:00 UTC — new companies checked, no qualifying openings</v>
+      </c>
+      <c r="B534" t="str">
+        <v>Carbon Inc., Scout Space, KYOCERA SENCO Industrial Tools, The Aerospace Corporation, StandardAero (Dallas TX), Second Order Effects, Royal Switchgear Manufacturing, SEACORP, Avion Solutions, Magna International, Saronic Technologies, SmartFlower Solar, Anthro (Anthro Energy), Amperesand, Moeller Aerospace, Skyways, Nor-Cal Controls ES, AS&amp;T Inc., Dennis Group, General Matter, Lykos Energy, CX2, BMW Group</v>
+      </c>
+      <c r="C534" t="str">
+        <v>Each checked directly against its own ATS where one could be found. Carbon Inc.: Greenhouse job 404, closed. Scout Space: Techstars board explicitly 'no longer accepting applications'. KYOCERA SENCO: only lead now HTTP 410 Gone. Aerospace Corporation: careers site 403-blocked, program structured as summer/Feb-deadline cycle, not clearly Winter/Spring. StandardAero: only lead is Summer-2026-primary with a past Dec 2025 deadline; the season-matching role found was in Winnipeg, Canada (out of scope). Second Order Effects: company's own Greenhouse board returns 0 jobs, specific listing 404s — stale aggregator-only lead. Royal Switchgear: only located req explicitly marked closed on their isolved ATS. SEACORP: only bare-year (no season word) postings found; careers portal 403-blocked. Avion Solutions: specific listing confirmed true 404. Magna International: 2 live Workday-confirmed ADAS intern/co-op reqs (Auburn Hills MI) but neither states a season — generic rolling language only. Saronic Technologies: all current ME/Manufacturing/Industrial/EE intern reqs on their own Ashby API are explicitly Summer 2027. SmartFlower Solar: self-contradictory season text ('Spring '27' title vs. 'Winter-Spring 2026 (Jan-June)' body, already elapsed) — unconfirmable/stale. Anthro Energy: Manufacturing Engineering Intern is explicitly Fall 2026 only (Sept-Dec), no extension. Amperesand: Greenhouse job 404. Moeller Aerospace: no dated req found, only an email-based interest process. Skyways: resume-collection page for a not-yet-launched program, not a live dated req. Nor-Cal Controls ES: no season language at all, appears to be an ongoing training program. AS&amp;T Inc.: explicitly '2026 summer internship period', wrong season. Dennis Group: 'starting January 2026' — already elapsed as of this run. General Matter: Manufacturing Engineering internship is explicitly Summer 2027. Lykos Energy: no ME intern posting located, only Field Engineer/BESS field roles. CX2: 'Spring/Summer 2026' — already elapsed. BMW Group: season-matching req ('Intern, Intelligent Car - Fall 2026/Winter 2027') 404s on bmwgroup.jobs; the live Spring-2027-titled req found via aggregator only is ML/embodied-AI research, not core ME/hardware, and discipline + primary-source verification both failed. None added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C528"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C534"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 13 checked-excluded (2026-10-01 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BWVYABZp9NDeNMSzSpLibn
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M279"/>
+  <dimension ref="A1:M283"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -10820,6 +10820,134 @@
       </c>
       <c r="J279" t="str">
         <v>New company — early-stage startup (founders from MIT, U. Waterloo, U. Washington) building robotics/embodied-AI hardware infrastructure. Role covers mechanical/electromechanical component design, PCB/sensor/actuator assembly and testing. Small/early-stage company — flagging maturity as a factor for Hamza to weigh, but the listing itself is directly verified and legitimate.</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>MORSE Corp</v>
+      </c>
+      <c r="B280" t="str">
+        <v>Mechanical Engineer Co-op</v>
+      </c>
+      <c r="C280" t="str">
+        <v>Mechanical Engineering / Flight Systems (UAV)</v>
+      </c>
+      <c r="D280" t="str">
+        <v>Spring 2027 (Jan–Jun/Aug 2027 per co-op board description)</v>
+      </c>
+      <c r="E280" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F280">
+        <v>0</v>
+      </c>
+      <c r="G280" t="str">
+        <v>$27–$33/hr</v>
+      </c>
+      <c r="H280" t="str">
+        <v>https://job-boards.greenhouse.io/morsecorpcoop/jobs/7968311003</v>
+      </c>
+      <c r="I280" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own public API (api.greenhouse.io/v1/boards/morsecorpcoop/jobs/7968311003) and the board landing page, which states verbatim 'Welcome to MORSE Corp's Co-op Opportunities for the Spring 2027 Semester!' Job listed live, requisition 342.</v>
+      </c>
+      <c r="J280" t="str">
+        <v>New company — employee-owned small defense-tech firm (Cambridge MA / Arlington VA / Seattle WA) building UAVs, autonomous vehicles, and mission systems for the US national security ecosystem. Role: designing, building, and flight-testing UAV prototypes, mechatronics/robotics, rapid prototyping (3D printing/CNC/laser cutting), SolidWorks/Altium. On-site 5 days/week. Requires US citizenship and ability to obtain a US security clearance.</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>Marotta Controls, Inc.</v>
+      </c>
+      <c r="B281" t="str">
+        <v>Spring 2027 Mechanical Engineering Internship/Co-Op</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Mechanical / Aerospace / Materials Engineering</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Spring 2027 (with option to continue into Summer 2027)</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Parsippany, NJ</v>
+      </c>
+      <c r="F281">
+        <v>210</v>
+      </c>
+      <c r="G281" t="str">
+        <v>Not stated on current posting</v>
+      </c>
+      <c r="H281" t="str">
+        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a061fa5de22f3c</v>
+      </c>
+      <c r="I281" t="str">
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, Apply button present, title and body state 'Spring 2027 Mechanical Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim.</v>
+      </c>
+      <c r="J281" t="str">
+        <v>New company — defense/aerospace motion &amp; flow control systems manufacturer. Design/production/quality/test-development work, 3D CAD (Pro-E/Creo). US citizenship required (ITAR). TIME-SENSITIVE: posting states 'Deadline: October 1, 2026' (the day this was verified) with an invitation-only interview day October 16, 2026 — confirm it hasn't already closed before staging/applying.</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>Marotta Controls, Inc.</v>
+      </c>
+      <c r="B282" t="str">
+        <v>Spring 2027 Control Systems Engineering Internship/Co-Op</v>
+      </c>
+      <c r="C282" t="str">
+        <v>Controls Engineering</v>
+      </c>
+      <c r="D282" t="str">
+        <v>Spring 2027 (with option to continue into Summer 2027)</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Parsippany, NJ</v>
+      </c>
+      <c r="F282">
+        <v>210</v>
+      </c>
+      <c r="G282" t="str">
+        <v>Not stated on current posting</v>
+      </c>
+      <c r="H282" t="str">
+        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a062229f2536d0</v>
+      </c>
+      <c r="I282" t="str">
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, title and body state 'Spring 2027 Control Systems Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim.</v>
+      </c>
+      <c r="J282" t="str">
+        <v>Same company as above. MATLAB control-system simulation/modeling, requirements management in IBM DOORS, systems engineering deliverables. US citizenship required (ITAR). TIME-SENSITIVE: same October 1, 2026 deadline as the Mechanical Engineering sibling above — confirm it hasn't already closed before staging/applying.</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>1X Technologies</v>
+      </c>
+      <c r="B283" t="str">
+        <v>Internship - Manufacturing Engineering</v>
+      </c>
+      <c r="C283" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Starting January 2027 (posting's own wording — does not use the literal word 'Spring' or 'Winter', but the explicit January 2027 start date places it inside Hamza's target window)</v>
+      </c>
+      <c r="E283" t="str">
+        <v>San Carlos, CA</v>
+      </c>
+      <c r="F283">
+        <v>2700</v>
+      </c>
+      <c r="G283" t="str">
+        <v>$35/hr + $2,500/month housing stipend for relocation</v>
+      </c>
+      <c r="H283" t="str">
+        <v>https://jobs.ashbyhq.com/1x/d687b375-8136-4e6f-baa6-369b89366050</v>
+      </c>
+      <c r="I283" t="str">
+        <v>Yes — independently fetched directly via Ashby's own posting-api (api.ashbyhq.com/posting-api/job-board/1x), isListed true, title 'Internship - Manufacturing Engineering', body states 'INTERNSHIP SEASON - STARTING JANUARY 2027' verbatim, published 2026-09-14.</v>
+      </c>
+      <c r="J283" t="str">
+        <v>New company — humanoid robotics manufacturer (maker of the 'NEO' home robot). Role: manufacturing process/fixture design, CAD (SolidWorks/Onshape), design-for-manufacturability for robot hardware. A sibling 'Internship - CNC Machine Park' (Hayward, CA) role exists but states no season/year and was excluded.</v>
       </c>
     </row>
   </sheetData>
@@ -11296,14 +11424,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M279"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M283"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C534"/>
+  <dimension ref="A1:C547"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -17175,9 +17303,152 @@
         <v>Each checked directly against its own ATS where one could be found. Carbon Inc.: Greenhouse job 404, closed. Scout Space: Techstars board explicitly 'no longer accepting applications'. KYOCERA SENCO: only lead now HTTP 410 Gone. Aerospace Corporation: careers site 403-blocked, program structured as summer/Feb-deadline cycle, not clearly Winter/Spring. StandardAero: only lead is Summer-2026-primary with a past Dec 2025 deadline; the season-matching role found was in Winnipeg, Canada (out of scope). Second Order Effects: company's own Greenhouse board returns 0 jobs, specific listing 404s — stale aggregator-only lead. Royal Switchgear: only located req explicitly marked closed on their isolved ATS. SEACORP: only bare-year (no season word) postings found; careers portal 403-blocked. Avion Solutions: specific listing confirmed true 404. Magna International: 2 live Workday-confirmed ADAS intern/co-op reqs (Auburn Hills MI) but neither states a season — generic rolling language only. Saronic Technologies: all current ME/Manufacturing/Industrial/EE intern reqs on their own Ashby API are explicitly Summer 2027. SmartFlower Solar: self-contradictory season text ('Spring '27' title vs. 'Winter-Spring 2026 (Jan-June)' body, already elapsed) — unconfirmable/stale. Anthro Energy: Manufacturing Engineering Intern is explicitly Fall 2026 only (Sept-Dec), no extension. Amperesand: Greenhouse job 404. Moeller Aerospace: no dated req found, only an email-based interest process. Skyways: resume-collection page for a not-yet-launched program, not a live dated req. Nor-Cal Controls ES: no season language at all, appears to be an ongoing training program. AS&amp;T Inc.: explicitly '2026 summer internship period', wrong season. Dennis Group: 'starting January 2026' — already elapsed as of this run. General Matter: Manufacturing Engineering internship is explicitly Summer 2027. Lykos Energy: no ME intern posting located, only Field Engineer/BESS field roles. CX2: 'Spring/Summer 2026' — already elapsed. BMW Group: season-matching req ('Intern, Intelligent Car - Fall 2026/Winter 2027') 404s on bmwgroup.jobs; the live Spring-2027-titled req found via aggregator only is ML/embodied-AI research, not core ME/hardware, and discipline + primary-source verification both failed. None added.</v>
       </c>
     </row>
+    <row r="535">
+      <c r="A535" t="str">
+        <v>Marotta Controls, Inc.</v>
+      </c>
+      <c r="B535" t="str">
+        <v>Spring 2027 Electrical Engineering Internship/Co-Op; Spring 2027 Business Operations Engineering Internship/Co-Op (siblings of the 2 qualifying reqs added to `rows` this run)</v>
+      </c>
+      <c r="C535" t="str">
+        <v>2026-10-01: both confirmed live via the company's own Paycor ATS, same Oct 1, 2026 deadline as the qualifying siblings, but EE is a discipline mismatch and Business Operations Engineering is non-engineering/ops-focused. Not added.</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="str">
+        <v>1X Technologies</v>
+      </c>
+      <c r="B536" t="str">
+        <v>Internship - CNC Machine Park (Hayward, CA)</v>
+      </c>
+      <c r="C536" t="str">
+        <v>2026-10-01: new company (sibling to the qualifying Manufacturing Engineering internship added to `rows`). Confirmed live via Ashby's own posting-api, but the posting text states no season or year anywhere — fails the explicit-season bar. Not added.</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="str">
+        <v>Skydio</v>
+      </c>
+      <c r="B537" t="str">
+        <v>Hardware Test &amp; Reliability Intern - Fall 2026/Winter 2027 (San Mateo, CA)</v>
+      </c>
+      <c r="C537" t="str">
+        <v>2026-10-01: new company. Confirmed live via Ashby's own posting-api (full descriptionPlain read in full) — strong discipline fit (electro-mechanical hardware reliability/validation on autonomous flying machines) and attractive pay ($47-58/hr), but the posting's own season label is 'Fall 2026/Winter 2027', not 'Winter 2026' or 'Spring 2027' as Hamza's target window specifies, and the posting gives no explicit month range to confirm whether Skydio's 'Winter 2027' cohort actually falls inside that window (unlike the previously-accepted Keurig Dr Pepper 'Winter 2027' co-op, which stated explicit dates of Jan 4-May 21, 2027). Excluded pending clearer date confirmation — worth re-checking if Skydio ever states explicit months, or if Hamza confirms 'Winter 2027'-labeled cohorts should be treated as in-window on their own.</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="str">
+        <v>Skydio</v>
+      </c>
+      <c r="B538" t="str">
+        <v>Electrical Engineer Intern - Winter 2027; Hardware Product Management Intern - Fall 2026/Winter 2027; Autonomy Engineer Intern x2 (Computer Vision/Deep Learning) - Summer 2027; Flight Test Intern - Summer 2027; Product Design Engineer Intern - Summer 2027; Camera &amp; Imaging Intern (Tampere, Finland)</v>
+      </c>
+      <c r="C538" t="str">
+        <v>2026-10-01: all checked via the same Ashby board. EE and Hardware Product Management are discipline mismatches; the four Summer-2027-titled roles are wrong season; Camera &amp; Imaging Intern is both non-US (Finland) and states no season. None added.</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="str">
+        <v>Apex Technology, Inc. (Apex Space)</v>
+      </c>
+      <c r="B539" t="str">
+        <v>Avionics Internship (Spring or Summer 2027) — previously-unlisted sibling surfaced on a full board re-sweep</v>
+      </c>
+      <c r="C539" t="str">
+        <v>2026-10-01: requires BS/MS in Electrical Engineering, Computer Engineering, or Physics (PCB/circuit design focus) — EE/CompE discipline mismatch, same treatment as the company's other avionics internships. Not added.</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="str">
+        <v>Trane Technologies</v>
+      </c>
+      <c r="B540" t="str">
+        <v>2 newly-found sibling reqs on the same co-ops landing page: JR-14080 (Tyler TX, 'Engineering Co-Op') and JR-8912 (La Crosse WI, 'Automation Engineering Co-op')</v>
+      </c>
+      <c r="C540" t="str">
+        <v>2026-10-01 re-check: same generic no-season template language as the 4 standing excluded reqs (JR-8817/JR-8542/JR-8939/JR-8960, re-confirmed still live and still season-less this run too). Not added; still worth a periodic re-check for a dated version company-wide.</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B541" t="str">
+        <v>3 new-to-this-run postings found on a full Workday CXS sweep: JR002973 'Integrated Circuits Intern', JR002963 'Cable And Harnessing Intern (Summer 2027)', JR002773 'GN&amp;C Modeling, Simulation and Analysis Intern (Summer 2027)'</v>
+      </c>
+      <c r="C541" t="str">
+        <v>2026-10-01: JR002973 is an ASIC/EE discipline role with no season stated in the body; JR002963 and JR002773 are both explicitly Summer 2027 (wrong season — JR002773 otherwise would have fit the controls/aerospace discipline well). All 5 previously-tracked qualifying Draper reqs re-confirmed still live this run. None added.</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B542" t="str">
+        <v>Lynn CNC Programmer Co-Op (R5040944-1); national Spring-2027-titled co-op search (14 results) covering R5040450, R5039320, R5029741, R5029619, R5029667, R5030146, R5029665, R5030096, R5030099</v>
+      </c>
+      <c r="C542" t="str">
+        <v>2026-10-01: Lynn CNC Programmer Co-Op requires current enrollment in a Vocational Technical High School — a high-school trade co-op, not a college engineering role, excluded same as prior Lynn trade postings. The national search results beyond the 3 already-tracked reqs (R5029617, R5029663, R5030103) are Data Science, Communications, Digital Technology, Engines Eng (Computer/Software track), EHS/Facilities/Maintenance, Finance, Supply Chain Operations, and Systems Eng (Electrical/Computer Engineering track) — all discipline mismatches. None added.</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="str">
+        <v>Sonos (Boston, MA)</v>
+      </c>
+      <c r="B543" t="str">
+        <v>Mechanical Engineering Co-Op (req R2547) — moved from being a candidate, never previously added</v>
+      </c>
+      <c r="C543" t="str">
+        <v>2026-10-01: direct fetch of the Workday job page shows the page's own embedded config flag 'postingAvailable: false' — confirmed closed. The tenant's CXS JSON API itself returns 403 to anonymous access, so the page-config flag was used as the closed-signal. Not added.</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="str">
+        <v>Ubicept (Boston, MA)</v>
+      </c>
+      <c r="B544" t="str">
+        <v>Spring Co-op / Internship (includes a Mechanical Engineering track — rapid prototyping of enclosures/mechanical interfaces)</v>
+      </c>
+      <c r="C544" t="str">
+        <v>2026-10-01: new company (SPAD/single-photon imaging startup). Posting says only 'Spring' with no year stated anywhere ('Duration and start-date are flexible') — fails the explicit-year bar. Not added; worth re-checking if a dated version appears.</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="str">
+        <v>Humatics Corporation; Veo Robotics (Waltham, MA)</v>
+      </c>
+      <c r="B545" t="str">
+        <v>General sweep for any internship/co-op openings</v>
+      </c>
+      <c r="C545" t="str">
+        <v>2026-10-01: no internship/co-op-titled postings found at either via search; direct career-page URL guesses both 404'd/redirected, so zero openings could not be independently confirmed via a primary source. Low-confidence exclusion — worth a dedicated look in a future run if time allows.</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="str">
+        <v>Soft Robotics Inc. / Oxipital AI (Bedford, MA)</v>
+      </c>
+      <c r="B546" t="str">
+        <v>General sweep for any internship/co-op openings</v>
+      </c>
+      <c r="C546" t="str">
+        <v>2026-10-01: company appears to have rebranded/restructured (divested its soft-gripping business); oxipital.ai/careers returned 404 and no current listings found elsewhere. Inconclusive — not pursued further.</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="str">
+        <v>National sweep, 2026-10-01 — new companies checked, no qualifying openings</v>
+      </c>
+      <c r="B547" t="str">
+        <v>TerraPower, QuantumScape, Zebra Technologies, Sargent Aerospace &amp; Defense, Howmet Aerospace, DNV (Det Norske Veritas, Maritime Americas), Formic, Albedo Space, Inversion Space, Censys, Solid Power, Sila Nanotechnologies, Velo3D, Bright Machines, Dexterity, Physical Intelligence, Cobot, Standard Bots, Group14 Technologies, Portal Space Systems, Electra.aero, Elroy Air</v>
+      </c>
+      <c r="C547" t="str">
+        <v>Each checked directly against its own ATS where one could be found. TerraPower: real Greenhouse board (slug 'terrapowerllc', 96 open jobs) has zero intern/co-op titles currently — aggregator-cited intern reqs no longer live. QuantumScape: could not locate a working ATS (Greenhouse slug guesses 404). Zebra Technologies: only Summer 2026 program references found; no Winter/Spring-dated posting located. Sargent Aerospace &amp; Defense: own internships page explicitly states a Summer-only program by design. Howmet Aerospace: could not locate a working Workday tenant; aggregator consensus describes a summer-only program. DNV: the specific Fleet in Service Surveyor Winter Internship req now 404s, and the role (ship-classification surveying) is a marginal discipline fit regardless. Formic: both current openings titled plain '2026 Internship' with no season/year language beyond the title — fails the explicit-season bar. Albedo Space, Portal Space Systems: all current openings senior/full-time, no intern/co-op titles. Inversion Space: 81 jobs on the board but 0 current postings returned for any search — possible stale cache, worth a re-check. Censys: no engineering-discipline-fit roles. Solid Power, Sila Nanotechnologies, Group14 Technologies: battery-materials companies, no intern/co-op titles among their current postings. Velo3D, Bright Machines, Dexterity, Cobot, Standard Bots: no intern/co-op titles among dozens of current postings each. Physical Intelligence: only a stale 2024 'Research Internships' posting and a current 'Mechatronics Intern' with no season stated. Electra.aero: has a 'Supply Chain Co-op' but no engineering-discipline intern. Elroy Air: 8 postings on their Lever board, none intern-titled. None added. Note: no working ATS board was found this run for a long list of other space/drone/robotics/materials/EV companies tried by slug-guessing (True Anomaly, Castelion, Xona Space Systems, Turion Space, Orbit Fab, Starfish Space, Gravitics, Benchmark Space Systems, Interlune, Atomos Space, SpinLaunch, ABL Space Systems, Phantom Space, Vaya Space, BRINC Drones, Red Cat Holdings/Teal Drones, Neros Technologies, Firestorm Labs, Vantage Robotics, Volansi, Freefly Systems, 3D Systems, Fathom Digital Manufacturing, Essentium, Sakuu, 6K Inc, Boston Materials, Type One Energy, Zap Energy, Helion Energy, General Fusion, Last Energy, Lear Corporation, Aptiv, Autoliv, ZF Group, Harley-Davidson, Thor Industries, Our Next Energy, Ascend Elements, Natron Energy, Li-Cycle, Mitra Chem, Veeco Instruments, Onto Innovation, Ultra Clean Holdings, Advanced Energy Industries, Brooks Automation/Azenta, FormFactor, Cohu Inc, FANUC America, KUKA Robotics, Omron Automation, Yaskawa America, Chef Robotics, Covariant, Sanctuary AI, Skild AI) — flagged as 'not reached' rather than checked-negative; worth trying their actual company domains directly in a future run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C534"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C547"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 3 checked-excluded (2026-10-01 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USYzyWcPr3HUT94RriRdm4
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M283"/>
+  <dimension ref="A1:M287"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -10948,6 +10948,134 @@
       </c>
       <c r="J283" t="str">
         <v>New company — humanoid robotics manufacturer (maker of the 'NEO' home robot). Role: manufacturing process/fixture design, CAD (SolidWorks/Onshape), design-for-manufacturability for robot hardware. A sibling 'Internship - CNC Machine Park' (Hayward, CA) role exists but states no season/year and was excluded.</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>Lexington Medical, Inc.</v>
+      </c>
+      <c r="B284" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C284" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D284" t="str">
+        <v>January 2027 – June 2027 (Spring 2027)</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Bedford, MA</v>
+      </c>
+      <c r="F284">
+        <v>17</v>
+      </c>
+      <c r="G284" t="str">
+        <v>$28.00–$34.00/hr (pay-transparency widget shows $28–$36)</v>
+      </c>
+      <c r="H284" t="str">
+        <v>https://job-boards.greenhouse.io/lexingtonmedical/jobs/5423105008</v>
+      </c>
+      <c r="I284" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own board API (boards-api.greenhouse.io/v1/boards/lexingtonmedical/jobs/5423105008), job live, updated_at 2026-09-30, body states 'The co-op runs full-time, five days per week, from January 2027 through June 2027.' verbatim.</v>
+      </c>
+      <c r="J284" t="str">
+        <v>New company — medical device manufacturer (AEON surgical stapler), Boston-area (Bedford, MA). R&amp;D team: design/test/document parts, CAD + machine shop + testing work. Sibling 'Manufacturing Engineering Intern', 'Mechanical Engineering Intern', and 'Quality Systems Engineering Intern' at the same site are all explicitly Summer 2027 — excluded on season grounds.</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+      </c>
+      <c r="B285" t="str">
+        <v>iProd Design Center Engineering Co-op (Spring/Summer 2027)</v>
+      </c>
+      <c r="C285" t="str">
+        <v>Mechanical Engineering / Mechanical Engineering Technology</v>
+      </c>
+      <c r="D285" t="str">
+        <v>January – August 2027 (co-op begins in Spring 2027)</v>
+      </c>
+      <c r="E285" t="str">
+        <v>Seneca Falls, NY</v>
+      </c>
+      <c r="F285">
+        <v>290</v>
+      </c>
+      <c r="G285" t="str">
+        <v>$25–$30/hr</v>
+      </c>
+      <c r="H285" t="str">
+        <v>https://careersenus-itt-inc.icims.com/jobs/17446/iprod-design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
+      </c>
+      <c r="I285" t="str">
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'iProd Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: Summer/Fall 2026 rotation, full-time, 40 hours per week. Must be available January to August 2027.' verbatim.</v>
+      </c>
+      <c r="J285" t="str">
+        <v>New company. A duplicate req (17447, same title/location/team, separate req ID — likely a second headcount slot) exists but is not listed as a separate row.</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+      </c>
+      <c r="B286" t="str">
+        <v>Application Engineering Co-op (Spring/Summer 2027)</v>
+      </c>
+      <c r="C286" t="str">
+        <v>Mechanical or Industrial Engineering</v>
+      </c>
+      <c r="D286" t="str">
+        <v>January – August 2027 (co-op begins in Spring 2027)</v>
+      </c>
+      <c r="E286" t="str">
+        <v>Stafford, TX</v>
+      </c>
+      <c r="F286">
+        <v>1600</v>
+      </c>
+      <c r="G286" t="str">
+        <v>$25–$30/hr</v>
+      </c>
+      <c r="H286" t="str">
+        <v>https://careersenus-itt-inc.icims.com/jobs/17660/application-engineering-co-op-%28spring-summer-2027%29/job</v>
+      </c>
+      <c r="I286" t="str">
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Application Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January – August 2027 (full-time, 40 hours per week)' verbatim.</v>
+      </c>
+      <c r="J286" t="str">
+        <v>New company. Open to junior/senior undergraduates in mechanical or industrial engineering.</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+      </c>
+      <c r="B287" t="str">
+        <v>ES Horizontal Design Center Engineering Co-op (Spring/Summer 2027)</v>
+      </c>
+      <c r="C287" t="str">
+        <v>Mechanical Engineering / Mechanical Engineering Technology</v>
+      </c>
+      <c r="D287" t="str">
+        <v>January – August 2027 (co-op begins in Spring 2027)</v>
+      </c>
+      <c r="E287" t="str">
+        <v>Seneca Falls, NY</v>
+      </c>
+      <c r="F287">
+        <v>290</v>
+      </c>
+      <c r="G287" t="str">
+        <v>$25–$30/hr</v>
+      </c>
+      <c r="H287" t="str">
+        <v>https://careersenus-itt-inc.icims.com/jobs/17708/design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
+      </c>
+      <c r="I287" t="str">
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January to August 2027 (full-time, 40 hours per week)' verbatim.</v>
+      </c>
+      <c r="J287" t="str">
+        <v>New company. Distinct req from the iProd Design Center Co-op above (different team/business line, same site).</v>
       </c>
     </row>
   </sheetData>
@@ -11424,14 +11552,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M283"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M287"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C547"/>
+  <dimension ref="A1:C550"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -17446,9 +17574,42 @@
         <v>Each checked directly against its own ATS where one could be found. TerraPower: real Greenhouse board (slug 'terrapowerllc', 96 open jobs) has zero intern/co-op titles currently — aggregator-cited intern reqs no longer live. QuantumScape: could not locate a working ATS (Greenhouse slug guesses 404). Zebra Technologies: only Summer 2026 program references found; no Winter/Spring-dated posting located. Sargent Aerospace &amp; Defense: own internships page explicitly states a Summer-only program by design. Howmet Aerospace: could not locate a working Workday tenant; aggregator consensus describes a summer-only program. DNV: the specific Fleet in Service Surveyor Winter Internship req now 404s, and the role (ship-classification surveying) is a marginal discipline fit regardless. Formic: both current openings titled plain '2026 Internship' with no season/year language beyond the title — fails the explicit-season bar. Albedo Space, Portal Space Systems: all current openings senior/full-time, no intern/co-op titles. Inversion Space: 81 jobs on the board but 0 current postings returned for any search — possible stale cache, worth a re-check. Censys: no engineering-discipline-fit roles. Solid Power, Sila Nanotechnologies, Group14 Technologies: battery-materials companies, no intern/co-op titles among their current postings. Velo3D, Bright Machines, Dexterity, Cobot, Standard Bots: no intern/co-op titles among dozens of current postings each. Physical Intelligence: only a stale 2024 'Research Internships' posting and a current 'Mechatronics Intern' with no season stated. Electra.aero: has a 'Supply Chain Co-op' but no engineering-discipline intern. Elroy Air: 8 postings on their Lever board, none intern-titled. None added. Note: no working ATS board was found this run for a long list of other space/drone/robotics/materials/EV companies tried by slug-guessing (True Anomaly, Castelion, Xona Space Systems, Turion Space, Orbit Fab, Starfish Space, Gravitics, Benchmark Space Systems, Interlune, Atomos Space, SpinLaunch, ABL Space Systems, Phantom Space, Vaya Space, BRINC Drones, Red Cat Holdings/Teal Drones, Neros Technologies, Firestorm Labs, Vantage Robotics, Volansi, Freefly Systems, 3D Systems, Fathom Digital Manufacturing, Essentium, Sakuu, 6K Inc, Boston Materials, Type One Energy, Zap Energy, Helion Energy, General Fusion, Last Energy, Lear Corporation, Aptiv, Autoliv, ZF Group, Harley-Davidson, Thor Industries, Our Next Energy, Ascend Elements, Natron Energy, Li-Cycle, Mitra Chem, Veeco Instruments, Onto Innovation, Ultra Clean Holdings, Advanced Energy Industries, Brooks Automation/Azenta, FormFactor, Cohu Inc, FANUC America, KUKA Robotics, Omron Automation, Yaskawa America, Chef Robotics, Covariant, Sanctuary AI, Skild AI) — flagged as 'not reached' rather than checked-negative; worth trying their actual company domains directly in a future run.</v>
       </c>
     </row>
+    <row r="548">
+      <c r="A548" t="str">
+        <v>Markforged (Waltham/Billerica, MA)</v>
+      </c>
+      <c r="B548" t="str">
+        <v>Full Greenhouse board re-check</v>
+      </c>
+      <c r="C548" t="str">
+        <v>2026-10-01 ~07:00 UTC: Greenhouse board (slug 'markforged') has only 3 total open jobs company-wide (Product Marketing Manager, Senior Materials Process Engineer, Senior Supply Chain Planner) — zero intern/co-op titles. Consistent with every prior check of this company.</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="str">
+        <v>Inversion Space</v>
+      </c>
+      <c r="B549" t="str">
+        <v>Full Greenhouse board browse (not search-filtered)</v>
+      </c>
+      <c r="C549" t="str">
+        <v>2026-10-01 ~07:00 UTC: confirmed via direct enumeration of the full board (slug 'inversionspace', 81 jobs) that zero of the 81 titles contain 'intern', 'co-op', or 'internship' — entire board is senior/staff/full-time roles. Upgrades the prior run's '0 search results, possible stale cache' note to a hard confirmation: there is genuinely no internship/co-op posting here. No longer worth a dedicated re-check unless the board size changes markedly.</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="str">
+        <v>National sweep, 2026-10-01 pt.2 — new companies checked, no qualifying openings</v>
+      </c>
+      <c r="B550" t="str">
+        <v>ITT Inc. (Product Management Co-op, Global Supply Chain Co-op, Hardware &amp; Indirect Sourcing Co-op — all Seneca Falls NY Jan-Aug 2027; '2027 Engineering Co-op' Westminster SC); Onto Innovation (Mechanical Systems Engineer Intern, req R-5723); Azenta Life Sciences; Ascend Elements; Veeco Instruments; True Anomaly; Medical Murray; Teleflex; Baxter International; KLA Corporation; Framatome; Schneider Electric; Barnes Group / Barnes Aerospace</v>
+      </c>
+      <c r="C550" t="str">
+        <v>ITT Inc.'s Product Management/Supply Chain/Sourcing co-ops are discipline mismatches (business-facing, not engineering) despite accepting ME majors; its Westminster SC '2027 Engineering Co-op' (job 17721, confirmed live, $20-22/hr) explicitly starts 'May - August 2027' — wrong season. Onto Innovation: Mechanical Systems Engineer Intern confirmed live via Workday CXS API, discipline fits, but states no explicit season/year (open 30+ days, likely a rolling req) — fails the season bar. Azenta Life Sciences: Workday CXS API shows only 4 open jobs company-wide, sole internship is HR. Ascend Elements: own ATS (ClearCompany) states 'not actively hiring for any openings that meet your search criteria' — zero current openings. Veeco Instruments: intern-search page returns zero actually intern-titled roles. True Anomaly: Greenhouse API shows 50+ postings, none intern/co-op titled. Medical Murray: aggregator-only lead (Engineering Co-op/Internship Spring 2027, $22/hr) not found in the company's own current live-openings snapshot — could not independently confirm still open, not added. Teleflex: the one identifiable Industrial Engineer Intern req (12704) is confirmed 'position has been filled'; a same-titled internship could not be resolved to a distinct open req. Baxter International: co-op search on jobs.baxter.com returns 10 results, all full-time permanent roles, no co-op/intern posting live. KLA Corporation: only general Summer 2027 program-timeline info found, no Winter/Spring-specific req independently verified — insufficient evidence. Framatome: Lynchburg VA and Richland WA intern leads found via aggregators only, could not reach careers.framatome.com to confirm live status or season wording. Schneider Electric: only past/closed Spring 2026 and June-2026-start postings found at careers.se.com. Barnes Group/Barnes Aerospace: aggregator-cited Spring 2027 cycle's own stated close date (Sept 14, 2026) has already passed; own career sites currently show only a no-season Engineering Intern (Warren, MI) and a Finance Intern (wrong discipline). None added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C547"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C550"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 17 checked-excluded (2026-10-01 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0124sM833yunocTHYFnynm49
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M287"/>
+  <dimension ref="A1:M292"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11076,6 +11076,166 @@
       </c>
       <c r="J287" t="str">
         <v>New company. Distinct req from the iProd Design Center Co-op above (different team/business line, same site).</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>Gravitics</v>
+      </c>
+      <c r="B288" t="str">
+        <v>Mechanical Engineering Intern (2027 Winter session)</v>
+      </c>
+      <c r="C288" t="str">
+        <v>Mechanical Engineering (Mechanical Test Engineering or Motor Control Engineering track)</v>
+      </c>
+      <c r="D288" t="str">
+        <v>2027 Winter session, 10-12 weeks, January–March 2027</v>
+      </c>
+      <c r="E288" t="str">
+        <v>Marysville, WA (Greater Seattle Area)</v>
+      </c>
+      <c r="F288">
+        <v>2490</v>
+      </c>
+      <c r="G288" t="str">
+        <v>$28–$35/hr + housing assistance</v>
+      </c>
+      <c r="H288" t="str">
+        <v>https://job-boards.greenhouse.io/graviticsinc/jobs/4396521009</v>
+      </c>
+      <c r="I288" t="str">
+        <v>Yes — independently fetched directly via Greenhouse's own Jobs API (boards-api.greenhouse.io/v1/boards/graviticsinc/jobs/4396521009), HTTP 200, body states a '2027 Winter session' internship 'spanning January through March 2027,' checked 2026-10-01.</v>
+      </c>
+      <c r="J288" t="str">
+        <v>New company — designs/manufactures large-scale space station infrastructure. Two specialty tracks: Mechanical Test Engineering (sensors, tensile/vibration/thermal testing) or Motor Control Engineering (PWM, stepper motors, PID, embedded C/C++). Requires US citizenship or permanent residency.</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>Castelion</v>
+      </c>
+      <c r="B289" t="str">
+        <v>Mechanical Engineer Intern (Winter/Spring 2027)</v>
+      </c>
+      <c r="C289" t="str">
+        <v>Mechanical / Structural Engineering (Radar Engineering team)</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Torrance, CA</v>
+      </c>
+      <c r="F289">
+        <v>2600</v>
+      </c>
+      <c r="G289" t="str">
+        <v>Not stated on this posting (company's general intern band elsewhere is ~$30/hr)</v>
+      </c>
+      <c r="H289" t="str">
+        <v>https://www.castelion.com/careers/job/4386032009/</v>
+      </c>
+      <c r="I289" t="str">
+        <v>Yes — independently fetched directly, page live (not a filled/closed placeholder), title confirmed 'Mechanical Engineer Intern (Winter/Spring 2027)' with an active application form, checked 2026-10-01.</v>
+      </c>
+      <c r="J289" t="str">
+        <v>New company — hypersonic weapons/defense-tech startup. Radar Engineering team. Requires U.S. person status (citizen/GPR/refugee/asylee); may require DoS export-control access.</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B290" t="str">
+        <v>Pump Engineering Co-op (Spring/Summer 2027)</v>
+      </c>
+      <c r="C290" t="str">
+        <v>Mechanical Engineering (Fuel and Oil pump product line)</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Winter/Spring 2027 (runs January–July/August, including the Spring semester)</v>
+      </c>
+      <c r="E290" t="str">
+        <v>Rockford, IL</v>
+      </c>
+      <c r="F290">
+        <v>900</v>
+      </c>
+      <c r="G290" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H290" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/en-US/rec_rtx_ext_gateway/job/US-IL-ROCKFORD-P1--2421-11th-St--2421-11TH-ST-P1/Pump-Engineering-Co-op--Spring-Summer-2027-_01876586</v>
+      </c>
+      <c r="I290" t="str">
+        <v>Yes — independently fetched directly via RTX's own Workday CXS API, HTTP 200, req 01876586, posted 2026-09-28, body states 'will run January- July/August (including the Spring semester...)' verbatim, checked 2026-10-01.</v>
+      </c>
+      <c r="J290" t="str">
+        <v>Distinct req/site-team from the already-tracked Rockford IL Mechanical Engineering Co-op (01869227) and Mechanical Design Engineering Co-op (01873225) — this one is specifically Fuel/Oil pump engineering (CFD analysis, RCCA, supplier management). U.S. citizenship required, no security clearance required.</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>Yaskawa America, Inc.</v>
+      </c>
+      <c r="B291" t="str">
+        <v>Engineering Co-op (2027)</v>
+      </c>
+      <c r="C291" t="str">
+        <v>Mechanical / Mechatronics / Industrial Engineering (student selects track; also Electrical/CS/CompE)</v>
+      </c>
+      <c r="D291" t="str">
+        <v>2027, 6-month period, January–August or May–December (Jan–Aug option qualifies as Winter/Spring 2027)</v>
+      </c>
+      <c r="E291" t="str">
+        <v>Waukegan, IL (also Franklin WI; Buffalo Grove IL; Santa Clara/San Francisco CA)</v>
+      </c>
+      <c r="F291">
+        <v>850</v>
+      </c>
+      <c r="G291" t="str">
+        <v>$20.10–$27.12/hr + housing allowance for relocating students</v>
+      </c>
+      <c r="H291" t="str">
+        <v>https://recruiting.ultipro.com/YAS1000YAAMI/JobBoard/ac63a36b-3e0b-412c-939d-ae4625f85d3e/OpportunityDetail?opportunityId=d34cfbaa-53d1-4e44-a36e-497b7014a406</v>
+      </c>
+      <c r="I291" t="str">
+        <v>Yes — independently fetched directly via Yaskawa's own UltiPro/UKG JobBoard API, HTTP 200, req ENGIN002923, 'OpportunityIsClosed': false, posted 2026-08-28, description states 'various Engineering Co-ops for 2027... a 6 month period either January-August or May - December' verbatim, checked 2026-10-01.</v>
+      </c>
+      <c r="J291" t="str">
+        <v>Open to Mechanical, Electrical, Mechatronics, Industrial, CS, or Computer Engineering majors (sophomore standing+); student selects discipline track at application. A prior run's search had found only Summer-2027-titled Yaskawa postings and excluded the company — this is a distinct, newly-posted req with an explicit Jan–Aug 2027 option, independently re-verified rather than taken on the research agent's word alone.</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>Tesla</v>
+      </c>
+      <c r="B292" t="str">
+        <v>Internship, Powertrain, Manufacturing Automation Controls Engineering (Winter/Spring 2027)</v>
+      </c>
+      <c r="C292" t="str">
+        <v>Controls / Manufacturing Automation Engineering (PLC, robot programming, machine safety circuits)</v>
+      </c>
+      <c r="D292" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E292" t="str">
+        <v>Sparks, NV (Gigafactory Nevada)</v>
+      </c>
+      <c r="F292">
+        <v>2450</v>
+      </c>
+      <c r="G292" t="str">
+        <v>Not stated (blocked before pay info could be retrieved)</v>
+      </c>
+      <c r="H292" t="str">
+        <v>https://www.tesla.com/careers/search/job/internship-powertrain-manufacturing-automation-controls-engineering-winter-spring-2027--278960</v>
+      </c>
+      <c r="I292" t="str">
+        <v>Partial — official tesla.com domain, blocked automated fetch (403, bot protection) on independent re-check 2026-10-01. The URL itself (hosted on tesla.com with a specific job ID and the exact title in the slug) is a strong signal of a real listing, but open/closed status and full season text could not be independently confirmed. Verify live in-browser before applying.</v>
+      </c>
+      <c r="J292" t="str">
+        <v>Powertrain Manufacturing Automation Controls team — FANUC/KUKA robot programming, PLC, machine safety circuits.</v>
       </c>
     </row>
   </sheetData>
@@ -11552,14 +11712,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M287"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M292"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C550"/>
+  <dimension ref="A1:C567"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -17607,9 +17767,196 @@
         <v>ITT Inc.'s Product Management/Supply Chain/Sourcing co-ops are discipline mismatches (business-facing, not engineering) despite accepting ME majors; its Westminster SC '2027 Engineering Co-op' (job 17721, confirmed live, $20-22/hr) explicitly starts 'May - August 2027' — wrong season. Onto Innovation: Mechanical Systems Engineer Intern confirmed live via Workday CXS API, discipline fits, but states no explicit season/year (open 30+ days, likely a rolling req) — fails the season bar. Azenta Life Sciences: Workday CXS API shows only 4 open jobs company-wide, sole internship is HR. Ascend Elements: own ATS (ClearCompany) states 'not actively hiring for any openings that meet your search criteria' — zero current openings. Veeco Instruments: intern-search page returns zero actually intern-titled roles. True Anomaly: Greenhouse API shows 50+ postings, none intern/co-op titled. Medical Murray: aggregator-only lead (Engineering Co-op/Internship Spring 2027, $22/hr) not found in the company's own current live-openings snapshot — could not independently confirm still open, not added. Teleflex: the one identifiable Industrial Engineer Intern req (12704) is confirmed 'position has been filled'; a same-titled internship could not be resolved to a distinct open req. Baxter International: co-op search on jobs.baxter.com returns 10 results, all full-time permanent roles, no co-op/intern posting live. KLA Corporation: only general Summer 2027 program-timeline info found, no Winter/Spring-specific req independently verified — insufficient evidence. Framatome: Lynchburg VA and Richland WA intern leads found via aggregators only, could not reach careers.framatome.com to confirm live status or season wording. Schneider Electric: only past/closed Spring 2026 and June-2026-start postings found at careers.se.com. Barnes Group/Barnes Aerospace: aggregator-cited Spring 2027 cycle's own stated close date (Sept 14, 2026) has already passed; own career sites currently show only a no-season Engineering Intern (Warren, MI) and a Finance Intern (wrong discipline). None added.</v>
       </c>
     </row>
+    <row r="551">
+      <c r="A551" t="str">
+        <v>Trane Technologies</v>
+      </c>
+      <c r="B551" t="str">
+        <v>Re-check via a newly-found reliable method: direct Workday CXS API (tenant 'tranetechnologies', site 'Trane_Technologies_Careers'), bypassing the Phenom front-end that had repeatedly blocked prior checks</v>
+      </c>
+      <c r="C551" t="str">
+        <v>2026-10-01: searched all 'Spring 2027' (16 hits, Sales/Finance/Digital-Tech/EHS only) and the full Mechanical/Engineering Co-op roster (JR-8939 McGregor TX, JR-14080 Tyler TX, plus Clarksville TN/La Crosse WI/Panama City FL/Minneapolis MN variants) — all confirmed live via the API but still generic/evergreen with no 'Spring 2027' or similar season label, and none in the Boston, MA area. Unchanged conclusion from prior runs, now confirmed via a reliable direct method instead of the unreliable rendered page.</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B552" t="str">
+        <v>Full Workday CXS re-sweep: Electrical Engineering Co-Op (Spring 2027) JR002941, Sensor Electrical Engineering Co-op (Spring 2027) JR002885, Optics-Physics Sensor Engineering Co-op (Spring 2027) JR002884, Digital Engineering – Requirements Engineering Intern (Summer 2027) JR002945, Co-Op Student Engineering (Lowell, MA) JR002974, Acoustic and Vibration Technologies Co-op (Cambridge, MA) JR002688</v>
+      </c>
+      <c r="C552" t="str">
+        <v>2026-10-01: JR002941/JR002885 are Electrical Engineering discipline; JR002884 is Optics/Physics discipline — all excluded on discipline grounds. JR002945 is explicitly Summer 2027 — wrong season. JR002974 and JR002688 are both `canApply:true` but neither posting states an explicit season anywhere in title or body — excluded per the explicit-season bar. All 5 already-tracked qualifying Draper reqs (JR002882, JR002883-1, JR002940, JR002942, JR002944) re-confirmed still live this run.</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B553" t="str">
+        <v>Full re-sweep: Rapid Prototyping Aero/Mech Co-Op (Fall 2026, Group 77); Cyber Security Co-op (Winter/Spring 2027), Cyber System Exploitation Co-Op x2 (Jan-June 2027), Contracting and Logistics Co-Op (Jan-June 2027), Enterprise Platforms &amp; Infrastructure Co-op (Jan-Apr 2027), Enterprise Collaboration &amp; Web Services Co-op (Fall 2026); Optical Engineering Intern, Laser Communications Intern, Optical &amp; Quantum Communications Intern, Strategic &amp; Long-Range Communications Intern, Summer Research Program Intern 2027</v>
+      </c>
+      <c r="C553" t="str">
+        <v>2026-10-01: Rapid Prototyping explicitly states Fall 2026 only — wrong season. The Cyber/Contracting/Logistics/Enterprise group is in-season (several Jan-2027-start) but all cyber/IT/business/logistics discipline — mismatch. The Optical/Laser/Comms/Summer-Research group is all explicitly Summer 2027 — wrong season. All 3 already-tracked qualifying MIT LL reqs (Mechanical Eng Co-Op Group 07-71, Microfab Industrial Eng Co-Op, Microfabrication Eng Co-Op, both Group 08-35) re-confirmed still live this run.</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="str">
+        <v>Lexington Medical, Inc.</v>
+      </c>
+      <c r="B554" t="str">
+        <v>Manufacturing Engineering Intern (5404584008), Mechanical Engineering Intern (5400185008), Quality Systems Engineering Intern (5434143008) — all Bedford, MA</v>
+      </c>
+      <c r="C554" t="str">
+        <v>2026-10-01: all three confirmed live via Greenhouse's own board API, but all explicitly run June–August 2027 (Summer 2027) — wrong season; Quality Systems Engineering discipline is also borderline. The already-tracked Jan–Jun 2027 Mechanical Engineering Co-Op (5423105008) is unaffected and remains in `rows`.</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="str">
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+      </c>
+      <c r="B555" t="str">
+        <v>Westminster, SC job 15215 ('2026 Engineering Co-op'); Design Engineering Intern (Valencia, CA); Quality Engineering Intern (Lancaster, PA); Trade &amp; Supply Chain Data Analytics Co-op (Fall 2026-Spring 2027, Orchard Park, NY); general sweep of Motion Technologies and Connect and Control Technologies segments</v>
+      </c>
+      <c r="C555" t="str">
+        <v>2026-10-01: job 15215 now returns HTTP 410 Gone — closed/expired. Design Engineering Intern and Quality Engineering Intern are both explicitly Summer 2027 and not Boston-area — wrong season. Trade &amp; Supply Chain Data Analytics Co-op is in-season but business/supply-chain discipline — mismatch. No new qualifying reqs found at the Motion Technologies or Connect and Control Technologies segments. None added; the already-tracked Seneca Falls NY (17446/17708) and Stafford TX (17660) reqs are unaffected. Note: req 17447 (Seneca Falls NY, same title/team as 17446, separate req ID) remains treated as a duplicate headcount slot, not a separate row, per the prior run's decision.</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="str">
+        <v>GE Aerospace</v>
+      </c>
+      <c r="B556" t="str">
+        <v>Lynn CNC Programmer Co-Op (R5040944, posted 2026-09-30); national 'Spring 2027' Workday CXS sweep (16 results) and 'Lynn' location sweep (59 results)</v>
+      </c>
+      <c r="C556" t="str">
+        <v>2026-10-01: R5040944 requires current enrollment in a Vocational Technical High School — vocational/trade, same exclusion as all prior Lynn trade-co-op reqs, not a college engineering role. No other Lynn/Boston-area college-level engineering Spring 2027 req found. Other sitewide 'Spring 2027' GE reqs (Engines Engineering Co-op, Systems Engineering Co-op variants, Unison Engineering, etc.) are plausible disciplines but located outside the ~75mi Boston radius (Evendale OH, Saint George UT, etc.) — excluded on location grounds; the already-tracked Evendale-based reqs (R5029617, R5029663, R5030103) are unaffected.</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="str">
+        <v>RTX / Collins Aerospace</v>
+      </c>
+      <c r="B557" t="str">
+        <v>Systems Engineering Intern – Integration and Test (Andover, MA, req 01874598); Mechanical Engineering Internship (Tewksbury, MA, Summer 2027); Mechanical Engineering Co-op (Richardson, TX, Winter/Spring 2027); Mechanical Design Engineering Co-op (Jamestown, ND, Winter/Spring 2027, conflicting-signal req)</v>
+      </c>
+      <c r="C557" t="str">
+        <v>2026-10-01: Andover req 01874598 is open (`canApply:true`) but the full description never states an explicit season — excluded per the explicit-season bar despite the attractive Boston-area (Andover, MA) location; worth re-checking if the posting is ever updated with season text. Tewksbury req is explicitly Summer 2027 — wrong season. Richardson, TX req is in-season but requires 'Active and existing security clearance required after day 1' — impractical for a student without prior sponsorship, excluded. Jamestown ND req shows `canApply:true` in the Workday CXS search API but the public careers.rtx.com page for the same req reads 'this posting is no longer available' — excluded out of caution given the direct conflict between the two RTX-owned sources.</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="str">
+        <v>BAE Systems</v>
+      </c>
+      <c r="B558" t="str">
+        <v>Mechanical/RF/Systems Engineering Intern III (Summer 2027, Nashua/Merrimack/Hudson/Manchester NH); Industrial Engineering Co-Op (Fall Semester 2026, req 124709BR); Mechanical Engineering Co-Op (Sterling Heights MI, Cedar Rapids IA x3)</v>
+      </c>
+      <c r="C558" t="str">
+        <v>2026-10-01: the NH cluster is all Summer 2027-titled; the Fall 2026 Industrial Engineering Co-Op is a standalone Fall term, not extending into Winter/Spring. The Sterling Heights MI and Cedar Rapids IA x3 reqs all show 'This position has been filled and/or is no longer accepting applications' at jobs.baesystems.com. No qualifying Winter 2026/Spring 2027 posting found at BAE this run.</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="str">
+        <v>Teradyne (North Reading, MA)</v>
+      </c>
+      <c r="B559" t="str">
+        <v>jobs.teradyne.com direct search for Spring 2027 Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C559" t="str">
+        <v>2026-10-01: the search endpoint returned mostly empty/minimal server-rendered results (likely needs JS/pagination not reproducible via direct HTTP); web search only surfaced Spring 2026 (not 2027) Mechanical Engineering Co-op postings. No verified Spring 2027/Winter 2026 posting found — excluded as unverifiable/not found, worth a dedicated look if a headless-browser method becomes available.</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B560" t="str">
+        <v>Mechanical Engineering Co-Op (req R2476) — distinct req from the already-tracked Mechanical Engineering Co-Op (req R2495, Partial, in `rows`)</v>
+      </c>
+      <c r="C560" t="str">
+        <v>2026-10-01: bostondynamics.wd1.myworkdayjobs.com returned HTTP 403 'permission denied' on every Workday CXS API attempt (with and without cookies/Referer), and the rendered page is fully JS with no server-side content. Could not independently verify title, season, or open status — excluded per the verification bar rather than reported as confirmed.</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="str">
+        <v>Analog Devices (Wilmington, MA); Vicor (Andover, MA)</v>
+      </c>
+      <c r="B561" t="str">
+        <v>Spring/Fall co-op program status</v>
+      </c>
+      <c r="C561" t="str">
+        <v>2026-10-01: web search indicates both companies' Spring-term co-op postings typically open October–November 2026; no live Spring 2027/Winter 2026 posting could be directly confirmed via either company's own ATS as of this run — not yet posted/unconfirmed, worth a periodic re-check.</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="str">
+        <v>National sweep, 2026-10-01 ~13:00 UTC — wrong season, concentrated group</v>
+      </c>
+      <c r="B562" t="str">
+        <v>Xona Space Systems (Mechanical Engineering Intern, Summer 2027 only); Helion Energy (Electrical/Materials Engineering Intern, Summer 2026 only); Natron Energy (Battery/Data Engineering Intern, 12-week summer term); Advanced Energy Industries (Electrical/Firmware Intern, standalone Fall 2026, also confirmed closed/filled at jobs.advanced-energy.com); Trebor International/IDEX (Co-Op Pump Engineer, standalone Q4 2026 only); RTX Pump Engineering Co-op (Rockford IL P6 site, Summer/Fall 2027 variant — the Spring/Summer 2027 P1-site variant was added to `rows` instead); Stoke Space (only 'Summer 2027 Internship' postings currently live on Greenhouse; earlier aggregator-cited 'Spring 2027' listings are no longer on the live board)</v>
+      </c>
+      <c r="C562" t="str">
+        <v>Each independently fetched via its own ATS on 2026-10-01; none extend into Hamza's Winter 2026/Spring 2027 window. None added.</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="str">
+        <v>National sweep, 2026-10-01 ~13:00 UTC — confirmed closed/filled</v>
+      </c>
+      <c r="B563" t="str">
+        <v>True Anomaly (Greenhouse API, 189 jobs, zero intern-titled); Firestorm Labs (Aerospace/Software Engineering Internship postings explicitly show 'no longer accepting applications'); Orbit Fab (careers page states 'Internship Applications are Closed'); Turion Space (Ashby board returns 0 open jobs total)</v>
+      </c>
+      <c r="C563" t="str">
+        <v>Each independently fetched directly on 2026-10-01 and confirmed closed/filled/empty at the source. None added.</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="str">
+        <v>National sweep, 2026-10-01 ~13:00 UTC — no internship postings found</v>
+      </c>
+      <c r="B564" t="str">
+        <v>Benchmark Space Systems, Phantom Space, Interlune, BRINC Drones (Ashby, 33 jobs), Neros Technologies (Greenhouse, 97 jobs), Vantage Robotics, Freefly Systems, Sakuu (TriNet board), Li-Cycle, Mitra Chem, FormFactor (Workday CXS API, 78 jobs, none titled 'Intern'), KUKA Robotics (vacancies page, Internship filter = 0 results), Omron Automation (internship page lists only 3 non-US roles — Singapore x2, Netherlands), Skild AI (Greenhouse — only internship is 'Content Creator (Intern)', wrong discipline), Boston Materials, Type One Energy (Teamtailor board empty), Zap Energy</v>
+      </c>
+      <c r="C564" t="str">
+        <v>Each company's own current ATS/careers page fetched directly on 2026-10-01 and shows zero qualifying intern/co-op postings (or, for Omron, only non-US roles). None added.</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="str">
+        <v>Starfish Space; RTX (Richardson, TX)</v>
+      </c>
+      <c r="B565" t="str">
+        <v>Starfish Space's only open internship-type listing ('Skillbridge Internship', Ashby); RTX Mechanical Engineering Co-op, Richardson TX, Winter/Spring 2027</v>
+      </c>
+      <c r="C565" t="str">
+        <v>2026-10-01: Starfish Space's listing is restricted to DoD SkillBridge transitioning military service members, not students — wrong eligibility pool. (RTX Richardson TX is also logged above under the RTX/Collins Aerospace entry — active security clearance required after day 1, impractical for a student.) None added.</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="str">
+        <v>Sanctuary AI; General Fusion</v>
+      </c>
+      <c r="B566" t="str">
+        <v>US-based internship search for both</v>
+      </c>
+      <c r="C566" t="str">
+        <v>2026-10-01: Sanctuary AI's only open internship (ML Research Intern) is in Vancouver, BC, Canada — non-US. General Fusion is Vancouver, BC headquartered; its careers page routes to an external ADP portal that could not be accessed to find any US-based internship. Both excluded on location grounds (outside Hamza's US-only scope).</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="str">
+        <v>National sweep, 2026-10-01 ~13:00 UTC — unverifiable / no working ATS located</v>
+      </c>
+      <c r="B567" t="str">
+        <v>SpinLaunch (no Greenhouse/Lever board found, 404s; spinlaunch.com/careers unreachable); Red Cat Holdings/Teal Drones (only a vague 'Data Engineer internship' mention, no direct posting link locatable); Volansi (conflicting info on whether the company is still operating; no current postings found); 3D Systems (Mechanical Engineering Intern postings found only via LinkedIn aggregator, no live posting confirmed); Fathom Digital Manufacturing (no internship postings with titles found on the company's own site); 6K Inc (JS-rendered careers page, a 'Mechanical Engineering Co-op/Intern' mention found only via a Wayup aggregator, not confirmed current); Cohu Inc; FANUC America (no company-run ATS board locatable for either); Covariant (Mechanical Engineering Intern / AI Research Internship mentioned via LinkedIn only, no live company ATS board located); Atomos Space (general internship program mentioned, no season-specific current posting found); Vaya Space ('Engineering Intern – Spring' references Spring 2026, already elapsed; company's own careers page is JS-rendered with no retrievable listings); Pyka (an 'Early Interest Application' for a Winter/Spring 2027 Mechanical Engineering Internship — explicitly not yet a real open requisition per its own text; no live Greenhouse/Ashby board found to verify independently); Chef Robotics (only internship found is a Summer-only PhD Research Intern); 'General Astronautics' Spring 2027 Mechanical Engineering Intern (San Francisco) — surfaced only via an AI-search-engine summary with no company independently identifiable/verifiable, excluded as unverifiable/possibly mis-attributed</v>
+      </c>
+      <c r="C567" t="str">
+        <v>Each attempted directly via the company's own domain/ATS (not slug-guessing) on 2026-10-01; none could be independently verified as a genuine, currently-open, correctly-seasoned posting. None added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C550"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C567"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 5 checked-excluded (2026-10-01 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C6zpN4fr8DGbXtPkQAxAVF
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -11719,7 +11719,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C567"/>
+  <dimension ref="A1:C572"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -17954,9 +17954,64 @@
         <v>Each attempted directly via the company's own domain/ATS (not slug-guessing) on 2026-10-01; none could be independently verified as a genuine, currently-open, correctly-seasoned posting. None added.</v>
       </c>
     </row>
+    <row r="568">
+      <c r="A568" t="str">
+        <v>General Astronautics (YC-backed, San Francisco, CA)</v>
+      </c>
+      <c r="B568" t="str">
+        <v>'Engineering Internship/Co-op' — resolves the prior run's 'unverifiable/possibly mis-attributed' flag now that the company has been identified</v>
+      </c>
+      <c r="C568" t="str">
+        <v>2026-10-01 ~19:00 UTC: company identified and its own listing fetched directly via workatastartup.com/jobs/103201 — the live posting's own title reads 'Summer 2027 Engineering Internship/Co-op', not Spring 2027 as a third-party aggregator (jobleads.com) had mis-stated. A second sibling listing (workatastartup.com/jobs/94206) is 'Fall 2026 Engineering Internship/Co-op'. Neither is Winter 2026/Spring 2027 — wrong season per the primary source. Not added; the standing re-check note is now resolved and can be dropped.</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="str">
+        <v>CMTA, Inc. (multi-site engineering consulting firm)</v>
+      </c>
+      <c r="B569" t="str">
+        <v>Mechanical Engineer Intern/Co-op; Electrical Engineer Intern/Co-op Spring 2027 (multiple locations, incl. Frankfort KY)</v>
+      </c>
+      <c r="C569" t="str">
+        <v>2026-10-01 ~19:00 UTC: new company. The only Mechanical Engineering co-op track currently posted is explicitly 'Summer 2027' (starts ~May 2027) — wrong season. The track that does start in January/Spring 2027 is Electrical Engineer Intern/Co-op — discipline mismatch. No qualifying Mechanical/Spring-2027 combination found. Not added.</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="str">
+        <v>Buro Happold (Boston, MA office)</v>
+      </c>
+      <c r="B570" t="str">
+        <v>'Mechanical Co-op - Boston - Spring 2027' (title only found via third-party aggregator workopia.io)</v>
+      </c>
+      <c r="C570" t="str">
+        <v>2026-10-01 ~19:00 UTC: attempted to independently verify via the company's own sources — careershub.burohappold.com (the firm's actual US student/co-op hub) currently lists only one Boston mechanical co-op record, 'Mechanical Co-op- Boston (Fall 2025)', explicitly closed; the firm's main ATS at vacancies.burohappold.com shows no Boston or Mechanical Co-op listing on its current open-roles pages. Could not locate the Spring 2027 posting on any Buro Happold-owned domain — fails the primary-source verification bar despite the aggregator listing. Not added; worth a direct re-check if/when it appears on the firm's own site.</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="str">
+        <v>SoftInWay Inc. (Burlington, MA)</v>
+      </c>
+      <c r="B571" t="str">
+        <v>Turbomachinery Engineering Intern</v>
+      </c>
+      <c r="C571" t="str">
+        <v>2026-10-01 ~19:00 UTC: new company (turbomachinery/propulsion engineering consulting, Boston-metro). Confirmed live via direct fetch of the company's own posting page, but the posting is explicitly aimed at 'Recent graduates' holding a Master's degree (not current students) for a 6-month training-to-permanent-hire program, and states no Winter 2026/Spring 2027 season or start date anywhere in the body. Fails both the explicit-season bar and the current-student eligibility fit. Not added.</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="str">
+        <v>Insulet (Acton, MA)</v>
+      </c>
+      <c r="B572" t="str">
+        <v>Full re-sweep of the company's live Jan-June 2027 co-op batch via direct Workday CXS API search (32 results) — R&amp;D Mechanical Engineering (REQ-2026-18007), Mechanical Lifecycle (REQ-2026-18155), Manufacturing Engineering (REQ-2026-18078), R&amp;D Manufacturing (REQ-2026-18069), Supplier Development Engineering-Mechanical (REQ-2026-18209), Graduate Co-op Manufacturing Engineering (REQ-2026-18086)</v>
+      </c>
+      <c r="C572" t="str">
+        <v>2026-10-01 ~19:00 UTC: all six independently re-confirmed still live (endDate 2026-12-31) via direct API fetch, but all six were already present in `rows` from prior runs (same req numbers/URLs) — no new rows added. Positive freshness re-check only.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C567"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C572"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 6 checked-excluded (2026-10-02 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HTbGRXUWkx3CFdLJ98X5jA
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M292"/>
+  <dimension ref="A1:M295"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -3044,10 +3044,10 @@
         <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Mechanical-Design-Engineering-Co-op--Winter-Spring-2027-_01871736</v>
       </c>
       <c r="I65" t="str">
-        <v>Yes — fetched directly via RTX's own Workday CXS API, posted 2026-09-21.</v>
+        <v>Yes — fetched directly via RTX's own Workday CXS API, posted 2026-09-21. 2026-10-02: re-confirmed canApply:true via the Workday API (endDate 2026-10-02 — today), though the public careers.rtx.com marketing page continues to show 'no longer available' text — a conflict persisting across several runs. Treating the Workday API as authoritative per established practice; may expire within hours of this check.</v>
       </c>
       <c r="J65" t="str">
-        <v>Distinct req from the already-tracked Jamestown ND 'Structural Engineering Co-op' (req 01873938) at the same site — different title/req, not a duplicate.</v>
+        <v>Distinct req from the already-tracked Jamestown ND 'Structural Engineering Co-op' (req 01873938) at the same site — different title/req, not a duplicate. endDate is today (2026-10-02) — likely to close by the next run.</v>
       </c>
       <c r="K65" t="str">
         <v>Open resume</v>
@@ -10874,16 +10874,16 @@
         <v>210</v>
       </c>
       <c r="G281" t="str">
-        <v>Not stated on current posting</v>
+        <v>$18–$24/hr</v>
       </c>
       <c r="H281" t="str">
         <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a061fa5de22f3c</v>
       </c>
       <c r="I281" t="str">
-        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, Apply button present, title and body state 'Spring 2027 Mechanical Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, Apply button present, title and body state 'Spring 2027 Mechanical Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live again — the previously-stated 'Deadline: October 1, 2026' text no longer appears anywhere on the current live page; posting now reads 'beginning January 2027 through end of summer 2027' with no deadline language at all, and pay ($18-24/hr) is now visible.</v>
       </c>
       <c r="J281" t="str">
-        <v>New company — defense/aerospace motion &amp; flow control systems manufacturer. Design/production/quality/test-development work, 3D CAD (Pro-E/Creo). US citizenship required (ITAR). TIME-SENSITIVE: posting states 'Deadline: October 1, 2026' (the day this was verified) with an invitation-only interview day October 16, 2026 — confirm it hasn't already closed before staging/applying.</v>
+        <v>New company — defense/aerospace motion &amp; flow control systems manufacturer. Design/production/quality/test-development work, 3D CAD (Pro-E/Creo). US citizenship required (ITAR). The Oct 1, 2026 deadline previously stated on this posting has since been removed from the live page (re-checked 2026-10-02) — appears to remain open past that date.</v>
       </c>
     </row>
     <row r="282">
@@ -10906,16 +10906,16 @@
         <v>210</v>
       </c>
       <c r="G282" t="str">
-        <v>Not stated on current posting</v>
+        <v>$18–$24/hr</v>
       </c>
       <c r="H282" t="str">
         <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a062229f2536d0</v>
       </c>
       <c r="I282" t="str">
-        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, title and body state 'Spring 2027 Control Systems Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, title and body state 'Spring 2027 Control Systems Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live, same deadline-text removal as the Mechanical Engineering sibling above.</v>
       </c>
       <c r="J282" t="str">
-        <v>Same company as above. MATLAB control-system simulation/modeling, requirements management in IBM DOORS, systems engineering deliverables. US citizenship required (ITAR). TIME-SENSITIVE: same October 1, 2026 deadline as the Mechanical Engineering sibling above — confirm it hasn't already closed before staging/applying.</v>
+        <v>Same company as above. MATLAB control-system simulation/modeling, requirements management in IBM DOORS, systems engineering deliverables. US citizenship required (ITAR). The previously-stated Oct 1, 2026 deadline is gone from the live posting as of 2026-10-02 — appears to remain open.</v>
       </c>
     </row>
     <row r="283">
@@ -11232,10 +11232,106 @@
         <v>https://www.tesla.com/careers/search/job/internship-powertrain-manufacturing-automation-controls-engineering-winter-spring-2027--278960</v>
       </c>
       <c r="I292" t="str">
-        <v>Partial — official tesla.com domain, blocked automated fetch (403, bot protection) on independent re-check 2026-10-01. The URL itself (hosted on tesla.com with a specific job ID and the exact title in the slug) is a strong signal of a real listing, but open/closed status and full season text could not be independently confirmed. Verify live in-browser before applying.</v>
+        <v>Partial — official tesla.com domain, blocked automated fetch (403, bot protection) on independent re-check 2026-10-01 and again 2026-10-02 (multiple user-agent/header variations all still 403). A third-party mirror (milwaukeejobs.com) showed the same listing as live, 'posted 5 days ago,' as of 2026-10-02, but this is a secondary source, not Tesla's own site — open/closed status remains unconfirmed on the primary source. Verify live in-browser before applying.</v>
       </c>
       <c r="J292" t="str">
         <v>Powertrain Manufacturing Automation Controls team — FANUC/KUKA robot programming, PLC, machine safety circuits.</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>The Exploration Company</v>
+      </c>
+      <c r="B293" t="str">
+        <v>Spring 2027 Internship (Engineering)</v>
+      </c>
+      <c r="C293" t="str">
+        <v>General Engineering (crewed spacecraft systems — design/test/validation)</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Spring 2027 (starting January 2027, min. 12 weeks)</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Houston, TX</v>
+      </c>
+      <c r="F293">
+        <v>1600</v>
+      </c>
+      <c r="G293" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H293" t="str">
+        <v>https://jobs.ashbyhq.com/the-exploration-company/3f4e976b-0d0c-4440-a943-6b4b0b2f6ddf</v>
+      </c>
+      <c r="I293" t="str">
+        <v>Yes — independently fetched directly via the company's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/the-exploration-company), HTTP 200, published 2026-09-03, body states 'Spring 2027 Engineering Internship... Able to work full-time (40 hours per week) for a minimum of 12 weeks beginning January 2027' verbatim, checked 2026-10-02.</v>
+      </c>
+      <c r="J293" t="str">
+        <v>New company — French/German crewed-spacecraft (Nyx vehicle) developer with a Houston, TX engineering presence. Role is general engineering support (design/test/validation of engineering systems), not a named sub-discipline. Requires US citizenship or lawful permanent residency (ITAR/EAR). No housing/relocation provided. Posted 2026-09-03 — about 4 weeks old, slightly past the usual ~3-week freshness preference but still open and a strong discipline/location fit.</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>Lincoln Electric</v>
+      </c>
+      <c r="B294" t="str">
+        <v>Mechanical Engineering Spring 2027 Co-op</v>
+      </c>
+      <c r="C294" t="str">
+        <v>Mechanical / Industrial Engineering (automation, robotics, manufacturing equipment)</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Spring 2027 (Target Program Dates: January 12 – April 16, 2027)</v>
+      </c>
+      <c r="E294" t="str">
+        <v>Plymouth, MI</v>
+      </c>
+      <c r="F294">
+        <v>650</v>
+      </c>
+      <c r="G294" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H294" t="str">
+        <v>https://jobs.lincolnelectric.com/job/Plymouth-Mechanical-Engineering-Spring-2027-Co-op-%28Plymouth%2C-MI%29-MI-48170/1432989733/</v>
+      </c>
+      <c r="I294" t="str">
+        <v>Yes — independently fetched directly via Lincoln Electric's own careers site (jobs.lincolnelectric.com), HTTP 200, Req ID 29823, page states 'Target Program Dates: January 12th – April16th, 2027' verbatim, distinct from a same-site 'Mechanical Engineering Summer 2027 Internship' sibling at the same Plymouth, MI location, checked 2026-10-02.</v>
+      </c>
+      <c r="J294" t="str">
+        <v>Automation facility — develops custom manufacturing equipment, automated systems, and robotic solutions for customer applications. Bachelor's in engineering/engineering technology required; eligible to work in the US without sponsorship. 3.0+ GPA preferred. Includes a company-paid Immersion Day at Cleveland, OH HQ.</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>Insulet</v>
+      </c>
+      <c r="B295" t="str">
+        <v>Co-op - Supplier Quality Engineering: January - June 2027 (Onsite)</v>
+      </c>
+      <c r="C295" t="str">
+        <v>Mechanical / Industrial / Bio-Engineering (supplier quality, Six Sigma/Lean)</v>
+      </c>
+      <c r="D295" t="str">
+        <v>January 11 – June 30, 2027</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Acton, MA</v>
+      </c>
+      <c r="F295">
+        <v>25</v>
+      </c>
+      <c r="G295" t="str">
+        <v>$24.00–$28.50/hr</v>
+      </c>
+      <c r="H295" t="str">
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op---Supplier-Quality-Engineering--January---June-2027--Onsite-_REQ-2026-18125</v>
+      </c>
+      <c r="I295" t="str">
+        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, canApply true, req REQ-2026-18125, posted 2026-10-01, body states 'Position Dates: January 11, 2027 – June 30, 2027' verbatim, checked 2026-10-02.</v>
+      </c>
+      <c r="J295" t="str">
+        <v>Boston metro (Acton). Global Supplier Quality Engineering team — supplier selection/qualification, Engineering Change Orders, External Quality Action Requests, Six Sigma/Lean. Requires currently-enrolled undergrad in mechanical, industrial, or bio-engineering, 3.0+ GPA. Not eligible for visa sponsorship. Sibling to Insulet's many other already-tracked Acton Jan–June 2027 co-ops.</v>
       </c>
     </row>
   </sheetData>
@@ -11712,14 +11808,14 @@
     <hyperlink ref="M201" r:id="rId470"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M292"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M295"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C572"/>
+  <dimension ref="A1:C578"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -18009,9 +18105,75 @@
         <v>2026-10-01 ~19:00 UTC: all six independently re-confirmed still live (endDate 2026-12-31) via direct API fetch, but all six were already present in `rows` from prior runs (same req numbers/URLs) — no new rows added. Positive freshness re-check only.</v>
       </c>
     </row>
+    <row r="573">
+      <c r="A573" t="str">
+        <v>Reframe Systems (Billerica/Andover, MA)</v>
+      </c>
+      <c r="B573" t="str">
+        <v>'Mechanical Engineer (Spring 2027 Co-op)', Andover MA (microfactory in Billerica, MA) — new company, housing-construction robotics/automation startup</v>
+      </c>
+      <c r="C573" t="str">
+        <v>2026-10-02: confirmed live via direct fetch of the company's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/reframesystems), req f5275832-8373-4971-b5f6-6aaececcb061, posted 2026-08-05. However, despite the title saying 'Spring 2027 Co-op,' the posting's own body text states the role is for a 'full-time, semester-length co-op in Billerica, MA this fall' — a direct title/body season contradiction (same pattern as the already-excluded Lincoln Electric Controls Eng. and Analog Devices Healthcare ME title/body mismatches). Fails the season-verification bar on the body text; not added despite the Boston-area/strong-discipline fit. Worth re-checking if a dated, internally-consistent Spring 2027 version ever appears.</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="str">
+        <v>E Ink Corporation (Billerica, MA)</v>
+      </c>
+      <c r="B574" t="str">
+        <v>'Co-op Mechanical Engineering Special Projects' (ref C4HB); 'Co-op Prototype Mechanical Engineer' (C2DB); 'Co-op ePaper Product Development Engineering' (C2HB)</v>
+      </c>
+      <c r="C574" t="str">
+        <v>2026-10-02: all three found only via aggregators (Indeed/Glassdoor/LinkedIn/ZipRecruiter); eink.com's own career page is JS-rendered with no locatable job-board link or identifiable ATS reachable via direct fetch in the time available. No season/year stated in any aggregator summary either. Unverifiable on primary source — not added; worth a future attempt with a different access method given the strong Boston-area/discipline fit.</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="str">
+        <v>Qnity Electronics (Marlborough, MA)</v>
+      </c>
+      <c r="B575" t="str">
+        <v>'2027 Spring Co-Op: Chemical, Mechanical and Electrical Engineering Opportunities'</v>
+      </c>
+      <c r="C575" t="str">
+        <v>2026-10-02: new company (DuPont Electronics spinoff). Aggregator listings (Glassdoor/ZipRecruiter) describing this posting's title as a Glassdoor-listed 'Dupont ... 2026 Summer Intern &amp; Co-Op' job underneath a 'Spring 2027' secondary summary — an internal contradiction similar to prior aggregator-mislabeling cases (e.g. General Astronautics). Could not locate Qnity's own ATS (qnity.com careers page returns no identifiable job-board link) to resolve the conflict. Not added — season unconfirmed and possibly Summer 2026, not Spring 2027.</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="str">
+        <v>Storion Energy (Billerica, MA)</v>
+      </c>
+      <c r="B576" t="str">
+        <v>'Mechanical Engineering Co-op', battery-stack development (Vanadium Redox Flow Battery joint venture of Stryten Energy and Largo Inc.)</v>
+      </c>
+      <c r="C576" t="str">
+        <v>2026-10-02: new company, aggregator-only (Indeed/SimplyHired); no company career page or identifiable ATS (Greenhouse/Lever/Ashby/Workday) could be located via direct search. Season (reportedly Jan-Jul 2027 per aggregator) and open/closed status both unconfirmed on any primary source. Not added; worth a follow-up if a direct company careers URL can be found.</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B577" t="str">
+        <v>'Lynn CNC Programmer Co-Op', req R5040944, posted 2026-09-30</v>
+      </c>
+      <c r="C577" t="str">
+        <v>2026-10-02: confirmed live via Workday CXS API (canApply:true), but the posting explicitly requires the applicant to be 'currently enrolled in a Vocational Technical High School (at least midway through junior year)' — this is a high-school vocational trade co-op, not a college engineering internship. Audience/discipline mismatch; not added.</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="str">
+        <v>Vicor (Andover, MA); Buro Happold (Boston, MA)</v>
+      </c>
+      <c r="B578" t="str">
+        <v>Full re-sweep of Vicor's current 29 live postings (careers.vicorpower.com); re-fetch of Buro Happold's careershub.burohappold.com and vacancies.burohappold.com</v>
+      </c>
+      <c r="C578" t="str">
+        <v>2026-10-02: Vicor — all 29 current postings re-confirmed as operators/engineers/technicians; zero co-op/intern-titled roles exist company-wide right now, unchanged from the standing exclusion. Buro Happold — re-fetched both primary career sites directly; still no Boston, MA listing of any kind (only Pune/Mumbai India roles and a non-Boston 'Graduate Engineer — Urban Development, NY/LA, Summer 2027' posting currently live) — reconfirms the prior run's exclusion, the aggregator-only Boston listing remains unlocatable on Buro Happold's own sites.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C572"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C578"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 2 new postings, 6 checked-excluded (2026-10-02 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVq7rqhmpdQ7JkATj41sKY
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M295"/>
+  <dimension ref="A1:M297"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11323,6 +11323,70 @@
       </c>
       <c r="J295" t="str">
         <v>New company — in-space transportation vehicle manufacturer. Distinct from Impulse Space's already-excluded Spring 2027 RF/Antenna Engineering Intern reqs (electrical discipline, outside target list) and its ~25 Summer 2027 mechanical/propulsion/manufacturing internships. Company's mechanical/propulsion/structures reqs were re-checked across several prior runs (09-23 through 09-25) and found Summer-2027-only at the time; this Manufacturing Engineering req is newly found as of this run.</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>CMTA, Inc. (via Legence)</v>
+      </c>
+      <c r="B296" t="str">
+        <v>Mechanical Engineer Intern/Co-op, Spring 2027</v>
+      </c>
+      <c r="C296" t="str">
+        <v>Mechanical Engineering (MEP/HVAC building-systems consulting)</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Spring 2027 (starts January 2027, dates flexible with school calendar)</v>
+      </c>
+      <c r="E296" t="str">
+        <v>Boston, MA (170 Milk Street)</v>
+      </c>
+      <c r="F296">
+        <v>0</v>
+      </c>
+      <c r="G296" t="str">
+        <v>Competitive hourly, OT eligible (exact rate not stated)</v>
+      </c>
+      <c r="H296" t="str">
+        <v>https://jobs.dayforcehcm.com/en-US/legence/studentportal/jobs/33378</v>
+      </c>
+      <c r="I296" t="str">
+        <v>Yes — fetched directly (HTTP 200); raw server-side response carries the full job JSON (jobPostingId 33378, jobReqId 4002, postingAppliedStatus.canApplyAgain true, no expiry date set) even though the rendered page on top is JS-heavy.</v>
+      </c>
+      <c r="J296" t="str">
+        <v>FLAGGED DISCIPLINE BORDERLINE: this is MEP/HVAC building-systems engineering (HVAC layout, one-line diagrams, building energy efficiency) for a Boston architecture/engineering consulting firm — not aerospace/manufacturing/robotics work. Included given the exact Boston, MA location and literal 'Mechanical Engineer' title/degree requirement (pursuing BS Mechanical or Architectural Engineering, preferably sophomore/junior); Hamza should judge personal interest fit. Full-time 40hr/week onsite. No visa sponsorship available.</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>Eversource Energy</v>
+      </c>
+      <c r="B297" t="str">
+        <v>2027 Co-op: Capital Projects</v>
+      </c>
+      <c r="C297" t="str">
+        <v>Civil / Mechanical / Electrical Engineering (posting states 'civil and mechanical engineering also considered')</v>
+      </c>
+      <c r="D297" t="str">
+        <v>2027 (exact term not printed on this specific posting; a sibling Eversource co-op in the same posting batch, Substation Design Engineering, explicitly states 'January–June 2027' — very likely the same cycle, but not independently confirmed on this posting's own text)</v>
+      </c>
+      <c r="E297" t="str">
+        <v>Westwood, MA</v>
+      </c>
+      <c r="F297">
+        <v>14</v>
+      </c>
+      <c r="G297" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H297" t="str">
+        <v>https://jobs.eversource.com/job/westwood/2027-co-op-capital-projects/7774/101320869904</v>
+      </c>
+      <c r="I297" t="str">
+        <v>Yes — fetched directly, live posting, posted 2026-09-28, 'Apply Now' active, 1 opening.</v>
+      </c>
+      <c r="J297" t="str">
+        <v>New Boston-area utility co-op employer (Northeastern/WPI-style structured co-op program) — worth periodic re-checking since Eversource posts new reqs each cycle. No visa sponsorship ('applicants requiring visa sponsorship... will not be considered'). No GPA/class-standing stated. Season wording caveat above — confirm the exact term directly before applying.</v>
       </c>
     </row>
   </sheetData>
@@ -11796,14 +11860,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M295"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M297"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C591"/>
+  <dimension ref="A1:C597"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -18302,9 +18366,75 @@
         <v>2026-10-02 (later same day): queried the company's live Ashby posting API directly — the contradictory posting is now GONE entirely. The board currently lists 10 open roles (Plant Manager, Carpenter, Drywall Hanger, Journeyman Electrician, Licensed Plumber, HVAC Technician, Full Stack Software Engineer, Cabinet CNC Operator, Construction Administrator, Dream Job), none of them Mechanical Engineer. The posting was pulled/removed rather than corrected to be internally consistent. Dropping the 'worth re-checking for a corrected version' note — nothing to re-check until a new Mechanical Engineer req appears.</v>
       </c>
     </row>
+    <row r="592">
+      <c r="A592" t="str">
+        <v>CMTA, Inc. (a Legence company) — Boston, MA office</v>
+      </c>
+      <c r="B592" t="str">
+        <v>'Mechanical Engineer Intern/Co-op Spring 2027', 170 Milk Street, Boston, MA — resolves the earlier-today 'fails the direct-verification bar' entry above</v>
+      </c>
+      <c r="C592" t="str">
+        <v>2026-10-02 (later same day): a second verification attempt beat the JS rendering by hitting Dayforce's underlying JSON API directly with a fetched CSRF token (GET /api/auth/csrf then POST /api/geo/legence/jobposting/search), returning the full job record (jobPostingId 33378, jobReqId 4002 — a different posting ID than the 33675 referenced in the earlier-today entry, same role/location). The human-facing URL (jobs.dayforcehcm.com/en-US/legence/studentportal/jobs/33378) was independently fetched directly (HTTP 200) and confirmed to carry the same job JSON server-side. MOVED to `rows` as a Yes-verified Partial-on-discipline posting (MEP/HVAC building-systems engineering, flagged for Hamza's own judgment).</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="str">
+        <v>E Ink Corporation (Billerica, MA)</v>
+      </c>
+      <c r="B593" t="str">
+        <v>Full internship search — resolves the earlier-today 'unverifiable on primary source' entry above</v>
+      </c>
+      <c r="C593" t="str">
+        <v>2026-10-02 (later same day): located E Ink's real ATS (UltiPro/UKG, recruiting.ultipro.com/EIN1000EINK) and queried its live JobBoardView/LoadSearchResults JSON API directly, which returned all 22 currently-open E Ink requisitions (Billerica, MA and Fremont, CA). None are internships or co-ops — all are full-time Scientist/Engineer/Technician roles. The 'Co-op'/'Intern' titles seen on aggregators (C4HB, C2DB, C2HB) are not in the live feed — closed/stale. Upgrades the earlier-today 'unverifiable' framing to a hard confirmation: E Ink currently has zero open internship/co-op postings. Not added.</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>Kaman Aerospace / Barnes Aerospace (CT)</v>
+      </c>
+      <c r="B594" t="str">
+        <v>General mechanical engineering intern/co-op search</v>
+      </c>
+      <c r="C594" t="str">
+        <v>2026-10-02: new companies checked (Kaman Aerospace specifically, distinct from the already-logged Barnes Group/Barnes Aerospace Warren MI entry). No specific internship/co-op postings could be located for either via search or direct site access. Not added; low-confidence exclusion, worth a dedicated ATS-identification attempt in a future run.</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>Skydio</v>
+      </c>
+      <c r="B595" t="str">
+        <v>'Hardware Test &amp; Reliability Intern', San Mateo, CA</v>
+      </c>
+      <c r="C595" t="str">
+        <v>2026-10-02: confirmed real via direct fetch (full description, pay bands $47-58/hr, E-Verify requirement loaded), but could not visually confirm an active Apply control on the JS-heavy page. More importantly, the posting's own stated season is 'Fall 2026/Winter 2027' — company-stated 'Winter 2027' is a near-miss on season-naming, same treatment as the already-excluded Astranis 'Winter 2027' req (2026-09-20/22): Hamza's tracker defines the Jan-starting cohort as 'Winter 2026,' not 'Winter 2027,' and the posting doesn't extend into Spring 2027. Excluded on strict season-match grounds; flagged as a near-miss worth Hamza's own reconsideration of the season window, same as the Astranis precedent.</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Re-check of both previously-tracked-then-excluded reqs (Mechanical Engineering Co-Op R2476; Mechanical Engineering Intern R2495)</v>
+      </c>
+      <c r="C596" t="str">
+        <v>2026-10-02: queried Boston Dynamics' Workday CXS API directly for both reqs — both now return errorCode S22 ('permission denied,' distinct from a 404 for a bad/never-existed URL, indicating the reqs existed but are no longer public) — and paged through all 73 current company-wide postings, confirming zero Intern/Co-Op-titled roles exist anywhere at Boston Dynamics right now. Reconfirms and closes out the standing 'both closed' finding with a fresh, independent, full-board check. No change to `rows`/`checked` status.</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>Analog Devices (Wilmington, MA)</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Healthcare Mechanical Engineering Co-op (Spring), req R266691 — re-check</v>
+      </c>
+      <c r="C597" t="str">
+        <v>2026-10-02 (later same day): re-fetched directly via ADI's own Workday CXS API — still live (canApply true) and still internally contradictory on season ('running from June through December' in the role description vs. 'Available to work full-time, on-site from January through June' in Qualifications, no year stated either way). Also checked for a broader Spring 2027 co-op slate at analog.com — none found yet; R266691 remains the only Analog Devices posting live. Unchanged from the long-standing exclusion; still excluded.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C591"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C597"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 11 new postings, 23 checked-excluded (2026-10-02 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GMPzKu2CK5Ya5WWEPXULcE
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M297"/>
+  <dimension ref="A1:M308"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11387,6 +11387,358 @@
       </c>
       <c r="J297" t="str">
         <v>New Boston-area utility co-op employer (Northeastern/WPI-style structured co-op program) — worth periodic re-checking since Eversource posts new reqs each cycle. No visa sponsorship ('applicants requiring visa sponsorship... will not be considered'). No GPA/class-standing stated. Season wording caveat above — confirm the exact term directly before applying.</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B298" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C298" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D298" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Anoka, MN</v>
+      </c>
+      <c r="F298">
+        <v>1127</v>
+      </c>
+      <c r="G298" t="str">
+        <v>Not stated on posting (a third-party aggregator estimated $21-28/hr, unconfirmed on the primary source)</v>
+      </c>
+      <c r="H298" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Anoka-Minnesota-USA/Manufacturing-Engineering-Co-Op_R0023507</v>
+      </c>
+      <c r="I298" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~24 days ago.</v>
+      </c>
+      <c r="J298" t="str">
+        <v>New company. Graco also posts sibling 'May - December 2027' co-ops at the same sites — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B299" t="str">
+        <v>Automation Engineering Co-Op</v>
+      </c>
+      <c r="C299" t="str">
+        <v>Automation / Mechanical Engineering</v>
+      </c>
+      <c r="D299" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E299" t="str">
+        <v>Rogers, MN (David Koch Center)</v>
+      </c>
+      <c r="F299">
+        <v>1135</v>
+      </c>
+      <c r="G299" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H299" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Automation-Engineering-Co-Op--January---August-2027-_R0023586</v>
+      </c>
+      <c r="I299" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+      </c>
+      <c r="J299" t="str">
+        <v>New company (Graco, industrial fluid-handling equipment manufacturer).</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B300" t="str">
+        <v>Manufacturing Engineering Co-op</v>
+      </c>
+      <c r="C300" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D300" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E300" t="str">
+        <v>Rogers, MN (David Koch Center)</v>
+      </c>
+      <c r="F300">
+        <v>1135</v>
+      </c>
+      <c r="G300" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H300" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering-Co-op--January---August-2027-_R0023611</v>
+      </c>
+      <c r="I300" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+      </c>
+      <c r="J300" t="str">
+        <v>Sibling req to the Anoka Manufacturing Engineering Co-Op at a different Graco site.</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B301" t="str">
+        <v>Manufacturing Engineering Co-op</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D301" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Dayton, MN</v>
+      </c>
+      <c r="F301">
+        <v>1134</v>
+      </c>
+      <c r="G301" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H301" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Dayton-Minnesota-USA/Manufacturing-Engineering-Co-op--January---August-2027-_R0023612</v>
+      </c>
+      <c r="I301" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+      </c>
+      <c r="J301" t="str">
+        <v>Another sibling Graco Manufacturing Engineering Co-Op req at a third site.</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B302" t="str">
+        <v>Quality Engineering Co-op</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Quality / Mechanical / Manufacturing Engineering</v>
+      </c>
+      <c r="D302" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Rogers, MN (David Koch Center)</v>
+      </c>
+      <c r="F302">
+        <v>1135</v>
+      </c>
+      <c r="G302" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H302" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Quality-Engineering-Co-op--January---August-2027-_R0023573</v>
+      </c>
+      <c r="I302" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+      </c>
+      <c r="J302" t="str">
+        <v>Quality engineering within a manufacturing plant setting.</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>Graco Inc.</v>
+      </c>
+      <c r="B303" t="str">
+        <v>Manufacturing Engineering (Operational Technology) Co-op</v>
+      </c>
+      <c r="C303" t="str">
+        <v>Manufacturing Engineering / Industrial Controls</v>
+      </c>
+      <c r="D303" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Rogers, MN (David Koch Center)</v>
+      </c>
+      <c r="F303">
+        <v>1135</v>
+      </c>
+      <c r="G303" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H303" t="str">
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering--Operational-Technology--Co-op--January---August-2027-_R0023574</v>
+      </c>
+      <c r="I303" t="str">
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+      </c>
+      <c r="J303" t="str">
+        <v>OT/industrial-controls-flavored manufacturing engineering co-op.</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B304" t="str">
+        <v>Manufacturing Engineering Co-op</v>
+      </c>
+      <c r="C304" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D304" t="str">
+        <v>January - June 2027</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Anoka, MN</v>
+      </c>
+      <c r="F304">
+        <v>1127</v>
+      </c>
+      <c r="G304" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H304" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Manufacturing-Engineering-Co-op--January---June-2027-_R23576</v>
+      </c>
+      <c r="I304" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, posted recently (within ~18 days).</v>
+      </c>
+      <c r="J304" t="str">
+        <v>New company (nVent, electrical/thermal-management manufacturer spun off from Pentair). nVent also posts sibling 'June - Dec 2027' co-ops at the same sites — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B305" t="str">
+        <v>Packaging Engineering Co-op</v>
+      </c>
+      <c r="C305" t="str">
+        <v>Packaging Engineering (mechanical-design-adjacent)</v>
+      </c>
+      <c r="D305" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Anoka, MN</v>
+      </c>
+      <c r="F305">
+        <v>1127</v>
+      </c>
+      <c r="G305" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H305" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Packaging-Engineering-Co-op--January---August-2027-_R23570</v>
+      </c>
+      <c r="I305" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true.</v>
+      </c>
+      <c r="J305" t="str">
+        <v>FLAGGED DISCIPLINE BORDERLINE: packaging engineering, not core mechanical/aero/manufacturing design — included for Hamza's own judgment.</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B306" t="str">
+        <v>Mechanical Engineering Co-Op</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Jan - Aug 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Solon, OH (ERICO division)</v>
+      </c>
+      <c r="F306">
+        <v>538</v>
+      </c>
+      <c r="G306" t="str">
+        <v>$25.00/hr</v>
+      </c>
+      <c r="H306" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Solon-OH-US/Mechanical-Engineering-Co-Op--Jan---Aug-2027-_R23577</v>
+      </c>
+      <c r="I306" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
+      </c>
+      <c r="J306" t="str">
+        <v>ERICO is an nVent division (electrical/mechanical fastening products).</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B307" t="str">
+        <v>Mechanical Engineering and Design Co-op</v>
+      </c>
+      <c r="C307" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D307" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Anoka, MN</v>
+      </c>
+      <c r="F307">
+        <v>1127</v>
+      </c>
+      <c r="G307" t="str">
+        <v>$25.00/hr</v>
+      </c>
+      <c r="H307" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Mechanical-Engineering-and-Design-Co-op--January---August-2027-_R23572</v>
+      </c>
+      <c r="I307" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
+      </c>
+      <c r="J307" t="str">
+        <v>Design-focused sibling to the Anoka Manufacturing Engineering Co-op.</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B308" t="str">
+        <v>Engineering Co-Op Opportunities</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Mechanical / Electrical / Industrial Engineering</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Spring 2027 (body text states 'Mechanical, Electrical, or Industrial Engineering Co-Op (Spring 2027)' verbatim)</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Richland, MS</v>
+      </c>
+      <c r="F308">
+        <v>1257</v>
+      </c>
+      <c r="G308" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H308" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Richland-MS-US/Engineering-Co-Op-Opportunities_R23659</v>
+      </c>
+      <c r="I308" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, explicit 'Spring 2027' wording confirmed in body text.</v>
+      </c>
+      <c r="J308" t="str">
+        <v>A general-opportunities req covering multiple disciplines at the Richland, MS site.</v>
       </c>
     </row>
   </sheetData>
@@ -11860,14 +12212,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M297"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M308"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C597"/>
+  <dimension ref="A1:C620"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -18432,9 +18784,262 @@
         <v>2026-10-02 (later same day): re-fetched directly via ADI's own Workday CXS API — still live (canApply true) and still internally contradictory on season ('running from June through December' in the role description vs. 'Available to work full-time, on-site from January through June' in Qualifications, no year stated either way). Also checked for a broader Spring 2027 co-op slate at analog.com — none found yet; R266691 remains the only Analog Devices posting live. Unchanged from the long-standing exclusion; still excluded.</v>
       </c>
     </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>Bose Corporation (Framingham, MA)</v>
+      </c>
+      <c r="B598" t="str">
+        <v>'Mechanical Engineer Co-op, Concept Prototyping', req R26422 — resolves the prior-run's repeated HTTP 500 block</v>
+      </c>
+      <c r="C598" t="str">
+        <v>2026-10-02 (later same day): root-caused the repeated 500s — prior attempts used the wrong Workday tenant subdomain (wd1, which redirects to a Workday maintenance page for this tenant). The correct tenant is wd503: https://boseallaboutme.wd503.myworkdayjobs.com/en-US/Bose_Careers/job/Mechanical-Engineer-Co-op--Concept-Prototyping_R26422 — fetched directly (HTTP 200), and the page's own embedded bootstrap JSON explicitly states postingAvailable: false. Confirmed CLOSED, not merely unconfirmed. Distinct from the already-logged older req R25833 at the same company. Not added.</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>Agility Robotics</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Possible 'Mechanical Engineer Intern, Spring 2027', Mountain View, CA — re-check of an aggregator-only lead</v>
+      </c>
+      <c r="C599" t="str">
+        <v>2026-10-02 (later same day): identified Agility's real ATS (Greenhouse, board slug agilityrobotics) and queried its live jobs API directly (HTTP 200) — all 78 current company-wide postings fetched. Zero postings contain 'Intern' or 'Co-op' in the title, and zero are located in Mountain View, CA (only Fremont CA, Pittsburgh PA, Salem OR, and a few other sites appear); the 5 live Mechanical-discipline reqs are senior/staff full-time roles. The original lead (aggregator-only, itself 403-blocked on direct fetch) cannot be corroborated on the employer's own live board. Treated as unconfirmed/likely stale. Not added.</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>Lutron Electronics</v>
+      </c>
+      <c r="B600" t="str">
+        <v>'Mechanical Engineering Co-Op', Boston, MA (1 Beacon St) — aggregator-sourced lead</v>
+      </c>
+      <c r="C600" t="str">
+        <v>2026-10-02: confirmed real Boston office via the company's own Jibe-powered careers API (careers.lutron.com/api/jobs), but the aggregator-sourced Boston co-op lead turned out to be a stale Spring 2026 (already-past) posting, not Spring 2027. Zero live Mechanical Engineering Co-Op postings for Spring 2027 exist company-wide; the only current intern-type posting anywhere is a Summer 2027 Manufacturing Engineering Intern in Ashland, VA (wrong season). Not added.</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>Field AI</v>
+      </c>
+      <c r="B601" t="str">
+        <v>'Mechanical Engineer, Robotics Hardware — Part-Time Internship' (Boston-tagged on an aggregator)</v>
+      </c>
+      <c r="C601" t="str">
+        <v>2026-10-02: queried the company's live Lever API directly (api.lever.co/v0/postings/field-ai, 97 postings fetched) — the only matching title is a full-time 'Mechanical Engineer, Robotics Hardware' role based in Irvine, CA, not an internship and not Boston. The aggregator lead is stale/unverifiable on the primary source. Not added.</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>United Launch Alliance (ULA)</v>
+      </c>
+      <c r="B602" t="str">
+        <v>Mechanical Engineering internship search</v>
+      </c>
+      <c r="C602" t="str">
+        <v>2026-10-02: only a Summer 2027 Mechanical Engineering Internship found; no Spring 2027 posting located. Wrong season.</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>Rolls-Royce North America (Indianapolis, IN)</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Co-op program (Mechanical/Aerospace/Systems/Materials)</v>
+      </c>
+      <c r="C603" t="str">
+        <v>2026-10-02: confirmed the co-op program exists for these majors, but the next application cycle doesn't open until late January/early February 2027 — no live Spring 2027 requisition currently posted. Not added; worth a re-check once the cycle opens.</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>SKF USA</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Mechanical/manufacturing engineering co-op/intern search</v>
+      </c>
+      <c r="C604" t="str">
+        <v>2026-10-02: no company-specific ATS posting found for any 2027 co-op/intern; only a generic program description page. Not added.</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>Ingersoll Rand</v>
+      </c>
+      <c r="B605" t="str">
+        <v>Manufacturing/Mechanical Engineering Intern (Quincy IL / Springfield MO / Bentleyville PA)</v>
+      </c>
+      <c r="C605" t="str">
+        <v>2026-10-02: only Summer 2027 postings found at all three sites. Wrong season.</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>Nordson Corporation</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Mechanical Engineering Intern (Ohio; East Providence, RI)</v>
+      </c>
+      <c r="C606" t="str">
+        <v>2026-10-02: current live postings don't state a 2027 season in the available sources; no Spring 2027-dated posting confirmed. Not added.</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>The Nuclear Company (Columbia, SC)</v>
+      </c>
+      <c r="B607" t="str">
+        <v>'TNC Nuclear Interns 2027'</v>
+      </c>
+      <c r="C607" t="str">
+        <v>2026-10-02: confirmed real but explicitly Summer 2027 (May/June–Aug/Sept). Wrong season.</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>Vestas</v>
+      </c>
+      <c r="B608" t="str">
+        <v>Mechanical engineering intern search</v>
+      </c>
+      <c r="C608" t="str">
+        <v>2026-10-02: no mechanical engineering intern posting found for any 2027 season; only a Service Technician Intern (MN) referenced. Not added.</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>Pentair</v>
+      </c>
+      <c r="B609" t="str">
+        <v>Engineering Leadership Development Internship Program</v>
+      </c>
+      <c r="C609" t="str">
+        <v>2026-10-02: explicitly Summer 2027. Wrong season.</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="str">
+        <v>Danfoss</v>
+      </c>
+      <c r="B610" t="str">
+        <v>Mechanical Engineering Internship (Product Development)</v>
+      </c>
+      <c r="C610" t="str">
+        <v>2026-10-02: only a Summer 2027 posting found. Wrong season.</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="str">
+        <v>Otis Elevator</v>
+      </c>
+      <c r="B611" t="str">
+        <v>2027 internship program</v>
+      </c>
+      <c r="C611" t="str">
+        <v>2026-10-02: confirmed real, but explicitly starts June 2027 (Summer). Wrong season.</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="str">
+        <v>Hamilton Company (Reno, NV)</v>
+      </c>
+      <c r="B612" t="str">
+        <v>Mechanical Engineering Intern</v>
+      </c>
+      <c r="C612" t="str">
+        <v>2026-10-02: posting is ASAP-start/rolling with no stated 2027 season, and is explicitly restricted to University of Nevada, Reno enrolled students. Excluded on season-ambiguity and eligibility-restriction grounds.</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="str">
+        <v>Agilent Technologies</v>
+      </c>
+      <c r="B613" t="str">
+        <v>Mechanical co-op/intern search</v>
+      </c>
+      <c r="C613" t="str">
+        <v>2026-10-02: no company-specific Spring 2027 mechanical co-op posting locatable; only a generic year-round program description. Not added.</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="str">
+        <v>Snap-on</v>
+      </c>
+      <c r="B614" t="str">
+        <v>Manufacturing engineering co-op/intern search</v>
+      </c>
+      <c r="C614" t="str">
+        <v>2026-10-02: no Spring 2027 (or any dated) manufacturing engineering co-op/intern posting found. Not added.</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="str">
+        <v>Gecko Robotics</v>
+      </c>
+      <c r="B615" t="str">
+        <v>Mechanical engineering internship search</v>
+      </c>
+      <c r="C615" t="str">
+        <v>2026-10-02: only Summer 2027 postings found company-wide (Test &amp; Reliability Engineering Intern – Pittsburgh; AI/ML Intern – NY); no current Mechanical Engineering posting of any season. Not added.</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="str">
+        <v>Oklo Inc. / Kairos Power</v>
+      </c>
+      <c r="B616" t="str">
+        <v>Mechanical Engineering internship pipelines</v>
+      </c>
+      <c r="C616" t="str">
+        <v>2026-10-02: both have Mechanical Engineering internship pipelines but both are explicitly labeled Summer 2027. Wrong season.</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="str">
+        <v>Blue Canyon Technologies</v>
+      </c>
+      <c r="B617" t="str">
+        <v>Internship search</v>
+      </c>
+      <c r="C617" t="str">
+        <v>2026-10-02: only past Summer internship postings found; no live 2027 req of any season. Not added.</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="str">
+        <v>Corning Incorporated (glass/materials — distinct from the already-tracked Owens Corning)</v>
+      </c>
+      <c r="B618" t="str">
+        <v>Rolling internship program</v>
+      </c>
+      <c r="C618" t="str">
+        <v>2026-10-02: program confirmed generally, but the only dated postings found are Summer 2027; no Spring 2027-specific req located. Not added.</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="str">
+        <v>Inkbit (Medford, MA) / Carbon (Carbon3D)</v>
+      </c>
+      <c r="B619" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C619" t="str">
+        <v>2026-10-02: no current internship/co-op postings of any kind found for either company. Not added.</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B620" t="str">
+        <v>'Engineering Lab Co-Op' — search-listing said Jan-Aug 2027</v>
+      </c>
+      <c r="C620" t="str">
+        <v>2026-10-02: the live page's own title contradicts the search-listing season — it actually reads 'Lab Internship (June - August 2027)'. Title/listing-vs-body season contradiction, same pattern as the earlier Reframe Systems/Analog Devices precedents. Excluded rather than reported as verified Winter/Spring.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C597"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C620"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 11 checked-excluded (2026-10-03 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017FPgMmpHUkQtJwiKjj75jY
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M308"/>
+  <dimension ref="A1:M311"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11739,6 +11739,102 @@
       </c>
       <c r="J308" t="str">
         <v>A general-opportunities req covering multiple disciplines at the Richland, MS site.</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
+      </c>
+      <c r="B309" t="str">
+        <v>Transducer Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Manufacturing / Mechanical / Industrial Engineering</v>
+      </c>
+      <c r="D309" t="str">
+        <v>January to June 2027 (per posting text)</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Waltham, MA</v>
+      </c>
+      <c r="F309">
+        <v>10</v>
+      </c>
+      <c r="G309" t="str">
+        <v>$25.00-$28.00/hr</v>
+      </c>
+      <c r="H309" t="str">
+        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015874986-transducer-manufacturing-engineering-co-op</v>
+      </c>
+      <c r="I309" t="str">
+        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116547, posted 2026-10-02.</v>
+      </c>
+      <c r="J309" t="str">
+        <v>Evident/Wabtec Inspection Technologies division. New employer for the tracker. Boston-area.</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
+      </c>
+      <c r="B310" t="str">
+        <v>Co-Op, Test Engineer - Transducer</v>
+      </c>
+      <c r="C310" t="str">
+        <v>Manufacturing / Test Engineering</v>
+      </c>
+      <c r="D310" t="str">
+        <v>January - June 2027 (stated in title)</v>
+      </c>
+      <c r="E310" t="str">
+        <v>State College, PA</v>
+      </c>
+      <c r="F310">
+        <v>390</v>
+      </c>
+      <c r="G310" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H310" t="str">
+        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015763566-co-op-test-engineer-transducer-january-june-2027-</v>
+      </c>
+      <c r="I310" t="str">
+        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116563, posted 2026-09-29.</v>
+      </c>
+      <c r="J310" t="str">
+        <v>Sibling req to the Waltham, MA transducer co-op above; hands-on fixture/test-system work.</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B311" t="str">
+        <v>Electrical/Controls Engineering Co-Op</v>
+      </c>
+      <c r="C311" t="str">
+        <v>Controls Engineering</v>
+      </c>
+      <c r="D311" t="str">
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Anoka, MN</v>
+      </c>
+      <c r="F311">
+        <v>1127</v>
+      </c>
+      <c r="G311" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H311" t="str">
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Electrical-Controls-Engineering-Co-Op--January---August-2027-_R23894</v>
+      </c>
+      <c r="I311" t="str">
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, req R23894, posted 2026-10-02/03.</v>
+      </c>
+      <c r="J311" t="str">
+        <v>Controls-discipline sibling to nVent's other already-tracked Jan-start Anoka, MN co-ops.</v>
       </c>
     </row>
   </sheetData>
@@ -12212,14 +12308,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M308"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M311"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C620"/>
+  <dimension ref="A1:C631"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -19037,9 +19133,130 @@
         <v>2026-10-02: the live page's own title contradicts the search-listing season — it actually reads 'Lab Internship (June - August 2027)'. Title/listing-vs-body season contradiction, same pattern as the earlier Reframe Systems/Analog Devices precedents. Excluded rather than reported as verified Winter/Spring.</v>
       </c>
     </row>
+    <row r="621">
+      <c r="A621" t="str">
+        <v>Axiom Space (Houston, TX)</v>
+      </c>
+      <c r="B621" t="str">
+        <v>'Spring 2027 Mechanical/Aerospace Engineering Intern' (aggregator-sourced lead)</v>
+      </c>
+      <c r="C621" t="str">
+        <v>2026-10-03 ~01:00 UTC: queried Axiom Space's own Workday CXS API directly with facet breakdown — workerSubType facet shows only 'Regular', zero Intern/Co-op reqs exist company-wide right now. Lead could not be substantiated on the live board. Not added.</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="str">
+        <v>Rockwell Automation</v>
+      </c>
+      <c r="B622" t="str">
+        <v>'Co-op, Mechanical Engineering (Spring 2027), Chelmsford, MA' (aggregator-sourced lead)</v>
+      </c>
+      <c r="C622" t="str">
+        <v>2026-10-03 ~01:00 UTC: queried Rockwell's own Workday CXS API directly (full Mechanical Engineering facet pull, 131 matches reviewed) — no such US req exists; the only live Mechanical/Manufacturing co-op company-wide is in Cambridge, Ontario, Canada (non-US, excluded on location). The Chelmsford MA aggregator lead appears stale/mis-indexed.</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="str">
+        <v>A.O. Smith (Milwaukee, WI)</v>
+      </c>
+      <c r="B623" t="str">
+        <v>Water Treatment Engineering Co-op; sibling Materials/Thermal/Electronics/Sensors Engineering Co-ops</v>
+      </c>
+      <c r="C623" t="str">
+        <v>2026-10-03 ~01:00 UTC: Water Treatment Engineering Co-op confirmed 'this position has been filled' directly on jobs.aosmith.com. Sibling co-op listings exist but state no season/year — not independently verified, not added.</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="str">
+        <v>Flint Hills Resources (Koch Industries, Rosemount, MN)</v>
+      </c>
+      <c r="B624" t="str">
+        <v>Mechanical Engineering Co-op, $32/hr</v>
+      </c>
+      <c r="C624" t="str">
+        <v>2026-10-03 ~01:00 UTC: confirmed live but structured as a part-time (10-20 hrs/week) ongoing role tied to 'anticipated Spring 2027 graduation date', not a discrete full-time Spring-2027-term co-op — fails the season/structure bar.</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="str">
+        <v>Wabtec</v>
+      </c>
+      <c r="B625" t="str">
+        <v>'Full-Time Spring Engineering Co-op' (Erie/Grove City, PA), req R0115355</v>
+      </c>
+      <c r="C625" t="str">
+        <v>2026-10-03 ~01:00 UTC: confirmed active:true via Wabtec's own SmartRecruiters API, broad in-discipline engineering disciplines, 30-week Jan-Aug program, posted 2026-08-28 — but no explicit calendar year appears anywhere in the posting body (grepped for '20xx', zero hits). Almost certainly the Jan 2027 cohort but excluded per the strict season-stated-in-posting bar rather than inferred.</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="str">
+        <v>Donaldson Company; SPX Technologies; Brooks Automation (Chelmsford, MA); Medrobotics (Raynham, MA); Activ Surgical; Inkbit (Medford, MA); Hyperfine</v>
+      </c>
+      <c r="B626" t="str">
+        <v>Internship/co-op search</v>
+      </c>
+      <c r="C626" t="str">
+        <v>2026-10-03 ~01:00 UTC: no live, dated Winter 2026/Spring 2027 mechanical/manufacturing co-op posting located for any of these companies this run.</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="str">
+        <v>RTX (Collins Aerospace, Cedar Rapids, IA)</v>
+      </c>
+      <c r="B627" t="str">
+        <v>'Industrial Engineering Co-Op (Spring/Summer 2027)', reqs 01870645 and 01871431</v>
+      </c>
+      <c r="C627" t="str">
+        <v>2026-10-03 ~01:00 UTC: both are single merged 'Spring/Summer 2027' co-op sessions with no distinct Spring-only dated sub-range confirmable (RTX's own Workday CXS API returns errorCode S22/403 on direct fetch; only aggregator-mirror title/location/pay corroborated) — same treatment as the prior Advanced Manufacturing Engineering Co-Op (req 01874253) and other RTX Spring/Summer-titled precedents. Not added.</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="str">
+        <v>RTX (Collins Aerospace, Rockford, IL)</v>
+      </c>
+      <c r="B628" t="str">
+        <v>'Manufacturing Engineering Ops Co-Op (Spring/Summer 2027)', req 01876912</v>
+      </c>
+      <c r="C628" t="str">
+        <v>2026-10-03 ~01:00 UTC: same merged-term, Workday-403-blocked treatment as the Cedar Rapids Industrial Engineering Co-Op reqs above. Not added.</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="str">
+        <v>Draper Laboratory (Lowell, MA)</v>
+      </c>
+      <c r="B629" t="str">
+        <v>'Co-Op Student Engineering', req JR002974</v>
+      </c>
+      <c r="C629" t="str">
+        <v>2026-10-03 ~01:00 UTC: direct Workday CXS fetch confirms canApply:true but endDate:None and no season/year stated anywhere in the body ('6 month period' with flexible timing). Full description reveals the role sits in Draper's Software Engineering Division (low-level software for real-time embedded systems) — discipline mismatch independent of the season problem. Excluded on both grounds.</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="str">
+        <v>nVent (Anoka, MN)</v>
+      </c>
+      <c r="B630" t="str">
+        <v>'Engineering Lab Co-Op (Jan - August 2027)', req R23537</v>
+      </c>
+      <c r="C630" t="str">
+        <v>2026-10-03 ~01:00 UTC: right season window, canApply:true, but discipline is generic R&amp;D Lab Co-Op / Lab Test Engineer support work, not a clean match to Hamza's target disciplines. Not added; his own call if reconsidered.</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="str">
+        <v>Graco Inc. (Dexter, MI)</v>
+      </c>
+      <c r="B631" t="str">
+        <v>'Application Engineering Intern', req R0023513</v>
+      </c>
+      <c r="C631" t="str">
+        <v>2026-10-03 ~01:00 UTC: discipline fits well (body explicitly wants Mechanical/Industrial Engineering majors for MFG co-op work) and canApply:true, but endDate:None and zero season/year stated anywhere in the posting — fails the explicit-season verification bar, consistent with how other no-season Graco/Hologic-style postings have been treated.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C620"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C631"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 8 new postings, 9 checked-excluded (2026-10-03 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XgRNZzN7eJxcv3jg9QqG4F
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M311"/>
+  <dimension ref="A1:M319"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11835,6 +11835,262 @@
       </c>
       <c r="J311" t="str">
         <v>Controls-discipline sibling to nVent's other already-tracked Jan-start Anoka, MN co-ops.</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>Schaeffler</v>
+      </c>
+      <c r="B312" t="str">
+        <v>Co-op Mechanical Engineering</v>
+      </c>
+      <c r="C312" t="str">
+        <v>Mechanical Engineering (Engine/Chassis R&amp;D)</v>
+      </c>
+      <c r="D312" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Troy, MI</v>
+      </c>
+      <c r="F312">
+        <v>720</v>
+      </c>
+      <c r="G312" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H312" t="str">
+        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechanical-Engineering-Winter-2027-MI-48083/1425401433/</v>
+      </c>
+      <c r="I312" t="str">
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present, no closed/expired message.</v>
+      </c>
+      <c r="J312" t="str">
+        <v>New employer for the tracker. Not Boston-area.</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>Schaeffler</v>
+      </c>
+      <c r="B313" t="str">
+        <v>Co-op Mechatronics Engineering</v>
+      </c>
+      <c r="C313" t="str">
+        <v>Mechatronics (Mechanical + Controls/Systems Integration)</v>
+      </c>
+      <c r="D313" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Troy, MI</v>
+      </c>
+      <c r="F313">
+        <v>720</v>
+      </c>
+      <c r="G313" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H313" t="str">
+        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechatronics-Engineering-Winter-2027-MI-48083/1425394833/</v>
+      </c>
+      <c r="I313" t="str">
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present.</v>
+      </c>
+      <c r="J313" t="str">
+        <v>Sibling req to the Mechanical Engineering co-op above, same site/season.</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>SSOE Group</v>
+      </c>
+      <c r="B314" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C314" t="str">
+        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Toledo, OH</v>
+      </c>
+      <c r="F314">
+        <v>700</v>
+      </c>
+      <c r="G314" t="str">
+        <v>Not independently confirmed this run (an older/cached listing cited $19-23/hr for a prior cycle)</v>
+      </c>
+      <c r="H314" t="str">
+        <v>https://careers-ssoe.icims.com/jobs/3885/mechanical-engineering-co-op---spring-2027/job</v>
+      </c>
+      <c r="I314" t="str">
+        <v>Partial — 2026-10-03 ~07:00 UTC: confirmed via direct fetch of careers-ssoe.icims.com's own search-results page (HTTP 200); job title/ID/location appear in the server-rendered HTML confirming the listing is currently live, but the individual job-detail page is JS-rendered and could not be independently fetched to confirm full description, pay, or Apply button.</v>
+      </c>
+      <c r="J314" t="str">
+        <v>New employer for the tracker (architecture/engineering design firm, MEP/HVAC discipline — borderline fit, Hamza's call). Job ID 3885.</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>SSOE Group</v>
+      </c>
+      <c r="B315" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C315" t="str">
+        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Nashville, TN</v>
+      </c>
+      <c r="F315">
+        <v>1090</v>
+      </c>
+      <c r="G315" t="str">
+        <v>Not independently confirmed this run</v>
+      </c>
+      <c r="H315" t="str">
+        <v>https://careers-ssoe.icims.com/jobs/3886/mechanical-engineering-co-op---spring-2027/job</v>
+      </c>
+      <c r="I315" t="str">
+        <v>Partial — 2026-10-03 ~07:00 UTC: same verification method as the Toledo, OH sibling req above — confirmed live via direct ATS search-results fetch (HTTP 200), job-detail page JS-rendered/unconfirmed.</v>
+      </c>
+      <c r="J315" t="str">
+        <v>Sibling req to the Toledo, OH SSOE Mechanical Engineering Co-op. Job ID 3886. MEP/HVAC discipline — borderline fit.</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>SSOE Group</v>
+      </c>
+      <c r="B316" t="str">
+        <v>Structural Engineering Co-op</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E316" t="str">
+        <v>Toledo, OH</v>
+      </c>
+      <c r="F316">
+        <v>700</v>
+      </c>
+      <c r="G316" t="str">
+        <v>Not independently confirmed this run</v>
+      </c>
+      <c r="H316" t="str">
+        <v>https://careers-ssoe.icims.com/jobs/3881/structural-engineering-co-op---spring-2027/job</v>
+      </c>
+      <c r="I316" t="str">
+        <v>Partial — 2026-10-03 ~07:00 UTC: same verification method as the SSOE Mechanical Engineering reqs above — confirmed live via direct ATS search-results fetch (HTTP 200), job-detail page JS-rendered/unconfirmed.</v>
+      </c>
+      <c r="J316" t="str">
+        <v>Job ID 3881. Structural Engineering is within Hamza's target discipline list.</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>Sanofi</v>
+      </c>
+      <c r="B317" t="str">
+        <v>2027 Spring Co-op Opportunities</v>
+      </c>
+      <c r="C317" t="str">
+        <v>Multi-track (Material Sciences, Process Chemistry, Laboratory Automation — process/materials-engineering-adjacent)</v>
+      </c>
+      <c r="D317" t="str">
+        <v>6-month duration starting January 2027</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Cambridge, MA</v>
+      </c>
+      <c r="F317">
+        <v>3</v>
+      </c>
+      <c r="G317" t="str">
+        <v>$27-$60/hr (stated on posting, varies by role/experience)</v>
+      </c>
+      <c r="H317" t="str">
+        <v>https://jobs.sanofi.com/en/job/cambridge/2027-spring-co-op-opportunities-cambridge-ma/2649/41259853312</v>
+      </c>
+      <c r="I317" t="str">
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.sanofi.com (employer's own career site), HTTP 200, 'Apply now' button present, application deadline Nov 13, 2026 stated on posting.</v>
+      </c>
+      <c r="J317" t="str">
+        <v>Right in the Boston metro. Sanofi is already tracked for Framingham, MA and Swiftwater, PA — this Cambridge req is a distinct posting/location. Multi-track req; Material Sciences/Process Chemistry/Lab Automation tracks are the closest fit to Hamza's target disciplines. A sibling Waltham, MA posting exists but is dominated by life-sciences tracks — excluded, see `checked`.</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B318" t="str">
+        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Lexington, MA</v>
+      </c>
+      <c r="F318">
+        <v>12</v>
+      </c>
+      <c r="G318" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H318" t="str">
+        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
+      </c>
+      <c r="I318" t="str">
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via careers.ll.mit.edu (employer's own SuccessFactors career site), HTTP 200, 'Apply now' link present, posted 2026-09-28.</v>
+      </c>
+      <c r="J318" t="str">
+        <v>Right in the Boston metro. Distinct from the already-tracked Microfabrication Industrial Eng Co-Op (Jan-Aug 2027) reqs — this is a separate Group 07-71 Mechanical Engineering req.</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>Symbotic</v>
+      </c>
+      <c r="B319" t="str">
+        <v>Co-op - Hardware Engineer</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Mechanical / Electro-Mechanical Engineering</v>
+      </c>
+      <c r="D319" t="str">
+        <v>Spring (January-May 2027)</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Wilmington, MA (ITC site)</v>
+      </c>
+      <c r="F319">
+        <v>17</v>
+      </c>
+      <c r="G319" t="str">
+        <v>$29.00-$40.00/hr</v>
+      </c>
+      <c r="H319" t="str">
+        <v>https://www.symbotic.com/careers/jobs/R7976/</v>
+      </c>
+      <c r="I319" t="str">
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via symbotic.com/careers (employer's own career site), season and pay range stated explicitly in body text, active 'Apply Now' button present (routes to Workday; not independently re-tested end-to-end due to a concurrent Workday platform-wide maintenance outage at check time).</v>
+      </c>
+      <c r="J319" t="str">
+        <v>Right in the Boston metro. CAD design/electro-mechanical debugging/SolidWorks/GD&amp;T/robotics work. Req R7976, distinct from the already-excluded 'Intern - Hardware Engineer' (R5394).</v>
       </c>
     </row>
   </sheetData>
@@ -12308,14 +12564,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M311"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M319"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C631"/>
+  <dimension ref="A1:C640"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -19254,9 +19510,108 @@
         <v>2026-10-03 ~01:00 UTC: discipline fits well (body explicitly wants Mechanical/Industrial Engineering majors for MFG co-op work) and canApply:true, but endDate:None and zero season/year stated anywhere in the posting — fails the explicit-season verification bar, consistent with how other no-season Graco/Hologic-style postings have been treated.</v>
       </c>
     </row>
+    <row r="632">
+      <c r="A632" t="str">
+        <v>Sanofi (Waltham, MA)</v>
+      </c>
+      <c r="B632" t="str">
+        <v>'2027 Spring Co-Op Opportunities, Waltham, MA'</v>
+      </c>
+      <c r="C632" t="str">
+        <v>2026-10-03 ~07:00 UTC: confirmed live/open via direct fetch of jobs.sanofi.com, but the posting is a single combined req dominated by life-sciences tracks (Purification Process Development, Analytical Development, Molecular Biology); only 'Upstream MSAT'/'Site Operations' sub-tracks are process/manufacturing-engineering-adjacent. Discipline fit too weak/diffuse to add as a clean match — Hamza's call if reconsidered. Distinct from the qualifying Cambridge, MA sibling req added to `rows`.</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="str">
+        <v>Schaeffler (Troy, MI)</v>
+      </c>
+      <c r="B633" t="str">
+        <v>'Co-Op - Humanoid Robotics (Mechanical Engineering) - 2027'</v>
+      </c>
+      <c r="C633" t="str">
+        <v>2026-10-03 ~07:00 UTC: confirmed live via direct fetch of jobs.schaeffler.com, 'Apply now' present, but the body text only states '2027' with no Winter/Spring/Summer wording — season unconfirmed from the posting itself. Not added; worth a re-check in case the listing is updated with explicit season language.</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="str">
+        <v>Bristol Myers Squibb (Devens, MA)</v>
+      </c>
+      <c r="B634" t="str">
+        <v>'Devens Spring Co-op Program (STEM)', req R1606920</v>
+      </c>
+      <c r="C634" t="str">
+        <v>2026-10-03 ~07:00 UTC: found via a mirror site (zapply.jobs) with a specific req ID, but BMS's own Workday instance was in a live platform-wide maintenance outage at check time (two fetch attempts ~20s apart both returned Workday's own maintenance page) — could not independently verify live status. Discipline also appears to be a broad STEM/Operational-Excellence pool rather than specifically mechanical. Not added; worth a re-check once Workday's outage clears.</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="str">
+        <v>CardioFocus (Marlborough, MA)</v>
+      </c>
+      <c r="B635" t="str">
+        <v>'Hardware R&amp;D Engineering Co-Op' (aggregator-sourced title)</v>
+      </c>
+      <c r="C635" t="str">
+        <v>2026-10-03 ~07:00 UTC: fetched the company's own live careers page directly — only 4 open roles listed (HR Specialist/Manager, NPI Manager, R&amp;D Catheter Technician, Catheter Process Engineer), no co-op posting present. Aggregator lead appears stale/closed. Not added.</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="str">
+        <v>Infrasynk Engineering</v>
+      </c>
+      <c r="B636" t="str">
+        <v>'Vehicle Integration &amp; Test Engineer Intern', Seattle, WA</v>
+      </c>
+      <c r="C636" t="str">
+        <v>2026-10-03 ~07:00 UTC: LinkedIn posting explicitly confirms a Summer start date. Wrong season.</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="str">
+        <v>GlobalFoundries</v>
+      </c>
+      <c r="B637" t="str">
+        <v>'Facility Engineering, Automation Intern (Jan-Jun 2027)'</v>
+      </c>
+      <c r="C637" t="str">
+        <v>2026-10-03 ~07:00 UTC: confirmed location is Woodlands, Singapore, not a US site — fails Hamza's US-only requirement. GlobalFoundries' own Workday CXS API is bot-protected (repeated HTTP 303 redirects to a challenge/maintenance page even with browser-like headers) — could not independently check for a separate US-based req this run. Not added; known blocker for a future run.</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="str">
+        <v>Toyota Motor Manufacturing (various US plants)</v>
+      </c>
+      <c r="B638" t="str">
+        <v>General 'STEM Co-op &amp; Internship' program page</v>
+      </c>
+      <c r="C638" t="str">
+        <v>2026-10-03 ~07:00 UTC: Toyota's own student careers page confirms co-ops run 'throughout spring, summer and fall' in Production/Manufacturing Engineering, but the page is a program description with no individual job requisitions visible — could not locate or verify a specific live Spring 2027 req/link. Inconclusive, not added.</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="str">
+        <v>Graco Inc. (Anoka, MN)</v>
+      </c>
+      <c r="B639" t="str">
+        <v>'Manufacturing Engineering Co-op (May - December 2027)', req R0023613</v>
+      </c>
+      <c r="C639" t="str">
+        <v>2026-10-03 ~07:00 UTC: new req found during the nVent/Graco liveness re-sweep, confirmed canApply:true via direct Workday CXS fetch, but explicitly 'May - December 2027' — wrong season (not Winter 2026/Spring 2027). Not added.</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="str">
+        <v>Symbotic (Wilmington, MA)</v>
+      </c>
+      <c r="B640" t="str">
+        <v>'Intern - Industrial Controls', req R7973; 'Co-op - Software Engineer', req R8111</v>
+      </c>
+      <c r="C640" t="str">
+        <v>2026-10-03 ~07:00 UTC: found during the same sweep that surfaced the qualifying Co-op - Hardware Engineer (R7976, added to `rows`). R7973 is explicitly 'Summer (May-Aug 2027)' — wrong season. R8111 is a software engineering co-op — discipline mismatch. Neither added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C631"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C640"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new postings, 18 checked-excluded (2026-10-03 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EpiftZQ8PumTqXAJrms1cs
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M319"/>
+  <dimension ref="A1:M320"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -12091,6 +12091,38 @@
       </c>
       <c r="J319" t="str">
         <v>Right in the Boston metro. CAD design/electro-mechanical debugging/SolidWorks/GD&amp;T/robotics work. Req R7976, distinct from the already-excluded 'Intern - Hardware Engineer' (R5394).</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>Analogic Corporation</v>
+      </c>
+      <c r="B320" t="str">
+        <v>Manufacturing Engineering Co-Op</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Spring 2027 Co-Op Program</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Salem, NH</v>
+      </c>
+      <c r="F320">
+        <v>28</v>
+      </c>
+      <c r="G320" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H320" t="str">
+        <v>https://recruiting.ultipro.com/ANA1003ALOG/JobBoard/a4de26ba-aa2d-4502-9d0f-577ea07dc7ca/OpportunityDetail?opportunityId=a25687db-ac1a-46ea-90a4-97fe04c715c6</v>
+      </c>
+      <c r="I320" t="str">
+        <v>Partial — 2026-10-03 ~13:00 UTC: confirmed live via a direct query of Analogic's own UltiPro ATS JSON search API (returned in the active-search result set, RequisitionNumber MANUF002804, PostedDate 2026-09-21, 'Spring 2027 Co-Op Program' stated as the literal first line of the body description). The human-facing detail page is a React SPA that did not render statically, so pay and full requirements could not be independently confirmed beyond the API's own fields.</v>
+      </c>
+      <c r="J320" t="str">
+        <v>Close to Boston (~28 mi). Distinct from Analogic's other open reqs at the same Salem, NH site: 'Engineering Co-Op' (ENGIN002794, security-imaging, no season stated) and 'Hardware/Software Engineering Co-Op' (COOPS002797, RF/electrical) — both excluded, see checked.</v>
       </c>
     </row>
   </sheetData>
@@ -12564,14 +12596,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M319"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M320"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C640"/>
+  <dimension ref="A1:C655"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -19609,9 +19641,174 @@
         <v>2026-10-03 ~07:00 UTC: found during the same sweep that surfaced the qualifying Co-op - Hardware Engineer (R7976, added to `rows`). R7973 is explicitly 'Summer (May-Aug 2027)' — wrong season. R8111 is a software engineering co-op — discipline mismatch. Neither added.</v>
       </c>
     </row>
+    <row r="641">
+      <c r="A641" t="str">
+        <v>Analogic Corporation (Salem, NH)</v>
+      </c>
+      <c r="B641" t="str">
+        <v>'Engineering Co-Op', req ENGIN002794; 'Hardware/Software Engineering Co-Op', req COOPS002797</v>
+      </c>
+      <c r="C641" t="str">
+        <v>2026-10-03 ~13:00 UTC: both confirmed open via Analogic's own UltiPro ATS API. ENGIN002794 (Security Imaging team) states no season anywhere in its description. COOPS002797 is RF-amplifier hardware/software work — discipline mismatch (electrical/software). Neither added; distinct from the qualifying Manufacturing Engineering Co-Op (MANUF002804) added to `rows`.</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="str">
+        <v>Realta Fusion (Madison, WI)</v>
+      </c>
+      <c r="B642" t="str">
+        <v>'Engineering Co-op' (Mechanical Design &amp; Fabrication track)</v>
+      </c>
+      <c r="C642" t="str">
+        <v>2026-10-03 ~13:00 UTC: posting states only 'fall or spring' generically with no year — fails the explicit-season verification bar. Not added.</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="str">
+        <v>Pacific Fusion (San Leandro/Fremont, CA; Los Lunas, NM)</v>
+      </c>
+      <c r="B643" t="str">
+        <v>Mechanical/Manufacturing internships</v>
+      </c>
+      <c r="C643" t="str">
+        <v>2026-10-03 ~13:00 UTC: explicitly Summer 2027 — wrong season.</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="str">
+        <v>Saronic Technologies (Austin, TX)</v>
+      </c>
+      <c r="B644" t="str">
+        <v>Mechanical/Manufacturing Engineer Intern</v>
+      </c>
+      <c r="C644" t="str">
+        <v>2026-10-03 ~13:00 UTC: explicitly Summer 2027 — wrong season.</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="str">
+        <v>Neros Technologies (Torrance/El Segundo, CA)</v>
+      </c>
+      <c r="B645" t="str">
+        <v>General mechanical intern/co-op search</v>
+      </c>
+      <c r="C645" t="str">
+        <v>2026-10-03 ~13:00 UTC: no dated Winter 2026/Spring 2027 posting located.</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="str">
+        <v>Gecko Robotics / Philips</v>
+      </c>
+      <c r="B646" t="str">
+        <v>Aggregator-sourced 'Manufacturing Engineering Co-op, Murrysville PA, Jan-June 2027' lead</v>
+      </c>
+      <c r="C646" t="str">
+        <v>2026-10-03 ~13:00 UTC: traced to a mislabeled aggregator entry — actually a Philips req (job 580754), which now 404s. Direct query of Philips' own live careers search confirms zero open co-op/internship postings company-wide, consistent with the existing Philips exclusion note. Not Gecko Robotics at all; not added.</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="str">
+        <v>Epirus (Torrance, CA)</v>
+      </c>
+      <c r="B647" t="str">
+        <v>Manufacturing/Mechanical Engineering Intern</v>
+      </c>
+      <c r="C647" t="str">
+        <v>2026-10-03 ~13:00 UTC: postings reference a graduation-eligibility window (12/2026-12/2027) but no explicit Winter/Spring season statement was retrievable — unresolved, not added.</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="str">
+        <v>Smith &amp; Nephew</v>
+      </c>
+      <c r="B648" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C648" t="str">
+        <v>2026-10-03 ~13:00 UTC: no co-op/internship postings of any kind found.</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="str">
+        <v>Hexagon Manufacturing Intelligence</v>
+      </c>
+      <c r="B649" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C649" t="str">
+        <v>2026-10-03 ~13:00 UTC: only a Summer 2027 Application Engineer Intern program found; no Spring 2027 mechanical/manufacturing posting located.</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B650" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C650" t="str">
+        <v>2026-10-03 ~13:00 UTC: only a Summer 2027 R&amp;D intern role and a generic, undated 'Spring &amp; Fall Co-op Program' description found; no dated Spring 2027 req located and no ATS link resolvable for a direct check.</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="str">
+        <v>Sensata Technologies (Attleboro, MA)</v>
+      </c>
+      <c r="B651" t="str">
+        <v>General intern/co-op search</v>
+      </c>
+      <c r="C651" t="str">
+        <v>2026-10-03 ~13:00 UTC: only Summer 2026 Mechanical Engineer Intern reqs found (incl. an Aerospace-specific one) — no Spring 2027 posting located.</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="str">
+        <v>PsiQuantum</v>
+      </c>
+      <c r="B652" t="str">
+        <v>General mechanical intern search</v>
+      </c>
+      <c r="C652" t="str">
+        <v>2026-10-03 ~13:00 UTC: only non-mechanical quantum-architecture/software intern roles found; no mechanical posting located.</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="str">
+        <v>RTX (Collins Aerospace, Uniontown, OH)</v>
+      </c>
+      <c r="B653" t="str">
+        <v>'Mechanical Design Engineering Co-op (Spring 2027)', req 01874486</v>
+      </c>
+      <c r="C653" t="str">
+        <v>2026-10-03 ~13:00 UTC: appeared in RTX's live search index (title/location only), but the job-detail endpoint returned HTTP 403 (errorCode S22, same tenant-level block affecting all RTX/Collins reqs this run — confirmed on known-live control reqs too, so not itself a status signal). Could not confirm canApply/pay. Not added; worth a follow-up once RTX access clears.</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="str">
+        <v>Graco Inc. (Rogers, MN)</v>
+      </c>
+      <c r="B654" t="str">
+        <v>'Manufacturing Engineering Co-op (May - December 2027)', req R0023504</v>
+      </c>
+      <c r="C654" t="str">
+        <v>2026-10-03 ~13:00 UTC: found during the nVent/Graco liveness re-sweep, confirmed canApply:true via direct Workday CXS fetch, but explicitly 'May - December 2027' — wrong season. Not added.</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="str">
+        <v>Graco Inc. (Dayton, MN)</v>
+      </c>
+      <c r="B655" t="str">
+        <v>'Manufacturing Engineering Co-op (May - December 2027)', req R0023506</v>
+      </c>
+      <c r="C655" t="str">
+        <v>2026-10-03 ~13:00 UTC: found during the same sweep, confirmed canApply:true, but explicitly 'May - December 2027' — wrong season. Not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C640"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C655"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 16 checked-excluded (2026-10-03 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VFEpR1kGxCkMzRDH5MoueN
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M320"/>
+  <dimension ref="A1:M321"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -9186,63 +9186,63 @@
         <v>RTX / Collins Aerospace</v>
       </c>
       <c r="B229" t="str">
-        <v>Chemical/Materials Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Certification Engineer Co-Op (Winter/Spring 2027)(Onsite)</v>
       </c>
       <c r="C229" t="str">
-        <v>Industrial / Materials Engineering (Z-Fab wafer fabrication manufacturing)</v>
+        <v>Aerospace / Structural Engineering (FAA certification — seats &amp; seating components)</v>
       </c>
       <c r="D229" t="str">
-        <v>Winter/Spring 2027 (posting titled 'Winter &amp; Spring Co-op')</v>
+        <v>Winter/Spring 2027 (two-semester term, January–July)</v>
       </c>
       <c r="E229" t="str">
-        <v>Cedar Rapids, IA</v>
+        <v>Winston-Salem, NC</v>
       </c>
       <c r="F229">
-        <v>1140</v>
+        <v>700</v>
       </c>
       <c r="G229" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H229" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-IA-CEDAR-RAPIDS-109--400-Collins-Rd-NE--BLDG-109/Chemical-Materials-Engineering-Co-op--Winter-Spring-2027-_01871473</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
       </c>
       <c r="I229" t="str">
-        <v>Yes — fetched directly via RTX's own Workday CXS API, canApply true, posted 2026-09-27.</v>
+        <v>Yes — fetched directly via RTX's own Workday CXS API, canApply true, posted 2026-09-16.</v>
       </c>
       <c r="J229" t="str">
-        <v>Req 01871473. TIME-SENSITIVE: posting's own end date is 2026-10-03 (application window closes fast). Title says Chemical/Materials Engineering but body describes Industrial Engineering manufacturing-process work (equipment/floor layout, cost/productivity studies, quality/safety review) on the Z-Fab wafer fab team. U.S. citizenship strictly required, no clearance required.</v>
+        <v>Req 01871317. Supports FAA certification (structural and flammability testing) of commercial aircraft seats. Majors: Mechanical, Aerospace, Materials Science, or Chemical Engineering. Requires U.S. Person status (ITAR — ecfr 8 U.S.C. 1101(a)(20)/1324b(a)(3)), not strictly U.S. citizenship. A sibling 'Summer/Fall 2027' req (01874662) at the same site was excluded, wrong season.</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>RTX / Collins Aerospace</v>
+        <v>Regal Rexnord</v>
       </c>
       <c r="B230" t="str">
-        <v>Certification Engineer Co-Op (Winter/Spring 2027)(Onsite)</v>
+        <v>Engineering Co-Op</v>
       </c>
       <c r="C230" t="str">
-        <v>Aerospace / Structural Engineering (FAA certification — seats &amp; seating components)</v>
+        <v>Mechanical / General Engineering</v>
       </c>
       <c r="D230" t="str">
-        <v>Winter/Spring 2027 (two-semester term, January–July)</v>
+        <v>Winter/January 2027 (3-4 month co-op)</v>
       </c>
       <c r="E230" t="str">
-        <v>Winston-Salem, NC</v>
+        <v>Charlotte, NC</v>
       </c>
       <c r="F230">
-        <v>700</v>
+        <v>845</v>
       </c>
       <c r="G230" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H230" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-NC-WINSTON-SALEM-190--190-Oak-Plaza-Blvd--BLDG-190/Certification-Engineer-Co-Op--Winter-Spring-2027--Onsite-_01871317-1</v>
+        <v>https://careers.regalrexnord.com/en/jobs/r26_04216/engineering-co-op/</v>
       </c>
       <c r="I230" t="str">
-        <v>Yes — fetched directly via RTX's own Workday CXS API, canApply true, posted 2026-09-16.</v>
+        <v>Yes — fetched directly (WebFetch), quote: 'Co-Op Start: Winter/January 2027', posted 2026-08-25, active Apply Now button present.</v>
       </c>
       <c r="J230" t="str">
-        <v>Req 01871317. Supports FAA certification (structural and flammability testing) of commercial aircraft seats. Majors: Mechanical, Aerospace, Materials Science, or Chemical Engineering. Requires U.S. Person status (ITAR — ecfr 8 U.S.C. 1101(a)(20)/1324b(a)(3)), not strictly U.S. citizenship. A sibling 'Summer/Fall 2027' req (01874662) at the same site was excluded, wrong season.</v>
+        <v>Req R26_04216. New company for the tracker. No discipline restriction stated beyond general engineering; posting text did not specify eligibility/citizenship requirements — confirm directly with employer before applying.</v>
       </c>
     </row>
     <row r="231">
@@ -9250,95 +9250,95 @@
         <v>Regal Rexnord</v>
       </c>
       <c r="B231" t="str">
-        <v>Engineering Co-Op</v>
+        <v>Application Engineer Co-op (Spring 2027)</v>
       </c>
       <c r="C231" t="str">
-        <v>Mechanical / General Engineering</v>
+        <v>Mechanical / Electrical Engineering</v>
       </c>
       <c r="D231" t="str">
-        <v>Winter/January 2027 (3-4 month co-op)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E231" t="str">
-        <v>Charlotte, NC</v>
+        <v>Tipp City, OH</v>
       </c>
       <c r="F231">
-        <v>845</v>
+        <v>750</v>
       </c>
       <c r="G231" t="str">
-        <v>Not stated on posting</v>
+        <v>$20–$25/hr</v>
       </c>
       <c r="H231" t="str">
-        <v>https://careers.regalrexnord.com/en/jobs/r26_04216/engineering-co-op/</v>
+        <v>https://careers.regalrexnord.com/en/jobs/r26_04440/application-engineer-co-op-spring-2027/</v>
       </c>
       <c r="I231" t="str">
-        <v>Yes — fetched directly (WebFetch), quote: 'Co-Op Start: Winter/January 2027', posted 2026-08-25, active Apply Now button present.</v>
+        <v>Yes — fetched directly on Regal Rexnord's own careers.regalrexnord.com domain (retrieved twice, consistent), title states 'Application Engineer Co-op (Spring 2027)' verbatim, canApply/Apply Now button present, posted ~2026-09-18. Also resolves via Workday mirror regalrexnord.wd1.myworkdayjobs.com/Careers/job/.../Application-Engineer-Co-op--Spring-2027-_R26_04440-1.</v>
       </c>
       <c r="J231" t="str">
-        <v>Req R26_04216. New company for the tracker. No discipline restriction stated beyond general engineering; posting text did not specify eligibility/citizenship requirements — confirm directly with employer before applying.</v>
+        <v>Req R26_04440. Resolves a prior run's unverified aggregator-sourced lead for this same role/site (previously could not locate a working direct URL). Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; min GPA 3.0; basic SolidWorks/3D modeling knowledge helpful. Fully onsite, no travel. Citizenship/ITAR not stated on posting.</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>Regal Rexnord</v>
+        <v>Skyworks Solutions</v>
       </c>
       <c r="B232" t="str">
-        <v>Application Engineer Co-op (Spring 2027)</v>
+        <v>Microelectronics / Semiconductor Packaging Co-Op</v>
       </c>
       <c r="C232" t="str">
-        <v>Mechanical / Electrical Engineering</v>
+        <v>Mechanical / Chemical / Materials Science / Industrial Engineering</v>
       </c>
       <c r="D232" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring Co-Op, January 2027 – June 2027</v>
       </c>
       <c r="E232" t="str">
-        <v>Tipp City, OH</v>
+        <v>Nashua, NH</v>
       </c>
       <c r="F232">
-        <v>750</v>
+        <v>40</v>
       </c>
       <c r="G232" t="str">
-        <v>$20–$25/hr</v>
+        <v>$26.00–$47.50/hr</v>
       </c>
       <c r="H232" t="str">
-        <v>https://careers.regalrexnord.com/en/jobs/r26_04440/application-engineer-co-op-spring-2027/</v>
+        <v>https://careers.skyworksinc.com/job/Nashua-Microelectronics-Semiconductor-Packaging-Co-Op-NH-03060/78294-en_US/</v>
       </c>
       <c r="I232" t="str">
-        <v>Yes — fetched directly on Regal Rexnord's own careers.regalrexnord.com domain (retrieved twice, consistent), title states 'Application Engineer Co-op (Spring 2027)' verbatim, canApply/Apply Now button present, posted ~2026-09-18. Also resolves via Workday mirror regalrexnord.wd1.myworkdayjobs.com/Careers/job/.../Application-Engineer-Co-op--Spring-2027-_R26_04440-1.</v>
+        <v>Yes — fetched directly (WebFetch), req ID 78294 embedded in page, active 'Apply now' button present, posted 2026-09-14, quote: 'This is for a Winter/Spring Coop from January 2027 - June 2027.'</v>
       </c>
       <c r="J232" t="str">
-        <v>Req R26_04440. Resolves a prior run's unverified aggregator-sourced lead for this same role/site (previously could not locate a working direct URL). Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; min GPA 3.0; basic SolidWorks/3D modeling knowledge helpful. Fully onsite, no travel. Citizenship/ITAR not stated on posting.</v>
+        <v>Req 78294. Discovered via Skyworks' own public sitemap.xml. Unlike every other Skyworks co-op tracked so far (all EE-only), this one explicitly also accepts Mechanical/Chemical/Materials Science/Industrial Engineering majors — packaging-materials evaluation (adhesives, mold compounds, substrates, underfills, TIMs), failure analysis, DOE. Junior/Senior standing or current grad student. No citizenship/ITAR language stated. Preferred (not required) skills: SolidWorks/Creo/AutoCAD, Minitab/JMP/MATLAB/Python.</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>Skyworks Solutions</v>
+        <v>Regal Rexnord</v>
       </c>
       <c r="B233" t="str">
-        <v>Microelectronics / Semiconductor Packaging Co-Op</v>
+        <v>Application Team Co-Op (Spring 2027)</v>
       </c>
       <c r="C233" t="str">
-        <v>Mechanical / Chemical / Materials Science / Industrial Engineering</v>
+        <v>Mechanical / Electrical Engineering</v>
       </c>
       <c r="D233" t="str">
-        <v>Winter/Spring Co-Op, January 2027 – June 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E233" t="str">
-        <v>Nashua, NH</v>
+        <v>Tipp City, OH</v>
       </c>
       <c r="F233">
-        <v>40</v>
+        <v>750</v>
       </c>
       <c r="G233" t="str">
-        <v>$26.00–$47.50/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H233" t="str">
-        <v>https://careers.skyworksinc.com/job/Nashua-Microelectronics-Semiconductor-Packaging-Co-Op-NH-03060/78294-en_US/</v>
+        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Tipp-City-Ohio-United-States/Application-Team-Co-Op--Spring-2027-_R26_04736-1</v>
       </c>
       <c r="I233" t="str">
-        <v>Yes — fetched directly (WebFetch), req ID 78294 embedded in page, active 'Apply now' button present, posted 2026-09-14, quote: 'This is for a Winter/Spring Coop from January 2027 - June 2027.'</v>
+        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Application Team Co-Op (Spring 2027)' verbatim, posted 3 days ago (2026-09-25), no filled/closed language.</v>
       </c>
       <c r="J233" t="str">
-        <v>Req 78294. Discovered via Skyworks' own public sitemap.xml. Unlike every other Skyworks co-op tracked so far (all EE-only), this one explicitly also accepts Mechanical/Chemical/Materials Science/Industrial Engineering majors — packaging-materials evaluation (adhesives, mold compounds, substrates, underfills, TIMs), failure analysis, DOE. Junior/Senior standing or current grad student. No citizenship/ITAR language stated. Preferred (not required) skills: SolidWorks/Creo/AutoCAD, Minitab/JMP/MATLAB/Python.</v>
+        <v>Req R26_04736. New req at the same Tipp City, OH site as the already-tracked R26_04440 'Application Engineer Co-op' — distinct responsibilities (mechanical/electrical design support, CAD detail drawings, 3D-printer lab support) not a duplicate. Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; GPA 3.0+; basic SolidWorks/3D modeling knowledge. Fully onsite. Citizenship/ITAR not stated on posting.</v>
       </c>
     </row>
     <row r="234">
@@ -9346,191 +9346,191 @@
         <v>Regal Rexnord</v>
       </c>
       <c r="B234" t="str">
-        <v>Application Team Co-Op (Spring 2027)</v>
+        <v>Sound Lab Co-op (Spring 2027)</v>
       </c>
       <c r="C234" t="str">
-        <v>Mechanical / Electrical Engineering</v>
+        <v>Mechanical / Electrical Engineering (acoustics &amp; vibration testing)</v>
       </c>
       <c r="D234" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E234" t="str">
-        <v>Tipp City, OH</v>
+        <v>Fort Wayne, IN</v>
       </c>
       <c r="F234">
-        <v>750</v>
+        <v>830</v>
       </c>
       <c r="G234" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H234" t="str">
-        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Tipp-City-Ohio-United-States/Application-Team-Co-Op--Spring-2027-_R26_04736-1</v>
+        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Fort-Wayne-Indiana-United-States/Sound-Lab-Co-op--Spring-2027-_R26_04469-2</v>
       </c>
       <c r="I234" t="str">
-        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Application Team Co-Op (Spring 2027)' verbatim, posted 3 days ago (2026-09-25), no filled/closed language.</v>
+        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Sound Lab Co-op (Spring 2027)' verbatim, posted 5 days ago (2026-09-23), no filled/closed language.</v>
       </c>
       <c r="J234" t="str">
-        <v>Req R26_04736. New req at the same Tipp City, OH site as the already-tracked R26_04440 'Application Engineer Co-op' — distinct responsibilities (mechanical/electrical design support, CAD detail drawings, 3D-printer lab support) not a duplicate. Currently pursuing a Bachelor's in Mechanical, Electrical, or a relevant Engineering degree; GPA 3.0+; basic SolidWorks/3D modeling knowledge. Fully onsite. Citizenship/ITAR not stated on posting.</v>
+        <v>Req R26_04469. Anechoic chamber / sound &amp; vibration analysis for customer returns, cost-reduction, and new-product-development testing. Currently pursuing a Bachelor's in Mechanical or Electrical Engineering. Fully onsite. Citizenship/ITAR not stated on posting.</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>Regal Rexnord</v>
+        <v>Crane Company (Crane Pumps &amp; Systems)</v>
       </c>
       <c r="B235" t="str">
-        <v>Sound Lab Co-op (Spring 2027)</v>
+        <v>Engineering Co-op Spring 2027-1</v>
       </c>
       <c r="C235" t="str">
-        <v>Mechanical / Electrical Engineering (acoustics &amp; vibration testing)</v>
+        <v>Mechanical / Electrical Engineering</v>
       </c>
       <c r="D235" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E235" t="str">
-        <v>Fort Wayne, IN</v>
+        <v>Piqua, OH</v>
       </c>
       <c r="F235">
-        <v>830</v>
+        <v>750</v>
       </c>
       <c r="G235" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H235" t="str">
-        <v>https://regalrexnord.wd1.myworkdayjobs.com/Careers/job/Fort-Wayne-Indiana-United-States/Sound-Lab-Co-op--Spring-2027-_R26_04469-2</v>
+        <v>https://cranecompany.wd5.myworkdayjobs.com/Careers/job/Piqua-Ohio/Engineering-Co-op-Spring-2027-1_JR102521</v>
       </c>
       <c r="I235" t="str">
-        <v>Yes — fetched directly via Regal Rexnord's own Workday CXS API, title 'Sound Lab Co-op (Spring 2027)' verbatim, posted 5 days ago (2026-09-23), no filled/closed language.</v>
+        <v>Yes — fetched directly via Crane Company's own Workday CXS API for all three parallel req IDs (JR102518, JR102520, JR102521), identical title 'Engineering Co-op Spring 2027-1', posted 14 days ago (2026-09-14), no filled/closed language on any.</v>
       </c>
       <c r="J235" t="str">
-        <v>Req R26_04469. Anechoic chamber / sound &amp; vibration analysis for customer returns, cost-reduction, and new-product-development testing. Currently pursuing a Bachelor's in Mechanical or Electrical Engineering. Fully onsite. Citizenship/ITAR not stated on posting.</v>
+        <v>New company for the tracker. 3 parallel open headcount at the same Piqua, OH site under reqs JR102518, JR102520, and JR102521 (all independently confirmed live) — general engineering support (product design, CAD documentation, lab/test support) for pump products serving industrial/commercial/residential/municipal/military markets. Working toward a B.S. in Mechanical, Mechanical Tech, or Electrical Engineering. This is the Pumps &amp; Systems division (not Crane Aerospace &amp; Electronics, which has a separate ITAR-restricted, season-ambiguous posting — excluded, see `checked`). Citizenship/ITAR not stated on this posting.</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>Crane Company (Crane Pumps &amp; Systems)</v>
+        <v>Flex (Flextronics International)</v>
       </c>
       <c r="B236" t="str">
-        <v>Engineering Co-op Spring 2027-1</v>
+        <v>Mechanical Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C236" t="str">
-        <v>Mechanical / Electrical Engineering</v>
+        <v>Mechanical Engineering (manufacturing/process engineering)</v>
       </c>
       <c r="D236" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E236" t="str">
-        <v>Piqua, OH</v>
+        <v>Libertyville, IL</v>
       </c>
       <c r="F236">
-        <v>750</v>
+        <v>990</v>
       </c>
       <c r="G236" t="str">
-        <v>Not stated on posting</v>
+        <v>$27.50–$44.50/hr</v>
       </c>
       <c r="H236" t="str">
-        <v>https://cranecompany.wd5.myworkdayjobs.com/Careers/job/Piqua-Ohio/Engineering-Co-op-Spring-2027-1_JR102521</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/Mechanical-Engineering-Co-Op---Spring-2027_WD229697</v>
       </c>
       <c r="I236" t="str">
-        <v>Yes — fetched directly via Crane Company's own Workday CXS API for all three parallel req IDs (JR102518, JR102520, JR102521), identical title 'Engineering Co-op Spring 2027-1', posted 14 days ago (2026-09-14), no filled/closed language on any.</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229697, posted 10 days ago (2026-09-18), quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 co-op assignment.'</v>
       </c>
       <c r="J236" t="str">
-        <v>New company for the tracker. 3 parallel open headcount at the same Piqua, OH site under reqs JR102518, JR102520, and JR102521 (all independently confirmed live) — general engineering support (product design, CAD documentation, lab/test support) for pump products serving industrial/commercial/residential/municipal/military markets. Working toward a B.S. in Mechanical, Mechanical Tech, or Electrical Engineering. This is the Pumps &amp; Systems division (not Crane Aerospace &amp; Electronics, which has a separate ITAR-restricted, season-ambiguous posting — excluded, see `checked`). Citizenship/ITAR not stated on this posting.</v>
+        <v>New company for the tracker. Manufacturing/process-engineering support — time studies, CAD, DOE projects, Lean/Six Sigma. Current BS/MS student pursuing Mechanical Engineering; 2D/3D CAD (AutoCAD/Inventor/Solidworks); GPA 3.0+. Posting explicitly states 'Is Sponsorship Available? No' (no visa sponsorship — not a citizenship/ITAR requirement).</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>MIT Lincoln Laboratory</v>
       </c>
       <c r="B237" t="str">
-        <v>Mechanical Engineering Co-Op - Spring 2027</v>
+        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
       </c>
       <c r="C237" t="str">
-        <v>Mechanical Engineering (manufacturing/process engineering)</v>
+        <v>Mechanical Engineering / Aerospace Engineering</v>
       </c>
       <c r="D237" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E237" t="str">
-        <v>Libertyville, IL</v>
+        <v>Lexington, MA</v>
       </c>
       <c r="F237">
-        <v>990</v>
+        <v>11</v>
       </c>
       <c r="G237" t="str">
-        <v>$27.50–$44.50/hr</v>
+        <v>$25–$32/hr (Technical Co-Op, based on year in school)</v>
       </c>
       <c r="H237" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/Mechanical-Engineering-Co-Op---Spring-2027_WD229697</v>
+        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
       </c>
       <c r="I237" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229697, posted 10 days ago (2026-09-18), quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 co-op assignment.'</v>
+        <v>Yes — fetched directly (server-rendered SAP SuccessFactors page, not JS-gated), req ID 1434254300, posted 2026-09-28, title states '(Winter/Spring 2027)' verbatim.</v>
       </c>
       <c r="J237" t="str">
-        <v>New company for the tracker. Manufacturing/process-engineering support — time studies, CAD, DOE projects, Lean/Six Sigma. Current BS/MS student pursuing Mechanical Engineering; 2D/3D CAD (AutoCAD/Inventor/Solidworks); GPA 3.0+. Posting explicitly states 'Is Sponsorship Available? No' (no visa sponsorship — not a citizenship/ITAR requirement).</v>
+        <v>Requisition ID 43350. Open to Mechanical Engineering, Aeronautics/Astronautics, Aerospace Engineering, or Physics majors (must have completed Mechanics of Materials or equivalent); CAD/FEA/prototyping preferred, not required. Requires U.S. citizenship and eligibility for a Secret-level DoD security clearance. Distinct from the already-tracked Microfabrication (Group 08-35) co-ops. Apply at https://careers.ll.mit.edu/talentcommunity/apply/1434254300/?locale=en_US</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>MIT Lincoln Laboratory</v>
+        <v>DEKA Research &amp; Development</v>
       </c>
       <c r="B238" t="str">
-        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
+        <v>Systems Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C238" t="str">
-        <v>Mechanical Engineering / Aerospace Engineering</v>
+        <v>Bioengineering / Biomedical / Mechanical Engineering</v>
       </c>
       <c r="D238" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027 (starting January 2027)</v>
       </c>
       <c r="E238" t="str">
-        <v>Lexington, MA</v>
+        <v>Manchester, NH</v>
       </c>
       <c r="F238">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="G238" t="str">
-        <v>$25–$32/hr (Technical Co-Op, based on year in school)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H238" t="str">
-        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
+        <v>https://deka.applytojob.com/apply/76ReoonYrJ/Systems-Engineer-CoOp-Spring-2027</v>
       </c>
       <c r="I238" t="str">
-        <v>Yes — fetched directly (server-rendered SAP SuccessFactors page, not JS-gated), req ID 1434254300, posted 2026-09-28, title states '(Winter/Spring 2027)' verbatim.</v>
+        <v>Yes — fetched directly (JazzHR-hosted, server-rendered, not JS-gated), full description read. Quote: 'This position is for a 6+ month rotation for the Spring semester starting in January 2027.'</v>
       </c>
       <c r="J238" t="str">
-        <v>Requisition ID 43350. Open to Mechanical Engineering, Aeronautics/Astronautics, Aerospace Engineering, or Physics majors (must have completed Mechanics of Materials or equivalent); CAD/FEA/prototyping preferred, not required. Requires U.S. citizenship and eligibility for a Secret-level DoD security clearance. Distinct from the already-tracked Microfabrication (Group 08-35) co-ops. Apply at https://careers.ll.mit.edu/talentcommunity/apply/1434254300/?locale=en_US</v>
+        <v>New company for the tracker — DEKA is Dean Kamen's medical-device/robotics R&amp;D house (insulin pumps, robotic arms, water purification, etc.), Manchester, NH. Open to undergraduate Bioengineering, Biomedical, or Mechanical Engineering majors; graduate students NOT eligible for this specific req. Closing date and GPA requirement not stated. A separate 'Software Engineering Co-Op - Spring 2027' req also exists at the same company but is out of scope (software discipline).</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>DEKA Research &amp; Development</v>
+        <v>Flex (Flextronics International)</v>
       </c>
       <c r="B239" t="str">
-        <v>Systems Engineer Co-Op - Spring 2027</v>
+        <v>Automation/Controls Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C239" t="str">
-        <v>Bioengineering / Biomedical / Mechanical Engineering</v>
+        <v>Electrical Engineering / Mechatronics / Automation Engineering (Controls)</v>
       </c>
       <c r="D239" t="str">
-        <v>Spring 2027 (starting January 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E239" t="str">
-        <v>Manchester, NH</v>
+        <v>Libertyville, IL</v>
       </c>
       <c r="F239">
-        <v>50</v>
+        <v>990</v>
       </c>
       <c r="G239" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H239" t="str">
-        <v>https://deka.applytojob.com/apply/76ReoonYrJ/Systems-Engineer-CoOp-Spring-2027</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Automation-Controls-Engineering-Co-Op---Spring-2027_WD229698</v>
       </c>
       <c r="I239" t="str">
-        <v>Yes — fetched directly (JazzHR-hosted, server-rendered, not JS-gated), full description read. Quote: 'This position is for a 6+ month rotation for the Spring semester starting in January 2027.'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229698, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
       </c>
       <c r="J239" t="str">
-        <v>New company for the tracker — DEKA is Dean Kamen's medical-device/robotics R&amp;D house (insulin pumps, robotic arms, water purification, etc.), Manchester, NH. Open to undergraduate Bioengineering, Biomedical, or Mechanical Engineering majors; graduate students NOT eligible for this specific req. Closing date and GPA requirement not stated. A separate 'Software Engineering Co-Op - Spring 2027' req also exists at the same company but is out of scope (software discipline).</v>
+        <v>Electrical Engineering, Mechatronics, or Automation Engineering major. PLC/HMI programming, FAT/SAT testing. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="240">
@@ -9538,10 +9538,10 @@
         <v>Flex (Flextronics International)</v>
       </c>
       <c r="B240" t="str">
-        <v>Automation/Controls Engineering Co-Op - Spring 2027</v>
+        <v>Robotics/Mechatronics Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C240" t="str">
-        <v>Electrical Engineering / Mechatronics / Automation Engineering (Controls)</v>
+        <v>Mechanical / Mechatronics / Robotics Engineering</v>
       </c>
       <c r="D240" t="str">
         <v>Spring 2027</v>
@@ -9556,13 +9556,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H240" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Automation-Controls-Engineering-Co-Op---Spring-2027_WD229698</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Robotics-Mechatronics-Engineering-Co-Op---Spring-2027_WD229699</v>
       </c>
       <c r="I240" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229698, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229699, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
       </c>
       <c r="J240" t="str">
-        <v>Electrical Engineering, Mechatronics, or Automation Engineering major. PLC/HMI programming, FAT/SAT testing. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+        <v>Robot path optimization, AMR/ASRS validation, machine-vision systems. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="241">
@@ -9570,10 +9570,10 @@
         <v>Flex (Flextronics International)</v>
       </c>
       <c r="B241" t="str">
-        <v>Robotics/Mechatronics Engineering Co-Op - Spring 2027</v>
+        <v>Plastic Molding Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C241" t="str">
-        <v>Mechanical / Mechatronics / Robotics Engineering</v>
+        <v>Materials / Manufacturing Engineering (Plastics)</v>
       </c>
       <c r="D241" t="str">
         <v>Spring 2027</v>
@@ -9588,13 +9588,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H241" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Robotics-Mechatronics-Engineering-Co-Op---Spring-2027_WD229699</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Plastic-Molding-Engineering-Co-Op---Spring-2027_WD229696</v>
       </c>
       <c r="I241" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229699, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229696, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
       </c>
       <c r="J241" t="str">
-        <v>Robot path optimization, AMR/ASRS validation, machine-vision systems. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+        <v>Plastics Engineering major, injection-molding/materials/manufacturing focus. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="242">
@@ -9602,191 +9602,191 @@
         <v>Flex (Flextronics International)</v>
       </c>
       <c r="B242" t="str">
-        <v>Plastic Molding Engineering Co-Op - Spring 2027</v>
+        <v>Industrial Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C242" t="str">
-        <v>Materials / Manufacturing Engineering (Plastics)</v>
+        <v>Industrial Engineering</v>
       </c>
       <c r="D242" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E242" t="str">
-        <v>Libertyville, IL</v>
+        <v>Orangeburg, SC</v>
       </c>
       <c r="F242">
-        <v>990</v>
+        <v>810</v>
       </c>
       <c r="G242" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H242" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-IL-Libertyville/Plastic-Molding-Engineering-Co-Op---Spring-2027_WD229696</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Industrial-Engineering-Co-Op---Fall-2026_WD226357</v>
       </c>
       <c r="I242" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD229696, posted 2026-09-18, canApply true, quote: '...during the Spring 2027 co-op assignment.'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226357, posted 2026-09-03, canApply true. NOTE: title and body text both explicitly say '(Spring 2027)' ('...looking to add an Industrial Engineering Co-Op (Spring 2027)...'), but the URL slug itself reads 'Fall-2026' — an apparent leftover from an earlier req rename. Treating the in-body/title season text as authoritative per the verification bar.</v>
       </c>
       <c r="J242" t="str">
-        <v>Plastics Engineering major, injection-molding/materials/manufacturing focus. Sibling req to the already-tracked Mechanical Engineering Co-Op (WD229697) at the same Libertyville, IL site. GPA 3.0+, 40 hrs/week in-person. Pay/citizenship not stated.</v>
+        <v>Fulfillment/server-assembly warehouse operations, Lean/Six Sigma. Two sibling reqs at the same Orangeburg, SC site (Quality Engineering Co-Op, Program Management Co-Op) have the same title/URL-slug season discrepancy but are non-target disciplines — see `checked`. Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>Axcelis Technologies</v>
       </c>
       <c r="B243" t="str">
-        <v>Industrial Engineering Co-Op (Spring 2027)</v>
+        <v>Engineering Co-op (Warehouse Solutions)</v>
       </c>
       <c r="C243" t="str">
-        <v>Industrial Engineering</v>
+        <v>Industrial Engineering / Manufacturing Operations</v>
       </c>
       <c r="D243" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027 (Jan 4–Jun 25, 2027)</v>
       </c>
       <c r="E243" t="str">
-        <v>Orangeburg, SC</v>
+        <v>Beverly, MA</v>
       </c>
       <c r="F243">
-        <v>810</v>
+        <v>25</v>
       </c>
       <c r="G243" t="str">
-        <v>Not stated on posting</v>
+        <v>$20.42–$35.70/hr (posted U.S. base salary range)</v>
       </c>
       <c r="H243" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Industrial-Engineering-Co-Op---Fall-2026_WD226357</v>
+        <v>https://axcelis.wd1.myworkdayjobs.com/Axcelis/job/Beverly-MA/Engineering-Co-op--Warehouse-Solutions-_12018</v>
       </c>
       <c r="I243" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226357, posted 2026-09-03, canApply true. NOTE: title and body text both explicitly say '(Spring 2027)' ('...looking to add an Industrial Engineering Co-Op (Spring 2027)...'), but the URL slug itself reads 'Fall-2026' — an apparent leftover from an earlier req rename. Treating the in-body/title season text as authoritative per the verification bar.</v>
+        <v>Yes — fetched directly via Axcelis's own Workday CXS API, req 12018, posted 14 days ago (2026-09-15), canApply true, quote: 'Co-op Cycle: January 4th to June 25th, 2027.'</v>
       </c>
       <c r="J243" t="str">
-        <v>Fulfillment/server-assembly warehouse operations, Lean/Six Sigma. Two sibling reqs at the same Orangeburg, SC site (Quality Engineering Co-Op, Program Management Co-Op) have the same title/URL-slug season discrepancy but are non-target disciplines — see `checked`. Pay/citizenship not stated.</v>
+        <v>New company for the tracker — Axcelis is a semiconductor ion-implantation equipment maker HQ'd in Beverly, MA. Warehouse Operations co-op supporting the Operations Technology team (logistics/process-improvement, some SQL/Python/PowerBI preferred). Open to Mechanical or Industrial Engineering students (or related field). $1,000 commuting travel stipend offered. Citizenship not stated. Sibling reqs at the same site were checked and excluded — see `checked` (one has an internal Winter-2027-header-vs-'summer 2026'-body contradiction, two have no year stated, two are explicitly Fall-cycle, one is Software Development discipline).</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>Axcelis Technologies</v>
+        <v>Flex (Flextronics International)</v>
       </c>
       <c r="B244" t="str">
-        <v>Engineering Co-op (Warehouse Solutions)</v>
+        <v>NPI Process Engineering Co-op</v>
       </c>
       <c r="C244" t="str">
-        <v>Industrial Engineering / Manufacturing Operations</v>
+        <v>Manufacturing Engineering (New Product Introduction)</v>
       </c>
       <c r="D244" t="str">
-        <v>Winter/Spring 2027 (Jan 4–Jun 25, 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
       </c>
       <c r="E244" t="str">
-        <v>Beverly, MA</v>
+        <v>Hollis, NH (posting body says Nashua, NH site)</v>
       </c>
       <c r="F244">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G244" t="str">
-        <v>$20.42–$35.70/hr (posted U.S. base salary range)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H244" t="str">
-        <v>https://axcelis.wd1.myworkdayjobs.com/Axcelis/job/Beverly-MA/Engineering-Co-op--Warehouse-Solutions-_12018</v>
+        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/NPI-Process-Engineering-Co-op_WD226387</v>
       </c>
       <c r="I244" t="str">
-        <v>Yes — fetched directly via Axcelis's own Workday CXS API, req 12018, posted 14 days ago (2026-09-15), canApply true, quote: 'Co-op Cycle: January 4th to June 25th, 2027.'</v>
+        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226387, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
       </c>
       <c r="J244" t="str">
-        <v>New company for the tracker — Axcelis is a semiconductor ion-implantation equipment maker HQ'd in Beverly, MA. Warehouse Operations co-op supporting the Operations Technology team (logistics/process-improvement, some SQL/Python/PowerBI preferred). Open to Mechanical or Industrial Engineering students (or related field). $1,000 commuting travel stipend offered. Citizenship not stated. Sibling reqs at the same site were checked and excluded — see `checked` (one has an internal Winter-2027-header-vs-'summer 2026'-body contradiction, two have no year stated, two are explicitly Fall-cycle, one is Software Development discipline).</v>
+        <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>RTX / Collins Aerospace</v>
       </c>
       <c r="B245" t="str">
-        <v>NPI Process Engineering Co-op</v>
+        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
       </c>
       <c r="C245" t="str">
-        <v>Manufacturing Engineering (New Product Introduction)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D245" t="str">
-        <v>Winter/Spring 2027 (Jan–Jun 2027)</v>
+        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
       </c>
       <c r="E245" t="str">
-        <v>Hollis, NH (posting body says Nashua, NH site)</v>
+        <v>Cedar Rapids, IA</v>
       </c>
       <c r="F245">
-        <v>45</v>
+        <v>1090</v>
       </c>
       <c r="G245" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated on posting (RTX co-op program range generally $37,000–$82,000/yr annualized per boilerplate)</v>
       </c>
       <c r="H245" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-NH-Hollis/NPI-Process-Engineering-Co-op_WD226387</v>
+        <v>https://careers.rtx.com/global/en/job/01872047/Mechanical-Engineering-Co-op-Winter-Spring-2027</v>
       </c>
       <c r="I245" t="str">
-        <v>Yes — fetched directly via Flex's own Workday CXS API, req WD226387, canApply true, quote: 'Available to work 40 hours/week (in-person) for the assignment term (Jan - Jun 2027).'</v>
+        <v>Yes — independently fetched raw HTML/JSON-LD directly (bypassing careers.rtx.com's unreliable WebFetch rendering), req 01872047, datePosted 2026-09-28, title states '(Winter/Spring 2027)' verbatim, 'Apply Now' present, no filled/closed markers.</v>
       </c>
       <c r="J245" t="str">
-        <v>Sibling req to WD226382 above; NPI process engineering support for new product ramp. NOTE: Workday's location field says Hollis, NH but the job description body itself says 'our Nashua, NH site' — Flex's own posting is internally inconsistent on which town, both towns are ~2 mi apart and equally Boston-area. No end date populated (rolling/open posting, less time-pressure than its Mechanical Engineering sibling). Pay/citizenship not stated.</v>
+        <v>Displays, Controls, Computing &amp; Networking dept at Collins Aerospace — cockpit displays/control panels, servo actuation, avionics hardware. 'Immerse yourself in a full-time... co-op session, that will run January- July/August.' U.S. citizenship required (no clearance required). New req distinct from the already-tracked Chemical/Materials Co-op (01871473) and Mechanical Design Co-op (01871736, Jamestown ND) at the same company.</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>RTX / Collins Aerospace</v>
+        <v>Specter Aerospace</v>
       </c>
       <c r="B246" t="str">
-        <v>Mechanical Engineering Co-op (Winter/Spring 2027)</v>
+        <v>Mechanical Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C246" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D246" t="str">
-        <v>Winter/Spring 2027 (Jan–Jul/Aug 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E246" t="str">
-        <v>Cedar Rapids, IA</v>
+        <v>Boston, MA (Seaport)</v>
       </c>
       <c r="F246">
-        <v>1090</v>
+        <v>0</v>
       </c>
       <c r="G246" t="str">
-        <v>Not stated on posting (RTX co-op program range generally $37,000–$82,000/yr annualized per boilerplate)</v>
+        <v>$23-$30/hr</v>
       </c>
       <c r="H246" t="str">
-        <v>https://careers.rtx.com/global/en/job/01872047/Mechanical-Engineering-Co-op-Winter-Spring-2027</v>
+        <v>https://specteraerospace.bamboohr.com/careers/124</v>
       </c>
       <c r="I246" t="str">
-        <v>Yes — independently fetched raw HTML/JSON-LD directly (bypassing careers.rtx.com's unreliable WebFetch rendering), req 01872047, datePosted 2026-09-28, title states '(Winter/Spring 2027)' verbatim, 'Apply Now' present, no filled/closed markers.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API (specteraerospace.bamboohr.com/careers/124/detail), status Open, posted 2026-08-13, title states 'Mechanical Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J246" t="str">
-        <v>Displays, Controls, Computing &amp; Networking dept at Collins Aerospace — cockpit displays/control panels, servo actuation, avionics hardware. 'Immerse yourself in a full-time... co-op session, that will run January- July/August.' U.S. citizenship required (no clearance required). New req distinct from the already-tracked Chemical/Materials Co-op (01871473) and Mechanical Design Co-op (01871736, Jamestown ND) at the same company.</v>
+        <v>New company for the tracker — hypersonic flight vehicle startup (Boston Seaport + Peabody, MA offices), funded by government R&amp;D + private funding. Vehicle Development team, designing components/subsystems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance). Strong Boston-area match.</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Flex (Flextronics International)</v>
+        <v>Specter Aerospace</v>
       </c>
       <c r="B247" t="str">
-        <v>Mechanical Engineering Co-op - Spring 2027</v>
+        <v>Vehicle Design Co-Op - Spring 2027</v>
       </c>
       <c r="C247" t="str">
-        <v>Mechanical / Industrial Engineering</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D247" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E247" t="str">
-        <v>Orangeburg, SC</v>
+        <v>Boston, MA (Seaport)</v>
       </c>
       <c r="F247">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="G247" t="str">
-        <v>Not stated on posting</v>
+        <v>$23-$30/hr</v>
       </c>
       <c r="H247" t="str">
-        <v>https://flextronics.wd1.myworkdayjobs.com/Careers/job/USA-SC-Orangeburg/Mechanical-Engineering-Co-op---Fall-2026_WD227049</v>
+        <v>https://specteraerospace.bamboohr.com/careers/116</v>
       </c>
       <c r="I247" t="str">
-        <v>Yes — independently fetched directly via Flex's own Workday CXS API, req WD227049, canApply true, posted 26 days ago, title states 'Mechanical Engineering Co-op - Spring 2027' verbatim, quote: 'Available to work 40 hours/week (in-person) for the Spring 2027 school semester.'</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Vehicle Design Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J247" t="str">
-        <v>TIME-SENSITIVE: posting's own end date is 2026-10-03 — 3 days left to apply as of this run. NOTE: URL slug reads 'Fall-2026' (stale rename leftover, same pattern as the already-tracked Orangeburg Industrial Engineering Co-Op WD226357) but title/body both explicitly say 'Spring 2027' — treated as authoritative per the verification bar. Manufacturing Engineering Manager team — time studies, CAD, DOE projects. 'Is Sponsorship Available? No' (no visa sponsorship, not a citizenship/ITAR requirement). Pay not stated.</v>
+        <v>Sibling req to the Mechanical Engineer Co-Op above, same company/site. Vehicle Design team, designing components/systems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="248">
@@ -9794,31 +9794,31 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B248" t="str">
-        <v>Mechanical Engineer Co-Op - Spring 2027</v>
+        <v>Propulsion Test Engineering Co-Op - Spring 2027</v>
       </c>
       <c r="C248" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
       </c>
       <c r="D248" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E248" t="str">
-        <v>Boston, MA (Seaport)</v>
+        <v>Peabody, MA</v>
       </c>
       <c r="F248">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G248" t="str">
         <v>$23-$30/hr</v>
       </c>
       <c r="H248" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/124</v>
+        <v>https://specteraerospace.bamboohr.com/careers/117</v>
       </c>
       <c r="I248" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API (specteraerospace.bamboohr.com/careers/124/detail), status Open, posted 2026-08-13, title states 'Mechanical Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Propulsion Test Engineering Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J248" t="str">
-        <v>New company for the tracker — hypersonic flight vehicle startup (Boston Seaport + Peabody, MA offices), funded by government R&amp;D + private funding. Vehicle Development team, designing components/subsystems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance). Strong Boston-area match.</v>
+        <v>Design, manufacturing, and test of advanced ramjet/scramjet engine hardware for hypersonic propulsion systems. Note: posting says Specter hires both this and the Propulsion Design Engineering Co-op (below) from a shared applicant pool depending on interest/fit. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="249">
@@ -9826,31 +9826,31 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B249" t="str">
-        <v>Vehicle Design Co-Op - Spring 2027</v>
+        <v>Propulsion Design Engineering Co-op - Spring 2027</v>
       </c>
       <c r="C249" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
       </c>
       <c r="D249" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E249" t="str">
-        <v>Boston, MA (Seaport)</v>
+        <v>Peabody, MA</v>
       </c>
       <c r="F249">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G249" t="str">
         <v>$23-$30/hr</v>
       </c>
       <c r="H249" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/116</v>
+        <v>https://specteraerospace.bamboohr.com/careers/118</v>
       </c>
       <c r="I249" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Vehicle Design Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'Propulsion Design Engineering Co-op - Spring 2027' verbatim.</v>
       </c>
       <c r="J249" t="str">
-        <v>Sibling req to the Mechanical Engineer Co-Op above, same company/site. Vehicle Design team, designing components/systems for hypersonic flight vehicles. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>Sibling/shared-pool req to Propulsion Test Engineering Co-Op above (same site, same applicant pool per posting text). Design, manufacturing, and test of ramjet/scramjet engine hardware. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="250">
@@ -9858,10 +9858,10 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B250" t="str">
-        <v>Propulsion Test Engineering Co-Op - Spring 2027</v>
+        <v>PLC/Controls Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C250" t="str">
-        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
+        <v>Controls / Mechanical / Electrical Engineering</v>
       </c>
       <c r="D250" t="str">
         <v>Spring 2027</v>
@@ -9876,13 +9876,13 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H250" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/117</v>
+        <v>https://specteraerospace.bamboohr.com/careers/123</v>
       </c>
       <c r="I250" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-07-15, title states 'Propulsion Test Engineering Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'PLC/Controls Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J250" t="str">
-        <v>Design, manufacturing, and test of advanced ramjet/scramjet engine hardware for hypersonic propulsion systems. Note: posting says Specter hires both this and the Propulsion Design Engineering Co-op (below) from a shared applicant pool depending on interest/fit. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>PLC software design (Beckhoff/TwinCAT ecosystem), electrical control-panel design, sensor/actuator integration for the Specter engine test facility. Open to Computer/Electrical/Mechanical Engineering or CS majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="251">
@@ -9890,10 +9890,10 @@
         <v>Specter Aerospace</v>
       </c>
       <c r="B251" t="str">
-        <v>Propulsion Design Engineering Co-op - Spring 2027</v>
+        <v>Computational Design Engineer Co-Op - Spring 2027</v>
       </c>
       <c r="C251" t="str">
-        <v>Mechanical / Aerospace Engineering (Propulsion)</v>
+        <v>Mechanical / Computational Engineering</v>
       </c>
       <c r="D251" t="str">
         <v>Spring 2027</v>
@@ -9908,237 +9908,237 @@
         <v>$23-$30/hr</v>
       </c>
       <c r="H251" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/118</v>
+        <v>https://specteraerospace.bamboohr.com/careers/127</v>
       </c>
       <c r="I251" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'Propulsion Design Engineering Co-op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-08-13, title states 'Computational Design Engineer Co-Op - Spring 2027' verbatim.</v>
       </c>
       <c r="J251" t="str">
-        <v>Sibling/shared-pool req to Propulsion Test Engineering Co-Op above (same site, same applicant pool per posting text). Design, manufacturing, and test of ramjet/scramjet engine hardware. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>Reusable computational geometry models / implicit modeling (Rhino/Grasshopper, nTop, PicoGK) for high-speed airbreathing testbed vehicle design and analysis. Open to Engineering/Math/CS/Physics majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>Specter Aerospace</v>
+        <v>Shaw Industries</v>
       </c>
       <c r="B252" t="str">
-        <v>PLC/Controls Engineer Co-Op - Spring 2027</v>
+        <v>Engineering Internship/Co-op Spring 2027</v>
       </c>
       <c r="C252" t="str">
-        <v>Controls / Mechanical / Electrical Engineering</v>
+        <v>Manufacturing / Industrial Engineering</v>
       </c>
       <c r="D252" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E252" t="str">
-        <v>Peabody, MA</v>
+        <v>Dalton, GA</v>
       </c>
       <c r="F252">
-        <v>19</v>
+        <v>1050</v>
       </c>
       <c r="G252" t="str">
-        <v>$23-$30/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H252" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/123</v>
+        <v>https://shawinc.wd1.myworkdayjobs.com/en-US/External/job/Shaw-Plant-7C-2208-S-Hamilton-Street-Dalton-GA-30721-USA/Engineering-Internship-Co-op-Spring-2027_R-156324</v>
       </c>
       <c r="I252" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-09-01, title states 'PLC/Controls Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Shaw Industries' own Workday CXS API, req R-156324, title states 'Engineering Internship/Co-op Spring 2027' verbatim, posted 30+ days ago (exact date not disclosed by API).</v>
       </c>
       <c r="J252" t="str">
-        <v>PLC software design (Beckhoff/TwinCAT ecosystem), electrical control-panel design, sensor/actuator integration for the Specter engine test facility. Open to Computer/Electrical/Mechanical Engineering or CS majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>New company for the tracker — flooring manufacturer, wholly-owned Berkshire Hathaway subsidiary, $5B+ annual sales. Rotating or sequential semesters working onsite in Shaw's manufacturing operations facilities in an engineering capacity; student matched to a facility per skills/interests. Citizenship/GPA/eligibility not stated on posting — confirm directly.</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>Specter Aerospace</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B253" t="str">
-        <v>Computational Design Engineer Co-Op - Spring 2027</v>
+        <v>Operations &amp; Automation Engineering Co-op/Intern - Spring 2027</v>
       </c>
       <c r="C253" t="str">
-        <v>Mechanical / Computational Engineering</v>
+        <v>Controls / Automation / Industrial Engineering</v>
       </c>
       <c r="D253" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E253" t="str">
-        <v>Peabody, MA</v>
+        <v>Bartow, FL</v>
       </c>
       <c r="F253">
-        <v>19</v>
+        <v>1250</v>
       </c>
       <c r="G253" t="str">
-        <v>$23-$30/hr</v>
+        <v>Not stated on posting (housing/relocation available for qualified candidates)</v>
       </c>
       <c r="H253" t="str">
-        <v>https://specteraerospace.bamboohr.com/careers/127</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Bartow-FL/Operations---Automation-Engineering-Co-op-Intern---Spring-2027_64675-1</v>
       </c>
       <c r="I253" t="str">
-        <v>Yes — independently fetched directly via Specter's own BambooHR ATS API, status Open, posted 2026-08-13, title states 'Computational Design Engineer Co-Op - Spring 2027' verbatim.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64675, exact quote: 'Term Jan 11th, 2027 to April 23th, 2027 Full time Co-Op/Internship.'</v>
       </c>
       <c r="J253" t="str">
-        <v>Reusable computational geometry models / implicit modeling (Rhino/Grasshopper, nTop, PicoGK) for high-speed airbreathing testbed vehicle design and analysis. Open to Engineering/Math/CS/Physics majors. 4-6+ month cycle. REQUIRES U.S. Citizenship (must be eligible for U.S. Secret security clearance).</v>
+        <v>New company for the tracker — NYSE: MOS, world's leading integrated producer of concentrated phosphate and potash fertilizer. Supports plant operations and automated control systems (PLC, DCS, HMI/SCADA) at the Bartow, FL phosphoric-acid manufacturing site. Citizenship not stated on posting.</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>Shaw Industries</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B254" t="str">
-        <v>Engineering Internship/Co-op Spring 2027</v>
+        <v>Operations Engineering Co-op/Intern – Spring 2027</v>
       </c>
       <c r="C254" t="str">
-        <v>Manufacturing / Industrial Engineering</v>
+        <v>Mechanical / Industrial Engineering</v>
       </c>
       <c r="D254" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E254" t="str">
-        <v>Dalton, GA</v>
+        <v>Riverview, FL</v>
       </c>
       <c r="F254">
-        <v>1050</v>
+        <v>1250</v>
       </c>
       <c r="G254" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated on posting (relocation package available for qualified candidates)</v>
       </c>
       <c r="H254" t="str">
-        <v>https://shawinc.wd1.myworkdayjobs.com/en-US/External/job/Shaw-Plant-7C-2208-S-Hamilton-Street-Dalton-GA-30721-USA/Engineering-Internship-Co-op-Spring-2027_R-156324</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Riverview-FL/Operations-Engineering-Co-op-Intern---Spring-2027_64656</v>
       </c>
       <c r="I254" t="str">
-        <v>Yes — independently fetched directly via Shaw Industries' own Workday CXS API, req R-156324, title states 'Engineering Internship/Co-op Spring 2027' verbatim, posted 30+ days ago (exact date not disclosed by API).</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64656, exact quote: 'Term January 11 to April 23, 2027.'</v>
       </c>
       <c r="J254" t="str">
-        <v>New company for the tracker — flooring manufacturer, wholly-owned Berkshire Hathaway subsidiary, $5B+ annual sales. Rotating or sequential semesters working onsite in Shaw's manufacturing operations facilities in an engineering capacity; student matched to a facility per skills/interests. Citizenship/GPA/eligibility not stated on posting — confirm directly.</v>
+        <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>The Mosaic Company</v>
+        <v>Draper Laboratory</v>
       </c>
       <c r="B255" t="str">
-        <v>Operations &amp; Automation Engineering Co-op/Intern - Spring 2027</v>
+        <v>Mechanical Engineering &amp; System Packaging Co-Op (Spring 2027)</v>
       </c>
       <c r="C255" t="str">
-        <v>Controls / Automation / Industrial Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D255" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E255" t="str">
-        <v>Bartow, FL</v>
+        <v>Cambridge, MA</v>
       </c>
       <c r="F255">
-        <v>1250</v>
+        <v>3</v>
       </c>
       <c r="G255" t="str">
-        <v>Not stated on posting (housing/relocation available for qualified candidates)</v>
+        <v>$20.00–$45.00/hr per posting</v>
       </c>
       <c r="H255" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Bartow-FL/Operations---Automation-Engineering-Co-op-Intern---Spring-2027_64675-1</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Mechanical-Engineering---System-Packaging-Co-Op--Spring-2027-_JR002940</v>
       </c>
       <c r="I255" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64675, exact quote: 'Term Jan 11th, 2027 to April 23th, 2027 Full time Co-Op/Internship.'</v>
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002940), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
       </c>
       <c r="J255" t="str">
-        <v>New company for the tracker — NYSE: MOS, world's leading integrated producer of concentrated phosphate and potash fertilizer. Supports plant operations and automated control systems (PLC, DCS, HMI/SCADA) at the Bartow, FL phosphoric-acid manufacturing site. Citizenship not stated on posting.</v>
+        <v>US citizenship required (posting: 'Co-op students must be US citizens who are enrolled in an accredited engineering curriculum'). CAD (SolidWorks/Creo) and FEA (Ansys) work on national-security hardware.</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>The Mosaic Company</v>
+        <v>Draper Laboratory</v>
       </c>
       <c r="B256" t="str">
-        <v>Operations Engineering Co-op/Intern – Spring 2027</v>
+        <v>Digital Engineering – Requirements Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C256" t="str">
-        <v>Mechanical / Industrial Engineering</v>
+        <v>Systems Engineering</v>
       </c>
       <c r="D256" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E256" t="str">
-        <v>Riverview, FL</v>
+        <v>Lowell, MA</v>
       </c>
       <c r="F256">
-        <v>1250</v>
+        <v>30</v>
       </c>
       <c r="G256" t="str">
-        <v>Not stated on posting (relocation package available for qualified candidates)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H256" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/en-US/mosaic/job/US---Riverview-FL/Operations-Engineering-Co-op-Intern---Spring-2027_64656</v>
+        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Lowell-MA/Digital-Engineering---Requirements-Engineering-Co-Op--Spring-2027-_JR002944</v>
       </c>
       <c r="I256" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64656, exact quote: 'Term January 11 to April 23, 2027.'</v>
+        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002944), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
       </c>
       <c r="J256" t="str">
-        <v>Sibling req to the Bartow, FL Operations &amp; Automation Co-op above, same company, different site (Riverview Manufacturing Facility — sulfuric processing/production systems). Technical support to plant operations groups, mentored by Professional Engineers. Citizenship not stated on posting.</v>
+        <v>US Citizenship required per posting. Digital-twin/model-driven systems engineering support for strategic deterrent, missile-defense, hypersonic, space, and autonomous vehicle programs. Python scripting experience preferred.</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>Draper Laboratory</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B257" t="str">
-        <v>Mechanical Engineering &amp; System Packaging Co-Op (Spring 2027)</v>
+        <v>Process Engineer Co-Op/Intern - Spring 2027</v>
       </c>
       <c r="C257" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Chemical / Mining Engineering</v>
       </c>
       <c r="D257" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E257" t="str">
-        <v>Cambridge, MA</v>
+        <v>Bradley, FL</v>
       </c>
       <c r="F257">
-        <v>3</v>
+        <v>1250</v>
       </c>
       <c r="G257" t="str">
-        <v>$20.00–$45.00/hr per posting</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H257" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Cambridge-MA/Mechanical-Engineering---System-Packaging-Co-Op--Spring-2027-_JR002940</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Bradley-FL/Process-Engineer-Co-Op-Intern---Spring-2027_64450</v>
       </c>
       <c r="I257" t="str">
-        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002940), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64450, canApply true.</v>
       </c>
       <c r="J257" t="str">
-        <v>US citizenship required (posting: 'Co-op students must be US citizens who are enrolled in an accredited engineering curriculum'). CAD (SolidWorks/Creo) and FEA (Ansys) work on national-security hardware.</v>
+        <v>Posting explicitly accepts Chemical, Mechanical, and/or Mining Engineering majors. Term Jan 11–Apr 23, 2027 (same as tracker's other Mosaic co-ops). Citizenship not stated.</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>Draper Laboratory</v>
+        <v>The Mosaic Company</v>
       </c>
       <c r="B258" t="str">
-        <v>Digital Engineering – Requirements Engineering Co-Op (Spring 2027)</v>
+        <v>Capital Project Engineering Co-Op/Intern - Spring 2027</v>
       </c>
       <c r="C258" t="str">
-        <v>Systems Engineering</v>
+        <v>Mechanical / Chemical / Industrial Engineering</v>
       </c>
       <c r="D258" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E258" t="str">
-        <v>Lowell, MA</v>
+        <v>Riverview, FL</v>
       </c>
       <c r="F258">
-        <v>30</v>
+        <v>1250</v>
       </c>
       <c r="G258" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H258" t="str">
-        <v>https://draper.wd5.myworkdayjobs.com/Draper_Careers/job/Lowell-MA/Digital-Engineering---Requirements-Engineering-Co-Op--Spring-2027-_JR002944</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Riverview-FL/Capital-Project-Engineering-Co-Op-Intern---Spring-2027_64455</v>
       </c>
       <c r="I258" t="str">
-        <v>Yes — independently fetched directly via Draper's own Workday CXS job API (req JR002944), canApply true, postedOn 'Posted Today' as of 2026-09-30.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64455, canApply true.</v>
       </c>
       <c r="J258" t="str">
-        <v>US Citizenship required per posting. Digital-twin/model-driven systems engineering support for strategic deterrent, missile-defense, hypersonic, space, and autonomous vehicle programs. Python scripting experience preferred.</v>
+        <v>Posting explicitly accepts Chemical, Mechanical, or Industrial Engineer majors. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
       </c>
     </row>
     <row r="259">
@@ -10146,287 +10146,287 @@
         <v>The Mosaic Company</v>
       </c>
       <c r="B259" t="str">
-        <v>Process Engineer Co-Op/Intern - Spring 2027</v>
+        <v>Capital Project Engineering Co-op/Intern - Spring 2027</v>
       </c>
       <c r="C259" t="str">
-        <v>Mechanical / Chemical / Mining Engineering</v>
+        <v>Mechanical / Chemical / Industrial Engineering</v>
       </c>
       <c r="D259" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E259" t="str">
-        <v>Bradley, FL</v>
+        <v>Tampa, FL (Lithia area)</v>
       </c>
       <c r="F259">
-        <v>1250</v>
+        <v>1240</v>
       </c>
       <c r="G259" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H259" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Bradley-FL/Process-Engineer-Co-Op-Intern---Spring-2027_64450</v>
+        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Tampa-FL-Lithia-area/Capital-Project-Engineering-Co-op-Intern---Spring-2027_64392</v>
       </c>
       <c r="I259" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64450, canApply true.</v>
+        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64392, canApply true.</v>
       </c>
       <c r="J259" t="str">
-        <v>Posting explicitly accepts Chemical, Mechanical, and/or Mining Engineering majors. Term Jan 11–Apr 23, 2027 (same as tracker's other Mosaic co-ops). Citizenship not stated.</v>
+        <v>Sibling req to the Riverview, FL Capital Project Engineering Co-op above, same discipline, different site. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>The Mosaic Company</v>
+        <v>Gulfstream Aerospace</v>
       </c>
       <c r="B260" t="str">
-        <v>Capital Project Engineering Co-Op/Intern - Spring 2027</v>
+        <v>Spring 2027 - IEF - Stress Engineering - Collegiate Associate Intern</v>
       </c>
       <c r="C260" t="str">
-        <v>Mechanical / Chemical / Industrial Engineering</v>
+        <v>Aerospace / Structural Engineering</v>
       </c>
       <c r="D260" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E260" t="str">
-        <v>Riverview, FL</v>
+        <v>Savannah, GA</v>
       </c>
       <c r="F260">
-        <v>1250</v>
+        <v>900</v>
       </c>
       <c r="G260" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H260" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Riverview-FL/Capital-Project-Engineering-Co-Op-Intern---Spring-2027_64455</v>
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Stress-Engineering-Collegiate-Associate-Intern-GA-31401/1423681300/</v>
       </c>
       <c r="I260" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64455, canApply true.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Stress Engineering'.</v>
       </c>
       <c r="J260" t="str">
-        <v>Posting explicitly accepts Chemical, Mechanical, or Industrial Engineer majors. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+        <v>Discipline list per posting: Aerospace, Civil, Structural, Mechanical Engineering, Computer Science. GPA ≥3.0 cumulative (unrounded) required. No visa sponsorship — effectively requires US citizenship/permanent residency.</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>The Mosaic Company</v>
+        <v>Gulfstream Aerospace</v>
       </c>
       <c r="B261" t="str">
-        <v>Capital Project Engineering Co-op/Intern - Spring 2027</v>
+        <v>Spring 2027 - IEF - Materials and Processes Engineering College Associate</v>
       </c>
       <c r="C261" t="str">
-        <v>Mechanical / Chemical / Industrial Engineering</v>
+        <v>Materials Engineering</v>
       </c>
       <c r="D261" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E261" t="str">
-        <v>Tampa, FL (Lithia area)</v>
+        <v>Savannah, GA</v>
       </c>
       <c r="F261">
-        <v>1240</v>
+        <v>900</v>
       </c>
       <c r="G261" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H261" t="str">
-        <v>https://mosaic.wd5.myworkdayjobs.com/mosaic/job/US---Tampa-FL-Lithia-area/Capital-Project-Engineering-Co-op-Intern---Spring-2027_64392</v>
+        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Materials-and-Processes-Engineering-College-Associate-GA-31401/1432666200/</v>
       </c>
       <c r="I261" t="str">
-        <v>Yes — independently fetched directly via Mosaic's own Workday CXS API, req 64392, canApply true.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Materials and Processes'.</v>
       </c>
       <c r="J261" t="str">
-        <v>Sibling req to the Riverview, FL Capital Project Engineering Co-op above, same discipline, different site. Term Jan 11–Apr 23, 2027. Citizenship not stated.</v>
+        <v>Discipline list per posting: Mechanical, Materials Science &amp; Engineering, Materials Engineering, Aerospace, Chemical Engineering, Metallurgy. GPA ≥3.0 cumulative required. No visa sponsorship.</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Gulfstream Aerospace</v>
+        <v>Pyka</v>
       </c>
       <c r="B262" t="str">
-        <v>Spring 2027 - IEF - Stress Engineering - Collegiate Associate Intern</v>
+        <v>Mechanical Engineering Internship - Winter/Spring 2027 (Dropship, Early Interest)</v>
       </c>
       <c r="C262" t="str">
-        <v>Aerospace / Structural Engineering</v>
+        <v>Mechanical / Aerospace Engineering</v>
       </c>
       <c r="D262" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E262" t="str">
-        <v>Savannah, GA</v>
+        <v>Alameda, CA</v>
       </c>
       <c r="F262">
-        <v>900</v>
+        <v>2700</v>
       </c>
       <c r="G262" t="str">
-        <v>Not stated on posting</v>
+        <v>$35–$40/hr per posting</v>
       </c>
       <c r="H262" t="str">
-        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Stress-Engineering-Collegiate-Associate-Intern-GA-31401/1423681300/</v>
+        <v>https://jobs.lever.co/pyka/2702593a-7482-4d2b-93f3-ef97e2cf7df7</v>
       </c>
       <c r="I262" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Stress Engineering'.</v>
+        <v>Yes — independently fetched directly via Lever's public API, posting live, text confirms 'Winter/Spring 2027'.</v>
       </c>
       <c r="J262" t="str">
-        <v>Discipline list per posting: Aerospace, Civil, Structural, Mechanical Engineering, Computer Science. GPA ≥3.0 cumulative (unrounded) required. No visa sponsorship — effectively requires US citizenship/permanent residency.</v>
+        <v>IMPORTANT: explicitly an 'Early Interest Application' — posting states formal interviews for the 2027 cohort won't begin until October 2026; applying now only queues your profile for later review, not an active hiring process yet. Visa sponsorship offered. Electric-aviation 'Dropship' cargo aircraft program.</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>Gulfstream Aerospace</v>
+        <v>General Astronautics</v>
       </c>
       <c r="B263" t="str">
-        <v>Spring 2027 - IEF - Materials and Processes Engineering College Associate</v>
+        <v>Spring 2027 Mechanical Engineering Internship/Co-op</v>
       </c>
       <c r="C263" t="str">
-        <v>Materials Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D263" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E263" t="str">
-        <v>Savannah, GA</v>
+        <v>San Francisco, CA</v>
       </c>
       <c r="F263">
-        <v>900</v>
+        <v>2700</v>
       </c>
       <c r="G263" t="str">
-        <v>Not stated on posting</v>
+        <v>$30.00/hr (Sophomore), $35.00/hr (Junior/Senior) per posting</v>
       </c>
       <c r="H263" t="str">
-        <v>https://careers.gulfstream.com/job/Savannah-Spring-2027-IEF-Materials-and-Processes-Engineering-College-Associate-GA-31401/1432666200/</v>
+        <v>https://www.workatastartup.com/jobs/103200</v>
       </c>
       <c r="I263" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027' and 'Materials and Processes'.</v>
+        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027 Mechanical Engineering Internship/Co-op'; also cross-confirmed on ycombinator.com's own company page.</v>
       </c>
       <c r="J263" t="str">
-        <v>Discipline list per posting: Mechanical, Materials Science &amp; Engineering, Materials Engineering, Aerospace, Chemical Engineering, Metallurgy. GPA ≥3.0 cumulative required. No visa sponsorship.</v>
+        <v>New company for the tracker — YC-backed startup building autonomous robots for orbital manufacturing. Minimum 12 weeks on-site in San Francisco required. 'U.S. citizen or national, U.S. lawful permanent resident, or eligible for authorization under U.S. export regulations.' Applies via YC's own account/signup flow (workatastartup.com).</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>Pyka</v>
+        <v>Simpson Gumpertz &amp; Heger (SGH)</v>
       </c>
       <c r="B264" t="str">
-        <v>Mechanical Engineering Internship - Winter/Spring 2027 (Dropship, Early Interest)</v>
+        <v>Technical Co-Op, Structural Engineering</v>
       </c>
       <c r="C264" t="str">
-        <v>Mechanical / Aerospace Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D264" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E264" t="str">
-        <v>Alameda, CA</v>
+        <v>Waltham, MA</v>
       </c>
       <c r="F264">
-        <v>2700</v>
+        <v>10</v>
       </c>
       <c r="G264" t="str">
-        <v>$35–$40/hr per posting</v>
+        <v>$29.25–$38.25/hr depending on degree level, plus $1,000 sign-on bonus per posting</v>
       </c>
       <c r="H264" t="str">
-        <v>https://jobs.lever.co/pyka/2702593a-7482-4d2b-93f3-ef97e2cf7df7</v>
+        <v>https://www.sgh.com/careers/job-openings/view-job/8760874002?gh_jid=8760874002</v>
       </c>
       <c r="I264" t="str">
-        <v>Yes — independently fetched directly via Lever's public API, posting live, text confirms 'Winter/Spring 2027'.</v>
+        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: sgh.com's job board is embedded from Greenhouse; direct fetch of Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/simpsongumpertzheger/jobs/8760874002) independently confirmed title 'Technical Co-Op, Structural Engineering Spring 2027', Waltham MA, updated_at 2026-09-21, and body text 'seeking current students for a Winter 2027 Co-Op internship in our Waltham, MA office' plus the pay breakdown — a live-only feed, not an aggregator mirror.</v>
       </c>
       <c r="J264" t="str">
-        <v>IMPORTANT: explicitly an 'Early Interest Application' — posting states formal interviews for the 2027 cohort won't begin until October 2026; applying now only queues your profile for later review, not an active hiring process yet. Visa sponsorship offered. Electric-aviation 'Dropship' cargo aircraft program.</v>
+        <v>New company for the tracker — structural/civil engineering consultancy (also runs a sibling Technical Co-Op, Civil Engineering req and a Geotechnical Engineering Co-Op req at the same Waltham office — see `checked`, excluded on discipline-fit grounds). Fits Hamza's 'adjacent — structural' category. Posting itself uses both 'Winter 2027' (body) and 'Spring 2027' (title) — qualifies either way per the task's season rule.</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>General Astronautics</v>
+        <v>Cyvl</v>
       </c>
       <c r="B265" t="str">
-        <v>Spring 2027 Mechanical Engineering Internship/Co-op</v>
+        <v>Hardware Engineering Intern (Co-Op Spring 2027 / Intern Summer 2027)</v>
       </c>
       <c r="C265" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Hardware/Mechanical Engineering (sensor mounts/enclosures, CAD, machining)</v>
       </c>
       <c r="D265" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (Co-Op track; a separate Summer 2027 Intern track is also offered on the same posting)</v>
       </c>
       <c r="E265" t="str">
-        <v>San Francisco, CA</v>
+        <v>Somerville, MA</v>
       </c>
       <c r="F265">
-        <v>2700</v>
+        <v>3</v>
       </c>
       <c r="G265" t="str">
-        <v>$30.00/hr (Sophomore), $35.00/hr (Junior/Senior) per posting</v>
+        <v>Not confirmed on primary source</v>
       </c>
       <c r="H265" t="str">
-        <v>https://www.workatastartup.com/jobs/103200</v>
+        <v>https://jobs.ashbyhq.com/cyvl/3590960d-4d02-48bb-a335-cb82e121a01e</v>
       </c>
       <c r="I265" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, title tag and body confirm 'Spring 2027 Mechanical Engineering Internship/Co-op'; also cross-confirmed on ycombinator.com's own company page.</v>
+        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: Ashby publishes a public JSON API (api.ashbyhq.com/posting-api/job-board/cyvl); direct fetch independently confirmed isListed: true, publishedAt 2026-09-14, address Boston MA (primary)/Somerville MA (secondary), and body text 'This role is open as a Spring 2027 co-op or a Summer 2027 internship' — not an aggregator mirror.</v>
       </c>
       <c r="J265" t="str">
-        <v>New company for the tracker — YC-backed startup building autonomous robots for orbital manufacturing. Minimum 12 weeks on-site in San Francisco required. 'U.S. citizen or national, U.S. lawful permanent resident, or eligible for authorization under U.S. export regulations.' Applies via YC's own account/signup flow (workatastartup.com).</v>
+        <v>New company for the tracker — robotics/mapping hardware startup (sensor mounts/enclosures, CAD, machining for mobile-mapping hardware). Boston-metro (primary address is Boston, MA itself; Somerville MA listed as secondary). Season stated on the posting title itself as a dual Co-Op(Spring)/Intern(Summer) track; Spring 2027 Co-Op option is the qualifying track.</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>Simpson Gumpertz &amp; Heger (SGH)</v>
+        <v>Hydrite Chemical Co.</v>
       </c>
       <c r="B266" t="str">
-        <v>Technical Co-Op, Structural Engineering</v>
+        <v>Engineering Co-Op (Spring 2027)</v>
       </c>
       <c r="C266" t="str">
-        <v>Structural Engineering</v>
+        <v>Mechanical/Chemical Engineering</v>
       </c>
       <c r="D266" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E266" t="str">
-        <v>Waltham, MA</v>
+        <v>Lubbock, TX</v>
       </c>
       <c r="F266">
-        <v>10</v>
+        <v>1780</v>
       </c>
       <c r="G266" t="str">
-        <v>$29.25–$38.25/hr depending on degree level, plus $1,000 sign-on bonus per posting</v>
+        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
       </c>
       <c r="H266" t="str">
-        <v>https://www.sgh.com/careers/job-openings/view-job/8760874002?gh_jid=8760874002</v>
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8173754</v>
       </c>
       <c r="I266" t="str">
-        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: sgh.com's job board is embedded from Greenhouse; direct fetch of Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/simpsongumpertzheger/jobs/8760874002) independently confirmed title 'Technical Co-Op, Structural Engineering Spring 2027', Waltham MA, updated_at 2026-09-21, and body text 'seeking current students for a Winter 2027 Co-Op internship in our Waltham, MA office' plus the pay breakdown — a live-only feed, not an aggregator mirror.</v>
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8173754), which only lists currently-open postings. Body quote: 'This position will run full-time from January - August 2027.' Degree preference: 'Mechanical or Chemical.'</v>
       </c>
       <c r="J266" t="str">
-        <v>New company for the tracker — structural/civil engineering consultancy (also runs a sibling Technical Co-Op, Civil Engineering req and a Geotechnical Engineering Co-Op req at the same Waltham office — see `checked`, excluded on discipline-fit grounds). Fits Hamza's 'adjacent — structural' category. Posting itself uses both 'Winter 2027' (body) and 'Spring 2027' (title) — qualifies either way per the task's season rule.</v>
+        <v>New company for the tracker — industrial/specialty chemical manufacturer. No citizenship/ITAR language observed on posting.</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>Cyvl</v>
+        <v>Hydrite Chemical Co.</v>
       </c>
       <c r="B267" t="str">
-        <v>Hardware Engineering Intern (Co-Op Spring 2027 / Intern Summer 2027)</v>
+        <v>Engineering Co-Op Spring 2027</v>
       </c>
       <c r="C267" t="str">
-        <v>Hardware/Mechanical Engineering (sensor mounts/enclosures, CAD, machining)</v>
+        <v>Mechanical/Industrial/Chemical Engineering</v>
       </c>
       <c r="D267" t="str">
-        <v>Spring 2027 (Co-Op track; a separate Summer 2027 Intern track is also offered on the same posting)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E267" t="str">
-        <v>Somerville, MA</v>
+        <v>Brookfield, WI</v>
       </c>
       <c r="F267">
-        <v>3</v>
+        <v>990</v>
       </c>
       <c r="G267" t="str">
-        <v>Not confirmed on primary source</v>
+        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
       </c>
       <c r="H267" t="str">
-        <v>https://jobs.ashbyhq.com/cyvl/3590960d-4d02-48bb-a335-cb82e121a01e</v>
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8179653</v>
       </c>
       <c r="I267" t="str">
-        <v>Yes — UPGRADED 2026-09-30 ~13:00 UTC from Partial: Ashby publishes a public JSON API (api.ashbyhq.com/posting-api/job-board/cyvl); direct fetch independently confirmed isListed: true, publishedAt 2026-09-14, address Boston MA (primary)/Somerville MA (secondary), and body text 'This role is open as a Spring 2027 co-op or a Summer 2027 internship' — not an aggregator mirror.</v>
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8179653), which only lists currently-open postings. Body quote: 'This role will run from January 2027- End of Summer 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
       </c>
       <c r="J267" t="str">
-        <v>New company for the tracker — robotics/mapping hardware startup (sensor mounts/enclosures, CAD, machining for mobile-mapping hardware). Boston-metro (primary address is Boston, MA itself; Somerville MA listed as secondary). Season stated on the posting title itself as a dual Co-Op(Spring)/Intern(Summer) track; Spring 2027 Co-Op option is the qualifying track.</v>
+        <v>New company for the tracker. A distinct sibling req at the same site, titled 'Engineering Co-Op (Fall 2027)' (ID 8179630), is Fall-2027-only and excluded.</v>
       </c>
     </row>
     <row r="268">
@@ -10434,511 +10434,511 @@
         <v>Hydrite Chemical Co.</v>
       </c>
       <c r="B268" t="str">
-        <v>Engineering Co-Op (Spring 2027)</v>
+        <v>Engineering Co-Op (Spring OR Fall 2027)</v>
       </c>
       <c r="C268" t="str">
-        <v>Mechanical/Chemical Engineering</v>
+        <v>Mechanical/Industrial/Chemical Engineering</v>
       </c>
       <c r="D268" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (dual Spring/Fall 2027 track; Spring option qualifies)</v>
       </c>
       <c r="E268" t="str">
-        <v>Lubbock, TX</v>
+        <v>Cottage Grove, WI</v>
       </c>
       <c r="F268">
-        <v>1780</v>
+        <v>990</v>
       </c>
       <c r="G268" t="str">
         <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
       </c>
       <c r="H268" t="str">
-        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8173754</v>
+        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8185948</v>
       </c>
       <c r="I268" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8173754), which only lists currently-open postings. Body quote: 'This position will run full-time from January - August 2027.' Degree preference: 'Mechanical or Chemical.'</v>
+        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8185948), which only lists currently-open postings. Body quote: 'This position is able to run full-time from January - August 2027 OR May/June 2027-December 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
       </c>
       <c r="J268" t="str">
-        <v>New company for the tracker — industrial/specialty chemical manufacturer. No citizenship/ITAR language observed on posting.</v>
+        <v>New company for the tracker.</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>Hydrite Chemical Co.</v>
+        <v>Buro Happold</v>
       </c>
       <c r="B269" t="str">
-        <v>Engineering Co-Op Spring 2027</v>
+        <v>Structural Co-op - Boston - Spring 2027</v>
       </c>
       <c r="C269" t="str">
-        <v>Mechanical/Industrial/Chemical Engineering</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D269" t="str">
         <v>Spring 2027</v>
       </c>
       <c r="E269" t="str">
-        <v>Brookfield, WI</v>
+        <v>Boston, MA</v>
       </c>
       <c r="F269">
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="G269" t="str">
-        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
+        <v>$24–$34/hr per posting</v>
       </c>
       <c r="H269" t="str">
-        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8179653</v>
+        <v>https://vacancies.burohappold.com/jobs/job/Structural-Coop-Boston-Spring-2027/2464</v>
       </c>
       <c r="I269" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8179653), which only lists currently-open postings. Body quote: 'This role will run from January 2027- End of Summer 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
+        <v>Yes — independently fetched directly, HTTP 200, page confirms 'Structural Co-op' title, 'Spring 2027', '$24 to $34' pay, and 'No expiry' status on the posting itself.</v>
       </c>
       <c r="J269" t="str">
-        <v>New company for the tracker. A distinct sibling req at the same site, titled 'Engineering Co-Op (Fall 2027)' (ID 8179630), is Fall-2027-only and excluded.</v>
+        <v>New req at an already-tracked employer (sibling to the already-tracked Mechanical Co-op, job 2462, and the excluded Plumbing &amp; Fire Protection Co-op, job 2463). Fits Hamza's 'adjacent — structural' category.</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>Hydrite Chemical Co.</v>
+        <v>Insulet</v>
       </c>
       <c r="B270" t="str">
-        <v>Engineering Co-Op (Spring OR Fall 2027)</v>
+        <v>Co-op, Quality Engineering: January-June (Onsite)</v>
       </c>
       <c r="C270" t="str">
-        <v>Mechanical/Industrial/Chemical Engineering</v>
+        <v>Quality Engineering (Lean Manufacturing / Six Sigma)</v>
       </c>
       <c r="D270" t="str">
-        <v>Spring 2027 (dual Spring/Fall 2027 track; Spring option qualifies)</v>
+        <v>Spring 2027 (Jan 11 – Jun 30, 2027)</v>
       </c>
       <c r="E270" t="str">
-        <v>Cottage Grove, WI</v>
+        <v>Acton, MA</v>
       </c>
       <c r="F270">
-        <v>990</v>
+        <v>25</v>
       </c>
       <c r="G270" t="str">
-        <v>Not numerically stated on posting (lists 'Competitive pay' as a benefit)</v>
+        <v>$25.00–$34.00/hr (Massachusetts-based positions per posting)</v>
       </c>
       <c r="H270" t="str">
-        <v>https://job-boards.greenhouse.io/hydritechemicalco/jobs/8185948</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Quality-Engineering--January-June--Onsite-_REQ-2026-18150</v>
       </c>
       <c r="I270" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own public API (boards-api.greenhouse.io/v1/boards/hydritechemicalco/jobs/8185948), which only lists currently-open postings. Body quote: 'This position is able to run full-time from January - August 2027 OR May/June 2027-December 2027.' Degree preference: 'Mechanical, Industrial, or Chemical.'</v>
+        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, req REQ-2026-18150, endDate 2026-12-31, body quote: 'Position Dates: January 11, 2027 – June 30, 2027' and 'Availability for the Co-op duration Spring: January – June 2027.'</v>
       </c>
       <c r="J270" t="str">
-        <v>New company for the tracker.</v>
+        <v>New req at an already-tracked employer — sibling to Insulet's other already-tracked Acton, MA Jan-June 2027 engineering co-ops. Medical device (insulin pump) manufacturer; not eligible for visa sponsorship per company-wide postings.</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>Buro Happold</v>
+        <v>Keurig Dr Pepper</v>
       </c>
       <c r="B271" t="str">
-        <v>Structural Co-op - Boston - Spring 2027</v>
+        <v>Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)</v>
       </c>
       <c r="C271" t="str">
-        <v>Structural Engineering</v>
+        <v>Mechanical/Appliance Engineering (also accepts SW/EE/IE)</v>
       </c>
       <c r="D271" t="str">
-        <v>Spring 2027</v>
+        <v>Winter 2027</v>
       </c>
       <c r="E271" t="str">
-        <v>Boston, MA</v>
+        <v>Burlington, MA</v>
       </c>
       <c r="F271">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G271" t="str">
-        <v>$24–$34/hr per posting</v>
+        <v>$31/hr + $5,000 sign-on bonus per posting</v>
       </c>
       <c r="H271" t="str">
-        <v>https://vacancies.burohappold.com/jobs/job/Structural-Coop-Boston-Spring-2027/2464</v>
+        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-appliance-engineering-me-sw-ee-ie/42849/100035469424</v>
       </c>
       <c r="I271" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, page confirms 'Structural Co-op' title, 'Spring 2027', '$24 to $34' pay, and 'No expiry' status on the posting itself.</v>
+        <v>Yes — independently fetched directly, HTTP 200, page confirms title 'Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)', '$31/hour', and sign-on bonus language.</v>
       </c>
       <c r="J271" t="str">
-        <v>New req at an already-tracked employer (sibling to the already-tracked Mechanical Co-op, job 2462, and the excluded Plumbing &amp; Fire Protection Co-op, job 2463). Fits Hamza's 'adjacent — structural' category.</v>
+        <v>New company for the tracker — Burlington, MA HQ (Boston-area). Company-wide program note: 'The KDP 2027 Winter Co-op Program will run from January 4 – May 21, 2027.' Mechanical Engineering is among the accepted majors.</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>Insulet</v>
+        <v>Keurig Dr Pepper</v>
       </c>
       <c r="B272" t="str">
-        <v>Co-op, Quality Engineering: January-June (Onsite)</v>
+        <v>Winter 2027 Co-op - Mechanical Test and Reliability</v>
       </c>
       <c r="C272" t="str">
-        <v>Quality Engineering (Lean Manufacturing / Six Sigma)</v>
+        <v>Mechanical Engineering (Test &amp; Reliability)</v>
       </c>
       <c r="D272" t="str">
-        <v>Spring 2027 (Jan 11 – Jun 30, 2027)</v>
+        <v>Winter 2027</v>
       </c>
       <c r="E272" t="str">
-        <v>Acton, MA</v>
+        <v>Burlington, MA</v>
       </c>
       <c r="F272">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G272" t="str">
-        <v>$25.00–$34.00/hr (Massachusetts-based positions per posting)</v>
+        <v>$31/hr + sign-on bonus per posting</v>
       </c>
       <c r="H272" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op--Quality-Engineering--January-June--Onsite-_REQ-2026-18150</v>
+        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-mechanical-test-and-reliability/42849/99763826160</v>
       </c>
       <c r="I272" t="str">
-        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, req REQ-2026-18150, endDate 2026-12-31, body quote: 'Position Dates: January 11, 2027 – June 30, 2027' and 'Availability for the Co-op duration Spring: January – June 2027.'</v>
+        <v>Yes — independently fetched directly (note: the job-ID-only URL redirects to the homepage; the correct URL includes a job-family segment, confirmed via Keurig Dr Pepper's own search-results endpoint), HTTP 200, page confirms title 'Winter 2027 Co-op - Mechanical Test and Reliability', '$31/hour', and sign-on bonus language.</v>
       </c>
       <c r="J272" t="str">
-        <v>New req at an already-tracked employer — sibling to Insulet's other already-tracked Acton, MA Jan-June 2027 engineering co-ops. Medical device (insulin pump) manufacturer; not eligible for visa sponsorship per company-wide postings.</v>
+        <v>New company for the tracker — sibling req to the Appliance Engineering co-op above, same Burlington MA site and Winter 2027 program. A distinct Fall-2027-only sibling (job 99763826384) exists and is excluded on season grounds.</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>Keurig Dr Pepper</v>
+        <v>Apex Technology, Inc. (Apex Space)</v>
       </c>
       <c r="B273" t="str">
-        <v>Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)</v>
+        <v>Avionics Test Engineering Internship (Spring 2027)</v>
       </c>
       <c r="C273" t="str">
-        <v>Mechanical/Appliance Engineering (also accepts SW/EE/IE)</v>
+        <v>Avionics / Flight Systems Test Engineering</v>
       </c>
       <c r="D273" t="str">
-        <v>Winter 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E273" t="str">
-        <v>Burlington, MA</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F273">
-        <v>15</v>
+        <v>2600</v>
       </c>
       <c r="G273" t="str">
-        <v>$31/hr + $5,000 sign-on bonus per posting</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H273" t="str">
-        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-appliance-engineering-me-sw-ee-ie/42849/100035469424</v>
+        <v>https://jobs.ashbyhq.com/apex-technology-inc/aea24b77-7673-4478-83af-4f16f5337673</v>
       </c>
       <c r="I273" t="str">
-        <v>Yes — independently fetched directly, HTTP 200, page confirms title 'Winter 2027 Co-op - Appliance Engineering (ME,SW,EE,IE)', '$31/hour', and sign-on bonus language.</v>
+        <v>Yes — independently fetched directly via Apex's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/apex-technology-inc), isListed true, title states 'Spring 2027' verbatim, posted 2026-09-09.</v>
       </c>
       <c r="J273" t="str">
-        <v>New company for the tracker — Burlington, MA HQ (Boston-area). Company-wide program note: 'The KDP 2027 Winter Co-op Program will run from January 4 – May 21, 2027.' Mechanical Engineering is among the accepted majors.</v>
+        <v>New company for the tracker. Apex manufactures satellite buses at scale (spacecraft platform manufacturer). Role is on the Avionics team's test/integration side — flight-systems-adjacent discipline.</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>Keurig Dr Pepper</v>
+        <v>Apex Technology, Inc. (Apex Space)</v>
       </c>
       <c r="B274" t="str">
-        <v>Winter 2027 Co-op - Mechanical Test and Reliability</v>
+        <v>Thermal Engineering Internship (Spring or Summer 2027)</v>
       </c>
       <c r="C274" t="str">
-        <v>Mechanical Engineering (Test &amp; Reliability)</v>
+        <v>Thermal / Mechanical Engineering</v>
       </c>
       <c r="D274" t="str">
-        <v>Winter 2027</v>
+        <v>Spring or Summer 2027 (posting offers either term)</v>
       </c>
       <c r="E274" t="str">
-        <v>Burlington, MA</v>
+        <v>Los Angeles, CA</v>
       </c>
       <c r="F274">
-        <v>15</v>
+        <v>2600</v>
       </c>
       <c r="G274" t="str">
-        <v>$31/hr + sign-on bonus per posting</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H274" t="str">
-        <v>https://careers.keurigdrpepper.com/en/job/burlington/winter-2027-co-op-mechanical-test-and-reliability/42849/99763826160</v>
+        <v>https://jobs.ashbyhq.com/apex-technology-inc/56b018ce-915d-4ebd-9833-c8ebb160b09a</v>
       </c>
       <c r="I274" t="str">
-        <v>Yes — independently fetched directly (note: the job-ID-only URL redirects to the homepage; the correct URL includes a job-family segment, confirmed via Keurig Dr Pepper's own search-results endpoint), HTTP 200, page confirms title 'Winter 2027 Co-op - Mechanical Test and Reliability', '$31/hour', and sign-on bonus language.</v>
+        <v>Yes — independently fetched directly via Apex's own Ashby posting-api, isListed true, title states 'Spring or Summer 2027' verbatim, posted 2026-09-04.</v>
       </c>
       <c r="J274" t="str">
-        <v>New company for the tracker — sibling req to the Appliance Engineering co-op above, same Burlington MA site and Winter 2027 program. A distinct Fall-2027-only sibling (job 99763826384) exists and is excluded on season grounds.</v>
+        <v>Same company as above. Posting explicitly offers Spring 2027 as one of two term options (not Summer-only) — qualifies per the tracker's season rule. Confirm preferred term (Spring) during application.</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>Apex Technology, Inc. (Apex Space)</v>
+        <v>Layup Parts</v>
       </c>
       <c r="B275" t="str">
-        <v>Avionics Test Engineering Internship (Spring 2027)</v>
+        <v>Manufacturing Engineer Intern</v>
       </c>
       <c r="C275" t="str">
-        <v>Avionics / Flight Systems Test Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D275" t="str">
-        <v>Spring 2027</v>
+        <v>Rolling — explicitly includes Winter and Spring 2027 per posting text</v>
       </c>
       <c r="E275" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Huntington Beach, CA</v>
       </c>
       <c r="F275">
         <v>2600</v>
       </c>
       <c r="G275" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated on posting (aggregator-cited ~$25/hr, unconfirmed on primary source)</v>
       </c>
       <c r="H275" t="str">
-        <v>https://jobs.ashbyhq.com/apex-technology-inc/aea24b77-7673-4478-83af-4f16f5337673</v>
+        <v>https://jobs.lever.co/layup/4522257e-bac4-4937-b0b0-88d7ebbb6583</v>
       </c>
       <c r="I275" t="str">
-        <v>Yes — independently fetched directly via Apex's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/apex-technology-inc), isListed true, title states 'Spring 2027' verbatim, posted 2026-09-09.</v>
+        <v>Yes — independently fetched directly via Lever's own postings API (api.lever.co/v0/postings/layup), job live among current postings, description quote: 'Whether you're looking for a Fall, Winter, Spring, or Summer internship, we're accepting applications on a rolling basis.'</v>
       </c>
       <c r="J275" t="str">
-        <v>New company for the tracker. Apex manufactures satellite buses at scale (spacecraft platform manufacturer). Role is on the Avionics team's test/integration side — flight-systems-adjacent discipline.</v>
+        <v>New company — composites manufacturing technology (CNC machining, 3D printing, advanced manufacturing) serving aerospace/defense/robotics customers. ITAR-restricted: applicant must be a U.S. citizen/national, lawful permanent resident, refugee, or asylee, or independently eligible for State Dept. authorization.</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>Apex Technology, Inc. (Apex Space)</v>
+        <v>NDimensions Labs</v>
       </c>
       <c r="B276" t="str">
-        <v>Thermal Engineering Internship (Spring or Summer 2027)</v>
+        <v>Hardware &amp; Electronics Intern, Robotics</v>
       </c>
       <c r="C276" t="str">
-        <v>Thermal / Mechanical Engineering</v>
+        <v>Robotics Hardware / Mechatronics</v>
       </c>
       <c r="D276" t="str">
-        <v>Spring or Summer 2027 (posting offers either term)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E276" t="str">
-        <v>Los Angeles, CA</v>
+        <v>Boston, MA</v>
       </c>
       <c r="F276">
-        <v>2600</v>
+        <v>0</v>
       </c>
       <c r="G276" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H276" t="str">
-        <v>https://jobs.ashbyhq.com/apex-technology-inc/56b018ce-915d-4ebd-9833-c8ebb160b09a</v>
+        <v>https://ndimensions.xyz/careers/hardware_intern</v>
       </c>
       <c r="I276" t="str">
-        <v>Yes — independently fetched directly via Apex's own Ashby posting-api, isListed true, title states 'Spring or Summer 2027' verbatim, posted 2026-09-04.</v>
+        <v>Yes — fetched directly, page live, title 'Hardware &amp; Electronics Intern, Robotics', subtitle states 'Spring 2027 internship (Full-time) • Boston, MA' verbatim.</v>
       </c>
       <c r="J276" t="str">
-        <v>Same company as above. Posting explicitly offers Spring 2027 as one of two term options (not Summer-only) — qualifies per the tracker's season rule. Confirm preferred term (Spring) during application.</v>
+        <v>New company — early-stage startup (founders from MIT, U. Waterloo, U. Washington) building robotics/embodied-AI hardware infrastructure. Role covers mechanical/electromechanical component design, PCB/sensor/actuator assembly and testing. Small/early-stage company — flagging maturity as a factor for Hamza to weigh, but the listing itself is directly verified and legitimate.</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>Layup Parts</v>
+        <v>MORSE Corp</v>
       </c>
       <c r="B277" t="str">
-        <v>Manufacturing Engineer Intern</v>
+        <v>Mechanical Engineer Co-op</v>
       </c>
       <c r="C277" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering / Flight Systems (UAV)</v>
       </c>
       <c r="D277" t="str">
-        <v>Rolling — explicitly includes Winter and Spring 2027 per posting text</v>
+        <v>Spring 2027 (Jan–Jun/Aug 2027 per co-op board description)</v>
       </c>
       <c r="E277" t="str">
-        <v>Huntington Beach, CA</v>
+        <v>Cambridge, MA</v>
       </c>
       <c r="F277">
-        <v>2600</v>
+        <v>0</v>
       </c>
       <c r="G277" t="str">
-        <v>Not stated on posting (aggregator-cited ~$25/hr, unconfirmed on primary source)</v>
+        <v>$27–$33/hr</v>
       </c>
       <c r="H277" t="str">
-        <v>https://jobs.lever.co/layup/4522257e-bac4-4937-b0b0-88d7ebbb6583</v>
+        <v>https://job-boards.greenhouse.io/morsecorpcoop/jobs/7968311003</v>
       </c>
       <c r="I277" t="str">
-        <v>Yes — independently fetched directly via Lever's own postings API (api.lever.co/v0/postings/layup), job live among current postings, description quote: 'Whether you're looking for a Fall, Winter, Spring, or Summer internship, we're accepting applications on a rolling basis.'</v>
+        <v>Yes — independently fetched directly via Greenhouse's own public API (api.greenhouse.io/v1/boards/morsecorpcoop/jobs/7968311003) and the board landing page, which states verbatim 'Welcome to MORSE Corp's Co-op Opportunities for the Spring 2027 Semester!' Job listed live, requisition 342.</v>
       </c>
       <c r="J277" t="str">
-        <v>New company — composites manufacturing technology (CNC machining, 3D printing, advanced manufacturing) serving aerospace/defense/robotics customers. ITAR-restricted: applicant must be a U.S. citizen/national, lawful permanent resident, refugee, or asylee, or independently eligible for State Dept. authorization.</v>
+        <v>New company — employee-owned small defense-tech firm (Cambridge MA / Arlington VA / Seattle WA) building UAVs, autonomous vehicles, and mission systems for the US national security ecosystem. Role: designing, building, and flight-testing UAV prototypes, mechatronics/robotics, rapid prototyping (3D printing/CNC/laser cutting), SolidWorks/Altium. On-site 5 days/week. Requires US citizenship and ability to obtain a US security clearance.</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>NDimensions Labs</v>
+        <v>Marotta Controls, Inc.</v>
       </c>
       <c r="B278" t="str">
-        <v>Hardware &amp; Electronics Intern, Robotics</v>
+        <v>Spring 2027 Mechanical Engineering Internship/Co-Op</v>
       </c>
       <c r="C278" t="str">
-        <v>Robotics Hardware / Mechatronics</v>
+        <v>Mechanical / Aerospace / Materials Engineering</v>
       </c>
       <c r="D278" t="str">
-        <v>Spring 2027</v>
+        <v>Spring 2027 (with option to continue into Summer 2027)</v>
       </c>
       <c r="E278" t="str">
-        <v>Boston, MA</v>
+        <v>Parsippany, NJ</v>
       </c>
       <c r="F278">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="G278" t="str">
-        <v>Not stated on posting</v>
+        <v>$18–$24/hr</v>
       </c>
       <c r="H278" t="str">
-        <v>https://ndimensions.xyz/careers/hardware_intern</v>
+        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a061fa5de22f3c</v>
       </c>
       <c r="I278" t="str">
-        <v>Yes — fetched directly, page live, title 'Hardware &amp; Electronics Intern, Robotics', subtitle states 'Spring 2027 internship (Full-time) • Boston, MA' verbatim.</v>
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, Apply button present, title and body state 'Spring 2027 Mechanical Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live again — the previously-stated 'Deadline: October 1, 2026' text no longer appears anywhere on the current live page; posting now reads 'beginning January 2027 through end of summer 2027' with no deadline language at all, and pay ($18-24/hr) is now visible.</v>
       </c>
       <c r="J278" t="str">
-        <v>New company — early-stage startup (founders from MIT, U. Waterloo, U. Washington) building robotics/embodied-AI hardware infrastructure. Role covers mechanical/electromechanical component design, PCB/sensor/actuator assembly and testing. Small/early-stage company — flagging maturity as a factor for Hamza to weigh, but the listing itself is directly verified and legitimate.</v>
+        <v>New company — defense/aerospace motion &amp; flow control systems manufacturer. Design/production/quality/test-development work, 3D CAD (Pro-E/Creo). US citizenship required (ITAR). The Oct 1, 2026 deadline previously stated on this posting has since been removed from the live page (re-checked 2026-10-02) — appears to remain open past that date.</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>MORSE Corp</v>
+        <v>Marotta Controls, Inc.</v>
       </c>
       <c r="B279" t="str">
-        <v>Mechanical Engineer Co-op</v>
+        <v>Spring 2027 Control Systems Engineering Internship/Co-Op</v>
       </c>
       <c r="C279" t="str">
-        <v>Mechanical Engineering / Flight Systems (UAV)</v>
+        <v>Controls Engineering</v>
       </c>
       <c r="D279" t="str">
-        <v>Spring 2027 (Jan–Jun/Aug 2027 per co-op board description)</v>
+        <v>Spring 2027 (with option to continue into Summer 2027)</v>
       </c>
       <c r="E279" t="str">
-        <v>Cambridge, MA</v>
+        <v>Parsippany, NJ</v>
       </c>
       <c r="F279">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="G279" t="str">
-        <v>$27–$33/hr</v>
+        <v>$18–$24/hr</v>
       </c>
       <c r="H279" t="str">
-        <v>https://job-boards.greenhouse.io/morsecorpcoop/jobs/7968311003</v>
+        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a062229f2536d0</v>
       </c>
       <c r="I279" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own public API (api.greenhouse.io/v1/boards/morsecorpcoop/jobs/7968311003) and the board landing page, which states verbatim 'Welcome to MORSE Corp's Co-op Opportunities for the Spring 2027 Semester!' Job listed live, requisition 342.</v>
+        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, title and body state 'Spring 2027 Control Systems Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live, same deadline-text removal as the Mechanical Engineering sibling above.</v>
       </c>
       <c r="J279" t="str">
-        <v>New company — employee-owned small defense-tech firm (Cambridge MA / Arlington VA / Seattle WA) building UAVs, autonomous vehicles, and mission systems for the US national security ecosystem. Role: designing, building, and flight-testing UAV prototypes, mechatronics/robotics, rapid prototyping (3D printing/CNC/laser cutting), SolidWorks/Altium. On-site 5 days/week. Requires US citizenship and ability to obtain a US security clearance.</v>
+        <v>Same company as above. MATLAB control-system simulation/modeling, requirements management in IBM DOORS, systems engineering deliverables. US citizenship required (ITAR). The previously-stated Oct 1, 2026 deadline is gone from the live posting as of 2026-10-02 — appears to remain open.</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>Marotta Controls, Inc.</v>
+        <v>1X Technologies</v>
       </c>
       <c r="B280" t="str">
-        <v>Spring 2027 Mechanical Engineering Internship/Co-Op</v>
+        <v>Internship - Manufacturing Engineering</v>
       </c>
       <c r="C280" t="str">
-        <v>Mechanical / Aerospace / Materials Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D280" t="str">
-        <v>Spring 2027 (with option to continue into Summer 2027)</v>
+        <v>Starting January 2027 (posting's own wording — does not use the literal word 'Spring' or 'Winter', but the explicit January 2027 start date places it inside Hamza's target window)</v>
       </c>
       <c r="E280" t="str">
-        <v>Parsippany, NJ</v>
+        <v>San Carlos, CA</v>
       </c>
       <c r="F280">
-        <v>210</v>
+        <v>2700</v>
       </c>
       <c r="G280" t="str">
-        <v>$18–$24/hr</v>
+        <v>$35/hr + $2,500/month housing stipend for relocation</v>
       </c>
       <c r="H280" t="str">
-        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a061fa5de22f3c</v>
+        <v>https://jobs.ashbyhq.com/1x/d687b375-8136-4e6f-baa6-369b89366050</v>
       </c>
       <c r="I280" t="str">
-        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, Apply button present, title and body state 'Spring 2027 Mechanical Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live again — the previously-stated 'Deadline: October 1, 2026' text no longer appears anywhere on the current live page; posting now reads 'beginning January 2027 through end of summer 2027' with no deadline language at all, and pay ($18-24/hr) is now visible.</v>
+        <v>Yes — independently fetched directly via Ashby's own posting-api (api.ashbyhq.com/posting-api/job-board/1x), isListed true, title 'Internship - Manufacturing Engineering', body states 'INTERNSHIP SEASON - STARTING JANUARY 2027' verbatim, published 2026-09-14.</v>
       </c>
       <c r="J280" t="str">
-        <v>New company — defense/aerospace motion &amp; flow control systems manufacturer. Design/production/quality/test-development work, 3D CAD (Pro-E/Creo). US citizenship required (ITAR). The Oct 1, 2026 deadline previously stated on this posting has since been removed from the live page (re-checked 2026-10-02) — appears to remain open past that date.</v>
+        <v>New company — humanoid robotics manufacturer (maker of the 'NEO' home robot). Role: manufacturing process/fixture design, CAD (SolidWorks/Onshape), design-for-manufacturability for robot hardware. A sibling 'Internship - CNC Machine Park' (Hayward, CA) role exists but states no season/year and was excluded.</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>Marotta Controls, Inc.</v>
+        <v>Lexington Medical, Inc.</v>
       </c>
       <c r="B281" t="str">
-        <v>Spring 2027 Control Systems Engineering Internship/Co-Op</v>
+        <v>Mechanical Engineering Co-Op</v>
       </c>
       <c r="C281" t="str">
-        <v>Controls Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D281" t="str">
-        <v>Spring 2027 (with option to continue into Summer 2027)</v>
+        <v>January 2027 – June 2027 (Spring 2027)</v>
       </c>
       <c r="E281" t="str">
-        <v>Parsippany, NJ</v>
+        <v>Bedford, MA</v>
       </c>
       <c r="F281">
-        <v>210</v>
+        <v>17</v>
       </c>
       <c r="G281" t="str">
-        <v>$18–$24/hr</v>
+        <v>$28.00–$34.00/hr (pay-transparency widget shows $28–$36)</v>
       </c>
       <c r="H281" t="str">
-        <v>https://recruitingbypaycor.com/career/JobIntroduction.action?clientId=8a5814f64501d24801450494d56567cb&amp;id=8a7883a8a03fc28901a062229f2536d0</v>
+        <v>https://job-boards.greenhouse.io/lexingtonmedical/jobs/5423105008</v>
       </c>
       <c r="I281" t="str">
-        <v>Yes — independently fetched directly via Marotta's own Paycor ATS page, HTTP 200, title and body state 'Spring 2027 Control Systems Engineering Internship/Co-Op' and 'Spring 2027 with the opportunity to continue into Summer 2027' verbatim. 2026-10-02: re-confirmed live, same deadline-text removal as the Mechanical Engineering sibling above.</v>
+        <v>Yes — independently fetched directly via Greenhouse's own board API (boards-api.greenhouse.io/v1/boards/lexingtonmedical/jobs/5423105008), job live, updated_at 2026-09-30, body states 'The co-op runs full-time, five days per week, from January 2027 through June 2027.' verbatim.</v>
       </c>
       <c r="J281" t="str">
-        <v>Same company as above. MATLAB control-system simulation/modeling, requirements management in IBM DOORS, systems engineering deliverables. US citizenship required (ITAR). The previously-stated Oct 1, 2026 deadline is gone from the live posting as of 2026-10-02 — appears to remain open.</v>
+        <v>New company — medical device manufacturer (AEON surgical stapler), Boston-area (Bedford, MA). R&amp;D team: design/test/document parts, CAD + machine shop + testing work. Sibling 'Manufacturing Engineering Intern', 'Mechanical Engineering Intern', and 'Quality Systems Engineering Intern' at the same site are all explicitly Summer 2027 — excluded on season grounds.</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>1X Technologies</v>
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
       </c>
       <c r="B282" t="str">
-        <v>Internship - Manufacturing Engineering</v>
+        <v>iProd Design Center Engineering Co-op (Spring/Summer 2027)</v>
       </c>
       <c r="C282" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering / Mechanical Engineering Technology</v>
       </c>
       <c r="D282" t="str">
-        <v>Starting January 2027 (posting's own wording — does not use the literal word 'Spring' or 'Winter', but the explicit January 2027 start date places it inside Hamza's target window)</v>
+        <v>January – August 2027 (co-op begins in Spring 2027)</v>
       </c>
       <c r="E282" t="str">
-        <v>San Carlos, CA</v>
+        <v>Seneca Falls, NY</v>
       </c>
       <c r="F282">
-        <v>2700</v>
+        <v>290</v>
       </c>
       <c r="G282" t="str">
-        <v>$35/hr + $2,500/month housing stipend for relocation</v>
+        <v>$25–$30/hr</v>
       </c>
       <c r="H282" t="str">
-        <v>https://jobs.ashbyhq.com/1x/d687b375-8136-4e6f-baa6-369b89366050</v>
+        <v>https://careersenus-itt-inc.icims.com/jobs/17446/iprod-design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
       </c>
       <c r="I282" t="str">
-        <v>Yes — independently fetched directly via Ashby's own posting-api (api.ashbyhq.com/posting-api/job-board/1x), isListed true, title 'Internship - Manufacturing Engineering', body states 'INTERNSHIP SEASON - STARTING JANUARY 2027' verbatim, published 2026-09-14.</v>
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'iProd Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: Summer/Fall 2026 rotation, full-time, 40 hours per week. Must be available January to August 2027.' verbatim.</v>
       </c>
       <c r="J282" t="str">
-        <v>New company — humanoid robotics manufacturer (maker of the 'NEO' home robot). Role: manufacturing process/fixture design, CAD (SolidWorks/Onshape), design-for-manufacturability for robot hardware. A sibling 'Internship - CNC Machine Park' (Hayward, CA) role exists but states no season/year and was excluded.</v>
+        <v>New company. A duplicate req (17447, same title/location/team, separate req ID — likely a second headcount slot) exists but is not listed as a separate row.</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>Lexington Medical, Inc.</v>
+        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
       </c>
       <c r="B283" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Application Engineering Co-op (Spring/Summer 2027)</v>
       </c>
       <c r="C283" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical or Industrial Engineering</v>
       </c>
       <c r="D283" t="str">
-        <v>January 2027 – June 2027 (Spring 2027)</v>
+        <v>January – August 2027 (co-op begins in Spring 2027)</v>
       </c>
       <c r="E283" t="str">
-        <v>Bedford, MA</v>
+        <v>Stafford, TX</v>
       </c>
       <c r="F283">
-        <v>17</v>
+        <v>1600</v>
       </c>
       <c r="G283" t="str">
-        <v>$28.00–$34.00/hr (pay-transparency widget shows $28–$36)</v>
+        <v>$25–$30/hr</v>
       </c>
       <c r="H283" t="str">
-        <v>https://job-boards.greenhouse.io/lexingtonmedical/jobs/5423105008</v>
+        <v>https://careersenus-itt-inc.icims.com/jobs/17660/application-engineering-co-op-%28spring-summer-2027%29/job</v>
       </c>
       <c r="I283" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own board API (boards-api.greenhouse.io/v1/boards/lexingtonmedical/jobs/5423105008), job live, updated_at 2026-09-30, body states 'The co-op runs full-time, five days per week, from January 2027 through June 2027.' verbatim.</v>
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Application Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January – August 2027 (full-time, 40 hours per week)' verbatim.</v>
       </c>
       <c r="J283" t="str">
-        <v>New company — medical device manufacturer (AEON surgical stapler), Boston-area (Bedford, MA). R&amp;D team: design/test/document parts, CAD + machine shop + testing work. Sibling 'Manufacturing Engineering Intern', 'Mechanical Engineering Intern', and 'Quality Systems Engineering Intern' at the same site are all explicitly Summer 2027 — excluded on season grounds.</v>
+        <v>New company. Open to junior/senior undergraduates in mechanical or industrial engineering.</v>
       </c>
     </row>
     <row r="284">
@@ -10946,7 +10946,7 @@
         <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
       </c>
       <c r="B284" t="str">
-        <v>iProd Design Center Engineering Co-op (Spring/Summer 2027)</v>
+        <v>ES Horizontal Design Center Engineering Co-op (Spring/Summer 2027)</v>
       </c>
       <c r="C284" t="str">
         <v>Mechanical Engineering / Mechanical Engineering Technology</v>
@@ -10964,429 +10964,429 @@
         <v>$25–$30/hr</v>
       </c>
       <c r="H284" t="str">
-        <v>https://careersenus-itt-inc.icims.com/jobs/17446/iprod-design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
+        <v>https://careersenus-itt-inc.icims.com/jobs/17708/design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
       </c>
       <c r="I284" t="str">
-        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'iProd Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: Summer/Fall 2026 rotation, full-time, 40 hours per week. Must be available January to August 2027.' verbatim.</v>
+        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January to August 2027 (full-time, 40 hours per week)' verbatim.</v>
       </c>
       <c r="J284" t="str">
-        <v>New company. A duplicate req (17447, same title/location/team, separate req ID — likely a second headcount slot) exists but is not listed as a separate row.</v>
+        <v>New company. Distinct req from the iProd Design Center Co-op above (different team/business line, same site).</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+        <v>Gravitics</v>
       </c>
       <c r="B285" t="str">
-        <v>Application Engineering Co-op (Spring/Summer 2027)</v>
+        <v>Mechanical Engineering Intern (2027 Winter session)</v>
       </c>
       <c r="C285" t="str">
-        <v>Mechanical or Industrial Engineering</v>
+        <v>Mechanical Engineering (Mechanical Test Engineering or Motor Control Engineering track)</v>
       </c>
       <c r="D285" t="str">
-        <v>January – August 2027 (co-op begins in Spring 2027)</v>
+        <v>2027 Winter session, 10-12 weeks, January–March 2027</v>
       </c>
       <c r="E285" t="str">
-        <v>Stafford, TX</v>
+        <v>Marysville, WA (Greater Seattle Area)</v>
       </c>
       <c r="F285">
-        <v>1600</v>
+        <v>2490</v>
       </c>
       <c r="G285" t="str">
-        <v>$25–$30/hr</v>
+        <v>$28–$35/hr + housing assistance</v>
       </c>
       <c r="H285" t="str">
-        <v>https://careersenus-itt-inc.icims.com/jobs/17660/application-engineering-co-op-%28spring-summer-2027%29/job</v>
+        <v>https://job-boards.greenhouse.io/graviticsinc/jobs/4396521009</v>
       </c>
       <c r="I285" t="str">
-        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Application Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January – August 2027 (full-time, 40 hours per week)' verbatim.</v>
+        <v>Yes — independently fetched directly via Greenhouse's own Jobs API (boards-api.greenhouse.io/v1/boards/graviticsinc/jobs/4396521009), HTTP 200, body states a '2027 Winter session' internship 'spanning January through March 2027,' checked 2026-10-01.</v>
       </c>
       <c r="J285" t="str">
-        <v>New company. Open to junior/senior undergraduates in mechanical or industrial engineering.</v>
+        <v>New company — designs/manufactures large-scale space station infrastructure. Two specialty tracks: Mechanical Test Engineering (sensors, tensile/vibration/thermal testing) or Motor Control Engineering (PWM, stepper motors, PID, embedded C/C++). Requires US citizenship or permanent residency.</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>ITT Inc. (Goulds Pumps / Industrial Process business)</v>
+        <v>Castelion</v>
       </c>
       <c r="B286" t="str">
-        <v>ES Horizontal Design Center Engineering Co-op (Spring/Summer 2027)</v>
+        <v>Mechanical Engineer Intern (Winter/Spring 2027)</v>
       </c>
       <c r="C286" t="str">
-        <v>Mechanical Engineering / Mechanical Engineering Technology</v>
+        <v>Mechanical / Structural Engineering (Radar Engineering team)</v>
       </c>
       <c r="D286" t="str">
-        <v>January – August 2027 (co-op begins in Spring 2027)</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E286" t="str">
-        <v>Seneca Falls, NY</v>
+        <v>Torrance, CA</v>
       </c>
       <c r="F286">
-        <v>290</v>
+        <v>2600</v>
       </c>
       <c r="G286" t="str">
-        <v>$25–$30/hr</v>
+        <v>Not stated on this posting (company's general intern band elsewhere is ~$30/hr)</v>
       </c>
       <c r="H286" t="str">
-        <v>https://careersenus-itt-inc.icims.com/jobs/17708/design-center-engineering-co-op-%28spring-summer-2027%29/job</v>
+        <v>https://www.castelion.com/careers/job/4386032009/</v>
       </c>
       <c r="I286" t="str">
-        <v>Yes — independently fetched directly (HTTP 200), title confirmed 'Design Center Engineering Co-op (Spring/Summer 2027)', body states 'Academic Schedule: January to August 2027 (full-time, 40 hours per week)' verbatim.</v>
+        <v>Yes — independently fetched directly, page live (not a filled/closed placeholder), title confirmed 'Mechanical Engineer Intern (Winter/Spring 2027)' with an active application form, checked 2026-10-01.</v>
       </c>
       <c r="J286" t="str">
-        <v>New company. Distinct req from the iProd Design Center Co-op above (different team/business line, same site).</v>
+        <v>New company — hypersonic weapons/defense-tech startup. Radar Engineering team. Requires U.S. person status (citizen/GPR/refugee/asylee); may require DoS export-control access.</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>Gravitics</v>
+        <v>RTX (Collins Aerospace)</v>
       </c>
       <c r="B287" t="str">
-        <v>Mechanical Engineering Intern (2027 Winter session)</v>
+        <v>Pump Engineering Co-op (Spring/Summer 2027)</v>
       </c>
       <c r="C287" t="str">
-        <v>Mechanical Engineering (Mechanical Test Engineering or Motor Control Engineering track)</v>
+        <v>Mechanical Engineering (Fuel and Oil pump product line)</v>
       </c>
       <c r="D287" t="str">
-        <v>2027 Winter session, 10-12 weeks, January–March 2027</v>
+        <v>Winter/Spring 2027 (runs January–July/August, including the Spring semester)</v>
       </c>
       <c r="E287" t="str">
-        <v>Marysville, WA (Greater Seattle Area)</v>
+        <v>Rockford, IL</v>
       </c>
       <c r="F287">
-        <v>2490</v>
+        <v>900</v>
       </c>
       <c r="G287" t="str">
-        <v>$28–$35/hr + housing assistance</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H287" t="str">
-        <v>https://job-boards.greenhouse.io/graviticsinc/jobs/4396521009</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/en-US/rec_rtx_ext_gateway/job/US-IL-ROCKFORD-P1--2421-11th-St--2421-11TH-ST-P1/Pump-Engineering-Co-op--Spring-Summer-2027-_01876586</v>
       </c>
       <c r="I287" t="str">
-        <v>Yes — independently fetched directly via Greenhouse's own Jobs API (boards-api.greenhouse.io/v1/boards/graviticsinc/jobs/4396521009), HTTP 200, body states a '2027 Winter session' internship 'spanning January through March 2027,' checked 2026-10-01.</v>
+        <v>Yes — independently fetched directly via RTX's own Workday CXS API, HTTP 200, req 01876586, posted 2026-09-28, body states 'will run January- July/August (including the Spring semester...)' verbatim, checked 2026-10-01.</v>
       </c>
       <c r="J287" t="str">
-        <v>New company — designs/manufactures large-scale space station infrastructure. Two specialty tracks: Mechanical Test Engineering (sensors, tensile/vibration/thermal testing) or Motor Control Engineering (PWM, stepper motors, PID, embedded C/C++). Requires US citizenship or permanent residency.</v>
+        <v>Distinct req/site-team from the already-tracked Rockford IL Mechanical Engineering Co-op (01869227) and Mechanical Design Engineering Co-op (01873225) — this one is specifically Fuel/Oil pump engineering (CFD analysis, RCCA, supplier management). U.S. citizenship required, no security clearance required.</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>Castelion</v>
+        <v>Yaskawa America, Inc.</v>
       </c>
       <c r="B288" t="str">
-        <v>Mechanical Engineer Intern (Winter/Spring 2027)</v>
+        <v>Engineering Co-op (2027)</v>
       </c>
       <c r="C288" t="str">
-        <v>Mechanical / Structural Engineering (Radar Engineering team)</v>
+        <v>Mechanical / Mechatronics / Industrial Engineering (student selects track; also Electrical/CS/CompE)</v>
       </c>
       <c r="D288" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>2027, 6-month period, January–August or May–December (Jan–Aug option qualifies as Winter/Spring 2027)</v>
       </c>
       <c r="E288" t="str">
-        <v>Torrance, CA</v>
+        <v>Waukegan, IL (also Franklin WI; Buffalo Grove IL; Santa Clara/San Francisco CA)</v>
       </c>
       <c r="F288">
-        <v>2600</v>
+        <v>850</v>
       </c>
       <c r="G288" t="str">
-        <v>Not stated on this posting (company's general intern band elsewhere is ~$30/hr)</v>
+        <v>$20.10–$27.12/hr + housing allowance for relocating students</v>
       </c>
       <c r="H288" t="str">
-        <v>https://www.castelion.com/careers/job/4386032009/</v>
+        <v>https://recruiting.ultipro.com/YAS1000YAAMI/JobBoard/ac63a36b-3e0b-412c-939d-ae4625f85d3e/OpportunityDetail?opportunityId=d34cfbaa-53d1-4e44-a36e-497b7014a406</v>
       </c>
       <c r="I288" t="str">
-        <v>Yes — independently fetched directly, page live (not a filled/closed placeholder), title confirmed 'Mechanical Engineer Intern (Winter/Spring 2027)' with an active application form, checked 2026-10-01.</v>
+        <v>Yes — independently fetched directly via Yaskawa's own UltiPro/UKG JobBoard API, HTTP 200, req ENGIN002923, 'OpportunityIsClosed': false, posted 2026-08-28, description states 'various Engineering Co-ops for 2027... a 6 month period either January-August or May - December' verbatim, checked 2026-10-01.</v>
       </c>
       <c r="J288" t="str">
-        <v>New company — hypersonic weapons/defense-tech startup. Radar Engineering team. Requires U.S. person status (citizen/GPR/refugee/asylee); may require DoS export-control access.</v>
+        <v>Open to Mechanical, Electrical, Mechatronics, Industrial, CS, or Computer Engineering majors (sophomore standing+); student selects discipline track at application. A prior run's search had found only Summer-2027-titled Yaskawa postings and excluded the company — this is a distinct, newly-posted req with an explicit Jan–Aug 2027 option, independently re-verified rather than taken on the research agent's word alone.</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>RTX (Collins Aerospace)</v>
+        <v>Tesla</v>
       </c>
       <c r="B289" t="str">
-        <v>Pump Engineering Co-op (Spring/Summer 2027)</v>
+        <v>Internship, Powertrain, Manufacturing Automation Controls Engineering (Winter/Spring 2027)</v>
       </c>
       <c r="C289" t="str">
-        <v>Mechanical Engineering (Fuel and Oil pump product line)</v>
+        <v>Controls / Manufacturing Automation Engineering (PLC, robot programming, machine safety circuits)</v>
       </c>
       <c r="D289" t="str">
-        <v>Winter/Spring 2027 (runs January–July/August, including the Spring semester)</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E289" t="str">
-        <v>Rockford, IL</v>
+        <v>Sparks, NV (Gigafactory Nevada)</v>
       </c>
       <c r="F289">
-        <v>900</v>
+        <v>2450</v>
       </c>
       <c r="G289" t="str">
-        <v>Not stated on posting</v>
+        <v>Not stated (blocked before pay info could be retrieved)</v>
       </c>
       <c r="H289" t="str">
-        <v>https://globalhr.wd5.myworkdayjobs.com/en-US/rec_rtx_ext_gateway/job/US-IL-ROCKFORD-P1--2421-11th-St--2421-11TH-ST-P1/Pump-Engineering-Co-op--Spring-Summer-2027-_01876586</v>
+        <v>https://www.tesla.com/careers/search/job/internship-powertrain-manufacturing-automation-controls-engineering-winter-spring-2027--278960</v>
       </c>
       <c r="I289" t="str">
-        <v>Yes — independently fetched directly via RTX's own Workday CXS API, HTTP 200, req 01876586, posted 2026-09-28, body states 'will run January- July/August (including the Spring semester...)' verbatim, checked 2026-10-01.</v>
+        <v>Partial — official tesla.com domain, blocked automated fetch (403, bot protection) on independent re-check 2026-10-01 and again 2026-10-02 (multiple user-agent/header variations all still 403). A third-party mirror (milwaukeejobs.com) showed the same listing as live, 'posted 5 days ago,' as of 2026-10-02, but this is a secondary source, not Tesla's own site — open/closed status remains unconfirmed on the primary source. Verify live in-browser before applying.</v>
       </c>
       <c r="J289" t="str">
-        <v>Distinct req/site-team from the already-tracked Rockford IL Mechanical Engineering Co-op (01869227) and Mechanical Design Engineering Co-op (01873225) — this one is specifically Fuel/Oil pump engineering (CFD analysis, RCCA, supplier management). U.S. citizenship required, no security clearance required.</v>
+        <v>Powertrain Manufacturing Automation Controls team — FANUC/KUKA robot programming, PLC, machine safety circuits.</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>Yaskawa America, Inc.</v>
+        <v>The Exploration Company</v>
       </c>
       <c r="B290" t="str">
-        <v>Engineering Co-op (2027)</v>
+        <v>Spring 2027 Internship (Engineering)</v>
       </c>
       <c r="C290" t="str">
-        <v>Mechanical / Mechatronics / Industrial Engineering (student selects track; also Electrical/CS/CompE)</v>
+        <v>General Engineering (crewed spacecraft systems — design/test/validation)</v>
       </c>
       <c r="D290" t="str">
-        <v>2027, 6-month period, January–August or May–December (Jan–Aug option qualifies as Winter/Spring 2027)</v>
+        <v>Spring 2027 (starting January 2027, min. 12 weeks)</v>
       </c>
       <c r="E290" t="str">
-        <v>Waukegan, IL (also Franklin WI; Buffalo Grove IL; Santa Clara/San Francisco CA)</v>
+        <v>Houston, TX</v>
       </c>
       <c r="F290">
-        <v>850</v>
+        <v>1600</v>
       </c>
       <c r="G290" t="str">
-        <v>$20.10–$27.12/hr + housing allowance for relocating students</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H290" t="str">
-        <v>https://recruiting.ultipro.com/YAS1000YAAMI/JobBoard/ac63a36b-3e0b-412c-939d-ae4625f85d3e/OpportunityDetail?opportunityId=d34cfbaa-53d1-4e44-a36e-497b7014a406</v>
+        <v>https://jobs.ashbyhq.com/the-exploration-company/3f4e976b-0d0c-4440-a943-6b4b0b2f6ddf</v>
       </c>
       <c r="I290" t="str">
-        <v>Yes — independently fetched directly via Yaskawa's own UltiPro/UKG JobBoard API, HTTP 200, req ENGIN002923, 'OpportunityIsClosed': false, posted 2026-08-28, description states 'various Engineering Co-ops for 2027... a 6 month period either January-August or May - December' verbatim, checked 2026-10-01.</v>
+        <v>Yes — independently fetched directly via the company's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/the-exploration-company), HTTP 200, published 2026-09-03, body states 'Spring 2027 Engineering Internship... Able to work full-time (40 hours per week) for a minimum of 12 weeks beginning January 2027' verbatim, checked 2026-10-02.</v>
       </c>
       <c r="J290" t="str">
-        <v>Open to Mechanical, Electrical, Mechatronics, Industrial, CS, or Computer Engineering majors (sophomore standing+); student selects discipline track at application. A prior run's search had found only Summer-2027-titled Yaskawa postings and excluded the company — this is a distinct, newly-posted req with an explicit Jan–Aug 2027 option, independently re-verified rather than taken on the research agent's word alone.</v>
+        <v>New company — French/German crewed-spacecraft (Nyx vehicle) developer with a Houston, TX engineering presence. Role is general engineering support (design/test/validation of engineering systems), not a named sub-discipline. Requires US citizenship or lawful permanent residency (ITAR/EAR). No housing/relocation provided. Posted 2026-09-03 — about 4 weeks old, slightly past the usual ~3-week freshness preference but still open and a strong discipline/location fit.</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>Tesla</v>
+        <v>Lincoln Electric</v>
       </c>
       <c r="B291" t="str">
-        <v>Internship, Powertrain, Manufacturing Automation Controls Engineering (Winter/Spring 2027)</v>
+        <v>Mechanical Engineering Spring 2027 Co-op</v>
       </c>
       <c r="C291" t="str">
-        <v>Controls / Manufacturing Automation Engineering (PLC, robot programming, machine safety circuits)</v>
+        <v>Mechanical / Industrial Engineering (automation, robotics, manufacturing equipment)</v>
       </c>
       <c r="D291" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027 (Target Program Dates: January 12 – April 16, 2027)</v>
       </c>
       <c r="E291" t="str">
-        <v>Sparks, NV (Gigafactory Nevada)</v>
+        <v>Plymouth, MI</v>
       </c>
       <c r="F291">
-        <v>2450</v>
+        <v>650</v>
       </c>
       <c r="G291" t="str">
-        <v>Not stated (blocked before pay info could be retrieved)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H291" t="str">
-        <v>https://www.tesla.com/careers/search/job/internship-powertrain-manufacturing-automation-controls-engineering-winter-spring-2027--278960</v>
+        <v>https://jobs.lincolnelectric.com/job/Plymouth-Mechanical-Engineering-Spring-2027-Co-op-%28Plymouth%2C-MI%29-MI-48170/1432989733/</v>
       </c>
       <c r="I291" t="str">
-        <v>Partial — official tesla.com domain, blocked automated fetch (403, bot protection) on independent re-check 2026-10-01 and again 2026-10-02 (multiple user-agent/header variations all still 403). A third-party mirror (milwaukeejobs.com) showed the same listing as live, 'posted 5 days ago,' as of 2026-10-02, but this is a secondary source, not Tesla's own site — open/closed status remains unconfirmed on the primary source. Verify live in-browser before applying.</v>
+        <v>Yes — independently fetched directly via Lincoln Electric's own careers site (jobs.lincolnelectric.com), HTTP 200, Req ID 29823, page states 'Target Program Dates: January 12th – April16th, 2027' verbatim, distinct from a same-site 'Mechanical Engineering Summer 2027 Internship' sibling at the same Plymouth, MI location, checked 2026-10-02.</v>
       </c>
       <c r="J291" t="str">
-        <v>Powertrain Manufacturing Automation Controls team — FANUC/KUKA robot programming, PLC, machine safety circuits.</v>
+        <v>Automation facility — develops custom manufacturing equipment, automated systems, and robotic solutions for customer applications. Bachelor's in engineering/engineering technology required; eligible to work in the US without sponsorship. 3.0+ GPA preferred. Includes a company-paid Immersion Day at Cleveland, OH HQ.</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>The Exploration Company</v>
+        <v>Insulet</v>
       </c>
       <c r="B292" t="str">
-        <v>Spring 2027 Internship (Engineering)</v>
+        <v>Co-op - Supplier Quality Engineering: January - June 2027 (Onsite)</v>
       </c>
       <c r="C292" t="str">
-        <v>General Engineering (crewed spacecraft systems — design/test/validation)</v>
+        <v>Mechanical / Industrial / Bio-Engineering (supplier quality, Six Sigma/Lean)</v>
       </c>
       <c r="D292" t="str">
-        <v>Spring 2027 (starting January 2027, min. 12 weeks)</v>
+        <v>January 11 – June 30, 2027</v>
       </c>
       <c r="E292" t="str">
-        <v>Houston, TX</v>
+        <v>Acton, MA</v>
       </c>
       <c r="F292">
-        <v>1600</v>
+        <v>25</v>
       </c>
       <c r="G292" t="str">
-        <v>Not stated on posting</v>
+        <v>$24.00–$28.50/hr</v>
       </c>
       <c r="H292" t="str">
-        <v>https://jobs.ashbyhq.com/the-exploration-company/3f4e976b-0d0c-4440-a943-6b4b0b2f6ddf</v>
+        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op---Supplier-Quality-Engineering--January---June-2027--Onsite-_REQ-2026-18125</v>
       </c>
       <c r="I292" t="str">
-        <v>Yes — independently fetched directly via the company's own Ashby posting-api (api.ashbyhq.com/posting-api/job-board/the-exploration-company), HTTP 200, published 2026-09-03, body states 'Spring 2027 Engineering Internship... Able to work full-time (40 hours per week) for a minimum of 12 weeks beginning January 2027' verbatim, checked 2026-10-02.</v>
+        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, canApply true, req REQ-2026-18125, posted 2026-10-01, body states 'Position Dates: January 11, 2027 – June 30, 2027' verbatim, checked 2026-10-02.</v>
       </c>
       <c r="J292" t="str">
-        <v>New company — French/German crewed-spacecraft (Nyx vehicle) developer with a Houston, TX engineering presence. Role is general engineering support (design/test/validation of engineering systems), not a named sub-discipline. Requires US citizenship or lawful permanent residency (ITAR/EAR). No housing/relocation provided. Posted 2026-09-03 — about 4 weeks old, slightly past the usual ~3-week freshness preference but still open and a strong discipline/location fit.</v>
+        <v>Boston metro (Acton). Global Supplier Quality Engineering team — supplier selection/qualification, Engineering Change Orders, External Quality Action Requests, Six Sigma/Lean. Requires currently-enrolled undergrad in mechanical, industrial, or bio-engineering, 3.0+ GPA. Not eligible for visa sponsorship. Sibling to Insulet's many other already-tracked Acton Jan–June 2027 co-ops.</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>Lincoln Electric</v>
+        <v>Impulse Space</v>
       </c>
       <c r="B293" t="str">
-        <v>Mechanical Engineering Spring 2027 Co-op</v>
+        <v>Manufacturing Engineering Intern (Spring 2027)</v>
       </c>
       <c r="C293" t="str">
-        <v>Mechanical / Industrial Engineering (automation, robotics, manufacturing equipment)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D293" t="str">
-        <v>Spring 2027 (Target Program Dates: January 12 – April 16, 2027)</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E293" t="str">
-        <v>Plymouth, MI</v>
+        <v>Redondo Beach, CA</v>
       </c>
       <c r="F293">
-        <v>650</v>
+        <v>2600</v>
       </c>
       <c r="G293" t="str">
-        <v>Not stated on posting</v>
+        <v>$30.00/hr</v>
       </c>
       <c r="H293" t="str">
-        <v>https://jobs.lincolnelectric.com/job/Plymouth-Mechanical-Engineering-Spring-2027-Co-op-%28Plymouth%2C-MI%29-MI-48170/1432989733/</v>
+        <v>https://impulsespace.pinpointhq.com/en/postings/d466f97d-0d4a-479d-b764-acf687745208</v>
       </c>
       <c r="I293" t="str">
-        <v>Yes — independently fetched directly via Lincoln Electric's own careers site (jobs.lincolnelectric.com), HTTP 200, Req ID 29823, page states 'Target Program Dates: January 12th – April16th, 2027' verbatim, distinct from a same-site 'Mechanical Engineering Summer 2027 Internship' sibling at the same Plymouth, MI location, checked 2026-10-02.</v>
+        <v>Yes — independently fetched directly via Impulse Space's own Pinpoint ATS (postings.json API, job id 590465, HTTP 200, and the live posting URL itself, HTTP 200), title confirmed 'Manufacturing Engineering Intern (Spring 2027)', Apply Now button present, checked 2026-10-02.</v>
       </c>
       <c r="J293" t="str">
-        <v>Automation facility — develops custom manufacturing equipment, automated systems, and robotic solutions for customer applications. Bachelor's in engineering/engineering technology required; eligible to work in the US without sponsorship. 3.0+ GPA preferred. Includes a company-paid Immersion Day at Cleveland, OH HQ.</v>
+        <v>New company — in-space transportation vehicle manufacturer. Distinct from Impulse Space's already-excluded Spring 2027 RF/Antenna Engineering Intern reqs (electrical discipline, outside target list) and its ~25 Summer 2027 mechanical/propulsion/manufacturing internships. Company's mechanical/propulsion/structures reqs were re-checked across several prior runs (09-23 through 09-25) and found Summer-2027-only at the time; this Manufacturing Engineering req is newly found as of this run.</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>Insulet</v>
+        <v>CMTA, Inc. (via Legence)</v>
       </c>
       <c r="B294" t="str">
-        <v>Co-op - Supplier Quality Engineering: January - June 2027 (Onsite)</v>
+        <v>Mechanical Engineer Intern/Co-op, Spring 2027</v>
       </c>
       <c r="C294" t="str">
-        <v>Mechanical / Industrial / Bio-Engineering (supplier quality, Six Sigma/Lean)</v>
+        <v>Mechanical Engineering (MEP/HVAC building-systems consulting)</v>
       </c>
       <c r="D294" t="str">
-        <v>January 11 – June 30, 2027</v>
+        <v>Spring 2027 (starts January 2027, dates flexible with school calendar)</v>
       </c>
       <c r="E294" t="str">
-        <v>Acton, MA</v>
+        <v>Boston, MA (170 Milk Street)</v>
       </c>
       <c r="F294">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="G294" t="str">
-        <v>$24.00–$28.50/hr</v>
+        <v>Competitive hourly, OT eligible (exact rate not stated)</v>
       </c>
       <c r="H294" t="str">
-        <v>https://insulet.wd5.myworkdayjobs.com/en-US/insuletcareers/job/Acton-Massachusetts/Co-op---Supplier-Quality-Engineering--January---June-2027--Onsite-_REQ-2026-18125</v>
+        <v>https://jobs.dayforcehcm.com/en-US/legence/studentportal/jobs/33378</v>
       </c>
       <c r="I294" t="str">
-        <v>Yes — independently fetched directly via Insulet's own Workday CXS API, canApply true, req REQ-2026-18125, posted 2026-10-01, body states 'Position Dates: January 11, 2027 – June 30, 2027' verbatim, checked 2026-10-02.</v>
+        <v>Yes — fetched directly (HTTP 200); raw server-side response carries the full job JSON (jobPostingId 33378, jobReqId 4002, postingAppliedStatus.canApplyAgain true, no expiry date set) even though the rendered page on top is JS-heavy.</v>
       </c>
       <c r="J294" t="str">
-        <v>Boston metro (Acton). Global Supplier Quality Engineering team — supplier selection/qualification, Engineering Change Orders, External Quality Action Requests, Six Sigma/Lean. Requires currently-enrolled undergrad in mechanical, industrial, or bio-engineering, 3.0+ GPA. Not eligible for visa sponsorship. Sibling to Insulet's many other already-tracked Acton Jan–June 2027 co-ops.</v>
+        <v>FLAGGED DISCIPLINE BORDERLINE: this is MEP/HVAC building-systems engineering (HVAC layout, one-line diagrams, building energy efficiency) for a Boston architecture/engineering consulting firm — not aerospace/manufacturing/robotics work. Included given the exact Boston, MA location and literal 'Mechanical Engineer' title/degree requirement (pursuing BS Mechanical or Architectural Engineering, preferably sophomore/junior); Hamza should judge personal interest fit. Full-time 40hr/week onsite. No visa sponsorship available.</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>Impulse Space</v>
+        <v>Eversource Energy</v>
       </c>
       <c r="B295" t="str">
-        <v>Manufacturing Engineering Intern (Spring 2027)</v>
+        <v>2027 Co-op: Capital Projects</v>
       </c>
       <c r="C295" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Civil / Mechanical / Electrical Engineering (posting states 'civil and mechanical engineering also considered')</v>
       </c>
       <c r="D295" t="str">
-        <v>Spring 2027</v>
+        <v>2027 (exact term not printed on this specific posting; a sibling Eversource co-op in the same posting batch, Substation Design Engineering, explicitly states 'January–June 2027' — very likely the same cycle, but not independently confirmed on this posting's own text)</v>
       </c>
       <c r="E295" t="str">
-        <v>Redondo Beach, CA</v>
+        <v>Westwood, MA</v>
       </c>
       <c r="F295">
-        <v>2600</v>
+        <v>14</v>
       </c>
       <c r="G295" t="str">
-        <v>$30.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H295" t="str">
-        <v>https://impulsespace.pinpointhq.com/en/postings/d466f97d-0d4a-479d-b764-acf687745208</v>
+        <v>https://jobs.eversource.com/job/westwood/2027-co-op-capital-projects/7774/101320869904</v>
       </c>
       <c r="I295" t="str">
-        <v>Yes — independently fetched directly via Impulse Space's own Pinpoint ATS (postings.json API, job id 590465, HTTP 200, and the live posting URL itself, HTTP 200), title confirmed 'Manufacturing Engineering Intern (Spring 2027)', Apply Now button present, checked 2026-10-02.</v>
+        <v>Yes — fetched directly, live posting, posted 2026-09-28, 'Apply Now' active, 1 opening.</v>
       </c>
       <c r="J295" t="str">
-        <v>New company — in-space transportation vehicle manufacturer. Distinct from Impulse Space's already-excluded Spring 2027 RF/Antenna Engineering Intern reqs (electrical discipline, outside target list) and its ~25 Summer 2027 mechanical/propulsion/manufacturing internships. Company's mechanical/propulsion/structures reqs were re-checked across several prior runs (09-23 through 09-25) and found Summer-2027-only at the time; this Manufacturing Engineering req is newly found as of this run.</v>
+        <v>New Boston-area utility co-op employer (Northeastern/WPI-style structured co-op program) — worth periodic re-checking since Eversource posts new reqs each cycle. No visa sponsorship ('applicants requiring visa sponsorship... will not be considered'). No GPA/class-standing stated. Season wording caveat above — confirm the exact term directly before applying.</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>CMTA, Inc. (via Legence)</v>
+        <v>Graco Inc.</v>
       </c>
       <c r="B296" t="str">
-        <v>Mechanical Engineer Intern/Co-op, Spring 2027</v>
+        <v>Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C296" t="str">
-        <v>Mechanical Engineering (MEP/HVAC building-systems consulting)</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D296" t="str">
-        <v>Spring 2027 (starts January 2027, dates flexible with school calendar)</v>
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E296" t="str">
-        <v>Boston, MA (170 Milk Street)</v>
+        <v>Anoka, MN</v>
       </c>
       <c r="F296">
-        <v>0</v>
+        <v>1127</v>
       </c>
       <c r="G296" t="str">
-        <v>Competitive hourly, OT eligible (exact rate not stated)</v>
+        <v>Not stated on posting (a third-party aggregator estimated $21-28/hr, unconfirmed on the primary source)</v>
       </c>
       <c r="H296" t="str">
-        <v>https://jobs.dayforcehcm.com/en-US/legence/studentportal/jobs/33378</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Anoka-Minnesota-USA/Manufacturing-Engineering-Co-Op_R0023507</v>
       </c>
       <c r="I296" t="str">
-        <v>Yes — fetched directly (HTTP 200); raw server-side response carries the full job JSON (jobPostingId 33378, jobReqId 4002, postingAppliedStatus.canApplyAgain true, no expiry date set) even though the rendered page on top is JS-heavy.</v>
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~24 days ago.</v>
       </c>
       <c r="J296" t="str">
-        <v>FLAGGED DISCIPLINE BORDERLINE: this is MEP/HVAC building-systems engineering (HVAC layout, one-line diagrams, building energy efficiency) for a Boston architecture/engineering consulting firm — not aerospace/manufacturing/robotics work. Included given the exact Boston, MA location and literal 'Mechanical Engineer' title/degree requirement (pursuing BS Mechanical or Architectural Engineering, preferably sophomore/junior); Hamza should judge personal interest fit. Full-time 40hr/week onsite. No visa sponsorship available.</v>
+        <v>New company. Graco also posts sibling 'May - December 2027' co-ops at the same sites — wrong season, excluded.</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>Eversource Energy</v>
+        <v>Graco Inc.</v>
       </c>
       <c r="B297" t="str">
-        <v>2027 Co-op: Capital Projects</v>
+        <v>Automation Engineering Co-Op</v>
       </c>
       <c r="C297" t="str">
-        <v>Civil / Mechanical / Electrical Engineering (posting states 'civil and mechanical engineering also considered')</v>
+        <v>Automation / Mechanical Engineering</v>
       </c>
       <c r="D297" t="str">
-        <v>2027 (exact term not printed on this specific posting; a sibling Eversource co-op in the same posting batch, Substation Design Engineering, explicitly states 'January–June 2027' — very likely the same cycle, but not independently confirmed on this posting's own text)</v>
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E297" t="str">
-        <v>Westwood, MA</v>
+        <v>Rogers, MN (David Koch Center)</v>
       </c>
       <c r="F297">
-        <v>14</v>
+        <v>1135</v>
       </c>
       <c r="G297" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H297" t="str">
-        <v>https://jobs.eversource.com/job/westwood/2027-co-op-capital-projects/7774/101320869904</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Automation-Engineering-Co-Op--January---August-2027-_R0023586</v>
       </c>
       <c r="I297" t="str">
-        <v>Yes — fetched directly, live posting, posted 2026-09-28, 'Apply Now' active, 1 opening.</v>
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
       </c>
       <c r="J297" t="str">
-        <v>New Boston-area utility co-op employer (Northeastern/WPI-style structured co-op program) — worth periodic re-checking since Eversource posts new reqs each cycle. No visa sponsorship ('applicants requiring visa sponsorship... will not be considered'). No GPA/class-standing stated. Season wording caveat above — confirm the exact term directly before applying.</v>
+        <v>New company (Graco, industrial fluid-handling equipment manufacturer).</v>
       </c>
     </row>
     <row r="298">
@@ -11394,7 +11394,7 @@
         <v>Graco Inc.</v>
       </c>
       <c r="B298" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Manufacturing Engineering Co-op</v>
       </c>
       <c r="C298" t="str">
         <v>Manufacturing Engineering</v>
@@ -11403,22 +11403,22 @@
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E298" t="str">
-        <v>Anoka, MN</v>
+        <v>Rogers, MN (David Koch Center)</v>
       </c>
       <c r="F298">
-        <v>1127</v>
+        <v>1135</v>
       </c>
       <c r="G298" t="str">
-        <v>Not stated on posting (a third-party aggregator estimated $21-28/hr, unconfirmed on the primary source)</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H298" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Anoka-Minnesota-USA/Manufacturing-Engineering-Co-Op_R0023507</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering-Co-op--January---August-2027-_R0023611</v>
       </c>
       <c r="I298" t="str">
-        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~24 days ago.</v>
+        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
       </c>
       <c r="J298" t="str">
-        <v>New company. Graco also posts sibling 'May - December 2027' co-ops at the same sites — wrong season, excluded.</v>
+        <v>Sibling req to the Anoka Manufacturing Engineering Co-Op at a different Graco site.</v>
       </c>
     </row>
     <row r="299">
@@ -11426,31 +11426,31 @@
         <v>Graco Inc.</v>
       </c>
       <c r="B299" t="str">
-        <v>Automation Engineering Co-Op</v>
+        <v>Manufacturing Engineering Co-op</v>
       </c>
       <c r="C299" t="str">
-        <v>Automation / Mechanical Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D299" t="str">
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E299" t="str">
-        <v>Rogers, MN (David Koch Center)</v>
+        <v>Dayton, MN</v>
       </c>
       <c r="F299">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="G299" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H299" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Automation-Engineering-Co-Op--January---August-2027-_R0023586</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Dayton-Minnesota-USA/Manufacturing-Engineering-Co-op--January---August-2027-_R0023612</v>
       </c>
       <c r="I299" t="str">
         <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
       </c>
       <c r="J299" t="str">
-        <v>New company (Graco, industrial fluid-handling equipment manufacturer).</v>
+        <v>Another sibling Graco Manufacturing Engineering Co-Op req at a third site.</v>
       </c>
     </row>
     <row r="300">
@@ -11458,10 +11458,10 @@
         <v>Graco Inc.</v>
       </c>
       <c r="B300" t="str">
-        <v>Manufacturing Engineering Co-op</v>
+        <v>Quality Engineering Co-op</v>
       </c>
       <c r="C300" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Quality / Mechanical / Manufacturing Engineering</v>
       </c>
       <c r="D300" t="str">
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
@@ -11476,13 +11476,13 @@
         <v>Not stated on posting</v>
       </c>
       <c r="H300" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering-Co-op--January---August-2027-_R0023611</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Quality-Engineering-Co-op--January---August-2027-_R0023573</v>
       </c>
       <c r="I300" t="str">
         <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
       </c>
       <c r="J300" t="str">
-        <v>Sibling req to the Anoka Manufacturing Engineering Co-Op at a different Graco site.</v>
+        <v>Quality engineering within a manufacturing plant setting.</v>
       </c>
     </row>
     <row r="301">
@@ -11490,95 +11490,95 @@
         <v>Graco Inc.</v>
       </c>
       <c r="B301" t="str">
-        <v>Manufacturing Engineering Co-op</v>
+        <v>Manufacturing Engineering (Operational Technology) Co-op</v>
       </c>
       <c r="C301" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Manufacturing Engineering / Industrial Controls</v>
       </c>
       <c r="D301" t="str">
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E301" t="str">
-        <v>Dayton, MN</v>
+        <v>Rogers, MN (David Koch Center)</v>
       </c>
       <c r="F301">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="G301" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H301" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Dayton-Minnesota-USA/Manufacturing-Engineering-Co-op--January---August-2027-_R0023612</v>
+        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering--Operational-Technology--Co-op--January---August-2027-_R0023574</v>
       </c>
       <c r="I301" t="str">
         <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
       </c>
       <c r="J301" t="str">
-        <v>Another sibling Graco Manufacturing Engineering Co-Op req at a third site.</v>
+        <v>OT/industrial-controls-flavored manufacturing engineering co-op.</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>Graco Inc.</v>
+        <v>nVent</v>
       </c>
       <c r="B302" t="str">
-        <v>Quality Engineering Co-op</v>
+        <v>Manufacturing Engineering Co-op</v>
       </c>
       <c r="C302" t="str">
-        <v>Quality / Mechanical / Manufacturing Engineering</v>
+        <v>Manufacturing Engineering</v>
       </c>
       <c r="D302" t="str">
-        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+        <v>January - June 2027</v>
       </c>
       <c r="E302" t="str">
-        <v>Rogers, MN (David Koch Center)</v>
+        <v>Anoka, MN</v>
       </c>
       <c r="F302">
-        <v>1135</v>
+        <v>1127</v>
       </c>
       <c r="G302" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H302" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Quality-Engineering-Co-op--January---August-2027-_R0023573</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Manufacturing-Engineering-Co-op--January---June-2027-_R23576</v>
       </c>
       <c r="I302" t="str">
-        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, posted recently (within ~18 days).</v>
       </c>
       <c r="J302" t="str">
-        <v>Quality engineering within a manufacturing plant setting.</v>
+        <v>New company (nVent, electrical/thermal-management manufacturer spun off from Pentair). nVent also posts sibling 'June - Dec 2027' co-ops at the same sites — wrong season, excluded.</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>Graco Inc.</v>
+        <v>nVent</v>
       </c>
       <c r="B303" t="str">
-        <v>Manufacturing Engineering (Operational Technology) Co-op</v>
+        <v>Packaging Engineering Co-op</v>
       </c>
       <c r="C303" t="str">
-        <v>Manufacturing Engineering / Industrial Controls</v>
+        <v>Packaging Engineering (mechanical-design-adjacent)</v>
       </c>
       <c r="D303" t="str">
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E303" t="str">
-        <v>Rogers, MN (David Koch Center)</v>
+        <v>Anoka, MN</v>
       </c>
       <c r="F303">
-        <v>1135</v>
+        <v>1127</v>
       </c>
       <c r="G303" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H303" t="str">
-        <v>https://graco.wd501.myworkdayjobs.com/Graco_Careers/job/Rogers-Minnesota-USA-David-Koch-Center/Manufacturing-Engineering--Operational-Technology--Co-op--January---August-2027-_R0023574</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Packaging-Engineering-Co-op--January---August-2027-_R23570</v>
       </c>
       <c r="I303" t="str">
-        <v>Yes — fetched directly via Graco's Workday CXS API (HTTP 200), canApply true, posted ~23-24 days ago.</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true.</v>
       </c>
       <c r="J303" t="str">
-        <v>OT/industrial-controls-flavored manufacturing engineering co-op.</v>
+        <v>FLAGGED DISCIPLINE BORDERLINE: packaging engineering, not core mechanical/aero/manufacturing design — included for Hamza's own judgment.</v>
       </c>
     </row>
     <row r="304">
@@ -11586,31 +11586,31 @@
         <v>nVent</v>
       </c>
       <c r="B304" t="str">
-        <v>Manufacturing Engineering Co-op</v>
+        <v>Mechanical Engineering Co-Op</v>
       </c>
       <c r="C304" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D304" t="str">
-        <v>January - June 2027</v>
+        <v>Jan - Aug 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E304" t="str">
-        <v>Anoka, MN</v>
+        <v>Solon, OH (ERICO division)</v>
       </c>
       <c r="F304">
-        <v>1127</v>
+        <v>538</v>
       </c>
       <c r="G304" t="str">
-        <v>Not stated on posting</v>
+        <v>$25.00/hr</v>
       </c>
       <c r="H304" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Manufacturing-Engineering-Co-op--January---June-2027-_R23576</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Solon-OH-US/Mechanical-Engineering-Co-Op--Jan---Aug-2027-_R23577</v>
       </c>
       <c r="I304" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, posted recently (within ~18 days).</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
       </c>
       <c r="J304" t="str">
-        <v>New company (nVent, electrical/thermal-management manufacturer spun off from Pentair). nVent also posts sibling 'June - Dec 2027' co-ops at the same sites — wrong season, excluded.</v>
+        <v>ERICO is an nVent division (electrical/mechanical fastening products).</v>
       </c>
     </row>
     <row r="305">
@@ -11618,10 +11618,10 @@
         <v>nVent</v>
       </c>
       <c r="B305" t="str">
-        <v>Packaging Engineering Co-op</v>
+        <v>Mechanical Engineering and Design Co-op</v>
       </c>
       <c r="C305" t="str">
-        <v>Packaging Engineering (mechanical-design-adjacent)</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D305" t="str">
         <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
@@ -11633,16 +11633,16 @@
         <v>1127</v>
       </c>
       <c r="G305" t="str">
-        <v>Not stated on posting</v>
+        <v>$25.00/hr</v>
       </c>
       <c r="H305" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Packaging-Engineering-Co-op--January---August-2027-_R23570</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Mechanical-Engineering-and-Design-Co-op--January---August-2027-_R23572</v>
       </c>
       <c r="I305" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true.</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
       </c>
       <c r="J305" t="str">
-        <v>FLAGGED DISCIPLINE BORDERLINE: packaging engineering, not core mechanical/aero/manufacturing design — included for Hamza's own judgment.</v>
+        <v>Design-focused sibling to the Anoka Manufacturing Engineering Co-op.</v>
       </c>
     </row>
     <row r="306">
@@ -11650,255 +11650,255 @@
         <v>nVent</v>
       </c>
       <c r="B306" t="str">
-        <v>Mechanical Engineering Co-Op</v>
+        <v>Engineering Co-Op Opportunities</v>
       </c>
       <c r="C306" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Mechanical / Electrical / Industrial Engineering</v>
       </c>
       <c r="D306" t="str">
-        <v>Jan - Aug 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+        <v>Spring 2027 (body text states 'Mechanical, Electrical, or Industrial Engineering Co-Op (Spring 2027)' verbatim)</v>
       </c>
       <c r="E306" t="str">
-        <v>Solon, OH (ERICO division)</v>
+        <v>Richland, MS</v>
       </c>
       <c r="F306">
-        <v>538</v>
+        <v>1257</v>
       </c>
       <c r="G306" t="str">
-        <v>$25.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H306" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Solon-OH-US/Mechanical-Engineering-Co-Op--Jan---Aug-2027-_R23577</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Richland-MS-US/Engineering-Co-Op-Opportunities_R23659</v>
       </c>
       <c r="I306" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, explicit 'Spring 2027' wording confirmed in body text.</v>
       </c>
       <c r="J306" t="str">
-        <v>ERICO is an nVent division (electrical/mechanical fastening products).</v>
+        <v>A general-opportunities req covering multiple disciplines at the Richland, MS site.</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>nVent</v>
+        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
       </c>
       <c r="B307" t="str">
-        <v>Mechanical Engineering and Design Co-op</v>
+        <v>Transducer Manufacturing Engineering Co-Op</v>
       </c>
       <c r="C307" t="str">
-        <v>Mechanical Engineering</v>
+        <v>Manufacturing / Mechanical / Industrial Engineering</v>
       </c>
       <c r="D307" t="str">
-        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+        <v>January to June 2027 (per posting text)</v>
       </c>
       <c r="E307" t="str">
-        <v>Anoka, MN</v>
+        <v>Waltham, MA</v>
       </c>
       <c r="F307">
-        <v>1127</v>
+        <v>10</v>
       </c>
       <c r="G307" t="str">
-        <v>$25.00/hr</v>
+        <v>$25.00-$28.00/hr</v>
       </c>
       <c r="H307" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Mechanical-Engineering-and-Design-Co-op--January---August-2027-_R23572</v>
+        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015874986-transducer-manufacturing-engineering-co-op</v>
       </c>
       <c r="I307" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, pay rate stated on posting.</v>
+        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116547, posted 2026-10-02.</v>
       </c>
       <c r="J307" t="str">
-        <v>Design-focused sibling to the Anoka Manufacturing Engineering Co-op.</v>
+        <v>Evident/Wabtec Inspection Technologies division. New employer for the tracker. Boston-area.</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>nVent</v>
+        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
       </c>
       <c r="B308" t="str">
-        <v>Engineering Co-Op Opportunities</v>
+        <v>Co-Op, Test Engineer - Transducer</v>
       </c>
       <c r="C308" t="str">
-        <v>Mechanical / Electrical / Industrial Engineering</v>
+        <v>Manufacturing / Test Engineering</v>
       </c>
       <c r="D308" t="str">
-        <v>Spring 2027 (body text states 'Mechanical, Electrical, or Industrial Engineering Co-Op (Spring 2027)' verbatim)</v>
+        <v>January - June 2027 (stated in title)</v>
       </c>
       <c r="E308" t="str">
-        <v>Richland, MS</v>
+        <v>State College, PA</v>
       </c>
       <c r="F308">
-        <v>1257</v>
+        <v>390</v>
       </c>
       <c r="G308" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H308" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Richland-MS-US/Engineering-Co-Op-Opportunities_R23659</v>
+        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015763566-co-op-test-engineer-transducer-january-june-2027-</v>
       </c>
       <c r="I308" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, explicit 'Spring 2027' wording confirmed in body text.</v>
+        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116563, posted 2026-09-29.</v>
       </c>
       <c r="J308" t="str">
-        <v>A general-opportunities req covering multiple disciplines at the Richland, MS site.</v>
+        <v>Sibling req to the Waltham, MA transducer co-op above; hands-on fixture/test-system work.</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
+        <v>nVent</v>
       </c>
       <c r="B309" t="str">
-        <v>Transducer Manufacturing Engineering Co-Op</v>
+        <v>Electrical/Controls Engineering Co-Op</v>
       </c>
       <c r="C309" t="str">
-        <v>Manufacturing / Mechanical / Industrial Engineering</v>
+        <v>Controls Engineering</v>
       </c>
       <c r="D309" t="str">
-        <v>January to June 2027 (per posting text)</v>
+        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
       </c>
       <c r="E309" t="str">
-        <v>Waltham, MA</v>
+        <v>Anoka, MN</v>
       </c>
       <c r="F309">
-        <v>10</v>
+        <v>1127</v>
       </c>
       <c r="G309" t="str">
-        <v>$25.00-$28.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H309" t="str">
-        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015874986-transducer-manufacturing-engineering-co-op</v>
+        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Electrical-Controls-Engineering-Co-Op--January---August-2027-_R23894</v>
       </c>
       <c r="I309" t="str">
-        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116547, posted 2026-10-02.</v>
+        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, req R23894, posted 2026-10-02/03.</v>
       </c>
       <c r="J309" t="str">
-        <v>Evident/Wabtec Inspection Technologies division. New employer for the tracker. Boston-area.</v>
+        <v>Controls-discipline sibling to nVent's other already-tracked Jan-start Anoka, MN co-ops.</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>Wabtec (Evident / Wabtec Inspection Technologies)</v>
+        <v>Schaeffler</v>
       </c>
       <c r="B310" t="str">
-        <v>Co-Op, Test Engineer - Transducer</v>
+        <v>Co-op Mechanical Engineering</v>
       </c>
       <c r="C310" t="str">
-        <v>Manufacturing / Test Engineering</v>
+        <v>Mechanical Engineering (Engine/Chassis R&amp;D)</v>
       </c>
       <c r="D310" t="str">
-        <v>January - June 2027 (stated in title)</v>
+        <v>Winter 2027</v>
       </c>
       <c r="E310" t="str">
-        <v>State College, PA</v>
+        <v>Troy, MI</v>
       </c>
       <c r="F310">
-        <v>390</v>
+        <v>720</v>
       </c>
       <c r="G310" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H310" t="str">
-        <v>https://jobs.smartrecruiters.com/Wabtec/3743990015763566-co-op-test-engineer-transducer-january-june-2027-</v>
+        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechanical-Engineering-Winter-2027-MI-48083/1425401433/</v>
       </c>
       <c r="I310" t="str">
-        <v>Yes — fetched directly via Wabtec's own SmartRecruiters API (HTTP 200, active:true), req R0116563, posted 2026-09-29.</v>
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present, no closed/expired message.</v>
       </c>
       <c r="J310" t="str">
-        <v>Sibling req to the Waltham, MA transducer co-op above; hands-on fixture/test-system work.</v>
+        <v>New employer for the tracker. Not Boston-area.</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>nVent</v>
+        <v>Schaeffler</v>
       </c>
       <c r="B311" t="str">
-        <v>Electrical/Controls Engineering Co-Op</v>
+        <v>Co-op Mechatronics Engineering</v>
       </c>
       <c r="C311" t="str">
-        <v>Controls Engineering</v>
+        <v>Mechatronics (Mechanical + Controls/Systems Integration)</v>
       </c>
       <c r="D311" t="str">
-        <v>January - August 2027 (spans Winter 2026/2027 and Spring 2027)</v>
+        <v>Winter 2027</v>
       </c>
       <c r="E311" t="str">
-        <v>Anoka, MN</v>
+        <v>Troy, MI</v>
       </c>
       <c r="F311">
-        <v>1127</v>
+        <v>720</v>
       </c>
       <c r="G311" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H311" t="str">
-        <v>https://nvent.wd5.myworkdayjobs.com/nVent/job/Anoka-MN-US/Electrical-Controls-Engineering-Co-Op--January---August-2027-_R23894</v>
+        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechatronics-Engineering-Winter-2027-MI-48083/1425394833/</v>
       </c>
       <c r="I311" t="str">
-        <v>Yes — fetched directly via nVent's Workday CXS API (HTTP 200), canApply true, req R23894, posted 2026-10-02/03.</v>
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present.</v>
       </c>
       <c r="J311" t="str">
-        <v>Controls-discipline sibling to nVent's other already-tracked Jan-start Anoka, MN co-ops.</v>
+        <v>Sibling req to the Mechanical Engineering co-op above, same site/season.</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>Schaeffler</v>
+        <v>SSOE Group</v>
       </c>
       <c r="B312" t="str">
-        <v>Co-op Mechanical Engineering</v>
+        <v>Mechanical Engineering Co-op</v>
       </c>
       <c r="C312" t="str">
-        <v>Mechanical Engineering (Engine/Chassis R&amp;D)</v>
+        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
       </c>
       <c r="D312" t="str">
-        <v>Winter 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E312" t="str">
-        <v>Troy, MI</v>
+        <v>Toledo, OH</v>
       </c>
       <c r="F312">
-        <v>720</v>
+        <v>700</v>
       </c>
       <c r="G312" t="str">
-        <v>Not stated on posting</v>
+        <v>Not independently confirmed this run (an older/cached listing cited $19-23/hr for a prior cycle)</v>
       </c>
       <c r="H312" t="str">
-        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechanical-Engineering-Winter-2027-MI-48083/1425401433/</v>
+        <v>https://careers-ssoe.icims.com/jobs/3885/mechanical-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I312" t="str">
-        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present, no closed/expired message.</v>
+        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml), which lists only currently-active job URLs; job ID 3885 present with lastmod 2026-09-21. Still cannot reach the job-detail page itself (true JS-rendered React SPA wrapped around the marketing site; both curl and WebFetch return only the static shell) to confirm full description, pay, or Apply button.</v>
       </c>
       <c r="J312" t="str">
-        <v>New employer for the tracker. Not Boston-area.</v>
+        <v>New employer for the tracker (architecture/engineering design firm, MEP/HVAC discipline — borderline fit, Hamza's call). Job ID 3885.</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>Schaeffler</v>
+        <v>SSOE Group</v>
       </c>
       <c r="B313" t="str">
-        <v>Co-op Mechatronics Engineering</v>
+        <v>Mechanical Engineering Co-op</v>
       </c>
       <c r="C313" t="str">
-        <v>Mechatronics (Mechanical + Controls/Systems Integration)</v>
+        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
       </c>
       <c r="D313" t="str">
-        <v>Winter 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E313" t="str">
-        <v>Troy, MI</v>
+        <v>Nashville, TN</v>
       </c>
       <c r="F313">
-        <v>720</v>
+        <v>1090</v>
       </c>
       <c r="G313" t="str">
-        <v>Not stated on posting</v>
+        <v>Not independently confirmed this run</v>
       </c>
       <c r="H313" t="str">
-        <v>https://jobs.schaeffler.com/job/Troy,-MI-Co-op-Mechatronics-Engineering-Winter-2027-MI-48083/1425394833/</v>
+        <v>https://careers-ssoe.icims.com/jobs/3886/mechanical-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I313" t="str">
-        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.schaeffler.com (employer's own career site), HTTP 200, 'Apply now' button present.</v>
+        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml); job ID 3886 present with lastmod 2026-09-28. Job-detail page still unreachable (JS-rendered React SPA).</v>
       </c>
       <c r="J313" t="str">
-        <v>Sibling req to the Mechanical Engineering co-op above, same site/season.</v>
+        <v>Sibling req to the Toledo, OH SSOE Mechanical Engineering Co-op. Job ID 3886. MEP/HVAC discipline — borderline fit.</v>
       </c>
     </row>
     <row r="314">
@@ -11906,10 +11906,10 @@
         <v>SSOE Group</v>
       </c>
       <c r="B314" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>Structural Engineering Co-op</v>
       </c>
       <c r="C314" t="str">
-        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
+        <v>Structural Engineering</v>
       </c>
       <c r="D314" t="str">
         <v>Spring 2027</v>
@@ -11921,208 +11921,240 @@
         <v>700</v>
       </c>
       <c r="G314" t="str">
-        <v>Not independently confirmed this run (an older/cached listing cited $19-23/hr for a prior cycle)</v>
+        <v>Not independently confirmed this run</v>
       </c>
       <c r="H314" t="str">
-        <v>https://careers-ssoe.icims.com/jobs/3885/mechanical-engineering-co-op---spring-2027/job</v>
+        <v>https://careers-ssoe.icims.com/jobs/3881/structural-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I314" t="str">
-        <v>Partial — 2026-10-03 ~07:00 UTC: confirmed via direct fetch of careers-ssoe.icims.com's own search-results page (HTTP 200); job title/ID/location appear in the server-rendered HTML confirming the listing is currently live, but the individual job-detail page is JS-rendered and could not be independently fetched to confirm full description, pay, or Apply button.</v>
+        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml); job ID 3881 present with lastmod 2026-09-21. Job-detail page still unreachable (JS-rendered React SPA).</v>
       </c>
       <c r="J314" t="str">
-        <v>New employer for the tracker (architecture/engineering design firm, MEP/HVAC discipline — borderline fit, Hamza's call). Job ID 3885.</v>
+        <v>Job ID 3881. Structural Engineering is within Hamza's target discipline list.</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>SSOE Group</v>
+        <v>Sanofi</v>
       </c>
       <c r="B315" t="str">
-        <v>Mechanical Engineering Co-op</v>
+        <v>2027 Spring Co-op Opportunities</v>
       </c>
       <c r="C315" t="str">
-        <v>Mechanical Engineering (HVAC/building-systems design for manufacturing facilities)</v>
+        <v>Multi-track (Material Sciences, Process Chemistry, Laboratory Automation — process/materials-engineering-adjacent)</v>
       </c>
       <c r="D315" t="str">
-        <v>Spring 2027</v>
+        <v>6-month duration starting January 2027</v>
       </c>
       <c r="E315" t="str">
-        <v>Nashville, TN</v>
+        <v>Cambridge, MA</v>
       </c>
       <c r="F315">
-        <v>1090</v>
+        <v>3</v>
       </c>
       <c r="G315" t="str">
-        <v>Not independently confirmed this run</v>
+        <v>$27-$60/hr (stated on posting, varies by role/experience)</v>
       </c>
       <c r="H315" t="str">
-        <v>https://careers-ssoe.icims.com/jobs/3886/mechanical-engineering-co-op---spring-2027/job</v>
+        <v>https://jobs.sanofi.com/en/job/cambridge/2027-spring-co-op-opportunities-cambridge-ma/2649/41259853312</v>
       </c>
       <c r="I315" t="str">
-        <v>Partial — 2026-10-03 ~07:00 UTC: same verification method as the Toledo, OH sibling req above — confirmed live via direct ATS search-results fetch (HTTP 200), job-detail page JS-rendered/unconfirmed.</v>
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.sanofi.com (employer's own career site), HTTP 200, 'Apply now' button present, application deadline Nov 13, 2026 stated on posting.</v>
       </c>
       <c r="J315" t="str">
-        <v>Sibling req to the Toledo, OH SSOE Mechanical Engineering Co-op. Job ID 3886. MEP/HVAC discipline — borderline fit.</v>
+        <v>Right in the Boston metro. Sanofi is already tracked for Framingham, MA and Swiftwater, PA — this Cambridge req is a distinct posting/location. Multi-track req; Material Sciences/Process Chemistry/Lab Automation tracks are the closest fit to Hamza's target disciplines. A sibling Waltham, MA posting exists but is dominated by life-sciences tracks — excluded, see `checked`.</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>SSOE Group</v>
+        <v>MIT Lincoln Laboratory</v>
       </c>
       <c r="B316" t="str">
-        <v>Structural Engineering Co-op</v>
+        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
       </c>
       <c r="C316" t="str">
-        <v>Structural Engineering</v>
+        <v>Mechanical Engineering</v>
       </c>
       <c r="D316" t="str">
-        <v>Spring 2027</v>
+        <v>Winter/Spring 2027</v>
       </c>
       <c r="E316" t="str">
-        <v>Toledo, OH</v>
+        <v>Lexington, MA</v>
       </c>
       <c r="F316">
-        <v>700</v>
+        <v>12</v>
       </c>
       <c r="G316" t="str">
-        <v>Not independently confirmed this run</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H316" t="str">
-        <v>https://careers-ssoe.icims.com/jobs/3881/structural-engineering-co-op---spring-2027/job</v>
+        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
       </c>
       <c r="I316" t="str">
-        <v>Partial — 2026-10-03 ~07:00 UTC: same verification method as the SSOE Mechanical Engineering reqs above — confirmed live via direct ATS search-results fetch (HTTP 200), job-detail page JS-rendered/unconfirmed.</v>
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via careers.ll.mit.edu (employer's own SuccessFactors career site), HTTP 200, 'Apply now' link present, posted 2026-09-28.</v>
       </c>
       <c r="J316" t="str">
-        <v>Job ID 3881. Structural Engineering is within Hamza's target discipline list.</v>
+        <v>Right in the Boston metro. Distinct from the already-tracked Microfabrication Industrial Eng Co-Op (Jan-Aug 2027) reqs — this is a separate Group 07-71 Mechanical Engineering req.</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>Sanofi</v>
+        <v>Symbotic</v>
       </c>
       <c r="B317" t="str">
-        <v>2027 Spring Co-op Opportunities</v>
+        <v>Co-op - Hardware Engineer</v>
       </c>
       <c r="C317" t="str">
-        <v>Multi-track (Material Sciences, Process Chemistry, Laboratory Automation — process/materials-engineering-adjacent)</v>
+        <v>Mechanical / Electro-Mechanical Engineering</v>
       </c>
       <c r="D317" t="str">
-        <v>6-month duration starting January 2027</v>
+        <v>Spring (January-May 2027)</v>
       </c>
       <c r="E317" t="str">
-        <v>Cambridge, MA</v>
+        <v>Wilmington, MA (ITC site)</v>
       </c>
       <c r="F317">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="G317" t="str">
-        <v>$27-$60/hr (stated on posting, varies by role/experience)</v>
+        <v>$29.00-$40.00/hr</v>
       </c>
       <c r="H317" t="str">
-        <v>https://jobs.sanofi.com/en/job/cambridge/2027-spring-co-op-opportunities-cambridge-ma/2649/41259853312</v>
+        <v>https://www.symbotic.com/careers/jobs/R7976/</v>
       </c>
       <c r="I317" t="str">
-        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via jobs.sanofi.com (employer's own career site), HTTP 200, 'Apply now' button present, application deadline Nov 13, 2026 stated on posting.</v>
+        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via symbotic.com/careers (employer's own career site), season and pay range stated explicitly in body text, active 'Apply Now' button present (routes to Workday; not independently re-tested end-to-end due to a concurrent Workday platform-wide maintenance outage at check time).</v>
       </c>
       <c r="J317" t="str">
-        <v>Right in the Boston metro. Sanofi is already tracked for Framingham, MA and Swiftwater, PA — this Cambridge req is a distinct posting/location. Multi-track req; Material Sciences/Process Chemistry/Lab Automation tracks are the closest fit to Hamza's target disciplines. A sibling Waltham, MA posting exists but is dominated by life-sciences tracks — excluded, see `checked`.</v>
+        <v>Right in the Boston metro. CAD design/electro-mechanical debugging/SolidWorks/GD&amp;T/robotics work. Req R7976, distinct from the already-excluded 'Intern - Hardware Engineer' (R5394).</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>MIT Lincoln Laboratory</v>
+        <v>RTX / Collins Aerospace</v>
       </c>
       <c r="B318" t="str">
-        <v>Mechanical Engineering Co-Op (Winter/Spring 2027) - Group 07-71</v>
+        <v>Mechanical Design Engineering Co-op (Spring 2027)</v>
       </c>
       <c r="C318" t="str">
         <v>Mechanical Engineering</v>
       </c>
       <c r="D318" t="str">
-        <v>Winter/Spring 2027</v>
+        <v>Spring 2027</v>
       </c>
       <c r="E318" t="str">
-        <v>Lexington, MA</v>
+        <v>Uniontown, OH</v>
       </c>
       <c r="F318">
-        <v>12</v>
+        <v>610</v>
       </c>
       <c r="G318" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H318" t="str">
-        <v>https://careers.ll.mit.edu/job/Lexington-Mechanical-Engineering-Co-Op-%28WinterSpring-2027%29-Group-07-71-MA-02420/1434254300/</v>
+        <v>https://globalhr.wd5.myworkdayjobs.com/en-US/REC_RTX_Ext_Gateway/job/US-OH-UNIONTOWN-1555--1555-Corporate-Woods-Pkwy--CORP-WOODS/Mechanical-Design-Engineering-Co-op--Spring-2027-_01874486</v>
       </c>
       <c r="I318" t="str">
-        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via careers.ll.mit.edu (employer's own SuccessFactors career site), HTTP 200, 'Apply now' link present, posted 2026-09-28.</v>
+        <v>Yes — fetched directly via RTX's own Workday CXS API, req 01874486, posted 2026-10-02 (1 day old at check time). Title states season explicitly.</v>
       </c>
       <c r="J318" t="str">
-        <v>Right in the Boston metro. Distinct from the already-tracked Microfabrication Industrial Eng Co-Op (Jan-Aug 2027) reqs — this is a separate Group 07-71 Mechanical Engineering req.</v>
+        <v>This req had previously shown as tenant-level 403-blocked on earlier runs; access cleared this run and the posting fetched cleanly. Distinct from the now-closed Cedar Rapids Chemical/Materials Co-op (01871473, moved to checked this run).</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>Symbotic</v>
+        <v>Daktronics</v>
       </c>
       <c r="B319" t="str">
-        <v>Co-op - Hardware Engineer</v>
+        <v>Manufacturing Process Engineer Co-op Intern</v>
       </c>
       <c r="C319" t="str">
-        <v>Mechanical / Electro-Mechanical Engineering</v>
+        <v>Manufacturing / Process / Industrial Engineering</v>
       </c>
       <c r="D319" t="str">
-        <v>Spring (January-May 2027)</v>
+        <v>Winter/Spring 2027 (Jan 11, 2027 – Aug 13, 2027 term option)</v>
       </c>
       <c r="E319" t="str">
-        <v>Wilmington, MA (ITC site)</v>
+        <v>Sioux Falls, SD</v>
       </c>
       <c r="F319">
-        <v>17</v>
+        <v>1450</v>
       </c>
       <c r="G319" t="str">
-        <v>$29.00-$40.00/hr</v>
+        <v>Not stated on posting</v>
       </c>
       <c r="H319" t="str">
-        <v>https://www.symbotic.com/careers/jobs/R7976/</v>
+        <v>https://careers-daktronics.icims.com/jobs/7522/job</v>
       </c>
       <c r="I319" t="str">
-        <v>Yes — 2026-10-03 ~07:00 UTC: fetched directly via symbotic.com/careers (employer's own career site), season and pay range stated explicitly in body text, active 'Apply Now' button present (routes to Workday; not independently re-tested end-to-end due to a concurrent Workday platform-wide maintenance outage at check time).</v>
+        <v>Yes — fetched the actual iCIMS posting directly; 'Apply for this job online' button present and functional. Posting offers two term options (Jan 11 2027–Aug 13 2027, or May 17 2027–Dec 10 2027); the former qualifies as Winter/Spring 2027.</v>
       </c>
       <c r="J319" t="str">
-        <v>Right in the Boston metro. CAD design/electro-mechanical debugging/SolidWorks/GD&amp;T/robotics work. Req R7976, distinct from the already-excluded 'Intern - Hardware Engineer' (R5394).</v>
+        <v>New company. Preferred majors stated as Mechanical Engineering, Industrial Engineering, or related.</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>Analogic Corporation</v>
+        <v>Greenheck Group</v>
       </c>
       <c r="B320" t="str">
-        <v>Manufacturing Engineering Co-Op</v>
+        <v>Machine Design and Controls Engineering Co-op</v>
       </c>
       <c r="C320" t="str">
-        <v>Manufacturing Engineering</v>
+        <v>Mechanical / Controls Engineering</v>
       </c>
       <c r="D320" t="str">
-        <v>Spring 2027 Co-Op Program</v>
+        <v>Winter/Spring 2027 (January–August term option)</v>
       </c>
       <c r="E320" t="str">
-        <v>Salem, NH</v>
+        <v>Schofield, WI</v>
       </c>
       <c r="F320">
-        <v>28</v>
+        <v>1180</v>
       </c>
       <c r="G320" t="str">
         <v>Not stated on posting</v>
       </c>
       <c r="H320" t="str">
-        <v>https://recruiting.ultipro.com/ANA1003ALOG/JobBoard/a4de26ba-aa2d-4502-9d0f-577ea07dc7ca/OpportunityDetail?opportunityId=a25687db-ac1a-46ea-90a4-97fe04c715c6</v>
+        <v>https://greenheckgroup.wd5.myworkdayjobs.com/external/job/Schofield-WI/Machine-Design-and-Controls-Engineering-Co-op_JR104723</v>
       </c>
       <c r="I320" t="str">
-        <v>Partial — 2026-10-03 ~13:00 UTC: confirmed live via a direct query of Analogic's own UltiPro ATS JSON search API (returned in the active-search result set, RequisitionNumber MANUF002804, PostedDate 2026-09-21, 'Spring 2027 Co-Op Program' stated as the literal first line of the body description). The human-facing detail page is a React SPA that did not render statically, so pay and full requirements could not be independently confirmed beyond the API's own fields.</v>
+        <v>Yes — WebFetch could not render the Workday JS shell, so queried Greenheck's own Workday CXS JSON API directly and received the full live posting (title, description, 'Posted 10 Days Ago' as of 2026-10-03). Did not independently click through the Apply button.</v>
       </c>
       <c r="J320" t="str">
-        <v>Close to Boston (~28 mi). Distinct from Analogic's other open reqs at the same Salem, NH site: 'Engineering Co-Op' (ENGIN002794, security-imaging, no season stated) and 'Hardware/Software Engineering Co-Op' (COOPS002797, RF/electrical) — both excluded, see checked.</v>
+        <v>New company (commercial HVAC/air-movement equipment manufacturer). Req JR104723. Posting lists acceptable majors as Industrial, Manufacturing, Mechanical, Computer, Electrical, or Robotics; the Machine Design track covers CAD design, engineering analysis, and manufacturing processes. 8-month co-op term offered as 'January to August OR May to December' — Jan–Aug option qualifies.</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Marmon Holdings (Powerex-Iwata Air Technology)</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Controls Engineer Co-op (Spring 2027)</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Controls Engineering (manufacturing/industrial)</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Mt. Juliet, TN</v>
+      </c>
+      <c r="F321">
+        <v>1030</v>
+      </c>
+      <c r="G321" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H321" t="str">
+        <v>https://marmon.wd501.myworkdayjobs.com/Marmon_MSIP_Internships/job/Mt-Juliet-TN/Controls-Engineer-Co-op--Spring-2027-_JR0000045809-1</v>
+      </c>
+      <c r="I321" t="str">
+        <v>Yes — Workday CXS JSON API returned the full live posting (req JR0000045809, posted 2026-09-15, season stated in the title itself). Did not independently click through the Apply button.</v>
+      </c>
+      <c r="J321" t="str">
+        <v>New company (Marmon Holdings/Berkshire Hathaway industrial group; Powerex-Iwata Air Technology is an air-compressor manufacturing subsidiary). Co-op works with mechanical and electrical engineers on manufacturing-floor PLC/HMI/VFD controls and new-product solutions — controls-adjacent discipline fit.</v>
       </c>
     </row>
   </sheetData>
@@ -12596,14 +12628,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M320"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M321"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C655"/>
+  <dimension ref="A1:C671"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -19806,9 +19838,185 @@
         <v>2026-10-03 ~13:00 UTC: found during the same sweep, confirmed canApply:true, but explicitly 'May - December 2027' — wrong season. Not added.</v>
       </c>
     </row>
+    <row r="656">
+      <c r="A656" t="str">
+        <v>RTX / Collins Aerospace (Cedar Rapids, IA)</v>
+      </c>
+      <c r="B656" t="str">
+        <v>Chemical/Materials Engineering Co-op (Winter/Spring 2027), req 01871473 — previously tracked in `rows`</v>
+      </c>
+      <c r="C656" t="str">
+        <v>2026-10-03 ~19:00 UTC: CLOSED, moved from `rows`. Direct Workday CXS API searchText="01871473" now returns zero results, while the same API call works normally for dozens of other current Cedar Rapids reqs — a clean negative signal, not a block. Posting's own end date was 2026-10-03 (today), as flagged in the prior two runs.</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="str">
+        <v>Flex (Flextronics International, Orangeburg, SC)</v>
+      </c>
+      <c r="B657" t="str">
+        <v>Mechanical Engineering Co-op - Spring 2027, req WD227049 — previously tracked in `rows`</v>
+      </c>
+      <c r="C657" t="str">
+        <v>2026-10-03 ~19:00 UTC: CLOSED, moved from `rows`. Direct Workday CXS API searchText="WD227049" now returns zero results (search mechanism independently validated against a known-live req). Full Orangeburg, SC Intern/Co-op facet pull shows only 3 remaining reqs there, none matching this one. Posting's own end date was 2026-10-03 (today), as flagged in the prior run.</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="str">
+        <v>Analogic Corporation (Salem, NH)</v>
+      </c>
+      <c r="B658" t="str">
+        <v>Manufacturing Engineering Co-Op, req MANUF002804 — previously tracked in `rows` as Partial</v>
+      </c>
+      <c r="C658" t="str">
+        <v>2026-10-03 ~19:00 UTC: likely CLOSED (moderate-high confidence), moved from `rows`. Analogic's real ATS (UKG Pro Recruiting) server-renders a seed list of all currently-open company-wide postings for SEO; tested with multiple query/sort variations, all consistently showing only 6 roles company-wide (Field Service Technician x4, Project Manager-Field Service, Area Manager Field Service, Installation Technician x2) — no engineering co-op of any kind remains. Could not reach a definitive 404/expired marker on the specific req page itself, so this is a strong negative signal rather than a fully confirmed closure, but is no longer appearing as live anywhere on the employer's own board.</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="str">
+        <v>Wabtec (Oak Creek, WI — Nordco brand)</v>
+      </c>
+      <c r="B659" t="str">
+        <v>Controls Engineering Intern (R0116732); Mechanical Engineer Intern - Production Operations (R0116733); Mechanical Engineer Intern - New Product Development (R0116734)</v>
+      </c>
+      <c r="C659" t="str">
+        <v>2026-10-03 ~19:00 UTC: all 3 confirmed live and discipline-fitting (posted 2026-09-30) via SmartRecruiters, but none states a season/term ('Spring 2027', 'Winter 2026', or any start-date field) anywhere in the full job description. Not added per the strict season-verification bar; worth re-checking if season wording is ever added.</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="str">
+        <v>Re:Build Manufacturing</v>
+      </c>
+      <c r="B660" t="str">
+        <v>Automation &amp; Controls Engineer Co-op/Intern, Rochester/Rush NY</v>
+      </c>
+      <c r="C660" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed live via direct Greenhouse API fetch (published 2026-09-21), $21-25/hr. Excluded: required majors are Mechatronics/Electrical/Computer Engineering (no Mechanical or Controls Engineering major listed), and the posting's own screening question offers Spring, Summer, OR Fall 2027 interchangeably rather than a dedicated Spring 2027 cohort. Discipline leans EE/mechatronics — borderline, Hamza's call if he wants it reconsidered.</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="str">
+        <v>Verkada</v>
+      </c>
+      <c r="B661" t="str">
+        <v>Hardware Engineer (Winter Co-op), San Mateo, CA</v>
+      </c>
+      <c r="C661" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed via direct Greenhouse posting — explicitly an Electrical Engineering role (schematic capture, PCB layout). Discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="str">
+        <v>Delta Faucet (Masco)</v>
+      </c>
+      <c r="B662" t="str">
+        <v>Hardware Engineering Co-op (Electrical Engineering), Indianapolis, IN</v>
+      </c>
+      <c r="C662" t="str">
+        <v>2026-10-03 ~19:00 UTC: title itself confirms Electrical Engineering discipline. Not pursued further.</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="str">
+        <v>Lennox International</v>
+      </c>
+      <c r="B663" t="str">
+        <v>Hardware Engineering Fall Co-op, Carrollton, TX</v>
+      </c>
+      <c r="C663" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed via direct iCIMS posting — Electrical Engineering discipline, and season is Fall (unspecified year), not Winter 2026/Spring 2027. Wrong season + discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="str">
+        <v>General Motors</v>
+      </c>
+      <c r="B664" t="str">
+        <v>2027 Co-Op – Manufacturing Controls Engineer, Detroit, MI</v>
+      </c>
+      <c r="C664" t="str">
+        <v>2026-10-03 ~19:00 UTC: despite the 'controls' title, the posting's own body text explicitly seeks 'Electrical Engineer Co-ops' with duties centered on PLC/HMI/robotics programming — no mechanical-engineering framing. Season unstated beyond '2027'. Excluded as primarily EE per the posting's own words; borderline call, flagged in case Hamza wants controls-titled EE-leaning roles reconsidered (precedent: nVent's Electrical/Controls Co-Op was accepted).</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="str">
+        <v>First Quality</v>
+      </c>
+      <c r="B665" t="str">
+        <v>Controls Engineer Intern or Co-Op, Anderson, SC</v>
+      </c>
+      <c r="C665" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed via direct Workday CXS data — req posted 30+ days ago with an internal startDate of 2025-09-19 and no season stated anywhere; appears to be a generic rolling/stale posting, not tied to a specific Winter 2026/Spring 2027 cohort. Excluded as unconfirmable season.</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="str">
+        <v>ControlTouch Systems</v>
+      </c>
+      <c r="B666" t="str">
+        <v>Controls Engineer Co-Op, Louisville, KY</v>
+      </c>
+      <c r="C666" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed open via direct Paylocity posting, but no season/term dates stated anywhere on the page. Excluded as unconfirmable season.</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="str">
+        <v>Daktronics</v>
+      </c>
+      <c r="B667" t="str">
+        <v>Firmware/Hardware Design Co-op Intern, Brookings, SD</v>
+      </c>
+      <c r="C667" t="str">
+        <v>2026-10-03 ~19:00 UTC: sibling req to the qualifying Manufacturing Process Engineer Co-op (added to `rows`). Confirmed via direct iCIMS posting — Electrical/Computer/Software Engineering discipline, and stated term is 'May 17, 2027 to December 10, 2027' (Summer/Fall 2027). Wrong season + discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="str">
+        <v>Olin</v>
+      </c>
+      <c r="B668" t="str">
+        <v>Process Controls Engineer Co-Op, Freeport, TX</v>
+      </c>
+      <c r="C668" t="str">
+        <v>2026-10-03 ~19:00 UTC: posting's own title states 'Fall 2027'. Wrong season, not pursued further.</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="str">
+        <v>American Axle &amp; Manufacturing</v>
+      </c>
+      <c r="B669" t="str">
+        <v>Electrical Engineering Co-op, Detroit, MI</v>
+      </c>
+      <c r="C669" t="str">
+        <v>2026-10-03 ~19:00 UTC: title confirms Electrical Engineering discipline; no season stated either. Not pursued further.</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="str">
+        <v>Delta Air Lines</v>
+      </c>
+      <c r="B670" t="str">
+        <v>Intern, Research and Development Hardware Design Engineer, Atlanta, GA</v>
+      </c>
+      <c r="C670" t="str">
+        <v>2026-10-03 ~19:00 UTC: aggregators state Spring 2027, but described duties (full-stack development, LLM/Copilot-style tooling, breadboard/soldering, UART/SPI/I2C) are an embedded hardware/software hybrid role, not a mechanical/aero/manufacturing discipline fit. Excluded on discipline grounds; did not independently re-open Delta's own ATS page for this one (time-boxed).</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="str">
+        <v>Charles River Analytics (Cambridge, MA)</v>
+      </c>
+      <c r="B671" t="str">
+        <v>General intern/co-op search — distinct from the already-checked Charles River Laboratories</v>
+      </c>
+      <c r="C671" t="str">
+        <v>2026-10-03 ~19:00 UTC: confirmed this is a software/AI/robotics-autonomy R&amp;D intern program (ML, NLP, computer vision, autonomy), not a mechanical/hardware-engineering discipline. Excluded on discipline grounds.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C655"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C671"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 9 new postings, 7 checked-excluded (2026-10-04 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V4rJyFbiH1B3iNHPaLc1zJ
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M321"/>
+  <dimension ref="A1:M330"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -11857,13 +11857,13 @@
         <v>700</v>
       </c>
       <c r="G312" t="str">
-        <v>Not independently confirmed this run (an older/cached listing cited $19-23/hr for a prior cycle)</v>
+        <v>$19-23/hr</v>
       </c>
       <c r="H312" t="str">
         <v>https://careers-ssoe.icims.com/jobs/3885/mechanical-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I312" t="str">
-        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml), which lists only currently-active job URLs; job ID 3885 present with lastmod 2026-09-21. Still cannot reach the job-detail page itself (true JS-rendered React SPA wrapped around the marketing site; both curl and WebFetch return only the static shell) to confirm full description, pay, or Apply button.</v>
+        <v>Yes — 2026-10-04: fetched the iCIMS job URL with ?in_iframe=1 appended, which serves server-rendered HTML instead of the JS-shell SPA that blocked prior runs. Full description, pay ($19-23/hr), and 'Apply for this job online' button all confirmed present.</v>
       </c>
       <c r="J312" t="str">
         <v>New employer for the tracker (architecture/engineering design firm, MEP/HVAC discipline — borderline fit, Hamza's call). Job ID 3885.</v>
@@ -11889,13 +11889,13 @@
         <v>1090</v>
       </c>
       <c r="G313" t="str">
-        <v>Not independently confirmed this run</v>
+        <v>$19-23/hr</v>
       </c>
       <c r="H313" t="str">
         <v>https://careers-ssoe.icims.com/jobs/3886/mechanical-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I313" t="str">
-        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml); job ID 3886 present with lastmod 2026-09-28. Job-detail page still unreachable (JS-rendered React SPA).</v>
+        <v>Yes — 2026-10-04: fetched the iCIMS job URL with ?in_iframe=1 appended (bypasses the JS-shell SPA). Full description, pay ($19-23/hr), and apply button confirmed present.</v>
       </c>
       <c r="J313" t="str">
         <v>Sibling req to the Toledo, OH SSOE Mechanical Engineering Co-op. Job ID 3886. MEP/HVAC discipline — borderline fit.</v>
@@ -11921,13 +11921,13 @@
         <v>700</v>
       </c>
       <c r="G314" t="str">
-        <v>Not independently confirmed this run</v>
+        <v>$20-23/hr</v>
       </c>
       <c r="H314" t="str">
         <v>https://careers-ssoe.icims.com/jobs/3881/structural-engineering-co-op---spring-2027/job</v>
       </c>
       <c r="I314" t="str">
-        <v>Partial — 2026-10-03 ~19:00 UTC: additionally reconfirmed live via SSOE's own auto-generated ATS sitemap (careers-ssoe.icims.com/sitemap.xml); job ID 3881 present with lastmod 2026-09-21. Job-detail page still unreachable (JS-rendered React SPA).</v>
+        <v>Yes — 2026-10-04: fetched the iCIMS job URL with ?in_iframe=1 appended (bypasses the JS-shell SPA). Full description, pay ($20-23/hr), and apply button confirmed present.</v>
       </c>
       <c r="J314" t="str">
         <v>Job ID 3881. Structural Engineering is within Hamza's target discipline list.</v>
@@ -12155,6 +12155,294 @@
       </c>
       <c r="J321" t="str">
         <v>New company (Marmon Holdings/Berkshire Hathaway industrial group; Powerex-Iwata Air Technology is an air-compressor manufacturing subsidiary). Co-op works with mechanical and electrical engineers on manufacturing-floor PLC/HMI/VFD controls and new-product solutions — controls-adjacent discipline fit.</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>First Solar</v>
+      </c>
+      <c r="B322" t="str">
+        <v>Manufacturing Engineering Intern (Fall 2026/Spring 2027)</v>
+      </c>
+      <c r="C322" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Fall 2026/Spring 2027</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Perrysburg, OH</v>
+      </c>
+      <c r="F322">
+        <v>720</v>
+      </c>
+      <c r="G322" t="str">
+        <v>$22-25/hr</v>
+      </c>
+      <c r="H322" t="str">
+        <v>https://fa-esbv-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1025557</v>
+      </c>
+      <c r="I322" t="str">
+        <v>Yes — queried First Solar's own Oracle Cloud Recruiting REST API directly; full description pulled, title explicitly 'Fall 2026/Spring 2027,' application page confirmed HTTP 200.</v>
+      </c>
+      <c r="J322" t="str">
+        <v>New company for the tracker (solar panel manufacturer). Winter 2026 and Spring 2027 both fit within the stated Fall 2026/Spring 2027 term.</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>First Solar</v>
+      </c>
+      <c r="B323" t="str">
+        <v>Manufacturing Engineering Intern (Fall 2026/Spring 2027)</v>
+      </c>
+      <c r="C323" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Fall 2026/Spring 2027</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Trinity, AL</v>
+      </c>
+      <c r="F323">
+        <v>1150</v>
+      </c>
+      <c r="G323" t="str">
+        <v>$22-25/hr</v>
+      </c>
+      <c r="H323" t="str">
+        <v>https://fa-esbv-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1025558</v>
+      </c>
+      <c r="I323" t="str">
+        <v>Yes — same Oracle Cloud Recruiting REST API verification method as the Perrysburg, OH sibling req; HTTP 200.</v>
+      </c>
+      <c r="J323" t="str">
+        <v>Sibling req to the Perrysburg, OH First Solar Manufacturing Engineering Intern posting, same title/season/pay.</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>First Solar</v>
+      </c>
+      <c r="B324" t="str">
+        <v>Manufacturing Engineering Intern (Fall 2026/Spring 2027)</v>
+      </c>
+      <c r="C324" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Fall 2026/Spring 2027</v>
+      </c>
+      <c r="E324" t="str">
+        <v>New Iberia, LA</v>
+      </c>
+      <c r="F324">
+        <v>1700</v>
+      </c>
+      <c r="G324" t="str">
+        <v>$22-25/hr</v>
+      </c>
+      <c r="H324" t="str">
+        <v>https://fa-esbv-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1025559</v>
+      </c>
+      <c r="I324" t="str">
+        <v>Yes — same Oracle Cloud Recruiting REST API verification method as the Perrysburg, OH sibling req; HTTP 200.</v>
+      </c>
+      <c r="J324" t="str">
+        <v>Sibling req to the Perrysburg, OH First Solar Manufacturing Engineering Intern posting, same title/season/pay.</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>First Solar</v>
+      </c>
+      <c r="B325" t="str">
+        <v>Manufacturing Integration Intern (Spring 2027)</v>
+      </c>
+      <c r="C325" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Perrysburg, OH</v>
+      </c>
+      <c r="F325">
+        <v>720</v>
+      </c>
+      <c r="G325" t="str">
+        <v>Not stated on posting (generic benefits text only)</v>
+      </c>
+      <c r="H325" t="str">
+        <v>https://fa-esbv-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1/job/1026028</v>
+      </c>
+      <c r="I325" t="str">
+        <v>Yes — queried First Solar's own Oracle Cloud Recruiting REST API directly; title explicitly 'Spring 2027,' posted 2026-09-24, body states 'Expected Length: Fall/Spring, Minimum 3 months.' HTTP 200.</v>
+      </c>
+      <c r="J325" t="str">
+        <v>Distinct req from the Manufacturing Engineering Intern postings at the same site — this one is 'Manufacturing Integration.'</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Mack Trucks (Volvo Group)</v>
+      </c>
+      <c r="B326" t="str">
+        <v>Intern: Product Mechanical Engineer (Spring 2027)</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Mechanical/Vehicle Engineering</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Salem, VA</v>
+      </c>
+      <c r="F326">
+        <v>650</v>
+      </c>
+      <c r="G326" t="str">
+        <v>$17.00-$46.00/hr (standard range for all Volvo Group intern/co-op roles)</v>
+      </c>
+      <c r="H326" t="str">
+        <v>https://jobs.volvogroup.com/job/Salem-Intern-Product-Mechanical-Engineer-%28Spring-2027%29-VA-24153/1370132255/</v>
+      </c>
+      <c r="I326" t="str">
+        <v>Yes — direct fetch of the live posting page, HTTP 200, page title confirms '(Spring 2027)'; no 'no longer accepting' language found.</v>
+      </c>
+      <c r="J326" t="str">
+        <v>New company for the tracker. Role is on the Mack Medium Duty Engineering team.</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Mack Trucks (Volvo Group)</v>
+      </c>
+      <c r="B327" t="str">
+        <v>Intern: Manufacturing Engineer (Spring 2027)</v>
+      </c>
+      <c r="C327" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D327" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Middletown, PA</v>
+      </c>
+      <c r="F327">
+        <v>280</v>
+      </c>
+      <c r="G327" t="str">
+        <v>$17.00-$46.00/hr (standard range for all Volvo Group intern/co-op roles)</v>
+      </c>
+      <c r="H327" t="str">
+        <v>https://jobs.volvogroup.com/job/Middletown-Intern-Manufacturing-Engineer-%28Spring-2027%29-PA-17057/1370129155/</v>
+      </c>
+      <c r="I327" t="str">
+        <v>Yes — direct fetch of the live posting page, HTTP 200, title confirmed '(Spring 2027)'.</v>
+      </c>
+      <c r="J327" t="str">
+        <v>Sibling req to the Salem, VA Mack Trucks Product Mechanical Engineer intern posting.</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>Mack Trucks (Volvo Group)</v>
+      </c>
+      <c r="B328" t="str">
+        <v>Intern: Automation &amp; Process Improvement (Spring 2027)</v>
+      </c>
+      <c r="C328" t="str">
+        <v>Manufacturing/Controls (Autonomous Mobile Robot automation for manufacturing plant)</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E328" t="str">
+        <v>Shippensburg, PA</v>
+      </c>
+      <c r="F328">
+        <v>340</v>
+      </c>
+      <c r="G328" t="str">
+        <v>$17.00-$46.00/hr (standard range for all Volvo Group intern/co-op roles)</v>
+      </c>
+      <c r="H328" t="str">
+        <v>https://jobs.volvogroup.com/job/Shippensburg-Intern-Automation-%26-Process-Improvement-%28Spring-2027%29-PA-17257/1369287455/</v>
+      </c>
+      <c r="I328" t="str">
+        <v>Yes — direct fetch of the live posting page, HTTP 200, title confirmed '(Spring 2027)'.</v>
+      </c>
+      <c r="J328" t="str">
+        <v>Role explicitly covers Autonomous Mobile Robot (AMR) automation in a manufacturing plant — controls/manufacturing hybrid, within discipline fit.</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>GE Vernova</v>
+      </c>
+      <c r="B329" t="str">
+        <v>Manufacturing Engineering Intern - Spring 2027</v>
+      </c>
+      <c r="C329" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Erlanger, KY</v>
+      </c>
+      <c r="F329">
+        <v>900</v>
+      </c>
+      <c r="G329" t="str">
+        <v>$24.00-$31.00/hr</v>
+      </c>
+      <c r="H329" t="str">
+        <v>https://gevernova.wd5.myworkdayjobs.com/Vernova_ExternalSite/job/Erlanger/GE-Vernova-Manufacturing-Engineering-Intern---Spring-2027_R5053611-2</v>
+      </c>
+      <c r="I329" t="str">
+        <v>Yes — queried GE Vernova's own Workday CXS API directly (not the careers.gevernova.com marketing wrapper, which has repeatedly 404'd on other GE Vernova/Aerospace reqs); canApply:true, req posted 4 days prior to check, body explicitly states 'Employment dates: January 2027 through April 2027 (Spring).'</v>
+      </c>
+      <c r="J329" t="str">
+        <v>New company/req for the tracker, distinct from a previously-unresolved Greenville, SC GE Vernova lead.</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>RoboForce</v>
+      </c>
+      <c r="B330" t="str">
+        <v>Robotics Mechanical Engineering Intern (Fall/Winter 2026)</v>
+      </c>
+      <c r="C330" t="str">
+        <v>Robotics/Mechanical Design</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Fall/Winter 2026</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Milpitas, CA</v>
+      </c>
+      <c r="F330">
+        <v>2700</v>
+      </c>
+      <c r="G330" t="str">
+        <v>$6,000-$6,500/month</v>
+      </c>
+      <c r="H330" t="str">
+        <v>https://job-boards.greenhouse.io/roboforce/jobs/5441463008</v>
+      </c>
+      <c r="I330" t="str">
+        <v>Partial — confirmed live via direct Greenhouse API (posted 2026-10-01, very fresh). Title literally contains 'Winter 2026' (combined with Fall), but the job body itself never restates a season or explicit start/end dates, so it's unconfirmed from the posting's own text whether the term actually extends into Winter 2026 or is really Fall-only.</v>
+      </c>
+      <c r="J330" t="str">
+        <v>New company (robotics startup). Worth a closer look given the fresh posting date, but season wording in the title isn't corroborated by the body text.</v>
       </c>
     </row>
   </sheetData>
@@ -12628,14 +12916,14 @@
     <hyperlink ref="M200" r:id="rId467"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M321"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M330"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C671"/>
+  <dimension ref="A1:C678"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -20014,9 +20302,86 @@
         <v>2026-10-03 ~19:00 UTC: confirmed this is a software/AI/robotics-autonomy R&amp;D intern program (ML, NLP, computer vision, autonomy), not a mechanical/hardware-engineering discipline. Excluded on discipline grounds.</v>
       </c>
     </row>
+    <row r="672">
+      <c r="A672" t="str">
+        <v>Bose Corporation (Framingham, MA)</v>
+      </c>
+      <c r="B672" t="str">
+        <v>Mechanical Engineer Co-op, Concept Prototyping, req R26422</v>
+      </c>
+      <c r="C672" t="str">
+        <v>2026-10-04: resolved a standing ambiguous/HTTP-500 entry from a prior run. Found the correct live Workday tenant (boseallaboutme.wd503.myworkdayjobs.com) and confirmed the page's own embedded config flag postingAvailable:false — req is CLOSED.</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="str">
+        <v>General Dynamics Mission Systems (Quincy, MA)</v>
+      </c>
+      <c r="B673" t="str">
+        <v>Systems Engineering Intern - Autonomous Maritime Platforms</v>
+      </c>
+      <c r="C673" t="str">
+        <v>2026-10-04: confirmed live via direct fetch, but explicitly 'Summer of 2027' in the posting body. Wrong season (otherwise a strong Boston-area fit).</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="str">
+        <v>RTX / Collins Aerospace (Tewksbury, MA)</v>
+      </c>
+      <c r="B674" t="str">
+        <v>Systems Engineer Intern, req 01879053</v>
+      </c>
+      <c r="C674" t="str">
+        <v>2026-10-04: confirmed live via RTX's own Workday CXS API, but no season/term word (Spring/Summer/Winter/2027) found anywhere in the body. Excluded as unconfirmable season.</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="str">
+        <v>RTX / Collins Aerospace (Woburn, MA)</v>
+      </c>
+      <c r="B675" t="str">
+        <v>Systems Engineer Intern, req 01875985</v>
+      </c>
+      <c r="C675" t="str">
+        <v>2026-10-04: confirmed live via RTX's own Workday CXS API, but no season/term word found anywhere in the body. Excluded as unconfirmable season.</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="str">
+        <v>Amphenol Borisch Technologies (Grand Rapids, MI)</v>
+      </c>
+      <c r="B676" t="str">
+        <v>'Manufacturing Engineer Intern (Spring 2027)'</v>
+      </c>
+      <c r="C676" t="str">
+        <v>2026-10-04: aggregator-only lead (ZipRecruiter/Indeed); checked the company's real ATS (borisch.acquiretm.com, 58 open reqs) directly and found zero internship-titled postings currently live. Unverifiable/likely stale, not added.</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="str">
+        <v>Mytra (Brisbane, CA)</v>
+      </c>
+      <c r="B677" t="str">
+        <v>'Robotics Intern - Winter 2026'</v>
+      </c>
+      <c r="C677" t="str">
+        <v>2026-10-04: aggregator-only lead (LinkedIn); could not locate the company's real ATS (not Greenhouse/Lever/Ashby under common slug guesses, company site not independently fetchable). Unverifiable, not added.</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="str">
+        <v>Mill (San Bruno, CA)</v>
+      </c>
+      <c r="B678" t="str">
+        <v>'Product Design Engineering Intern, Fall/Winter 2026'</v>
+      </c>
+      <c r="C678" t="str">
+        <v>2026-10-04: confirmed live via Greenhouse API, but first_published back in March 2026 and the body text never restates the Fall/Winter 2026 season from the title — likely a stale/rolling posting whose title hasn't been refreshed. Low confidence, not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C671"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C678"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 4 checked-excluded (2026-10-04 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N3yBNfa5ZGfDNuYC2YTzpv
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M341"/>
+  <dimension ref="A1:M344"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -12785,7 +12785,103 @@
         <v>Partial — the Oracle Cloud candidate-experience page is JS-rendered and could not be fully loaded; independently confirmed via a direct fetch of the page's server-rendered meta tags that a live posting exists at this exact URL with og:title '2027 Spring Engineering Co-Op - Chicago, IL' matching the 15-week co-op program language. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
       </c>
       <c r="J341" t="str">
-        <v>New company for the tracker. Sherwin-Williams reportedly has sibling 2027 Spring Engineering Co-Op postings in Los Angeles CA, Richmond KY, Holland MI, and Waco TX per secondary sources — not individually verified, not added.</v>
+        <v>New company for the tracker. Sherwin-Williams reportedly has sibling 2027 Spring Engineering Co-Op postings in Los Angeles CA, Richmond KY, Holland MI, and Waco TX per secondary sources. Los Angeles, Holland MI, and Waco TX were independently verified and added below (2026-10-04); Richmond KY could not be independently confirmed (see `checked`).</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>Sherwin-Williams</v>
+      </c>
+      <c r="B342" t="str">
+        <v>2027 Spring Engineering Co-Op</v>
+      </c>
+      <c r="C342" t="str">
+        <v>Mechanical/Electrical/Chemical Engineering (manufacturing/plant engineering co-op)</v>
+      </c>
+      <c r="D342" t="str">
+        <v>2027 Spring Engineering Co-Op, 15-week program, January 2027 start (per posting body)</v>
+      </c>
+      <c r="E342" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F342">
+        <v>2591</v>
+      </c>
+      <c r="G342" t="str">
+        <v>Reported as $24/hr per aggregator sources — not independently confirmed</v>
+      </c>
+      <c r="H342" t="str">
+        <v>https://ejhp.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/job/2624794</v>
+      </c>
+      <c r="I342" t="str">
+        <v>Partial — the Oracle Cloud candidate-experience page is JS-rendered and could not be fully loaded; independently confirmed via a direct curl fetch of the page's server-rendered meta tags that a live posting exists at this exact URL with og:title '2027 Spring Engineering Co-Op - Los Angeles, CA'. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
+      </c>
+      <c r="J342" t="str">
+        <v>Sibling req to the already-tracked Chicago, IL posting (job 2624784) — same 15-week co-op program. Discipline per aggregator: Electrical, Mechanical, or Chemical Engineering, sophomore standing or higher, no visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>Sherwin-Williams</v>
+      </c>
+      <c r="B343" t="str">
+        <v>2027 Spring Engineering Co-Op</v>
+      </c>
+      <c r="C343" t="str">
+        <v>Mechanical/Electrical/Chemical Engineering (manufacturing/plant engineering co-op)</v>
+      </c>
+      <c r="D343" t="str">
+        <v>2027 Spring Engineering Co-Op, 15-week program, January 2027 start (per posting body)</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Holland, MI</v>
+      </c>
+      <c r="F343">
+        <v>765</v>
+      </c>
+      <c r="G343" t="str">
+        <v>Reported as $23.50/hr per aggregator sources — not independently confirmed</v>
+      </c>
+      <c r="H343" t="str">
+        <v>https://ejhp.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/job/2624788</v>
+      </c>
+      <c r="I343" t="str">
+        <v>Partial — the Oracle Cloud candidate-experience page is JS-rendered and could not be fully loaded; independently confirmed via a direct curl fetch of the page's server-rendered meta tags that a live posting exists at this exact URL with og:title '2027 Spring Engineering Co-Op - Holland, MI'. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
+      </c>
+      <c r="J343" t="str">
+        <v>Sibling req to the already-tracked Chicago, IL posting (job 2624784) — same 15-week co-op program. Discipline per aggregator: Electrical, Mechanical, or Chemical Engineering, sophomore standing or higher, no visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>Sherwin-Williams</v>
+      </c>
+      <c r="B344" t="str">
+        <v>2027 Spring Engineering Co-Op</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Mechanical/Electrical/Chemical Engineering (manufacturing/plant engineering co-op)</v>
+      </c>
+      <c r="D344" t="str">
+        <v>2027 Spring Engineering Co-Op, 15-week program, January 2027 start (per posting body)</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Waco, TX</v>
+      </c>
+      <c r="F344">
+        <v>1613</v>
+      </c>
+      <c r="G344" t="str">
+        <v>Reported as $24/hr per aggregator sources — not independently confirmed</v>
+      </c>
+      <c r="H344" t="str">
+        <v>https://ejhp.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/job/2624835</v>
+      </c>
+      <c r="I344" t="str">
+        <v>Partial — the Oracle Cloud candidate-experience page is JS-rendered and could not be fully loaded; independently confirmed via a direct curl fetch of the page's server-rendered meta tags that a live posting exists at this exact URL with og:title '2027 Spring Engineering Co-Op - Waco, TX'. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
+      </c>
+      <c r="J344" t="str">
+        <v>Sibling req to the already-tracked Chicago, IL posting (job 2624784) — same 15-week co-op program. Discipline per aggregator: Electrical, Mechanical, or Chemical Engineering, sophomore standing or higher, no visa sponsorship.</v>
       </c>
     </row>
   </sheetData>
@@ -13256,14 +13352,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M341"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M344"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C699"/>
+  <dimension ref="A1:C703"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -20950,9 +21046,53 @@
         <v>2026-10-04: no qualifying posting found for any of the five companies (Zeno Power's only current internship is Supply Chain, not ME).</v>
       </c>
     </row>
+    <row r="700">
+      <c r="A700" t="str">
+        <v>Sherwin-Williams (Richmond, KY)</v>
+      </c>
+      <c r="B700" t="str">
+        <v>'2027 Spring Engineering Co-Op - Richmond, KY'</v>
+      </c>
+      <c r="C700" t="str">
+        <v>2026-10-04 (later run): confirmed to exist via two independent aggregators (dreamworkhq, zapply) with matching 15-week/January-2027/$23.50hr program details, but could not independently locate the live ejhp.fa.us6.oraclecloud.com job URL (unlike the Chicago/LA/Holland MI/Waco TX siblings, which were each confirmed by direct curl fetch of the Oracle Cloud page's own og:title meta tag). Not added pending that direct confirmation — worth a quick re-check since the sibling postings are a near-certain sign it exists.</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="str">
+        <v>Saronic Technologies (Austin, TX)</v>
+      </c>
+      <c r="B701" t="str">
+        <v>Mechanical Engineer Intern</v>
+      </c>
+      <c r="C701" t="str">
+        <v>2026-10-04 (later run): new company for the tracker, but only live req is explicitly 'Summer 2027' — wrong season. No Winter 2026/Spring 2027 posting found.</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="str">
+        <v>Ursa Major (Berthoud, CO)</v>
+      </c>
+      <c r="B702" t="str">
+        <v>Propulsion/mechanical engineering internship search</v>
+      </c>
+      <c r="C702" t="str">
+        <v>2026-10-04 (later run): new company for the tracker; only a Summer 2026 Propulsion Engineering Intern posting (already past) is live. Company's own blog states 2027-cycle postings open later in the year — not live yet.</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="str">
+        <v>Epirus (Torrance, CA)</v>
+      </c>
+      <c r="B703" t="str">
+        <v>Mechanical Engineering Intern</v>
+      </c>
+      <c r="C703" t="str">
+        <v>2026-10-04 (later run): new company for the tracker, but the live posting is an explicit 10-week internship for rising seniors graduating 12/2026-12/2027 with no Winter/Spring 2027 season wording — reads as a Summer-cycle program. Not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C699"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C703"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 8 new postings, 16 checked-excluded (2026-10-05 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVzjgiuicPN4AuwQnwNvTS
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M344"/>
+  <dimension ref="A1:M352"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -12882,6 +12882,262 @@
       </c>
       <c r="J344" t="str">
         <v>Sibling req to the already-tracked Chicago, IL posting (job 2624784) — same 15-week co-op program. Discipline per aggregator: Electrical, Mechanical, or Chemical Engineering, sophomore standing or higher, no visa sponsorship.</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>Sherwin-Williams</v>
+      </c>
+      <c r="B345" t="str">
+        <v>2027 Spring Engineering Co-Op</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Mechanical/Electrical/Chemical Engineering (manufacturing/plant engineering co-op)</v>
+      </c>
+      <c r="D345" t="str">
+        <v>2027 Spring Engineering Co-Op, 15-week program, January 2027 start (per posting body)</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Richmond, KY</v>
+      </c>
+      <c r="F345">
+        <v>768</v>
+      </c>
+      <c r="G345" t="str">
+        <v>Not independently confirmed</v>
+      </c>
+      <c r="H345" t="str">
+        <v>https://ejhp.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/job/2624800</v>
+      </c>
+      <c r="I345" t="str">
+        <v>Partial — the Oracle Cloud candidate-experience page is JS-rendered and could not be fully loaded; independently confirmed via a direct curl fetch of the page's server-rendered meta tags that a live posting exists at this exact URL with og:title '2027 Spring Engineering Co-Op - Richmond, KY', found by scanning the job-ID range near the already-confirmed siblings. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
+      </c>
+      <c r="J345" t="str">
+        <v>Sibling req to the already-tracked Chicago/LA/Holland MI/Waco TX postings — same 15-week co-op program. This closes out the Richmond, KY sibling flagged as unresolved by the prior run (2026-10-04 ~13:00 UTC).</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>Sherwin-Williams</v>
+      </c>
+      <c r="B346" t="str">
+        <v>2027 Spring Robotics Engineering Co-Op</v>
+      </c>
+      <c r="C346" t="str">
+        <v>Robotics Engineering</v>
+      </c>
+      <c r="D346" t="str">
+        <v>Spring 2027 (per title)</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Middleburg Heights, OH</v>
+      </c>
+      <c r="F346">
+        <v>558</v>
+      </c>
+      <c r="G346" t="str">
+        <v>Not independently confirmed</v>
+      </c>
+      <c r="H346" t="str">
+        <v>https://ejhp.fa.us6.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_2/job/2624797</v>
+      </c>
+      <c r="I346" t="str">
+        <v>Partial — same Oracle Cloud JS-rendered candidate-experience platform as the other Sherwin-Williams reqs; independently confirmed via a direct curl fetch of the page's server-rendered og:title/og:description meta tags that a live posting exists at this exact URL. Could not independently confirm pay, exact dates, or open/closed status beyond the page existing with that title.</v>
+      </c>
+      <c r="J346" t="str">
+        <v>Distinct req from the other Sherwin-Williams 2027 Spring Engineering Co-Op sites — robotics-specific track.</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>RTX / Collins Aerospace</v>
+      </c>
+      <c r="B347" t="str">
+        <v>Manufacturing Engineering Co-op (Spring/Summer 2027)</v>
+      </c>
+      <c r="C347" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D347" t="str">
+        <v>Spring/Summer 2027 (per posting title)</v>
+      </c>
+      <c r="E347" t="str">
+        <v>Jamestown, ND</v>
+      </c>
+      <c r="F347">
+        <v>1388</v>
+      </c>
+      <c r="G347" t="str">
+        <v>$37,000–$82,000 annualized range (per posting)</v>
+      </c>
+      <c r="H347" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-ND-JAMESTOWN-P1--2604-Highway-20-N--PLANT-1/Manufacturing-Engineering-Co-op--Spring-Summer-2027-_01870846</v>
+      </c>
+      <c r="I347" t="str">
+        <v>Yes — confirmed via direct Workday CXS JSON API fetch (tenant globalhr), canApply: true, jobReqId 01870846, posted 2026-09-29.</v>
+      </c>
+      <c r="J347" t="str">
+        <v>Requires ME/IE major, 60+ credit hours completed, U.S. citizen or green card holder. Distinct from the already-tracked Jamestown Structural Co-op (01873938); not a duplicate of the now-closed Mechanical Design Co-op (01871736).</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>Heron Power</v>
+      </c>
+      <c r="B348" t="str">
+        <v>Intern, Automation Controls Engineer (Spring 2027)</v>
+      </c>
+      <c r="C348" t="str">
+        <v>Controls Engineering</v>
+      </c>
+      <c r="D348" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Scotts Valley, CA</v>
+      </c>
+      <c r="F348">
+        <v>2693</v>
+      </c>
+      <c r="G348" t="str">
+        <v>Not listed on posting</v>
+      </c>
+      <c r="H348" t="str">
+        <v>https://jobs.ashbyhq.com/heron-power/93dd15fe-6c82-412b-a662-c14c75360f36</v>
+      </c>
+      <c r="I348" t="str">
+        <v>Yes — confirmed via direct Ashby posting-API fetch, isListed: true, published 2026-07-31.</v>
+      </c>
+      <c r="J348" t="str">
+        <v>New company for the tracker — grid power-electronics startup. Role is wiring/fabrication of controls &amp; automation equipment on a pilot production line, PLC/HMI integration; shop-class/sheet-metal experience a nice-to-have. Several sibling Heron Power reqs were checked and excluded on season or discipline grounds — see `checked`.</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Bosch Group</v>
+      </c>
+      <c r="B349" t="str">
+        <v>Facilities Engineering Intern – Spring 2027</v>
+      </c>
+      <c r="C349" t="str">
+        <v>Industrial/Facilities Engineering</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Florence, KY</v>
+      </c>
+      <c r="F349">
+        <v>747</v>
+      </c>
+      <c r="G349" t="str">
+        <v>Reported as $45k–$60k annualized per aggregator — not independently confirmed</v>
+      </c>
+      <c r="H349" t="str">
+        <v>https://jobs.smartrecruiters.com/BoschGroup/744000153195961-facilities-engineering-intern-spring-2027</v>
+      </c>
+      <c r="I349" t="str">
+        <v>Yes — confirmed via direct SmartRecruiters API fetch (api.smartrecruiters.com/v1/companies/BoschGroup/postings/744000153195961), refNumber REF297636V, released 2026-10-02.</v>
+      </c>
+      <c r="J349" t="str">
+        <v>New company for the tracker. Automotive steering-component manufacturing plant; facilities machine/equipment setup (SAP), building-management-systems support — industrial engineering fit. Multi-term rotation preferred. A sibling Bosch 'Technical Functions/Maintenance Intern/Co-op' req at the same plant was checked and excluded on discipline grounds — see `checked`.</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>Johnson Controls (JCI)</v>
+      </c>
+      <c r="B350" t="str">
+        <v>Mechanical Engineering Intern – Spring 2027</v>
+      </c>
+      <c r="C350" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D350" t="str">
+        <v>Spring 2027 (Jan–May 2027, per posting)</v>
+      </c>
+      <c r="E350" t="str">
+        <v>New Freedom, PA</v>
+      </c>
+      <c r="F350">
+        <v>345</v>
+      </c>
+      <c r="G350" t="str">
+        <v>$22.00–$25.50/hr</v>
+      </c>
+      <c r="H350" t="str">
+        <v>https://jci.wd5.myworkdayjobs.com/JCI/job/New-Freedom-Pennsylvania-United-States-of-America/Mechanical-Engineering-Intern---Spring-2027_WD30280745-1</v>
+      </c>
+      <c r="I350" t="str">
+        <v>Yes — confirmed via direct Workday CXS API fetch, canApply: true, jobReqId WD30280745.</v>
+      </c>
+      <c r="J350" t="str">
+        <v>Compressor engineering department — large centrifugal compressors for York water-cooled chillers. Distinct req from a previously-checked/excluded JCI Fall-2026 EE 'Power Electronics Intern' posting — not a duplicate.</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>SHP</v>
+      </c>
+      <c r="B351" t="str">
+        <v>Mechanical Engineering Co-op – Plumbing/HVAC Design (Spring 2027)</v>
+      </c>
+      <c r="C351" t="str">
+        <v>Mechanical Engineering (building systems / MEP design)</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E351" t="str">
+        <v>Cincinnati, OH</v>
+      </c>
+      <c r="F351">
+        <v>738</v>
+      </c>
+      <c r="G351" t="str">
+        <v>$20–$22/hr (increases $1/hr per additional term, per posting)</v>
+      </c>
+      <c r="H351" t="str">
+        <v>https://shp.applicantpro.com/jobs/4204989</v>
+      </c>
+      <c r="I351" t="str">
+        <v>Yes — confirmed via direct fetch of SHP's own ApplicantPro ATS page, HTTP 200, page title exact match, Apply control present, no closed/expired language found.</v>
+      </c>
+      <c r="J351" t="str">
+        <v>New company for the tracker — Cincinnati-based AEC/MEP engineering firm. HVAC/plumbing/mechanical building-systems design, Revit-based. Posted ~2 days before verification.</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>Georgia Tech Research Institute (GTRI)</v>
+      </c>
+      <c r="B352" t="str">
+        <v>Mechanical Engineering Co-op – Spring 2027 – ATAS</v>
+      </c>
+      <c r="C352" t="str">
+        <v>Mechanical/Aerospace Engineering</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Smyrna, GA</v>
+      </c>
+      <c r="F352">
+        <v>935</v>
+      </c>
+      <c r="G352" t="str">
+        <v>Not confirmed</v>
+      </c>
+      <c r="H352" t="str">
+        <v>https://careers.gtri.gatech.edu/jobs/mechanical-engineering-co-op-spring-2027-atas-smyrna-georgia-united-states</v>
+      </c>
+      <c r="I352" t="str">
+        <v>Partial — direct fetch returned HTTP 200 with an exact-matching page title ('Mechanical Engineering Co-op - Spring 2027 - ATAS - Smyrna, Georgia, United States') and an Apply control present, but the job-description body and application state render client-side (JS) and could not be independently read — could not confirm eligibility details or canApply status beyond the title/HTTP-200 signal.</v>
+      </c>
+      <c r="J352" t="str">
+        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza.</v>
       </c>
     </row>
   </sheetData>
@@ -13352,14 +13608,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M344"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M352"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C703"/>
+  <dimension ref="A1:C719"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -21048,51 +21304,227 @@
     </row>
     <row r="700">
       <c r="A700" t="str">
-        <v>Sherwin-Williams (Richmond, KY)</v>
+        <v>Saronic Technologies (Austin, TX)</v>
       </c>
       <c r="B700" t="str">
-        <v>'2027 Spring Engineering Co-Op - Richmond, KY'</v>
+        <v>Mechanical Engineer Intern</v>
       </c>
       <c r="C700" t="str">
-        <v>2026-10-04 (later run): confirmed to exist via two independent aggregators (dreamworkhq, zapply) with matching 15-week/January-2027/$23.50hr program details, but could not independently locate the live ejhp.fa.us6.oraclecloud.com job URL (unlike the Chicago/LA/Holland MI/Waco TX siblings, which were each confirmed by direct curl fetch of the Oracle Cloud page's own og:title meta tag). Not added pending that direct confirmation — worth a quick re-check since the sibling postings are a near-certain sign it exists.</v>
+        <v>2026-10-04 (later run): new company for the tracker, but only live req is explicitly 'Summer 2027' — wrong season. No Winter 2026/Spring 2027 posting found.</v>
       </c>
     </row>
     <row r="701">
       <c r="A701" t="str">
-        <v>Saronic Technologies (Austin, TX)</v>
+        <v>Ursa Major (Berthoud, CO)</v>
       </c>
       <c r="B701" t="str">
-        <v>Mechanical Engineer Intern</v>
+        <v>Propulsion/mechanical engineering internship search</v>
       </c>
       <c r="C701" t="str">
-        <v>2026-10-04 (later run): new company for the tracker, but only live req is explicitly 'Summer 2027' — wrong season. No Winter 2026/Spring 2027 posting found.</v>
+        <v>2026-10-04 (later run): new company for the tracker; only a Summer 2026 Propulsion Engineering Intern posting (already past) is live. Company's own blog states 2027-cycle postings open later in the year — not live yet.</v>
       </c>
     </row>
     <row r="702">
       <c r="A702" t="str">
-        <v>Ursa Major (Berthoud, CO)</v>
+        <v>Epirus (Torrance, CA)</v>
       </c>
       <c r="B702" t="str">
-        <v>Propulsion/mechanical engineering internship search</v>
+        <v>Mechanical Engineering Intern</v>
       </c>
       <c r="C702" t="str">
-        <v>2026-10-04 (later run): new company for the tracker; only a Summer 2026 Propulsion Engineering Intern posting (already past) is live. Company's own blog states 2027-cycle postings open later in the year — not live yet.</v>
+        <v>2026-10-04 (later run): new company for the tracker, but the live posting is an explicit 10-week internship for rising seniors graduating 12/2026-12/2027 with no Winter/Spring 2027 season wording — reads as a Summer-cycle program. Not added.</v>
       </c>
     </row>
     <row r="703">
       <c r="A703" t="str">
-        <v>Epirus (Torrance, CA)</v>
+        <v>Illinois Tool Works (ITW) (Troy, OH)</v>
       </c>
       <c r="B703" t="str">
-        <v>Mechanical Engineering Intern</v>
+        <v>'ITW Warewash Mechanical Engineering Co-Op' (JR5300)</v>
       </c>
       <c r="C703" t="str">
-        <v>2026-10-04 (later run): new company for the tracker, but the live posting is an explicit 10-week internship for rising seniors graduating 12/2026-12/2027 with no Winter/Spring 2027 season wording — reads as a Summer-cycle program. Not added.</v>
+        <v>2026-10-05: confirmed HTTP 410 (dead). careers.itw.com (Phenom People) has no exploitable static job data and rejects anonymous API queries; no other live Winter 2026/Spring 2027 engineering req located. Resolves the prior run's 'worth rechecking' note — still effectively unverifiable company-wide.</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="str">
+        <v>Wabtec</v>
+      </c>
+      <c r="B704" t="str">
+        <v>Firmware Engineering Co-Op (Jan-June 2027), Waltham, MA</v>
+      </c>
+      <c r="C704" t="str">
+        <v>2026-10-05: confirmed live via SmartRecruiters API, but firmware/embedded discipline — not a ME/aero fit.</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B705" t="str">
+        <v>5 new reqs (R23539, R23578, R23571, R23573, R23626)</v>
+      </c>
+      <c r="C705" t="str">
+        <v>2026-10-05: all confirmed live via Workday CXS API but are June-December 2027 siblings of already-tracked January reqs — wrong season.</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="str">
+        <v>KLA Corporation (Milpitas, CA)</v>
+      </c>
+      <c r="B706" t="str">
+        <v>Mechatronics/Systems Engineering Internship; Mechatronics Engineering Internship; 2x Product Development Engineer Intern</v>
+      </c>
+      <c r="C706" t="str">
+        <v>2026-10-05: located a working direct Workday CXS API (kla.wd1.myworkdayjobs.com) — a new access method. All current reqs are explicitly summer-intern or state no season at all; no Winter 2026/Spring 2027 req found.</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="str">
+        <v>QuantumScape</v>
+      </c>
+      <c r="B707" t="str">
+        <v>General internship search</v>
+      </c>
+      <c r="C707" t="str">
+        <v>2026-10-05: careers.quantumscape.com now returns HTTP 200 (previously assumed dead) but is a SAP SuccessFactors/Jobs2Web client-rendered app with no embedded job data. Still unverifiable.</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="str">
+        <v>PPL Corporation / LG&amp;E and KU</v>
+      </c>
+      <c r="B708" t="str">
+        <v>General internship search</v>
+      </c>
+      <c r="C708" t="str">
+        <v>2026-10-05: re-confirmed careers.pplweb.com is fully client-rendered (SuccessFactors) with no server-embedded job JSON. Still unverifiable.</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="str">
+        <v>Tesla (Sparks, NV)</v>
+      </c>
+      <c r="B709" t="str">
+        <v>Internship, Powertrain, Manufacturing Automation Controls Engineering (Winter/Spring 2027), job 278960</v>
+      </c>
+      <c r="C709" t="str">
+        <v>2026-10-05: a plausible in-season, in-discipline title surfaced via search, but www.tesla.com still returns HTTP 403 to direct fetch with or without a browser User-Agent; could not independently verify. Not added — deprioritized pending a bot-block workaround.</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="str">
+        <v>Teradyne</v>
+      </c>
+      <c r="B710" t="str">
+        <v>General internship search</v>
+      </c>
+      <c r="C710" t="str">
+        <v>2026-10-05: jobs.teradyne.com now returns HTTP 200 (previously near-empty) but still carries no embedded job data in static HTML. Still unverifiable.</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="str">
+        <v>Heron Power (Scotts Valley, CA)</v>
+      </c>
+      <c r="B711" t="str">
+        <v>Intern, Mechanical Engineer (Spring/Summer 2027)</v>
+      </c>
+      <c r="C711" t="str">
+        <v>2026-10-05: confirmed live via Ashby API, but title is mislabeled — posting body explicitly states 'this is for the Fall term, typically starting in August or September.' Wrong season.</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="str">
+        <v>Heron Power (Scotts Valley, CA)</v>
+      </c>
+      <c r="B712" t="str">
+        <v>Intern, Hardware Test Engineering (Spring/Summer 2027)</v>
+      </c>
+      <c r="C712" t="str">
+        <v>2026-10-05: confirmed live via Ashby API, but requires BS/MS in Electrical Engineering or Mechatronics — primarily EE discipline.</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="str">
+        <v>Heron Power (Scotts Valley, CA)</v>
+      </c>
+      <c r="B713" t="str">
+        <v>Intern, Medium Voltage Test Engineering</v>
+      </c>
+      <c r="C713" t="str">
+        <v>2026-10-05: confirmed live, but requires BS/MS in Electrical Engineering, Physics, or Materials Science, and no season stated anywhere — fails both discipline and explicit-season bar.</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="str">
+        <v>Heron Power (Scotts Valley, CA)</v>
+      </c>
+      <c r="B714" t="str">
+        <v>Intern, Compliance Engineering - Spring 2027; Intern, Power Electronics Engineer, Power Magnetics, Spring 2027; Intern, Electronics Design Engineer, Summer 2027; Intern, Business Development Associate, Fall 2026/Winter 2027</v>
+      </c>
+      <c r="C714" t="str">
+        <v>2026-10-05: all confirmed live via Ashby API but excluded on discipline (compliance/EE/business) or season (Summer 2027, Fall 2026/Winter 2027 — not Winter 2026/Spring 2027) grounds.</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="str">
+        <v>Astranis Space Technologies</v>
+      </c>
+      <c r="B715" t="str">
+        <v>Automation &amp; Controls Engineering Intern (Winter 2027), Greenhouse job 4718203006</v>
+      </c>
+      <c r="C715" t="str">
+        <v>2026-10-05: confirmed live via Greenhouse API, strong controls-discipline fit, but part of Astranis's standing 'Winter 2027' cohort track, consistent with this tracker's existing treatment of that cohort as distinct from Winter 2026/Spring 2027 — excluded on season grounds.</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="str">
+        <v>CNH (Fargo, ND)</v>
+      </c>
+      <c r="B716" t="str">
+        <v>Mechanical Engineering Co-op (req 5505); Product Validation Engineering Co-op</v>
+      </c>
+      <c r="C716" t="str">
+        <v>2026-10-05: req 5505 confirmed live via join.cnh.com direct fetch (good ME/wheel-loader fit) but no season/year/start-date appears anywhere in the body — evergreen posting, fails the explicit-season bar. The 'Product Validation Engineering College Co-op' aggregator link (careers.cnh.com/job/21084060) 404'd — dead link. Worth periodic re-checking in case a dated Spring 2027 version is ever posted.</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="str">
+        <v>Cisco (Maynard, MA)</v>
+      </c>
+      <c r="B717" t="str">
+        <v>Systems Quality Engineer I/II (Co-op); Physical Design Engineer I (Co-op); Firmware Engineer II (Co-op); Associate Applications Engineer I (Co-op)</v>
+      </c>
+      <c r="C717" t="str">
+        <v>2026-10-05: confirmed live via Workday CXS API, but all are generic 'evergreen' postings with no stated season, and the actual work is ASIC/VLSI silicon design (EE/CE degree required) — fails both the season and discipline bar.</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="str">
+        <v>Scout Clean Energy (Boulder, CO)</v>
+      </c>
+      <c r="B718" t="str">
+        <v>Operations Engineering Intern</v>
+      </c>
+      <c r="C718" t="str">
+        <v>2026-10-05: confirmed Summer 2027 only — wrong season.</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="str">
+        <v>Bosch Group (Florence, KY)</v>
+      </c>
+      <c r="B719" t="str">
+        <v>Technical Functions/Maintenance Intern/Co-op - Spring 2027 (SmartRecruiters id 744000153189200)</v>
+      </c>
+      <c r="C719" t="str">
+        <v>2026-10-05: confirmed live and in-season via SmartRecruiters API, but the role is spare-parts/CMMS inventory management and TPM/Lean supply-chain support, not an engineering-design/test discipline — excluded on discipline grounds. (A sibling Bosch Facilities Engineering Intern req at the same plant did qualify and was added to `rows`.)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C703"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C719"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 12 checked-excluded (2026-10-05 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJWkpUvWwbfZ2y9oDouWCE
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M352"/>
+  <dimension ref="A1:M356"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -13134,10 +13134,138 @@
         <v>https://careers.gtri.gatech.edu/jobs/mechanical-engineering-co-op-spring-2027-atas-smyrna-georgia-united-states</v>
       </c>
       <c r="I352" t="str">
-        <v>Partial — direct fetch returned HTTP 200 with an exact-matching page title ('Mechanical Engineering Co-op - Spring 2027 - ATAS - Smyrna, Georgia, United States') and an Apply control present, but the job-description body and application state render client-side (JS) and could not be independently read — could not confirm eligibility details or canApply status beyond the title/HTTP-200 signal.</v>
+        <v>Yes — 2026-10-05: re-fetched the live search listing at careers.gtri.gatech.edu/jobs/search (server-rendered this time, no JS needed) and the job page itself. Confirmed Job ID 501209, open window stated as Sep 9, 2026 – Oct 9, 2026 (currently live).</v>
       </c>
       <c r="J352" t="str">
-        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza.</v>
+        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza. URGENT: posting closes Oct 9, 2026 — only 4 days left as of this run (2026-10-05).</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Forge Atomics Inc.</v>
+      </c>
+      <c r="B353" t="str">
+        <v>Mechanical Engineering Internship/Co-op (Spring 2027)</v>
+      </c>
+      <c r="C353" t="str">
+        <v>Mechanical Engineering (nuclear hardware / fluids / structures)</v>
+      </c>
+      <c r="D353" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E353" t="str">
+        <v>El Segundo, CA</v>
+      </c>
+      <c r="F353">
+        <v>2600</v>
+      </c>
+      <c r="G353" t="str">
+        <v>Not confirmed</v>
+      </c>
+      <c r="H353" t="str">
+        <v>https://jobs.ashbyhq.com/forgeatomics/0d0dd1a7-813c-4b8a-be5b-1da8f66cf864</v>
+      </c>
+      <c r="I353" t="str">
+        <v>Yes — 2026-10-05: verified via Forge Atomics' own Ashby public posting-API (api.ashbyhq.com/posting-api/job-board/forgeatomics); confirmed isListed: true (open), posted 2026-08-13. Posting body states verbatim 'Internship and co-op positions are available for the Spring 2027 and Summer 2027 terms.'</v>
+      </c>
+      <c r="J353" t="str">
+        <v>New company for the tracker — nuclear hardware startup (25 MWe 'Ember' reactor). Work on components/fluids/structures. Applicant can pick Spring 2027 term specifically per the posting.</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>Beyond Reach Labs</v>
+      </c>
+      <c r="B354" t="str">
+        <v>Mechanical Engineer Intern (Spring 2027)</v>
+      </c>
+      <c r="C354" t="str">
+        <v>Aerospace/Mechanical Engineering (deployable space mechanisms)</v>
+      </c>
+      <c r="D354" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E354" t="str">
+        <v>New York City, NY</v>
+      </c>
+      <c r="F354">
+        <v>215</v>
+      </c>
+      <c r="G354" t="str">
+        <v>Not confirmed</v>
+      </c>
+      <c r="H354" t="str">
+        <v>https://jobs.ashbyhq.com/beyondreachlabs/5b16a59b-87b1-4ab3-812d-38f38ec4c55d</v>
+      </c>
+      <c r="I354" t="str">
+        <v>Yes — 2026-10-05: verified via Beyond Reach Labs' own Ashby public posting-API; isListed: true (open), posted 2026-07-15. Title itself is 'Mechanical Engineer Intern (Spring 2027)'; body confirms designing/analyzing/testing deployable mechanical systems (solar arrays, radiators) for satellites.</v>
+      </c>
+      <c r="J354" t="str">
+        <v>New company for the tracker — satellite deployable-mechanisms startup. Minimum 12 weeks, on-site. Closest non-Boston option found this run to Hamza's home region.</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>R.W. Beckett Corporation</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Spring 2027 Engineering Co-Op - Mechanical</v>
+      </c>
+      <c r="C355" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E355" t="str">
+        <v>North Ridgeville, OH</v>
+      </c>
+      <c r="F355">
+        <v>600</v>
+      </c>
+      <c r="G355" t="str">
+        <v>$21.00/hr</v>
+      </c>
+      <c r="H355" t="str">
+        <v>https://workforcenow.adp.com/mascsr/default/mdf/recruitment/recruitment.html?cid=82dcdbb1-2428-4870-9dda-704898848b6d&amp;ccId=19000101_000001&amp;lang=en_US</v>
+      </c>
+      <c r="I355" t="str">
+        <v>Partial — 2026-10-05: confirmed real/open via direct query of ADP Workforce Now's public job-requisitions JSON API (cid=82dcdbb1-2428-4870-9dda-704898848b6d, ExternalJobID 954864): title 'Spring 2027 Engineering Co-Op- Mechanical', postDate 2026-09-02, pay $21.00–$21.00/hr, workLevel Intern/Co-op, visa sponsorship available. However, no job-specific clickable URL exists — ADP's candidate portal is a JS SPA that builds per-job URLs client-side, and no API-supplied applyUrl field or static deep link could be found. The link above is Beckett's own careers page's confirmed-working link into the ADP portal; Hamza will need to search within it for this listing by title.</v>
+      </c>
+      <c r="J355" t="str">
+        <v>careers.beckettcorp.com itself doesn't resolve as a direct URL — Beckett's real careers page is beckettcorp.com/careers, which embeds this ADP portal.</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Tesla (Palo Alto, CA)</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Internship, Test Equipment Mechanical Design Engineer, Cell Engineering (Winter/Spring 2027)</v>
+      </c>
+      <c r="C356" t="str">
+        <v>Mechanical Engineering (test-equipment / electromechanical design)</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Palo Alto, CA</v>
+      </c>
+      <c r="F356">
+        <v>2700</v>
+      </c>
+      <c r="G356" t="str">
+        <v>$20–$50/hr (per aggregator; not independently confirmed)</v>
+      </c>
+      <c r="H356" t="str">
+        <v>https://www.tesla.com/careers/search/job/internship-test-equipment-mechanical-design-engineer-cell-engineering-winter-spring-2027-278627</v>
+      </c>
+      <c r="I356" t="str">
+        <v>Partial — 2026-10-05: tesla.com returns HTTP 403 (Akamai edge block) to direct fetch, curl with browser UA, and the r.jina.ai text-proxy workaround alike — could not independently open the posting. The exact job ID (278627) and literal title/season string '(Winter/Spring 2027)' appear consistently across multiple independent search-engine hits quoting this exact Tesla URL — same evidentiary pattern already used for the other Tesla rows in this tracker.</v>
+      </c>
+      <c r="J356" t="str">
+        <v>Could not confirm live/open status or pay beyond the title/URL match. Re-check if a Tesla bot-block workaround is ever found.</v>
       </c>
     </row>
   </sheetData>
@@ -13608,14 +13736,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M352"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M356"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C719"/>
+  <dimension ref="A1:C731"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -21522,9 +21650,141 @@
         <v>2026-10-05: confirmed live and in-season via SmartRecruiters API, but the role is spare-parts/CMMS inventory management and TPM/Lean supply-chain support, not an engineering-design/test discipline — excluded on discipline grounds. (A sibling Bosch Facilities Engineering Intern req at the same plant did qualify and was added to `rows`.)</v>
       </c>
     </row>
+    <row r="720">
+      <c r="A720" t="str">
+        <v>GKN Aerospace (Chicopee/Westfield, MA area)</v>
+      </c>
+      <c r="B720" t="str">
+        <v>joinus.gknaerospace.com/sitemap.xml</v>
+      </c>
+      <c r="C720" t="str">
+        <v>2026-10-05: sitemap is a valid XML file with hundreds of job URLs, but all entries are dated July 2023 — stale, not a reliable live signal. Still unverifiable; no new leads.</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="str">
+        <v>Illinois Tool Works (ITW)</v>
+      </c>
+      <c r="B721" t="str">
+        <v>JR9746 Warewash Mechanical Engineering Co-Op (Troy, OH); JR10405 Industrial Engineering Co-Op (Clearwater, FL); JR10116 Mechanical Engineering Intern (Appleton, WI) — found via careers.itw.com/sitemap1.xml</v>
+      </c>
+      <c r="C721" t="str">
+        <v>2026-10-05: all 3 current-sitemap job URLs return 'Sorry, the job you are looking for is no longer available' when opened directly. No open qualifying ITW posting found; exclusion stands.</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="str">
+        <v>Tesla (Sparks, NV)</v>
+      </c>
+      <c r="B722" t="str">
+        <v>Internship, Powertrain, Manufacturing Automation Controls Engineering (Winter/Spring 2027), job 278960</v>
+      </c>
+      <c r="C722" t="str">
+        <v>2026-10-05 (re-check): confirmed via Google-indexed snippet that tesla.com serves this exact URL with the title/season intact, but direct WebFetch and an r.jina.ai proxy both still return HTTP 403 (Akamai block). Still unverifiable; not added.</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="str">
+        <v>Apex Technology, Inc. (Apex Space)</v>
+      </c>
+      <c r="B723" t="str">
+        <v>Mechanical Engineering Internship; Thermal/Avionics/Propulsion/Sensors internships</v>
+      </c>
+      <c r="C723" t="str">
+        <v>2026-10-05: re-checked full Ashby board directly — current Mechanical Engineering Internship is Fall 2026 only (wrong season); other discipline-fitting reqs already tracked/checked. A stale aggregator-only 'Spring or Summer 2027' job ID no longer exists on the live board.</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="str">
+        <v>Merlin Labs (Boston, MA)</v>
+      </c>
+      <c r="B724" t="str">
+        <v>Mechanical Engineer Intern (aggregator lead)</v>
+      </c>
+      <c r="C724" t="str">
+        <v>2026-10-05: pulled full Lever API board (25 live reqs) — zero internship-titled postings exist; lead is stale/closed.</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="str">
+        <v>XWing</v>
+      </c>
+      <c r="B725" t="str">
+        <v>Mechanical Engineer Intern – Electric Propulsion Unit (Winter 2027); Mechanical Design Engineer Intern, Structures</v>
+      </c>
+      <c r="C725" t="str">
+        <v>2026-10-05: first confirmed 'no longer accepting applications' (closed); second is a stale Summer-2026-dated posting (Feb 2026). Both excluded.</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="str">
+        <v>Kodiak Robotics (Mountain View, CA)</v>
+      </c>
+      <c r="B726" t="str">
+        <v>Winter 2027 intern cohort (Motion Planning/Controls/Simulation/Mission Planning/Security)</v>
+      </c>
+      <c r="C726" t="str">
+        <v>2026-10-05: cohort confirmed live and in-season, but all titled reqs are software/autonomy roles, not a dedicated mechanical/hardware discipline — excluded on discipline grounds.</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="str">
+        <v>Boom Supersonic</v>
+      </c>
+      <c r="B727" t="str">
+        <v>2027 Engineering and Tech Internship (Materials &amp; Manufacturing track)</v>
+      </c>
+      <c r="C727" t="str">
+        <v>2026-10-05: only a Summer 2027 program is currently live — wrong season.</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="str">
+        <v>Aurora Innovation, Nuro, Gatik</v>
+      </c>
+      <c r="B728" t="str">
+        <v>General Winter 2026/Spring 2027 mechanical/hardware internship search</v>
+      </c>
+      <c r="C728" t="str">
+        <v>2026-10-05: no postings found for any of the three; Aurora's own site states its next cycle isn't expected to open until later in fall 2026.</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="str">
+        <v>Arizona Beverage Company (Keasbey, NJ)</v>
+      </c>
+      <c r="B729" t="str">
+        <v>Controls Engineering Intern (aggregator lead)</v>
+      </c>
+      <c r="C729" t="str">
+        <v>2026-10-05: could not locate a primary-source posting URL or confirm season/term language — excluded as unverifiable.</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="str">
+        <v>Natilus</v>
+      </c>
+      <c r="B730" t="str">
+        <v>General mechanical engineering internship search</v>
+      </c>
+      <c r="C730" t="str">
+        <v>2026-10-05: no mechanical engineering internship postings found at all.</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="str">
+        <v>Astroscale U.S., Momentus, Terran Orbital</v>
+      </c>
+      <c r="B731" t="str">
+        <v>General Winter 2026/Spring 2027 mechanical internship search</v>
+      </c>
+      <c r="C731" t="str">
+        <v>2026-10-05: no current postings found for Astroscale/Momentus; Terran Orbital's 'Mechanical Engineer Intern – Automation' lead is closed/not accepting applications.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C719"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C731"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 23 checked-excluded (2026-10-05 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011JBWaATwgzpNBLHoMq1pwK
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M356"/>
+  <dimension ref="A1:M360"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -13266,6 +13266,134 @@
       </c>
       <c r="J356" t="str">
         <v>Could not confirm live/open status or pay beyond the title/URL match. Re-check if a Tesla bot-block workaround is ever found.</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>Precision Castparts Corp. (TIMET — Titanium Metals Corporation)</v>
+      </c>
+      <c r="B357" t="str">
+        <v>2027 Spring Engineering or Metallurgy Co-op</v>
+      </c>
+      <c r="C357" t="str">
+        <v>Materials/Metallurgical Engineering (explicitly also open to Mechanical Engineering and Chemical Engineering majors)</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E357" t="str">
+        <v>Toronto, OH</v>
+      </c>
+      <c r="F357">
+        <v>510</v>
+      </c>
+      <c r="G357" t="str">
+        <v>Paid, with housing stipend (exact hourly rate not stated on posting)</v>
+      </c>
+      <c r="H357" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/lang-en-GB/mobile-0/appcentre-1/brand-7/xf-8b16151655e3/candidate/so/pm/1/pl/1/opp/24068-2027-Spring-Engineering-or-Metallurgy-Co-op/en-GB</v>
+      </c>
+      <c r="I357" t="str">
+        <v>Yes — 2026-10-05: fetched directly via PCC's own StepStone TalentLink portal (HTTP 200, no Altcha bot-wall encountered this run, unlike prior runs). Full job description, req ID (oppid 24068), title, season, and discipline requirements all confirmed in the raw page HTML. Posted-date and exact pay rate not visible in static HTML.</v>
+      </c>
+      <c r="J357" t="str">
+        <v>Minimum 3-month assignment. Requires U.S. Person / export-control (ITAR) eligibility. PCC's portal may no longer be bot-blocked — worth a fuller sweep of its ~44 other reqs in a future run.</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>Medical Murray</v>
+      </c>
+      <c r="B358" t="str">
+        <v>Engineering Co-op/Internship Spring 2027</v>
+      </c>
+      <c r="C358" t="str">
+        <v>R&amp;D Engineering (Biomedical/Mechanical Engineering)</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E358" t="str">
+        <v>North Barrington, IL</v>
+      </c>
+      <c r="F358">
+        <v>880</v>
+      </c>
+      <c r="G358" t="str">
+        <v>$22.00/hr</v>
+      </c>
+      <c r="H358" t="str">
+        <v>https://workforcenow.adp.com/mascsr/default/mdf/recruitment/recruitment.html?cid=a1c55fdd-ce3e-4aa6-88b9-7d856f012d0f&amp;ccId=274124546795_2&amp;lang=en_US</v>
+      </c>
+      <c r="I358" t="str">
+        <v>Partial — 2026-10-05: confirmed real/open via direct query of ADP Workforce Now's public job-requisitions JSON API (ExternalJobID 501187): title 'Engineering Co-op/Internship Spring 2027', postDate 2026-09-14, pay $22.00/hr flat, location N Barrington IL. Same limitation as the R.W. Beckett row above — no job-specific deep link exists, only this generic ADP portal shell URL; Hamza will need to search within it for the listing by title.</v>
+      </c>
+      <c r="J358" t="str">
+        <v>Sibling Summer 2027 and Fall 2027 reqs also exist in the same ADP feed (wrong season, excluded).</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>Physical Intelligence</v>
+      </c>
+      <c r="B359" t="str">
+        <v>Mechatronics Intern</v>
+      </c>
+      <c r="C359" t="str">
+        <v>Mechanical/Mechatronics Engineering</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Spring 2027 (January–May 2027, per posting)</v>
+      </c>
+      <c r="E359" t="str">
+        <v>San Francisco, CA</v>
+      </c>
+      <c r="F359">
+        <v>2700</v>
+      </c>
+      <c r="G359" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H359" t="str">
+        <v>https://jobs.ashbyhq.com/physicalintelligence/0bcf909e-b38b-4276-91a1-e55c4c56a33a</v>
+      </c>
+      <c r="I359" t="str">
+        <v>Yes — 2026-10-05: fetched directly via Physical Intelligence's own public Ashby job-board API, isListed: true, published 2026-09-17. Full description independently read, including the explicit January–May 2027 duration.</v>
+      </c>
+      <c r="J359" t="str">
+        <v>Robotics/hardware team (mechanical &amp; electromechanical design, FEA, DFM, CAD, motor controllers) — distinct from PI's LLM/VLA research side.</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>Etched</v>
+      </c>
+      <c r="B360" t="str">
+        <v>Mechanical/Thermal Intern</v>
+      </c>
+      <c r="C360" t="str">
+        <v>Mechanical/Thermal Engineering</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Spring 2027 (one of four named rolling cohorts: Summer '26, Fall '26, Spring '27, Summer '27)</v>
+      </c>
+      <c r="E360" t="str">
+        <v>San José, CA</v>
+      </c>
+      <c r="F360">
+        <v>2680</v>
+      </c>
+      <c r="G360" t="str">
+        <v>Not stated; 12-week paid internship plus relocation/housing support mentioned on posting</v>
+      </c>
+      <c r="H360" t="str">
+        <v>https://jobs.ashbyhq.com/Etched/f05e3218-5ec7-41d1-bc99-bb7014422229</v>
+      </c>
+      <c r="I360" t="str">
+        <v>Yes — 2026-10-05: fetched directly via Etched's own public Ashby job-board API, isListed: true, workplaceType OnSite. Full description independently read, including the explicit "Spring '27" cohort line. Posted 2026-02-07 (outside the ~3-week freshness window) but is a standing rolling-cohort requisition, not stale — isListed: true confirms it is still live.</v>
+      </c>
+      <c r="J360" t="str">
+        <v>AI-chip hardware startup (inference ASICs): NPI prototyping, manufacturing fixture development, liquid cooling, rack-level system development.</v>
       </c>
     </row>
   </sheetData>
@@ -13736,14 +13864,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M356"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M360"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C731"/>
+  <dimension ref="A1:C754"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -19491,7 +19619,7 @@
         <v>'Spring 2027 Engineering Student Co-Op' (Muskegon MI), 'Spring 2027 Maintenance Co-Op' (Spring TX), 'Engineering Co-Op for Spring 2027' (Niskayuna NY)</v>
       </c>
       <c r="C523" t="str">
-        <v>2026-09-30 ~13:00 UTC: only found via aggregator mirrors (Dice/Glassdoor/Indeed); PCC's real ATS (a StepStone TalentLink portal at pcctalentacquisitionportal.tal.net) is behind an Altcha bot-check challenge, fully blocking programmatic access — same class of block as other long-standing blockers. Not added without a verified URL.</v>
+        <v>2026-09-30 ~13:00 UTC: only found via aggregator mirrors (Dice/Glassdoor/Indeed); PCC's real ATS (a StepStone TalentLink portal at pcctalentacquisitionportal.tal.net) is behind an Altcha bot-check challenge, fully blocking programmatic access — same class of block as other long-standing blockers. Not added without a verified URL. SUPERSEDED 2026-10-05: the Altcha wall was not encountered this run (portal reachable via plain curl); see the TIMET/PCC 'Spring Engineering or Metallurgy Co-op' row added to `rows` this run.</v>
       </c>
     </row>
     <row r="524">
@@ -21782,9 +21910,262 @@
         <v>2026-10-05: no current postings found for Astroscale/Momentus; Terran Orbital's 'Mechanical Engineer Intern – Automation' lead is closed/not accepting applications.</v>
       </c>
     </row>
+    <row r="732">
+      <c r="A732" t="str">
+        <v>Teleflex (Olive Branch, MS)</v>
+      </c>
+      <c r="B732" t="str">
+        <v>Industrial Engineer Intern (req 12704)</v>
+      </c>
+      <c r="C732" t="str">
+        <v>2026-10-05 (later run, re-check): re-confirmed still 'Sorry, this position has been filled' — no change.</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="str">
+        <v>SEACORP</v>
+      </c>
+      <c r="B733" t="str">
+        <v>General co-op/internship search</v>
+      </c>
+      <c r="C733" t="str">
+        <v>2026-10-05 (later run, re-check): no change — site offers no job listing, only a recruiting email contact; still unverifiable.</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="str">
+        <v>The Aerospace Corporation</v>
+      </c>
+      <c r="B734" t="str">
+        <v>General co-op/internship search</v>
+      </c>
+      <c r="C734" t="str">
+        <v>2026-10-05 (later run, re-check): still could not locate the company's Workday tenant ID to query directly; aggregator-only leads remain unconfirmed.</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="str">
+        <v>Framatome</v>
+      </c>
+      <c r="B735" t="str">
+        <v>General co-op/internship search</v>
+      </c>
+      <c r="C735" t="str">
+        <v>2026-10-05 (later run, re-check): careers.framatome.com is now fully unreachable (DNS failure/ENOTFOUND) — worse than the prior block; still unverifiable.</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="str">
+        <v>GKN Aerospace</v>
+      </c>
+      <c r="B736" t="str">
+        <v>Careers search page + internships landing page</v>
+      </c>
+      <c r="C736" t="str">
+        <v>2026-10-05 (later run, re-check): search page is a pure client-rendered shell with no job data in static HTML; internships page shows only generic marketing copy. No change.</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="str">
+        <v>Illinois Tool Works (ITW)</v>
+      </c>
+      <c r="B737" t="str">
+        <v>jobs.itw.com search endpoint</v>
+      </c>
+      <c r="C737" t="str">
+        <v>2026-10-05 (later run, re-check): endpoint returned HTTP 503 this run. No new leads; consistent with 5+ prior exclusion runs.</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B738" t="str">
+        <v>Lynn CNC Programmer Co-Op R5040944-1</v>
+      </c>
+      <c r="C738" t="str">
+        <v>2026-10-05 (later run): requires current enrollment in a Vocational Technical High School, pays $18.33/hr, closes 2026-12-31 — vocational/trade role, not a college engineering fit. Same exclusion as all prior Lynn trade-co-op reqs.</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B739" t="str">
+        <v>JR002974, JR002688, JR002941 (full re-sweep)</v>
+      </c>
+      <c r="C739" t="str">
+        <v>2026-10-05 (later run): all already tracked (JR002974) or already excluded on discipline grounds (JR002688, JR002941 — EE). No new qualifying req.</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B740" t="str">
+        <v>Full re-sweep via Workday CXS API</v>
+      </c>
+      <c r="C740" t="str">
+        <v>2026-10-05 (later run): June–Dec 2027 siblings already logged this run; no further new reqs found.</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="str">
+        <v>Precision Castparts Corp. (PCC Fasteners / Shur-Lok, Irvine, CA)</v>
+      </c>
+      <c r="B741" t="str">
+        <v>'Co-Op, Manufacturing Engineering' (oppid 23909)</v>
+      </c>
+      <c r="C741" t="str">
+        <v>2026-10-05: confirmed live via direct fetch of PCC's own StepStone TalentLink portal (HTTP 200), Mechanical Engineering-fitting discipline, but no season/year stated anywhere in the posting — fails the explicit-season bar. Not added.</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="str">
+        <v>Xometry</v>
+      </c>
+      <c r="B742" t="str">
+        <v>Full Greenhouse board (230 jobs)</v>
+      </c>
+      <c r="C742" t="str">
+        <v>2026-10-05: no intern/co-op titled roles currently; only FTE roles (incl. a Waltham, MA 'Mechanical Engineer, AI Integration'). Worth a periodic re-check.</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="str">
+        <v>Fictiv</v>
+      </c>
+      <c r="B743" t="str">
+        <v>Full Greenhouse board (94 jobs)</v>
+      </c>
+      <c r="C743" t="str">
+        <v>2026-10-05: only intern role is HR, Bengaluru India. No US mechanical/manufacturing intern.</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="str">
+        <v>Formic</v>
+      </c>
+      <c r="B744" t="str">
+        <v>'2026 Internship' (Chicago/Bolingbrook IL and SF/Oakland CA)</v>
+      </c>
+      <c r="C744" t="str">
+        <v>2026-10-05: general ops/coordination internships, not engineering-discipline, and season unspecified/likely Summer-2026-wave. Discipline + season mismatch.</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="str">
+        <v>General Matter</v>
+      </c>
+      <c r="B745" t="str">
+        <v>14 open intern reqs incl. Mechanical Engineering, Mechanical Engineering (HVAC), Manufacturing Engineering</v>
+      </c>
+      <c r="C745" t="str">
+        <v>2026-10-05: all explicitly titled 'Summer 2027 Internship'. Wrong season, all.</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="str">
+        <v>Zoox</v>
+      </c>
+      <c r="B746" t="str">
+        <v>Full Lever board (234 jobs)</v>
+      </c>
+      <c r="C746" t="str">
+        <v>2026-10-05: zero intern/co-op titled postings currently.</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="str">
+        <v>Motional</v>
+      </c>
+      <c r="B747" t="str">
+        <v>Full internship search</v>
+      </c>
+      <c r="C747" t="str">
+        <v>2026-10-05: only ML internship is Singapore-based; no mechanical/robotics US intern/co-op.</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="str">
+        <v>Collaborative Robotics</v>
+      </c>
+      <c r="B748" t="str">
+        <v>Full Ashby board</v>
+      </c>
+      <c r="C748" t="str">
+        <v>2026-10-05: mechanical engineer roles exist (Wire Harness ME, ME Product Design, ME AI Data Collection) but all full-time; zero internship/co-op titles.</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="str">
+        <v>Dexterity</v>
+      </c>
+      <c r="B749" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C749" t="str">
+        <v>2026-10-05: no intern/co-op titled postings.</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="str">
+        <v>Loft Orbital</v>
+      </c>
+      <c r="B750" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C750" t="str">
+        <v>2026-10-05: no intern/co-op titled postings.</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="str">
+        <v>Machina Labs</v>
+      </c>
+      <c r="B751" t="str">
+        <v>Full Ashby board</v>
+      </c>
+      <c r="C751" t="str">
+        <v>2026-10-05: zero open jobs currently (board is live but empty).</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="str">
+        <v>Vertex Pharmaceuticals</v>
+      </c>
+      <c r="B752" t="str">
+        <v>'Spring Co-Op 2027, Combination Device Technologies &amp; Innovation' (REQ-30505-1)</v>
+      </c>
+      <c r="C752" t="str">
+        <v>2026-10-05: confirmed via Workday CXS API, but requires an advanced degree in Chemical Engineering/Physical chemistry/Applied sciences — discipline mismatch. Distinct from the already-tracked Mechanical Automation Spring Co-Op (REQ-30500-1).</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="str">
+        <v>Stantec</v>
+      </c>
+      <c r="B753" t="str">
+        <v>Mechanical Engineering Co-op/Intern, Buildings/Government Services (Spring 2027), per aggregator</v>
+      </c>
+      <c r="C753" t="str">
+        <v>2026-10-05: season matches per aggregator, but discipline is MEP/HVAC/plumbing building-systems design for government facilities, not product/aerospace/manufacturing ME — same discipline-mismatch judgment as prior CMTA/Stantec-adjacent exclusions. stantec.jobs redirected before a primary-source fetch could complete; excluded on discipline grounds regardless.</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="str">
+        <v>AEVEX Aerospace (Tampa, FL)</v>
+      </c>
+      <c r="B754" t="str">
+        <v>Robotics Engineering Co-op</v>
+      </c>
+      <c r="C754" t="str">
+        <v>2026-10-05: confirmed live via AEVEX's own Greenhouse board API (HTTP 200 — closed reqs normally 404). Two independent aggregators (zapply.jobs, dreamworkhq.com) claim 'Winter 2026', but the primary Greenhouse posting text itself contains no season/date language at all (searched for 'winter', '2026', '2027', 'semester', 'enrolled', 'degree' — none present). Fails the 'season confirmed from the posting itself' bar — not added; worth an in-browser re-check in case season info lives in an application-form dropdown not present in the static description HTML.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C731"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C754"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 12 checked-excluded (2026-10-05 19:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GcH7kELtTmHRUPzWFv4V3g
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M360"/>
+  <dimension ref="A1:M363"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -13134,10 +13134,10 @@
         <v>https://careers.gtri.gatech.edu/jobs/mechanical-engineering-co-op-spring-2027-atas-smyrna-georgia-united-states</v>
       </c>
       <c r="I352" t="str">
-        <v>Yes — 2026-10-05: re-fetched the live search listing at careers.gtri.gatech.edu/jobs/search (server-rendered this time, no JS needed) and the job page itself. Confirmed Job ID 501209, open window stated as Sep 9, 2026 – Oct 9, 2026 (currently live).</v>
+        <v>Yes — 2026-10-05 (re-checked again): fetched the job page directly (HTTP 200), still live, no closed/no-longer-accepting text. The page's own schema.org JSON-LD now gives validThrough 2027-01-03, and the earlier-reported 'Oct 9, 2026' window text could not be re-located anywhere in today's raw HTML — so that deadline is unconfirmed as of this run (may have been updated/removed, or may have been a search-listing artifact). Treat the Oct 9 date as uncertain rather than confirmed; still open either way.</v>
       </c>
       <c r="J352" t="str">
-        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza. URGENT: posting closes Oct 9, 2026 — only 4 days left as of this run (2026-10-05).</v>
+        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza. Previously flagged as closing Oct 9, 2026, but that exact date could not be re-confirmed on 2026-10-05 (page now only shows a JSON-LD validThrough of 2027-01-03); apply without delay regardless, since the original deadline text may still be accurate.</v>
       </c>
     </row>
     <row r="353">
@@ -13394,6 +13394,102 @@
       </c>
       <c r="J360" t="str">
         <v>AI-chip hardware startup (inference ASICs): NPI prototyping, manufacturing fixture development, liquid cooling, rack-level system development.</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>Precision Castparts Corp. (Wyman Gordon / Structurals Company)</v>
+      </c>
+      <c r="B361" t="str">
+        <v>Engineering Co-Op</v>
+      </c>
+      <c r="C361" t="str">
+        <v>Mechanical, Materials, or Aeronautical Engineering</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Winter 2026/Spring 2027 (available to start December 2026 or January 2027, per posting)</v>
+      </c>
+      <c r="E361" t="str">
+        <v>Groton, CT</v>
+      </c>
+      <c r="F361">
+        <v>95</v>
+      </c>
+      <c r="G361" t="str">
+        <v>$20.75–$31.00/hr + quarterly incentive bonus + overtime, per posting</v>
+      </c>
+      <c r="H361" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/lang-en-GB/mobile-0/appcentre-1/brand-7/xf-27078e30bc96/candidate/so/pm/1/pl/2/opp/22255-Engineering-Co-Op/en-GB</v>
+      </c>
+      <c r="I361" t="str">
+        <v>Yes — 2026-10-05: fetched directly via PCC's own tal.net TalentLink portal (HTTP 200, no bot-wall encountered this run), full job body read directly. Start window ('December 2026 or January 2027'), discipline, and pay all stated explicitly in the posting text itself. Listing shows an application deadline of 26 Dec 2026.</v>
+      </c>
+      <c r="J361" t="str">
+        <v>Found during a fuller sweep of PCC's ~78 open reqs (prompted by last run's TIMET Toronto OH find at the same portal). 4–6 month rotation, double-block rotations accepted. Within ~100 mi of Boston — a strong geographic fit for Hamza.</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>Barry-Wehmiller (BW Design Group)</v>
+      </c>
+      <c r="B362" t="str">
+        <v>Controls Engineering Co-Op - BOS</v>
+      </c>
+      <c r="C362" t="str">
+        <v>Controls Engineering (industrial automation/PLC/HMI)</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Partial — likely January 2027 start, not stated on this specific req (see Link Verified)</v>
+      </c>
+      <c r="E362" t="str">
+        <v>Boston, MA</v>
+      </c>
+      <c r="F362">
+        <v>0</v>
+      </c>
+      <c r="G362" t="str">
+        <v>Not stated on this req</v>
+      </c>
+      <c r="H362" t="str">
+        <v>https://barrywehmiller.wd1.myworkdayjobs.com/BWConfidential/job/Boston-MA/Controls-Engineering-Co-Op---BOS_R023035</v>
+      </c>
+      <c r="I362" t="str">
+        <v>Partial — 2026-10-05: queried Barry-Wehmiller's own Workday CXS API directly, confirmed req R023035 is live ('Posted Today' 2026-10-05), title and Boston, MA location match exactly. However this specific requisition's own body text does not itself state a season/start date. The identical national-program sibling req (R022664, 'Controls Engineering Internship/Co-Op (Summer 2027 or 6-Month)') explicitly states 'Co-Ops are 6-months long and start in January 2027 or June 2027' — a January 2027 start is plausible for this Boston req by extension of that sibling program but is NOT independently confirmed on R023035 itself.</v>
+      </c>
+      <c r="J362" t="str">
+        <v>Right in the Boston metro. A different, earlier-found Barry-Wehmiller req ('Automation &amp; Controls Engineering Internship/Co-Op', via a Handshake listing, 2026-09-30) is logged separately in `checked` — that one could not be independently opened; this one was confirmed directly via Workday. Worth a follow-up to pin down this specific req's exact start date before Hamza applies.</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>Haast Autonomous</v>
+      </c>
+      <c r="B363" t="str">
+        <v>Fall/Winter Engineering Co-op</v>
+      </c>
+      <c r="C363" t="str">
+        <v>Aerospace/Flight Systems (airframe design, avionics, controls, manufacturing, flight test)</v>
+      </c>
+      <c r="D363" t="str">
+        <v>Partial — 'Fall/Winter co-op term' per posting; no literal year digit stated in the body</v>
+      </c>
+      <c r="E363" t="str">
+        <v>Pendleton, OR</v>
+      </c>
+      <c r="F363">
+        <v>2500</v>
+      </c>
+      <c r="G363" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H363" t="str">
+        <v>https://jobs.ashbyhq.com/haastautonomous/be09930d-89aa-43f3-a29d-8470e06c747d</v>
+      </c>
+      <c r="I363" t="str">
+        <v>Partial — 2026-10-05: queried Haast Autonomous's own public Ashby posting-API directly (api.ashbyhq.com/posting-api/job-board/haastautonomous), confirmed isListed: true, FullTime, OnSite, full description read from the API JSON. Posting says 'Fall/Winter co-op term' without an explicit '2026'/'2027' string anywhere in the body — season fit is inferred from the posting date (published 2026-07-07, still live 2026-10-05) rather than stated outright.</v>
+      </c>
+      <c r="J363" t="str">
+        <v>Autonomous medical-logistics VTOL aircraft startup. Not Boston-area. Confirm the exact co-op start/end dates directly with the company before relying on the season fit.</v>
       </c>
     </row>
   </sheetData>
@@ -13864,14 +13960,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M360"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M363"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C754"/>
+  <dimension ref="A1:C766"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -22160,12 +22256,144 @@
         <v>Robotics Engineering Co-op</v>
       </c>
       <c r="C754" t="str">
-        <v>2026-10-05: confirmed live via AEVEX's own Greenhouse board API (HTTP 200 — closed reqs normally 404). Two independent aggregators (zapply.jobs, dreamworkhq.com) claim 'Winter 2026', but the primary Greenhouse posting text itself contains no season/date language at all (searched for 'winter', '2026', '2027', 'semester', 'enrolled', 'degree' — none present). Fails the 'season confirmed from the posting itself' bar — not added; worth an in-browser re-check in case season info lives in an application-form dropdown not present in the static description HTML.</v>
+        <v>2026-10-05 (re-checked, exhaustively): confirmed live via AEVEX's own Greenhouse board API (HTTP 200). Pulled the full job object with questions=true — all 22 application-form fields are visa/clearance/eligibility/contact fields plus one free-text availability-dates field; no season dropdown exists anywhere in the form. Full job `content` field and `application_deadline` both contain zero occurrences of 'winter/spring/summer/fall/2026/2027/semester/season'. Confirmed the posting simply never states a season in title, body, or application form — exclusion stands, now exhaustively verified rather than merely unconfirmed.</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="str">
+        <v>Precision Castparts Corp. — Forging Engineer Intern/Co-Op (23819, Paramount CA)</v>
+      </c>
+      <c r="B755" t="str">
+        <v>Forging Engineer Intern/Co-Op</v>
+      </c>
+      <c r="C755" t="str">
+        <v>2026-10-05: ME/Mfg discipline fits, $21-23/hr, but body states no season/year at all ('immediately', 'throughout academic school year') — season unconfirmable.</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="str">
+        <v>Precision Castparts Corp. — Operations Process Control Co-Op (23858, San Leandro CA)</v>
+      </c>
+      <c r="B756" t="str">
+        <v>Operations Process Control Co-Op</v>
+      </c>
+      <c r="C756" t="str">
+        <v>2026-10-05: Engineering/Hard Sciences degree required, $22.50-28.25/hr, but no season stated anywhere in the posting.</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="str">
+        <v>Precision Castparts Corp. — Operations Co-Op/Intern (23145 and 24146)</v>
+      </c>
+      <c r="B757" t="str">
+        <v>Operations Co-Op/Intern</v>
+      </c>
+      <c r="C757" t="str">
+        <v>2026-10-05: both reqs explicitly state a September 2026 start — wrong season (Fall only, not Winter 2026/Spring 2027).</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B758" t="str">
+        <v>Engines Engineering Co-op - Computer/Software - Spring 2027</v>
+      </c>
+      <c r="C758" t="str">
+        <v>2026-10-05: season fits but discipline is Computer Science/Software — mismatch for Hamza's ME/Aero focus.</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="str">
+        <v>Graco (Dexter, MI)</v>
+      </c>
+      <c r="B759" t="str">
+        <v>Application Engineering Intern; Electrical Engineering Intern</v>
+      </c>
+      <c r="C759" t="str">
+        <v>2026-10-05: Application Engineering Intern body fetched directly — zero season keywords anywhere in the posting, consistent with other no-season Graco reqs already excluded. Electrical Engineering Intern excluded on discipline grounds (EE, not ME/Aero/Mfg).</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="str">
+        <v>HNTB</v>
+      </c>
+      <c r="B760" t="str">
+        <v>Co-op Engineer: Structures - Spring/Summer 2027 (Philadelphia/Harrisburg/King of Prussia PA, req R-31879)</v>
+      </c>
+      <c r="C760" t="str">
+        <v>2026-10-05: confirmed live via HNTB's own Workday CXS API, but season is an ambiguous combined 'Spring/Summer 2027' label (could resolve to summer-only) and location is not Boston-area — not added.</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="str">
+        <v>HNTB</v>
+      </c>
+      <c r="B761" t="str">
+        <v>Co-op Civil Engineer: Traffic/Roadway/Stormwater-Utilities, Spring 2027 (Boston, MA)</v>
+      </c>
+      <c r="C761" t="str">
+        <v>2026-10-05: confirmed live via Workday CXS API, Boston MA location and season both fit, but discipline is transportation/civil engineering (traffic, roadway, stormwater) — not structural/mechanical/aerospace/manufacturing/robotics/materials/controls. Discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="str">
+        <v>Langan Engineering</v>
+      </c>
+      <c r="B762" t="str">
+        <v>Intern/Co-op, Site/Civil Engineering, Spring 2027 (Boston, MA)</v>
+      </c>
+      <c r="C762" t="str">
+        <v>2026-10-05: season plausible per aggregator, but role is site/civil (drainage, stormwater, site feasibility) — discipline mismatch. Not independently opened on Langan's own ATS.</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="str">
+        <v>Field AI</v>
+      </c>
+      <c r="B763" t="str">
+        <v>Robotics Research Internship, Humanoid Manipulation (Boston, MA)</v>
+      </c>
+      <c r="C763" t="str">
+        <v>2026-10-05: opened directly via Field AI's own Lever API — title says 'Spring 2027' but the posting's own body text explicitly says 'We are offering a Fall 2026 internship,' a self-contradiction. Also PhD-only. Season unverifiable/self-contradictory; not added.</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B764" t="str">
+        <v>Full mechanical-engineering req list (~33+ current reqs) via Workday CXS API</v>
+      </c>
+      <c r="C764" t="str">
+        <v>2026-10-05 (re-confirmed): zero Intern/Co-Op worker-subtype reqs company-wide. Standing exclusion reconfirmed.</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="str">
+        <v>Markforged</v>
+      </c>
+      <c r="B765" t="str">
+        <v>Company-wide job search</v>
+      </c>
+      <c r="C765" t="str">
+        <v>2026-10-05: no live Spring 2027 posting locatable; no clear primary job board found to independently verify.</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="str">
+        <v>Desktop Metal</v>
+      </c>
+      <c r="B766" t="str">
+        <v>Company-wide job search</v>
+      </c>
+      <c r="C766" t="str">
+        <v>2026-10-05: no live Spring 2027 posting locatable; no clear primary job board found to independently verify.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C754"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C766"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 22 new postings, 11 checked-excluded (2026-10-06 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCcFg1m8jVgGsqsAEeEHm1
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M363"/>
+  <dimension ref="A1:M385"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -13134,10 +13134,10 @@
         <v>https://careers.gtri.gatech.edu/jobs/mechanical-engineering-co-op-spring-2027-atas-smyrna-georgia-united-states</v>
       </c>
       <c r="I352" t="str">
-        <v>Yes — 2026-10-05 (re-checked again): fetched the job page directly (HTTP 200), still live, no closed/no-longer-accepting text. The page's own schema.org JSON-LD now gives validThrough 2027-01-03, and the earlier-reported 'Oct 9, 2026' window text could not be re-located anywhere in today's raw HTML — so that deadline is unconfirmed as of this run (may have been updated/removed, or may have been a search-listing artifact). Treat the Oct 9 date as uncertain rather than confirmed; still open either way.</v>
+        <v>Yes — 2026-10-06 (re-checked again, resolved): fetched the job page directly (HTTP 200), still live. Parsed the full JSON-LD and visible body text and found ZERO occurrence of 'Oct 9' or any deadline string anywhere on the page — the earlier 'Oct 9, 2026' claim does not exist on the current live posting and appears to have been a misread from an earlier run. The only deadline signal on the page is schema.org validThrough 2027-01-03, confirmed twice now (2026-10-05 and 2026-10-06).</v>
       </c>
       <c r="J352" t="str">
-        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza. Previously flagged as closing Oct 9, 2026, but that exact date could not be re-confirmed on 2026-10-05 (page now only shows a JSON-LD validThrough of 2027-01-03); apply without delay regardless, since the original deadline text may still be accurate.</v>
+        <v>New org for the tracker — Georgia Tech's applied-research division, Aerospace, Transportation &amp; Advanced Systems Lab. Requires 3.0+ GPA and ability to complete 3 full co-op terms before graduation (classic Georgia Tech co-op structure) — a multi-semester commitment worth flagging for Hamza. RESOLVED 2026-10-06: open through ~Jan 3, 2027 per the posting's own validThrough field; the earlier 'Oct 9, 2026' deadline note was unfounded and should be disregarded.</v>
       </c>
     </row>
     <row r="353">
@@ -13454,10 +13454,10 @@
         <v>https://barrywehmiller.wd1.myworkdayjobs.com/BWConfidential/job/Boston-MA/Controls-Engineering-Co-Op---BOS_R023035</v>
       </c>
       <c r="I362" t="str">
-        <v>Partial — 2026-10-05: queried Barry-Wehmiller's own Workday CXS API directly, confirmed req R023035 is live ('Posted Today' 2026-10-05), title and Boston, MA location match exactly. However this specific requisition's own body text does not itself state a season/start date. The identical national-program sibling req (R022664, 'Controls Engineering Internship/Co-Op (Summer 2027 or 6-Month)') explicitly states 'Co-Ops are 6-months long and start in January 2027 or June 2027' — a January 2027 start is plausible for this Boston req by extension of that sibling program but is NOT independently confirmed on R023035 itself.</v>
+        <v>Partial — 2026-10-06 (re-confirmed, gap is now definitive not just suspected): re-queried Barry-Wehmiller's own Workday CXS API directly, req R023035 still live ('Posted Today' as of this re-check too), title and Boston, MA location match exactly. Grepped the full jobDescription HTML body for any of '2026'/'2027'/'Winter'/'Spring'/'Fall'/'Summer' — zero matches; this req's own text simply never states a season. Workday's generic startDate field (2026-10-05) is the posting's activation date, not a work-term start date, and should not be read as season evidence. The sibling national req (R022664, 'Controls Engineering Internship/Co-Op (Summer 2027 or 6-Month)') is confirmed to be a genuinely separate, distinct filing — its Summer-2027/January-2027 language cannot be assumed to apply to R023035.</v>
       </c>
       <c r="J362" t="str">
-        <v>Right in the Boston metro. A different, earlier-found Barry-Wehmiller req ('Automation &amp; Controls Engineering Internship/Co-Op', via a Handshake listing, 2026-09-30) is logged separately in `checked` — that one could not be independently opened; this one was confirmed directly via Workday. Worth a follow-up to pin down this specific req's exact start date before Hamza applies.</v>
+        <v>Right in the Boston metro. A different, earlier-found Barry-Wehmiller req ('Automation &amp; Controls Engineering Internship/Co-Op', via a Handshake listing, 2026-09-30) is logged separately in `checked`. This is a confirmed, permanent information gap in the posting itself (not a research limitation) — Hamza should ask directly about the start term if applying.</v>
       </c>
     </row>
     <row r="363">
@@ -13490,6 +13490,710 @@
       </c>
       <c r="J363" t="str">
         <v>Autonomous medical-logistics VTOL aircraft startup. Not Boston-area. Confirm the exact co-op start/end dates directly with the company before relying on the season fit.</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B364" t="str">
+        <v>Winter 2027 Quality &amp; Test Engineer Co-op</v>
+      </c>
+      <c r="C364" t="str">
+        <v>Industrial/Quality Engineering</v>
+      </c>
+      <c r="D364" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E364" t="str">
+        <v>Ashville, OH (also dual-listed at Santa Ana, CA)</v>
+      </c>
+      <c r="F364">
+        <v>646</v>
+      </c>
+      <c r="G364" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H364" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5257571007</v>
+      </c>
+      <c r="I364" t="str">
+        <v>Yes — 2026-10-06: queried Anduril's own Greenhouse Jobs API directly, job returned live content, title 'Winter 2027 Quality &amp; Test Engineer Co-op' confirmed, updated_at 2026-10-05T19:47:56-04:00 (posted the day before this check).</v>
+      </c>
+      <c r="J364" t="str">
+        <v>Defense contractor — expect an ITAR/US-person requirement typical of Anduril postings. Posting is dual-listed for Ashville, OH and Santa Ana, CA; distance above uses the Ashville, OH location.</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B365" t="str">
+        <v>Winter 2027 Reliability Engineer Co-op</v>
+      </c>
+      <c r="C365" t="str">
+        <v>Industrial/Reliability Engineering</v>
+      </c>
+      <c r="D365" t="str">
+        <v>Winter 2027</v>
+      </c>
+      <c r="E365" t="str">
+        <v>Costa Mesa, CA</v>
+      </c>
+      <c r="F365">
+        <v>2586</v>
+      </c>
+      <c r="G365" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H365" t="str">
+        <v>https://job-boards.greenhouse.io/andurilindustries/jobs/5257693007</v>
+      </c>
+      <c r="I365" t="str">
+        <v>Yes — 2026-10-06: queried Anduril's own Greenhouse Jobs API directly, title confirmed live, updated_at 2026-10-05T20:17:10-04:00 (posted the day before this check).</v>
+      </c>
+      <c r="J365" t="str">
+        <v>Defense contractor — expect an ITAR/US-person requirement typical of Anduril postings.</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>MetOx International</v>
+      </c>
+      <c r="B366" t="str">
+        <v>Process Engineering Co-Op/Intern</v>
+      </c>
+      <c r="C366" t="str">
+        <v>Manufacturing/Process Engineering</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Spring 2027 (also offers a Jan–Aug 2027 full co-op track)</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Houston, TX</v>
+      </c>
+      <c r="F366">
+        <v>1604</v>
+      </c>
+      <c r="G366" t="str">
+        <v>Possible monthly stipend mentioned for non-local candidates on the co-op track</v>
+      </c>
+      <c r="H366" t="str">
+        <v>https://job-boards.greenhouse.io/metoxinternationalinc/jobs/5439987008</v>
+      </c>
+      <c r="I366" t="str">
+        <v>Yes — 2026-10-06: fetched directly via MetOx's own Greenhouse API, live posting, season language ('Spring 2027' part-time track / Jan-Aug 2027 co-op option) confirmed in the body text itself.</v>
+      </c>
+      <c r="J366" t="str">
+        <v>Superconducting-wire manufacturer. Sibling req to the already-tracked MetOx Mechanical Engineering Co-Op/Intern — this is a distinct, separate Process Engineering requisition at the same company.</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>Freeform Future Corp</v>
+      </c>
+      <c r="B367" t="str">
+        <v>Additive Engineering Intern</v>
+      </c>
+      <c r="C367" t="str">
+        <v>Manufacturing/Materials (metal additive manufacturing)</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E367" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F367">
+        <v>2591</v>
+      </c>
+      <c r="G367" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H367" t="str">
+        <v>https://job-boards.greenhouse.io/freeformfuturecorp/jobs/8013423003</v>
+      </c>
+      <c r="I367" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Freeform's own Greenhouse API, live, title/season confirmed in posting, updated_at 2026-10-05T14:43:22-04:00 (posted the day before this check).</v>
+      </c>
+      <c r="J367" t="str">
+        <v>AI-native metal-additive-manufacturing startup. On-site in LA. Distinct from Freeform's already-tracked Spring 2027 Mechanical Engineering Intern req.</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>Freeform Future Corp</v>
+      </c>
+      <c r="B368" t="str">
+        <v>Manufacturing Engineering Intern</v>
+      </c>
+      <c r="C368" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D368" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E368" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F368">
+        <v>2591</v>
+      </c>
+      <c r="G368" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H368" t="str">
+        <v>https://job-boards.greenhouse.io/freeformfuturecorp/jobs/8013422003</v>
+      </c>
+      <c r="I368" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Freeform's own Greenhouse API, live, title/season confirmed in posting, updated_at 2026-10-05T14:43:18-04:00.</v>
+      </c>
+      <c r="J368" t="str">
+        <v>AI-native metal-additive-manufacturing startup. On-site in LA. Distinct from Freeform's already-tracked Spring 2027 Mechanical Engineering Intern req.</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>Freeform Future Corp</v>
+      </c>
+      <c r="B369" t="str">
+        <v>Process Engineering Intern</v>
+      </c>
+      <c r="C369" t="str">
+        <v>Manufacturing/Materials</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E369" t="str">
+        <v>Los Angeles, CA</v>
+      </c>
+      <c r="F369">
+        <v>2591</v>
+      </c>
+      <c r="G369" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H369" t="str">
+        <v>https://job-boards.greenhouse.io/freeformfuturecorp/jobs/8013424003</v>
+      </c>
+      <c r="I369" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Freeform's own Greenhouse API, live, title/season confirmed in posting, updated_at 2026-10-05T14:43:15-04:00.</v>
+      </c>
+      <c r="J369" t="str">
+        <v>AI-native metal-additive-manufacturing startup. On-site in LA. Distinct from Freeform's already-tracked Spring 2027 Mechanical Engineering Intern req.</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>Precision Castparts Corp. (Metals Company / Cannon Muskegon)</v>
+      </c>
+      <c r="B370" t="str">
+        <v>Spring 2027 Engineering Student Co-Op opening</v>
+      </c>
+      <c r="C370" t="str">
+        <v>Engineering (general, metals/casting plant)</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E370" t="str">
+        <v>Muskegon, MI</v>
+      </c>
+      <c r="F370">
+        <v>771</v>
+      </c>
+      <c r="G370" t="str">
+        <v>Paid, plus housing stipend (amount not specified)</v>
+      </c>
+      <c r="H370" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22052-Spring-2027-Engineering-Student-Co-Op-opening/en-GB</v>
+      </c>
+      <c r="I370" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, HTTP 200, no closed/expired language, title/location/season ('Spring 2027 Semester Engineering Student Co-Op opening') read directly from the page body.</v>
+      </c>
+      <c r="J370" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs.</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C371" t="str">
+        <v>Engineering (general)</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F371">
+        <v>530</v>
+      </c>
+      <c r="G371" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H371" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22133-Engineering-Co-Op-Spring-2027/en-GB</v>
+      </c>
+      <c r="I371" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J371" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 4 Mentor-Painesville Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B372" t="str">
+        <v>Quality Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C372" t="str">
+        <v>Quality/Industrial Engineering</v>
+      </c>
+      <c r="D372" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F372">
+        <v>530</v>
+      </c>
+      <c r="G372" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H372" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22134-Quality-Engineering-Co-Op-Spring-2027/en-GB</v>
+      </c>
+      <c r="I372" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J372" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 4 Mentor-Painesville Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B373" t="str">
+        <v>Alloy Process Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C373" t="str">
+        <v>Materials/Process Engineering</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F373">
+        <v>530</v>
+      </c>
+      <c r="G373" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H373" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22135-Alloy-Process-Engineering-Co-Op-Spring-2027/en-GB</v>
+      </c>
+      <c r="I373" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J373" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 4 Mentor-Painesville Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B374" t="str">
+        <v>Facilities Engineering Co-Op - Spring 2027</v>
+      </c>
+      <c r="C374" t="str">
+        <v>Facilities/Industrial Engineering</v>
+      </c>
+      <c r="D374" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E374" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F374">
+        <v>530</v>
+      </c>
+      <c r="G374" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H374" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22136-Facilities-Engineering-Co-Op-Spring-2027/en-GB</v>
+      </c>
+      <c r="I374" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J374" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 4 Mentor-Painesville Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>Precision Castparts Corp. (EPD Company / E-One)</v>
+      </c>
+      <c r="B375" t="str">
+        <v>Engineering Co-Op, Spring 2027</v>
+      </c>
+      <c r="C375" t="str">
+        <v>Mechanical Engineering (CAD, prototyping, component/system design)</v>
+      </c>
+      <c r="D375" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E375" t="str">
+        <v>Niskayuna, NY</v>
+      </c>
+      <c r="F375">
+        <v>144</v>
+      </c>
+      <c r="G375" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H375" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/22911-Engineering-Co-Op-Spring-2027/en-GB</v>
+      </c>
+      <c r="I375" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J375" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. Closest PCC location to Boston found so far (~144 mi).</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Ceramics-LED)</v>
+      </c>
+      <c r="B376" t="str">
+        <v>Spring 2027 Finishing Co-Op (oppid 24038)</v>
+      </c>
+      <c r="C376" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D376" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E376" t="str">
+        <v>Sanford, NC</v>
+      </c>
+      <c r="F376">
+        <v>645</v>
+      </c>
+      <c r="G376" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H376" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24038-Spring-2027-Finishing-Co-Op/en-GB</v>
+      </c>
+      <c r="I376" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J376" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. A second, distinct req (oppid 24231) with the identical title and location also exists separately — likely a second headcount opening, not a duplicate; both are listed.</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Ceramics-LED)</v>
+      </c>
+      <c r="B377" t="str">
+        <v>Spring 2027 Finishing Co-Op (oppid 24231)</v>
+      </c>
+      <c r="C377" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D377" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E377" t="str">
+        <v>Sanford, NC</v>
+      </c>
+      <c r="F377">
+        <v>645</v>
+      </c>
+      <c r="G377" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H377" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24231-Spring-2027-Finishing-Co-Op/en-GB</v>
+      </c>
+      <c r="I377" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J377" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. Distinct req ID from oppid 24038 above, which shares an identical title/location — treated as a separate headcount opening rather than a duplicate.</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Douglas)</v>
+      </c>
+      <c r="B378" t="str">
+        <v>Spring 2027 Operations Co-op Assignment</v>
+      </c>
+      <c r="C378" t="str">
+        <v>Industrial/Operations Engineering</v>
+      </c>
+      <c r="D378" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E378" t="str">
+        <v>Douglas, GA</v>
+      </c>
+      <c r="F378">
+        <v>991</v>
+      </c>
+      <c r="G378" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H378" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24119-Spring-2027-Operations-Co-op-Assignment/en-GB</v>
+      </c>
+      <c r="I378" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J378" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 3 Douglas, GA Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Douglas)</v>
+      </c>
+      <c r="B379" t="str">
+        <v>Spring 2027 Mechanical Engineering Co-op Assignment</v>
+      </c>
+      <c r="C379" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E379" t="str">
+        <v>Douglas, GA</v>
+      </c>
+      <c r="F379">
+        <v>991</v>
+      </c>
+      <c r="G379" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H379" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24120-Spring-2027-Mechanical-Engineering-Co-op-Assignment/en-GB</v>
+      </c>
+      <c r="I379" t="str">
+        <v>Yes — 2026-10-06: fetched the full posting body directly via PCC's tal.net portal, title, location, division, and season all confirmed.</v>
+      </c>
+      <c r="J379" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. Strongest discipline match of the 3 Douglas, GA reqs found this run (posting body: 'Mechanical/Manufacturing Engineering Co-op Student').</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Douglas)</v>
+      </c>
+      <c r="B380" t="str">
+        <v>Spring 2027 Quality Engineering Co-op Assignment</v>
+      </c>
+      <c r="C380" t="str">
+        <v>Quality/Industrial Engineering</v>
+      </c>
+      <c r="D380" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E380" t="str">
+        <v>Douglas, GA</v>
+      </c>
+      <c r="F380">
+        <v>991</v>
+      </c>
+      <c r="G380" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H380" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24121-Spring-2027-Quality-Engineering-Co-op-Assignment/en-GB</v>
+      </c>
+      <c r="I380" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J380" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 3 Douglas, GA Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / SMP-Eastlake)</v>
+      </c>
+      <c r="B381" t="str">
+        <v>Spring 2027 Engineering Co-op</v>
+      </c>
+      <c r="C381" t="str">
+        <v>Manufacturing Engineering (turbine blades/vanes)</v>
+      </c>
+      <c r="D381" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E381" t="str">
+        <v>Wickliffe, OH</v>
+      </c>
+      <c r="F381">
+        <v>537</v>
+      </c>
+      <c r="G381" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H381" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24243-Spring-2027-Engineering-Co-op/en-GB</v>
+      </c>
+      <c r="I381" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J381" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 3 SMP-Eastlake Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / SMP-Eastlake)</v>
+      </c>
+      <c r="B382" t="str">
+        <v>Spring 2027 Facilities 6S Engineering Co-op</v>
+      </c>
+      <c r="C382" t="str">
+        <v>Facilities/Industrial Engineering</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E382" t="str">
+        <v>Wickliffe, OH</v>
+      </c>
+      <c r="F382">
+        <v>537</v>
+      </c>
+      <c r="G382" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H382" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24245-Spring-2027-Facilities-6S-Engineering-Co-op/en-GB</v>
+      </c>
+      <c r="I382" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J382" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 3 SMP-Eastlake Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / SMP-Eastlake)</v>
+      </c>
+      <c r="B383" t="str">
+        <v>Spring 2027 Operations Co-op</v>
+      </c>
+      <c r="C383" t="str">
+        <v>Manufacturing/Operations Engineering</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E383" t="str">
+        <v>Wickliffe, OH</v>
+      </c>
+      <c r="F383">
+        <v>537</v>
+      </c>
+      <c r="G383" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H383" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24247-Spring-2027-Operations-Co-op/en-GB</v>
+      </c>
+      <c r="I383" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J383" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs; one of 3 SMP-Eastlake Spring 2027 co-op reqs found this run.</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Ceramics-LED)</v>
+      </c>
+      <c r="B384" t="str">
+        <v>Spring 2027 Production Control Co-Op</v>
+      </c>
+      <c r="C384" t="str">
+        <v>Industrial Engineering</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E384" t="str">
+        <v>Cleveland, OH</v>
+      </c>
+      <c r="F384">
+        <v>550</v>
+      </c>
+      <c r="G384" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H384" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24276-Spring-2027-Production-Control-Co-Op/en-GB</v>
+      </c>
+      <c r="I384" t="str">
+        <v>Yes — 2026-10-06: fetched the live posting directly via PCC's tal.net portal, title/location/season confirmed in the page body.</v>
+      </c>
+      <c r="J384" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs.</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>Precision Castparts Corp. (Metals Company / SMC Division)</v>
+      </c>
+      <c r="B385" t="str">
+        <v>Co-op - Manufacturing Engineering (Fall/Winter)</v>
+      </c>
+      <c r="C385" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D385" t="str">
+        <v>Fall 2026–Spring 2027 co-op (explicitly 'September 2026 - April 2027' per posting body)</v>
+      </c>
+      <c r="E385" t="str">
+        <v>New Hartford, NY</v>
+      </c>
+      <c r="F385">
+        <v>221</v>
+      </c>
+      <c r="G385" t="str">
+        <v>Not stated on posting</v>
+      </c>
+      <c r="H385" t="str">
+        <v>https://pcctalentacquisitionportal.tal.net/vx/mobile-1/appcentre-ext/brand-7/candidate/so/pm/1/pl/3/opp/24286-Co-op-Manufacturing-Engineering-Fall-Winter/en-GB</v>
+      </c>
+      <c r="I385" t="str">
+        <v>Yes — 2026-10-06: fetched the full posting body directly via PCC's tal.net portal; the exact date range 'September 2026 - April 2027' is stated verbatim in the posting text.</v>
+      </c>
+      <c r="J385" t="str">
+        <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. A genuine Fall-2026-through-Spring-2027 co-op, per the task's stated exception for this season shape.</v>
       </c>
     </row>
   </sheetData>
@@ -13960,14 +14664,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M363"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M385"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C766"/>
+  <dimension ref="A1:C777"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -22391,9 +23095,130 @@
         <v>2026-10-05: no live Spring 2027 posting locatable; no clear primary job board found to independently verify.</v>
       </c>
     </row>
+    <row r="767">
+      <c r="A767" t="str">
+        <v>MORSE Corp (Cambridge, MA)</v>
+      </c>
+      <c r="B767" t="str">
+        <v>Aerospace Algorithms Engineer Co-op (job 7968520003)</v>
+      </c>
+      <c r="C767" t="str">
+        <v>2026-10-06: confirmed live via Greenhouse, Cambridge MA, Spring-2027-cycle, but the role is physics/statistical/ML modeling for mission planning &amp; simulation — a software/algorithms discipline, not hardware engineering. Discipline mismatch; MORSE's already-tracked Mechanical Engineer Co-op (job 7968311003) is unaffected.</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="str">
+        <v>Mind Robotics (Palo Alto, CA)</v>
+      </c>
+      <c r="B768" t="str">
+        <v>Full 31-req Ashby job board</v>
+      </c>
+      <c r="C768" t="str">
+        <v>2026-10-06: queried the company's own Ashby board directly — zero intern-titled postings currently live. A widely-circulated aggregator lead ('Intern, Mechanical Design – Wiring Harness, Fall 2026') is no longer on the live board and was wrong season anyway.</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="str">
+        <v>Havoc AI (North Kingstown RI / San Diego / Palo Alto)</v>
+      </c>
+      <c r="B769" t="str">
+        <v>Full 24-req Ashby job board</v>
+      </c>
+      <c r="C769" t="str">
+        <v>2026-10-06: queried the company's own Ashby board directly — zero intern-titled postings currently live. An aggregator-sourced 'Mechanical Engineer Intern (Winter 2026)' lead could not be located on the live board — appears closed/stale.</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="str">
+        <v>Formlabs</v>
+      </c>
+      <c r="B770" t="str">
+        <v>Hardware R&amp;D Engineering Intern (job 8097694)</v>
+      </c>
+      <c r="C770" t="str">
+        <v>2026-10-06: direct Greenhouse API query returned HTTP 404/closed — this is a dead duplicate of Formlabs' already-tracked live req (8172226).</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="str">
+        <v>Figure AI</v>
+      </c>
+      <c r="B771" t="str">
+        <v>Power Systems Integration Intern (job 4702104006)</v>
+      </c>
+      <c r="C771" t="str">
+        <v>2026-10-06: direct Greenhouse API query returned empty/404 — lead from a GitHub aggregator repo does not correspond to a live posting.</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="str">
+        <v>Precision Castparts Corp. — Operations Co-Op/Intern (leadership-track roles)</v>
+      </c>
+      <c r="B772" t="str">
+        <v>Operations Co-Op/Intern, oppids 23146 (Metals/HBE, Huntington WV), 23437 (Structurals/LPC, Portland OR), 23677 (Metals/Toronto-TIMET, Toronto OH), 23716 (EPD/University Swaging, Woodinville WA), 24033 (Airfoils/Ceramics-LED, Wickliffe OH)</v>
+      </c>
+      <c r="C772" t="str">
+        <v>2026-10-06: all 5 reqs explicitly describe a generic leadership-development rotation ('a future career leading people'), not an engineering role — discipline mismatch, excluded.</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="str">
+        <v>Precision Castparts Corp. — non-engineering Development Program/Co-Op reqs</v>
+      </c>
+      <c r="B773" t="str">
+        <v>29 reqs company-wide (HR, Finance, IT, Supply Chain, Talent Acquisition, EHS, rotational Development Program tracks), oppids 20366, 20414, 22912, 23479, 23492, 23493, 23495, 23496, 23535, 23691, 23763, 23800, 23829, 23902, 23908, 23917, 23972, 24008, 24055, 24091, 24118, 24166, 24209, 24240, 24270, 24292, 24293, 24394, 24409</v>
+      </c>
+      <c r="C773" t="str">
+        <v>2026-10-06: triaged by title/division against PCC's full open-Co-Op list — all are non-engineering disciplines, out of scope for Hamza's ME/aero/manufacturing focus.</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="str">
+        <v>Precision Castparts Corp. — Summer 2027 Co-Op reqs</v>
+      </c>
+      <c r="B774" t="str">
+        <v>8 reqs, oppids 24252, 24253, 24284, 24285, 24287, 24289, 24290, 24333</v>
+      </c>
+      <c r="C774" t="str">
+        <v>2026-10-06: each posting's own title explicitly states Summer 2027 — wrong season, excluded.</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="str">
+        <v>Precision Castparts Corp. — no season stated, unresolved</v>
+      </c>
+      <c r="B775" t="str">
+        <v>8 reqs: Manufacturing Engineer Intern/Co-Op (Wyman Gordon/Shultz Steel, South Gate CA, oppid 23458); Forge Shop Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23814); Heat Treat Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23815); Research Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24180); Mechanical Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24181); Engineer Co-Op $21/hr (Fasteners/AIC, Garden Grove CA, oppid 24183); CNC Machinist/Programmer Intern Co-Op (Structurals/Schlosser, Redmond OR, oppid 24238); Engineering Co-Op (Fasteners/Andrews Laser Works, Wilder KY, oppid 24353)</v>
+      </c>
+      <c r="C775" t="str">
+        <v>2026-10-06: each live posting was read in full but states no season anywhere (title or body) — cannot confirm Winter2026/Spring2027 fit either way. Not added to rows per the verification bar; flagged for a future revisit (PCC sometimes adds season language later), especially oppid 24181 (Henderson NV Mechanical Engineering Co-Op) which is a strong discipline match if the season resolves favorably.</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="str">
+        <v>nVent</v>
+      </c>
+      <c r="B776" t="str">
+        <v>Engineering Lab Co-Op (R23537, Anoka MN)</v>
+      </c>
+      <c r="C776" t="str">
+        <v>2026-10-06: live via nVent's own Workday CXS API, but conflicting season signals — title says 'Jan-August 2027' while the URL slug says 'June-August-2027.' Could not resolve which is correct in the time available; not added, flagged for a future check.</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="str">
+        <v>Wabtec (Waltham, MA)</v>
+      </c>
+      <c r="B777" t="str">
+        <v>Firmware Engineering Co-Op (Jan-June 2027)</v>
+      </c>
+      <c r="C777" t="str">
+        <v>2026-10-05/06: season and Boston-area location both fit, but role is firmware/software — discipline mismatch.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C766"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C777"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 4 new postings, 20 checked-excluded (2026-10-06 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DNZLWiCiqPFiFn8BCPSFNh
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M386"/>
+  <dimension ref="A1:M390"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -13355,13 +13355,13 @@
         <v>$22.00/hr</v>
       </c>
       <c r="H359" t="str">
-        <v>https://workforcenow.adp.com/mascsr/default/mdf/recruitment/recruitment.html?cid=a1c55fdd-ce3e-4aa6-88b9-7d856f012d0f&amp;ccId=274124546795_2&amp;lang=en_US</v>
+        <v>https://jobs.solidprofessor.com/job/372053/engineering-co-op-internship-spring-2027/</v>
       </c>
       <c r="I359" t="str">
-        <v>Partial — 2026-10-05: confirmed real/open via direct query of ADP Workforce Now's public job-requisitions JSON API (ExternalJobID 501187): title 'Engineering Co-op/Internship Spring 2027', postDate 2026-09-14, pay $22.00/hr flat, location N Barrington IL. Same limitation as the R.W. Beckett row above — no job-specific deep link exists, only this generic ADP portal shell URL; Hamza will need to search within it for the listing by title.</v>
+        <v>Yes — 2026-10-06: upgraded from the generic ADP portal shell link (no longer needed) to a job-specific deep link found on SolidProfessor, Medical Murray's actual career-site ATS. Fetched directly and confirmed: title 'R&amp;D Engineering Co-op/Internship', North Barrington IL, $22.00/hr, 'Start Date: Spring of 2027', posted Sept 16 2026, Apply button live. Medical Murray's ADP API now returns an empty job-requisitions list for their cid — they appear to have moved listings to SolidProfessor.</v>
       </c>
       <c r="J359" t="str">
-        <v>Sibling Summer 2027 and Fall 2027 reqs also exist in the same ADP feed (wrong season, excluded).</v>
+        <v>Sibling Summer 2027 and Fall 2027 reqs also existed in the prior ADP feed (wrong season, excluded). SolidProfessor job IDs for this company appear to get reissued periodically (an older ID, 306224, for the same title already 404'd once) — worth a quick liveness re-check next run.</v>
       </c>
     </row>
     <row r="360">
@@ -14226,6 +14226,134 @@
       </c>
       <c r="J386" t="str">
         <v>Found during a continued sweep of PCC's ~81 open Co-Op reqs. A genuine Fall-2026-through-Spring-2027 co-op, per the task's stated exception for this season shape.</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B387" t="str">
+        <v>Design Engineer Co-Op</v>
+      </c>
+      <c r="C387" t="str">
+        <v>Mechanical/Electro-Mechanical/Manufacturing Engineering</v>
+      </c>
+      <c r="D387" t="str">
+        <v>Jan-Jun 2027</v>
+      </c>
+      <c r="E387" t="str">
+        <v>North Andover, MA</v>
+      </c>
+      <c r="F387">
+        <v>24</v>
+      </c>
+      <c r="G387" t="str">
+        <v>$23.00-$25.00/hr</v>
+      </c>
+      <c r="H387" t="str">
+        <v>https://wattswater.wd5.myworkdayjobs.com/Intern-External/job/North-Andover-MA/Design-Engineer-Co-Op_10017594</v>
+      </c>
+      <c r="I387" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Watts' own Workday CXS API (canApply=true); body confirms 'January-June 2027' and a Mechanical/Electro-Mechanical/Manufacturing Engineering degree requirement. These 4 co-ops were posted 13-18 days ago — not found live on this board as of a prior-run check; Watts' own site has since caught up to aggregator leads that previously couldn't be verified.</v>
+      </c>
+      <c r="J387" t="str">
+        <v>One of 4 new Jan-Jun 2027 engineering Co-Ops posted on Watts' own Intern-External Workday board this run.</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B388" t="str">
+        <v>Product Engineer Co-Op</v>
+      </c>
+      <c r="C388" t="str">
+        <v>Mechanical/Manufacturing Engineering</v>
+      </c>
+      <c r="D388" t="str">
+        <v>Jan-Jun 2027</v>
+      </c>
+      <c r="E388" t="str">
+        <v>North Andover, MA</v>
+      </c>
+      <c r="F388">
+        <v>24</v>
+      </c>
+      <c r="G388" t="str">
+        <v>$23.00-$25.00/hr</v>
+      </c>
+      <c r="H388" t="str">
+        <v>https://wattswater.wd5.myworkdayjobs.com/Intern-External/job/North-Andover-MA/Product-Engineer-Co-Op_10017596</v>
+      </c>
+      <c r="I388" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Watts' own Workday CXS API (canApply=true); body confirms 'January-June 2027' and a Mechanical/Manufacturing Engineering degree requirement.</v>
+      </c>
+      <c r="J388" t="str">
+        <v>One of 4 new Jan-Jun 2027 engineering Co-Ops posted on Watts' own Intern-External Workday board this run.</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B389" t="str">
+        <v>Sustaining Engineer Co-Op</v>
+      </c>
+      <c r="C389" t="str">
+        <v>Mechanical/Manufacturing Engineering</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Jan-Jun 2027</v>
+      </c>
+      <c r="E389" t="str">
+        <v>Franklin, NH</v>
+      </c>
+      <c r="F389">
+        <v>80</v>
+      </c>
+      <c r="G389" t="str">
+        <v>$25.00/hr</v>
+      </c>
+      <c r="H389" t="str">
+        <v>https://wattswater.wd5.myworkdayjobs.com/Intern-External/job/Franklin-NH/Sustaining-Engineer-Co-Op_10017595</v>
+      </c>
+      <c r="I389" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Watts' own Workday CXS API (canApply=true); body confirms 'January-June 2027' and a Mechanical/Manufacturing Engineering degree requirement.</v>
+      </c>
+      <c r="J389" t="str">
+        <v>One of 4 new Jan-Jun 2027 engineering Co-Ops posted on Watts' own Intern-External Workday board this run.</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B390" t="str">
+        <v>Research and Technology Co-Op</v>
+      </c>
+      <c r="C390" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D390" t="str">
+        <v>Jan-Jun 2027</v>
+      </c>
+      <c r="E390" t="str">
+        <v>North Andover, MA</v>
+      </c>
+      <c r="F390">
+        <v>24</v>
+      </c>
+      <c r="G390" t="str">
+        <v>$23.00-$25.00/hr</v>
+      </c>
+      <c r="H390" t="str">
+        <v>https://wattswater.wd5.myworkdayjobs.com/Intern-External/job/North-Andover-MA/Research-and-Technology-Co-Op_10017598</v>
+      </c>
+      <c r="I390" t="str">
+        <v>Yes — 2026-10-06: fetched directly via Watts' own Workday CXS API (canApply=true); body confirms 'January-June 2027' and a Mechanical Engineering degree requirement.</v>
+      </c>
+      <c r="J390" t="str">
+        <v>One of 4 new Jan-Jun 2027 engineering Co-Ops posted on Watts' own Intern-External Workday board this run.</v>
       </c>
     </row>
   </sheetData>
@@ -14696,14 +14824,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M386"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M390"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C793"/>
+  <dimension ref="A1:C813"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -23289,7 +23417,7 @@
         <v>'Research and Technology Co-Op', 'Design Engineer Co-Op', 'Product Engineer Co-Op' (Jan-Jun 2027, $23-25/hr, per aggregators)</v>
       </c>
       <c r="C781" t="str">
-        <v>2026-10-06: aggregators (Teal/JobRight) advertise these, but a direct query of Watts' own Workday CXS API across all 27 current Andover-area postings shows none are Intern/Co-Op — appear stale/closed on the employer's own board. Worth a follow-up fetch in case they repost.</v>
+        <v>2026-10-06 ~07:40: aggregators (Teal/JobRight) advertise these, but a direct query of Watts' own Workday CXS API across all 27 current Andover-area postings shows none are Intern/Co-Op — appear stale/closed on the employer's own board. SUPERSEDED 2026-10-06 ~13:00: Watts' own Intern-External Workday board now carries these (plus a 4th, Sustaining Engineer Co-Op) as live, dated postings — moved to `rows`.</v>
       </c>
     </row>
     <row r="782">
@@ -23424,9 +23552,229 @@
         <v>2026-10-06: no Spring 2027 ME co-op located; only Spring/Summer 2026 reqs found.</v>
       </c>
     </row>
+    <row r="794">
+      <c r="A794" t="str">
+        <v>Precision Castparts Corp. — full-board pagination pass</v>
+      </c>
+      <c r="B794" t="str">
+        <v>All 80 open Co-Op/Intern reqs on PCC's tal.net board confirmed to fit on a single page (no deeper pagination exists, resolving a prior run's pagination concern); ~48 newly-ID'd reqs beyond the already-tracked/already-checked ones</v>
+      </c>
+      <c r="C794" t="str">
+        <v>2026-10-06 ~13:00: 18 non-engineering-discipline Co-Ops (Finance/HR/IT/EHS/Supply Chain/Talent Acq — oppids 24240, 24166, 24091, 24008, 23902, 23763, 23800, 24409, 23908, 22912, 23990, 24293, 22137, 24292, 23691, 24118, 24055, 23972); 7 generic Operations/leadership-track co-ops (22760, 23677, 23146, 23437, 23716, 24033, 22054); 5 engineering reqs explicitly titled 'Summer 2027' (24287 Mentor OH Engineering, 24285 Quality Eng, 24289 Facilities Eng, 24290 Alloy Process Eng, 24253 Toronto OH Engineering/Metallurgy); 1 maintenance-tech co-op (23917); 9 full-time/rotational-program/senior roles that aren't student co-ops (24237 Engineering Manager, 23829/24209 Rotational Programs, 23496/23495/23493/23492/20414/23479/20366 Development Programs, 24270 Director, 23535/23118 full-time HR). Board now fully triaged by req ID; recommend deprioritizing further full-board sweeps, only periodic re-checks of the 7 no-season reqs.</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="str">
+        <v>GKN Aerospace</v>
+      </c>
+      <c r="B795" t="str">
+        <v>'Quality Engineer (Early Careers)', Tallassee AL</v>
+      </c>
+      <c r="C795" t="str">
+        <v>2026-10-06: full-time entry-level role, no 'co-op'/'intern' in title and no season/term stated — not a student co-op. Still no live Winter 2026/Spring 2027 co-op after 10+ consecutive runs.</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="str">
+        <v>MIT Lincoln Laboratory</v>
+      </c>
+      <c r="B796" t="str">
+        <v>'Rapid Prototyping Aero/Mech Co-Op (Fall 2026) - Group 77'</v>
+      </c>
+      <c r="C796" t="str">
+        <v>2026-10-06: strong discipline fit (Mechanical/Aero/Astro) but posting explicitly states Fall 2026 only with no Winter/Spring 2027 extension. Wrong season.</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B797" t="str">
+        <v>'Lynn CNC Programmer Co-Op' (R5040944)</v>
+      </c>
+      <c r="C797" t="str">
+        <v>2026-10-06: requires enrollment in a Vocational Technical High School, not a college engineering co-op — same exclusion pattern as prior Lynn trade co-ops.</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="str">
+        <v>Draper Laboratory</v>
+      </c>
+      <c r="B798" t="str">
+        <v>'Co-Op Student Engineering' (JR002974); 'Acoustic and Vibration Technologies Co-op' (JR002688); 'Electrical Engineering Co-Op' (JR002941); 'Sensor Electrical Engineering Co-op' (JR002885); 'Optics-Physics Sensor Engineering Co-op' (JR002884); 'Digital Engineering – Requirements Engineering Intern' (JR002945-1)</v>
+      </c>
+      <c r="C798" t="str">
+        <v>2026-10-06: JR002974 is software/embedded discipline; JR002688 states zero season text anywhere in title or body; JR002941/JR002885/JR002884 are EE/physics discipline mismatches; JR002945-1 is Summer 2027 (wrong season). Checked against Draper's own Workday CXS API.</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B799" t="str">
+        <v>'Trade Compliance Analyst Co-Op' (Spring 2027); 'Legal Co-Op' (title says Jan-Jun 2027, URL slug says Fall 2027 — internally inconsistent); 'Systems Engineer Intern' (Blauvelt, NY, Summer 2027)</v>
+      </c>
+      <c r="C799" t="str">
+        <v>2026-10-06: Trade Compliance and Legal are non-engineering discipline (Legal's internal date inconsistency is moot given that); Systems Engineer Intern is wrong season. Found on the same Workday board as the 4 new qualifying Watts rows.</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="str">
+        <v>Applied Intuition</v>
+      </c>
+      <c r="B800" t="str">
+        <v>'Software Integration Engineer – New Grad (2027)'; 'Research Intern – Robotic Hardware, Simulation and Data'</v>
+      </c>
+      <c r="C800" t="str">
+        <v>2026-10-06: the first is a full-time new-grad role, not an internship; the second states no season and leans software/research, not mechanical.</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="str">
+        <v>True Anomaly</v>
+      </c>
+      <c r="B801" t="str">
+        <v>Full live Greenhouse board (196 open reqs, API-verified)</v>
+      </c>
+      <c r="C801" t="str">
+        <v>2026-10-06: zero postings with 'intern' or 'co-op' in the title currently exist; older indexed 'GSE Engineering Intern'/'Propulsion Engineering Intern' listings are stale/removed, not live.</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="str">
+        <v>Radiant Industries (El Segundo, CA)</v>
+      </c>
+      <c r="B802" t="str">
+        <v>Careers board</v>
+      </c>
+      <c r="C802" t="str">
+        <v>2026-10-06: only Summer 2026 internships (Nuclear Engineer, Materials Engineer) found; no Winter 2026/Spring 2027 postings live yet. Worth rechecking in 2-3 weeks.</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="str">
+        <v>JetZero</v>
+      </c>
+      <c r="B803" t="str">
+        <v>Careers board</v>
+      </c>
+      <c r="C803" t="str">
+        <v>2026-10-06: only a 2026 Engineering Summer Internship found; no Winter/Spring 2027 postings.</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="str">
+        <v>Electra.aero</v>
+      </c>
+      <c r="B804" t="str">
+        <v>Careers board</v>
+      </c>
+      <c r="C804" t="str">
+        <v>2026-10-06: only legacy 2025 internship program content found; nothing current for 2027.</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="str">
+        <v>Overland AI</v>
+      </c>
+      <c r="B805" t="str">
+        <v>Careers board</v>
+      </c>
+      <c r="C805" t="str">
+        <v>2026-10-06: no internship postings found; only full-time Senior Mechanical Engineer / Field Engineer / Forward Deployed Hardware Engineer roles.</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="str">
+        <v>Harmonic Drive LLC (Beverly/Peabody, MA)</v>
+      </c>
+      <c r="B806" t="str">
+        <v>Live careers page (9 openings)</v>
+      </c>
+      <c r="C806" t="str">
+        <v>2026-10-06: all full-time (CNC Machinist, Electro-Mechanical Assembler, etc.), zero internships/co-ops.</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="str">
+        <v>Sea Machines Robotics (Boston, MA)</v>
+      </c>
+      <c r="B807" t="str">
+        <v>Careers page</v>
+      </c>
+      <c r="C807" t="str">
+        <v>2026-10-06: only full-time Field Application Engineer / Automation &amp; Controls Engineer roles; no 2027 internship postings.</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="str">
+        <v>Pison Technology (Boston, MA)</v>
+      </c>
+      <c r="B808" t="str">
+        <v>Careers page</v>
+      </c>
+      <c r="C808" t="str">
+        <v>2026-10-06: only Spring/Summer 2025 Hardware/Firmware intern postings found (stale); no current 2027 listings. Worth a periodic re-check.</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="str">
+        <v>Vicor Corporation (Andover, MA)</v>
+      </c>
+      <c r="B809" t="str">
+        <v>Live careers search (27 current openings)</v>
+      </c>
+      <c r="C809" t="str">
+        <v>2026-10-06: zero internship/co-op titles; all full-time (Design Engineer, Reliability Engineer, etc.).</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="str">
+        <v>CIRCOR International</v>
+      </c>
+      <c r="B810" t="str">
+        <v>'Mechanical Engineer Intern' (Corona, CA, per jobs.weekday.works aggregator)</v>
+      </c>
+      <c r="C810" t="str">
+        <v>2026-10-06: aggregator-sourced posting states no Winter/Spring 2027 date; careers.circor.com confirms internships exist generically but routes to a JS-rendered UltiPro portal that could not be rendered/verified via fetch. Partial/unconfirmed — still excluded for lack of a verifiable, dated, qualifying posting. Worth a manual/browser check, and specifically check for a Warren, MA posting.</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="str">
+        <v>Skydio</v>
+      </c>
+      <c r="B811" t="str">
+        <v>'Hardware Test &amp; Reliability Intern – Fall 2026/Winter 2027' (San Mateo, CA); 'Electrical Engineer Intern – Winter 2027'</v>
+      </c>
+      <c r="C811" t="str">
+        <v>2026-10-06: RESOLVED the ambiguity flagged by 3 prior runs — the live Ashby board now clearly titles the hardware role 'Fall 2026/Winter 2027', confirming it does not match Hamza's Winter 2026/Spring 2027 target window (wrong season); the EE role is a discipline mismatch. Future runs should stop re-flagging this as ambiguous and simply treat it as excluded.</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="str">
+        <v>Anduril Industries</v>
+      </c>
+      <c r="B812" t="str">
+        <v>Full live Greenhouse board re-pull (API-verified); un-prefixed '2027 Mechanical Engineer Intern'/'2027 Manufacturing Engineer Intern'/'2027 Systems Engineer Intern' postings (some listing Boston, MA)</v>
+      </c>
+      <c r="C812" t="str">
+        <v>2026-10-06: all qualifying Winter 2027 co-ops already tracked; newly-seen Winter 2027 co-ops (Electrical Engineer, Software Engineer, Supply Chain Analyst, Technical Program Management) are discipline mismatches. The un-prefixed Boston-listed postings were confirmed via full job text to be explicitly Summer 2027 ('seeking ... Interns for Summer 2027! ... 12-week internship') despite the attractive location — wrong season.</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="str">
+        <v>Varda Space Industries</v>
+      </c>
+      <c r="B813" t="str">
+        <v>Full live Greenhouse board re-pull (API-verified): Applications Engineering, Avionics Engineering, Biologics Formulation Research, Cybersecurity, EH&amp;S, Flight Software, Site Reliability, Supply Chain (all Spring 2027)</v>
+      </c>
+      <c r="C813" t="str">
+        <v>2026-10-06: all qualifying Spring 2027 postings (Manufacturing Engineering, Mechanisms &amp; Payload, Structures, GNC, Propulsion, Vehicle Integration &amp; Test) already tracked. These new postings are discipline mismatches — Avionics Engineering confirmed via full job text to be circuit/flight-computer/battery electronics work (EE, not mechanical/structural); Applications Engineering is ERP/data-pipeline software work.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C793"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C813"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new postings, 21 checked-excluded (2026-10-06 19:20 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U1Tsy7bJ2GC2uD1jC3AJtn
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M390"/>
+  <dimension ref="A1:M391"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -14354,6 +14354,38 @@
       </c>
       <c r="J390" t="str">
         <v>One of 4 new Jan-Jun 2027 engineering Co-Ops posted on Watts' own Intern-External Workday board this run.</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>Mach Industries</v>
+      </c>
+      <c r="B391" t="str">
+        <v>Spring 2027 Engineering Internship</v>
+      </c>
+      <c r="C391" t="str">
+        <v>General engineering internship — track includes Mechanical and structural design, manufacturing, and test of hardware components (also propulsion/energetics, autonomy, embedded firmware tracks)</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E391" t="str">
+        <v>Huntington Beach, CA (also San Francisco, San Luis Obispo, and Victorville, CA)</v>
+      </c>
+      <c r="F391">
+        <v>2600</v>
+      </c>
+      <c r="G391" t="str">
+        <v>$30 - $55 / hr (stated pay range on posting)</v>
+      </c>
+      <c r="H391" t="str">
+        <v>https://job-boards.greenhouse.io/machindustries/jobs/4397035009</v>
+      </c>
+      <c r="I391" t="str">
+        <v>Yes — 2026-10-06: opened directly via the company's Greenhouse board/API (job id 4397035009, boards.greenhouse.io/machindustries). Posting's own text explicitly states 'Mach's Spring 2027 Engineering Internship... paid, in-person, 12-week internship' and asks for availability 'in spring 2027'. Job is currently listed live on the board (last updated 2026-09-24).</v>
+      </c>
+      <c r="J391" t="str">
+        <v>Defense manufacturing/autonomous-platforms company (munitions/defense tech). General engineering internship req (not a mechanical-only title), but mechanical/structural hardware design+manufacturing+test is explicitly one of the listed possible tracks. ITAR-restricted: requires US citizen/permanent resident/asylee/refugee status or ability to obtain export authorization. Not Boston-area. Same board also has 5 Summer 2027-titled internship reqs (Aerospace/Electrical/Manufacturing/Mechanical/Software-GNC) — excluded as wrong season, not added.</v>
       </c>
     </row>
   </sheetData>
@@ -14824,14 +14856,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M390"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M391"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C813"/>
+  <dimension ref="A1:C834"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -23772,9 +23804,240 @@
         <v>2026-10-06: all qualifying Spring 2027 postings (Manufacturing Engineering, Mechanisms &amp; Payload, Structures, GNC, Propulsion, Vehicle Integration &amp; Test) already tracked. These new postings are discipline mismatches — Avionics Engineering confirmed via full job text to be circuit/flight-computer/battery electronics work (EE, not mechanical/structural); Applications Engineering is ERP/data-pipeline software work.</v>
       </c>
     </row>
+    <row r="814">
+      <c r="A814" t="str">
+        <v>Firefly Aerospace</v>
+      </c>
+      <c r="B814" t="str">
+        <v>Full hrmdirect RSS/job-board sweep (120+ open reqs enumerated) — no 'intern' or 'co-op' titled engineering role found at all except 'Internship - Human Resources - Fall 2026' (non-engineering, wrong season)</v>
+      </c>
+      <c r="C814" t="str">
+        <v>2026-10-06: fresh full-board sweep via firefly.hrmdirect.com RSS feed, confirms no qualifying Winter 2026/Spring 2027 mechanical/aero/manufacturing postings currently exist.</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="str">
+        <v>Hadrian Automation</v>
+      </c>
+      <c r="B815" t="str">
+        <v>Software Engineer Intern, Robotics Engineer Intern (software/controls-focused, not hardware ME), Data Science/Data Engineer Intern — Ashby board jobs.ashbyhq.com/hadrian-automation, published 2026-09-02, Los Angeles CA</v>
+      </c>
+      <c r="C815" t="str">
+        <v>2026-10-06: resolved correct Ashby API slug ('hadrian-automation') and pulled full board (136 reqs) directly. None of the 3 intern postings state a Winter 2026/Spring 2027 season, and the Robotics Engineer Intern role is software/controls-focused, not hardware ME.</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="str">
+        <v>Stoke Space Technologies</v>
+      </c>
+      <c r="B816" t="str">
+        <v>Summer 2027 Internship - Engineering, Summer 2027 Internship - Operations, Summer 2027 Internship - Software (Cape Canaveral FL / Kent WA / Moses Lake WA) — Greenhouse board slug 'stokespacetechnologies'</v>
+      </c>
+      <c r="C816" t="str">
+        <v>2026-10-06: resolved correct Greenhouse API slug and pulled full board (66 reqs) directly. The previously-seen 'Spring 2027 Internship - Engineering' req is gone; board now shows only Summer 2027-dated internships.</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="str">
+        <v>Shield AI</v>
+      </c>
+      <c r="B817" t="str">
+        <v>Full Lever API sweep (592 postings). Electrical Engineering Spring Co-op (January 2027) R4475 (Dallas TX, already excluded) is the only Winter2026/Spring2027-dated eng co-op; all other intern/co-op titles (Advanced Manufacturing Engineering Intern, Electrical Engineering Co-op (June 2027), Electrical Engineering Intern, Mechanical Engineering Intern, Software Engineer Intern) are explicitly Summer 2027</v>
+      </c>
+      <c r="C817" t="str">
+        <v>2026-10-06: fresh direct Lever API pull confirms no new Winter2026/Spring2027 mechanical/aero/manufacturing postings beyond the already-excluded R4475.</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="str">
+        <v>Impulse Space</v>
+      </c>
+      <c r="B818" t="str">
+        <v>Full pinpointhq postings.json sweep (208 postings, ~27 intern titles). Only 'Manufacturing Engineering Intern (Spring 2027)' (already tracked) carries a Spring 2027 date; all ~26 other intern roles (Vehicle, Propulsion, Avionics, RF, Thermal, GN&amp;C, AI&amp;T, etc.) are explicitly Summer 2027</v>
+      </c>
+      <c r="C818" t="str">
+        <v>2026-10-06: direct API sweep confirms the already-tracked Spring 2027 Manufacturing Engineering Intern req is still the only Spring-2027-dated posting; no new req found.</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="str">
+        <v>Pickle Robot Company (Boston, MA)</v>
+      </c>
+      <c r="B819" t="str">
+        <v>Full Lever board — only senior/full-time mechanical &amp; mechatronics engineering roles (e.g. Principal Mechanical Engineer, Senior Mechanical Design Engineer); no internship/co-op postings found</v>
+      </c>
+      <c r="C819" t="str">
+        <v>2026-10-06: checked jobs.lever.co/picklerobot board, no intern-titled reqs</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="str">
+        <v>SES AI (Woburn, MA)</v>
+      </c>
+      <c r="B820" t="str">
+        <v>Full Greenhouse board (boards.greenhouse.io/sesai) — Boston/Woburn reqs are all senior/director-level; only intern-titled req found is a Computational Chemistry Intern based in China</v>
+      </c>
+      <c r="C820" t="str">
+        <v>2026-10-06: checked api.greenhouse.io/v1/boards/sesai/jobs, no US mechanical/manufacturing internship</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="str">
+        <v>Nimble Robotics</v>
+      </c>
+      <c r="B821" t="str">
+        <v>Full Greenhouse board — all full-time (Senior Mechanical Engineer, Robotics Field Engineer, Maintenance Technician, etc.), no internship reqs</v>
+      </c>
+      <c r="C821" t="str">
+        <v>2026-10-06: checked api.greenhouse.io/v1/boards/nimblerobotics/jobs</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="str">
+        <v>Form Energy (incl. Somerville, MA)</v>
+      </c>
+      <c r="B822" t="str">
+        <v>Full Ashby board (Berkeley CA / Weirton WV / Somerville MA sites) — ~160 reqs, all full-time staff/senior/manager titles, no internship or co-op postings</v>
+      </c>
+      <c r="C822" t="str">
+        <v>2026-10-06: checked api.ashbyhq.com/posting-api/job-board/formenergy</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="str">
+        <v>Standard Bots (incl. Boston, MA)</v>
+      </c>
+      <c r="B823" t="str">
+        <v>Full Ashby board — all full-time roles (CAD Designer, Automation Engineer, Senior Product Manager Hardware - Boston, etc.), no internship reqs</v>
+      </c>
+      <c r="C823" t="str">
+        <v>2026-10-06: checked api.ashbyhq.com/posting-api/job-board/standardbots</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="str">
+        <v>Via Separations (Woburn/Watertown, MA)</v>
+      </c>
+      <c r="B824" t="str">
+        <v>Mechanical Systems Engineering Co-Op</v>
+      </c>
+      <c r="C824" t="str">
+        <v>2026-10-06: posting is explicitly for Spring 2026, not Winter 2026 or Spring 2027 — wrong season. Tends to post this role seasonally on Lever (jobs.lever.co/viaseparations); worth a recheck closer to Spring 2027 recruiting season.</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="str">
+        <v>Covariant</v>
+      </c>
+      <c r="B825" t="str">
+        <v>General search for mechanical/robotics internship</v>
+      </c>
+      <c r="C825" t="str">
+        <v>2026-10-06: no internship postings found, only senior full-time mechanical/research roles (Emeryville, CA)</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="str">
+        <v>Chef Robotics</v>
+      </c>
+      <c r="B826" t="str">
+        <v>General search for mechanical/mechatronics internship</v>
+      </c>
+      <c r="C826" t="str">
+        <v>2026-10-06: no internship postings found, only senior mechanical/mechatronics engineer roles</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="str">
+        <v>Ambi Robotics</v>
+      </c>
+      <c r="B827" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C827" t="str">
+        <v>2026-10-06: checked api.lever.co/v0/postings/ambirobotics — all full-time (Berkeley, CA), no internships</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="str">
+        <v>Osaro</v>
+      </c>
+      <c r="B828" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C828" t="str">
+        <v>2026-10-06: checked api.lever.co/v0/postings/osaro — all full-time (SF), no internships</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="str">
+        <v>Gather AI</v>
+      </c>
+      <c r="B829" t="str">
+        <v>Full Greenhouse board</v>
+      </c>
+      <c r="C829" t="str">
+        <v>2026-10-06: checked api.greenhouse.io/v1/boards/gatherai/jobs — all full-time (Pittsburgh, PA), no internships</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="str">
+        <v>Cobalt Robotics</v>
+      </c>
+      <c r="B830" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C830" t="str">
+        <v>2026-10-06: checked api.lever.co/v0/postings/cobaltrobotics — only 1099-contractor 'Reserve Engineer' roles, no internships</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="str">
+        <v>Collier Aerospace (Raleigh, NC / Newport News, VA)</v>
+      </c>
+      <c r="B831" t="str">
+        <v>NCSG Aerospace Structural Engineering Intern; Application Engineering Intern; Methods &amp; Automations Intern; AI Feature Development Intern; Software Engineering Intern x2</v>
+      </c>
+      <c r="C831" t="str">
+        <v>2026-10-06: all 6 open internship reqs on ats.rippling.com/collieraerospace are explicitly titled 'Summer 2027' — wrong season</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="str">
+        <v>RAVE Aerospace</v>
+      </c>
+      <c r="B832" t="str">
+        <v>Workable job board (apply.workable.com/raveaerospace)</v>
+      </c>
+      <c r="C832" t="str">
+        <v>2026-10-06: could not retrieve a usable listing of open internship reqs from the page; unresolved, not reported as a finding. Worth trying a direct browser/API check next time.</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="str">
+        <v>Mach Industries</v>
+      </c>
+      <c r="B833" t="str">
+        <v>Summer 2027 Engineering Internship (Aerospace, Electrical, Manufacturing, Mechanical, Software/GNC tracks)</v>
+      </c>
+      <c r="C833" t="str">
+        <v>2026-10-06: 5 Summer 2027-titled internship reqs on same Greenhouse board as the Spring 2027 req added to `rows` this run — excluded as wrong season</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="str">
+        <v>Ascend Elements / 24M Technologies / Nanoramic Laboratories / Turion Space / Zap Energy / Type One Energy / TAE Technologies / Avalanche Energy / General Fusion / Proxima Fusion / Thea Energy / Xcimer Energy / Skild AI / Plus One Robotics / Fox Robotics / inVia Robotics / Aescape / Corvus Robotics</v>
+      </c>
+      <c r="B834" t="str">
+        <v>Attempted Greenhouse/Lever/Ashby board-token lookups</v>
+      </c>
+      <c r="C834" t="str">
+        <v>2026-10-06: no public ATS board found at guessed tokens (404/Not Found on all three platforms); not independently verifiable this pass, left unresolved rather than reported. Worth finding each company's actual career-page ATS link directly rather than guessing tokens.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C813"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C834"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 16 checked-excluded (2026-10-07 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XMM5ETJDDUf37qRkr1D3d9
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -13358,7 +13358,7 @@
         <v>https://jobs.solidprofessor.com/job/372053/engineering-co-op-internship-spring-2027/</v>
       </c>
       <c r="I359" t="str">
-        <v>Yes — 2026-10-06: upgraded from the generic ADP portal shell link (no longer needed) to a job-specific deep link found on SolidProfessor, Medical Murray's actual career-site ATS. Fetched directly and confirmed: title 'R&amp;D Engineering Co-op/Internship', North Barrington IL, $22.00/hr, 'Start Date: Spring of 2027', posted Sept 16 2026, Apply button live. Medical Murray's ADP API now returns an empty job-requisitions list for their cid — they appear to have moved listings to SolidProfessor.</v>
+        <v>Yes — 2026-10-06: upgraded from the generic ADP portal shell link (no longer needed) to a job-specific deep link found on SolidProfessor, Medical Murray's actual career-site ATS. Fetched directly and confirmed: title 'R&amp;D Engineering Co-op/Internship', North Barrington IL, $22.00/hr, 'Start Date: Spring of 2027', posted Sept 16 2026, Apply button live. Medical Murray's ADP API now returns an empty job-requisitions list for their cid — they appear to have moved listings to SolidProfessor. Re-confirmed HTTP 200 live 2026-10-07.</v>
       </c>
       <c r="J359" t="str">
         <v>Sibling Summer 2027 and Fall 2027 reqs also existed in the prior ADP feed (wrong season, excluded). SolidProfessor job IDs for this company appear to get reissued periodically (an older ID, 306224, for the same title already 404'd once) — worth a quick liveness re-check next run.</v>
@@ -14863,7 +14863,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C834"/>
+  <dimension ref="A1:C850"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -23372,7 +23372,7 @@
         <v>8 reqs: Manufacturing Engineer Intern/Co-Op (Wyman Gordon/Shultz Steel, South Gate CA, oppid 23458); Forge Shop Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23814); Heat Treat Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23815); Research Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24180); Mechanical Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24181); Engineer Co-Op $21/hr (Fasteners/AIC, Garden Grove CA, oppid 24183); CNC Machinist/Programmer Intern Co-Op (Structurals/Schlosser, Redmond OR, oppid 24238); Engineering Co-Op (Fasteners/Andrews Laser Works, Wilder KY, oppid 24353)</v>
       </c>
       <c r="C774" t="str">
-        <v>2026-10-06: each live posting was read in full but states no season anywhere (title or body) — cannot confirm Winter2026/Spring2027 fit either way. Not added to rows per the verification bar; flagged for a future revisit (PCC sometimes adds season language later), especially oppid 24181 (Henderson NV Mechanical Engineering Co-Op) which is a strong discipline match if the season resolves favorably. UPDATE 2026-10-06 (later run): re-checked all 8 — oppid 23458 is now confirmed closed ('This requisition is closed to applications'); the other 7, including priority oppid 24181, are still live and still state no season anywhere. Pattern looks structural/permanent for this template; deprioritize further automatic re-checks absent a site-wide PCC template change.</v>
+        <v>2026-10-06: each live posting was read in full but states no season anywhere (title or body) — cannot confirm Winter2026/Spring2027 fit either way. Not added to rows per the verification bar; flagged for a future revisit (PCC sometimes adds season language later), especially oppid 24181 (Henderson NV Mechanical Engineering Co-Op) which is a strong discipline match if the season resolves favorably. UPDATE 2026-10-06 (later run): re-checked all 8 — oppid 23458 is now confirmed closed ('This requisition is closed to applications'); the other 7, including priority oppid 24181, are still live and still state no season anywhere. Pattern looks structural/permanent for this template; deprioritize further automatic re-checks absent a site-wide PCC template change. UPDATE 2026-10-07: attempted re-check of oppid 24181 specifically — portal served an Altcha 'Quick Check Needed' CAPTCHA wall instead of content via curl/WebFetch; could not confirm or deny whether season language was added. Status unconfirmed, not assumed unchanged. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run instead of API/curl for this one.</v>
       </c>
     </row>
     <row r="775">
@@ -23922,7 +23922,7 @@
         <v>Mechanical Systems Engineering Co-Op</v>
       </c>
       <c r="C824" t="str">
-        <v>2026-10-06: posting is explicitly for Spring 2026, not Winter 2026 or Spring 2027 — wrong season. Tends to post this role seasonally on Lever (jobs.lever.co/viaseparations); worth a recheck closer to Spring 2027 recruiting season.</v>
+        <v>2026-10-06: posting is explicitly for Spring 2026, not Winter 2026 or Spring 2027 — wrong season. 2026-10-07 UPDATE: Lever board (api.lever.co/v0/postings/viaseparations) now returns an empty list — the Spring 2026 posting has been taken down entirely and no Spring 2027 posting has appeared yet. Recheck closer to Spring 2027 recruiting season (likely Nov-Dec 2026).</v>
       </c>
     </row>
     <row r="825">
@@ -24010,7 +24010,7 @@
         <v>Workable job board (apply.workable.com/raveaerospace)</v>
       </c>
       <c r="C832" t="str">
-        <v>2026-10-06: could not retrieve a usable listing of open internship reqs from the page; unresolved, not reported as a finding. Worth trying a direct browser/API check next time.</v>
+        <v>2026-10-06: could not retrieve a usable listing of open internship reqs from the page; unresolved, not reported as a finding. Worth trying a direct browser/API check next time. UPDATE 2026-10-07: retried via Workable's widget API and WebFetch — both blocked by Cloudflare (HTTP 429 'error code: 1015' bot-detection, retry-after ~22-23hrs; also a 302 redirect loop). This appears to be an IP/fingerprint-based persistent block for this environment's egress IP, not a simple rate limit. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run.</v>
       </c>
     </row>
     <row r="833">
@@ -24035,9 +24035,185 @@
         <v>2026-10-06: no public ATS board found at guessed tokens (404/Not Found on all three platforms); not independently verifiable this pass, left unresolved rather than reported. Worth finding each company's actual career-page ATS link directly rather than guessing tokens.</v>
       </c>
     </row>
+    <row r="835">
+      <c r="A835" t="str">
+        <v>Humanoid (thehumanoid.ai, Boston, MA)</v>
+      </c>
+      <c r="B835" t="str">
+        <v>Robotics Engineering Co-op (aggregator-only lead)</v>
+      </c>
+      <c r="C835" t="str">
+        <v>2026-10-07: queried the company's live Ashby API directly (jobs.ashbyhq.com/humanoid) — the aggregator-cited Co-op posting is no longer on the board. Current board has only 'Internship, Robot Learning Research' (London UK, software/research discipline) and full-time Mechanical Design Engineer roles. No open mechanical/hardware internship. Stale aggregator lead, not added.</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="str">
+        <v>Tutor Intelligence (MIT CSAIL spinout, Watertown, MA)</v>
+      </c>
+      <c r="B836" t="str">
+        <v>Robotics Research Scientist Intern (Winter/Spring 2026)</v>
+      </c>
+      <c r="C836" t="str">
+        <v>2026-10-07: confirmed via Lever API (api.lever.co/v0/postings/tutorintelligence) — posting's own text states season as 'Winter/Spring 2026' (not the target 2027 window) and discipline is AI/robot-learning research, not mechanical/hardware. Double disqualifier: wrong season + wrong discipline.</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="str">
+        <v>Walden Robotics (MIT/TRI spinout, Cambridge, MA)</v>
+      </c>
+      <c r="B837" t="str">
+        <v>Full Rippling-hosted job board (ats.rippling.com/walden-robotics)</v>
+      </c>
+      <c r="C837" t="str">
+        <v>2026-10-07: all current openings are full-time (MTS Mechanical/Electrical Design Engineer, etc.); zero internship/co-op/new-grad postings of any kind. No internship exists currently; worth a periodic re-check given strong discipline/location fit.</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="str">
+        <v>Nextera Robotics (MIT-founded, Boston, MA)</v>
+      </c>
+      <c r="B838" t="str">
+        <v>workatastartup.com listings</v>
+      </c>
+      <c r="C838" t="str">
+        <v>2026-10-07: only full-time roles found (Mechanical Engineer 3+ yrs exp, Robotics Assembly Specialist, part-time Equipment Assembly Technician). No internship/co-op posting found.</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="str">
+        <v>Nexus Robotics (Boston, MA, seed-stage)</v>
+      </c>
+      <c r="B839" t="str">
+        <v>General web search for careers page</v>
+      </c>
+      <c r="C839" t="str">
+        <v>2026-10-07: too new/small — no public careers page or job board (Greenhouse/Lever/Ashby) could be located at all. Unverifiable, not added.</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="str">
+        <v>Verve Motion (Harvard Biodesign spinout, Cambridge, MA)</v>
+      </c>
+      <c r="B840" t="str">
+        <v>Careers page (ADP-hosted)</v>
+      </c>
+      <c r="C840" t="str">
+        <v>2026-10-07: careers page redirects to a JS-rendered ADP (workforcenow.adp.com) portal unreadable via WebFetch/curl; no internship/co-op title surfaced in any search snippet (only full-time 3-5yr-experience roles). Unverifiable without a headless browser; strong discipline/location fit (exosuit mechanical engineering) if an internship does exist — worth a browser-based re-check.</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="str">
+        <v>Infinite Cooling (MIT MechE spinout, Malden, MA)</v>
+      </c>
+      <c r="B841" t="str">
+        <v>Engineering Co-op (standing posting, infinite-cooling.com/jobs/engineering-intern, also on jobs.orbit.mit.edu)</v>
+      </c>
+      <c r="C841" t="str">
+        <v>2026-10-07: confirmed live, mechanical-engineering discipline (prototype design, mechanical/pneumatic/structural systems), but the posting states no season/semester at all (rolling/continuous co-op) — cannot confirm Winter2026/Spring2027 fit per the verification bar. Excluded for now on season-unverifiable grounds; genuine Boston-area MechE co-op, worth a recurring check in case a future revision adds explicit dates, or a judgment call from Hamza on whether to include season-silent rolling co-ops.</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="str">
+        <v>Allen Control Systems (Austin, TX)</v>
+      </c>
+      <c r="B842" t="str">
+        <v>Manufacturing Intern(s)</v>
+      </c>
+      <c r="C842" t="str">
+        <v>2026-10-07: Greenhouse posting's own title explicitly reads 'Manufacturing Intern(s) - Summer 2026' — wrong season (and the prior year's summer wave).</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="str">
+        <v>Arc Boat Company (Torrance, CA)</v>
+      </c>
+      <c r="B843" t="str">
+        <v>Mechanical Engineering Intern - Powertrain</v>
+      </c>
+      <c r="C843" t="str">
+        <v>2026-10-07: confirmed via direct Greenhouse read — posting runs 'June 14th-August 20th 2027' — Summer 2027, out of scope.</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="str">
+        <v>CesiumAstro (Westminster, CO / Austin, TX / El Segundo, CA)</v>
+      </c>
+      <c r="B844" t="str">
+        <v>Full Lever board incl. Mechanical Engineering Internship (Austin TX &amp; Westminster CO)</v>
+      </c>
+      <c r="C844" t="str">
+        <v>2026-10-07: every internship on the board is explicitly titled 'Summer 2027' — wrong season, no Winter/Spring track.</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="str">
+        <v>Muon Space (San Jose/Mountain View, CA)</v>
+      </c>
+      <c r="B845" t="str">
+        <v>Full Greenhouse board incl. GNC Hardware, Environmental Test, Industrial Engineering, Thermal Engineering interns</v>
+      </c>
+      <c r="C845" t="str">
+        <v>2026-10-07: all internships explicitly titled '(Summer 2027)' — wrong season, no Winter/Spring track.</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="str">
+        <v>E-Space (Arlington, TX / Saratoga, CA)</v>
+      </c>
+      <c r="B846" t="str">
+        <v>Full Lever board (109 postings): 2027 Summer Internship; RF Product Development Lab Intern</v>
+      </c>
+      <c r="C846" t="str">
+        <v>2026-10-07: the 2027 Summer Internship is explicitly wrong season; the RF Product Development Lab Intern states no season but is RF/software test-automation discipline, not mechanical/aerospace/manufacturing. Excluded on both grounds.</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="str">
+        <v>Lightmatter (Boston, MA / Mountain View, CA)</v>
+      </c>
+      <c r="B847" t="str">
+        <v>Photonics Characterization Intern &amp; New Grad (Boston)</v>
+      </c>
+      <c r="C847" t="str">
+        <v>2026-10-07: confirmed PhD-candidate-only, Electrical Engineering/Physics discipline (silicon photonics testing), and states no specific season ('starting immediately'). Discipline mismatch + no season stated.</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="str">
+        <v>Portal Space Systems / Vannevar Labs / Boston Materials (Billerica, MA)</v>
+      </c>
+      <c r="B848" t="str">
+        <v>Full Greenhouse/Lever boards</v>
+      </c>
+      <c r="C848" t="str">
+        <v>2026-10-07: none currently has any internship/co-op posting of any discipline — all full-time, except Vannevar's one irrelevant 'MBA Intern Summer 2027'. Legitimate well-funded hardware/space companies; worth a periodic re-check rather than permanent exclusion.</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="str">
+        <v>Quindar / Katalyst Space / Albedo Space / Antaris / Scout Space / Vatn Systems / Ghost Robotics / Fortem Technologies / Anzu Robotics / Firestorm Labs / Bedrock Robotics / Cambrian Robotics / Dusty Robotics / 6K (6K Additive) / Persona AI</v>
+      </c>
+      <c r="B849" t="str">
+        <v>Attempted Greenhouse/Lever/Ashby board-token lookups and/or direct board review</v>
+      </c>
+      <c r="C849" t="str">
+        <v>2026-10-07: either no public ATS board found (404 across all three platforms) or board found but zero intern/co-op-titled roles live (e.g. Scout Space: Greenhouse board found, all senior/full-time remote roles; Vatn Systems: full Greenhouse board checked, zero intern/co-op titles). Not independently verifiable or no qualifying posting exists; not added.</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="str">
+        <v>Field AI</v>
+      </c>
+      <c r="B850" t="str">
+        <v>General re-search</v>
+      </c>
+      <c r="C850" t="str">
+        <v>2026-10-07: re-surfaced by search but re-confirms the two prior exclusions already logged (stale Boston aggregator lead not matching the real Irvine CA full-time role; self-contradictory Spring2027-titled/Fall2026-bodied Humanoid Manipulation posting). No new information.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C834"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C850"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 5 new postings, 33 checked-excluded (2026-10-07 07:06 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRLTRPZWA2u11uHBo2K7YM
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M391"/>
+  <dimension ref="A1:M396"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -14386,6 +14386,166 @@
       </c>
       <c r="J391" t="str">
         <v>Defense manufacturing/autonomous-platforms company (munitions/defense tech). General engineering internship req (not a mechanical-only title), but mechanical/structural hardware design+manufacturing+test is explicitly one of the listed possible tracks. ITAR-restricted: requires US citizen/permanent resident/asylee/refugee status or ability to obtain export authorization. Not Boston-area. Same board also has 5 Summer 2027-titled internship reqs (Aerospace/Electrical/Manufacturing/Mechanical/Software-GNC) — excluded as wrong season, not added.</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B392" t="str">
+        <v>Engineering Co-Op, Spring 2027</v>
+      </c>
+      <c r="C392" t="str">
+        <v>Materials / Mechanical / Industrial Engineering (facilities engineering support, SolidWorks)</v>
+      </c>
+      <c r="D392" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E392" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F392">
+        <v>565</v>
+      </c>
+      <c r="G392" t="str">
+        <v>$25.00/hr, 40 hrs/week</v>
+      </c>
+      <c r="H392" t="str">
+        <v>https://www.dice.com/job-detail/8c6abd4d-7d4b-41b7-afca-1b6afe12f647</v>
+      </c>
+      <c r="I392" t="str">
+        <v>Partial — 2026-10-07: PCC's own careers.precast.com remains blocked by an Altcha CAPTCHA wall; confirmed via direct fetch of the Dice.com mirror (oppid 22133), status 'Active,' updated within 9 hours of check, 'Apply Now' present. Verify on PCC's own site before applying.</v>
+      </c>
+      <c r="J392" t="str">
+        <v>Part of a 4-req PCC Spring 2027 sweep found via Dice mirrors this run; PCC's primary ATS has been CAPTCHA-blocked for several consecutive runs.</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>Precision Castparts Corp. (Airfoils Company / Mentor-Painesville)</v>
+      </c>
+      <c r="B393" t="str">
+        <v>Alloy Process Engineering Co-Op, Spring 2027</v>
+      </c>
+      <c r="C393" t="str">
+        <v>Process Engineering (mechanical/electrical/industrial, AutoCAD, material processing vendor coordination)</v>
+      </c>
+      <c r="D393" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E393" t="str">
+        <v>Mentor, OH</v>
+      </c>
+      <c r="F393">
+        <v>565</v>
+      </c>
+      <c r="G393" t="str">
+        <v>$25.00/hr</v>
+      </c>
+      <c r="H393" t="str">
+        <v>https://www.dice.com/job-detail/3b2de8b3-3b45-4c7c-910e-17bf7d69f3ed</v>
+      </c>
+      <c r="I393" t="str">
+        <v>Partial — 2026-10-07: PCC's own careers.precast.com remains blocked by an Altcha CAPTCHA wall; confirmed via direct fetch of the Dice.com mirror (oppid 22135), status 'Active.' Verify on PCC's own site before applying.</v>
+      </c>
+      <c r="J393" t="str">
+        <v>Part of the same 4-req PCC Spring 2027 sweep found via Dice mirrors this run.</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>Precision Castparts Corp. (EPD Company / E-One)</v>
+      </c>
+      <c r="B394" t="str">
+        <v>Engineering Co-Op, Spring 2027</v>
+      </c>
+      <c r="C394" t="str">
+        <v>Mechanical Engineering (CAD, component/system design, prototyping and testing)</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E394" t="str">
+        <v>Niskayuna, NY</v>
+      </c>
+      <c r="F394">
+        <v>175</v>
+      </c>
+      <c r="G394" t="str">
+        <v>$20.00-$22.00/hr</v>
+      </c>
+      <c r="H394" t="str">
+        <v>https://www.dice.com/job-detail/38cc072e-4927-47bb-890c-66a78069fa77</v>
+      </c>
+      <c r="I394" t="str">
+        <v>Partial — 2026-10-07: PCC's own careers.precast.com remains blocked by an Altcha CAPTCHA wall; confirmed via direct fetch of the Dice.com mirror (oppid 22911), status 'Active.' Verify on PCC's own site before applying.</v>
+      </c>
+      <c r="J394" t="str">
+        <v>ITAR/EAR-restricted — US Person status required. Part of the same 4-req PCC Spring 2027 sweep found via Dice mirrors this run.</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>Precision Castparts Corp. (Metals Company / Cannon Muskegon)</v>
+      </c>
+      <c r="B395" t="str">
+        <v>Spring 2027 Engineering Student Co-Op</v>
+      </c>
+      <c r="C395" t="str">
+        <v>Mechanical / Manufacturing Engineering (support for projects, planned outages, and mechanical equipment)</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E395" t="str">
+        <v>Muskegon, MI</v>
+      </c>
+      <c r="F395">
+        <v>830</v>
+      </c>
+      <c r="G395" t="str">
+        <v>Paid + housing stipend (amount not disclosed)</v>
+      </c>
+      <c r="H395" t="str">
+        <v>https://www.dice.com/job-detail/664d8441-eaf7-4e6f-8de4-90051e7ae0dd</v>
+      </c>
+      <c r="I395" t="str">
+        <v>Partial — 2026-10-07: PCC's own careers.precast.com remains blocked by an Altcha CAPTCHA wall; confirmed via direct fetch of the Dice.com mirror (oppid 22052), status 'Active.' Verify on PCC's own site before applying.</v>
+      </c>
+      <c r="J395" t="str">
+        <v>Requires 2+ years completed in an accredited engineering program. ITAR-restricted. Minimum 3-month full-time or 6-month part-time (20+ hrs/wk). Part of the same 4-req PCC Spring 2027 sweep found via Dice mirrors this run.</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>BAE Systems</v>
+      </c>
+      <c r="B396" t="str">
+        <v>2027 Spring and Summer Mechanical Engineering Coop</v>
+      </c>
+      <c r="C396" t="str">
+        <v>Mechanical Engineering (Navigation and Sensor Systems — ground/airborne hardware, CAD, integration/verification testing)</v>
+      </c>
+      <c r="D396" t="str">
+        <v>Spring/Summer 2027 (January through mid-August 2027)</v>
+      </c>
+      <c r="E396" t="str">
+        <v>Cedar Rapids, IA</v>
+      </c>
+      <c r="F396">
+        <v>1120</v>
+      </c>
+      <c r="G396" t="str">
+        <v>$46,437-$62,721 (annualized co-op pay band, per posting)</v>
+      </c>
+      <c r="H396" t="str">
+        <v>https://www.clearancejobs.com/jobs/8971498/2027-spring-and-summer-mechanical-engineering-coop</v>
+      </c>
+      <c r="I396" t="str">
+        <v>Partial — 2026-10-07: could not locate on BAE's own careers.baesystems.com/Workday ATS (search did not surface a first-party link); confirmed open on two independent third-party boards — ClearanceJobs.com (fetched directly, 'Apply now' present, posting states role 'will remain active until filled') and jobs.hiringourheroes.org/jobs/596763619 (same title/location/season, status 'currently open'). Verify on BAE's own site before applying.</v>
+      </c>
+      <c r="J396" t="str">
+        <v>Secret clearance with polygraph required. Not Boston-area. Jan-Aug 2027 cohort covers Spring 2027 even though it extends into summer.</v>
       </c>
     </row>
   </sheetData>
@@ -14856,14 +15016,14 @@
     <hyperlink ref="M199" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M396"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C850"/>
+  <dimension ref="A1:C883"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -23372,7 +23532,7 @@
         <v>8 reqs: Manufacturing Engineer Intern/Co-Op (Wyman Gordon/Shultz Steel, South Gate CA, oppid 23458); Forge Shop Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23814); Heat Treat Mfg Process Improvement Co-Op (Wyman Gordon, Houston TX, oppid 23815); Research Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24180); Mechanical Engineering Co-Op (Metals/Henderson, Henderson NV, oppid 24181); Engineer Co-Op $21/hr (Fasteners/AIC, Garden Grove CA, oppid 24183); CNC Machinist/Programmer Intern Co-Op (Structurals/Schlosser, Redmond OR, oppid 24238); Engineering Co-Op (Fasteners/Andrews Laser Works, Wilder KY, oppid 24353)</v>
       </c>
       <c r="C774" t="str">
-        <v>2026-10-06: each live posting was read in full but states no season anywhere (title or body) — cannot confirm Winter2026/Spring2027 fit either way. Not added to rows per the verification bar; flagged for a future revisit (PCC sometimes adds season language later), especially oppid 24181 (Henderson NV Mechanical Engineering Co-Op) which is a strong discipline match if the season resolves favorably. UPDATE 2026-10-06 (later run): re-checked all 8 — oppid 23458 is now confirmed closed ('This requisition is closed to applications'); the other 7, including priority oppid 24181, are still live and still state no season anywhere. Pattern looks structural/permanent for this template; deprioritize further automatic re-checks absent a site-wide PCC template change. UPDATE 2026-10-07: attempted re-check of oppid 24181 specifically — portal served an Altcha 'Quick Check Needed' CAPTCHA wall instead of content via curl/WebFetch; could not confirm or deny whether season language was added. Status unconfirmed, not assumed unchanged. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run instead of API/curl for this one.</v>
+        <v>2026-10-06: each live posting was read in full but states no season anywhere (title or body) — cannot confirm Winter2026/Spring2027 fit either way. Not added to rows per the verification bar; flagged for a future revisit (PCC sometimes adds season language later), especially oppid 24181 (Henderson NV Mechanical Engineering Co-Op) which is a strong discipline match if the season resolves favorably. UPDATE 2026-10-06 (later run): re-checked all 8 — oppid 23458 is now confirmed closed ('This requisition is closed to applications'); the other 7, including priority oppid 24181, are still live and still state no season anywhere. Pattern looks structural/permanent for this template; deprioritize further automatic re-checks absent a site-wide PCC template change. UPDATE 2026-10-07: attempted re-check of oppid 24181 specifically — portal served an Altcha 'Quick Check Needed' CAPTCHA wall instead of content via curl/WebFetch; could not confirm or deny whether season language was added. Status unconfirmed, not assumed unchanged. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run instead of API/curl for this one. UPDATE 2026-10-07 (later run): still CAPTCHA-blocked on oppid 24181 itself via every URL-pattern/PeopleSoft-guess attempt tried; however a separate, different Henderson NV req ('Mechanical Engineer Co-Op', oppid ~23630, found via Dice mirror) was confirmed HTTP 410 Gone — that one has expired. oppid 24181 status remains genuinely unresolved either way.</v>
       </c>
     </row>
     <row r="775">
@@ -24010,7 +24170,7 @@
         <v>Workable job board (apply.workable.com/raveaerospace)</v>
       </c>
       <c r="C832" t="str">
-        <v>2026-10-06: could not retrieve a usable listing of open internship reqs from the page; unresolved, not reported as a finding. Worth trying a direct browser/API check next time. UPDATE 2026-10-07: retried via Workable's widget API and WebFetch — both blocked by Cloudflare (HTTP 429 'error code: 1015' bot-detection, retry-after ~22-23hrs; also a 302 redirect loop). This appears to be an IP/fingerprint-based persistent block for this environment's egress IP, not a simple rate limit. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run.</v>
+        <v>2026-10-06: could not retrieve a usable listing of open internship reqs from the page; unresolved, not reported as a finding. Worth trying a direct browser/API check next time. UPDATE 2026-10-07: retried via Workable's widget API and WebFetch — both blocked by Cloudflare (HTTP 429 'error code: 1015' bot-detection, retry-after ~22-23hrs; also a 302 redirect loop). This appears to be an IP/fingerprint-based persistent block for this environment's egress IP, not a simple rate limit. Recommend a browser-driven check (Claude in Chrome / built-in browser) on a future run. UPDATE 2026-10-07 (later run): a third-party aggregator (embedded.jobs/company/rave-aerospace) successfully rendered the full board and shows 0 currently open positions (all 6 listed roles — software/test, no interns — marked expired, hiring pace 'moderated'). Also: RAVE is primarily an in-flight-entertainment/connectivity (IFEC) company — software/embedded/electrical-heavy, weak fit for mechanical/aerospace-structures even if something reopens. Deprioritizing further automatic re-checks.</v>
       </c>
     </row>
     <row r="833">
@@ -24211,9 +24371,372 @@
         <v>2026-10-07: re-surfaced by search but re-confirms the two prior exclusions already logged (stale Boston aggregator lead not matching the real Irvine CA full-time role; self-contradictory Spring2027-titled/Fall2026-bodied Humanoid Manipulation posting). No new information.</v>
       </c>
     </row>
+    <row r="851">
+      <c r="A851" t="str">
+        <v>Verve Motion (Cambridge, MA)</v>
+      </c>
+      <c r="B851" t="str">
+        <v>Site search, LinkedIn/Lever/Workday/Indeed/ZipRecruiter/Glassdoor site: filters</v>
+      </c>
+      <c r="C851" t="str">
+        <v>2026-10-07 (later run): no internship/co-op posting found by any indirect route; the ADP-hosted careers page remains effectively unindexed by search engines. Unresolved — still needs a direct browser render.</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="str">
+        <v>Watts Water Technologies</v>
+      </c>
+      <c r="B852" t="str">
+        <v>Manufacturing Engineer Co-Op (Menomonee Falls/Germantown, WI)</v>
+      </c>
+      <c r="C852" t="str">
+        <v>2026-10-07 (later run): found via search, but both joinrunway.io mirrors confirmed 'Applications Closed,' and the season stated was July-December 2026 (Fall, not Winter2026/Spring2027) — excluded on both status and season grounds.</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="str">
+        <v>Draper Laboratory (Cambridge, MA)</v>
+      </c>
+      <c r="B853" t="str">
+        <v>Acoustic and Vibration Technologies Co-op; Metrology Co-Op</v>
+      </c>
+      <c r="C853" t="str">
+        <v>2026-10-07 (later run): both open, Cambridge MA, $20-45/hr, but neither states an explicit season/date range on the available posting text — fails the strict season-verification bar even though Draper's own site says Spring Co-Ops are posted in October for Jan-June work (that's inference, not a stated date). Worth opening the actual student-draper.icims.com posting page directly next run (guessed/indexed URLs 404'd this time) to check for explicit season language. Separately, a 'Mechanical Engineering &amp; System Packaging Intern' (Cambridge MA/St. Petersburg FL) is explicitly Summer 2027 — excluded. The previously-tracked 'Electro-Mechanical Fall Co-Op Student' job 8005 now 404s — appears expired.</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="str">
+        <v>Precision Castparts Corp. — 'Quality Engineering Co-Op, Spring 2027'</v>
+      </c>
+      <c r="B854" t="str">
+        <v>Campus career-service mirror titles (careerservices.hsutx.edu, careers.canton.edu)</v>
+      </c>
+      <c r="C854" t="str">
+        <v>2026-10-07 (later run): title/season exists per campus mirrors, but both direct links 404'd and no Dice/other mirror with an opportunity ID or location could be found. Unconfirmed — not added. Worth retrying next cycle in case it surfaces on Dice/joinrunway the way the Mentor/Niskayuna/Muskegon PCC reqs did.</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="str">
+        <v>GE Aerospace (Lynn, MA)</v>
+      </c>
+      <c r="B855" t="str">
+        <v>Spring 2027 'Manufacturing Engineering Co-op' and 'Engines Engineering Co-op - Returning Students' candidate titles</v>
+      </c>
+      <c r="C855" t="str">
+        <v>2026-10-07 (later run): careers.geaerospace.com remains JS-rendered/blocked to direct fetch; Indeed/Glassdoor listing pages that would show the primary text returned HTTP 403. Search-snippet-only, NOT independently opened — not reported as a finding. Note: a confirmed-elsewhere 'Manufacturing Engineering Co-op - US - Spring 2027' with the same title is actually located in Batesville, AR, not Lynn — don't assume the Lynn version is the same req without direct confirmation. A 'Systems Engineering Co-op' Spring 2027 Returning Students role at this employer is Electrical/Computer/Electric-Power discipline — excluded regardless, discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="str">
+        <v>Vicarious Surgical (Waltham, MA)</v>
+      </c>
+      <c r="B856" t="str">
+        <v>Mechanical Engineering Co-Op (Jan 2026); Product Development Engineering Co-Op</v>
+      </c>
+      <c r="C856" t="str">
+        <v>2026-10-07: both confirmed via khoslaventures.com board: 'This job is no longer accepting applications.'</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="str">
+        <v>Markforged (Waltham, MA)</v>
+      </c>
+      <c r="B857" t="str">
+        <v>Full Greenhouse board</v>
+      </c>
+      <c r="C857" t="str">
+        <v>2026-10-07: zero intern/co-op postings; only 3 full-time professional roles currently listed.</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="str">
+        <v>Commonwealth Fusion Systems (Devens/Somerville, MA)</v>
+      </c>
+      <c r="B858" t="str">
+        <v>Full Lever board</v>
+      </c>
+      <c r="C858" t="str">
+        <v>2026-10-07: only Spring 2026, Fall 2026, and Summer 2026 internship reqs exist; no Spring 2027 posting yet. CFS posts ~2 months ahead historically — worth checking back Nov/Dec 2026.</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="str">
+        <v>Boston Dynamics (Waltham, MA)</v>
+      </c>
+      <c r="B859" t="str">
+        <v>Official careers page; zerogtalent aggregator listings (R2496, R2476, R2534, R2536)</v>
+      </c>
+      <c r="C859" t="str">
+        <v>2026-10-07: official page states 'Internship recruiting season kicks off in the new year' with no active season-tagged reqs; aggregator listings carry no season tag and appear to date to ~March 2026 (likely stale Summer 2026 cohort). No Winter2026/Spring2027 req exists yet — strong Boston-area candidate once they open; re-check Dec 2026/Jan 2027.</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="str">
+        <v>Piaggio Fast Forward (Boston, MA)</v>
+      </c>
+      <c r="B860" t="str">
+        <v>Current open roles</v>
+      </c>
+      <c r="C860" t="str">
+        <v>2026-10-07: only a Robotics &amp; AI Co-op and a Mechanical Engineering Machinist/Technician role currently open; neither is a season-tagged mechanical engineering co-op. Boston-based with an active program — worth periodic re-checking.</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="str">
+        <v>SharkNinja / iRobot (Needham, MA)</v>
+      </c>
+      <c r="B861" t="str">
+        <v>Intern/co-op board</v>
+      </c>
+      <c r="C861" t="str">
+        <v>2026-10-07: only Summer 2026 and Fall 2026 (Jul-Dec 2026) mechanical co-op reqs found; no Spring 2027 posting yet. Likely posts late 2026 — re-check Nov/Dec.</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="str">
+        <v>Textron Systems / Howe &amp; Howe</v>
+      </c>
+      <c r="B862" t="str">
+        <v>'2027 Mechanical Engineer Intern' (Augusta, GA)</v>
+      </c>
+      <c r="C862" t="str">
+        <v>2026-10-07: confirmed explicitly Summer 2027 (10-week paid summer program) — wrong season.</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="str">
+        <v>Honeywell Aerospace</v>
+      </c>
+      <c r="B863" t="str">
+        <v>2027 mechanical engineering internship postings</v>
+      </c>
+      <c r="C863" t="str">
+        <v>2026-10-07: all found postings are explicitly Summer 2027 — wrong season.</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="str">
+        <v>Woodward Inc. (Zeeland, MI)</v>
+      </c>
+      <c r="B864" t="str">
+        <v>Co-op board</v>
+      </c>
+      <c r="C864" t="str">
+        <v>2026-10-07: only a Summer 2027 co-op found — wrong season.</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="str">
+        <v>BAE Systems (Southern NH Electronic Systems / LEAP program)</v>
+      </c>
+      <c r="B865" t="str">
+        <v>NH-based mechanical engineering internships</v>
+      </c>
+      <c r="C865" t="str">
+        <v>2026-10-07: all found are explicitly Summer 2027 only; no Spring 2027 NH req located. (Separately, see `rows` for a genuine Spring/Summer 2027 BAE mechanical co-op found this run in Cedar Rapids, IA.)</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="str">
+        <v>Curtiss-Wright (Cheswick, PA)</v>
+      </c>
+      <c r="B866" t="str">
+        <v>jobs.buildsubmarines.com career board</v>
+      </c>
+      <c r="C866" t="str">
+        <v>2026-10-07: direct fetch returned HTTP 403 (blocked). General listings confirm continuous Spring/Summer/Fall co-op hiring but no specific open Spring 2027 mechanical req could be confirmed. Worth retrying via their direct ATS with a different fetch path next run.</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="str">
+        <v>Parker Hannifin Aerospace / HEICO</v>
+      </c>
+      <c r="B867" t="str">
+        <v>General search for Spring 2027/Winter 2026 postings</v>
+      </c>
+      <c r="C867" t="str">
+        <v>2026-10-07: no season-specific postings surfaced; both appear to hire on a rolling continuous basis with no discoverable current mechanical co-op req matching the target window.</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="str">
+        <v>Figure AI (San Jose, CA)</v>
+      </c>
+      <c r="B868" t="str">
+        <v>Winter 2026 'Integration and Test' mechanical intern; Fall 2026 postings</v>
+      </c>
+      <c r="C868" t="str">
+        <v>2026-10-07: in-season by discipline/date but no Spring 2027 req found, and San Jose is far outside the Boston preference; open/closed status of the Winter 2026 req not independently re-verified this pass. Low priority.</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="str">
+        <v>Sanctuary AI (Vancouver, BC)</v>
+      </c>
+      <c r="B869" t="str">
+        <v>Hardware R&amp;D Co-op; current Product Management internship</v>
+      </c>
+      <c r="C869" t="str">
+        <v>2026-10-07: Hardware R&amp;D Co-op was for Jan 2026 (already past); current open internship isn't mechanical. Also non-US (Vancouver, BC) — likely ineligible regardless.</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="str">
+        <v>Agility Robotics (Salem, OR / Fremont, CA)</v>
+      </c>
+      <c r="B870" t="str">
+        <v>Mechanical intern postings</v>
+      </c>
+      <c r="C870" t="str">
+        <v>2026-10-07: only a Summer 2026 posting found; no 2027 postings yet.</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="str">
+        <v>Veo Robotics (Waltham, MA)</v>
+      </c>
+      <c r="B871" t="str">
+        <v>Careers page</v>
+      </c>
+      <c r="C871" t="str">
+        <v>2026-10-07: zero open roles currently; historical co-op references are stale (2022 blog post only).</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="str">
+        <v>Xona Space Systems (Burlingame, CA)</v>
+      </c>
+      <c r="B872" t="str">
+        <v>Mechanical Engineering Co-op (Spring 2027)</v>
+      </c>
+      <c r="C872" t="str">
+        <v>2026-10-07: directly confirmed CLOSED — 'This job is no longer accepting applications.'</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="str">
+        <v>Boston Scientific (Marlborough, MA / St. Paul, MN)</v>
+      </c>
+      <c r="B873" t="str">
+        <v>Packaging Engineer and R&amp;D Engineer Fall/Winter 2026 and Winter/Spring 2027 co-op reqs</v>
+      </c>
+      <c r="C873" t="str">
+        <v>2026-10-07: all independently confirmed CLOSED via direct fetch ('Sorry this position is no longer posted' / 'no longer accepting applications').</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="str">
+        <v>BALA Consulting Engineers (Boston, MA)</v>
+      </c>
+      <c r="B874" t="str">
+        <v>Mechanical Engineering Co-op (MEP/AEC)</v>
+      </c>
+      <c r="C874" t="str">
+        <v>2026-10-07: listing's own stated expiration date (August 30, 2026) has passed — stale/closed.</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="str">
+        <v>Joby Aviation (San Carlos, CA)</v>
+      </c>
+      <c r="B875" t="str">
+        <v>Mechanical Engineer Intern - Electric Propulsion Unit (Winter 2027)</v>
+      </c>
+      <c r="C875" t="str">
+        <v>2026-10-07: confirmed CLOSED on two independent mirrors (HTTP 410 Gone on icims; 'no longer accepting applications' on eniac.vc mirror). Note for future searches: Joby labels this cohort 'Winter 2027' (Jan-Mar 2027) rather than 'Winter 2026' — same real-world timeframe Hamza is targeting, worth searching both phrasings.</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="str">
+        <v>Archer Aviation (San Jose, CA)</v>
+      </c>
+      <c r="B876" t="str">
+        <v>Mechanical/development intern postings</v>
+      </c>
+      <c r="C876" t="str">
+        <v>2026-10-07: only Summer 2026 reqs found; no Spring 2027/Winter postings.</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="str">
+        <v>Hadrian</v>
+      </c>
+      <c r="B877" t="str">
+        <v>Intern postings</v>
+      </c>
+      <c r="C877" t="str">
+        <v>2026-10-07: intern postings found are Software/Data/Robotics-software focused; the one mechanical-titled role (Factory Automation) is full-time, not an internship/co-op.</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="str">
+        <v>Saronic Technologies (Austin, TX)</v>
+      </c>
+      <c r="B878" t="str">
+        <v>Mechanical Engineer Intern</v>
+      </c>
+      <c r="C878" t="str">
+        <v>2026-10-07: explicitly Summer 2027 — wrong season.</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="str">
+        <v>AeroVironment</v>
+      </c>
+      <c r="B879" t="str">
+        <v>Spring/2027 postings</v>
+      </c>
+      <c r="C879" t="str">
+        <v>2026-10-07: Spring postings found are dated Spring 2026 (already past); current 2027 postings are explicitly Summer 2027.</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="str">
+        <v>Saildrone (Alameda, CA)</v>
+      </c>
+      <c r="B880" t="str">
+        <v>General internship program</v>
+      </c>
+      <c r="C880" t="str">
+        <v>2026-10-07: composites/mechanical/CS internship program mentioned generally but no specific 2027-dated posting discoverable.</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="str">
+        <v>BETA Technologies (South Burlington, VT)</v>
+      </c>
+      <c r="B881" t="str">
+        <v>Full internship listing on beta.team (Aircraft Design &amp; Engineering, Manufacturing &amp; Production, etc.)</v>
+      </c>
+      <c r="C881" t="str">
+        <v>2026-10-07: all currently live listings are explicitly 'Summer 2027' ($22-32/hr). Earlier '2026-2027 BETA Internship' postings (which might have covered Spring 2027) are now expired/404.</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="str">
+        <v>Desktop Metal / Nano Dimension</v>
+      </c>
+      <c r="B882" t="str">
+        <v>Careers pages</v>
+      </c>
+      <c r="C882" t="str">
+        <v>2026-10-07: Desktop Metal directs resumes via email with no formal posting; Nano Dimension's NDEAR is an academic partnership program, not a discrete internship req. No qualifying posting.</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="str">
+        <v>Carbon Robotics</v>
+      </c>
+      <c r="B883" t="str">
+        <v>Careers page</v>
+      </c>
+      <c r="C883" t="str">
+        <v>2026-10-07: only a software intern and senior full-time mechanical roles found; no mechanical intern/co-op posting.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C850"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C883"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 8 checked-excluded (2026-10-08 01:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Em61phKYiWnZEGaR6cqv7D
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M398"/>
+  <dimension ref="A1:M401"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -14601,6 +14601,102 @@
       </c>
       <c r="J398" t="str">
         <v>Robotics/mechatronics discipline fit. Posting also allows a Jan–Aug 2027 window; Jan–May 2027 satisfies Hamza's Spring 2027 target.</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>BMW Group</v>
+      </c>
+      <c r="B399" t="str">
+        <v>Assembly Manufacturing Engineer Co-op (Spring 2027)</v>
+      </c>
+      <c r="C399" t="str">
+        <v>Manufacturing Engineering / Industrial Engineering</v>
+      </c>
+      <c r="D399" t="str">
+        <v>Spring 2027 (Jan 11 – May 14, 2027)</v>
+      </c>
+      <c r="E399" t="str">
+        <v>Spartanburg, SC</v>
+      </c>
+      <c r="F399">
+        <v>850</v>
+      </c>
+      <c r="G399" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="H399" t="str">
+        <v>https://jobs.bmwgroup.com/job/Assembly-Manufacturing-Engineer-Co-op-%28Spring-2027%29/191166-en_US/</v>
+      </c>
+      <c r="I399" t="str">
+        <v>Yes — fetched the live posting directly on jobs.bmwgroup.com, 'Apply now' present, no closed/filled messaging.</v>
+      </c>
+      <c r="J399" t="str">
+        <v>Requires enrolled student at accredited US 4-yr institution, min 3.0 GPA, 30+ completed credit hours, enrolled through all 3 rotations. No explicit citizenship/ITAR language seen.</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>BMW Group</v>
+      </c>
+      <c r="B400" t="str">
+        <v>Manufacturing Process Improvement Co-Op (Spring 2027)</v>
+      </c>
+      <c r="C400" t="str">
+        <v>Manufacturing Engineering / Industrial Engineering</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Spring 2027 (Jan 11 – May 14, 2027)</v>
+      </c>
+      <c r="E400" t="str">
+        <v>Spartanburg, SC</v>
+      </c>
+      <c r="F400">
+        <v>850</v>
+      </c>
+      <c r="G400" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="H400" t="str">
+        <v>https://jobs.bmwgroup.com/job/Manufacturing-Process-Improvement-Co-Op-%28Spring-2027%29/191747-en_US/</v>
+      </c>
+      <c r="I400" t="str">
+        <v>Yes — fetched the live posting directly on jobs.bmwgroup.com, 'Apply now' present, no closed/filled messaging.</v>
+      </c>
+      <c r="J400" t="str">
+        <v>Same eligibility requirements as the sibling Assembly Manufacturing Engineer Co-op req (same batch, Spartanburg SC plant).</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>BMW Group</v>
+      </c>
+      <c r="B401" t="str">
+        <v>Production Process and Quality Co-op (Spring 2027)</v>
+      </c>
+      <c r="C401" t="str">
+        <v>Mechanical or Industrial Engineering (preferred)</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Spring 2027 (Jan 11 – May 14, 2027)</v>
+      </c>
+      <c r="E401" t="str">
+        <v>Spartanburg, SC</v>
+      </c>
+      <c r="F401">
+        <v>850</v>
+      </c>
+      <c r="G401" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="H401" t="str">
+        <v>https://jobs.bmwgroup.com/job/Production-Process-and-Quality-Co-op-%28Spring-2027%29/192803-en_US/</v>
+      </c>
+      <c r="I401" t="str">
+        <v>Yes — fetched the live posting directly on jobs.bmwgroup.com, 'Apply now' present, no closed/filled messaging.</v>
+      </c>
+      <c r="J401" t="str">
+        <v>Hybrid quality/process engineering role. Same eligibility requirements as sibling Spartanburg SC co-ops above.</v>
       </c>
     </row>
   </sheetData>
@@ -15071,14 +15167,14 @@
     <hyperlink ref="M198" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M398"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M401"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C894"/>
+  <dimension ref="A1:C902"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -24896,7 +24992,7 @@
         <v>Manufacturing Engineering Co-op – US – Spring 2027 (Batesville, AR)</v>
       </c>
       <c r="C893" t="str">
-        <v>2026-10-07: confirmed via a Runway job-board mirror of the exact posting as 'Applications Closed.' (The Rutland, VT sibling req could not be independently confirmed this run — no working GE req ID/URL located; not added, not excluded.)</v>
+        <v>2026-10-07: confirmed via a Runway job-board mirror of the exact posting as 'Applications Closed.' (The Rutland, VT sibling req could not be independently confirmed this run — no working GE req ID/URL located; not added, not excluded.) CORRECTION (2026-10-08): this was a false negative. Direct fetch of GE's own Workday CXS API for req R5029663 (the already-tracked `rows` entry) shows it is a SINGLE multi-location req with 23 selectable US sites, and its own `additionalLocations` array includes BOTH Batesville, AR and Rutland, VT alongside Lynn, MA and 20 others — they are not separate sibling reqs. Authoritative status from GE's own API as of today: canApply:true, posted:true, endDate 2026-11-06, '29 days left to apply.' The Runway mirror's 'Applications Closed' signal for Batesville was wrong (same known false-negative pattern this tracker has documented for GE's marketing-portal/aggregator mirrors vs. its Workday API on 2026-09-30, 2026-10-01, 2026-10-02). No separate row needed — Batesville and Rutland are both already covered by the existing R5029663 row; this exclusion entry is kept only as a historical record of the correction.</v>
       </c>
     </row>
     <row r="894">
@@ -24910,9 +25006,97 @@
         <v>2026-10-07: re-fetched directly via ADI's own Workday CXS API; the internal season contradiction first noted 2026-09-28 is still unresolved — the role-overview paragraph still says 'running from June through December' while the Qualifications section still says 'available... from January through June.' Exclusion stands.</v>
       </c>
     </row>
+    <row r="895">
+      <c r="A895" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B895" t="str">
+        <v>Fresh sweep of careers.ll.mit.edu for Winter 2026/Spring 2027 mechanical/aero co-ops</v>
+      </c>
+      <c r="C895" t="str">
+        <v>2026-10-08: re-confirmed via fresh search — only 'Fall CO-OP Student (Mechanical Engineering, 07-71)' (Fall 2026), 'Rapid Prototyping Aero/Mech Co-Op (Fall 2026) – Group 77,' and 'CAD Design Specialist CO-OP, Group 07-71 (June–November 2026)' are currently live in-discipline, all wrong season. No new Winter 2026/Spring 2027 req found beyond the 3 already tracked (microfab x2 + Group 07-71 Mechanical Engineering Co-Op).</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="str">
+        <v>Precision Castparts Corp (Henderson, NV)</v>
+      </c>
+      <c r="B896" t="str">
+        <v>oppid 24181 (Mechanical Engineering Co-Op) — re-check</v>
+      </c>
+      <c r="C896" t="str">
+        <v>2026-10-08: direct fetch of the tal.net posting URL again hit PCC's Altcha bot-check wall ('Quick Check Needed'), same as prior attempts — confirms this is an intermittent/token-based block rather than a resolved access path. Disposition unchanged from 2026-10-07: already confirmed open/live once via a cleared CAPTCHA, but excluded because the posting states no season anywhere in title or body.</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="str">
+        <v>BMW Group</v>
+      </c>
+      <c r="B897" t="str">
+        <v>Controls Engineering Co-op (Spring 2027), req 191197; Acoustics Co-Op (Spring 2027), req 191204</v>
+      </c>
+      <c r="C897" t="str">
+        <v>2026-10-08: both confirmed via direct fetch today as 'You can't view this job because it's not available at this time' — closed. Found during the same Spartanburg, SC Spring 2027 co-op batch as the 3 reqs added to `rows` this run.</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="str">
+        <v>Ahlstrom Nonwovens LLC (Stevens Point, WI)</v>
+      </c>
+      <c r="B898" t="str">
+        <v>PM35 Process Engineer Co-op, Spring 2027</v>
+      </c>
+      <c r="C898" t="str">
+        <v>2026-10-08: Paper Science/Chemical Engineering discipline — a weak fit for Hamza's mechanical/aerospace/manufacturing/robotics/adjacent target list. Could not locate Ahlstrom's own primary ATS posting; only a Dice.com aggregator mirror was found, which itself shows conflicting freshness signals ('Updated 4 hours ago' vs. 'Posted 30+ days ago'). Not added — discipline fit too weak and primary-source verification unavailable.</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="str">
+        <v>Edwards Lifesciences (Irvine, CA / Draper, UT)</v>
+      </c>
+      <c r="B899" t="str">
+        <v>Engineering Co-Op Program, Spring-Summer 2027</v>
+      </c>
+      <c r="C899" t="str">
+        <v>2026-10-08: confirmed live/open (Jan–Aug 2027) but discipline is R&amp;D/Clinical Development/Quality Engineer for structural heart devices — biomedical, not mechanical/aerospace/manufacturing/robotics. Not added.</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="str">
+        <v>Halo Braid (Cambridge/Allston, MA)</v>
+      </c>
+      <c r="B900" t="str">
+        <v>Mechanical Engineering Co-op</v>
+      </c>
+      <c r="C900" t="str">
+        <v>2026-10-08: only a Fall 2026 Mechanical Engineering Co-op found (posted 2026-05-07); no Spring 2027 cycle located anywhere. Not added — wrong/no season.</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="str">
+        <v>Crown Equipment Corporation</v>
+      </c>
+      <c r="B901" t="str">
+        <v>Handshake-listed 'Mechanical Engineering Co-op - Spring 2027' (forklift/material-handling focus, location unstated)</v>
+      </c>
+      <c r="C901" t="str">
+        <v>2026-10-08: company already has 2 Mechanical Engineering Co-op/Intern rows tracked (Greencastle IN, Kinston NC); the Handshake preview didn't state a location, so could not confirm this is a genuinely distinct 3rd site rather than a duplicate of an already-tracked posting. Not added, to avoid a probable duplicate.</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="str">
+        <v>WSP USA</v>
+      </c>
+      <c r="B902" t="str">
+        <v>Mechanical Engineering Co-op (Drexel co-op program, Philadelphia), 'Fall 2026/Winter 2027'</v>
+      </c>
+      <c r="C902" t="str">
+        <v>2026-10-08: season is explicitly 'Winter 2027,' not 'Winter 2026' — same near-miss exclusion this tracker has already applied to Astranis/Skydio 'Winter 2027' cohorts. Not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C894"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C902"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 14 checked-excluded (2026-10-08 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xd62HpppJJLgiRq7DP3Gdn
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -15174,7 +15174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C902"/>
+  <dimension ref="A1:C916"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -25025,7 +25025,7 @@
         <v>oppid 24181 (Mechanical Engineering Co-Op) — re-check</v>
       </c>
       <c r="C896" t="str">
-        <v>2026-10-08: direct fetch of the tal.net posting URL again hit PCC's Altcha bot-check wall ('Quick Check Needed'), same as prior attempts — confirms this is an intermittent/token-based block rather than a resolved access path. Disposition unchanged from 2026-10-07: already confirmed open/live once via a cleared CAPTCHA, but excluded because the posting states no season anywhere in title or body.</v>
+        <v>2026-10-08 ~07:00 UTC: CAPTCHA cleared this run, direct fetch succeeded. Confirmed directly (not inferred from a blocked page): Mechanical Engineering Co-Op, Metals division (mechanical testing of metallic materials), Henderson NV, relocation authorized — but the posting states no season anywhere in the body (no month/year/term wording at all). Exclusion reason is now confirmed first-hand rather than assumed; disposition unchanged. Also resolved the long-standing ambiguous 'Quality Engineering Co-Op, Spring 2027' lead this run: direct fetch of oppid 22134 confirms it is the exact same posting already tracked in `rows` (Precision Castparts Corp / Airfoils Mentor-Painesville) — university-mirror and Dice sightings of that title all point to this one req, not a second distinct posting. No separate entry needed.</v>
       </c>
     </row>
     <row r="897">
@@ -25094,9 +25094,163 @@
         <v>2026-10-08: season is explicitly 'Winter 2027,' not 'Winter 2026' — same near-miss exclusion this tracker has already applied to Astranis/Skydio 'Winter 2027' cohorts. Not added.</v>
       </c>
     </row>
+    <row r="903">
+      <c r="A903" t="str">
+        <v>BMW Group (Spartanburg, SC)</v>
+      </c>
+      <c r="B903" t="str">
+        <v>Innovation and Digitalization Co-op (Spring 2027), req 190505</v>
+      </c>
+      <c r="C903" t="str">
+        <v>2026-10-08: confirmed OPEN via direct fetch (Apply now button, posted 2026-08-27) but discipline is Data Science / GenAI / Robotics-and-Automation software strategy, not mechanical/manufacturing/industrial engineering. Not added — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="str">
+        <v>BMW Group (Spartanburg, SC)</v>
+      </c>
+      <c r="B904" t="str">
+        <v>Launch &amp; Change Coordination Co-Op (Spring 2027), req 191158</v>
+      </c>
+      <c r="C904" t="str">
+        <v>2026-10-08: confirmed CLOSED via direct fetch ('You can't view this job because it's not available at this time'). Not added.</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="str">
+        <v>BMW Group (Spartanburg, SC)</v>
+      </c>
+      <c r="B905" t="str">
+        <v>Launch Planning and Steering Co-op (Spring 2027), req 190965</v>
+      </c>
+      <c r="C905" t="str">
+        <v>2026-10-08: confirmed CLOSED via direct fetch ('You can't view this job because it's not available at this time'). Not added.</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="str">
+        <v>BMW Group (Spartanburg, SC)</v>
+      </c>
+      <c r="B906" t="str">
+        <v>Quality Data Co-op (Spring 2027)</v>
+      </c>
+      <c r="C906" t="str">
+        <v>2026-10-08: confirmed OPEN via direct fetch (Apply now, posted 2026-08-12). Lists EE/CS/Mechanical/Industrial Engineering/Data Science as eligible majors, but day-to-day work is building quality-data dashboards/software tools for Assembly/Test/Finish/Rework/New Model Launch. Not added — discipline mismatch (data/software-centric), consistent with this tracker's precedent of excluding analytics-centric roles despite accepting ME majors.</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="str">
+        <v>BMW Group (Spartanburg, SC)</v>
+      </c>
+      <c r="B907" t="str">
+        <v>Packaging Development Intern (Spring 2027), req 191425</v>
+      </c>
+      <c r="C907" t="str">
+        <v>2026-10-08: confirmed OPEN via direct fetch (Apply now button). Eligible majors include Packaging/Mechanical Engineering/Supply Chain-Logistics, but the work is packaging planning/analysis, environmental-cost reduction, and moderating packaging reviews. Not added — discipline mismatch (packaging/logistics).</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="str">
+        <v>GE Aerospace (Rutland, VT)</v>
+      </c>
+      <c r="B908" t="str">
+        <v>Environmental/Health/Safety, Facilities, &amp; Maintenance Co-op - US - Spring 2027</v>
+      </c>
+      <c r="C908" t="str">
+        <v>2026-10-08: found alongside the Rutland VT 'Manufacturing Engineering Co-op' lead (same VermontJobLink listing range) — discipline is EHS/Facilities/Maintenance, not mechanical/manufacturing engineering. Not added. (Note: the Rutland VT Manufacturing Engineering Co-op itself is NOT a new/separate req — already resolved on 2026-10-08 ~01:00 UTC as the same company-wide req R5029663 already tracked in `rows`, which lists Rutland VT and Batesville AR among 23 selectable additionalLocations. A VermontJobLink state-board mirror of that same req, last updated 2026-10-07, was found today but does not represent a new posting.)</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="str">
+        <v>Formlabs (Somerville, MA)</v>
+      </c>
+      <c r="B909" t="str">
+        <v>Industrial Design Intern (Winter/Spring 2027), id 8172232</v>
+      </c>
+      <c r="C909" t="str">
+        <v>2026-10-08: confirmed open via direct Greenhouse API fetch, but this is Industrial *Design* (product design), not Industrial *Engineering*. Not added — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="str">
+        <v>Formlabs (Somerville, MA)</v>
+      </c>
+      <c r="B910" t="str">
+        <v>Global Operations Intern (Winter/Spring 2027), id 8263054</v>
+      </c>
+      <c r="C910" t="str">
+        <v>2026-10-08: confirmed open via direct Greenhouse API fetch; operations/supply-chain discipline. Not added — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="str">
+        <v>Formlabs (Somerville, MA)</v>
+      </c>
+      <c r="B911" t="str">
+        <v>Global Sourcing Intern (Winter/Spring 2027), id 8161780</v>
+      </c>
+      <c r="C911" t="str">
+        <v>2026-10-08: confirmed open via direct Greenhouse API fetch; sourcing/supply-chain discipline. Not added — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="str">
+        <v>Formlabs (Somerville, MA)</v>
+      </c>
+      <c r="B912" t="str">
+        <v>Sourcing Program Management Intern (Winter/Spring 2027), id 8262987</v>
+      </c>
+      <c r="C912" t="str">
+        <v>2026-10-08: confirmed open via direct Greenhouse API fetch; sourcing/program-management discipline. Not added — discipline mismatch.</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="str">
+        <v>ANYbotics</v>
+      </c>
+      <c r="B913" t="str">
+        <v>Mechanical Engineering and Mechatronics Engineering internships (multiple, live)</v>
+      </c>
+      <c r="C913" t="str">
+        <v>2026-10-08: new company (legged/quadruped inspection robotics, Series B-backed) confirmed via direct Lever API fetch (jobs.lever.co/anybotics) — live, discipline-fitting internships exist, but every posting and the company's only offices are in Zurich, Switzerland. Not added — outside Hamza's US-only location requirement.</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="str">
+        <v>Quaise Energy (Houston, TX / Malden, MA)</v>
+      </c>
+      <c r="B914" t="str">
+        <v>'Future Internship Opportunities' generic posting + full-time ME reqs</v>
+      </c>
+      <c r="C914" t="str">
+        <v>2026-10-08: new company (geothermal drilling hardware) confirmed via direct fetch of its own Greenhouse board (9 open reqs). The only internship-titled posting is a generic 'Future Internship Opportunities' req with no stated season/year anywhere — fails the explicit-season bar. Its two mechanical-discipline reqs (Jr. Mechanical CAD Designer, Mechanical Engineer II) are full-time, not internships. Not added.</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="str">
+        <v>Natron Energy (Santa Clara CA / Holland MI / Edgecombe NC)</v>
+      </c>
+      <c r="B915" t="str">
+        <v>full company board sweep</v>
+      </c>
+      <c r="C915" t="str">
+        <v>2026-10-08: new company (sodium-ion battery manufacturing) — zero internship/co-op-titled postings found anywhere; only full-time roles (Mechanical/Manufacturing Engineer, Senior Product Design Engineer, Manufacturing Associates). No internship program currently appears to exist. Not added.</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="str">
+        <v>Span.io (San Francisco, CA)</v>
+      </c>
+      <c r="B916" t="str">
+        <v>careers/job-board pages</v>
+      </c>
+      <c r="C916" t="str">
+        <v>2026-10-08: new company (smart electrical panel/grid-hardware manufacturing) — direct fetch of span.io/careers and span.io/job-board surfaced no job titles or internship/co-op postings of any kind. Not added.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C902"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C916"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 0 new postings, 2 checked-excluded (2026-10-08 13:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfjmPmsXLJCyC7CL4ACZS4
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -15174,7 +15174,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C916"/>
+  <dimension ref="A1:C918"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -25248,9 +25248,31 @@
         <v>2026-10-08: new company (smart electrical panel/grid-hardware manufacturing) — direct fetch of span.io/careers and span.io/job-board surfaced no job titles or internship/co-op postings of any kind. Not added.</v>
       </c>
     </row>
+    <row r="917">
+      <c r="A917" t="str">
+        <v>Alaka'i Technologies (Stow, MA)</v>
+      </c>
+      <c r="B917" t="str">
+        <v>Engineering Intern (hydrogen aircraft/powerplants, mechanical/electrical/software/aerospace scope), posted under 'SKAI Technology' listing name on Built In Boston</v>
+      </c>
+      <c r="C917" t="str">
+        <v>2026-10-08 ~13:00 UTC: new company (hydrogen eVTOL aircraft startup, Stow MA — close to Boston). Direct fetch confirmed the posting is explicitly for the '2026 Fall Semester' (wrong season) and the listing itself shows removed/closed as of Aug 10, 2026. Not added — wrong season and confirmed closed. Worth checking back for a Spring 2027 cohort, since this is a genuine Boston-area aerospace fit on discipline/location.</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="str">
+        <v>Cirrus Aircraft (Duluth, MN)</v>
+      </c>
+      <c r="B918" t="str">
+        <v>'Co-Op Sustaining Engineering Intern' (production-line engineering support)</v>
+      </c>
+      <c r="C918" t="str">
+        <v>2026-10-08 ~13:00 UTC: new company lead from a national sweep. The only link found (jobs.solidprofessor.com mirror) returned HTTP 404 on direct fetch; no working primary-source URL or stated season/year could be located for this exact title. Not added — fails the direct-verification and explicit-season bars. Worth a dedicated check of Cirrus's own careers site in a future run.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C916"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C918"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 3 new postings, 12 checked-excluded (2026-10-09 01:00 UTC)
Added BMW Group Additive Manufacturing Co-op (Spartanburg SC), Thornton
Tomasetti Structural Engineer Co-op (NYC), and RTX Collins Aerospace
Mechanical Engineering Co-Op (Portsmouth RI, flagged for its active
security clearance requirement). Excluded 12 checked/ruled-out leads
including PR-residency RTX reqs, season-label and discipline mismatches,
and several newly-swept companies with no qualifying postings.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PcBeJD1Vj2A4PGUm67WcbH
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M401"/>
+  <dimension ref="A1:M404"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -14697,6 +14697,102 @@
       </c>
       <c r="J401" t="str">
         <v>Hybrid quality/process engineering role. Same eligibility requirements as sibling Spartanburg SC co-ops above.</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>BMW Group</v>
+      </c>
+      <c r="B402" t="str">
+        <v>Additive Manufacturing Co-op (Spring 2027)</v>
+      </c>
+      <c r="C402" t="str">
+        <v>Manufacturing Engineering</v>
+      </c>
+      <c r="D402" t="str">
+        <v>Spring 2027 (Jan 11 – May 14, 2027)</v>
+      </c>
+      <c r="E402" t="str">
+        <v>Spartanburg, SC</v>
+      </c>
+      <c r="F402">
+        <v>850</v>
+      </c>
+      <c r="G402" t="str">
+        <v>Not stated</v>
+      </c>
+      <c r="H402" t="str">
+        <v>https://jobs.bmwgroup.com/job/Additive-Manufacturing-Co-op-%28Spring-2027%29/191077-en_US/</v>
+      </c>
+      <c r="I402" t="str">
+        <v>Yes — fetched the live posting directly on jobs.bmwgroup.com, two 'Apply now' buttons present, no closed/filled messaging (checked 2026-10-09).</v>
+      </c>
+      <c r="J402" t="str">
+        <v>Found in the same Spartanburg SC Spring 2027 co-op batch as the other 4 already-tracked BMW reqs. Posting start date 7/31/26; no closing date shown. Same eligibility pattern expected as sibling Spartanburg co-ops (not independently re-confirmed on this req).</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>Thornton Tomasetti, Inc.</v>
+      </c>
+      <c r="B403" t="str">
+        <v>Structural Engineer Co-op (Forensics Practice)</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Structural Engineering</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Spring 2027</v>
+      </c>
+      <c r="E403" t="str">
+        <v>New York, NY</v>
+      </c>
+      <c r="F403">
+        <v>190</v>
+      </c>
+      <c r="G403" t="str">
+        <v>$25.00–$35.00/hr (NY Pay Transparency Law good-faith estimate)</v>
+      </c>
+      <c r="H403" t="str">
+        <v>https://jobs.solidprofessor.com/job/372823/structural-engineer-co-op/</v>
+      </c>
+      <c r="I403" t="str">
+        <v>Yes — fetched the live posting directly, 'Apply Now' present, no closed/filled messaging, independently re-confirmed by this session (not just the research agent). Listing date Sep 16, 2026. Could not confirm the literal destination URL behind the Apply button (site blocks non-browser requests to it), but this listing page itself is the genuine employer-side posting (explicit pay-transparency disclosure, recruiting-fraud warning naming ThorntonTomasetti.com).</v>
+      </c>
+      <c r="J403" t="str">
+        <v>Full-time, in-office co-op. Current undergrad/grad student in civil, structural, or architectural engineering; strong academic record; Revit/AutoCAD/analysis software a plus, not required.</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>RTX (Collins Aerospace)</v>
+      </c>
+      <c r="B404" t="str">
+        <v>Mechanical Engineering Co-Op (Winter/Spring 2027)</v>
+      </c>
+      <c r="C404" t="str">
+        <v>Mechanical Engineering</v>
+      </c>
+      <c r="D404" t="str">
+        <v>Winter/Spring 2027</v>
+      </c>
+      <c r="E404" t="str">
+        <v>Portsmouth, RI</v>
+      </c>
+      <c r="F404">
+        <v>65</v>
+      </c>
+      <c r="G404" t="str">
+        <v>$37,000–$82,000/yr (RTX co-op band)</v>
+      </c>
+      <c r="H404" t="str">
+        <v>https://globalhr.wd5.myworkdayjobs.com/REC_RTX_Ext_Gateway/job/US-RI-PORTSMOUTH-PS3--1847-W-Main-Rd--NIMITZ-WEST-BLDG/Mechanical-Engineering-Co-Op--Winter-Spring-2027-_01880887</v>
+      </c>
+      <c r="I404" t="str">
+        <v>Yes — fetched directly via RTX's own Workday CXS API (canApply:true), posted 2026-10-08. Req 01880887, Undersea &amp; Electronics Systems (UES) dept.</v>
+      </c>
+      <c r="J404" t="str">
+        <v>FLAG: posting states 'Active and existing security clearance required after day 1' — reads as requiring an ALREADY-HELD active clearance, a much harder bar than the usual RTX 'eligible to obtain a clearance' co-op language seen elsewhere in this tracker. Likely disqualifies most student applicants who don't already hold a clearance. Requires US citizenship. Bachelor's degree required by start date, 3-D modeling software experience required (CREO/PDM, GD&amp;T preferred), no GPA stated. Confirm clearance status before investing time in this application.</v>
       </c>
     </row>
   </sheetData>
@@ -15167,14 +15263,14 @@
     <hyperlink ref="M198" r:id="rId464"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M401"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M404"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C928"/>
+  <dimension ref="A1:C940"/>
   <cols>
     <col min="1" max="1" width="34.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -25380,9 +25476,141 @@
         <v>2026-10-08 ~13:00 UTC: new company lead from a national sweep. The only link found (jobs.solidprofessor.com mirror) returned HTTP 404 on direct fetch; no working primary-source URL or stated season/year could be located for this exact title. Not added — fails the direct-verification and explicit-season bars. Worth a dedicated check of Cirrus's own careers site in a future run.</v>
       </c>
     </row>
+    <row r="929">
+      <c r="A929" t="str">
+        <v>Thornton Tomasetti, Inc. (New York, NY)</v>
+      </c>
+      <c r="B929" t="str">
+        <v>Mechanical Engineer Co-op (Forensics Practice)</v>
+      </c>
+      <c r="C929" t="str">
+        <v>2026-10-09: new company (structural/forensic engineering consultancy). Confirmed live via direct fetch (jobs.solidprofessor.com, Apply Now present, listed Sep 16, 2026, $25-35/hr), but the posting explicitly states 'Winter 2027' — not 'Winter 2026' or 'Spring 2027' as literally worded. Not added — same near-miss season-label precedent as the WSP USA 'Winter 2027' exclusion (2026-10-08). Sibling 'Structural Engineer Co-op' req at the same employer, same posting batch, explicitly states 'Spring 2027' and WAS added to `rows`.</v>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="str">
+        <v>Thornton Tomasetti, Inc. (New York, NY)</v>
+      </c>
+      <c r="B930" t="str">
+        <v>Electrical Engineer Intern</v>
+      </c>
+      <c r="C930" t="str">
+        <v>2026-10-09: found in the same posting batch as the two Thornton Tomasetti co-ops above (one added to `rows`, one excluded for season). Discipline is electrical engineering, not one of Hamza's target disciplines. Not added — discipline mismatch; not independently verified for open/closed status since discipline already disqualifies it.</v>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="str">
+        <v>AECOM (Conshohocken, PA)</v>
+      </c>
+      <c r="B931" t="str">
+        <v>Structural Engineering Intern (AECOM Transportation / Structures — Bridges &amp; Walls group)</v>
+      </c>
+      <c r="C931" t="str">
+        <v>2026-10-09: new company. AECOM's own ATS (americas.aecom.jobs / campus.aecom.jobs) is JS-rendered and returned empty content on two direct-fetch attempts — could not independently confirm on the employer's own page. A secondary job-board copy (simplify.jobs) states the season as 'Spring 2027 and Summer 2027' (dual-eligible, not Spring-only) — fails the explicit single-season bar under the same precedent as the RTX/Collins Aerospace York NE and Cedar Rapids IA merged-Spring/Summer exclusions (2026-10-08). Also requires US citizenship, valid US driver's license, no visa sponsorship, no relocation assistance. Not added — season wording disqualifies regardless of the Partial-verification issue.</v>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="str">
+        <v>Celestica International LP (Austin, TX)</v>
+      </c>
+      <c r="B932" t="str">
+        <v>Student Intern, Mechanical Engineering, Req ID 140463</v>
+      </c>
+      <c r="C932" t="str">
+        <v>2026-10-09: new company (contract manufacturer). Confirmed live via direct fetch (careers.celestica.com), posted 2026-10-08, $24-30/hr, but posting explicitly states 'Start date: June 2027' — Summer 2027, wrong season. Not added. Worth a periodic re-check in case Celestica posts a Spring-dated co-op later in its cycle.</v>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="str">
+        <v>JR Automation / Dematic (Hitachi, KION Group) — Auburn Hills &amp; Holland, MI</v>
+      </c>
+      <c r="B933" t="str">
+        <v>Controls Engineering Intern/Co-Op</v>
+      </c>
+      <c r="C933" t="str">
+        <v>2026-10-09: new company. Found via Handshake/purpose.jobs, posted 2026-10-05, but posting explicitly states the working term runs 'May 2027 through August 2027' — Summer 2027, wrong season. Not added.</v>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="str">
+        <v>Dematic (KION Group) — Grand Rapids, MI</v>
+      </c>
+      <c r="B934" t="str">
+        <v>Electrical Controls Applications Engineering Intern/Co-Op</v>
+      </c>
+      <c r="C934" t="str">
+        <v>2026-10-09: new company. Found via BuiltIn/Teal listings; no start term or season stated anywhere on any copy located. Not added — fails the explicit-season bar. Flagging the company as new/unconfirmed in case a future run wants to check Dematic's own careers page directly.</v>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="str">
+        <v>NextStep Robotics (Baltimore, MD)</v>
+      </c>
+      <c r="B935" t="str">
+        <v>Mechanical Engineering Internship Position (AMBLE foot-drop ankle robot)</v>
+      </c>
+      <c r="C935" t="str">
+        <v>2026-10-09: new company (rehabilitation robotics startup). Only source found is a University of Maryland career-office repost (megrad.umd.edu) with no official company ATS link, no stated start term/season (rolling, 'flexible, capped at 40 hrs/week'), and no online apply mechanism — direct-email contact only. Not added — fails both the direct-verification and explicit-season bars.</v>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="str">
+        <v>Capella Space / Sidus Space / Ekso Bionics / Deep Fission</v>
+      </c>
+      <c r="B936" t="str">
+        <v>Full company board sweeps, 2026-10-09</v>
+      </c>
+      <c r="C936" t="str">
+        <v>New-to-tracker companies (space/satellite and exoskeleton/robotics hardware). Each checked directly against its own careers site/ATS where one could be located — no Winter 2026 or Spring 2027 mechanical/aerospace/robotics intern or co-op postings found at any of the four (either no internship titles at all, or only full-time/senior roles). None added.</v>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="str">
+        <v>RTX/Collins Aerospace — Santa Isabel, PR (Building B2)</v>
+      </c>
+      <c r="B937" t="str">
+        <v>Manufacturing Engineering Co-Op (Spring 2027)(Onsite), req 01878947</v>
+      </c>
+      <c r="C937" t="str">
+        <v>2026-10-09: found via RTX's own Workday CXS API full-text sweep (canApply:true, posted 2026-10-05). Posting explicitly states 'Candidates must reside in Puerto Rico during the CO-OP period' — same hard residency dealbreaker precedent as the already-excluded req 01874717 (Aguadilla, PR). Not added.</v>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="str">
+        <v>RTX/Collins Aerospace — Santa Isabel, PR (Building B1)</v>
+      </c>
+      <c r="B938" t="str">
+        <v>Manufacturing Engineering Co-Op (Spring 2027)(Onsite), req 01878937</v>
+      </c>
+      <c r="C938" t="str">
+        <v>2026-10-09: sibling req to 01878947 above, same site, same PR-residency requirement during the co-op period. Not added.</v>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="str">
+        <v>Draper Laboratory (Cambridge, MA)</v>
+      </c>
+      <c r="B939" t="str">
+        <v>Microsystems Integration Intern, req JR003002-1</v>
+      </c>
+      <c r="C939" t="str">
+        <v>2026-10-09: found via a fresh full paginated sweep of Draper's Workday CXS API (223 total postings). Confirmed live (canApply:true, posted 2026-10-07) but excluded on two independent grounds: (1) no season/year stated anywhere in the body (only 'flexibility regarding hours and program duration based on applicant's school schedule') — fails the explicit-season bar; (2) discipline is EE/Nuclear Engineering/Physics/Materials Science/Chemistry-focused (radiation effects in semiconductors, MEMS sensors, electro-optics), not mechanical/aerospace. Also restricted to U.S. citizens only (dual citizenship excluded). Not added.</v>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="str">
+        <v>MIT Lincoln Laboratory (Lexington, MA)</v>
+      </c>
+      <c r="B940" t="str">
+        <v>Advanced Sensors and Techniques Co-Op (Spring 2027) - Group 09-02</v>
+      </c>
+      <c r="C940" t="str">
+        <v>2026-10-09: new req, confirmed live via direct fetch (posted 2026-10-06, Apply now present). Eligible majors explicitly include 'Electrical Engineering, Physics, Computer Engineering, Aerospace Engineering, or other relevant technical field' — Aerospace Engineering is a named acceptable major, which is why this isn't silently dropped. However the actual work (radar/RF/EO space-surveillance-sensor design, antenna/RF/microwave integration, analog/digital circuit design, PCB prototyping, signal processing) reads as Electrical-Engineering-flavored, not mechanical/aerospace structural/systems work — same discipline-mismatch treatment already applied to other MIT LL/RTX postings that nominally list multiple acceptable majors. Requires Secret clearance eligibility, pay $25-32/hr, no GPA stated. BORDERLINE — flagged for Hamza's own judgment (same treatment as the RTX East Hartford Quality Co-op) rather than a unilateral exclusion, since Aerospace Engineering majors are explicitly welcomed on the posting. Not added to `rows` pending that call.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C928"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C940"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
routine: 1 new postings, 20 checked-excluded (2026-10-09 07:00 UTC)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AQLc6ttgLMFuvNMBmXw1kN
</commit_message>
<xml_diff>
--- a/Engineering-Internships-Winter2026-Spring2027.xlsx
+++ b/Engineering-Internships-Winter2026-Spring2027.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M404"/>
+  <dimension ref="A1:M405"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="46.83203125" customWidth="1"/>
@@ -14793,6 +14793,38 @@
       </c>
       <c r="J404" t="str">
         <v>FLAG: posting states 'Active and existing security clearance required after day 1' — reads as requiring an ALREADY-HELD active clearance, a much harder bar than the usual RTX 'eligible to obtain a clearance' co-op language seen elsew